<commit_message>
Force update data to Friday (2026-03-27) close
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -489,7 +489,7 @@
         <v>100</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="3">
@@ -519,7 +519,7 @@
         <v>100</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         <v>100</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="5">
@@ -579,7 +579,7 @@
         <v>100</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="6">
@@ -609,7 +609,7 @@
         <v>100</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="7">
@@ -639,7 +639,7 @@
         <v>100</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="8">
@@ -669,7 +669,7 @@
         <v>100</v>
       </c>
       <c r="H8" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="9">
@@ -699,7 +699,7 @@
         <v>100</v>
       </c>
       <c r="H9" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="10">
@@ -729,7 +729,7 @@
         <v>100</v>
       </c>
       <c r="H10" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="11">
@@ -759,7 +759,7 @@
         <v>100</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="12">
@@ -789,7 +789,7 @@
         <v>100</v>
       </c>
       <c r="H12" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="13">
@@ -819,7 +819,7 @@
         <v>100</v>
       </c>
       <c r="H13" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="14">
@@ -849,7 +849,7 @@
         <v>100</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="15">
@@ -879,7 +879,7 @@
         <v>100</v>
       </c>
       <c r="H15" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="16">
@@ -909,7 +909,7 @@
         <v>100</v>
       </c>
       <c r="H16" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="17">
@@ -939,7 +939,7 @@
         <v>100</v>
       </c>
       <c r="H17" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="18">
@@ -969,7 +969,7 @@
         <v>100</v>
       </c>
       <c r="H18" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="19">
@@ -999,7 +999,7 @@
         <v>100</v>
       </c>
       <c r="H19" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="20">
@@ -1029,7 +1029,7 @@
         <v>100</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="21">
@@ -1059,7 +1059,7 @@
         <v>100</v>
       </c>
       <c r="H21" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="22">
@@ -1089,7 +1089,7 @@
         <v>100</v>
       </c>
       <c r="H22" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="23">
@@ -1119,7 +1119,7 @@
         <v>100</v>
       </c>
       <c r="H23" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="24">
@@ -1149,7 +1149,7 @@
         <v>100</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="25">
@@ -1179,7 +1179,7 @@
         <v>100</v>
       </c>
       <c r="H25" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="26">
@@ -1209,7 +1209,7 @@
         <v>100</v>
       </c>
       <c r="H26" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="27">
@@ -1239,7 +1239,7 @@
         <v>100</v>
       </c>
       <c r="H27" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="28">
@@ -1269,7 +1269,7 @@
         <v>100</v>
       </c>
       <c r="H28" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="29">
@@ -1299,7 +1299,7 @@
         <v>100</v>
       </c>
       <c r="H29" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="30">
@@ -1329,7 +1329,7 @@
         <v>100</v>
       </c>
       <c r="H30" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="31">
@@ -1359,7 +1359,7 @@
         <v>100</v>
       </c>
       <c r="H31" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="32">
@@ -1389,7 +1389,7 @@
         <v>100</v>
       </c>
       <c r="H32" s="1" t="n">
-        <v>46111</v>
+        <v>46108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Apr  3 22:01:50 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,42 +433,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>行业代码</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>行业名称</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>TTM市盈率</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>市净率</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>PE分位%</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PB分位%</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>行业温度</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
@@ -465,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>21.71</v>
+        <v>15.84</v>
       </c>
       <c r="D2" t="n">
-        <v>2.37</v>
+        <v>1.28</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -488,26 +500,26 @@
       <c r="G2" t="n">
         <v>100</v>
       </c>
-      <c r="H2" s="1" t="n">
-        <v>46108</v>
+      <c r="H2" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.61</v>
+        <v>28.32</v>
       </c>
       <c r="D3" t="n">
-        <v>2.63</v>
+        <v>2.7</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -518,26 +530,26 @@
       <c r="G3" t="n">
         <v>100</v>
       </c>
-      <c r="H3" s="1" t="n">
-        <v>46108</v>
+      <c r="H3" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22.04</v>
+        <v>19.9</v>
       </c>
       <c r="D4" t="n">
-        <v>1.18</v>
+        <v>4.16</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
@@ -548,26 +560,26 @@
       <c r="G4" t="n">
         <v>100</v>
       </c>
-      <c r="H4" s="1" t="n">
-        <v>46108</v>
+      <c r="H4" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25.65</v>
+        <v>26.47</v>
       </c>
       <c r="D5" t="n">
-        <v>3.7</v>
+        <v>2.51</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
@@ -578,26 +590,26 @@
       <c r="G5" t="n">
         <v>100</v>
       </c>
-      <c r="H5" s="1" t="n">
-        <v>46108</v>
+      <c r="H5" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>55.11</v>
+        <v>26.55</v>
       </c>
       <c r="D6" t="n">
-        <v>5.18</v>
+        <v>1.54</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
@@ -608,668 +620,668 @@
       <c r="G6" t="n">
         <v>100</v>
       </c>
-      <c r="H6" s="1" t="n">
-        <v>46108</v>
+      <c r="H6" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25.07</v>
+        <v>6.93</v>
       </c>
       <c r="D7" t="n">
-        <v>2.45</v>
+        <v>0.67</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
-      </c>
-      <c r="H7" s="1" t="n">
-        <v>46108</v>
+        <v>87.5</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14.35</v>
+        <v>29.93</v>
       </c>
       <c r="D8" t="n">
-        <v>2.38</v>
+        <v>2.06</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
-      </c>
-      <c r="H8" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19.69</v>
+        <v>10.51</v>
       </c>
       <c r="D9" t="n">
-        <v>4.07</v>
+        <v>0.75</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
-      </c>
-      <c r="H9" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.6</v>
+        <v>23.93</v>
       </c>
       <c r="D10" t="n">
-        <v>1.76</v>
+        <v>2.26</v>
       </c>
       <c r="E10" t="n">
         <v>100</v>
       </c>
       <c r="F10" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>100</v>
-      </c>
-      <c r="H10" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>23.2</v>
+        <v>69.73999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>2.31</v>
+        <v>2.85</v>
       </c>
       <c r="E11" t="n">
         <v>100</v>
       </c>
       <c r="F11" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G11" t="n">
-        <v>100</v>
-      </c>
-      <c r="H11" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>27</v>
+        <v>33.9</v>
       </c>
       <c r="D12" t="n">
-        <v>2.62</v>
+        <v>2.86</v>
       </c>
       <c r="E12" t="n">
         <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G12" t="n">
-        <v>100</v>
-      </c>
-      <c r="H12" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.89</v>
+        <v>14.39</v>
       </c>
       <c r="D13" t="n">
-        <v>1.93</v>
+        <v>2.35</v>
       </c>
       <c r="E13" t="n">
         <v>100</v>
       </c>
       <c r="F13" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G13" t="n">
-        <v>100</v>
-      </c>
-      <c r="H13" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.44</v>
+        <v>26.51</v>
       </c>
       <c r="D14" t="n">
-        <v>1.26</v>
+        <v>3.63</v>
       </c>
       <c r="E14" t="n">
         <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G14" t="n">
-        <v>100</v>
-      </c>
-      <c r="H14" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>32.29</v>
+        <v>19.59</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.76</v>
       </c>
       <c r="E15" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F15" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G15" t="n">
-        <v>100</v>
-      </c>
-      <c r="H15" s="1" t="n">
-        <v>46108</v>
+        <v>62.5</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30.85</v>
+        <v>53.85</v>
       </c>
       <c r="D16" t="n">
-        <v>2.04</v>
+        <v>5.02</v>
       </c>
       <c r="E16" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F16" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G16" t="n">
-        <v>100</v>
-      </c>
-      <c r="H16" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>35</v>
+        <v>30.77</v>
       </c>
       <c r="D17" t="n">
-        <v>2.62</v>
+        <v>0.9</v>
       </c>
       <c r="E17" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F17" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G17" t="n">
-        <v>100</v>
-      </c>
-      <c r="H17" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6.84</v>
+        <v>18.53</v>
       </c>
       <c r="D18" t="n">
-        <v>0.67</v>
+        <v>1.79</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G18" t="n">
-        <v>100</v>
-      </c>
-      <c r="H18" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.29</v>
+        <v>22.89</v>
       </c>
       <c r="D19" t="n">
-        <v>1.31</v>
+        <v>2.24</v>
       </c>
       <c r="E19" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F19" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G19" t="n">
-        <v>100</v>
-      </c>
-      <c r="H19" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>58.93</v>
+        <v>24.12</v>
       </c>
       <c r="D20" t="n">
-        <v>2.91</v>
+        <v>2.37</v>
       </c>
       <c r="E20" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F20" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G20" t="n">
-        <v>100</v>
-      </c>
-      <c r="H20" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>25.89</v>
+        <v>21.89</v>
       </c>
       <c r="D21" t="n">
-        <v>1.51</v>
+        <v>1.16</v>
       </c>
       <c r="E21" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F21" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G21" t="n">
-        <v>100</v>
-      </c>
-      <c r="H21" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9.77</v>
+        <v>27.09</v>
       </c>
       <c r="D22" t="n">
-        <v>0.77</v>
+        <v>2.53</v>
       </c>
       <c r="E22" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F22" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G22" t="n">
-        <v>100</v>
-      </c>
-      <c r="H22" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>35.1</v>
+        <v>10.1</v>
       </c>
       <c r="D23" t="n">
-        <v>3.9</v>
+        <v>1.28</v>
       </c>
       <c r="E23" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F23" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>100</v>
-      </c>
-      <c r="H23" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>33.68</v>
+        <v>32.92</v>
       </c>
       <c r="D24" t="n">
-        <v>2.91</v>
+        <v>2.54</v>
       </c>
       <c r="E24" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F24" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H24" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>74.81999999999999</v>
+        <v>32.46</v>
       </c>
       <c r="D25" t="n">
-        <v>4.04</v>
+        <v>3.56</v>
       </c>
       <c r="E25" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F25" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G25" t="n">
-        <v>100</v>
-      </c>
-      <c r="H25" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>48.96</v>
+        <v>69.88</v>
       </c>
       <c r="D26" t="n">
-        <v>4.25</v>
+        <v>3.94</v>
       </c>
       <c r="E26" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F26" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H26" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25.7</v>
+        <v>48.73</v>
       </c>
       <c r="D27" t="n">
-        <v>2.31</v>
+        <v>4.11</v>
       </c>
       <c r="E27" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F27" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H27" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25.75</v>
+        <v>25.28</v>
       </c>
       <c r="D28" t="n">
-        <v>2.44</v>
+        <v>2.27</v>
       </c>
       <c r="E28" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F28" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G28" t="n">
-        <v>100</v>
-      </c>
-      <c r="H28" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="29">
@@ -1284,22 +1296,22 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>19.12</v>
+        <v>18.43</v>
       </c>
       <c r="D29" t="n">
-        <v>1.86</v>
+        <v>1.78</v>
       </c>
       <c r="E29" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F29" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G29" t="n">
-        <v>100</v>
-      </c>
-      <c r="H29" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="30">
@@ -1314,22 +1326,22 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>16.77</v>
+        <v>16.65</v>
       </c>
       <c r="D30" t="n">
-        <v>1.58</v>
+        <v>1.55</v>
       </c>
       <c r="E30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G30" t="n">
-        <v>100</v>
-      </c>
-      <c r="H30" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="31">
@@ -1344,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>24.43</v>
+        <v>23.49</v>
       </c>
       <c r="D31" t="n">
-        <v>1.72</v>
+        <v>1.64</v>
       </c>
       <c r="E31" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F31" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G31" t="n">
-        <v>100</v>
-      </c>
-      <c r="H31" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
     <row r="32">
@@ -1374,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>31.22</v>
+        <v>31.17</v>
       </c>
       <c r="D32" t="n">
-        <v>2.78</v>
+        <v>2.73</v>
       </c>
       <c r="E32" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F32" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G32" t="n">
-        <v>100</v>
-      </c>
-      <c r="H32" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>46115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Apr  4 11:03:52 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>1.28</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.7</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>4.16</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.51</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.54</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>0.67</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F7" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="G7" t="n">
         <v>75</v>
       </c>
-      <c r="G7" t="n">
-        <v>87.5</v>
-      </c>
       <c r="H7" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="8">
@@ -675,13 +675,13 @@
         <v>50</v>
       </c>
       <c r="F8" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G8" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>0.75</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F9" t="n">
         <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.26</v>
       </c>
       <c r="E10" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F10" t="n">
         <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.85</v>
       </c>
       <c r="E11" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F11" t="n">
         <v>50</v>
       </c>
       <c r="G11" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.86</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F12" t="n">
         <v>50</v>
       </c>
       <c r="G12" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>2.35</v>
       </c>
       <c r="E13" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F13" t="n">
         <v>50</v>
       </c>
       <c r="G13" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>3.63</v>
       </c>
       <c r="E14" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F14" t="n">
         <v>50</v>
       </c>
       <c r="G14" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="15">
@@ -885,13 +885,13 @@
         <v>50</v>
       </c>
       <c r="F15" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="G15" t="n">
-        <v>62.5</v>
+        <v>58.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="16">
@@ -921,7 +921,7 @@
         <v>50</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="17">
@@ -951,7 +951,7 @@
         <v>50</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="18">
@@ -981,7 +981,7 @@
         <v>50</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="19">
@@ -1011,7 +1011,7 @@
         <v>50</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="20">
@@ -1041,7 +1041,7 @@
         <v>50</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="21">
@@ -1071,7 +1071,7 @@
         <v>50</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="22">
@@ -1101,7 +1101,7 @@
         <v>50</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="23">
@@ -1131,7 +1131,7 @@
         <v>50</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="24">
@@ -1161,7 +1161,7 @@
         <v>50</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="25">
@@ -1191,7 +1191,7 @@
         <v>50</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="26">
@@ -1221,7 +1221,7 @@
         <v>50</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="27">
@@ -1251,7 +1251,7 @@
         <v>50</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="28">
@@ -1281,7 +1281,7 @@
         <v>50</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="29">
@@ -1311,7 +1311,7 @@
         <v>50</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="30">
@@ -1341,7 +1341,7 @@
         <v>50</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="31">
@@ -1371,7 +1371,7 @@
         <v>50</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
     <row r="32">
@@ -1401,7 +1401,7 @@
         <v>50</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Apr  5 11:05:22 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>1.28</v>
       </c>
       <c r="E2" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F2" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G2" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.7</v>
       </c>
       <c r="E3" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F3" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G3" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>4.16</v>
       </c>
       <c r="E4" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F4" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G4" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.51</v>
       </c>
       <c r="E5" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G5" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.54</v>
       </c>
       <c r="E6" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G6" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>0.67</v>
       </c>
       <c r="E7" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F7" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="G7" t="n">
-        <v>75</v>
+        <v>68.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="8">
@@ -675,13 +675,13 @@
         <v>50</v>
       </c>
       <c r="F8" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G8" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>0.75</v>
       </c>
       <c r="E9" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F9" t="n">
         <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.26</v>
       </c>
       <c r="E10" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F10" t="n">
         <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.85</v>
       </c>
       <c r="E11" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F11" t="n">
         <v>50</v>
       </c>
       <c r="G11" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.86</v>
       </c>
       <c r="E12" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F12" t="n">
         <v>50</v>
       </c>
       <c r="G12" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>2.35</v>
       </c>
       <c r="E13" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F13" t="n">
         <v>50</v>
       </c>
       <c r="G13" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>3.63</v>
       </c>
       <c r="E14" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F14" t="n">
         <v>50</v>
       </c>
       <c r="G14" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="15">
@@ -885,13 +885,13 @@
         <v>50</v>
       </c>
       <c r="F15" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="G15" t="n">
-        <v>58.3</v>
+        <v>56.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="16">
@@ -921,7 +921,7 @@
         <v>50</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="17">
@@ -951,7 +951,7 @@
         <v>50</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="18">
@@ -981,7 +981,7 @@
         <v>50</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="19">
@@ -1011,7 +1011,7 @@
         <v>50</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="20">
@@ -1041,7 +1041,7 @@
         <v>50</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="21">
@@ -1071,7 +1071,7 @@
         <v>50</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="22">
@@ -1101,7 +1101,7 @@
         <v>50</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="23">
@@ -1131,7 +1131,7 @@
         <v>50</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="24">
@@ -1161,7 +1161,7 @@
         <v>50</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="25">
@@ -1191,7 +1191,7 @@
         <v>50</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="26">
@@ -1221,7 +1221,7 @@
         <v>50</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="27">
@@ -1251,7 +1251,7 @@
         <v>50</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="28">
@@ -1281,7 +1281,7 @@
         <v>50</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="29">
@@ -1311,7 +1311,7 @@
         <v>50</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="30">
@@ -1341,7 +1341,7 @@
         <v>50</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="31">
@@ -1371,7 +1371,7 @@
         <v>50</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="32">
@@ -1401,7 +1401,7 @@
         <v>50</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Apr 10 22:01:38 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,42 +433,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>行业代码</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>行业名称</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>TTM市盈率</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>市净率</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>PE分位%</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PB分位%</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>行业温度</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
@@ -465,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>21.71</v>
+        <v>22.19</v>
       </c>
       <c r="D2" t="n">
-        <v>2.37</v>
+        <v>1.19</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -488,26 +500,26 @@
       <c r="G2" t="n">
         <v>100</v>
       </c>
-      <c r="H2" s="1" t="n">
-        <v>46108</v>
+      <c r="H2" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.61</v>
+        <v>59.49</v>
       </c>
       <c r="D3" t="n">
-        <v>2.63</v>
+        <v>5.55</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -518,26 +530,26 @@
       <c r="G3" t="n">
         <v>100</v>
       </c>
-      <c r="H3" s="1" t="n">
-        <v>46108</v>
+      <c r="H3" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22.04</v>
+        <v>27.98</v>
       </c>
       <c r="D4" t="n">
-        <v>1.18</v>
+        <v>3.84</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
@@ -548,26 +560,26 @@
       <c r="G4" t="n">
         <v>100</v>
       </c>
-      <c r="H4" s="1" t="n">
-        <v>46108</v>
+      <c r="H4" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25.65</v>
+        <v>25.17</v>
       </c>
       <c r="D5" t="n">
-        <v>3.7</v>
+        <v>2.48</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
@@ -578,26 +590,26 @@
       <c r="G5" t="n">
         <v>100</v>
       </c>
-      <c r="H5" s="1" t="n">
-        <v>46108</v>
+      <c r="H5" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>55.11</v>
+        <v>14.68</v>
       </c>
       <c r="D6" t="n">
-        <v>5.18</v>
+        <v>2.4</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
@@ -608,26 +620,26 @@
       <c r="G6" t="n">
         <v>100</v>
       </c>
-      <c r="H6" s="1" t="n">
-        <v>46108</v>
+      <c r="H6" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25.07</v>
+        <v>20.05</v>
       </c>
       <c r="D7" t="n">
-        <v>2.45</v>
+        <v>1.81</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
@@ -638,26 +650,26 @@
       <c r="G7" t="n">
         <v>100</v>
       </c>
-      <c r="H7" s="1" t="n">
-        <v>46108</v>
+      <c r="H7" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14.35</v>
+        <v>19.85</v>
       </c>
       <c r="D8" t="n">
-        <v>2.38</v>
+        <v>4.15</v>
       </c>
       <c r="E8" t="n">
         <v>100</v>
@@ -668,26 +680,26 @@
       <c r="G8" t="n">
         <v>100</v>
       </c>
-      <c r="H8" s="1" t="n">
-        <v>46108</v>
+      <c r="H8" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19.69</v>
+        <v>15.84</v>
       </c>
       <c r="D9" t="n">
-        <v>4.07</v>
+        <v>1.28</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
@@ -698,26 +710,26 @@
       <c r="G9" t="n">
         <v>100</v>
       </c>
-      <c r="H9" s="1" t="n">
-        <v>46108</v>
+      <c r="H9" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.6</v>
+        <v>30.87</v>
       </c>
       <c r="D10" t="n">
-        <v>1.76</v>
+        <v>2.12</v>
       </c>
       <c r="E10" t="n">
         <v>100</v>
@@ -728,8 +740,8 @@
       <c r="G10" t="n">
         <v>100</v>
       </c>
-      <c r="H10" s="1" t="n">
-        <v>46108</v>
+      <c r="H10" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="11">
@@ -744,10 +756,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>23.2</v>
+        <v>23.76</v>
       </c>
       <c r="D11" t="n">
-        <v>2.31</v>
+        <v>2.32</v>
       </c>
       <c r="E11" t="n">
         <v>100</v>
@@ -758,8 +770,8 @@
       <c r="G11" t="n">
         <v>100</v>
       </c>
-      <c r="H11" s="1" t="n">
-        <v>46108</v>
+      <c r="H11" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="12">
@@ -774,10 +786,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>27</v>
+        <v>28.58</v>
       </c>
       <c r="D12" t="n">
-        <v>2.62</v>
+        <v>2.72</v>
       </c>
       <c r="E12" t="n">
         <v>100</v>
@@ -788,26 +800,26 @@
       <c r="G12" t="n">
         <v>100</v>
       </c>
-      <c r="H12" s="1" t="n">
-        <v>46108</v>
+      <c r="H12" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.89</v>
+        <v>27.75</v>
       </c>
       <c r="D13" t="n">
-        <v>1.93</v>
+        <v>1.64</v>
       </c>
       <c r="E13" t="n">
         <v>100</v>
@@ -818,26 +830,26 @@
       <c r="G13" t="n">
         <v>100</v>
       </c>
-      <c r="H13" s="1" t="n">
-        <v>46108</v>
+      <c r="H13" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.44</v>
+        <v>10.85</v>
       </c>
       <c r="D14" t="n">
-        <v>1.26</v>
+        <v>0.78</v>
       </c>
       <c r="E14" t="n">
         <v>100</v>
@@ -848,26 +860,26 @@
       <c r="G14" t="n">
         <v>100</v>
       </c>
-      <c r="H14" s="1" t="n">
-        <v>46108</v>
+      <c r="H14" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>32.29</v>
+        <v>10.42</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.32</v>
       </c>
       <c r="E15" t="n">
         <v>100</v>
@@ -878,26 +890,26 @@
       <c r="G15" t="n">
         <v>100</v>
       </c>
-      <c r="H15" s="1" t="n">
-        <v>46108</v>
+      <c r="H15" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30.85</v>
+        <v>99.73999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>2.04</v>
+        <v>2.95</v>
       </c>
       <c r="E16" t="n">
         <v>100</v>
@@ -908,26 +920,26 @@
       <c r="G16" t="n">
         <v>100</v>
       </c>
-      <c r="H16" s="1" t="n">
-        <v>46108</v>
+      <c r="H16" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>35</v>
+        <v>36.2</v>
       </c>
       <c r="D17" t="n">
-        <v>2.62</v>
+        <v>3.05</v>
       </c>
       <c r="E17" t="n">
         <v>100</v>
@@ -938,26 +950,26 @@
       <c r="G17" t="n">
         <v>100</v>
       </c>
-      <c r="H17" s="1" t="n">
-        <v>46108</v>
+      <c r="H17" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6.84</v>
+        <v>28.25</v>
       </c>
       <c r="D18" t="n">
-        <v>0.67</v>
+        <v>2.68</v>
       </c>
       <c r="E18" t="n">
         <v>100</v>
@@ -968,26 +980,26 @@
       <c r="G18" t="n">
         <v>100</v>
       </c>
-      <c r="H18" s="1" t="n">
-        <v>46108</v>
+      <c r="H18" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.29</v>
+        <v>26.76</v>
       </c>
       <c r="D19" t="n">
-        <v>1.31</v>
+        <v>2.38</v>
       </c>
       <c r="E19" t="n">
         <v>100</v>
@@ -998,26 +1010,26 @@
       <c r="G19" t="n">
         <v>100</v>
       </c>
-      <c r="H19" s="1" t="n">
-        <v>46108</v>
+      <c r="H19" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>58.93</v>
+        <v>51.75</v>
       </c>
       <c r="D20" t="n">
-        <v>2.91</v>
+        <v>4.35</v>
       </c>
       <c r="E20" t="n">
         <v>100</v>
@@ -1028,368 +1040,368 @@
       <c r="G20" t="n">
         <v>100</v>
       </c>
-      <c r="H20" s="1" t="n">
-        <v>46108</v>
+      <c r="H20" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>25.89</v>
+        <v>28.61</v>
       </c>
       <c r="D21" t="n">
-        <v>1.51</v>
+        <v>2.68</v>
       </c>
       <c r="E21" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>100</v>
-      </c>
-      <c r="H21" s="1" t="n">
-        <v>46108</v>
+        <v>87.5</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9.77</v>
+        <v>31.43</v>
       </c>
       <c r="D22" t="n">
-        <v>0.77</v>
+        <v>2.76</v>
       </c>
       <c r="E22" t="n">
         <v>100</v>
       </c>
       <c r="F22" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G22" t="n">
-        <v>100</v>
-      </c>
-      <c r="H22" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>35.1</v>
+        <v>24.43</v>
       </c>
       <c r="D23" t="n">
-        <v>3.9</v>
+        <v>2.3</v>
       </c>
       <c r="E23" t="n">
         <v>100</v>
       </c>
       <c r="F23" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>100</v>
-      </c>
-      <c r="H23" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>33.68</v>
+        <v>72.8</v>
       </c>
       <c r="D24" t="n">
-        <v>2.91</v>
+        <v>4.1</v>
       </c>
       <c r="E24" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F24" t="n">
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H24" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>74.81999999999999</v>
+        <v>34.13</v>
       </c>
       <c r="D25" t="n">
-        <v>4.04</v>
+        <v>2.62</v>
       </c>
       <c r="E25" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F25" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G25" t="n">
-        <v>100</v>
-      </c>
-      <c r="H25" s="1" t="n">
-        <v>46108</v>
+        <v>62.5</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>48.96</v>
+        <v>24.39</v>
       </c>
       <c r="D26" t="n">
-        <v>4.25</v>
+        <v>1.72</v>
       </c>
       <c r="E26" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F26" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H26" s="1" t="n">
-        <v>46108</v>
+        <v>62.5</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25.7</v>
+        <v>30.96</v>
       </c>
       <c r="D27" t="n">
-        <v>2.31</v>
+        <v>0.92</v>
       </c>
       <c r="E27" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F27" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H27" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25.75</v>
+        <v>18.59</v>
       </c>
       <c r="D28" t="n">
-        <v>2.44</v>
+        <v>1.79</v>
       </c>
       <c r="E28" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F28" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G28" t="n">
-        <v>100</v>
-      </c>
-      <c r="H28" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>19.12</v>
+        <v>34.74</v>
       </c>
       <c r="D29" t="n">
-        <v>1.86</v>
+        <v>3.81</v>
       </c>
       <c r="E29" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F29" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G29" t="n">
-        <v>100</v>
-      </c>
-      <c r="H29" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>16.77</v>
+        <v>6.79</v>
       </c>
       <c r="D30" t="n">
-        <v>1.58</v>
+        <v>0.66</v>
       </c>
       <c r="E30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G30" t="n">
-        <v>100</v>
-      </c>
-      <c r="H30" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>24.43</v>
+        <v>16.4</v>
       </c>
       <c r="D31" t="n">
-        <v>1.72</v>
+        <v>1.53</v>
       </c>
       <c r="E31" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F31" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G31" t="n">
-        <v>100</v>
-      </c>
-      <c r="H31" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>31.22</v>
+        <v>18.4</v>
       </c>
       <c r="D32" t="n">
-        <v>2.78</v>
+        <v>1.75</v>
       </c>
       <c r="E32" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F32" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G32" t="n">
-        <v>100</v>
-      </c>
-      <c r="H32" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>46122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Apr 11 11:06:16 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>1.19</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>5.55</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.84</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.48</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.4</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.81</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F7" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>4.15</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F8" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.28</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F9" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.12</v>
       </c>
       <c r="E10" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F10" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G10" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.32</v>
       </c>
       <c r="E11" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F11" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G11" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.72</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F12" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G12" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.64</v>
       </c>
       <c r="E13" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F13" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G13" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>0.78</v>
       </c>
       <c r="E14" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F14" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G14" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.32</v>
       </c>
       <c r="E15" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F15" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G15" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.95</v>
       </c>
       <c r="E16" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F16" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G16" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.05</v>
       </c>
       <c r="E17" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F17" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G17" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.68</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G18" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.38</v>
       </c>
       <c r="E19" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F19" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G19" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>4.35</v>
       </c>
       <c r="E20" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F20" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G20" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.68</v>
       </c>
       <c r="E21" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F21" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="G21" t="n">
         <v>75</v>
       </c>
-      <c r="F21" t="n">
-        <v>100</v>
-      </c>
-      <c r="G21" t="n">
-        <v>87.5</v>
-      </c>
       <c r="H21" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.76</v>
       </c>
       <c r="E22" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F22" t="n">
         <v>50</v>
       </c>
       <c r="G22" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.3</v>
       </c>
       <c r="E23" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F23" t="n">
         <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="24">
@@ -1155,13 +1155,13 @@
         <v>50</v>
       </c>
       <c r="F24" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G24" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="25">
@@ -1185,13 +1185,13 @@
         <v>50</v>
       </c>
       <c r="F25" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="G25" t="n">
-        <v>62.5</v>
+        <v>58.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="26">
@@ -1215,13 +1215,13 @@
         <v>50</v>
       </c>
       <c r="F26" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="G26" t="n">
-        <v>62.5</v>
+        <v>58.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="27">
@@ -1251,7 +1251,7 @@
         <v>50</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="28">
@@ -1281,7 +1281,7 @@
         <v>50</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="29">
@@ -1311,7 +1311,7 @@
         <v>50</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="30">
@@ -1341,7 +1341,7 @@
         <v>50</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="31">
@@ -1371,7 +1371,7 @@
         <v>50</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="32">
@@ -1401,7 +1401,7 @@
         <v>50</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Apr 12 11:24:14 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>1.19</v>
       </c>
       <c r="E2" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F2" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G2" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>5.55</v>
       </c>
       <c r="E3" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F3" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G3" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.84</v>
       </c>
       <c r="E4" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F4" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G4" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.48</v>
       </c>
       <c r="E5" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G5" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.4</v>
       </c>
       <c r="E6" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G6" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.81</v>
       </c>
       <c r="E7" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F7" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G7" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>4.15</v>
       </c>
       <c r="E8" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F8" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G8" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.28</v>
       </c>
       <c r="E9" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F9" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G9" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.12</v>
       </c>
       <c r="E10" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F10" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G10" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.32</v>
       </c>
       <c r="E11" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F11" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G11" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.72</v>
       </c>
       <c r="E12" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F12" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G12" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.64</v>
       </c>
       <c r="E13" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F13" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G13" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>0.78</v>
       </c>
       <c r="E14" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F14" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G14" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.32</v>
       </c>
       <c r="E15" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F15" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G15" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.95</v>
       </c>
       <c r="E16" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F16" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G16" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.05</v>
       </c>
       <c r="E17" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F17" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G17" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.68</v>
       </c>
       <c r="E18" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F18" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G18" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.38</v>
       </c>
       <c r="E19" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F19" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G19" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>4.35</v>
       </c>
       <c r="E20" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F20" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G20" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.68</v>
       </c>
       <c r="E21" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="F21" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G21" t="n">
-        <v>75</v>
+        <v>68.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.76</v>
       </c>
       <c r="E22" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F22" t="n">
         <v>50</v>
       </c>
       <c r="G22" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.3</v>
       </c>
       <c r="E23" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F23" t="n">
         <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="24">
@@ -1155,13 +1155,13 @@
         <v>50</v>
       </c>
       <c r="F24" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G24" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="25">
@@ -1185,13 +1185,13 @@
         <v>50</v>
       </c>
       <c r="F25" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="G25" t="n">
-        <v>58.3</v>
+        <v>56.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="26">
@@ -1215,13 +1215,13 @@
         <v>50</v>
       </c>
       <c r="F26" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="G26" t="n">
-        <v>58.3</v>
+        <v>56.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="27">
@@ -1251,7 +1251,7 @@
         <v>50</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="28">
@@ -1281,7 +1281,7 @@
         <v>50</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="29">
@@ -1311,7 +1311,7 @@
         <v>50</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="30">
@@ -1341,7 +1341,7 @@
         <v>50</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="31">
@@ -1371,7 +1371,7 @@
         <v>50</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="32">
@@ -1401,7 +1401,7 @@
         <v>50</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Apr 24 22:01:26 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,42 +433,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>行业代码</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>行业名称</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>TTM市盈率</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>市净率</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>PE分位%</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PB分位%</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>行业温度</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
@@ -465,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>21.71</v>
+        <v>29.26</v>
       </c>
       <c r="D2" t="n">
-        <v>2.37</v>
+        <v>2.68</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -488,26 +500,26 @@
       <c r="G2" t="n">
         <v>100</v>
       </c>
-      <c r="H2" s="1" t="n">
-        <v>46108</v>
+      <c r="H2" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.61</v>
+        <v>23.84</v>
       </c>
       <c r="D3" t="n">
-        <v>2.63</v>
+        <v>1.23</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -518,26 +530,26 @@
       <c r="G3" t="n">
         <v>100</v>
       </c>
-      <c r="H3" s="1" t="n">
-        <v>46108</v>
+      <c r="H3" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22.04</v>
+        <v>65.14</v>
       </c>
       <c r="D4" t="n">
-        <v>1.18</v>
+        <v>6.06</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
@@ -548,26 +560,26 @@
       <c r="G4" t="n">
         <v>100</v>
       </c>
-      <c r="H4" s="1" t="n">
-        <v>46108</v>
+      <c r="H4" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25.65</v>
+        <v>15.13</v>
       </c>
       <c r="D5" t="n">
-        <v>3.7</v>
+        <v>2.46</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
@@ -578,26 +590,26 @@
       <c r="G5" t="n">
         <v>100</v>
       </c>
-      <c r="H5" s="1" t="n">
-        <v>46108</v>
+      <c r="H5" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>55.11</v>
+        <v>25.7</v>
       </c>
       <c r="D6" t="n">
-        <v>5.18</v>
+        <v>2.48</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
@@ -608,26 +620,26 @@
       <c r="G6" t="n">
         <v>100</v>
       </c>
-      <c r="H6" s="1" t="n">
-        <v>46108</v>
+      <c r="H6" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25.07</v>
+        <v>20.97</v>
       </c>
       <c r="D7" t="n">
-        <v>2.45</v>
+        <v>1.84</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
@@ -638,26 +650,26 @@
       <c r="G7" t="n">
         <v>100</v>
       </c>
-      <c r="H7" s="1" t="n">
-        <v>46108</v>
+      <c r="H7" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14.35</v>
+        <v>20.75</v>
       </c>
       <c r="D8" t="n">
-        <v>2.38</v>
+        <v>4.09</v>
       </c>
       <c r="E8" t="n">
         <v>100</v>
@@ -668,26 +680,26 @@
       <c r="G8" t="n">
         <v>100</v>
       </c>
-      <c r="H8" s="1" t="n">
-        <v>46108</v>
+      <c r="H8" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19.69</v>
+        <v>15.78</v>
       </c>
       <c r="D9" t="n">
-        <v>4.07</v>
+        <v>1.27</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
@@ -698,26 +710,26 @@
       <c r="G9" t="n">
         <v>100</v>
       </c>
-      <c r="H9" s="1" t="n">
-        <v>46108</v>
+      <c r="H9" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.6</v>
+        <v>29.96</v>
       </c>
       <c r="D10" t="n">
-        <v>1.76</v>
+        <v>2.77</v>
       </c>
       <c r="E10" t="n">
         <v>100</v>
@@ -728,8 +740,8 @@
       <c r="G10" t="n">
         <v>100</v>
       </c>
-      <c r="H10" s="1" t="n">
-        <v>46108</v>
+      <c r="H10" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="11">
@@ -744,10 +756,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>23.2</v>
+        <v>24.46</v>
       </c>
       <c r="D11" t="n">
-        <v>2.31</v>
+        <v>2.35</v>
       </c>
       <c r="E11" t="n">
         <v>100</v>
@@ -758,26 +770,26 @@
       <c r="G11" t="n">
         <v>100</v>
       </c>
-      <c r="H11" s="1" t="n">
-        <v>46108</v>
+      <c r="H11" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>27</v>
+        <v>36.83</v>
       </c>
       <c r="D12" t="n">
-        <v>2.62</v>
+        <v>3.09</v>
       </c>
       <c r="E12" t="n">
         <v>100</v>
@@ -788,26 +800,26 @@
       <c r="G12" t="n">
         <v>100</v>
       </c>
-      <c r="H12" s="1" t="n">
-        <v>46108</v>
+      <c r="H12" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.89</v>
+        <v>32.43</v>
       </c>
       <c r="D13" t="n">
-        <v>1.93</v>
+        <v>1.82</v>
       </c>
       <c r="E13" t="n">
         <v>100</v>
@@ -818,26 +830,26 @@
       <c r="G13" t="n">
         <v>100</v>
       </c>
-      <c r="H13" s="1" t="n">
-        <v>46108</v>
+      <c r="H13" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.44</v>
+        <v>101.2</v>
       </c>
       <c r="D14" t="n">
-        <v>1.26</v>
+        <v>3.25</v>
       </c>
       <c r="E14" t="n">
         <v>100</v>
@@ -848,26 +860,26 @@
       <c r="G14" t="n">
         <v>100</v>
       </c>
-      <c r="H14" s="1" t="n">
-        <v>46108</v>
+      <c r="H14" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>32.29</v>
+        <v>7.02</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="E15" t="n">
         <v>100</v>
@@ -878,26 +890,26 @@
       <c r="G15" t="n">
         <v>100</v>
       </c>
-      <c r="H15" s="1" t="n">
-        <v>46108</v>
+      <c r="H15" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30.85</v>
+        <v>35.46</v>
       </c>
       <c r="D16" t="n">
-        <v>2.04</v>
+        <v>2.68</v>
       </c>
       <c r="E16" t="n">
         <v>100</v>
@@ -908,26 +920,26 @@
       <c r="G16" t="n">
         <v>100</v>
       </c>
-      <c r="H16" s="1" t="n">
-        <v>46108</v>
+      <c r="H16" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>35</v>
+        <v>24.67</v>
       </c>
       <c r="D17" t="n">
-        <v>2.62</v>
+        <v>1.75</v>
       </c>
       <c r="E17" t="n">
         <v>100</v>
@@ -938,26 +950,26 @@
       <c r="G17" t="n">
         <v>100</v>
       </c>
-      <c r="H17" s="1" t="n">
-        <v>46108</v>
+      <c r="H17" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6.84</v>
+        <v>29.21</v>
       </c>
       <c r="D18" t="n">
-        <v>0.67</v>
+        <v>2.75</v>
       </c>
       <c r="E18" t="n">
         <v>100</v>
@@ -968,26 +980,26 @@
       <c r="G18" t="n">
         <v>100</v>
       </c>
-      <c r="H18" s="1" t="n">
-        <v>46108</v>
+      <c r="H18" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.29</v>
+        <v>28.68</v>
       </c>
       <c r="D19" t="n">
-        <v>1.31</v>
+        <v>2.39</v>
       </c>
       <c r="E19" t="n">
         <v>100</v>
@@ -998,26 +1010,26 @@
       <c r="G19" t="n">
         <v>100</v>
       </c>
-      <c r="H19" s="1" t="n">
-        <v>46108</v>
+      <c r="H19" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>58.93</v>
+        <v>74.87</v>
       </c>
       <c r="D20" t="n">
-        <v>2.91</v>
+        <v>4.31</v>
       </c>
       <c r="E20" t="n">
         <v>100</v>
@@ -1028,26 +1040,26 @@
       <c r="G20" t="n">
         <v>100</v>
       </c>
-      <c r="H20" s="1" t="n">
-        <v>46108</v>
+      <c r="H20" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>25.89</v>
+        <v>51.83</v>
       </c>
       <c r="D21" t="n">
-        <v>1.51</v>
+        <v>4.39</v>
       </c>
       <c r="E21" t="n">
         <v>100</v>
@@ -1058,26 +1070,26 @@
       <c r="G21" t="n">
         <v>100</v>
       </c>
-      <c r="H21" s="1" t="n">
-        <v>46108</v>
+      <c r="H21" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9.77</v>
+        <v>36.1</v>
       </c>
       <c r="D22" t="n">
-        <v>0.77</v>
+        <v>3.99</v>
       </c>
       <c r="E22" t="n">
         <v>100</v>
@@ -1088,308 +1100,308 @@
       <c r="G22" t="n">
         <v>100</v>
       </c>
-      <c r="H22" s="1" t="n">
-        <v>46108</v>
+      <c r="H22" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>35.1</v>
+        <v>11.39</v>
       </c>
       <c r="D23" t="n">
-        <v>3.9</v>
+        <v>0.77</v>
       </c>
       <c r="E23" t="n">
         <v>100</v>
       </c>
       <c r="F23" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G23" t="n">
-        <v>100</v>
-      </c>
-      <c r="H23" s="1" t="n">
-        <v>46108</v>
+        <v>87.5</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>33.68</v>
+        <v>31.27</v>
       </c>
       <c r="D24" t="n">
-        <v>2.91</v>
+        <v>2.31</v>
       </c>
       <c r="E24" t="n">
         <v>100</v>
       </c>
       <c r="F24" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H24" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>74.81999999999999</v>
+        <v>33.77</v>
       </c>
       <c r="D25" t="n">
-        <v>4.04</v>
+        <v>2.75</v>
       </c>
       <c r="E25" t="n">
         <v>100</v>
       </c>
       <c r="F25" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G25" t="n">
-        <v>100</v>
-      </c>
-      <c r="H25" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>48.96</v>
+        <v>28.56</v>
       </c>
       <c r="D26" t="n">
-        <v>4.25</v>
+        <v>2.17</v>
       </c>
       <c r="E26" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F26" t="n">
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H26" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25.7</v>
+        <v>35.94</v>
       </c>
       <c r="D27" t="n">
-        <v>2.31</v>
+        <v>0.91</v>
       </c>
       <c r="E27" t="n">
         <v>100</v>
       </c>
       <c r="F27" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H27" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25.75</v>
+        <v>25.63</v>
       </c>
       <c r="D28" t="n">
-        <v>2.44</v>
+        <v>3.81</v>
       </c>
       <c r="E28" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F28" t="n">
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>100</v>
-      </c>
-      <c r="H28" s="1" t="n">
-        <v>46108</v>
+        <v>75</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>19.12</v>
+        <v>19.64</v>
       </c>
       <c r="D29" t="n">
-        <v>1.86</v>
+        <v>1.89</v>
       </c>
       <c r="E29" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F29" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G29" t="n">
-        <v>100</v>
-      </c>
-      <c r="H29" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>16.77</v>
+        <v>10.19</v>
       </c>
       <c r="D30" t="n">
-        <v>1.58</v>
+        <v>1.29</v>
       </c>
       <c r="E30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G30" t="n">
-        <v>100</v>
-      </c>
-      <c r="H30" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>24.43</v>
+        <v>16.08</v>
       </c>
       <c r="D31" t="n">
-        <v>1.72</v>
+        <v>1.51</v>
       </c>
       <c r="E31" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F31" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G31" t="n">
-        <v>100</v>
-      </c>
-      <c r="H31" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>31.22</v>
+        <v>18.75</v>
       </c>
       <c r="D32" t="n">
-        <v>2.78</v>
+        <v>1.8</v>
       </c>
       <c r="E32" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F32" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G32" t="n">
-        <v>100</v>
-      </c>
-      <c r="H32" s="1" t="n">
-        <v>46108</v>
+        <v>50</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>46136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Apr 25 11:56:56 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.68</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.23</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>6.06</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.46</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.48</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.84</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F7" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>4.09</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F8" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.27</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F9" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.77</v>
       </c>
       <c r="E10" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F10" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G10" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.35</v>
       </c>
       <c r="E11" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F11" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G11" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.09</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F12" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G12" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.82</v>
       </c>
       <c r="E13" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F13" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G13" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>3.25</v>
       </c>
       <c r="E14" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F14" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G14" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>0.68</v>
       </c>
       <c r="E15" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F15" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G15" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.68</v>
       </c>
       <c r="E16" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F16" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G16" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.75</v>
       </c>
       <c r="E17" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F17" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G17" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.75</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G18" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.39</v>
       </c>
       <c r="E19" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F19" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G19" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>4.31</v>
       </c>
       <c r="E20" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F20" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G20" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>4.39</v>
       </c>
       <c r="E21" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F21" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G21" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>3.99</v>
       </c>
       <c r="E22" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F22" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G22" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.77</v>
       </c>
       <c r="E23" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F23" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="G23" t="n">
         <v>75</v>
       </c>
-      <c r="G23" t="n">
-        <v>87.5</v>
-      </c>
       <c r="H23" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.31</v>
       </c>
       <c r="E24" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F24" t="n">
         <v>50</v>
       </c>
       <c r="G24" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.75</v>
       </c>
       <c r="E25" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F25" t="n">
         <v>50</v>
       </c>
       <c r="G25" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="26">
@@ -1215,13 +1215,13 @@
         <v>50</v>
       </c>
       <c r="F26" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G26" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>0.91</v>
       </c>
       <c r="E27" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F27" t="n">
         <v>50</v>
       </c>
       <c r="G27" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="28">
@@ -1275,13 +1275,13 @@
         <v>50</v>
       </c>
       <c r="F28" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G28" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="29">
@@ -1311,7 +1311,7 @@
         <v>50</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="30">
@@ -1341,7 +1341,7 @@
         <v>50</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="31">
@@ -1371,7 +1371,7 @@
         <v>50</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="32">
@@ -1401,7 +1401,7 @@
         <v>50</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Apr 26 10:31:30 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.68</v>
       </c>
       <c r="E2" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F2" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G2" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.23</v>
       </c>
       <c r="E3" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F3" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G3" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>6.06</v>
       </c>
       <c r="E4" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F4" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G4" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.46</v>
       </c>
       <c r="E5" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G5" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.48</v>
       </c>
       <c r="E6" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G6" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.84</v>
       </c>
       <c r="E7" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F7" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G7" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>4.09</v>
       </c>
       <c r="E8" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F8" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G8" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.27</v>
       </c>
       <c r="E9" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F9" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G9" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.77</v>
       </c>
       <c r="E10" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F10" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G10" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.35</v>
       </c>
       <c r="E11" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F11" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G11" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.09</v>
       </c>
       <c r="E12" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F12" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G12" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.82</v>
       </c>
       <c r="E13" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F13" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G13" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>3.25</v>
       </c>
       <c r="E14" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F14" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G14" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>0.68</v>
       </c>
       <c r="E15" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F15" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G15" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.68</v>
       </c>
       <c r="E16" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F16" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G16" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.75</v>
       </c>
       <c r="E17" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F17" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G17" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.75</v>
       </c>
       <c r="E18" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F18" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G18" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.39</v>
       </c>
       <c r="E19" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F19" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G19" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>4.31</v>
       </c>
       <c r="E20" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F20" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G20" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>4.39</v>
       </c>
       <c r="E21" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F21" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G21" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>3.99</v>
       </c>
       <c r="E22" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F22" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G22" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.77</v>
       </c>
       <c r="E23" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F23" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="G23" t="n">
-        <v>75</v>
+        <v>68.8</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.31</v>
       </c>
       <c r="E24" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F24" t="n">
         <v>50</v>
       </c>
       <c r="G24" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.75</v>
       </c>
       <c r="E25" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F25" t="n">
         <v>50</v>
       </c>
       <c r="G25" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="26">
@@ -1215,13 +1215,13 @@
         <v>50</v>
       </c>
       <c r="F26" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G26" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>0.91</v>
       </c>
       <c r="E27" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="F27" t="n">
         <v>50</v>
       </c>
       <c r="G27" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="28">
@@ -1275,13 +1275,13 @@
         <v>50</v>
       </c>
       <c r="F28" t="n">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="G28" t="n">
-        <v>66.7</v>
+        <v>62.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="29">
@@ -1311,7 +1311,7 @@
         <v>50</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="30">
@@ -1341,7 +1341,7 @@
         <v>50</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="31">
@@ -1371,7 +1371,7 @@
         <v>50</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="32">
@@ -1401,7 +1401,7 @@
         <v>50</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46137</v>
+        <v>46138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Apr 27 11:28:05 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,61 +477,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>29.26</v>
+        <v>15.32</v>
       </c>
       <c r="D2" t="n">
-        <v>2.68</v>
+        <v>2.47</v>
       </c>
       <c r="E2" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>23.84</v>
+        <v>25.86</v>
       </c>
       <c r="D3" t="n">
-        <v>1.23</v>
+        <v>2.49</v>
       </c>
       <c r="E3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="4">
@@ -546,862 +546,862 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>65.14</v>
+        <v>67.75</v>
       </c>
       <c r="D4" t="n">
-        <v>6.06</v>
+        <v>6.39</v>
       </c>
       <c r="E4" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15.13</v>
+        <v>21.38</v>
       </c>
       <c r="D5" t="n">
-        <v>2.46</v>
+        <v>1.87</v>
       </c>
       <c r="E5" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>25.7</v>
+        <v>36.21</v>
       </c>
       <c r="D6" t="n">
-        <v>2.48</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.97</v>
+        <v>37.8</v>
       </c>
       <c r="D7" t="n">
-        <v>1.84</v>
+        <v>3.16</v>
       </c>
       <c r="E7" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20.75</v>
+        <v>101.53</v>
       </c>
       <c r="D8" t="n">
-        <v>4.09</v>
+        <v>3.27</v>
       </c>
       <c r="E8" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15.78</v>
+        <v>76.76000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>1.27</v>
+        <v>4.33</v>
       </c>
       <c r="E9" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>29.96</v>
+        <v>28.57</v>
       </c>
       <c r="D10" t="n">
-        <v>2.77</v>
+        <v>2.19</v>
       </c>
       <c r="E10" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F10" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>24.46</v>
+        <v>29.57</v>
       </c>
       <c r="D11" t="n">
-        <v>2.35</v>
+        <v>2.68</v>
       </c>
       <c r="E11" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F11" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G11" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>36.83</v>
+        <v>36.08</v>
       </c>
       <c r="D12" t="n">
-        <v>3.09</v>
+        <v>2.68</v>
       </c>
       <c r="E12" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G12" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>32.43</v>
+        <v>24.9</v>
       </c>
       <c r="D13" t="n">
-        <v>1.82</v>
+        <v>2.35</v>
       </c>
       <c r="E13" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F13" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G13" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>101.2</v>
+        <v>36.15</v>
       </c>
       <c r="D14" t="n">
-        <v>3.25</v>
+        <v>0.91</v>
       </c>
       <c r="E14" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="G14" t="n">
         <v>75</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7.02</v>
+        <v>29.31</v>
       </c>
       <c r="D15" t="n">
-        <v>0.68</v>
+        <v>2.74</v>
       </c>
       <c r="E15" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="G15" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>35.46</v>
+        <v>30.05</v>
       </c>
       <c r="D16" t="n">
-        <v>2.68</v>
+        <v>2.76</v>
       </c>
       <c r="E16" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F16" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="G16" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>24.67</v>
+        <v>33.65</v>
       </c>
       <c r="D17" t="n">
-        <v>1.75</v>
+        <v>2.79</v>
       </c>
       <c r="E17" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="F17" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>29.21</v>
+        <v>16.12</v>
       </c>
       <c r="D18" t="n">
-        <v>2.75</v>
+        <v>1.51</v>
       </c>
       <c r="E18" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F18" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="G18" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>28.68</v>
+        <v>24.29</v>
       </c>
       <c r="D19" t="n">
-        <v>2.39</v>
+        <v>3.88</v>
       </c>
       <c r="E19" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="F19" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>74.87</v>
+        <v>28.58</v>
       </c>
       <c r="D20" t="n">
-        <v>4.31</v>
+        <v>2.39</v>
       </c>
       <c r="E20" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="F20" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G20" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>51.83</v>
+        <v>31.79</v>
       </c>
       <c r="D21" t="n">
-        <v>4.39</v>
+        <v>1.82</v>
       </c>
       <c r="E21" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="F21" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G21" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>36.1</v>
+        <v>24.2</v>
       </c>
       <c r="D22" t="n">
-        <v>3.99</v>
+        <v>1.75</v>
       </c>
       <c r="E22" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="F22" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G22" t="n">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>11.39</v>
+        <v>23.68</v>
       </c>
       <c r="D23" t="n">
-        <v>0.77</v>
+        <v>1.19</v>
       </c>
       <c r="E23" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="F23" t="n">
-        <v>62.5</v>
+        <v>40</v>
       </c>
       <c r="G23" t="n">
-        <v>68.8</v>
+        <v>40</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>31.27</v>
+        <v>51.7</v>
       </c>
       <c r="D24" t="n">
-        <v>2.31</v>
+        <v>4.36</v>
       </c>
       <c r="E24" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="F24" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G24" t="n">
-        <v>62.5</v>
+        <v>40</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>33.77</v>
+        <v>10.24</v>
       </c>
       <c r="D25" t="n">
-        <v>2.75</v>
+        <v>1.28</v>
       </c>
       <c r="E25" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F25" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G25" t="n">
-        <v>62.5</v>
+        <v>38</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>28.56</v>
+        <v>18.92</v>
       </c>
       <c r="D26" t="n">
-        <v>2.17</v>
+        <v>1.74</v>
       </c>
       <c r="E26" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="F26" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="G26" t="n">
-        <v>62.5</v>
+        <v>38</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>35.94</v>
+        <v>6.96</v>
       </c>
       <c r="D27" t="n">
-        <v>0.91</v>
+        <v>0.67</v>
       </c>
       <c r="E27" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="F27" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G27" t="n">
-        <v>62.5</v>
+        <v>35</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25.63</v>
+        <v>15.47</v>
       </c>
       <c r="D28" t="n">
-        <v>3.81</v>
+        <v>1.26</v>
       </c>
       <c r="E28" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F28" t="n">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="G28" t="n">
-        <v>62.5</v>
+        <v>35</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>19.64</v>
+        <v>31.13</v>
       </c>
       <c r="D29" t="n">
-        <v>1.89</v>
+        <v>2.28</v>
       </c>
       <c r="E29" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F29" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G29" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>10.19</v>
+        <v>20.28</v>
       </c>
       <c r="D30" t="n">
-        <v>1.29</v>
+        <v>3.91</v>
       </c>
       <c r="E30" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F30" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G30" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>16.08</v>
+        <v>11.35</v>
       </c>
       <c r="D31" t="n">
-        <v>1.51</v>
+        <v>0.76</v>
       </c>
       <c r="E31" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F31" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G31" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18.75</v>
+        <v>19.58</v>
       </c>
       <c r="D32" t="n">
-        <v>1.8</v>
+        <v>1.88</v>
       </c>
       <c r="E32" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F32" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G32" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Apr 28 11:27:48 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>15.32</v>
+        <v>108.35</v>
       </c>
       <c r="D2" t="n">
-        <v>2.47</v>
+        <v>3.29</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,907 +501,907 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>25.86</v>
+        <v>37.81</v>
       </c>
       <c r="D3" t="n">
-        <v>2.49</v>
+        <v>3.14</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>91.7</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>67.75</v>
+        <v>7.03</v>
       </c>
       <c r="D4" t="n">
-        <v>6.39</v>
+        <v>0.68</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21.38</v>
+        <v>16.32</v>
       </c>
       <c r="D5" t="n">
-        <v>1.87</v>
+        <v>1.54</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>36.21</v>
+        <v>21.72</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>1.84</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>58.3</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>79.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>37.8</v>
+        <v>32.41</v>
       </c>
       <c r="D7" t="n">
-        <v>3.16</v>
+        <v>1.83</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>101.53</v>
+        <v>19.81</v>
       </c>
       <c r="D8" t="n">
-        <v>3.27</v>
+        <v>1.89</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F8" t="n">
-        <v>100</v>
+        <v>58.3</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>70.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>76.76000000000001</v>
+        <v>10.27</v>
       </c>
       <c r="D9" t="n">
-        <v>4.33</v>
+        <v>1.29</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F9" t="n">
-        <v>100</v>
+        <v>58.3</v>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>70.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28.57</v>
+        <v>28.68</v>
       </c>
       <c r="D10" t="n">
-        <v>2.19</v>
+        <v>2.39</v>
       </c>
       <c r="E10" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F10" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="G10" t="n">
-        <v>90</v>
+        <v>70.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>29.57</v>
+        <v>23.98</v>
       </c>
       <c r="D11" t="n">
-        <v>2.68</v>
+        <v>1.19</v>
       </c>
       <c r="E11" t="n">
         <v>100</v>
       </c>
       <c r="F11" t="n">
-        <v>70</v>
+        <v>41.7</v>
       </c>
       <c r="G11" t="n">
-        <v>85</v>
+        <v>70.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>36.08</v>
+        <v>19.59</v>
       </c>
       <c r="D12" t="n">
-        <v>2.68</v>
+        <v>1.79</v>
       </c>
       <c r="E12" t="n">
         <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>70</v>
+        <v>33.3</v>
       </c>
       <c r="G12" t="n">
-        <v>85</v>
+        <v>66.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>24.9</v>
+        <v>32.41</v>
       </c>
       <c r="D13" t="n">
-        <v>2.35</v>
+        <v>2.3</v>
       </c>
       <c r="E13" t="n">
         <v>100</v>
       </c>
       <c r="F13" t="n">
-        <v>70</v>
+        <v>33.3</v>
       </c>
       <c r="G13" t="n">
-        <v>85</v>
+        <v>66.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>36.15</v>
+        <v>30.11</v>
       </c>
       <c r="D14" t="n">
-        <v>0.91</v>
+        <v>2.75</v>
       </c>
       <c r="E14" t="n">
         <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="G14" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>29.31</v>
+        <v>15.53</v>
       </c>
       <c r="D15" t="n">
-        <v>2.74</v>
+        <v>2.45</v>
       </c>
       <c r="E15" t="n">
         <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="G15" t="n">
-        <v>70</v>
+        <v>66.7</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30.05</v>
+        <v>29.42</v>
       </c>
       <c r="D16" t="n">
-        <v>2.76</v>
+        <v>2.66</v>
       </c>
       <c r="E16" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="F16" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="G16" t="n">
-        <v>70</v>
+        <v>58.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>33.65</v>
+        <v>24.58</v>
       </c>
       <c r="D17" t="n">
-        <v>2.79</v>
+        <v>1.75</v>
       </c>
       <c r="E17" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F17" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="G17" t="n">
-        <v>70</v>
+        <v>58.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>16.12</v>
+        <v>64.3</v>
       </c>
       <c r="D18" t="n">
-        <v>1.51</v>
+        <v>6.3</v>
       </c>
       <c r="E18" t="n">
-        <v>80</v>
+        <v>33.3</v>
       </c>
       <c r="F18" t="n">
-        <v>50</v>
+        <v>83.3</v>
       </c>
       <c r="G18" t="n">
-        <v>65</v>
+        <v>58.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>24.29</v>
+        <v>15.41</v>
       </c>
       <c r="D19" t="n">
-        <v>3.88</v>
+        <v>1.28</v>
       </c>
       <c r="E19" t="n">
-        <v>20</v>
+        <v>16.7</v>
       </c>
       <c r="F19" t="n">
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>60</v>
+        <v>58.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>28.58</v>
+        <v>11.78</v>
       </c>
       <c r="D20" t="n">
-        <v>2.39</v>
+        <v>1.16</v>
       </c>
       <c r="E20" t="n">
-        <v>40</v>
+        <v>16.7</v>
       </c>
       <c r="F20" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>55</v>
+        <v>58.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>31.79</v>
+        <v>23.39</v>
       </c>
       <c r="D21" t="n">
-        <v>1.82</v>
+        <v>3.81</v>
       </c>
       <c r="E21" t="n">
-        <v>40</v>
+        <v>16.7</v>
       </c>
       <c r="F21" t="n">
-        <v>70</v>
+        <v>58.3</v>
       </c>
       <c r="G21" t="n">
-        <v>55</v>
+        <v>37.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>24.2</v>
+        <v>33.38</v>
       </c>
       <c r="D22" t="n">
-        <v>1.75</v>
+        <v>2.75</v>
       </c>
       <c r="E22" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="F22" t="n">
-        <v>70</v>
+        <v>41.7</v>
       </c>
       <c r="G22" t="n">
-        <v>45</v>
+        <v>37.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>23.68</v>
+        <v>24.51</v>
       </c>
       <c r="D23" t="n">
-        <v>1.19</v>
+        <v>2.3</v>
       </c>
       <c r="E23" t="n">
-        <v>40</v>
+        <v>83.3</v>
       </c>
       <c r="F23" t="n">
-        <v>40</v>
+        <v>16.7</v>
       </c>
       <c r="G23" t="n">
-        <v>40</v>
+        <v>36.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>51.7</v>
+        <v>35.5</v>
       </c>
       <c r="D24" t="n">
-        <v>4.36</v>
+        <v>3.92</v>
       </c>
       <c r="E24" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="F24" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="G24" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10.24</v>
+        <v>28.86</v>
       </c>
       <c r="D25" t="n">
-        <v>1.28</v>
+        <v>2.71</v>
       </c>
       <c r="E25" t="n">
-        <v>80</v>
+        <v>33.3</v>
       </c>
       <c r="F25" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="G25" t="n">
-        <v>38</v>
+        <v>33.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18.92</v>
+        <v>50.94</v>
       </c>
       <c r="D26" t="n">
-        <v>1.74</v>
+        <v>4.29</v>
       </c>
       <c r="E26" t="n">
-        <v>80</v>
+        <v>33.3</v>
       </c>
       <c r="F26" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="G26" t="n">
-        <v>38</v>
+        <v>33.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6.96</v>
+        <v>11.29</v>
       </c>
       <c r="D27" t="n">
-        <v>0.67</v>
+        <v>0.76</v>
       </c>
       <c r="E27" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="F27" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G27" t="n">
-        <v>35</v>
+        <v>27.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>15.47</v>
+        <v>20.33</v>
       </c>
       <c r="D28" t="n">
-        <v>1.26</v>
+        <v>3.9</v>
       </c>
       <c r="E28" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F28" t="n">
-        <v>30</v>
+        <v>16.7</v>
       </c>
       <c r="G28" t="n">
-        <v>35</v>
+        <v>26.7</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>31.13</v>
+        <v>34.81</v>
       </c>
       <c r="D29" t="n">
-        <v>2.28</v>
+        <v>2.63</v>
       </c>
       <c r="E29" t="n">
-        <v>40</v>
+        <v>16.7</v>
       </c>
       <c r="F29" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="G29" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>20.28</v>
+        <v>28.05</v>
       </c>
       <c r="D30" t="n">
-        <v>3.91</v>
+        <v>2.16</v>
       </c>
       <c r="E30" t="n">
-        <v>40</v>
+        <v>16.7</v>
       </c>
       <c r="F30" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="G30" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>11.35</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="D31" t="n">
-        <v>0.76</v>
+        <v>4.26</v>
       </c>
       <c r="E31" t="n">
-        <v>40</v>
+        <v>16.7</v>
       </c>
       <c r="F31" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="G31" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>19.58</v>
+        <v>25.63</v>
       </c>
       <c r="D32" t="n">
-        <v>1.88</v>
+        <v>2.44</v>
       </c>
       <c r="E32" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="F32" t="n">
-        <v>20</v>
+        <v>16.7</v>
       </c>
       <c r="G32" t="n">
-        <v>20</v>
+        <v>21.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Apr 29 11:21:01 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>108.35</v>
+        <v>29.81</v>
       </c>
       <c r="D2" t="n">
-        <v>3.29</v>
+        <v>2.69</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,217 +501,217 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>37.81</v>
+        <v>109.23</v>
       </c>
       <c r="D3" t="n">
-        <v>3.14</v>
+        <v>3.31</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7.03</v>
+        <v>37.85</v>
       </c>
       <c r="D4" t="n">
-        <v>0.68</v>
+        <v>3.23</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>87.5</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>16.32</v>
+        <v>34.12</v>
       </c>
       <c r="D5" t="n">
-        <v>1.54</v>
+        <v>1.9</v>
       </c>
       <c r="E5" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>21.72</v>
+        <v>36.94</v>
       </c>
       <c r="D6" t="n">
-        <v>1.84</v>
+        <v>4.08</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>58.3</v>
+        <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>79.2</v>
+        <v>100</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>32.41</v>
+        <v>36.24</v>
       </c>
       <c r="D7" t="n">
-        <v>1.83</v>
+        <v>2.7</v>
       </c>
       <c r="E7" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.81</v>
+        <v>32.96</v>
       </c>
       <c r="D8" t="n">
-        <v>1.89</v>
+        <v>2.37</v>
       </c>
       <c r="E8" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>58.3</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>70.8</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10.27</v>
+        <v>25.43</v>
       </c>
       <c r="D9" t="n">
-        <v>1.29</v>
+        <v>2.35</v>
       </c>
       <c r="E9" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>58.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>70.8</v>
+        <v>85.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="10">
@@ -726,112 +726,112 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28.68</v>
+        <v>30.82</v>
       </c>
       <c r="D10" t="n">
         <v>2.39</v>
       </c>
       <c r="E10" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F10" t="n">
-        <v>66.7</v>
+        <v>64.3</v>
       </c>
       <c r="G10" t="n">
-        <v>70.8</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>23.98</v>
+        <v>19.64</v>
       </c>
       <c r="D11" t="n">
-        <v>1.19</v>
+        <v>1.8</v>
       </c>
       <c r="E11" t="n">
         <v>100</v>
       </c>
       <c r="F11" t="n">
-        <v>41.7</v>
+        <v>64.3</v>
       </c>
       <c r="G11" t="n">
-        <v>70.8</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>19.59</v>
+        <v>10.42</v>
       </c>
       <c r="D12" t="n">
-        <v>1.79</v>
+        <v>1.29</v>
       </c>
       <c r="E12" t="n">
         <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>33.3</v>
+        <v>57.1</v>
       </c>
       <c r="G12" t="n">
-        <v>66.7</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>32.41</v>
+        <v>22.16</v>
       </c>
       <c r="D13" t="n">
-        <v>2.3</v>
+        <v>1.84</v>
       </c>
       <c r="E13" t="n">
         <v>100</v>
       </c>
       <c r="F13" t="n">
-        <v>33.3</v>
+        <v>57.1</v>
       </c>
       <c r="G13" t="n">
-        <v>66.7</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="14">
@@ -846,202 +846,202 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>30.11</v>
+        <v>30.16</v>
       </c>
       <c r="D14" t="n">
-        <v>2.75</v>
+        <v>2.76</v>
       </c>
       <c r="E14" t="n">
         <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="G14" t="n">
-        <v>66.7</v>
+        <v>75</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>15.53</v>
+        <v>16.29</v>
       </c>
       <c r="D15" t="n">
-        <v>2.45</v>
+        <v>1.54</v>
       </c>
       <c r="E15" t="n">
-        <v>100</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>33.3</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>66.7</v>
+        <v>75</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>29.42</v>
+        <v>15.47</v>
       </c>
       <c r="D16" t="n">
-        <v>2.66</v>
+        <v>1.28</v>
       </c>
       <c r="E16" t="n">
-        <v>83.3</v>
+        <v>50</v>
       </c>
       <c r="F16" t="n">
-        <v>33.3</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>58.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>24.58</v>
+        <v>26.78</v>
       </c>
       <c r="D17" t="n">
-        <v>1.75</v>
+        <v>2.46</v>
       </c>
       <c r="E17" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F17" t="n">
-        <v>66.7</v>
+        <v>42.9</v>
       </c>
       <c r="G17" t="n">
-        <v>58.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>64.3</v>
+        <v>24.48</v>
       </c>
       <c r="D18" t="n">
-        <v>6.3</v>
+        <v>1.76</v>
       </c>
       <c r="E18" t="n">
-        <v>33.3</v>
+        <v>42.9</v>
       </c>
       <c r="F18" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>58.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15.41</v>
+        <v>16.23</v>
       </c>
       <c r="D19" t="n">
-        <v>1.28</v>
+        <v>2.45</v>
       </c>
       <c r="E19" t="n">
-        <v>16.7</v>
+        <v>100</v>
       </c>
       <c r="F19" t="n">
-        <v>100</v>
+        <v>35.7</v>
       </c>
       <c r="G19" t="n">
-        <v>58.3</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>11.78</v>
+        <v>33.06</v>
       </c>
       <c r="D20" t="n">
-        <v>1.16</v>
+        <v>2.8</v>
       </c>
       <c r="E20" t="n">
-        <v>16.7</v>
+        <v>28.6</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>58.3</v>
+        <v>64.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="21">
@@ -1056,292 +1056,292 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>23.39</v>
+        <v>23.58</v>
       </c>
       <c r="D21" t="n">
-        <v>3.81</v>
+        <v>3.92</v>
       </c>
       <c r="E21" t="n">
-        <v>16.7</v>
+        <v>28.6</v>
       </c>
       <c r="F21" t="n">
-        <v>58.3</v>
+        <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>37.5</v>
+        <v>64.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>33.38</v>
+        <v>11.87</v>
       </c>
       <c r="D22" t="n">
-        <v>2.75</v>
+        <v>1.16</v>
       </c>
       <c r="E22" t="n">
-        <v>33.3</v>
+        <v>28.6</v>
       </c>
       <c r="F22" t="n">
-        <v>41.7</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>37.5</v>
+        <v>60.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24.51</v>
+        <v>61.93</v>
       </c>
       <c r="D23" t="n">
-        <v>2.3</v>
+        <v>6.22</v>
       </c>
       <c r="E23" t="n">
-        <v>83.3</v>
+        <v>28.6</v>
       </c>
       <c r="F23" t="n">
-        <v>16.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>36.7</v>
+        <v>50</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>35.5</v>
+        <v>11.4</v>
       </c>
       <c r="D24" t="n">
-        <v>3.92</v>
+        <v>0.76</v>
       </c>
       <c r="E24" t="n">
-        <v>33.3</v>
+        <v>100</v>
       </c>
       <c r="F24" t="n">
-        <v>33.3</v>
+        <v>28.6</v>
       </c>
       <c r="G24" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.86</v>
+        <v>51.59</v>
       </c>
       <c r="D25" t="n">
-        <v>2.71</v>
+        <v>4.34</v>
       </c>
       <c r="E25" t="n">
-        <v>33.3</v>
+        <v>42.9</v>
       </c>
       <c r="F25" t="n">
-        <v>33.3</v>
+        <v>42.9</v>
       </c>
       <c r="G25" t="n">
-        <v>33.3</v>
+        <v>42.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>50.94</v>
+        <v>19.93</v>
       </c>
       <c r="D26" t="n">
-        <v>4.29</v>
+        <v>1.87</v>
       </c>
       <c r="E26" t="n">
-        <v>33.3</v>
+        <v>100</v>
       </c>
       <c r="F26" t="n">
-        <v>33.3</v>
+        <v>14.3</v>
       </c>
       <c r="G26" t="n">
-        <v>33.3</v>
+        <v>40</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>11.29</v>
+        <v>27.88</v>
       </c>
       <c r="D27" t="n">
-        <v>0.76</v>
+        <v>2.17</v>
       </c>
       <c r="E27" t="n">
-        <v>33.3</v>
+        <v>14.3</v>
       </c>
       <c r="F27" t="n">
-        <v>25</v>
+        <v>64.3</v>
       </c>
       <c r="G27" t="n">
-        <v>27.5</v>
+        <v>39.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>20.33</v>
+        <v>28.84</v>
       </c>
       <c r="D28" t="n">
-        <v>3.9</v>
+        <v>2.72</v>
       </c>
       <c r="E28" t="n">
-        <v>50</v>
+        <v>28.6</v>
       </c>
       <c r="F28" t="n">
-        <v>16.7</v>
+        <v>42.9</v>
       </c>
       <c r="G28" t="n">
-        <v>26.7</v>
+        <v>35.7</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>34.81</v>
+        <v>6.99</v>
       </c>
       <c r="D29" t="n">
-        <v>2.63</v>
+        <v>0.67</v>
       </c>
       <c r="E29" t="n">
-        <v>16.7</v>
+        <v>42.9</v>
       </c>
       <c r="F29" t="n">
-        <v>33.3</v>
+        <v>28.6</v>
       </c>
       <c r="G29" t="n">
-        <v>25</v>
+        <v>32.9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>28.05</v>
+        <v>20.74</v>
       </c>
       <c r="D30" t="n">
-        <v>2.16</v>
+        <v>3.89</v>
       </c>
       <c r="E30" t="n">
-        <v>16.7</v>
+        <v>57.1</v>
       </c>
       <c r="F30" t="n">
-        <v>33.3</v>
+        <v>14.3</v>
       </c>
       <c r="G30" t="n">
-        <v>25</v>
+        <v>27.1</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="31">
@@ -1356,52 +1356,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>72.84999999999999</v>
+        <v>71.18000000000001</v>
       </c>
       <c r="D31" t="n">
         <v>4.26</v>
       </c>
       <c r="E31" t="n">
-        <v>16.7</v>
+        <v>14.3</v>
       </c>
       <c r="F31" t="n">
-        <v>33.3</v>
+        <v>35.7</v>
       </c>
       <c r="G31" t="n">
         <v>25</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.63</v>
+        <v>20.77</v>
       </c>
       <c r="D32" t="n">
-        <v>2.44</v>
+        <v>1.14</v>
       </c>
       <c r="E32" t="n">
-        <v>33.3</v>
+        <v>14.3</v>
       </c>
       <c r="F32" t="n">
-        <v>16.7</v>
+        <v>14.3</v>
       </c>
       <c r="G32" t="n">
-        <v>21.7</v>
+        <v>14.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Apr 30 11:20:37 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>29.81</v>
+        <v>130.93</v>
       </c>
       <c r="D2" t="n">
-        <v>2.69</v>
+        <v>4.91</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,25 +501,25 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>109.23</v>
+        <v>38.54</v>
       </c>
       <c r="D3" t="n">
-        <v>3.31</v>
+        <v>3.25</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -531,697 +531,697 @@
         <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37.85</v>
+        <v>32.34</v>
       </c>
       <c r="D4" t="n">
-        <v>3.23</v>
+        <v>2.4</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>34.12</v>
+        <v>36.66</v>
       </c>
       <c r="D5" t="n">
-        <v>1.9</v>
+        <v>4.01</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>36.94</v>
+        <v>33.47</v>
       </c>
       <c r="D6" t="n">
-        <v>4.08</v>
+        <v>1.86</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>36.24</v>
+        <v>25.97</v>
       </c>
       <c r="D7" t="n">
-        <v>2.7</v>
+        <v>2.35</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>100</v>
+        <v>68.8</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>32.96</v>
+        <v>19.68</v>
       </c>
       <c r="D8" t="n">
-        <v>2.37</v>
+        <v>1.8</v>
       </c>
       <c r="E8" t="n">
         <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>92.90000000000001</v>
+        <v>62.5</v>
       </c>
       <c r="G8" t="n">
-        <v>96.40000000000001</v>
+        <v>81.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>25.43</v>
+        <v>26.73</v>
       </c>
       <c r="D9" t="n">
-        <v>2.35</v>
+        <v>2.48</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="F9" t="n">
-        <v>71.40000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="G9" t="n">
-        <v>85.7</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>30.82</v>
+        <v>52.4</v>
       </c>
       <c r="D10" t="n">
-        <v>2.39</v>
+        <v>4.3</v>
       </c>
       <c r="E10" t="n">
         <v>100</v>
       </c>
       <c r="F10" t="n">
-        <v>64.3</v>
+        <v>37.5</v>
       </c>
       <c r="G10" t="n">
-        <v>82.09999999999999</v>
+        <v>68.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.64</v>
+        <v>16.22</v>
       </c>
       <c r="D11" t="n">
-        <v>1.8</v>
+        <v>1.53</v>
       </c>
       <c r="E11" t="n">
-        <v>100</v>
+        <v>62.5</v>
       </c>
       <c r="F11" t="n">
-        <v>64.3</v>
+        <v>62.5</v>
       </c>
       <c r="G11" t="n">
-        <v>82.09999999999999</v>
+        <v>62.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10.42</v>
+        <v>15.53</v>
       </c>
       <c r="D12" t="n">
-        <v>1.29</v>
+        <v>1.27</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>62.5</v>
       </c>
       <c r="F12" t="n">
-        <v>57.1</v>
+        <v>56.2</v>
       </c>
       <c r="G12" t="n">
-        <v>78.59999999999999</v>
+        <v>59.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>22.16</v>
+        <v>61.6</v>
       </c>
       <c r="D13" t="n">
-        <v>1.84</v>
+        <v>6.35</v>
       </c>
       <c r="E13" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="F13" t="n">
-        <v>57.1</v>
+        <v>87.5</v>
       </c>
       <c r="G13" t="n">
-        <v>78.59999999999999</v>
+        <v>56.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>30.16</v>
+        <v>12.69</v>
       </c>
       <c r="D14" t="n">
-        <v>2.76</v>
+        <v>1.15</v>
       </c>
       <c r="E14" t="n">
-        <v>100</v>
+        <v>37.5</v>
       </c>
       <c r="F14" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G14" t="n">
-        <v>75</v>
+        <v>56.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>16.29</v>
+        <v>16.28</v>
       </c>
       <c r="D15" t="n">
-        <v>1.54</v>
+        <v>2.41</v>
       </c>
       <c r="E15" t="n">
-        <v>71.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>78.59999999999999</v>
+        <v>25</v>
       </c>
       <c r="G15" t="n">
-        <v>75</v>
+        <v>47.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15.47</v>
+        <v>22.9</v>
       </c>
       <c r="D16" t="n">
-        <v>1.28</v>
+        <v>3.87</v>
       </c>
       <c r="E16" t="n">
-        <v>50</v>
+        <v>12.5</v>
       </c>
       <c r="F16" t="n">
-        <v>92.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="G16" t="n">
-        <v>71.40000000000001</v>
+        <v>43.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>26.78</v>
+        <v>21.9</v>
       </c>
       <c r="D17" t="n">
-        <v>2.46</v>
+        <v>1.82</v>
       </c>
       <c r="E17" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="F17" t="n">
-        <v>42.9</v>
+        <v>25</v>
       </c>
       <c r="G17" t="n">
-        <v>71.40000000000001</v>
+        <v>43.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>24.48</v>
+        <v>33</v>
       </c>
       <c r="D18" t="n">
-        <v>1.76</v>
+        <v>2.76</v>
       </c>
       <c r="E18" t="n">
-        <v>42.9</v>
+        <v>25</v>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>62.5</v>
       </c>
       <c r="G18" t="n">
-        <v>71.40000000000001</v>
+        <v>43.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>16.23</v>
+        <v>10.52</v>
       </c>
       <c r="D19" t="n">
-        <v>2.45</v>
+        <v>1.28</v>
       </c>
       <c r="E19" t="n">
         <v>100</v>
       </c>
       <c r="F19" t="n">
-        <v>35.7</v>
+        <v>18.8</v>
       </c>
       <c r="G19" t="n">
-        <v>67.90000000000001</v>
+        <v>43.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>33.06</v>
+        <v>11.72</v>
       </c>
       <c r="D20" t="n">
-        <v>2.8</v>
+        <v>0.75</v>
       </c>
       <c r="E20" t="n">
-        <v>28.6</v>
+        <v>100</v>
       </c>
       <c r="F20" t="n">
-        <v>100</v>
+        <v>12.5</v>
       </c>
       <c r="G20" t="n">
-        <v>64.3</v>
+        <v>38.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>23.58</v>
+        <v>35.11</v>
       </c>
       <c r="D21" t="n">
-        <v>3.92</v>
+        <v>2.67</v>
       </c>
       <c r="E21" t="n">
-        <v>28.6</v>
+        <v>37.5</v>
       </c>
       <c r="F21" t="n">
-        <v>100</v>
+        <v>37.5</v>
       </c>
       <c r="G21" t="n">
-        <v>64.3</v>
+        <v>37.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>11.87</v>
+        <v>28.66</v>
       </c>
       <c r="D22" t="n">
-        <v>1.16</v>
+        <v>2.72</v>
       </c>
       <c r="E22" t="n">
-        <v>28.6</v>
+        <v>25</v>
       </c>
       <c r="F22" t="n">
-        <v>92.90000000000001</v>
+        <v>43.8</v>
       </c>
       <c r="G22" t="n">
-        <v>60.7</v>
+        <v>34.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>61.93</v>
+        <v>65.68000000000001</v>
       </c>
       <c r="D23" t="n">
-        <v>6.22</v>
+        <v>4.27</v>
       </c>
       <c r="E23" t="n">
-        <v>28.6</v>
+        <v>12.5</v>
       </c>
       <c r="F23" t="n">
-        <v>71.40000000000001</v>
+        <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>50</v>
+        <v>31.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>11.4</v>
+        <v>29.11</v>
       </c>
       <c r="D24" t="n">
-        <v>0.76</v>
+        <v>2.67</v>
       </c>
       <c r="E24" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="F24" t="n">
-        <v>28.6</v>
+        <v>37.5</v>
       </c>
       <c r="G24" t="n">
-        <v>50</v>
+        <v>31.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>51.59</v>
+        <v>29.95</v>
       </c>
       <c r="D25" t="n">
-        <v>4.34</v>
+        <v>2.73</v>
       </c>
       <c r="E25" t="n">
-        <v>42.9</v>
+        <v>25</v>
       </c>
       <c r="F25" t="n">
-        <v>42.9</v>
+        <v>25</v>
       </c>
       <c r="G25" t="n">
-        <v>42.9</v>
+        <v>25</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>19.93</v>
+        <v>23.88</v>
       </c>
       <c r="D26" t="n">
-        <v>1.87</v>
+        <v>1.74</v>
       </c>
       <c r="E26" t="n">
-        <v>100</v>
+        <v>12.5</v>
       </c>
       <c r="F26" t="n">
-        <v>14.3</v>
+        <v>25</v>
       </c>
       <c r="G26" t="n">
-        <v>40</v>
+        <v>21.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="27">
@@ -1236,142 +1236,142 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>27.88</v>
+        <v>26.19</v>
       </c>
       <c r="D27" t="n">
-        <v>2.17</v>
+        <v>2.15</v>
       </c>
       <c r="E27" t="n">
-        <v>14.3</v>
+        <v>12.5</v>
       </c>
       <c r="F27" t="n">
-        <v>64.3</v>
+        <v>25</v>
       </c>
       <c r="G27" t="n">
-        <v>39.3</v>
+        <v>21.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>28.84</v>
+        <v>28.26</v>
       </c>
       <c r="D28" t="n">
-        <v>2.72</v>
+        <v>2.31</v>
       </c>
       <c r="E28" t="n">
-        <v>28.6</v>
+        <v>25</v>
       </c>
       <c r="F28" t="n">
-        <v>42.9</v>
+        <v>18.8</v>
       </c>
       <c r="G28" t="n">
-        <v>35.7</v>
+        <v>20.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6.99</v>
+        <v>20.3</v>
       </c>
       <c r="D29" t="n">
-        <v>0.67</v>
+        <v>3.81</v>
       </c>
       <c r="E29" t="n">
-        <v>42.9</v>
+        <v>37.5</v>
       </c>
       <c r="F29" t="n">
-        <v>28.6</v>
+        <v>12.5</v>
       </c>
       <c r="G29" t="n">
-        <v>32.9</v>
+        <v>20</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>20.74</v>
+        <v>19.62</v>
       </c>
       <c r="D30" t="n">
-        <v>3.89</v>
+        <v>1.83</v>
       </c>
       <c r="E30" t="n">
-        <v>57.1</v>
+        <v>25</v>
       </c>
       <c r="F30" t="n">
-        <v>14.3</v>
+        <v>12.5</v>
       </c>
       <c r="G30" t="n">
-        <v>27.1</v>
+        <v>16.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>71.18000000000001</v>
+        <v>6.94</v>
       </c>
       <c r="D31" t="n">
-        <v>4.26</v>
+        <v>0.66</v>
       </c>
       <c r="E31" t="n">
-        <v>14.3</v>
+        <v>25</v>
       </c>
       <c r="F31" t="n">
-        <v>35.7</v>
+        <v>12.5</v>
       </c>
       <c r="G31" t="n">
-        <v>25</v>
+        <v>16.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>20.77</v>
+        <v>20.14</v>
       </c>
       <c r="D32" t="n">
-        <v>1.14</v>
+        <v>1.12</v>
       </c>
       <c r="E32" t="n">
-        <v>14.3</v>
+        <v>12.5</v>
       </c>
       <c r="F32" t="n">
-        <v>14.3</v>
+        <v>12.5</v>
       </c>
       <c r="G32" t="n">
-        <v>14.3</v>
+        <v>12.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri May  1 10:58:01 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>4.91</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.25</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.4</v>
       </c>
       <c r="E4" t="n">
-        <v>75</v>
+        <v>72.2</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>4.01</v>
       </c>
       <c r="E5" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="F5" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="G5" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.86</v>
       </c>
       <c r="E6" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="F6" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="G6" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.35</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>68.8</v>
+        <v>66.7</v>
       </c>
       <c r="G7" t="n">
-        <v>84.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.8</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>62.5</v>
+        <v>61.1</v>
       </c>
       <c r="G8" t="n">
-        <v>81.2</v>
+        <v>77.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.48</v>
       </c>
       <c r="E9" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="F9" t="n">
-        <v>68.8</v>
+        <v>66.7</v>
       </c>
       <c r="G9" t="n">
-        <v>78.09999999999999</v>
+        <v>75</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>4.3</v>
       </c>
       <c r="E10" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>37.5</v>
+        <v>38.9</v>
       </c>
       <c r="G10" t="n">
-        <v>68.8</v>
+        <v>66.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.53</v>
       </c>
       <c r="E11" t="n">
-        <v>62.5</v>
+        <v>61.1</v>
       </c>
       <c r="F11" t="n">
-        <v>62.5</v>
+        <v>61.1</v>
       </c>
       <c r="G11" t="n">
-        <v>62.5</v>
+        <v>61.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.27</v>
       </c>
       <c r="E12" t="n">
-        <v>62.5</v>
+        <v>61.1</v>
       </c>
       <c r="F12" t="n">
-        <v>56.2</v>
+        <v>55.6</v>
       </c>
       <c r="G12" t="n">
-        <v>59.4</v>
+        <v>58.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>6.35</v>
       </c>
       <c r="E13" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="F13" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="G13" t="n">
-        <v>56.2</v>
+        <v>55.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.15</v>
       </c>
       <c r="E14" t="n">
-        <v>37.5</v>
+        <v>38.9</v>
       </c>
       <c r="F14" t="n">
-        <v>75</v>
+        <v>72.2</v>
       </c>
       <c r="G14" t="n">
-        <v>56.2</v>
+        <v>55.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.41</v>
       </c>
       <c r="E15" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="G15" t="n">
-        <v>47.5</v>
+        <v>47.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>3.87</v>
       </c>
       <c r="E16" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="F16" t="n">
-        <v>75</v>
+        <v>72.2</v>
       </c>
       <c r="G16" t="n">
-        <v>43.8</v>
+        <v>44.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.82</v>
       </c>
       <c r="E17" t="n">
-        <v>87.5</v>
+        <v>83.3</v>
       </c>
       <c r="F17" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="G17" t="n">
-        <v>43.8</v>
+        <v>44.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.76</v>
       </c>
       <c r="E18" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="F18" t="n">
-        <v>62.5</v>
+        <v>61.1</v>
       </c>
       <c r="G18" t="n">
-        <v>43.8</v>
+        <v>44.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.28</v>
       </c>
       <c r="E19" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>18.8</v>
+        <v>22.2</v>
       </c>
       <c r="G19" t="n">
-        <v>43.1</v>
+        <v>43.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.75</v>
       </c>
       <c r="E20" t="n">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F20" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="G20" t="n">
-        <v>38.8</v>
+        <v>40</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.67</v>
       </c>
       <c r="E21" t="n">
-        <v>37.5</v>
+        <v>38.9</v>
       </c>
       <c r="F21" t="n">
-        <v>37.5</v>
+        <v>38.9</v>
       </c>
       <c r="G21" t="n">
-        <v>37.5</v>
+        <v>38.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.72</v>
       </c>
       <c r="E22" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="F22" t="n">
-        <v>43.8</v>
+        <v>44.4</v>
       </c>
       <c r="G22" t="n">
-        <v>34.4</v>
+        <v>36.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>4.27</v>
       </c>
       <c r="E23" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="F23" t="n">
         <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>31.2</v>
+        <v>33.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.67</v>
       </c>
       <c r="E24" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="F24" t="n">
-        <v>37.5</v>
+        <v>38.9</v>
       </c>
       <c r="G24" t="n">
-        <v>31.2</v>
+        <v>33.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.73</v>
       </c>
       <c r="E25" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="F25" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="G25" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>1.74</v>
       </c>
       <c r="E26" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="F26" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="G26" t="n">
-        <v>21.2</v>
+        <v>24.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.15</v>
       </c>
       <c r="E27" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="F27" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="G27" t="n">
-        <v>21.2</v>
+        <v>24.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.31</v>
       </c>
       <c r="E28" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="F28" t="n">
-        <v>18.8</v>
+        <v>22.2</v>
       </c>
       <c r="G28" t="n">
-        <v>20.6</v>
+        <v>23.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.81</v>
       </c>
       <c r="E29" t="n">
-        <v>37.5</v>
+        <v>38.9</v>
       </c>
       <c r="F29" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="G29" t="n">
-        <v>20</v>
+        <v>23.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.83</v>
       </c>
       <c r="E30" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="F30" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="G30" t="n">
-        <v>16.2</v>
+        <v>20</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>0.66</v>
       </c>
       <c r="E31" t="n">
-        <v>25</v>
+        <v>27.8</v>
       </c>
       <c r="F31" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="G31" t="n">
-        <v>16.2</v>
+        <v>20</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.12</v>
       </c>
       <c r="E32" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="F32" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="G32" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat May  2 10:35:18 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>4.91</v>
       </c>
       <c r="E2" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="F2" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="G2" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.25</v>
       </c>
       <c r="E3" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="F3" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="G3" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.4</v>
       </c>
       <c r="E4" t="n">
-        <v>72.2</v>
+        <v>70</v>
       </c>
       <c r="F4" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="G4" t="n">
-        <v>83.3</v>
+        <v>80</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>4.01</v>
       </c>
       <c r="E5" t="n">
-        <v>83.3</v>
+        <v>80</v>
       </c>
       <c r="F5" t="n">
-        <v>83.3</v>
+        <v>80</v>
       </c>
       <c r="G5" t="n">
-        <v>83.3</v>
+        <v>80</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.86</v>
       </c>
       <c r="E6" t="n">
-        <v>83.3</v>
+        <v>80</v>
       </c>
       <c r="F6" t="n">
-        <v>83.3</v>
+        <v>80</v>
       </c>
       <c r="G6" t="n">
-        <v>83.3</v>
+        <v>80</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.35</v>
       </c>
       <c r="E7" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="F7" t="n">
-        <v>66.7</v>
+        <v>65</v>
       </c>
       <c r="G7" t="n">
-        <v>80.59999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.8</v>
       </c>
       <c r="E8" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="F8" t="n">
-        <v>61.1</v>
+        <v>60</v>
       </c>
       <c r="G8" t="n">
-        <v>77.8</v>
+        <v>75</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.48</v>
       </c>
       <c r="E9" t="n">
-        <v>83.3</v>
+        <v>80</v>
       </c>
       <c r="F9" t="n">
-        <v>66.7</v>
+        <v>65</v>
       </c>
       <c r="G9" t="n">
-        <v>75</v>
+        <v>72.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="10">
@@ -732,226 +732,226 @@
         <v>4.3</v>
       </c>
       <c r="E10" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="F10" t="n">
-        <v>38.9</v>
+        <v>40</v>
       </c>
       <c r="G10" t="n">
-        <v>66.7</v>
+        <v>65</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16.22</v>
+        <v>16.28</v>
       </c>
       <c r="D11" t="n">
-        <v>1.53</v>
+        <v>2.41</v>
       </c>
       <c r="E11" t="n">
-        <v>61.1</v>
+        <v>90</v>
       </c>
       <c r="F11" t="n">
-        <v>61.1</v>
+        <v>30</v>
       </c>
       <c r="G11" t="n">
-        <v>61.1</v>
+        <v>60</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15.53</v>
+        <v>16.22</v>
       </c>
       <c r="D12" t="n">
-        <v>1.27</v>
+        <v>1.53</v>
       </c>
       <c r="E12" t="n">
-        <v>61.1</v>
+        <v>60</v>
       </c>
       <c r="F12" t="n">
-        <v>55.6</v>
+        <v>60</v>
       </c>
       <c r="G12" t="n">
-        <v>58.3</v>
+        <v>60</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>61.6</v>
+        <v>15.53</v>
       </c>
       <c r="D13" t="n">
-        <v>6.35</v>
+        <v>1.27</v>
       </c>
       <c r="E13" t="n">
-        <v>27.8</v>
+        <v>60</v>
       </c>
       <c r="F13" t="n">
-        <v>83.3</v>
+        <v>55</v>
       </c>
       <c r="G13" t="n">
-        <v>55.6</v>
+        <v>57.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12.69</v>
+        <v>21.9</v>
       </c>
       <c r="D14" t="n">
-        <v>1.15</v>
+        <v>1.82</v>
       </c>
       <c r="E14" t="n">
-        <v>38.9</v>
+        <v>80</v>
       </c>
       <c r="F14" t="n">
-        <v>72.2</v>
+        <v>30</v>
       </c>
       <c r="G14" t="n">
-        <v>55.6</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>16.28</v>
+        <v>61.6</v>
       </c>
       <c r="D15" t="n">
-        <v>2.41</v>
+        <v>6.35</v>
       </c>
       <c r="E15" t="n">
-        <v>94.40000000000001</v>
+        <v>30</v>
       </c>
       <c r="F15" t="n">
-        <v>27.8</v>
+        <v>80</v>
       </c>
       <c r="G15" t="n">
-        <v>47.8</v>
+        <v>55</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>22.9</v>
+        <v>12.69</v>
       </c>
       <c r="D16" t="n">
-        <v>3.87</v>
+        <v>1.15</v>
       </c>
       <c r="E16" t="n">
-        <v>16.7</v>
+        <v>40</v>
       </c>
       <c r="F16" t="n">
-        <v>72.2</v>
+        <v>70</v>
       </c>
       <c r="G16" t="n">
-        <v>44.4</v>
+        <v>55</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>21.9</v>
+        <v>22.9</v>
       </c>
       <c r="D17" t="n">
-        <v>1.82</v>
+        <v>3.87</v>
       </c>
       <c r="E17" t="n">
-        <v>83.3</v>
+        <v>20</v>
       </c>
       <c r="F17" t="n">
-        <v>27.8</v>
+        <v>70</v>
       </c>
       <c r="G17" t="n">
-        <v>44.4</v>
+        <v>45</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.76</v>
       </c>
       <c r="E18" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="F18" t="n">
-        <v>61.1</v>
+        <v>60</v>
       </c>
       <c r="G18" t="n">
-        <v>44.4</v>
+        <v>45</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.28</v>
       </c>
       <c r="E19" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="F19" t="n">
-        <v>22.2</v>
+        <v>25</v>
       </c>
       <c r="G19" t="n">
-        <v>43.9</v>
+        <v>44.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.75</v>
       </c>
       <c r="E20" t="n">
-        <v>94.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="F20" t="n">
-        <v>16.7</v>
+        <v>20</v>
       </c>
       <c r="G20" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.67</v>
       </c>
       <c r="E21" t="n">
-        <v>38.9</v>
+        <v>40</v>
       </c>
       <c r="F21" t="n">
-        <v>38.9</v>
+        <v>40</v>
       </c>
       <c r="G21" t="n">
-        <v>38.9</v>
+        <v>40</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.72</v>
       </c>
       <c r="E22" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="F22" t="n">
-        <v>44.4</v>
+        <v>45</v>
       </c>
       <c r="G22" t="n">
-        <v>36.1</v>
+        <v>37.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>4.27</v>
       </c>
       <c r="E23" t="n">
-        <v>16.7</v>
+        <v>20</v>
       </c>
       <c r="F23" t="n">
         <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>33.3</v>
+        <v>35</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.67</v>
       </c>
       <c r="E24" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="F24" t="n">
-        <v>38.9</v>
+        <v>40</v>
       </c>
       <c r="G24" t="n">
-        <v>33.3</v>
+        <v>35</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="25">
@@ -1182,136 +1182,136 @@
         <v>2.73</v>
       </c>
       <c r="E25" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="F25" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="G25" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>23.88</v>
+        <v>28.26</v>
       </c>
       <c r="D26" t="n">
-        <v>1.74</v>
+        <v>2.31</v>
       </c>
       <c r="E26" t="n">
-        <v>16.7</v>
+        <v>30</v>
       </c>
       <c r="F26" t="n">
-        <v>27.8</v>
+        <v>25</v>
       </c>
       <c r="G26" t="n">
-        <v>24.4</v>
+        <v>26.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>26.19</v>
+        <v>20.3</v>
       </c>
       <c r="D27" t="n">
-        <v>2.15</v>
+        <v>3.81</v>
       </c>
       <c r="E27" t="n">
-        <v>16.7</v>
+        <v>40</v>
       </c>
       <c r="F27" t="n">
-        <v>27.8</v>
+        <v>20</v>
       </c>
       <c r="G27" t="n">
-        <v>24.4</v>
+        <v>26</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>28.26</v>
+        <v>26.19</v>
       </c>
       <c r="D28" t="n">
-        <v>2.31</v>
+        <v>2.15</v>
       </c>
       <c r="E28" t="n">
-        <v>27.8</v>
+        <v>20</v>
       </c>
       <c r="F28" t="n">
-        <v>22.2</v>
+        <v>30</v>
       </c>
       <c r="G28" t="n">
-        <v>23.9</v>
+        <v>25</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>20.3</v>
+        <v>23.88</v>
       </c>
       <c r="D29" t="n">
-        <v>3.81</v>
+        <v>1.74</v>
       </c>
       <c r="E29" t="n">
-        <v>38.9</v>
+        <v>20</v>
       </c>
       <c r="F29" t="n">
-        <v>16.7</v>
+        <v>30</v>
       </c>
       <c r="G29" t="n">
-        <v>23.3</v>
+        <v>25</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.83</v>
       </c>
       <c r="E30" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="F30" t="n">
-        <v>16.7</v>
+        <v>20</v>
       </c>
       <c r="G30" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>0.66</v>
       </c>
       <c r="E31" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="F31" t="n">
-        <v>16.7</v>
+        <v>20</v>
       </c>
       <c r="G31" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.12</v>
       </c>
       <c r="E32" t="n">
-        <v>16.7</v>
+        <v>20</v>
       </c>
       <c r="F32" t="n">
-        <v>16.7</v>
+        <v>20</v>
       </c>
       <c r="G32" t="n">
-        <v>16.7</v>
+        <v>20</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun May  3 10:38:15 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>4.91</v>
       </c>
       <c r="E2" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.25</v>
       </c>
       <c r="E3" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.4</v>
       </c>
       <c r="E4" t="n">
-        <v>70</v>
+        <v>68.2</v>
       </c>
       <c r="F4" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>4.01</v>
       </c>
       <c r="E5" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="F5" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="G5" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.86</v>
       </c>
       <c r="E6" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="F6" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="G6" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.35</v>
       </c>
       <c r="E7" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>65</v>
+        <v>63.6</v>
       </c>
       <c r="G7" t="n">
-        <v>77.5</v>
+        <v>75</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.8</v>
       </c>
       <c r="E8" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>60</v>
+        <v>59.1</v>
       </c>
       <c r="G8" t="n">
-        <v>75</v>
+        <v>72.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.48</v>
       </c>
       <c r="E9" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="F9" t="n">
-        <v>65</v>
+        <v>63.6</v>
       </c>
       <c r="G9" t="n">
-        <v>72.5</v>
+        <v>70.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>4.3</v>
       </c>
       <c r="E10" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>40</v>
+        <v>40.9</v>
       </c>
       <c r="G10" t="n">
-        <v>65</v>
+        <v>63.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.41</v>
       </c>
       <c r="E11" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="G11" t="n">
-        <v>60</v>
+        <v>59.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.53</v>
       </c>
       <c r="E12" t="n">
-        <v>60</v>
+        <v>59.1</v>
       </c>
       <c r="F12" t="n">
-        <v>60</v>
+        <v>59.1</v>
       </c>
       <c r="G12" t="n">
-        <v>60</v>
+        <v>59.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.27</v>
       </c>
       <c r="E13" t="n">
-        <v>60</v>
+        <v>59.1</v>
       </c>
       <c r="F13" t="n">
-        <v>55</v>
+        <v>54.5</v>
       </c>
       <c r="G13" t="n">
-        <v>57.5</v>
+        <v>56.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.82</v>
       </c>
       <c r="E14" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="F14" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="G14" t="n">
-        <v>55</v>
+        <v>54.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>6.35</v>
       </c>
       <c r="E15" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="F15" t="n">
-        <v>80</v>
+        <v>77.3</v>
       </c>
       <c r="G15" t="n">
-        <v>55</v>
+        <v>54.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.15</v>
       </c>
       <c r="E16" t="n">
-        <v>40</v>
+        <v>40.9</v>
       </c>
       <c r="F16" t="n">
-        <v>70</v>
+        <v>68.2</v>
       </c>
       <c r="G16" t="n">
-        <v>55</v>
+        <v>54.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.87</v>
       </c>
       <c r="E17" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="F17" t="n">
-        <v>70</v>
+        <v>68.2</v>
       </c>
       <c r="G17" t="n">
-        <v>45</v>
+        <v>45.5</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.76</v>
       </c>
       <c r="E18" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="F18" t="n">
-        <v>60</v>
+        <v>59.1</v>
       </c>
       <c r="G18" t="n">
-        <v>45</v>
+        <v>45.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.28</v>
       </c>
       <c r="E19" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>25</v>
+        <v>27.3</v>
       </c>
       <c r="G19" t="n">
-        <v>44.5</v>
+        <v>45</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.75</v>
       </c>
       <c r="E20" t="n">
-        <v>90</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F20" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="G20" t="n">
-        <v>41</v>
+        <v>41.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.67</v>
       </c>
       <c r="E21" t="n">
-        <v>40</v>
+        <v>40.9</v>
       </c>
       <c r="F21" t="n">
-        <v>40</v>
+        <v>40.9</v>
       </c>
       <c r="G21" t="n">
-        <v>40</v>
+        <v>40.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.72</v>
       </c>
       <c r="E22" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="F22" t="n">
-        <v>45</v>
+        <v>45.5</v>
       </c>
       <c r="G22" t="n">
-        <v>37.5</v>
+        <v>38.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>4.27</v>
       </c>
       <c r="E23" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="F23" t="n">
         <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>35</v>
+        <v>36.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.67</v>
       </c>
       <c r="E24" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="F24" t="n">
-        <v>40</v>
+        <v>40.9</v>
       </c>
       <c r="G24" t="n">
-        <v>35</v>
+        <v>36.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.73</v>
       </c>
       <c r="E25" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="F25" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="G25" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.31</v>
       </c>
       <c r="E26" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="F26" t="n">
-        <v>25</v>
+        <v>27.3</v>
       </c>
       <c r="G26" t="n">
-        <v>26.5</v>
+        <v>28.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.81</v>
       </c>
       <c r="E27" t="n">
-        <v>40</v>
+        <v>40.9</v>
       </c>
       <c r="F27" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="G27" t="n">
-        <v>26</v>
+        <v>28.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.15</v>
       </c>
       <c r="E28" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="F28" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="G28" t="n">
-        <v>25</v>
+        <v>27.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.74</v>
       </c>
       <c r="E29" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="F29" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="G29" t="n">
-        <v>25</v>
+        <v>27.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.83</v>
       </c>
       <c r="E30" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="F30" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="G30" t="n">
-        <v>23</v>
+        <v>25.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>0.66</v>
       </c>
       <c r="E31" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="F31" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="G31" t="n">
-        <v>23</v>
+        <v>25.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.12</v>
       </c>
       <c r="E32" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="F32" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="G32" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon May  4 11:27:20 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>4.91</v>
       </c>
       <c r="E2" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="F2" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="G2" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.25</v>
       </c>
       <c r="E3" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="F3" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="G3" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.4</v>
       </c>
       <c r="E4" t="n">
-        <v>68.2</v>
+        <v>66.7</v>
       </c>
       <c r="F4" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="G4" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>4.01</v>
       </c>
       <c r="E5" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="G5" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.86</v>
       </c>
       <c r="E6" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="G6" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.35</v>
       </c>
       <c r="E7" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="F7" t="n">
-        <v>63.6</v>
+        <v>62.5</v>
       </c>
       <c r="G7" t="n">
-        <v>75</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.8</v>
       </c>
       <c r="E8" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="F8" t="n">
-        <v>59.1</v>
+        <v>58.3</v>
       </c>
       <c r="G8" t="n">
-        <v>72.7</v>
+        <v>70.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.48</v>
       </c>
       <c r="E9" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="F9" t="n">
-        <v>63.6</v>
+        <v>62.5</v>
       </c>
       <c r="G9" t="n">
-        <v>70.5</v>
+        <v>68.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>4.3</v>
       </c>
       <c r="E10" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="F10" t="n">
-        <v>40.9</v>
+        <v>41.7</v>
       </c>
       <c r="G10" t="n">
-        <v>63.6</v>
+        <v>62.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.41</v>
       </c>
       <c r="E11" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="F11" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="G11" t="n">
-        <v>59.1</v>
+        <v>58.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.53</v>
       </c>
       <c r="E12" t="n">
-        <v>59.1</v>
+        <v>58.3</v>
       </c>
       <c r="F12" t="n">
-        <v>59.1</v>
+        <v>58.3</v>
       </c>
       <c r="G12" t="n">
-        <v>59.1</v>
+        <v>58.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.27</v>
       </c>
       <c r="E13" t="n">
-        <v>59.1</v>
+        <v>58.3</v>
       </c>
       <c r="F13" t="n">
-        <v>54.5</v>
+        <v>54.2</v>
       </c>
       <c r="G13" t="n">
-        <v>56.8</v>
+        <v>56.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.82</v>
       </c>
       <c r="E14" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="F14" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="G14" t="n">
-        <v>54.5</v>
+        <v>54.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>6.35</v>
       </c>
       <c r="E15" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="F15" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="G15" t="n">
-        <v>54.5</v>
+        <v>54.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.15</v>
       </c>
       <c r="E16" t="n">
-        <v>40.9</v>
+        <v>41.7</v>
       </c>
       <c r="F16" t="n">
-        <v>68.2</v>
+        <v>66.7</v>
       </c>
       <c r="G16" t="n">
-        <v>54.5</v>
+        <v>54.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.87</v>
       </c>
       <c r="E17" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="F17" t="n">
-        <v>68.2</v>
+        <v>66.7</v>
       </c>
       <c r="G17" t="n">
-        <v>45.5</v>
+        <v>45.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.76</v>
       </c>
       <c r="E18" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="F18" t="n">
-        <v>59.1</v>
+        <v>58.3</v>
       </c>
       <c r="G18" t="n">
-        <v>45.5</v>
+        <v>45.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.28</v>
       </c>
       <c r="E19" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="F19" t="n">
-        <v>27.3</v>
+        <v>29.2</v>
       </c>
       <c r="G19" t="n">
-        <v>45</v>
+        <v>45.4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.75</v>
       </c>
       <c r="E20" t="n">
-        <v>86.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="F20" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="G20" t="n">
-        <v>41.8</v>
+        <v>42.5</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.67</v>
       </c>
       <c r="E21" t="n">
-        <v>40.9</v>
+        <v>41.7</v>
       </c>
       <c r="F21" t="n">
-        <v>40.9</v>
+        <v>41.7</v>
       </c>
       <c r="G21" t="n">
-        <v>40.9</v>
+        <v>41.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.72</v>
       </c>
       <c r="E22" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="F22" t="n">
-        <v>45.5</v>
+        <v>45.8</v>
       </c>
       <c r="G22" t="n">
-        <v>38.6</v>
+        <v>39.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>4.27</v>
       </c>
       <c r="E23" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="F23" t="n">
         <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>36.4</v>
+        <v>37.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.67</v>
       </c>
       <c r="E24" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="F24" t="n">
-        <v>40.9</v>
+        <v>41.7</v>
       </c>
       <c r="G24" t="n">
-        <v>36.4</v>
+        <v>37.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.73</v>
       </c>
       <c r="E25" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="F25" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="G25" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.31</v>
       </c>
       <c r="E26" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="F26" t="n">
-        <v>27.3</v>
+        <v>29.2</v>
       </c>
       <c r="G26" t="n">
-        <v>28.6</v>
+        <v>30.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.81</v>
       </c>
       <c r="E27" t="n">
-        <v>40.9</v>
+        <v>41.7</v>
       </c>
       <c r="F27" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="G27" t="n">
-        <v>28.2</v>
+        <v>30</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.15</v>
       </c>
       <c r="E28" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="F28" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="G28" t="n">
-        <v>27.3</v>
+        <v>29.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.74</v>
       </c>
       <c r="E29" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="F29" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="G29" t="n">
-        <v>27.3</v>
+        <v>29.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.83</v>
       </c>
       <c r="E30" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="F30" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="G30" t="n">
-        <v>25.5</v>
+        <v>27.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>0.66</v>
       </c>
       <c r="E31" t="n">
-        <v>31.8</v>
+        <v>33.3</v>
       </c>
       <c r="F31" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="G31" t="n">
-        <v>25.5</v>
+        <v>27.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.12</v>
       </c>
       <c r="E32" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="F32" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="G32" t="n">
-        <v>22.7</v>
+        <v>25</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue May  5 11:06:41 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>4.91</v>
       </c>
       <c r="E2" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="F2" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="G2" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.25</v>
       </c>
       <c r="E3" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="F3" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="G3" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.4</v>
       </c>
       <c r="E4" t="n">
-        <v>66.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="G4" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>4.01</v>
       </c>
       <c r="E5" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.86</v>
       </c>
       <c r="E6" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.35</v>
       </c>
       <c r="E7" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="F7" t="n">
-        <v>62.5</v>
+        <v>61.5</v>
       </c>
       <c r="G7" t="n">
-        <v>72.90000000000001</v>
+        <v>71.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.8</v>
       </c>
       <c r="E8" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="F8" t="n">
-        <v>58.3</v>
+        <v>57.7</v>
       </c>
       <c r="G8" t="n">
-        <v>70.8</v>
+        <v>69.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.48</v>
       </c>
       <c r="E9" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>62.5</v>
+        <v>61.5</v>
       </c>
       <c r="G9" t="n">
-        <v>68.8</v>
+        <v>67.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>4.3</v>
       </c>
       <c r="E10" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="F10" t="n">
-        <v>41.7</v>
+        <v>42.3</v>
       </c>
       <c r="G10" t="n">
-        <v>62.5</v>
+        <v>61.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.41</v>
       </c>
       <c r="E11" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="F11" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="G11" t="n">
-        <v>58.3</v>
+        <v>57.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="12">
@@ -792,76 +792,76 @@
         <v>1.53</v>
       </c>
       <c r="E12" t="n">
-        <v>58.3</v>
+        <v>57.7</v>
       </c>
       <c r="F12" t="n">
-        <v>58.3</v>
+        <v>57.7</v>
       </c>
       <c r="G12" t="n">
-        <v>58.3</v>
+        <v>57.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>15.53</v>
+        <v>10.52</v>
       </c>
       <c r="D13" t="n">
-        <v>1.27</v>
+        <v>1.28</v>
       </c>
       <c r="E13" t="n">
-        <v>58.3</v>
+        <v>80.8</v>
       </c>
       <c r="F13" t="n">
-        <v>54.2</v>
+        <v>30.8</v>
       </c>
       <c r="G13" t="n">
-        <v>56.2</v>
+        <v>55.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21.9</v>
+        <v>15.53</v>
       </c>
       <c r="D14" t="n">
-        <v>1.82</v>
+        <v>1.27</v>
       </c>
       <c r="E14" t="n">
-        <v>75</v>
+        <v>57.7</v>
       </c>
       <c r="F14" t="n">
-        <v>33.3</v>
+        <v>53.8</v>
       </c>
       <c r="G14" t="n">
-        <v>54.2</v>
+        <v>55.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>6.35</v>
       </c>
       <c r="E15" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="F15" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>54.2</v>
+        <v>53.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="16">
@@ -912,46 +912,46 @@
         <v>1.15</v>
       </c>
       <c r="E16" t="n">
-        <v>41.7</v>
+        <v>42.3</v>
       </c>
       <c r="F16" t="n">
-        <v>66.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>54.2</v>
+        <v>53.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>22.9</v>
+        <v>21.9</v>
       </c>
       <c r="D17" t="n">
-        <v>3.87</v>
+        <v>1.82</v>
       </c>
       <c r="E17" t="n">
-        <v>25</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>66.7</v>
+        <v>34.6</v>
       </c>
       <c r="G17" t="n">
-        <v>45.8</v>
+        <v>53.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="18">
@@ -972,46 +972,46 @@
         <v>2.76</v>
       </c>
       <c r="E18" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="F18" t="n">
-        <v>58.3</v>
+        <v>57.7</v>
       </c>
       <c r="G18" t="n">
-        <v>45.8</v>
+        <v>46.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.52</v>
+        <v>22.9</v>
       </c>
       <c r="D19" t="n">
-        <v>1.28</v>
+        <v>3.87</v>
       </c>
       <c r="E19" t="n">
-        <v>83.3</v>
+        <v>26.9</v>
       </c>
       <c r="F19" t="n">
-        <v>29.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>45.4</v>
+        <v>46.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.75</v>
       </c>
       <c r="E20" t="n">
-        <v>83.3</v>
+        <v>80.8</v>
       </c>
       <c r="F20" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="G20" t="n">
-        <v>42.5</v>
+        <v>43.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.67</v>
       </c>
       <c r="E21" t="n">
-        <v>41.7</v>
+        <v>42.3</v>
       </c>
       <c r="F21" t="n">
-        <v>41.7</v>
+        <v>42.3</v>
       </c>
       <c r="G21" t="n">
-        <v>41.7</v>
+        <v>42.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.72</v>
       </c>
       <c r="E22" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="F22" t="n">
-        <v>45.8</v>
+        <v>46.2</v>
       </c>
       <c r="G22" t="n">
-        <v>39.6</v>
+        <v>40.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>4.27</v>
       </c>
       <c r="E23" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="F23" t="n">
         <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>37.5</v>
+        <v>38.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.67</v>
       </c>
       <c r="E24" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="F24" t="n">
-        <v>41.7</v>
+        <v>42.3</v>
       </c>
       <c r="G24" t="n">
-        <v>37.5</v>
+        <v>38.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.73</v>
       </c>
       <c r="E25" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="F25" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="G25" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.31</v>
       </c>
       <c r="E26" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="F26" t="n">
-        <v>29.2</v>
+        <v>30.8</v>
       </c>
       <c r="G26" t="n">
-        <v>30.4</v>
+        <v>32.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.81</v>
       </c>
       <c r="E27" t="n">
-        <v>41.7</v>
+        <v>42.3</v>
       </c>
       <c r="F27" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="G27" t="n">
-        <v>30</v>
+        <v>31.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.15</v>
       </c>
       <c r="E28" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="F28" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="G28" t="n">
-        <v>29.2</v>
+        <v>30.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.74</v>
       </c>
       <c r="E29" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="F29" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="G29" t="n">
-        <v>29.2</v>
+        <v>30.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.83</v>
       </c>
       <c r="E30" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="F30" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="G30" t="n">
-        <v>27.5</v>
+        <v>29.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>0.66</v>
       </c>
       <c r="E31" t="n">
-        <v>33.3</v>
+        <v>34.6</v>
       </c>
       <c r="F31" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="G31" t="n">
-        <v>27.5</v>
+        <v>29.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.12</v>
       </c>
       <c r="E32" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="F32" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="G32" t="n">
-        <v>25</v>
+        <v>26.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed May  6 11:30:32 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,31 +477,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>130.93</v>
+        <v>38.18</v>
       </c>
       <c r="D2" t="n">
-        <v>4.91</v>
+        <v>4.11</v>
       </c>
       <c r="E2" t="n">
-        <v>80.8</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>80.8</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>80.8</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="3">
@@ -516,592 +516,592 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>38.54</v>
+        <v>39.3</v>
       </c>
       <c r="D3" t="n">
-        <v>3.25</v>
+        <v>3.31</v>
       </c>
       <c r="E3" t="n">
-        <v>80.8</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>80.8</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>80.8</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>32.34</v>
+        <v>53.99</v>
       </c>
       <c r="D4" t="n">
-        <v>2.4</v>
+        <v>4.44</v>
       </c>
       <c r="E4" t="n">
-        <v>65.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>80.8</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>73.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>36.66</v>
+        <v>35.34</v>
       </c>
       <c r="D5" t="n">
-        <v>4.01</v>
+        <v>1.96</v>
       </c>
       <c r="E5" t="n">
-        <v>73.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>73.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>73.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>33.47</v>
+        <v>138.34</v>
       </c>
       <c r="D6" t="n">
-        <v>1.86</v>
+        <v>5.18</v>
       </c>
       <c r="E6" t="n">
-        <v>73.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>73.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>73.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25.97</v>
+        <v>10.59</v>
       </c>
       <c r="D7" t="n">
-        <v>2.35</v>
+        <v>1.29</v>
       </c>
       <c r="E7" t="n">
-        <v>80.8</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>61.5</v>
+        <v>75</v>
       </c>
       <c r="G7" t="n">
-        <v>71.2</v>
+        <v>87.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.68</v>
+        <v>29.37</v>
       </c>
       <c r="D8" t="n">
-        <v>1.8</v>
+        <v>2.69</v>
       </c>
       <c r="E8" t="n">
-        <v>80.8</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>57.7</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>69.2</v>
+        <v>87.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>26.73</v>
+        <v>32.42</v>
       </c>
       <c r="D9" t="n">
-        <v>2.48</v>
+        <v>2.4</v>
       </c>
       <c r="E9" t="n">
-        <v>73.09999999999999</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>61.5</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>67.3</v>
+        <v>85.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>52.4</v>
+        <v>15.65</v>
       </c>
       <c r="D10" t="n">
-        <v>4.3</v>
+        <v>1.28</v>
       </c>
       <c r="E10" t="n">
-        <v>80.8</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>42.3</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>61.5</v>
+        <v>85.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16.28</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>2.41</v>
+        <v>6.61</v>
       </c>
       <c r="E11" t="n">
-        <v>80.8</v>
+        <v>64.3</v>
       </c>
       <c r="F11" t="n">
-        <v>34.6</v>
+        <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>57.7</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>16.22</v>
+        <v>23.7</v>
       </c>
       <c r="D12" t="n">
-        <v>1.53</v>
+        <v>4.01</v>
       </c>
       <c r="E12" t="n">
-        <v>57.7</v>
+        <v>64.3</v>
       </c>
       <c r="F12" t="n">
-        <v>57.7</v>
+        <v>100</v>
       </c>
       <c r="G12" t="n">
-        <v>57.7</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.52</v>
+        <v>13.06</v>
       </c>
       <c r="D13" t="n">
-        <v>1.28</v>
+        <v>1.17</v>
       </c>
       <c r="E13" t="n">
-        <v>80.8</v>
+        <v>64.3</v>
       </c>
       <c r="F13" t="n">
-        <v>30.8</v>
+        <v>100</v>
       </c>
       <c r="G13" t="n">
-        <v>55.8</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.53</v>
+        <v>29.08</v>
       </c>
       <c r="D14" t="n">
-        <v>1.27</v>
+        <v>2.75</v>
       </c>
       <c r="E14" t="n">
-        <v>57.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>53.8</v>
+        <v>89.3</v>
       </c>
       <c r="G14" t="n">
-        <v>55.8</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>61.6</v>
+        <v>26.03</v>
       </c>
       <c r="D15" t="n">
-        <v>6.35</v>
+        <v>2.35</v>
       </c>
       <c r="E15" t="n">
-        <v>34.6</v>
+        <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>73.09999999999999</v>
+        <v>60.7</v>
       </c>
       <c r="G15" t="n">
-        <v>53.8</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>12.69</v>
+        <v>26.97</v>
       </c>
       <c r="D16" t="n">
-        <v>1.15</v>
+        <v>2.48</v>
       </c>
       <c r="E16" t="n">
-        <v>42.3</v>
+        <v>100</v>
       </c>
       <c r="F16" t="n">
-        <v>65.40000000000001</v>
+        <v>60.7</v>
       </c>
       <c r="G16" t="n">
-        <v>53.8</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>21.9</v>
+        <v>16.39</v>
       </c>
       <c r="D17" t="n">
-        <v>1.82</v>
+        <v>2.42</v>
       </c>
       <c r="E17" t="n">
-        <v>73.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="F17" t="n">
-        <v>34.6</v>
+        <v>57.1</v>
       </c>
       <c r="G17" t="n">
-        <v>53.8</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>33</v>
+        <v>30.13</v>
       </c>
       <c r="D18" t="n">
-        <v>2.76</v>
+        <v>2.75</v>
       </c>
       <c r="E18" t="n">
-        <v>34.6</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>57.7</v>
+        <v>60.7</v>
       </c>
       <c r="G18" t="n">
-        <v>46.2</v>
+        <v>76.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22.9</v>
+        <v>33.34</v>
       </c>
       <c r="D19" t="n">
-        <v>3.87</v>
+        <v>2.79</v>
       </c>
       <c r="E19" t="n">
-        <v>26.9</v>
+        <v>64.3</v>
       </c>
       <c r="F19" t="n">
-        <v>65.40000000000001</v>
+        <v>89.3</v>
       </c>
       <c r="G19" t="n">
-        <v>46.2</v>
+        <v>76.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>11.72</v>
+        <v>24.2</v>
       </c>
       <c r="D20" t="n">
-        <v>0.75</v>
+        <v>1.78</v>
       </c>
       <c r="E20" t="n">
-        <v>80.8</v>
+        <v>53.6</v>
       </c>
       <c r="F20" t="n">
-        <v>26.9</v>
+        <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>43.1</v>
+        <v>76.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>35.11</v>
+        <v>19.94</v>
       </c>
       <c r="D21" t="n">
-        <v>2.67</v>
+        <v>1.86</v>
       </c>
       <c r="E21" t="n">
-        <v>42.3</v>
+        <v>100</v>
       </c>
       <c r="F21" t="n">
-        <v>42.3</v>
+        <v>50</v>
       </c>
       <c r="G21" t="n">
-        <v>42.3</v>
+        <v>75</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28.66</v>
+        <v>28.79</v>
       </c>
       <c r="D22" t="n">
-        <v>2.72</v>
+        <v>2.35</v>
       </c>
       <c r="E22" t="n">
-        <v>34.6</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>46.2</v>
+        <v>57.1</v>
       </c>
       <c r="G22" t="n">
-        <v>40.4</v>
+        <v>75</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="23">
@@ -1116,292 +1116,292 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>65.68000000000001</v>
+        <v>66.84</v>
       </c>
       <c r="D23" t="n">
-        <v>4.27</v>
+        <v>4.34</v>
       </c>
       <c r="E23" t="n">
-        <v>26.9</v>
+        <v>50</v>
       </c>
       <c r="F23" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>38.5</v>
+        <v>75</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>29.11</v>
+        <v>21.95</v>
       </c>
       <c r="D24" t="n">
-        <v>2.67</v>
+        <v>1.83</v>
       </c>
       <c r="E24" t="n">
-        <v>34.6</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>42.3</v>
+        <v>57.1</v>
       </c>
       <c r="G24" t="n">
-        <v>38.5</v>
+        <v>75</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29.95</v>
+        <v>19.65</v>
       </c>
       <c r="D25" t="n">
-        <v>2.73</v>
+        <v>1.8</v>
       </c>
       <c r="E25" t="n">
-        <v>34.6</v>
+        <v>57.1</v>
       </c>
       <c r="F25" t="n">
-        <v>34.6</v>
+        <v>57.1</v>
       </c>
       <c r="G25" t="n">
-        <v>34.6</v>
+        <v>57.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>28.26</v>
+        <v>11.79</v>
       </c>
       <c r="D26" t="n">
-        <v>2.31</v>
+        <v>0.75</v>
       </c>
       <c r="E26" t="n">
-        <v>34.6</v>
+        <v>100</v>
       </c>
       <c r="F26" t="n">
-        <v>30.8</v>
+        <v>28.6</v>
       </c>
       <c r="G26" t="n">
-        <v>32.7</v>
+        <v>50</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>20.3</v>
+        <v>20.34</v>
       </c>
       <c r="D27" t="n">
-        <v>3.81</v>
+        <v>1.13</v>
       </c>
       <c r="E27" t="n">
-        <v>42.3</v>
+        <v>50</v>
       </c>
       <c r="F27" t="n">
-        <v>26.9</v>
+        <v>50</v>
       </c>
       <c r="G27" t="n">
-        <v>31.5</v>
+        <v>50</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>26.19</v>
+        <v>21.87</v>
       </c>
       <c r="D28" t="n">
-        <v>2.15</v>
+        <v>3.8</v>
       </c>
       <c r="E28" t="n">
-        <v>26.9</v>
+        <v>100</v>
       </c>
       <c r="F28" t="n">
-        <v>34.6</v>
+        <v>7.1</v>
       </c>
       <c r="G28" t="n">
-        <v>30.8</v>
+        <v>35</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>23.88</v>
+        <v>26.19</v>
       </c>
       <c r="D29" t="n">
-        <v>1.74</v>
+        <v>2.15</v>
       </c>
       <c r="E29" t="n">
-        <v>26.9</v>
+        <v>28.6</v>
       </c>
       <c r="F29" t="n">
-        <v>34.6</v>
+        <v>35.7</v>
       </c>
       <c r="G29" t="n">
-        <v>30.8</v>
+        <v>32.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.62</v>
+        <v>6.87</v>
       </c>
       <c r="D30" t="n">
-        <v>1.83</v>
+        <v>0.65</v>
       </c>
       <c r="E30" t="n">
-        <v>34.6</v>
+        <v>14.3</v>
       </c>
       <c r="F30" t="n">
-        <v>26.9</v>
+        <v>7.1</v>
       </c>
       <c r="G30" t="n">
-        <v>29.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>6.94</v>
+        <v>34.21</v>
       </c>
       <c r="D31" t="n">
-        <v>0.66</v>
+        <v>2.61</v>
       </c>
       <c r="E31" t="n">
-        <v>34.6</v>
+        <v>7.1</v>
       </c>
       <c r="F31" t="n">
-        <v>26.9</v>
+        <v>7.1</v>
       </c>
       <c r="G31" t="n">
-        <v>29.2</v>
+        <v>7.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>20.14</v>
+        <v>15.79</v>
       </c>
       <c r="D32" t="n">
-        <v>1.12</v>
+        <v>1.49</v>
       </c>
       <c r="E32" t="n">
-        <v>26.9</v>
+        <v>7.1</v>
       </c>
       <c r="F32" t="n">
-        <v>26.9</v>
+        <v>7.1</v>
       </c>
       <c r="G32" t="n">
-        <v>26.9</v>
+        <v>7.1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu May  7 11:29:41 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>38.18</v>
+        <v>27.34</v>
       </c>
       <c r="D2" t="n">
-        <v>4.11</v>
+        <v>2.52</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,25 +501,25 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>39.3</v>
+        <v>26.26</v>
       </c>
       <c r="D3" t="n">
-        <v>3.31</v>
+        <v>2.38</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -531,25 +531,25 @@
         <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>53.99</v>
+        <v>29.81</v>
       </c>
       <c r="D4" t="n">
-        <v>4.44</v>
+        <v>2.82</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
@@ -561,25 +561,25 @@
         <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>35.34</v>
+        <v>54.89</v>
       </c>
       <c r="D5" t="n">
-        <v>1.96</v>
+        <v>4.52</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
@@ -591,25 +591,25 @@
         <v>100</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>138.34</v>
+        <v>40.39</v>
       </c>
       <c r="D6" t="n">
-        <v>5.18</v>
+        <v>3.41</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
@@ -621,127 +621,127 @@
         <v>100</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10.59</v>
+        <v>36.22</v>
       </c>
       <c r="D7" t="n">
-        <v>1.29</v>
+        <v>2.01</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>87.5</v>
+        <v>100</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>29.37</v>
+        <v>144.85</v>
       </c>
       <c r="D8" t="n">
-        <v>2.69</v>
+        <v>5.43</v>
       </c>
       <c r="E8" t="n">
-        <v>78.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>96.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>87.5</v>
+        <v>100</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>32.42</v>
+        <v>24.76</v>
       </c>
       <c r="D9" t="n">
-        <v>2.4</v>
+        <v>1.82</v>
       </c>
       <c r="E9" t="n">
-        <v>92.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>78.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>15.65</v>
+        <v>29.37</v>
       </c>
       <c r="D10" t="n">
-        <v>1.28</v>
+        <v>2.4</v>
       </c>
       <c r="E10" t="n">
-        <v>78.59999999999999</v>
+        <v>93.3</v>
       </c>
       <c r="F10" t="n">
-        <v>92.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>85.7</v>
+        <v>96.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="11">
@@ -756,232 +756,232 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>64.09999999999999</v>
+        <v>65.81</v>
       </c>
       <c r="D11" t="n">
-        <v>6.61</v>
+        <v>6.79</v>
       </c>
       <c r="E11" t="n">
-        <v>64.3</v>
+        <v>93.3</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>82.09999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>23.7</v>
+        <v>12.06</v>
       </c>
       <c r="D12" t="n">
-        <v>4.01</v>
+        <v>0.77</v>
       </c>
       <c r="E12" t="n">
-        <v>64.3</v>
+        <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>100</v>
+        <v>86.7</v>
       </c>
       <c r="G12" t="n">
-        <v>82.09999999999999</v>
+        <v>93.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>13.06</v>
+        <v>38.1</v>
       </c>
       <c r="D13" t="n">
-        <v>1.17</v>
+        <v>4.1</v>
       </c>
       <c r="E13" t="n">
-        <v>64.3</v>
+        <v>93.3</v>
       </c>
       <c r="F13" t="n">
-        <v>100</v>
+        <v>93.3</v>
       </c>
       <c r="G13" t="n">
-        <v>82.09999999999999</v>
+        <v>93.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>29.08</v>
+        <v>10.64</v>
       </c>
       <c r="D14" t="n">
-        <v>2.75</v>
+        <v>1.29</v>
       </c>
       <c r="E14" t="n">
-        <v>71.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>89.3</v>
+        <v>73.3</v>
       </c>
       <c r="G14" t="n">
-        <v>80.40000000000001</v>
+        <v>86.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26.03</v>
+        <v>15.7</v>
       </c>
       <c r="D15" t="n">
-        <v>2.35</v>
+        <v>1.28</v>
       </c>
       <c r="E15" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F15" t="n">
-        <v>60.7</v>
+        <v>90</v>
       </c>
       <c r="G15" t="n">
-        <v>80.40000000000001</v>
+        <v>85</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26.97</v>
+        <v>13.15</v>
       </c>
       <c r="D16" t="n">
-        <v>2.48</v>
+        <v>1.19</v>
       </c>
       <c r="E16" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="F16" t="n">
-        <v>60.7</v>
+        <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>80.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>16.39</v>
+        <v>23.81</v>
       </c>
       <c r="D17" t="n">
-        <v>2.42</v>
+        <v>4.03</v>
       </c>
       <c r="E17" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="F17" t="n">
-        <v>57.1</v>
+        <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>78.59999999999999</v>
+        <v>83.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>30.13</v>
+        <v>20.19</v>
       </c>
       <c r="D18" t="n">
-        <v>2.75</v>
+        <v>1.88</v>
       </c>
       <c r="E18" t="n">
-        <v>92.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F18" t="n">
-        <v>60.7</v>
+        <v>63.3</v>
       </c>
       <c r="G18" t="n">
-        <v>76.8</v>
+        <v>81.7</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="19">
@@ -996,322 +996,322 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>33.34</v>
+        <v>33.37</v>
       </c>
       <c r="D19" t="n">
-        <v>2.79</v>
+        <v>2.8</v>
       </c>
       <c r="E19" t="n">
-        <v>64.3</v>
+        <v>66.7</v>
       </c>
       <c r="F19" t="n">
-        <v>89.3</v>
+        <v>96.7</v>
       </c>
       <c r="G19" t="n">
-        <v>76.8</v>
+        <v>81.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>24.2</v>
+        <v>16.46</v>
       </c>
       <c r="D20" t="n">
-        <v>1.78</v>
+        <v>2.43</v>
       </c>
       <c r="E20" t="n">
-        <v>53.6</v>
+        <v>100</v>
       </c>
       <c r="F20" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="G20" t="n">
-        <v>76.8</v>
+        <v>80</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>19.94</v>
+        <v>67.37</v>
       </c>
       <c r="D21" t="n">
-        <v>1.86</v>
+        <v>4.38</v>
       </c>
       <c r="E21" t="n">
-        <v>100</v>
+        <v>53.3</v>
       </c>
       <c r="F21" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>75</v>
+        <v>76.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28.79</v>
+        <v>22.04</v>
       </c>
       <c r="D22" t="n">
-        <v>2.35</v>
+        <v>1.83</v>
       </c>
       <c r="E22" t="n">
-        <v>92.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="F22" t="n">
-        <v>57.1</v>
+        <v>56.7</v>
       </c>
       <c r="G22" t="n">
         <v>75</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>66.84</v>
+        <v>30</v>
       </c>
       <c r="D23" t="n">
-        <v>4.34</v>
+        <v>2.76</v>
       </c>
       <c r="E23" t="n">
-        <v>50</v>
+        <v>73.3</v>
       </c>
       <c r="F23" t="n">
-        <v>100</v>
+        <v>73.3</v>
       </c>
       <c r="G23" t="n">
-        <v>75</v>
+        <v>73.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>21.95</v>
+        <v>26.31</v>
       </c>
       <c r="D24" t="n">
-        <v>1.83</v>
+        <v>2.16</v>
       </c>
       <c r="E24" t="n">
-        <v>92.90000000000001</v>
+        <v>53.3</v>
       </c>
       <c r="F24" t="n">
-        <v>57.1</v>
+        <v>63.3</v>
       </c>
       <c r="G24" t="n">
-        <v>75</v>
+        <v>58.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>19.65</v>
+        <v>32.05</v>
       </c>
       <c r="D25" t="n">
-        <v>1.8</v>
+        <v>2.38</v>
       </c>
       <c r="E25" t="n">
-        <v>57.1</v>
+        <v>40</v>
       </c>
       <c r="F25" t="n">
-        <v>57.1</v>
+        <v>53.3</v>
       </c>
       <c r="G25" t="n">
-        <v>57.1</v>
+        <v>46.7</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>11.79</v>
+        <v>20.2</v>
       </c>
       <c r="D26" t="n">
-        <v>0.75</v>
+        <v>1.12</v>
       </c>
       <c r="E26" t="n">
-        <v>100</v>
+        <v>46.7</v>
       </c>
       <c r="F26" t="n">
-        <v>28.6</v>
+        <v>26.7</v>
       </c>
       <c r="G26" t="n">
-        <v>50</v>
+        <v>32.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>20.34</v>
+        <v>21.84</v>
       </c>
       <c r="D27" t="n">
-        <v>1.13</v>
+        <v>3.79</v>
       </c>
       <c r="E27" t="n">
-        <v>50</v>
+        <v>93.3</v>
       </c>
       <c r="F27" t="n">
-        <v>50</v>
+        <v>6.7</v>
       </c>
       <c r="G27" t="n">
-        <v>50</v>
+        <v>32.7</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>21.87</v>
+        <v>34.49</v>
       </c>
       <c r="D28" t="n">
-        <v>3.8</v>
+        <v>2.63</v>
       </c>
       <c r="E28" t="n">
-        <v>100</v>
+        <v>13.3</v>
       </c>
       <c r="F28" t="n">
-        <v>7.1</v>
+        <v>23.3</v>
       </c>
       <c r="G28" t="n">
-        <v>35</v>
+        <v>20.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26.19</v>
+        <v>28.99</v>
       </c>
       <c r="D29" t="n">
-        <v>2.15</v>
+        <v>2.66</v>
       </c>
       <c r="E29" t="n">
-        <v>28.6</v>
+        <v>13.3</v>
       </c>
       <c r="F29" t="n">
-        <v>35.7</v>
+        <v>16.7</v>
       </c>
       <c r="G29" t="n">
-        <v>32.1</v>
+        <v>15.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="30">
@@ -1326,82 +1326,82 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6.87</v>
+        <v>6.85</v>
       </c>
       <c r="D30" t="n">
         <v>0.65</v>
       </c>
       <c r="E30" t="n">
-        <v>14.3</v>
+        <v>13.3</v>
       </c>
       <c r="F30" t="n">
-        <v>7.1</v>
+        <v>10</v>
       </c>
       <c r="G30" t="n">
-        <v>9.300000000000001</v>
+        <v>11</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>34.21</v>
+        <v>15.07</v>
       </c>
       <c r="D31" t="n">
-        <v>2.61</v>
+        <v>1.42</v>
       </c>
       <c r="E31" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="F31" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="G31" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>15.79</v>
+        <v>18.63</v>
       </c>
       <c r="D32" t="n">
-        <v>1.49</v>
+        <v>1.7</v>
       </c>
       <c r="E32" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="F32" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="G32" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri May  8 10:57:43 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.52</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.38</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.82</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>4.52</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>3.41</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.01</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>5.43</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.82</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.4</v>
       </c>
       <c r="E10" t="n">
-        <v>93.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>96.7</v>
+        <v>93.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>6.79</v>
       </c>
       <c r="E11" t="n">
-        <v>93.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F11" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>96.7</v>
+        <v>93.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>0.77</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>86.7</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>93.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>4.1</v>
       </c>
       <c r="E13" t="n">
-        <v>93.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>93.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>93.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.29</v>
       </c>
       <c r="E14" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>73.3</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>86.7</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.28</v>
       </c>
       <c r="E15" t="n">
-        <v>80</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>90</v>
+        <v>87.5</v>
       </c>
       <c r="G15" t="n">
-        <v>85</v>
+        <v>82.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.19</v>
       </c>
       <c r="E16" t="n">
-        <v>66.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>83.3</v>
+        <v>81.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>4.03</v>
       </c>
       <c r="E17" t="n">
-        <v>66.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>83.3</v>
+        <v>81.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.88</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>63.3</v>
+        <v>62.5</v>
       </c>
       <c r="G18" t="n">
-        <v>81.7</v>
+        <v>79.7</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.8</v>
       </c>
       <c r="E19" t="n">
-        <v>66.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="F19" t="n">
-        <v>96.7</v>
+        <v>93.8</v>
       </c>
       <c r="G19" t="n">
-        <v>81.7</v>
+        <v>79.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>2.43</v>
       </c>
       <c r="E20" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F20" t="n">
-        <v>60</v>
+        <v>59.4</v>
       </c>
       <c r="G20" t="n">
-        <v>80</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>4.38</v>
       </c>
       <c r="E21" t="n">
-        <v>53.3</v>
+        <v>53.1</v>
       </c>
       <c r="F21" t="n">
-        <v>100</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>76.7</v>
+        <v>75</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.83</v>
       </c>
       <c r="E22" t="n">
-        <v>93.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>56.7</v>
+        <v>56.2</v>
       </c>
       <c r="G22" t="n">
-        <v>75</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.76</v>
       </c>
       <c r="E23" t="n">
-        <v>73.3</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>73.3</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>73.3</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.16</v>
       </c>
       <c r="E24" t="n">
-        <v>53.3</v>
+        <v>53.1</v>
       </c>
       <c r="F24" t="n">
-        <v>63.3</v>
+        <v>62.5</v>
       </c>
       <c r="G24" t="n">
-        <v>58.3</v>
+        <v>57.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.38</v>
       </c>
       <c r="E25" t="n">
-        <v>40</v>
+        <v>40.6</v>
       </c>
       <c r="F25" t="n">
-        <v>53.3</v>
+        <v>53.1</v>
       </c>
       <c r="G25" t="n">
-        <v>46.7</v>
+        <v>46.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>1.12</v>
       </c>
       <c r="E26" t="n">
-        <v>46.7</v>
+        <v>46.9</v>
       </c>
       <c r="F26" t="n">
-        <v>26.7</v>
+        <v>28.1</v>
       </c>
       <c r="G26" t="n">
-        <v>32.7</v>
+        <v>33.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.79</v>
       </c>
       <c r="E27" t="n">
-        <v>93.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F27" t="n">
-        <v>6.7</v>
+        <v>9.4</v>
       </c>
       <c r="G27" t="n">
-        <v>32.7</v>
+        <v>33.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.63</v>
       </c>
       <c r="E28" t="n">
-        <v>13.3</v>
+        <v>15.6</v>
       </c>
       <c r="F28" t="n">
-        <v>23.3</v>
+        <v>25</v>
       </c>
       <c r="G28" t="n">
-        <v>20.3</v>
+        <v>22.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>2.66</v>
       </c>
       <c r="E29" t="n">
-        <v>13.3</v>
+        <v>15.6</v>
       </c>
       <c r="F29" t="n">
-        <v>16.7</v>
+        <v>18.8</v>
       </c>
       <c r="G29" t="n">
-        <v>15.7</v>
+        <v>17.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>0.65</v>
       </c>
       <c r="E30" t="n">
-        <v>13.3</v>
+        <v>15.6</v>
       </c>
       <c r="F30" t="n">
-        <v>10</v>
+        <v>12.5</v>
       </c>
       <c r="G30" t="n">
-        <v>11</v>
+        <v>13.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.42</v>
       </c>
       <c r="E31" t="n">
-        <v>6.7</v>
+        <v>9.4</v>
       </c>
       <c r="F31" t="n">
-        <v>6.7</v>
+        <v>9.4</v>
       </c>
       <c r="G31" t="n">
-        <v>6.7</v>
+        <v>9.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.7</v>
       </c>
       <c r="E32" t="n">
-        <v>6.7</v>
+        <v>9.4</v>
       </c>
       <c r="F32" t="n">
-        <v>6.7</v>
+        <v>9.4</v>
       </c>
       <c r="G32" t="n">
-        <v>6.7</v>
+        <v>9.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat May  9 10:38:07 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,112 +486,112 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>27.34</v>
+        <v>27.51</v>
       </c>
       <c r="D2" t="n">
-        <v>2.52</v>
+        <v>2.53</v>
       </c>
       <c r="E2" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>26.26</v>
+        <v>15.89</v>
       </c>
       <c r="D3" t="n">
-        <v>2.38</v>
+        <v>1.29</v>
       </c>
       <c r="E3" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>29.81</v>
+        <v>26.61</v>
       </c>
       <c r="D4" t="n">
-        <v>2.82</v>
+        <v>2.41</v>
       </c>
       <c r="E4" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>54.89</v>
+        <v>30.16</v>
       </c>
       <c r="D5" t="n">
-        <v>4.52</v>
+        <v>2.85</v>
       </c>
       <c r="E5" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="6">
@@ -606,82 +606,82 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40.39</v>
+        <v>40.67</v>
       </c>
       <c r="D6" t="n">
-        <v>3.41</v>
+        <v>3.43</v>
       </c>
       <c r="E6" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>36.22</v>
+        <v>22.18</v>
       </c>
       <c r="D7" t="n">
-        <v>2.01</v>
+        <v>1.85</v>
       </c>
       <c r="E7" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>96.90000000000001</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>96.90000000000001</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>144.85</v>
+        <v>54.94</v>
       </c>
       <c r="D8" t="n">
-        <v>5.43</v>
+        <v>4.52</v>
       </c>
       <c r="E8" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>96.90000000000001</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>96.90000000000001</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="9">
@@ -696,82 +696,82 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>24.76</v>
+        <v>24.77</v>
       </c>
       <c r="D9" t="n">
         <v>1.82</v>
       </c>
       <c r="E9" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>96.90000000000001</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>96.90000000000001</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>29.37</v>
+        <v>36.15</v>
       </c>
       <c r="D10" t="n">
-        <v>2.4</v>
+        <v>2.02</v>
       </c>
       <c r="E10" t="n">
-        <v>90.59999999999999</v>
+        <v>88.2</v>
       </c>
       <c r="F10" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>93.8</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>65.81</v>
+        <v>16.64</v>
       </c>
       <c r="D11" t="n">
-        <v>6.79</v>
+        <v>2.46</v>
       </c>
       <c r="E11" t="n">
-        <v>90.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="F11" t="n">
-        <v>96.90000000000001</v>
+        <v>85.3</v>
       </c>
       <c r="G11" t="n">
-        <v>93.8</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="12">
@@ -786,142 +786,142 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>12.06</v>
+        <v>12.11</v>
       </c>
       <c r="D12" t="n">
         <v>0.77</v>
       </c>
       <c r="E12" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>84.40000000000001</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>90.59999999999999</v>
+        <v>91.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>38.1</v>
+        <v>20.2</v>
       </c>
       <c r="D13" t="n">
-        <v>4.1</v>
+        <v>1.89</v>
       </c>
       <c r="E13" t="n">
-        <v>90.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="F13" t="n">
-        <v>90.59999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>90.59999999999999</v>
+        <v>91.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10.64</v>
+        <v>29.34</v>
       </c>
       <c r="D14" t="n">
-        <v>1.29</v>
+        <v>2.4</v>
       </c>
       <c r="E14" t="n">
-        <v>96.90000000000001</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>71.90000000000001</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>84.40000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>15.7</v>
+        <v>33.59</v>
       </c>
       <c r="D15" t="n">
-        <v>1.28</v>
+        <v>2.81</v>
       </c>
       <c r="E15" t="n">
-        <v>78.09999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="F15" t="n">
-        <v>87.5</v>
+        <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>82.8</v>
+        <v>88.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>13.15</v>
+        <v>65.17</v>
       </c>
       <c r="D16" t="n">
-        <v>1.19</v>
+        <v>6.73</v>
       </c>
       <c r="E16" t="n">
-        <v>65.59999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>96.90000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="G16" t="n">
-        <v>81.2</v>
+        <v>85.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="17">
@@ -936,412 +936,412 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.81</v>
+        <v>23.87</v>
       </c>
       <c r="D17" t="n">
-        <v>4.03</v>
+        <v>4.04</v>
       </c>
       <c r="E17" t="n">
-        <v>65.59999999999999</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>81.2</v>
+        <v>85.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>20.19</v>
+        <v>13.31</v>
       </c>
       <c r="D18" t="n">
-        <v>1.88</v>
+        <v>1.2</v>
       </c>
       <c r="E18" t="n">
-        <v>96.90000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="F18" t="n">
-        <v>62.5</v>
+        <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>79.7</v>
+        <v>85.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>33.37</v>
+        <v>137.88</v>
       </c>
       <c r="D19" t="n">
-        <v>2.8</v>
+        <v>5.18</v>
       </c>
       <c r="E19" t="n">
-        <v>65.59999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>93.8</v>
+        <v>85.3</v>
       </c>
       <c r="G19" t="n">
-        <v>79.7</v>
+        <v>83.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>16.46</v>
+        <v>69.5</v>
       </c>
       <c r="D20" t="n">
-        <v>2.43</v>
+        <v>4.52</v>
       </c>
       <c r="E20" t="n">
-        <v>96.90000000000001</v>
+        <v>58.8</v>
       </c>
       <c r="F20" t="n">
-        <v>59.4</v>
+        <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>78.09999999999999</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>67.37</v>
+        <v>37.45</v>
       </c>
       <c r="D21" t="n">
-        <v>4.38</v>
+        <v>4.03</v>
       </c>
       <c r="E21" t="n">
-        <v>53.1</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>96.90000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="G21" t="n">
-        <v>75</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22.04</v>
+        <v>10.59</v>
       </c>
       <c r="D22" t="n">
-        <v>1.83</v>
+        <v>1.29</v>
       </c>
       <c r="E22" t="n">
-        <v>90.59999999999999</v>
+        <v>85.3</v>
       </c>
       <c r="F22" t="n">
-        <v>56.2</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="G22" t="n">
-        <v>73.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>30</v>
+        <v>26.34</v>
       </c>
       <c r="D23" t="n">
-        <v>2.76</v>
+        <v>2.17</v>
       </c>
       <c r="E23" t="n">
-        <v>71.90000000000001</v>
+        <v>58.8</v>
       </c>
       <c r="F23" t="n">
-        <v>71.90000000000001</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>71.90000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>26.31</v>
+        <v>31.9</v>
       </c>
       <c r="D24" t="n">
-        <v>2.16</v>
+        <v>2.37</v>
       </c>
       <c r="E24" t="n">
-        <v>53.1</v>
+        <v>35.3</v>
       </c>
       <c r="F24" t="n">
-        <v>62.5</v>
+        <v>41.2</v>
       </c>
       <c r="G24" t="n">
-        <v>57.8</v>
+        <v>38.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>32.05</v>
+        <v>20.25</v>
       </c>
       <c r="D25" t="n">
-        <v>2.38</v>
+        <v>1.12</v>
       </c>
       <c r="E25" t="n">
-        <v>40.6</v>
+        <v>52.9</v>
       </c>
       <c r="F25" t="n">
-        <v>53.1</v>
+        <v>29.4</v>
       </c>
       <c r="G25" t="n">
-        <v>46.9</v>
+        <v>36.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>20.2</v>
+        <v>34.84</v>
       </c>
       <c r="D26" t="n">
-        <v>1.12</v>
+        <v>2.65</v>
       </c>
       <c r="E26" t="n">
-        <v>46.9</v>
+        <v>29.4</v>
       </c>
       <c r="F26" t="n">
-        <v>28.1</v>
+        <v>35.3</v>
       </c>
       <c r="G26" t="n">
-        <v>33.8</v>
+        <v>32.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>21.84</v>
+        <v>29.81</v>
       </c>
       <c r="D27" t="n">
-        <v>3.79</v>
+        <v>2.74</v>
       </c>
       <c r="E27" t="n">
-        <v>90.59999999999999</v>
+        <v>11.8</v>
       </c>
       <c r="F27" t="n">
-        <v>9.4</v>
+        <v>47.1</v>
       </c>
       <c r="G27" t="n">
-        <v>33.8</v>
+        <v>29.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>34.49</v>
+        <v>21.77</v>
       </c>
       <c r="D28" t="n">
-        <v>2.63</v>
+        <v>3.78</v>
       </c>
       <c r="E28" t="n">
-        <v>15.6</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F28" t="n">
-        <v>25</v>
+        <v>5.9</v>
       </c>
       <c r="G28" t="n">
-        <v>22.2</v>
+        <v>28.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>28.99</v>
+        <v>6.86</v>
       </c>
       <c r="D29" t="n">
-        <v>2.66</v>
+        <v>0.65</v>
       </c>
       <c r="E29" t="n">
-        <v>15.6</v>
+        <v>23.5</v>
       </c>
       <c r="F29" t="n">
-        <v>18.8</v>
+        <v>14.7</v>
       </c>
       <c r="G29" t="n">
-        <v>17.8</v>
+        <v>17.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6.85</v>
+        <v>28.91</v>
       </c>
       <c r="D30" t="n">
-        <v>0.65</v>
+        <v>2.65</v>
       </c>
       <c r="E30" t="n">
-        <v>15.6</v>
+        <v>11.8</v>
       </c>
       <c r="F30" t="n">
-        <v>12.5</v>
+        <v>11.8</v>
       </c>
       <c r="G30" t="n">
-        <v>13.4</v>
+        <v>11.8</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>15.07</v>
+        <v>14.97</v>
       </c>
       <c r="D31" t="n">
-        <v>1.42</v>
+        <v>1.41</v>
       </c>
       <c r="E31" t="n">
-        <v>9.4</v>
+        <v>5.9</v>
       </c>
       <c r="F31" t="n">
-        <v>9.4</v>
+        <v>5.9</v>
       </c>
       <c r="G31" t="n">
-        <v>9.4</v>
+        <v>5.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18.63</v>
+        <v>18.45</v>
       </c>
       <c r="D32" t="n">
-        <v>1.7</v>
+        <v>1.69</v>
       </c>
       <c r="E32" t="n">
-        <v>9.4</v>
+        <v>5.9</v>
       </c>
       <c r="F32" t="n">
-        <v>9.4</v>
+        <v>5.9</v>
       </c>
       <c r="G32" t="n">
-        <v>9.4</v>
+        <v>5.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun May 10 10:48:21 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.53</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.29</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.41</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.85</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>3.43</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.85</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F7" t="n">
-        <v>94.09999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="G7" t="n">
-        <v>97.09999999999999</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>4.52</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F8" t="n">
-        <v>94.09999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="G8" t="n">
-        <v>97.09999999999999</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.82</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F9" t="n">
-        <v>94.09999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="G9" t="n">
-        <v>97.09999999999999</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.02</v>
       </c>
       <c r="E10" t="n">
-        <v>88.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G10" t="n">
-        <v>94.09999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.46</v>
       </c>
       <c r="E11" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F11" t="n">
-        <v>85.3</v>
+        <v>83.3</v>
       </c>
       <c r="G11" t="n">
-        <v>92.59999999999999</v>
+        <v>90.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>0.77</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F12" t="n">
-        <v>82.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>91.2</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.89</v>
       </c>
       <c r="E13" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="F13" t="n">
-        <v>82.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>91.2</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.4</v>
       </c>
       <c r="E14" t="n">
-        <v>82.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>94.09999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="G14" t="n">
-        <v>88.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.81</v>
       </c>
       <c r="E15" t="n">
-        <v>76.5</v>
+        <v>75</v>
       </c>
       <c r="F15" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G15" t="n">
-        <v>88.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>6.73</v>
       </c>
       <c r="E16" t="n">
-        <v>82.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>88.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>85.3</v>
+        <v>83.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>4.04</v>
       </c>
       <c r="E17" t="n">
-        <v>70.59999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G17" t="n">
-        <v>85.3</v>
+        <v>83.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.2</v>
       </c>
       <c r="E18" t="n">
-        <v>70.59999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G18" t="n">
-        <v>85.3</v>
+        <v>83.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>5.18</v>
       </c>
       <c r="E19" t="n">
-        <v>82.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="F19" t="n">
-        <v>85.3</v>
+        <v>83.3</v>
       </c>
       <c r="G19" t="n">
-        <v>83.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>4.52</v>
       </c>
       <c r="E20" t="n">
-        <v>58.8</v>
+        <v>58.3</v>
       </c>
       <c r="F20" t="n">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="G20" t="n">
-        <v>79.40000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>4.03</v>
       </c>
       <c r="E21" t="n">
-        <v>82.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>76.5</v>
+        <v>75</v>
       </c>
       <c r="G21" t="n">
-        <v>79.40000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.29</v>
       </c>
       <c r="E22" t="n">
-        <v>85.3</v>
+        <v>83.3</v>
       </c>
       <c r="F22" t="n">
-        <v>70.59999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>77.90000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="23">
@@ -1122,76 +1122,76 @@
         <v>2.17</v>
       </c>
       <c r="E23" t="n">
-        <v>58.8</v>
+        <v>58.3</v>
       </c>
       <c r="F23" t="n">
-        <v>82.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>70.59999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>31.9</v>
+        <v>20.25</v>
       </c>
       <c r="D24" t="n">
-        <v>2.37</v>
+        <v>1.12</v>
       </c>
       <c r="E24" t="n">
-        <v>35.3</v>
+        <v>52.8</v>
       </c>
       <c r="F24" t="n">
-        <v>41.2</v>
+        <v>30.6</v>
       </c>
       <c r="G24" t="n">
-        <v>38.2</v>
+        <v>41.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20.25</v>
+        <v>31.9</v>
       </c>
       <c r="D25" t="n">
-        <v>1.12</v>
+        <v>2.37</v>
       </c>
       <c r="E25" t="n">
-        <v>52.9</v>
+        <v>36.1</v>
       </c>
       <c r="F25" t="n">
-        <v>29.4</v>
+        <v>41.7</v>
       </c>
       <c r="G25" t="n">
-        <v>36.5</v>
+        <v>38.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.65</v>
       </c>
       <c r="E26" t="n">
-        <v>29.4</v>
+        <v>30.6</v>
       </c>
       <c r="F26" t="n">
-        <v>35.3</v>
+        <v>36.1</v>
       </c>
       <c r="G26" t="n">
-        <v>32.4</v>
+        <v>33.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.74</v>
       </c>
       <c r="E27" t="n">
-        <v>11.8</v>
+        <v>13.9</v>
       </c>
       <c r="F27" t="n">
-        <v>47.1</v>
+        <v>47.2</v>
       </c>
       <c r="G27" t="n">
-        <v>29.4</v>
+        <v>30.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>3.78</v>
       </c>
       <c r="E28" t="n">
-        <v>82.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="F28" t="n">
-        <v>5.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>28.8</v>
+        <v>30</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>0.65</v>
       </c>
       <c r="E29" t="n">
-        <v>23.5</v>
+        <v>25</v>
       </c>
       <c r="F29" t="n">
-        <v>14.7</v>
+        <v>16.7</v>
       </c>
       <c r="G29" t="n">
-        <v>17.4</v>
+        <v>19.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.65</v>
       </c>
       <c r="E30" t="n">
-        <v>11.8</v>
+        <v>13.9</v>
       </c>
       <c r="F30" t="n">
-        <v>11.8</v>
+        <v>13.9</v>
       </c>
       <c r="G30" t="n">
-        <v>11.8</v>
+        <v>13.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.41</v>
       </c>
       <c r="E31" t="n">
-        <v>5.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F31" t="n">
-        <v>5.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>5.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.69</v>
       </c>
       <c r="E32" t="n">
-        <v>5.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F32" t="n">
-        <v>5.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G32" t="n">
-        <v>5.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46151</v>
+        <v>46152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon May 11 12:32:49 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,331 +477,331 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>27.51</v>
+        <v>68.3</v>
       </c>
       <c r="D2" t="n">
-        <v>2.53</v>
+        <v>7.05</v>
       </c>
       <c r="E2" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>15.89</v>
+        <v>26.76</v>
       </c>
       <c r="D3" t="n">
-        <v>1.29</v>
+        <v>2.42</v>
       </c>
       <c r="E3" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>26.61</v>
+        <v>30.28</v>
       </c>
       <c r="D4" t="n">
-        <v>2.41</v>
+        <v>2.79</v>
       </c>
       <c r="E4" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>30.16</v>
+        <v>55.24</v>
       </c>
       <c r="D5" t="n">
-        <v>2.85</v>
+        <v>4.55</v>
       </c>
       <c r="E5" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40.67</v>
+        <v>36.52</v>
       </c>
       <c r="D6" t="n">
-        <v>3.43</v>
+        <v>2.04</v>
       </c>
       <c r="E6" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>22.18</v>
+        <v>41.55</v>
       </c>
       <c r="D7" t="n">
-        <v>1.85</v>
+        <v>3.51</v>
       </c>
       <c r="E7" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>94.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>54.94</v>
+        <v>12.2</v>
       </c>
       <c r="D8" t="n">
-        <v>4.52</v>
+        <v>0.78</v>
       </c>
       <c r="E8" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>94.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>24.77</v>
+        <v>30.93</v>
       </c>
       <c r="D9" t="n">
-        <v>1.82</v>
+        <v>2.93</v>
       </c>
       <c r="E9" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>94.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>36.15</v>
+        <v>16.72</v>
       </c>
       <c r="D10" t="n">
-        <v>2.02</v>
+        <v>2.47</v>
       </c>
       <c r="E10" t="n">
-        <v>86.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="F10" t="n">
-        <v>97.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>91.7</v>
+        <v>98.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16.64</v>
+        <v>22.28</v>
       </c>
       <c r="D11" t="n">
-        <v>2.46</v>
+        <v>1.87</v>
       </c>
       <c r="E11" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F11" t="n">
-        <v>83.3</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>90.3</v>
+        <v>98.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>12.11</v>
+        <v>10.72</v>
       </c>
       <c r="D12" t="n">
-        <v>0.77</v>
+        <v>1.3</v>
       </c>
       <c r="E12" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>80.59999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="G12" t="n">
-        <v>88.90000000000001</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="13">
@@ -816,592 +816,592 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>20.2</v>
+        <v>20.5</v>
       </c>
       <c r="D13" t="n">
-        <v>1.89</v>
+        <v>1.91</v>
       </c>
       <c r="E13" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="F13" t="n">
-        <v>80.59999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="G13" t="n">
-        <v>88.90000000000001</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>29.34</v>
+        <v>27.51</v>
       </c>
       <c r="D14" t="n">
-        <v>2.4</v>
+        <v>2.53</v>
       </c>
       <c r="E14" t="n">
-        <v>80.59999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="F14" t="n">
-        <v>91.7</v>
+        <v>94.7</v>
       </c>
       <c r="G14" t="n">
-        <v>86.09999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>33.59</v>
+        <v>13.61</v>
       </c>
       <c r="D15" t="n">
-        <v>2.81</v>
+        <v>1.23</v>
       </c>
       <c r="E15" t="n">
-        <v>75</v>
+        <v>73.7</v>
       </c>
       <c r="F15" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>86.09999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>65.17</v>
+        <v>24.04</v>
       </c>
       <c r="D16" t="n">
-        <v>6.73</v>
+        <v>4.06</v>
       </c>
       <c r="E16" t="n">
-        <v>80.59999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="F16" t="n">
-        <v>86.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>83.3</v>
+        <v>86.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.87</v>
+        <v>38.08</v>
       </c>
       <c r="D17" t="n">
-        <v>4.04</v>
+        <v>4.1</v>
       </c>
       <c r="E17" t="n">
-        <v>69.40000000000001</v>
+        <v>84.2</v>
       </c>
       <c r="F17" t="n">
-        <v>97.2</v>
+        <v>89.5</v>
       </c>
       <c r="G17" t="n">
-        <v>83.3</v>
+        <v>86.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>13.31</v>
+        <v>70.39</v>
       </c>
       <c r="D18" t="n">
-        <v>1.2</v>
+        <v>4.58</v>
       </c>
       <c r="E18" t="n">
-        <v>69.40000000000001</v>
+        <v>63.2</v>
       </c>
       <c r="F18" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>83.3</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>137.88</v>
+        <v>15.75</v>
       </c>
       <c r="D19" t="n">
-        <v>5.18</v>
+        <v>1.28</v>
       </c>
       <c r="E19" t="n">
-        <v>80.59999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="F19" t="n">
-        <v>83.3</v>
+        <v>76.3</v>
       </c>
       <c r="G19" t="n">
-        <v>81.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>69.5</v>
+        <v>136.94</v>
       </c>
       <c r="D20" t="n">
-        <v>4.52</v>
+        <v>5.14</v>
       </c>
       <c r="E20" t="n">
-        <v>58.3</v>
+        <v>73.7</v>
       </c>
       <c r="F20" t="n">
-        <v>97.2</v>
+        <v>73.7</v>
       </c>
       <c r="G20" t="n">
-        <v>77.8</v>
+        <v>73.7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>37.45</v>
+        <v>24.63</v>
       </c>
       <c r="D21" t="n">
-        <v>4.03</v>
+        <v>1.81</v>
       </c>
       <c r="E21" t="n">
-        <v>80.59999999999999</v>
+        <v>63.2</v>
       </c>
       <c r="F21" t="n">
-        <v>75</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>77.8</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10.59</v>
+        <v>29.17</v>
       </c>
       <c r="D22" t="n">
-        <v>1.29</v>
+        <v>2.38</v>
       </c>
       <c r="E22" t="n">
-        <v>83.3</v>
+        <v>73.7</v>
       </c>
       <c r="F22" t="n">
-        <v>69.40000000000001</v>
+        <v>47.4</v>
       </c>
       <c r="G22" t="n">
-        <v>76.40000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>26.34</v>
+        <v>33.34</v>
       </c>
       <c r="D23" t="n">
-        <v>2.17</v>
+        <v>2.79</v>
       </c>
       <c r="E23" t="n">
-        <v>58.3</v>
+        <v>50</v>
       </c>
       <c r="F23" t="n">
-        <v>80.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>69.40000000000001</v>
+        <v>59.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>20.25</v>
+        <v>26.33</v>
       </c>
       <c r="D24" t="n">
-        <v>1.12</v>
+        <v>2.16</v>
       </c>
       <c r="E24" t="n">
-        <v>52.8</v>
+        <v>52.6</v>
       </c>
       <c r="F24" t="n">
-        <v>30.6</v>
+        <v>55.3</v>
       </c>
       <c r="G24" t="n">
-        <v>41.7</v>
+        <v>53.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>31.9</v>
+        <v>29.11</v>
       </c>
       <c r="D25" t="n">
-        <v>2.37</v>
+        <v>2.67</v>
       </c>
       <c r="E25" t="n">
-        <v>36.1</v>
+        <v>47.4</v>
       </c>
       <c r="F25" t="n">
-        <v>41.7</v>
+        <v>52.6</v>
       </c>
       <c r="G25" t="n">
-        <v>38.9</v>
+        <v>50</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>34.84</v>
+        <v>32.03</v>
       </c>
       <c r="D26" t="n">
-        <v>2.65</v>
+        <v>2.38</v>
       </c>
       <c r="E26" t="n">
-        <v>30.6</v>
+        <v>42.1</v>
       </c>
       <c r="F26" t="n">
-        <v>36.1</v>
+        <v>57.9</v>
       </c>
       <c r="G26" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>29.81</v>
+        <v>20.16</v>
       </c>
       <c r="D27" t="n">
-        <v>2.74</v>
+        <v>1.12</v>
       </c>
       <c r="E27" t="n">
-        <v>13.9</v>
+        <v>36.8</v>
       </c>
       <c r="F27" t="n">
-        <v>47.2</v>
+        <v>31.6</v>
       </c>
       <c r="G27" t="n">
-        <v>30.6</v>
+        <v>34.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>21.77</v>
+        <v>34.7</v>
       </c>
       <c r="D28" t="n">
-        <v>3.78</v>
+        <v>2.64</v>
       </c>
       <c r="E28" t="n">
-        <v>80.59999999999999</v>
+        <v>21.1</v>
       </c>
       <c r="F28" t="n">
-        <v>8.300000000000001</v>
+        <v>31.6</v>
       </c>
       <c r="G28" t="n">
-        <v>30</v>
+        <v>26.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6.86</v>
+        <v>21.7</v>
       </c>
       <c r="D29" t="n">
-        <v>0.65</v>
+        <v>3.77</v>
       </c>
       <c r="E29" t="n">
-        <v>25</v>
+        <v>73.7</v>
       </c>
       <c r="F29" t="n">
-        <v>16.7</v>
+        <v>5.3</v>
       </c>
       <c r="G29" t="n">
-        <v>19.2</v>
+        <v>25.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>28.91</v>
+        <v>6.84</v>
       </c>
       <c r="D30" t="n">
-        <v>2.65</v>
+        <v>0.65</v>
       </c>
       <c r="E30" t="n">
-        <v>13.9</v>
+        <v>7.9</v>
       </c>
       <c r="F30" t="n">
-        <v>13.9</v>
+        <v>18.4</v>
       </c>
       <c r="G30" t="n">
-        <v>13.9</v>
+        <v>15.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>14.97</v>
+        <v>18.46</v>
       </c>
       <c r="D31" t="n">
-        <v>1.41</v>
+        <v>1.69</v>
       </c>
       <c r="E31" t="n">
-        <v>8.300000000000001</v>
+        <v>15.8</v>
       </c>
       <c r="F31" t="n">
-        <v>8.300000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="G31" t="n">
-        <v>8.300000000000001</v>
+        <v>12.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18.45</v>
+        <v>14.96</v>
       </c>
       <c r="D32" t="n">
-        <v>1.69</v>
+        <v>1.41</v>
       </c>
       <c r="E32" t="n">
-        <v>8.300000000000001</v>
+        <v>5.3</v>
       </c>
       <c r="F32" t="n">
-        <v>8.300000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="G32" t="n">
-        <v>8.300000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue May 12 11:34:51 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>68.3</v>
+        <v>31.37</v>
       </c>
       <c r="D2" t="n">
-        <v>7.05</v>
+        <v>2.97</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,127 +501,127 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>26.76</v>
+        <v>20.71</v>
       </c>
       <c r="D3" t="n">
-        <v>2.42</v>
+        <v>1.93</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>97.5</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>98.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30.28</v>
+        <v>36.61</v>
       </c>
       <c r="D4" t="n">
-        <v>2.79</v>
+        <v>2.03</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>97.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>55.24</v>
+        <v>68.25</v>
       </c>
       <c r="D5" t="n">
-        <v>4.55</v>
+        <v>7.05</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>97.5</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>96.2</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>36.52</v>
+        <v>12.14</v>
       </c>
       <c r="D6" t="n">
-        <v>2.04</v>
+        <v>0.78</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>97.5</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>96.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="7">
@@ -636,382 +636,382 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>41.55</v>
+        <v>41.16</v>
       </c>
       <c r="D7" t="n">
-        <v>3.51</v>
+        <v>3.48</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="F7" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>12.2</v>
+        <v>30.17</v>
       </c>
       <c r="D8" t="n">
-        <v>0.78</v>
+        <v>2.78</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="F8" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30.93</v>
+        <v>10.69</v>
       </c>
       <c r="D9" t="n">
-        <v>2.93</v>
+        <v>1.3</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="F9" t="n">
-        <v>100</v>
+        <v>92.5</v>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>93.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>16.72</v>
+        <v>22.15</v>
       </c>
       <c r="D10" t="n">
-        <v>2.47</v>
+        <v>1.86</v>
       </c>
       <c r="E10" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F10" t="n">
-        <v>97.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="G10" t="n">
-        <v>98.7</v>
+        <v>85</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>22.28</v>
+        <v>26.59</v>
       </c>
       <c r="D11" t="n">
-        <v>1.87</v>
+        <v>2.4</v>
       </c>
       <c r="E11" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="F11" t="n">
-        <v>97.40000000000001</v>
+        <v>85</v>
       </c>
       <c r="G11" t="n">
-        <v>98.7</v>
+        <v>85</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10.72</v>
+        <v>13.48</v>
       </c>
       <c r="D12" t="n">
-        <v>1.3</v>
+        <v>1.23</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F12" t="n">
-        <v>94.7</v>
+        <v>97.5</v>
       </c>
       <c r="G12" t="n">
-        <v>97.40000000000001</v>
+        <v>83.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>20.5</v>
+        <v>23.91</v>
       </c>
       <c r="D13" t="n">
-        <v>1.91</v>
+        <v>4.04</v>
       </c>
       <c r="E13" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F13" t="n">
-        <v>94.7</v>
+        <v>90</v>
       </c>
       <c r="G13" t="n">
-        <v>97.40000000000001</v>
+        <v>80</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>27.51</v>
+        <v>37.68</v>
       </c>
       <c r="D14" t="n">
-        <v>2.53</v>
+        <v>4.05</v>
       </c>
       <c r="E14" t="n">
-        <v>94.7</v>
+        <v>80</v>
       </c>
       <c r="F14" t="n">
-        <v>94.7</v>
+        <v>75</v>
       </c>
       <c r="G14" t="n">
-        <v>94.7</v>
+        <v>77.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>13.61</v>
+        <v>69.88</v>
       </c>
       <c r="D15" t="n">
-        <v>1.23</v>
+        <v>4.54</v>
       </c>
       <c r="E15" t="n">
-        <v>73.7</v>
+        <v>60</v>
       </c>
       <c r="F15" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G15" t="n">
-        <v>86.8</v>
+        <v>77.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>24.04</v>
+        <v>27.26</v>
       </c>
       <c r="D16" t="n">
-        <v>4.06</v>
+        <v>2.51</v>
       </c>
       <c r="E16" t="n">
-        <v>73.7</v>
+        <v>75</v>
       </c>
       <c r="F16" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G16" t="n">
-        <v>86.8</v>
+        <v>75</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>38.08</v>
+        <v>54.16</v>
       </c>
       <c r="D17" t="n">
-        <v>4.1</v>
+        <v>4.46</v>
       </c>
       <c r="E17" t="n">
-        <v>84.2</v>
+        <v>75</v>
       </c>
       <c r="F17" t="n">
-        <v>89.5</v>
+        <v>75</v>
       </c>
       <c r="G17" t="n">
-        <v>86.8</v>
+        <v>75</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>70.39</v>
+        <v>15.73</v>
       </c>
       <c r="D18" t="n">
-        <v>4.58</v>
+        <v>1.28</v>
       </c>
       <c r="E18" t="n">
-        <v>63.2</v>
+        <v>70</v>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G18" t="n">
-        <v>81.59999999999999</v>
+        <v>72.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15.75</v>
+        <v>16.58</v>
       </c>
       <c r="D19" t="n">
-        <v>1.28</v>
+        <v>2.45</v>
       </c>
       <c r="E19" t="n">
-        <v>73.7</v>
+        <v>85</v>
       </c>
       <c r="F19" t="n">
-        <v>76.3</v>
+        <v>60</v>
       </c>
       <c r="G19" t="n">
-        <v>75</v>
+        <v>72.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="20">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>136.94</v>
+        <v>132.48</v>
       </c>
       <c r="D20" t="n">
-        <v>5.14</v>
+        <v>4.97</v>
       </c>
       <c r="E20" t="n">
-        <v>73.7</v>
+        <v>70</v>
       </c>
       <c r="F20" t="n">
-        <v>73.7</v>
+        <v>70</v>
       </c>
       <c r="G20" t="n">
-        <v>73.7</v>
+        <v>70</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="21">
@@ -1056,22 +1056,22 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>24.63</v>
+        <v>24.45</v>
       </c>
       <c r="D21" t="n">
-        <v>1.81</v>
+        <v>1.8</v>
       </c>
       <c r="E21" t="n">
-        <v>63.2</v>
+        <v>50</v>
       </c>
       <c r="F21" t="n">
-        <v>78.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="G21" t="n">
-        <v>71.09999999999999</v>
+        <v>62.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="22">
@@ -1086,322 +1086,322 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>29.17</v>
+        <v>28.82</v>
       </c>
       <c r="D22" t="n">
-        <v>2.38</v>
+        <v>2.36</v>
       </c>
       <c r="E22" t="n">
-        <v>73.7</v>
+        <v>70</v>
       </c>
       <c r="F22" t="n">
-        <v>47.4</v>
+        <v>45</v>
       </c>
       <c r="G22" t="n">
-        <v>60.5</v>
+        <v>57.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>33.34</v>
+        <v>31.36</v>
       </c>
       <c r="D23" t="n">
-        <v>2.79</v>
+        <v>2.32</v>
       </c>
       <c r="E23" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F23" t="n">
-        <v>68.40000000000001</v>
+        <v>30</v>
       </c>
       <c r="G23" t="n">
-        <v>59.2</v>
+        <v>30</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>26.33</v>
+        <v>28.98</v>
       </c>
       <c r="D24" t="n">
-        <v>2.16</v>
+        <v>2.66</v>
       </c>
       <c r="E24" t="n">
-        <v>52.6</v>
+        <v>20</v>
       </c>
       <c r="F24" t="n">
-        <v>55.3</v>
+        <v>27.5</v>
       </c>
       <c r="G24" t="n">
-        <v>53.9</v>
+        <v>25.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29.11</v>
+        <v>21.49</v>
       </c>
       <c r="D25" t="n">
-        <v>2.67</v>
+        <v>3.73</v>
       </c>
       <c r="E25" t="n">
-        <v>47.4</v>
+        <v>70</v>
       </c>
       <c r="F25" t="n">
-        <v>52.6</v>
+        <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>50</v>
+        <v>24.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>32.03</v>
+        <v>6.84</v>
       </c>
       <c r="D26" t="n">
-        <v>2.38</v>
+        <v>0.65</v>
       </c>
       <c r="E26" t="n">
-        <v>42.1</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>57.9</v>
+        <v>20</v>
       </c>
       <c r="G26" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>20.16</v>
+        <v>14.99</v>
       </c>
       <c r="D27" t="n">
-        <v>1.12</v>
+        <v>1.41</v>
       </c>
       <c r="E27" t="n">
-        <v>36.8</v>
+        <v>20</v>
       </c>
       <c r="F27" t="n">
-        <v>31.6</v>
+        <v>12.5</v>
       </c>
       <c r="G27" t="n">
-        <v>34.2</v>
+        <v>14.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>34.7</v>
+        <v>25.94</v>
       </c>
       <c r="D28" t="n">
-        <v>2.64</v>
+        <v>2.13</v>
       </c>
       <c r="E28" t="n">
-        <v>21.1</v>
+        <v>5</v>
       </c>
       <c r="F28" t="n">
-        <v>31.6</v>
+        <v>10</v>
       </c>
       <c r="G28" t="n">
-        <v>26.3</v>
+        <v>8.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>21.7</v>
+        <v>32.71</v>
       </c>
       <c r="D29" t="n">
-        <v>3.77</v>
+        <v>2.74</v>
       </c>
       <c r="E29" t="n">
-        <v>73.7</v>
+        <v>10</v>
       </c>
       <c r="F29" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="G29" t="n">
-        <v>25.8</v>
+        <v>6.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6.84</v>
+        <v>19.94</v>
       </c>
       <c r="D30" t="n">
-        <v>0.65</v>
+        <v>1.1</v>
       </c>
       <c r="E30" t="n">
-        <v>7.9</v>
+        <v>5</v>
       </c>
       <c r="F30" t="n">
-        <v>18.4</v>
+        <v>5</v>
       </c>
       <c r="G30" t="n">
-        <v>15.3</v>
+        <v>5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>18.46</v>
+        <v>34.18</v>
       </c>
       <c r="D31" t="n">
-        <v>1.69</v>
+        <v>2.6</v>
       </c>
       <c r="E31" t="n">
-        <v>15.8</v>
+        <v>5</v>
       </c>
       <c r="F31" t="n">
-        <v>10.5</v>
+        <v>5</v>
       </c>
       <c r="G31" t="n">
-        <v>12.1</v>
+        <v>5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>14.96</v>
+        <v>18.37</v>
       </c>
       <c r="D32" t="n">
-        <v>1.41</v>
+        <v>1.68</v>
       </c>
       <c r="E32" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
-        <v>10.5</v>
+        <v>5</v>
       </c>
       <c r="G32" t="n">
-        <v>8.9</v>
+        <v>5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed May 13 11:51:45 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>31.37</v>
+        <v>70.87</v>
       </c>
       <c r="D2" t="n">
-        <v>2.97</v>
+        <v>7.32</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,7 +501,7 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="3">
@@ -516,562 +516,562 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.71</v>
+        <v>21.09</v>
       </c>
       <c r="D3" t="n">
-        <v>1.93</v>
+        <v>1.97</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>97.5</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>98.8</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>36.61</v>
+        <v>38.41</v>
       </c>
       <c r="D4" t="n">
-        <v>2.03</v>
+        <v>4.13</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>97.5</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>68.25</v>
+        <v>41.92</v>
       </c>
       <c r="D5" t="n">
-        <v>7.05</v>
+        <v>3.54</v>
       </c>
       <c r="E5" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>97.5</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>96.2</v>
+        <v>100</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>12.14</v>
+        <v>32.03</v>
       </c>
       <c r="D6" t="n">
-        <v>0.78</v>
+        <v>3.03</v>
       </c>
       <c r="E6" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>97.5</v>
+        <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>96.2</v>
+        <v>100</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>41.16</v>
+        <v>36.73</v>
       </c>
       <c r="D7" t="n">
-        <v>3.48</v>
+        <v>2.04</v>
       </c>
       <c r="E7" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>95</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>95</v>
+        <v>98.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>30.17</v>
+        <v>12.24</v>
       </c>
       <c r="D8" t="n">
-        <v>2.78</v>
+        <v>0.78</v>
       </c>
       <c r="E8" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>95</v>
+        <v>95.2</v>
       </c>
       <c r="G8" t="n">
-        <v>95</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10.69</v>
+        <v>55.13</v>
       </c>
       <c r="D9" t="n">
-        <v>1.3</v>
+        <v>4.54</v>
       </c>
       <c r="E9" t="n">
-        <v>95</v>
+        <v>95.2</v>
       </c>
       <c r="F9" t="n">
-        <v>92.5</v>
+        <v>95.2</v>
       </c>
       <c r="G9" t="n">
-        <v>93.8</v>
+        <v>95.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>22.15</v>
+        <v>24.8</v>
       </c>
       <c r="D10" t="n">
-        <v>1.86</v>
+        <v>1.82</v>
       </c>
       <c r="E10" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F10" t="n">
-        <v>90</v>
+        <v>90.5</v>
       </c>
       <c r="G10" t="n">
-        <v>85</v>
+        <v>95.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>26.59</v>
+        <v>27.35</v>
       </c>
       <c r="D11" t="n">
-        <v>2.4</v>
+        <v>2.53</v>
       </c>
       <c r="E11" t="n">
-        <v>85</v>
+        <v>85.7</v>
       </c>
       <c r="F11" t="n">
-        <v>85</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>85</v>
+        <v>89.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>13.48</v>
+        <v>24.1</v>
       </c>
       <c r="D12" t="n">
-        <v>1.23</v>
+        <v>4.07</v>
       </c>
       <c r="E12" t="n">
-        <v>70</v>
+        <v>76.2</v>
       </c>
       <c r="F12" t="n">
-        <v>97.5</v>
+        <v>100</v>
       </c>
       <c r="G12" t="n">
-        <v>83.8</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>23.91</v>
+        <v>16.64</v>
       </c>
       <c r="D13" t="n">
-        <v>4.04</v>
+        <v>2.46</v>
       </c>
       <c r="E13" t="n">
-        <v>70</v>
+        <v>90.5</v>
       </c>
       <c r="F13" t="n">
-        <v>90</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>80</v>
+        <v>84.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>37.68</v>
+        <v>70.42</v>
       </c>
       <c r="D14" t="n">
-        <v>4.05</v>
+        <v>4.58</v>
       </c>
       <c r="E14" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
       <c r="F14" t="n">
-        <v>75</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>77.5</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>69.88</v>
+        <v>26.46</v>
       </c>
       <c r="D15" t="n">
-        <v>4.54</v>
+        <v>2.39</v>
       </c>
       <c r="E15" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="F15" t="n">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="G15" t="n">
-        <v>77.5</v>
+        <v>81</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>27.26</v>
+        <v>13.32</v>
       </c>
       <c r="D16" t="n">
-        <v>2.51</v>
+        <v>1.21</v>
       </c>
       <c r="E16" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="F16" t="n">
-        <v>75</v>
+        <v>90.5</v>
       </c>
       <c r="G16" t="n">
-        <v>75</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>54.16</v>
+        <v>22.1</v>
       </c>
       <c r="D17" t="n">
-        <v>4.46</v>
+        <v>1.85</v>
       </c>
       <c r="E17" t="n">
-        <v>75</v>
+        <v>76.2</v>
       </c>
       <c r="F17" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="G17" t="n">
-        <v>75</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>15.73</v>
+        <v>137.51</v>
       </c>
       <c r="D18" t="n">
-        <v>1.28</v>
+        <v>5.16</v>
       </c>
       <c r="E18" t="n">
-        <v>70</v>
+        <v>76.2</v>
       </c>
       <c r="F18" t="n">
-        <v>75</v>
+        <v>76.2</v>
       </c>
       <c r="G18" t="n">
-        <v>72.5</v>
+        <v>76.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>16.58</v>
+        <v>15.75</v>
       </c>
       <c r="D19" t="n">
-        <v>2.45</v>
+        <v>1.28</v>
       </c>
       <c r="E19" t="n">
-        <v>85</v>
+        <v>73.8</v>
       </c>
       <c r="F19" t="n">
-        <v>60</v>
+        <v>73.8</v>
       </c>
       <c r="G19" t="n">
-        <v>72.5</v>
+        <v>73.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>132.48</v>
+        <v>29.2</v>
       </c>
       <c r="D20" t="n">
-        <v>4.97</v>
+        <v>2.68</v>
       </c>
       <c r="E20" t="n">
-        <v>70</v>
+        <v>66.7</v>
       </c>
       <c r="F20" t="n">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="G20" t="n">
-        <v>70</v>
+        <v>73.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>24.45</v>
+        <v>30</v>
       </c>
       <c r="D21" t="n">
-        <v>1.8</v>
+        <v>2.76</v>
       </c>
       <c r="E21" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="F21" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="G21" t="n">
-        <v>62.5</v>
+        <v>66.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="22">
@@ -1086,172 +1086,172 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28.82</v>
+        <v>29.03</v>
       </c>
       <c r="D22" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="E22" t="n">
-        <v>70</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>45</v>
+        <v>47.6</v>
       </c>
       <c r="G22" t="n">
-        <v>57.5</v>
+        <v>59.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>31.36</v>
+        <v>10.56</v>
       </c>
       <c r="D23" t="n">
-        <v>2.32</v>
+        <v>1.28</v>
       </c>
       <c r="E23" t="n">
-        <v>30</v>
+        <v>66.7</v>
       </c>
       <c r="F23" t="n">
-        <v>30</v>
+        <v>21.4</v>
       </c>
       <c r="G23" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>28.98</v>
+        <v>31.33</v>
       </c>
       <c r="D24" t="n">
-        <v>2.66</v>
+        <v>2.32</v>
       </c>
       <c r="E24" t="n">
-        <v>20</v>
+        <v>28.6</v>
       </c>
       <c r="F24" t="n">
-        <v>27.5</v>
+        <v>31</v>
       </c>
       <c r="G24" t="n">
-        <v>25.2</v>
+        <v>29.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21.49</v>
+        <v>32.95</v>
       </c>
       <c r="D25" t="n">
-        <v>3.73</v>
+        <v>2.76</v>
       </c>
       <c r="E25" t="n">
-        <v>70</v>
+        <v>14.3</v>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>42.9</v>
       </c>
       <c r="G25" t="n">
-        <v>24.5</v>
+        <v>28.6</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6.84</v>
+        <v>21.34</v>
       </c>
       <c r="D26" t="n">
-        <v>0.65</v>
+        <v>3.7</v>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>66.7</v>
       </c>
       <c r="F26" t="n">
-        <v>20</v>
+        <v>4.8</v>
       </c>
       <c r="G26" t="n">
-        <v>17</v>
+        <v>23.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>14.99</v>
+        <v>34.44</v>
       </c>
       <c r="D27" t="n">
-        <v>1.41</v>
+        <v>2.62</v>
       </c>
       <c r="E27" t="n">
-        <v>20</v>
+        <v>14.3</v>
       </c>
       <c r="F27" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="G27" t="n">
-        <v>14.8</v>
+        <v>16</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="28">
@@ -1266,52 +1266,52 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25.94</v>
+        <v>26.06</v>
       </c>
       <c r="D28" t="n">
-        <v>2.13</v>
+        <v>2.14</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>9.5</v>
       </c>
       <c r="F28" t="n">
-        <v>10</v>
+        <v>14.3</v>
       </c>
       <c r="G28" t="n">
-        <v>8.5</v>
+        <v>12.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>32.71</v>
+        <v>14.93</v>
       </c>
       <c r="D29" t="n">
-        <v>2.74</v>
+        <v>1.41</v>
       </c>
       <c r="E29" t="n">
-        <v>10</v>
+        <v>4.8</v>
       </c>
       <c r="F29" t="n">
-        <v>5</v>
+        <v>14.3</v>
       </c>
       <c r="G29" t="n">
-        <v>6.5</v>
+        <v>11.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="30">
@@ -1326,52 +1326,52 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.94</v>
+        <v>19.75</v>
       </c>
       <c r="D30" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="E30" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="F30" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="G30" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>34.18</v>
+        <v>6.77</v>
       </c>
       <c r="D31" t="n">
-        <v>2.6</v>
+        <v>0.64</v>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="F31" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="G31" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18.37</v>
+        <v>18.2</v>
       </c>
       <c r="D32" t="n">
-        <v>1.68</v>
+        <v>1.66</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="F32" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="G32" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu May 14 11:29:02 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>70.87</v>
+        <v>32.13</v>
       </c>
       <c r="D2" t="n">
-        <v>7.32</v>
+        <v>3.04</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,67 +501,67 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>21.09</v>
+        <v>68.95</v>
       </c>
       <c r="D3" t="n">
-        <v>1.97</v>
+        <v>7.12</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>95.5</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>95.5</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>95.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>38.41</v>
+        <v>20.7</v>
       </c>
       <c r="D4" t="n">
-        <v>4.13</v>
+        <v>1.93</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="5">
@@ -576,832 +576,832 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>41.92</v>
+        <v>40.93</v>
       </c>
       <c r="D5" t="n">
-        <v>3.54</v>
+        <v>3.46</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>32.03</v>
+        <v>36.07</v>
       </c>
       <c r="D6" t="n">
-        <v>3.03</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>68.2</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>68.2</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>68.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>36.73</v>
+        <v>133.41</v>
       </c>
       <c r="D7" t="n">
-        <v>2.04</v>
+        <v>5.01</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>68.2</v>
       </c>
       <c r="F7" t="n">
-        <v>97.59999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="G7" t="n">
-        <v>98.8</v>
+        <v>68.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>12.24</v>
+        <v>26.15</v>
       </c>
       <c r="D8" t="n">
-        <v>0.78</v>
+        <v>2.36</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>68.2</v>
       </c>
       <c r="F8" t="n">
-        <v>95.2</v>
+        <v>68.2</v>
       </c>
       <c r="G8" t="n">
-        <v>97.59999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>55.13</v>
+        <v>11.97</v>
       </c>
       <c r="D9" t="n">
-        <v>4.54</v>
+        <v>0.77</v>
       </c>
       <c r="E9" t="n">
-        <v>95.2</v>
+        <v>68.2</v>
       </c>
       <c r="F9" t="n">
-        <v>95.2</v>
+        <v>68.2</v>
       </c>
       <c r="G9" t="n">
-        <v>95.2</v>
+        <v>68.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>24.8</v>
+        <v>16.56</v>
       </c>
       <c r="D10" t="n">
-        <v>1.82</v>
+        <v>2.45</v>
       </c>
       <c r="E10" t="n">
-        <v>100</v>
+        <v>77.3</v>
       </c>
       <c r="F10" t="n">
-        <v>90.5</v>
+        <v>56.8</v>
       </c>
       <c r="G10" t="n">
-        <v>95.2</v>
+        <v>67</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.35</v>
+        <v>15.67</v>
       </c>
       <c r="D11" t="n">
-        <v>2.53</v>
+        <v>1.28</v>
       </c>
       <c r="E11" t="n">
-        <v>85.7</v>
+        <v>54.5</v>
       </c>
       <c r="F11" t="n">
-        <v>92.90000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="G11" t="n">
-        <v>89.3</v>
+        <v>63.6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>24.1</v>
+        <v>53.22</v>
       </c>
       <c r="D12" t="n">
-        <v>4.07</v>
+        <v>4.38</v>
       </c>
       <c r="E12" t="n">
-        <v>76.2</v>
+        <v>63.6</v>
       </c>
       <c r="F12" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G12" t="n">
-        <v>88.09999999999999</v>
+        <v>56.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>16.64</v>
+        <v>13.11</v>
       </c>
       <c r="D13" t="n">
-        <v>2.46</v>
+        <v>1.18</v>
       </c>
       <c r="E13" t="n">
-        <v>90.5</v>
+        <v>45.5</v>
       </c>
       <c r="F13" t="n">
-        <v>78.59999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="G13" t="n">
-        <v>84.5</v>
+        <v>56.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>70.42</v>
+        <v>24.29</v>
       </c>
       <c r="D14" t="n">
-        <v>4.58</v>
+        <v>1.78</v>
       </c>
       <c r="E14" t="n">
-        <v>66.7</v>
+        <v>40.9</v>
       </c>
       <c r="F14" t="n">
-        <v>97.59999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>82.09999999999999</v>
+        <v>53.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26.46</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>2.39</v>
+        <v>4.36</v>
       </c>
       <c r="E15" t="n">
-        <v>81</v>
+        <v>36.4</v>
       </c>
       <c r="F15" t="n">
-        <v>81</v>
+        <v>68.2</v>
       </c>
       <c r="G15" t="n">
-        <v>81</v>
+        <v>52.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>13.32</v>
+        <v>26.89</v>
       </c>
       <c r="D16" t="n">
-        <v>1.21</v>
+        <v>2.48</v>
       </c>
       <c r="E16" t="n">
-        <v>66.7</v>
+        <v>63.6</v>
       </c>
       <c r="F16" t="n">
-        <v>90.5</v>
+        <v>40.9</v>
       </c>
       <c r="G16" t="n">
-        <v>78.59999999999999</v>
+        <v>52.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>22.1</v>
+        <v>23.26</v>
       </c>
       <c r="D17" t="n">
-        <v>1.85</v>
+        <v>3.93</v>
       </c>
       <c r="E17" t="n">
-        <v>76.2</v>
+        <v>31.8</v>
       </c>
       <c r="F17" t="n">
-        <v>81</v>
+        <v>63.6</v>
       </c>
       <c r="G17" t="n">
-        <v>78.59999999999999</v>
+        <v>47.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>137.51</v>
+        <v>37.18</v>
       </c>
       <c r="D18" t="n">
-        <v>5.16</v>
+        <v>4</v>
       </c>
       <c r="E18" t="n">
-        <v>76.2</v>
+        <v>63.6</v>
       </c>
       <c r="F18" t="n">
-        <v>76.2</v>
+        <v>29.5</v>
       </c>
       <c r="G18" t="n">
-        <v>76.2</v>
+        <v>39.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15.75</v>
+        <v>21.83</v>
       </c>
       <c r="D19" t="n">
-        <v>1.28</v>
+        <v>1.83</v>
       </c>
       <c r="E19" t="n">
-        <v>73.8</v>
+        <v>31.8</v>
       </c>
       <c r="F19" t="n">
-        <v>73.8</v>
+        <v>43.2</v>
       </c>
       <c r="G19" t="n">
-        <v>73.8</v>
+        <v>37.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29.2</v>
+        <v>31.3</v>
       </c>
       <c r="D20" t="n">
-        <v>2.68</v>
+        <v>2.32</v>
       </c>
       <c r="E20" t="n">
-        <v>66.7</v>
+        <v>27.3</v>
       </c>
       <c r="F20" t="n">
-        <v>81</v>
+        <v>31.8</v>
       </c>
       <c r="G20" t="n">
-        <v>73.8</v>
+        <v>29.5</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>30</v>
+        <v>21.33</v>
       </c>
       <c r="D21" t="n">
-        <v>2.76</v>
+        <v>3.7</v>
       </c>
       <c r="E21" t="n">
-        <v>66.7</v>
+        <v>63.6</v>
       </c>
       <c r="F21" t="n">
-        <v>66.7</v>
+        <v>6.8</v>
       </c>
       <c r="G21" t="n">
-        <v>66.7</v>
+        <v>23.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>29.03</v>
+        <v>6.82</v>
       </c>
       <c r="D22" t="n">
-        <v>2.37</v>
+        <v>0.65</v>
       </c>
       <c r="E22" t="n">
-        <v>71.40000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="F22" t="n">
-        <v>47.6</v>
+        <v>25</v>
       </c>
       <c r="G22" t="n">
-        <v>59.5</v>
+        <v>20.2</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10.56</v>
+        <v>14.94</v>
       </c>
       <c r="D23" t="n">
-        <v>1.28</v>
+        <v>1.41</v>
       </c>
       <c r="E23" t="n">
-        <v>66.7</v>
+        <v>9.1</v>
       </c>
       <c r="F23" t="n">
-        <v>21.4</v>
+        <v>15.9</v>
       </c>
       <c r="G23" t="n">
-        <v>35</v>
+        <v>13.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>31.33</v>
+        <v>10.36</v>
       </c>
       <c r="D24" t="n">
-        <v>2.32</v>
+        <v>1.26</v>
       </c>
       <c r="E24" t="n">
-        <v>28.6</v>
+        <v>31.8</v>
       </c>
       <c r="F24" t="n">
-        <v>31</v>
+        <v>4.5</v>
       </c>
       <c r="G24" t="n">
-        <v>29.8</v>
+        <v>12.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>32.95</v>
+        <v>29.31</v>
       </c>
       <c r="D25" t="n">
-        <v>2.76</v>
+        <v>2.7</v>
       </c>
       <c r="E25" t="n">
-        <v>14.3</v>
+        <v>9.1</v>
       </c>
       <c r="F25" t="n">
-        <v>42.9</v>
+        <v>9.1</v>
       </c>
       <c r="G25" t="n">
-        <v>28.6</v>
+        <v>9.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>21.34</v>
+        <v>25.79</v>
       </c>
       <c r="D26" t="n">
-        <v>3.7</v>
+        <v>2.12</v>
       </c>
       <c r="E26" t="n">
-        <v>66.7</v>
+        <v>4.5</v>
       </c>
       <c r="F26" t="n">
-        <v>4.8</v>
+        <v>9.1</v>
       </c>
       <c r="G26" t="n">
-        <v>23.3</v>
+        <v>7.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>34.44</v>
+        <v>28.67</v>
       </c>
       <c r="D27" t="n">
-        <v>2.62</v>
+        <v>2.63</v>
       </c>
       <c r="E27" t="n">
-        <v>14.3</v>
+        <v>9.1</v>
       </c>
       <c r="F27" t="n">
-        <v>16.7</v>
+        <v>6.8</v>
       </c>
       <c r="G27" t="n">
-        <v>16</v>
+        <v>7.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>26.06</v>
+        <v>18.16</v>
       </c>
       <c r="D28" t="n">
-        <v>2.14</v>
+        <v>1.66</v>
       </c>
       <c r="E28" t="n">
-        <v>9.5</v>
+        <v>4.5</v>
       </c>
       <c r="F28" t="n">
-        <v>14.3</v>
+        <v>6.8</v>
       </c>
       <c r="G28" t="n">
-        <v>12.9</v>
+        <v>6.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>14.93</v>
+        <v>32.31</v>
       </c>
       <c r="D29" t="n">
-        <v>1.41</v>
+        <v>2.71</v>
       </c>
       <c r="E29" t="n">
-        <v>4.8</v>
+        <v>9.1</v>
       </c>
       <c r="F29" t="n">
-        <v>14.3</v>
+        <v>4.5</v>
       </c>
       <c r="G29" t="n">
-        <v>11.4</v>
+        <v>5.9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.75</v>
+        <v>28.01</v>
       </c>
       <c r="D30" t="n">
-        <v>1.09</v>
+        <v>2.29</v>
       </c>
       <c r="E30" t="n">
-        <v>4.8</v>
+        <v>9.1</v>
       </c>
       <c r="F30" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="G30" t="n">
-        <v>4.8</v>
+        <v>5.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>6.77</v>
+        <v>19.41</v>
       </c>
       <c r="D31" t="n">
-        <v>0.64</v>
+        <v>1.08</v>
       </c>
       <c r="E31" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="F31" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="G31" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18.2</v>
+        <v>33.7</v>
       </c>
       <c r="D32" t="n">
-        <v>1.66</v>
+        <v>2.57</v>
       </c>
       <c r="E32" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="F32" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="G32" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri May 15 11:37:24 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,31 +477,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>32.13</v>
+        <v>16.7</v>
       </c>
       <c r="D2" t="n">
-        <v>3.04</v>
+        <v>2.47</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>95.7</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>95.7</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>95.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="3">
@@ -516,142 +516,142 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>68.95</v>
+        <v>68.44</v>
       </c>
       <c r="D3" t="n">
-        <v>7.12</v>
+        <v>7.07</v>
       </c>
       <c r="E3" t="n">
-        <v>95.5</v>
+        <v>91.3</v>
       </c>
       <c r="F3" t="n">
-        <v>95.5</v>
+        <v>91.3</v>
       </c>
       <c r="G3" t="n">
-        <v>95.5</v>
+        <v>91.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20.7</v>
+        <v>41.42</v>
       </c>
       <c r="D4" t="n">
-        <v>1.93</v>
+        <v>3.5</v>
       </c>
       <c r="E4" t="n">
-        <v>90.90000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="F4" t="n">
-        <v>90.90000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="G4" t="n">
-        <v>90.90000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>40.93</v>
+        <v>31.57</v>
       </c>
       <c r="D5" t="n">
-        <v>3.46</v>
+        <v>2.99</v>
       </c>
       <c r="E5" t="n">
-        <v>86.40000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="F5" t="n">
-        <v>86.40000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="G5" t="n">
-        <v>86.40000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>36.07</v>
+        <v>20.58</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1.92</v>
       </c>
       <c r="E6" t="n">
-        <v>68.2</v>
+        <v>87</v>
       </c>
       <c r="F6" t="n">
-        <v>68.2</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>68.2</v>
+        <v>84.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>133.41</v>
+        <v>26.93</v>
       </c>
       <c r="D7" t="n">
-        <v>5.01</v>
+        <v>2.5</v>
       </c>
       <c r="E7" t="n">
-        <v>68.2</v>
+        <v>65.2</v>
       </c>
       <c r="F7" t="n">
-        <v>68.2</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>68.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="8">
@@ -666,322 +666,322 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>26.15</v>
+        <v>26.13</v>
       </c>
       <c r="D8" t="n">
         <v>2.36</v>
       </c>
       <c r="E8" t="n">
-        <v>68.2</v>
+        <v>65.2</v>
       </c>
       <c r="F8" t="n">
-        <v>68.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>68.2</v>
+        <v>66.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>11.97</v>
+        <v>34.63</v>
       </c>
       <c r="D9" t="n">
-        <v>0.77</v>
+        <v>1.93</v>
       </c>
       <c r="E9" t="n">
-        <v>68.2</v>
+        <v>60.9</v>
       </c>
       <c r="F9" t="n">
-        <v>68.2</v>
+        <v>60.9</v>
       </c>
       <c r="G9" t="n">
-        <v>68.2</v>
+        <v>60.9</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>16.56</v>
+        <v>52.75</v>
       </c>
       <c r="D10" t="n">
-        <v>2.45</v>
+        <v>4.35</v>
       </c>
       <c r="E10" t="n">
-        <v>77.3</v>
+        <v>60.9</v>
       </c>
       <c r="F10" t="n">
-        <v>56.8</v>
+        <v>43.5</v>
       </c>
       <c r="G10" t="n">
-        <v>67</v>
+        <v>52.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>15.67</v>
+        <v>12.94</v>
       </c>
       <c r="D11" t="n">
-        <v>1.28</v>
+        <v>1.16</v>
       </c>
       <c r="E11" t="n">
-        <v>54.5</v>
+        <v>39.1</v>
       </c>
       <c r="F11" t="n">
-        <v>72.7</v>
+        <v>56.5</v>
       </c>
       <c r="G11" t="n">
-        <v>63.6</v>
+        <v>47.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>53.22</v>
+        <v>15.1</v>
       </c>
       <c r="D12" t="n">
-        <v>4.38</v>
+        <v>1.42</v>
       </c>
       <c r="E12" t="n">
-        <v>63.6</v>
+        <v>39.1</v>
       </c>
       <c r="F12" t="n">
-        <v>50</v>
+        <v>34.8</v>
       </c>
       <c r="G12" t="n">
-        <v>56.8</v>
+        <v>37</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>13.11</v>
+        <v>65.84999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>1.18</v>
+        <v>4.28</v>
       </c>
       <c r="E13" t="n">
-        <v>45.5</v>
+        <v>30.4</v>
       </c>
       <c r="F13" t="n">
-        <v>68.2</v>
+        <v>43.5</v>
       </c>
       <c r="G13" t="n">
-        <v>56.8</v>
+        <v>37</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>24.29</v>
+        <v>130.12</v>
       </c>
       <c r="D14" t="n">
-        <v>1.78</v>
+        <v>4.88</v>
       </c>
       <c r="E14" t="n">
-        <v>40.9</v>
+        <v>34.8</v>
       </c>
       <c r="F14" t="n">
-        <v>65.90000000000001</v>
+        <v>34.8</v>
       </c>
       <c r="G14" t="n">
-        <v>53.4</v>
+        <v>34.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>67.15000000000001</v>
+        <v>11.86</v>
       </c>
       <c r="D15" t="n">
-        <v>4.36</v>
+        <v>0.75</v>
       </c>
       <c r="E15" t="n">
-        <v>36.4</v>
+        <v>65.2</v>
       </c>
       <c r="F15" t="n">
-        <v>68.2</v>
+        <v>19.6</v>
       </c>
       <c r="G15" t="n">
-        <v>52.3</v>
+        <v>33.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26.89</v>
+        <v>36.97</v>
       </c>
       <c r="D16" t="n">
-        <v>2.48</v>
+        <v>3.98</v>
       </c>
       <c r="E16" t="n">
-        <v>63.6</v>
+        <v>60.9</v>
       </c>
       <c r="F16" t="n">
-        <v>40.9</v>
+        <v>13</v>
       </c>
       <c r="G16" t="n">
-        <v>52.3</v>
+        <v>27.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.26</v>
+        <v>23.86</v>
       </c>
       <c r="D17" t="n">
-        <v>3.93</v>
+        <v>1.75</v>
       </c>
       <c r="E17" t="n">
-        <v>31.8</v>
+        <v>4.3</v>
       </c>
       <c r="F17" t="n">
-        <v>63.6</v>
+        <v>45.7</v>
       </c>
       <c r="G17" t="n">
-        <v>47.7</v>
+        <v>25</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>37.18</v>
+        <v>18.45</v>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>1.69</v>
       </c>
       <c r="E18" t="n">
-        <v>63.6</v>
+        <v>21.7</v>
       </c>
       <c r="F18" t="n">
-        <v>29.5</v>
+        <v>23.9</v>
       </c>
       <c r="G18" t="n">
-        <v>39.8</v>
+        <v>23.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="19">
@@ -996,172 +996,172 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>21.83</v>
+        <v>21.7</v>
       </c>
       <c r="D19" t="n">
-        <v>1.83</v>
+        <v>1.82</v>
       </c>
       <c r="E19" t="n">
-        <v>31.8</v>
+        <v>26.1</v>
       </c>
       <c r="F19" t="n">
-        <v>43.2</v>
+        <v>21.7</v>
       </c>
       <c r="G19" t="n">
-        <v>37.5</v>
+        <v>23</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>31.3</v>
+        <v>21.04</v>
       </c>
       <c r="D20" t="n">
-        <v>2.32</v>
+        <v>3.65</v>
       </c>
       <c r="E20" t="n">
-        <v>27.3</v>
+        <v>60.9</v>
       </c>
       <c r="F20" t="n">
-        <v>31.8</v>
+        <v>4.3</v>
       </c>
       <c r="G20" t="n">
-        <v>29.5</v>
+        <v>21.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>21.33</v>
+        <v>31.02</v>
       </c>
       <c r="D21" t="n">
-        <v>3.7</v>
+        <v>2.3</v>
       </c>
       <c r="E21" t="n">
-        <v>63.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>6.8</v>
+        <v>10.9</v>
       </c>
       <c r="G21" t="n">
-        <v>23.9</v>
+        <v>10.2</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>6.82</v>
+        <v>15.46</v>
       </c>
       <c r="D22" t="n">
-        <v>0.65</v>
+        <v>1.26</v>
       </c>
       <c r="E22" t="n">
-        <v>9.1</v>
+        <v>13</v>
       </c>
       <c r="F22" t="n">
-        <v>25</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G22" t="n">
-        <v>20.2</v>
+        <v>10</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>14.94</v>
+        <v>28.12</v>
       </c>
       <c r="D23" t="n">
-        <v>1.41</v>
+        <v>2.3</v>
       </c>
       <c r="E23" t="n">
-        <v>9.1</v>
+        <v>13</v>
       </c>
       <c r="F23" t="n">
-        <v>15.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>13.9</v>
+        <v>10</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10.36</v>
+        <v>28.66</v>
       </c>
       <c r="D24" t="n">
-        <v>1.26</v>
+        <v>2.63</v>
       </c>
       <c r="E24" t="n">
-        <v>31.8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>4.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G24" t="n">
-        <v>12.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="25">
@@ -1176,112 +1176,112 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29.31</v>
+        <v>29.11</v>
       </c>
       <c r="D25" t="n">
-        <v>2.7</v>
+        <v>2.68</v>
       </c>
       <c r="E25" t="n">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F25" t="n">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G25" t="n">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25.79</v>
+        <v>22.29</v>
       </c>
       <c r="D26" t="n">
-        <v>2.12</v>
+        <v>3.77</v>
       </c>
       <c r="E26" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="F26" t="n">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>28.67</v>
+        <v>25.33</v>
       </c>
       <c r="D27" t="n">
-        <v>2.63</v>
+        <v>2.08</v>
       </c>
       <c r="E27" t="n">
-        <v>9.1</v>
+        <v>4.3</v>
       </c>
       <c r="F27" t="n">
-        <v>6.8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G27" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18.16</v>
+        <v>6.8</v>
       </c>
       <c r="D28" t="n">
-        <v>1.66</v>
+        <v>0.64</v>
       </c>
       <c r="E28" t="n">
-        <v>4.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F28" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="G28" t="n">
-        <v>6.1</v>
+        <v>7.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="29">
@@ -1296,112 +1296,112 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>32.31</v>
+        <v>31.79</v>
       </c>
       <c r="D29" t="n">
-        <v>2.71</v>
+        <v>2.66</v>
       </c>
       <c r="E29" t="n">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F29" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="G29" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>28.01</v>
+        <v>19.03</v>
       </c>
       <c r="D30" t="n">
-        <v>2.29</v>
+        <v>1.06</v>
       </c>
       <c r="E30" t="n">
-        <v>9.1</v>
+        <v>4.3</v>
       </c>
       <c r="F30" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="G30" t="n">
-        <v>5.9</v>
+        <v>4.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>19.41</v>
+        <v>33.53</v>
       </c>
       <c r="D31" t="n">
-        <v>1.08</v>
+        <v>2.55</v>
       </c>
       <c r="E31" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="F31" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="G31" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>33.7</v>
+        <v>10.14</v>
       </c>
       <c r="D32" t="n">
-        <v>2.57</v>
+        <v>1.23</v>
       </c>
       <c r="E32" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="F32" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="G32" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat May 16 10:49:07 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.47</v>
       </c>
       <c r="E2" t="n">
-        <v>95.7</v>
+        <v>93.8</v>
       </c>
       <c r="F2" t="n">
-        <v>95.7</v>
+        <v>93.8</v>
       </c>
       <c r="G2" t="n">
-        <v>95.7</v>
+        <v>93.8</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>7.07</v>
       </c>
       <c r="E3" t="n">
-        <v>91.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>91.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>91.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.5</v>
       </c>
       <c r="E4" t="n">
-        <v>91.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>91.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>91.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.99</v>
       </c>
       <c r="E5" t="n">
-        <v>91.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>91.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>91.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.92</v>
       </c>
       <c r="E6" t="n">
-        <v>87</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>82.59999999999999</v>
+        <v>81.2</v>
       </c>
       <c r="G6" t="n">
-        <v>84.8</v>
+        <v>83.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.5</v>
       </c>
       <c r="E7" t="n">
-        <v>65.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>69.59999999999999</v>
+        <v>68.8</v>
       </c>
       <c r="G7" t="n">
-        <v>67.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.36</v>
       </c>
       <c r="E8" t="n">
-        <v>65.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>67.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="G8" t="n">
-        <v>66.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.93</v>
       </c>
       <c r="E9" t="n">
-        <v>60.9</v>
+        <v>60.4</v>
       </c>
       <c r="F9" t="n">
-        <v>60.9</v>
+        <v>60.4</v>
       </c>
       <c r="G9" t="n">
-        <v>60.9</v>
+        <v>60.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>4.35</v>
       </c>
       <c r="E10" t="n">
-        <v>60.9</v>
+        <v>60.4</v>
       </c>
       <c r="F10" t="n">
-        <v>43.5</v>
+        <v>43.8</v>
       </c>
       <c r="G10" t="n">
-        <v>52.2</v>
+        <v>52.1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.16</v>
       </c>
       <c r="E11" t="n">
-        <v>39.1</v>
+        <v>39.6</v>
       </c>
       <c r="F11" t="n">
-        <v>56.5</v>
+        <v>56.2</v>
       </c>
       <c r="G11" t="n">
-        <v>47.8</v>
+        <v>47.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.42</v>
       </c>
       <c r="E12" t="n">
-        <v>39.1</v>
+        <v>39.6</v>
       </c>
       <c r="F12" t="n">
-        <v>34.8</v>
+        <v>35.4</v>
       </c>
       <c r="G12" t="n">
-        <v>37</v>
+        <v>37.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>4.28</v>
       </c>
       <c r="E13" t="n">
-        <v>30.4</v>
+        <v>31.2</v>
       </c>
       <c r="F13" t="n">
-        <v>43.5</v>
+        <v>43.8</v>
       </c>
       <c r="G13" t="n">
-        <v>37</v>
+        <v>37.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>4.88</v>
       </c>
       <c r="E14" t="n">
-        <v>34.8</v>
+        <v>35.4</v>
       </c>
       <c r="F14" t="n">
-        <v>34.8</v>
+        <v>35.4</v>
       </c>
       <c r="G14" t="n">
-        <v>34.8</v>
+        <v>35.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>0.75</v>
       </c>
       <c r="E15" t="n">
-        <v>65.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>19.6</v>
+        <v>20.8</v>
       </c>
       <c r="G15" t="n">
-        <v>33.3</v>
+        <v>34</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>3.98</v>
       </c>
       <c r="E16" t="n">
-        <v>60.9</v>
+        <v>60.4</v>
       </c>
       <c r="F16" t="n">
-        <v>13</v>
+        <v>14.6</v>
       </c>
       <c r="G16" t="n">
-        <v>27.4</v>
+        <v>28.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.75</v>
       </c>
       <c r="E17" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="F17" t="n">
-        <v>45.7</v>
+        <v>45.8</v>
       </c>
       <c r="G17" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.69</v>
       </c>
       <c r="E18" t="n">
-        <v>21.7</v>
+        <v>22.9</v>
       </c>
       <c r="F18" t="n">
-        <v>23.9</v>
+        <v>25</v>
       </c>
       <c r="G18" t="n">
-        <v>23.3</v>
+        <v>24.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.82</v>
       </c>
       <c r="E19" t="n">
-        <v>26.1</v>
+        <v>27.1</v>
       </c>
       <c r="F19" t="n">
-        <v>21.7</v>
+        <v>22.9</v>
       </c>
       <c r="G19" t="n">
-        <v>23</v>
+        <v>24.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>3.65</v>
       </c>
       <c r="E20" t="n">
-        <v>60.9</v>
+        <v>60.4</v>
       </c>
       <c r="F20" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="G20" t="n">
-        <v>21.3</v>
+        <v>22.5</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.3</v>
       </c>
       <c r="E21" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="F21" t="n">
-        <v>10.9</v>
+        <v>12.5</v>
       </c>
       <c r="G21" t="n">
-        <v>10.2</v>
+        <v>11.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.26</v>
       </c>
       <c r="E22" t="n">
-        <v>13</v>
+        <v>14.6</v>
       </c>
       <c r="F22" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G22" t="n">
-        <v>10</v>
+        <v>11.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.3</v>
       </c>
       <c r="E23" t="n">
-        <v>13</v>
+        <v>14.6</v>
       </c>
       <c r="F23" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G23" t="n">
-        <v>10</v>
+        <v>11.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.63</v>
       </c>
       <c r="E24" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="F24" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G24" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.68</v>
       </c>
       <c r="E25" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="F25" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G25" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.77</v>
       </c>
       <c r="E26" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="F26" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G26" t="n">
-        <v>7.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.08</v>
       </c>
       <c r="E27" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="F27" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G27" t="n">
-        <v>7.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>0.64</v>
       </c>
       <c r="E28" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="F28" t="n">
-        <v>6.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>7.2</v>
+        <v>9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>2.66</v>
       </c>
       <c r="E29" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="F29" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="G29" t="n">
-        <v>5.7</v>
+        <v>7.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.06</v>
       </c>
       <c r="E30" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="F30" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="G30" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>2.55</v>
       </c>
       <c r="E31" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="F31" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="G31" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.23</v>
       </c>
       <c r="E32" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="F32" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="G32" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun May 17 10:56:23 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.47</v>
       </c>
       <c r="E2" t="n">
-        <v>93.8</v>
+        <v>92</v>
       </c>
       <c r="F2" t="n">
-        <v>93.8</v>
+        <v>92</v>
       </c>
       <c r="G2" t="n">
-        <v>93.8</v>
+        <v>92</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>7.07</v>
       </c>
       <c r="E3" t="n">
-        <v>89.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="F3" t="n">
-        <v>89.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="G3" t="n">
-        <v>89.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.5</v>
       </c>
       <c r="E4" t="n">
-        <v>89.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="F4" t="n">
-        <v>89.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="G4" t="n">
-        <v>89.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.99</v>
       </c>
       <c r="E5" t="n">
-        <v>89.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="F5" t="n">
-        <v>89.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="G5" t="n">
-        <v>89.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.92</v>
       </c>
       <c r="E6" t="n">
-        <v>85.40000000000001</v>
+        <v>84</v>
       </c>
       <c r="F6" t="n">
-        <v>81.2</v>
+        <v>80</v>
       </c>
       <c r="G6" t="n">
-        <v>83.3</v>
+        <v>82</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.5</v>
       </c>
       <c r="E7" t="n">
-        <v>64.59999999999999</v>
+        <v>64</v>
       </c>
       <c r="F7" t="n">
-        <v>68.8</v>
+        <v>68</v>
       </c>
       <c r="G7" t="n">
-        <v>66.7</v>
+        <v>66</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.36</v>
       </c>
       <c r="E8" t="n">
-        <v>64.59999999999999</v>
+        <v>64</v>
       </c>
       <c r="F8" t="n">
-        <v>66.7</v>
+        <v>66</v>
       </c>
       <c r="G8" t="n">
-        <v>65.59999999999999</v>
+        <v>65</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.93</v>
       </c>
       <c r="E9" t="n">
-        <v>60.4</v>
+        <v>60</v>
       </c>
       <c r="F9" t="n">
-        <v>60.4</v>
+        <v>60</v>
       </c>
       <c r="G9" t="n">
-        <v>60.4</v>
+        <v>60</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>4.35</v>
       </c>
       <c r="E10" t="n">
-        <v>60.4</v>
+        <v>60</v>
       </c>
       <c r="F10" t="n">
-        <v>43.8</v>
+        <v>44</v>
       </c>
       <c r="G10" t="n">
-        <v>52.1</v>
+        <v>52</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.16</v>
       </c>
       <c r="E11" t="n">
-        <v>39.6</v>
+        <v>40</v>
       </c>
       <c r="F11" t="n">
-        <v>56.2</v>
+        <v>56</v>
       </c>
       <c r="G11" t="n">
-        <v>47.9</v>
+        <v>48</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.42</v>
       </c>
       <c r="E12" t="n">
-        <v>39.6</v>
+        <v>40</v>
       </c>
       <c r="F12" t="n">
-        <v>35.4</v>
+        <v>36</v>
       </c>
       <c r="G12" t="n">
-        <v>37.5</v>
+        <v>38</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>4.28</v>
       </c>
       <c r="E13" t="n">
-        <v>31.2</v>
+        <v>32</v>
       </c>
       <c r="F13" t="n">
-        <v>43.8</v>
+        <v>44</v>
       </c>
       <c r="G13" t="n">
-        <v>37.5</v>
+        <v>38</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>4.88</v>
       </c>
       <c r="E14" t="n">
-        <v>35.4</v>
+        <v>36</v>
       </c>
       <c r="F14" t="n">
-        <v>35.4</v>
+        <v>36</v>
       </c>
       <c r="G14" t="n">
-        <v>35.4</v>
+        <v>36</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>0.75</v>
       </c>
       <c r="E15" t="n">
-        <v>64.59999999999999</v>
+        <v>64</v>
       </c>
       <c r="F15" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="G15" t="n">
-        <v>34</v>
+        <v>34.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>3.98</v>
       </c>
       <c r="E16" t="n">
-        <v>60.4</v>
+        <v>60</v>
       </c>
       <c r="F16" t="n">
-        <v>14.6</v>
+        <v>16</v>
       </c>
       <c r="G16" t="n">
-        <v>28.3</v>
+        <v>29.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.75</v>
       </c>
       <c r="E17" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
-        <v>45.8</v>
+        <v>46</v>
       </c>
       <c r="G17" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.69</v>
       </c>
       <c r="E18" t="n">
-        <v>22.9</v>
+        <v>24</v>
       </c>
       <c r="F18" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G18" t="n">
-        <v>24.4</v>
+        <v>25.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.82</v>
       </c>
       <c r="E19" t="n">
-        <v>27.1</v>
+        <v>28</v>
       </c>
       <c r="F19" t="n">
-        <v>22.9</v>
+        <v>24</v>
       </c>
       <c r="G19" t="n">
-        <v>24.2</v>
+        <v>25.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>3.65</v>
       </c>
       <c r="E20" t="n">
-        <v>60.4</v>
+        <v>60</v>
       </c>
       <c r="F20" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="G20" t="n">
-        <v>22.5</v>
+        <v>23.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.3</v>
       </c>
       <c r="E21" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="F21" t="n">
-        <v>12.5</v>
+        <v>14</v>
       </c>
       <c r="G21" t="n">
-        <v>11.9</v>
+        <v>13.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.26</v>
       </c>
       <c r="E22" t="n">
-        <v>14.6</v>
+        <v>16</v>
       </c>
       <c r="F22" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="G22" t="n">
-        <v>11.7</v>
+        <v>13.2</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.3</v>
       </c>
       <c r="E23" t="n">
-        <v>14.6</v>
+        <v>16</v>
       </c>
       <c r="F23" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="G23" t="n">
-        <v>11.7</v>
+        <v>13.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.63</v>
       </c>
       <c r="E24" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="F24" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="G24" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.68</v>
       </c>
       <c r="E25" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="F25" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="G25" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.77</v>
       </c>
       <c r="E26" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="F26" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="G26" t="n">
-        <v>9.199999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.08</v>
       </c>
       <c r="E27" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="F27" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="G27" t="n">
-        <v>9.199999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>0.64</v>
       </c>
       <c r="E28" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="F28" t="n">
-        <v>8.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="G28" t="n">
-        <v>9</v>
+        <v>10.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>2.66</v>
       </c>
       <c r="E29" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="F29" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="G29" t="n">
-        <v>7.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.06</v>
       </c>
       <c r="E30" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="F30" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="G30" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>2.55</v>
       </c>
       <c r="E31" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="F31" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="G31" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.23</v>
       </c>
       <c r="E32" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="F32" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="G32" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon May 18 12:56:43 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,31 +477,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>16.7</v>
+        <v>32.19</v>
       </c>
       <c r="D2" t="n">
-        <v>2.47</v>
+        <v>3.05</v>
       </c>
       <c r="E2" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="3">
@@ -516,82 +516,82 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>68.44</v>
+        <v>69.53</v>
       </c>
       <c r="D3" t="n">
-        <v>7.07</v>
+        <v>7.19</v>
       </c>
       <c r="E3" t="n">
-        <v>88</v>
+        <v>96.2</v>
       </c>
       <c r="F3" t="n">
-        <v>88</v>
+        <v>96.2</v>
       </c>
       <c r="G3" t="n">
-        <v>88</v>
+        <v>96.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>41.42</v>
+        <v>16.7</v>
       </c>
       <c r="D4" t="n">
-        <v>3.5</v>
+        <v>2.47</v>
       </c>
       <c r="E4" t="n">
-        <v>88</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>88</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>88</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>31.57</v>
+        <v>41.47</v>
       </c>
       <c r="D5" t="n">
-        <v>2.99</v>
+        <v>3.5</v>
       </c>
       <c r="E5" t="n">
-        <v>88</v>
+        <v>92.3</v>
       </c>
       <c r="F5" t="n">
-        <v>88</v>
+        <v>86.5</v>
       </c>
       <c r="G5" t="n">
-        <v>88</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="6">
@@ -606,382 +606,382 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>20.58</v>
+        <v>20.63</v>
       </c>
       <c r="D6" t="n">
-        <v>1.92</v>
+        <v>1.93</v>
       </c>
       <c r="E6" t="n">
-        <v>84</v>
+        <v>88.5</v>
       </c>
       <c r="F6" t="n">
-        <v>80</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>82</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>26.93</v>
+        <v>53.16</v>
       </c>
       <c r="D7" t="n">
-        <v>2.5</v>
+        <v>4.38</v>
       </c>
       <c r="E7" t="n">
-        <v>64</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>68</v>
+        <v>55.8</v>
       </c>
       <c r="G7" t="n">
-        <v>66</v>
+        <v>60.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>26.13</v>
+        <v>34.44</v>
       </c>
       <c r="D8" t="n">
-        <v>2.36</v>
+        <v>1.92</v>
       </c>
       <c r="E8" t="n">
-        <v>64</v>
+        <v>53.8</v>
       </c>
       <c r="F8" t="n">
-        <v>66</v>
+        <v>53.8</v>
       </c>
       <c r="G8" t="n">
-        <v>65</v>
+        <v>53.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>34.63</v>
+        <v>37.13</v>
       </c>
       <c r="D9" t="n">
-        <v>1.93</v>
+        <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>60</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>60</v>
+        <v>38.5</v>
       </c>
       <c r="G9" t="n">
-        <v>60</v>
+        <v>51.9</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>52.75</v>
+        <v>11.77</v>
       </c>
       <c r="D10" t="n">
-        <v>4.35</v>
+        <v>0.76</v>
       </c>
       <c r="E10" t="n">
-        <v>60</v>
+        <v>53.8</v>
       </c>
       <c r="F10" t="n">
-        <v>44</v>
+        <v>48.1</v>
       </c>
       <c r="G10" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>12.94</v>
+        <v>15.15</v>
       </c>
       <c r="D11" t="n">
-        <v>1.16</v>
+        <v>1.43</v>
       </c>
       <c r="E11" t="n">
-        <v>40</v>
+        <v>46.2</v>
       </c>
       <c r="F11" t="n">
-        <v>56</v>
+        <v>46.2</v>
       </c>
       <c r="G11" t="n">
-        <v>48</v>
+        <v>46.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15.1</v>
+        <v>18.72</v>
       </c>
       <c r="D12" t="n">
-        <v>1.42</v>
+        <v>1.71</v>
       </c>
       <c r="E12" t="n">
-        <v>40</v>
+        <v>46.2</v>
       </c>
       <c r="F12" t="n">
-        <v>36</v>
+        <v>46.2</v>
       </c>
       <c r="G12" t="n">
-        <v>38</v>
+        <v>46.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>65.84999999999999</v>
+        <v>130.06</v>
       </c>
       <c r="D13" t="n">
-        <v>4.28</v>
+        <v>4.88</v>
       </c>
       <c r="E13" t="n">
-        <v>32</v>
+        <v>30.8</v>
       </c>
       <c r="F13" t="n">
-        <v>44</v>
+        <v>36.5</v>
       </c>
       <c r="G13" t="n">
-        <v>38</v>
+        <v>33.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>130.12</v>
+        <v>23.87</v>
       </c>
       <c r="D14" t="n">
-        <v>4.88</v>
+        <v>1.75</v>
       </c>
       <c r="E14" t="n">
-        <v>36</v>
+        <v>15.4</v>
       </c>
       <c r="F14" t="n">
-        <v>36</v>
+        <v>46.2</v>
       </c>
       <c r="G14" t="n">
-        <v>36</v>
+        <v>30.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>11.86</v>
+        <v>12.51</v>
       </c>
       <c r="D15" t="n">
-        <v>0.75</v>
+        <v>1.13</v>
       </c>
       <c r="E15" t="n">
-        <v>64</v>
+        <v>11.5</v>
       </c>
       <c r="F15" t="n">
-        <v>22</v>
+        <v>23.1</v>
       </c>
       <c r="G15" t="n">
-        <v>34.6</v>
+        <v>19.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>36.97</v>
+        <v>20.89</v>
       </c>
       <c r="D16" t="n">
-        <v>3.98</v>
+        <v>3.64</v>
       </c>
       <c r="E16" t="n">
-        <v>60</v>
+        <v>53.8</v>
       </c>
       <c r="F16" t="n">
-        <v>16</v>
+        <v>3.8</v>
       </c>
       <c r="G16" t="n">
-        <v>29.2</v>
+        <v>18.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.86</v>
+        <v>26.65</v>
       </c>
       <c r="D17" t="n">
-        <v>1.75</v>
+        <v>2.46</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>26.9</v>
       </c>
       <c r="F17" t="n">
-        <v>46</v>
+        <v>13.5</v>
       </c>
       <c r="G17" t="n">
-        <v>27</v>
+        <v>17.5</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>18.45</v>
+        <v>25.59</v>
       </c>
       <c r="D18" t="n">
-        <v>1.69</v>
+        <v>2.31</v>
       </c>
       <c r="E18" t="n">
-        <v>24</v>
+        <v>30.8</v>
       </c>
       <c r="F18" t="n">
-        <v>26</v>
+        <v>9.6</v>
       </c>
       <c r="G18" t="n">
-        <v>25.4</v>
+        <v>16</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="19">
@@ -996,352 +996,352 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>21.7</v>
+        <v>21.47</v>
       </c>
       <c r="D19" t="n">
-        <v>1.82</v>
+        <v>1.8</v>
       </c>
       <c r="E19" t="n">
-        <v>28</v>
+        <v>23.1</v>
       </c>
       <c r="F19" t="n">
-        <v>24</v>
+        <v>7.7</v>
       </c>
       <c r="G19" t="n">
-        <v>25.2</v>
+        <v>12.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>21.04</v>
+        <v>6.75</v>
       </c>
       <c r="D20" t="n">
-        <v>3.65</v>
+        <v>0.64</v>
       </c>
       <c r="E20" t="n">
-        <v>60</v>
+        <v>3.8</v>
       </c>
       <c r="F20" t="n">
-        <v>8</v>
+        <v>11.5</v>
       </c>
       <c r="G20" t="n">
-        <v>23.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>31.02</v>
+        <v>65.54000000000001</v>
       </c>
       <c r="D21" t="n">
-        <v>2.3</v>
+        <v>4.26</v>
       </c>
       <c r="E21" t="n">
-        <v>12</v>
+        <v>3.8</v>
       </c>
       <c r="F21" t="n">
-        <v>14</v>
+        <v>11.5</v>
       </c>
       <c r="G21" t="n">
-        <v>13.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>15.46</v>
+        <v>28.58</v>
       </c>
       <c r="D22" t="n">
-        <v>1.26</v>
+        <v>2.63</v>
       </c>
       <c r="E22" t="n">
-        <v>16</v>
+        <v>7.7</v>
       </c>
       <c r="F22" t="n">
-        <v>12</v>
+        <v>7.7</v>
       </c>
       <c r="G22" t="n">
-        <v>13.2</v>
+        <v>7.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>28.12</v>
+        <v>22.05</v>
       </c>
       <c r="D23" t="n">
-        <v>2.3</v>
+        <v>3.73</v>
       </c>
       <c r="E23" t="n">
-        <v>16</v>
+        <v>3.8</v>
       </c>
       <c r="F23" t="n">
-        <v>12</v>
+        <v>7.7</v>
       </c>
       <c r="G23" t="n">
-        <v>13.2</v>
+        <v>6.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>28.66</v>
+        <v>25.17</v>
       </c>
       <c r="D24" t="n">
-        <v>2.63</v>
+        <v>2.07</v>
       </c>
       <c r="E24" t="n">
-        <v>12</v>
+        <v>3.8</v>
       </c>
       <c r="F24" t="n">
-        <v>12</v>
+        <v>7.7</v>
       </c>
       <c r="G24" t="n">
-        <v>12</v>
+        <v>6.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29.11</v>
+        <v>27.89</v>
       </c>
       <c r="D25" t="n">
-        <v>2.68</v>
+        <v>2.28</v>
       </c>
       <c r="E25" t="n">
-        <v>12</v>
+        <v>7.7</v>
       </c>
       <c r="F25" t="n">
-        <v>12</v>
+        <v>3.8</v>
       </c>
       <c r="G25" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>22.29</v>
+        <v>31.31</v>
       </c>
       <c r="D26" t="n">
-        <v>3.77</v>
+        <v>2.63</v>
       </c>
       <c r="E26" t="n">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="F26" t="n">
-        <v>12</v>
+        <v>3.8</v>
       </c>
       <c r="G26" t="n">
-        <v>10.8</v>
+        <v>5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25.33</v>
+        <v>30.3</v>
       </c>
       <c r="D27" t="n">
-        <v>2.08</v>
+        <v>2.25</v>
       </c>
       <c r="E27" t="n">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="F27" t="n">
-        <v>12</v>
+        <v>3.8</v>
       </c>
       <c r="G27" t="n">
-        <v>10.8</v>
+        <v>5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6.8</v>
+        <v>18.7</v>
       </c>
       <c r="D28" t="n">
-        <v>0.64</v>
+        <v>1.04</v>
       </c>
       <c r="E28" t="n">
-        <v>12</v>
+        <v>3.8</v>
       </c>
       <c r="F28" t="n">
-        <v>10</v>
+        <v>3.8</v>
       </c>
       <c r="G28" t="n">
-        <v>10.6</v>
+        <v>3.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>31.79</v>
+        <v>15.33</v>
       </c>
       <c r="D29" t="n">
-        <v>2.66</v>
+        <v>1.25</v>
       </c>
       <c r="E29" t="n">
-        <v>12</v>
+        <v>3.8</v>
       </c>
       <c r="F29" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="G29" t="n">
-        <v>9.199999999999999</v>
+        <v>3.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.03</v>
+        <v>28.38</v>
       </c>
       <c r="D30" t="n">
-        <v>1.06</v>
+        <v>2.61</v>
       </c>
       <c r="E30" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="F30" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="G30" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>33.53</v>
+        <v>33.33</v>
       </c>
       <c r="D31" t="n">
-        <v>2.55</v>
+        <v>2.54</v>
       </c>
       <c r="E31" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="F31" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="G31" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>10.14</v>
+        <v>10.06</v>
       </c>
       <c r="D32" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="E32" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="F32" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="G32" t="n">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue May 19 12:31:23 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>32.19</v>
+        <v>21.24</v>
       </c>
       <c r="D2" t="n">
-        <v>3.05</v>
+        <v>1.98</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,817 +501,817 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>69.53</v>
+        <v>32.27</v>
       </c>
       <c r="D3" t="n">
-        <v>7.19</v>
+        <v>3.06</v>
       </c>
       <c r="E3" t="n">
-        <v>96.2</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>96.2</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>96.2</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>16.7</v>
+        <v>41.98</v>
       </c>
       <c r="D4" t="n">
-        <v>2.47</v>
+        <v>3.55</v>
       </c>
       <c r="E4" t="n">
-        <v>90.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>90.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>90.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>41.47</v>
+        <v>70.66</v>
       </c>
       <c r="D5" t="n">
-        <v>3.5</v>
+        <v>7.3</v>
       </c>
       <c r="E5" t="n">
-        <v>92.3</v>
+        <v>96.3</v>
       </c>
       <c r="F5" t="n">
-        <v>86.5</v>
+        <v>96.3</v>
       </c>
       <c r="G5" t="n">
-        <v>89.40000000000001</v>
+        <v>96.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>20.63</v>
+        <v>54.1</v>
       </c>
       <c r="D6" t="n">
-        <v>1.93</v>
+        <v>4.46</v>
       </c>
       <c r="E6" t="n">
-        <v>88.5</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>90.40000000000001</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>89.40000000000001</v>
+        <v>75</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>53.16</v>
+        <v>37.41</v>
       </c>
       <c r="D7" t="n">
-        <v>4.38</v>
+        <v>4.03</v>
       </c>
       <c r="E7" t="n">
-        <v>65.40000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>55.8</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>60.6</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>34.44</v>
+        <v>132.1</v>
       </c>
       <c r="D8" t="n">
-        <v>1.92</v>
+        <v>4.96</v>
       </c>
       <c r="E8" t="n">
-        <v>53.8</v>
+        <v>66.7</v>
       </c>
       <c r="F8" t="n">
-        <v>53.8</v>
+        <v>66.7</v>
       </c>
       <c r="G8" t="n">
-        <v>53.8</v>
+        <v>66.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>37.13</v>
+        <v>16.59</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>2.45</v>
       </c>
       <c r="E9" t="n">
-        <v>65.40000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>38.5</v>
+        <v>48.1</v>
       </c>
       <c r="G9" t="n">
-        <v>51.9</v>
+        <v>59.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>11.77</v>
+        <v>34.61</v>
       </c>
       <c r="D10" t="n">
-        <v>0.76</v>
+        <v>1.93</v>
       </c>
       <c r="E10" t="n">
-        <v>53.8</v>
+        <v>55.6</v>
       </c>
       <c r="F10" t="n">
-        <v>48.1</v>
+        <v>61.1</v>
       </c>
       <c r="G10" t="n">
-        <v>51</v>
+        <v>58.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>15.15</v>
+        <v>24.04</v>
       </c>
       <c r="D11" t="n">
-        <v>1.43</v>
+        <v>1.77</v>
       </c>
       <c r="E11" t="n">
-        <v>46.2</v>
+        <v>40.7</v>
       </c>
       <c r="F11" t="n">
-        <v>46.2</v>
+        <v>66.7</v>
       </c>
       <c r="G11" t="n">
-        <v>46.2</v>
+        <v>53.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>18.72</v>
+        <v>11.84</v>
       </c>
       <c r="D12" t="n">
-        <v>1.71</v>
+        <v>0.76</v>
       </c>
       <c r="E12" t="n">
-        <v>46.2</v>
+        <v>59.3</v>
       </c>
       <c r="F12" t="n">
-        <v>46.2</v>
+        <v>48.1</v>
       </c>
       <c r="G12" t="n">
-        <v>46.2</v>
+        <v>53.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>130.06</v>
+        <v>18.73</v>
       </c>
       <c r="D13" t="n">
-        <v>4.88</v>
+        <v>1.71</v>
       </c>
       <c r="E13" t="n">
-        <v>30.8</v>
+        <v>48.1</v>
       </c>
       <c r="F13" t="n">
-        <v>36.5</v>
+        <v>46.3</v>
       </c>
       <c r="G13" t="n">
-        <v>33.7</v>
+        <v>47.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>23.87</v>
+        <v>15.14</v>
       </c>
       <c r="D14" t="n">
-        <v>1.75</v>
+        <v>1.42</v>
       </c>
       <c r="E14" t="n">
-        <v>15.4</v>
+        <v>44.4</v>
       </c>
       <c r="F14" t="n">
-        <v>46.2</v>
+        <v>35.2</v>
       </c>
       <c r="G14" t="n">
-        <v>30.8</v>
+        <v>39.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>12.51</v>
+        <v>28.21</v>
       </c>
       <c r="D15" t="n">
-        <v>1.13</v>
+        <v>2.31</v>
       </c>
       <c r="E15" t="n">
-        <v>11.5</v>
+        <v>25.9</v>
       </c>
       <c r="F15" t="n">
-        <v>23.1</v>
+        <v>35.2</v>
       </c>
       <c r="G15" t="n">
-        <v>19.6</v>
+        <v>30.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>20.89</v>
+        <v>26.76</v>
       </c>
       <c r="D16" t="n">
-        <v>3.64</v>
+        <v>2.47</v>
       </c>
       <c r="E16" t="n">
-        <v>53.8</v>
+        <v>51.9</v>
       </c>
       <c r="F16" t="n">
-        <v>3.8</v>
+        <v>18.5</v>
       </c>
       <c r="G16" t="n">
-        <v>18.8</v>
+        <v>28.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>26.65</v>
+        <v>6.79</v>
       </c>
       <c r="D17" t="n">
-        <v>2.46</v>
+        <v>0.65</v>
       </c>
       <c r="E17" t="n">
-        <v>26.9</v>
+        <v>11.1</v>
       </c>
       <c r="F17" t="n">
-        <v>13.5</v>
+        <v>37</v>
       </c>
       <c r="G17" t="n">
-        <v>17.5</v>
+        <v>24.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>25.59</v>
+        <v>12.63</v>
       </c>
       <c r="D18" t="n">
-        <v>2.31</v>
+        <v>1.14</v>
       </c>
       <c r="E18" t="n">
-        <v>30.8</v>
+        <v>14.8</v>
       </c>
       <c r="F18" t="n">
-        <v>9.6</v>
+        <v>25.9</v>
       </c>
       <c r="G18" t="n">
-        <v>16</v>
+        <v>22.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>21.47</v>
+        <v>15.48</v>
       </c>
       <c r="D19" t="n">
-        <v>1.8</v>
+        <v>1.26</v>
       </c>
       <c r="E19" t="n">
-        <v>23.1</v>
+        <v>33.3</v>
       </c>
       <c r="F19" t="n">
-        <v>7.7</v>
+        <v>16.7</v>
       </c>
       <c r="G19" t="n">
-        <v>12.3</v>
+        <v>21.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6.75</v>
+        <v>25.53</v>
       </c>
       <c r="D20" t="n">
-        <v>0.64</v>
+        <v>2.1</v>
       </c>
       <c r="E20" t="n">
-        <v>3.8</v>
+        <v>18.5</v>
       </c>
       <c r="F20" t="n">
-        <v>11.5</v>
+        <v>22.2</v>
       </c>
       <c r="G20" t="n">
-        <v>9.199999999999999</v>
+        <v>21.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>65.54000000000001</v>
+        <v>20.91</v>
       </c>
       <c r="D21" t="n">
-        <v>4.26</v>
+        <v>3.64</v>
       </c>
       <c r="E21" t="n">
-        <v>3.8</v>
+        <v>55.6</v>
       </c>
       <c r="F21" t="n">
-        <v>11.5</v>
+        <v>5.6</v>
       </c>
       <c r="G21" t="n">
-        <v>9.199999999999999</v>
+        <v>20.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28.58</v>
+        <v>25.76</v>
       </c>
       <c r="D22" t="n">
-        <v>2.63</v>
+        <v>2.33</v>
       </c>
       <c r="E22" t="n">
-        <v>7.7</v>
+        <v>33.3</v>
       </c>
       <c r="F22" t="n">
-        <v>7.7</v>
+        <v>14.8</v>
       </c>
       <c r="G22" t="n">
-        <v>7.7</v>
+        <v>20.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22.05</v>
+        <v>21.55</v>
       </c>
       <c r="D23" t="n">
-        <v>3.73</v>
+        <v>1.81</v>
       </c>
       <c r="E23" t="n">
-        <v>3.8</v>
+        <v>25.9</v>
       </c>
       <c r="F23" t="n">
-        <v>7.7</v>
+        <v>11.1</v>
       </c>
       <c r="G23" t="n">
-        <v>6.5</v>
+        <v>15.6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>25.17</v>
+        <v>33.52</v>
       </c>
       <c r="D24" t="n">
-        <v>2.07</v>
+        <v>2.55</v>
       </c>
       <c r="E24" t="n">
-        <v>3.8</v>
+        <v>7.4</v>
       </c>
       <c r="F24" t="n">
-        <v>7.7</v>
+        <v>13</v>
       </c>
       <c r="G24" t="n">
-        <v>6.5</v>
+        <v>11.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>27.89</v>
+        <v>10.12</v>
       </c>
       <c r="D25" t="n">
-        <v>2.28</v>
+        <v>1.23</v>
       </c>
       <c r="E25" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="F25" t="n">
-        <v>3.8</v>
+        <v>13</v>
       </c>
       <c r="G25" t="n">
-        <v>5</v>
+        <v>11.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>31.31</v>
+        <v>28.73</v>
       </c>
       <c r="D26" t="n">
-        <v>2.63</v>
+        <v>2.64</v>
       </c>
       <c r="E26" t="n">
-        <v>7.7</v>
+        <v>11.1</v>
       </c>
       <c r="F26" t="n">
-        <v>3.8</v>
+        <v>11.1</v>
       </c>
       <c r="G26" t="n">
-        <v>5</v>
+        <v>11.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>30.3</v>
+        <v>65.39</v>
       </c>
       <c r="D27" t="n">
-        <v>2.25</v>
+        <v>4.25</v>
       </c>
       <c r="E27" t="n">
-        <v>7.7</v>
+        <v>3.7</v>
       </c>
       <c r="F27" t="n">
-        <v>3.8</v>
+        <v>7.4</v>
       </c>
       <c r="G27" t="n">
-        <v>5</v>
+        <v>6.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18.7</v>
+        <v>30.18</v>
       </c>
       <c r="D28" t="n">
-        <v>1.04</v>
+        <v>2.24</v>
       </c>
       <c r="E28" t="n">
-        <v>3.8</v>
+        <v>7.4</v>
       </c>
       <c r="F28" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="G28" t="n">
-        <v>3.8</v>
+        <v>4.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>15.33</v>
+        <v>18.6</v>
       </c>
       <c r="D29" t="n">
-        <v>1.25</v>
+        <v>1.03</v>
       </c>
       <c r="E29" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="F29" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="G29" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="30">
@@ -1326,82 +1326,82 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>28.38</v>
+        <v>28.2</v>
       </c>
       <c r="D30" t="n">
-        <v>2.61</v>
+        <v>2.59</v>
       </c>
       <c r="E30" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="F30" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="G30" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>33.33</v>
+        <v>21.81</v>
       </c>
       <c r="D31" t="n">
-        <v>2.54</v>
+        <v>3.69</v>
       </c>
       <c r="E31" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="F31" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="G31" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>10.06</v>
+        <v>31.12</v>
       </c>
       <c r="D32" t="n">
-        <v>1.22</v>
+        <v>2.61</v>
       </c>
       <c r="E32" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="F32" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="G32" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed May 20 12:12:07 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>21.24</v>
+        <v>72.52</v>
       </c>
       <c r="D2" t="n">
-        <v>1.98</v>
+        <v>7.5</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,25 +501,25 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>32.27</v>
+        <v>42.24</v>
       </c>
       <c r="D3" t="n">
-        <v>3.06</v>
+        <v>3.57</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -531,157 +531,157 @@
         <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>41.98</v>
+        <v>31.96</v>
       </c>
       <c r="D4" t="n">
-        <v>3.55</v>
+        <v>3.03</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>85.7</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>70.66</v>
+        <v>37.75</v>
       </c>
       <c r="D5" t="n">
-        <v>7.3</v>
+        <v>4.07</v>
       </c>
       <c r="E5" t="n">
-        <v>96.3</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>96.3</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>96.3</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>54.1</v>
+        <v>132.53</v>
       </c>
       <c r="D6" t="n">
-        <v>4.46</v>
+        <v>4.97</v>
       </c>
       <c r="E6" t="n">
-        <v>74.09999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>75.90000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>75</v>
+        <v>70.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>37.41</v>
+        <v>34.95</v>
       </c>
       <c r="D7" t="n">
-        <v>4.03</v>
+        <v>1.95</v>
       </c>
       <c r="E7" t="n">
-        <v>70.40000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>70.40000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>70.40000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>132.1</v>
+        <v>53.27</v>
       </c>
       <c r="D8" t="n">
-        <v>4.96</v>
+        <v>4.43</v>
       </c>
       <c r="E8" t="n">
-        <v>66.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>66.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>66.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="9">
@@ -696,112 +696,112 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>16.59</v>
+        <v>16.58</v>
       </c>
       <c r="D9" t="n">
-        <v>2.45</v>
+        <v>2.46</v>
       </c>
       <c r="E9" t="n">
-        <v>70.40000000000001</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>48.1</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>59.3</v>
+        <v>67</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>34.61</v>
+        <v>20.39</v>
       </c>
       <c r="D10" t="n">
-        <v>1.93</v>
+        <v>1.9</v>
       </c>
       <c r="E10" t="n">
-        <v>55.6</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>61.1</v>
+        <v>64.3</v>
       </c>
       <c r="G10" t="n">
-        <v>58.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>24.04</v>
+        <v>15.25</v>
       </c>
       <c r="D11" t="n">
-        <v>1.77</v>
+        <v>1.44</v>
       </c>
       <c r="E11" t="n">
-        <v>40.7</v>
+        <v>50</v>
       </c>
       <c r="F11" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="G11" t="n">
-        <v>53.7</v>
+        <v>50</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>11.84</v>
+        <v>15.49</v>
       </c>
       <c r="D12" t="n">
-        <v>0.76</v>
+        <v>1.27</v>
       </c>
       <c r="E12" t="n">
-        <v>59.3</v>
+        <v>35.7</v>
       </c>
       <c r="F12" t="n">
-        <v>48.1</v>
+        <v>44.6</v>
       </c>
       <c r="G12" t="n">
-        <v>53.7</v>
+        <v>40.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="13">
@@ -816,442 +816,442 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>18.73</v>
+        <v>18.58</v>
       </c>
       <c r="D13" t="n">
-        <v>1.71</v>
+        <v>1.7</v>
       </c>
       <c r="E13" t="n">
-        <v>48.1</v>
+        <v>35.7</v>
       </c>
       <c r="F13" t="n">
-        <v>46.3</v>
+        <v>39.3</v>
       </c>
       <c r="G13" t="n">
-        <v>47.2</v>
+        <v>37.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.14</v>
+        <v>23.82</v>
       </c>
       <c r="D14" t="n">
-        <v>1.42</v>
+        <v>1.75</v>
       </c>
       <c r="E14" t="n">
-        <v>44.4</v>
+        <v>3.6</v>
       </c>
       <c r="F14" t="n">
-        <v>35.2</v>
+        <v>44.6</v>
       </c>
       <c r="G14" t="n">
-        <v>39.8</v>
+        <v>24.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>28.21</v>
+        <v>11.7</v>
       </c>
       <c r="D15" t="n">
-        <v>2.31</v>
+        <v>0.75</v>
       </c>
       <c r="E15" t="n">
-        <v>25.9</v>
+        <v>28.6</v>
       </c>
       <c r="F15" t="n">
-        <v>35.2</v>
+        <v>21.4</v>
       </c>
       <c r="G15" t="n">
-        <v>30.6</v>
+        <v>23.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26.76</v>
+        <v>12.43</v>
       </c>
       <c r="D16" t="n">
-        <v>2.47</v>
+        <v>1.13</v>
       </c>
       <c r="E16" t="n">
-        <v>51.9</v>
+        <v>10.7</v>
       </c>
       <c r="F16" t="n">
-        <v>18.5</v>
+        <v>23.2</v>
       </c>
       <c r="G16" t="n">
-        <v>28.5</v>
+        <v>19.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6.79</v>
+        <v>25.58</v>
       </c>
       <c r="D17" t="n">
-        <v>0.65</v>
+        <v>2.32</v>
       </c>
       <c r="E17" t="n">
-        <v>11.1</v>
+        <v>28.6</v>
       </c>
       <c r="F17" t="n">
-        <v>37</v>
+        <v>14.3</v>
       </c>
       <c r="G17" t="n">
-        <v>24.1</v>
+        <v>18.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>12.63</v>
+        <v>20.88</v>
       </c>
       <c r="D18" t="n">
-        <v>1.14</v>
+        <v>3.63</v>
       </c>
       <c r="E18" t="n">
-        <v>14.8</v>
+        <v>50</v>
       </c>
       <c r="F18" t="n">
-        <v>25.9</v>
+        <v>3.6</v>
       </c>
       <c r="G18" t="n">
-        <v>22.6</v>
+        <v>17.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15.48</v>
+        <v>21.39</v>
       </c>
       <c r="D19" t="n">
-        <v>1.26</v>
+        <v>1.8</v>
       </c>
       <c r="E19" t="n">
-        <v>33.3</v>
+        <v>21.4</v>
       </c>
       <c r="F19" t="n">
-        <v>16.7</v>
+        <v>8.9</v>
       </c>
       <c r="G19" t="n">
-        <v>21.7</v>
+        <v>12.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>25.53</v>
+        <v>26.38</v>
       </c>
       <c r="D20" t="n">
-        <v>2.1</v>
+        <v>2.44</v>
       </c>
       <c r="E20" t="n">
-        <v>18.5</v>
+        <v>25</v>
       </c>
       <c r="F20" t="n">
-        <v>22.2</v>
+        <v>5.4</v>
       </c>
       <c r="G20" t="n">
-        <v>21.1</v>
+        <v>11.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20.91</v>
+        <v>6.7</v>
       </c>
       <c r="D21" t="n">
-        <v>3.64</v>
+        <v>0.64</v>
       </c>
       <c r="E21" t="n">
-        <v>55.6</v>
+        <v>3.6</v>
       </c>
       <c r="F21" t="n">
-        <v>5.6</v>
+        <v>12.5</v>
       </c>
       <c r="G21" t="n">
-        <v>20.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>25.76</v>
+        <v>28.58</v>
       </c>
       <c r="D22" t="n">
-        <v>2.33</v>
+        <v>2.63</v>
       </c>
       <c r="E22" t="n">
-        <v>33.3</v>
+        <v>8.9</v>
       </c>
       <c r="F22" t="n">
-        <v>14.8</v>
+        <v>8.9</v>
       </c>
       <c r="G22" t="n">
-        <v>20.4</v>
+        <v>8.9</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>21.55</v>
+        <v>21.81</v>
       </c>
       <c r="D23" t="n">
-        <v>1.81</v>
+        <v>3.7</v>
       </c>
       <c r="E23" t="n">
-        <v>25.9</v>
+        <v>5.4</v>
       </c>
       <c r="F23" t="n">
-        <v>11.1</v>
+        <v>8.9</v>
       </c>
       <c r="G23" t="n">
-        <v>15.6</v>
+        <v>7.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>33.52</v>
+        <v>25.15</v>
       </c>
       <c r="D24" t="n">
-        <v>2.55</v>
+        <v>2.07</v>
       </c>
       <c r="E24" t="n">
-        <v>7.4</v>
+        <v>3.6</v>
       </c>
       <c r="F24" t="n">
-        <v>13</v>
+        <v>8.9</v>
       </c>
       <c r="G24" t="n">
-        <v>11.3</v>
+        <v>7.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10.12</v>
+        <v>28.35</v>
       </c>
       <c r="D25" t="n">
-        <v>1.23</v>
+        <v>2.6</v>
       </c>
       <c r="E25" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="F25" t="n">
-        <v>13</v>
+        <v>7.1</v>
       </c>
       <c r="G25" t="n">
-        <v>11.3</v>
+        <v>7.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>28.73</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="D26" t="n">
-        <v>2.64</v>
+        <v>4.23</v>
       </c>
       <c r="E26" t="n">
-        <v>11.1</v>
+        <v>3.6</v>
       </c>
       <c r="F26" t="n">
-        <v>11.1</v>
+        <v>7.1</v>
       </c>
       <c r="G26" t="n">
-        <v>11.1</v>
+        <v>6.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>65.39</v>
+        <v>10.06</v>
       </c>
       <c r="D27" t="n">
-        <v>4.25</v>
+        <v>1.22</v>
       </c>
       <c r="E27" t="n">
-        <v>3.7</v>
+        <v>5.4</v>
       </c>
       <c r="F27" t="n">
-        <v>7.4</v>
+        <v>5.4</v>
       </c>
       <c r="G27" t="n">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="28">
@@ -1266,112 +1266,112 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>30.18</v>
+        <v>29.83</v>
       </c>
       <c r="D28" t="n">
-        <v>2.24</v>
+        <v>2.21</v>
       </c>
       <c r="E28" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="F28" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="G28" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.6</v>
+        <v>27.66</v>
       </c>
       <c r="D29" t="n">
-        <v>1.03</v>
+        <v>2.26</v>
       </c>
       <c r="E29" t="n">
-        <v>3.7</v>
+        <v>7.1</v>
       </c>
       <c r="F29" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="G29" t="n">
-        <v>3.7</v>
+        <v>4.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>28.2</v>
+        <v>18.43</v>
       </c>
       <c r="D30" t="n">
-        <v>2.59</v>
+        <v>1.02</v>
       </c>
       <c r="E30" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="F30" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="G30" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>21.81</v>
+        <v>33.07</v>
       </c>
       <c r="D31" t="n">
-        <v>3.69</v>
+        <v>2.52</v>
       </c>
       <c r="E31" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="F31" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="G31" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>31.12</v>
+        <v>30.83</v>
       </c>
       <c r="D32" t="n">
-        <v>2.61</v>
+        <v>2.59</v>
       </c>
       <c r="E32" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="F32" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="G32" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu May 21 12:35:33 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>72.52</v>
+        <v>69.89</v>
       </c>
       <c r="D2" t="n">
-        <v>7.5</v>
+        <v>7.23</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>89.7</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>89.7</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>89.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42.24</v>
+        <v>41.44</v>
       </c>
       <c r="D3" t="n">
-        <v>3.57</v>
+        <v>3.5</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>82.8</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>79.3</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="4">
@@ -546,832 +546,832 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>31.96</v>
+        <v>30.51</v>
       </c>
       <c r="D4" t="n">
-        <v>3.03</v>
+        <v>2.89</v>
       </c>
       <c r="E4" t="n">
-        <v>85.7</v>
+        <v>65.5</v>
       </c>
       <c r="F4" t="n">
-        <v>87.5</v>
+        <v>65.5</v>
       </c>
       <c r="G4" t="n">
-        <v>86.59999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>37.75</v>
+        <v>34.55</v>
       </c>
       <c r="D5" t="n">
-        <v>4.07</v>
+        <v>1.92</v>
       </c>
       <c r="E5" t="n">
-        <v>82.09999999999999</v>
+        <v>51.7</v>
       </c>
       <c r="F5" t="n">
-        <v>78.59999999999999</v>
+        <v>50</v>
       </c>
       <c r="G5" t="n">
-        <v>80.40000000000001</v>
+        <v>50.9</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>132.53</v>
+        <v>16.51</v>
       </c>
       <c r="D6" t="n">
-        <v>4.97</v>
+        <v>2.44</v>
       </c>
       <c r="E6" t="n">
-        <v>71.40000000000001</v>
+        <v>58.6</v>
       </c>
       <c r="F6" t="n">
-        <v>69.59999999999999</v>
+        <v>37.9</v>
       </c>
       <c r="G6" t="n">
-        <v>70.5</v>
+        <v>48.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>34.95</v>
+        <v>20.01</v>
       </c>
       <c r="D7" t="n">
-        <v>1.95</v>
+        <v>1.87</v>
       </c>
       <c r="E7" t="n">
-        <v>67.90000000000001</v>
+        <v>51.7</v>
       </c>
       <c r="F7" t="n">
-        <v>67.90000000000001</v>
+        <v>29.3</v>
       </c>
       <c r="G7" t="n">
-        <v>67.90000000000001</v>
+        <v>36</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>53.27</v>
+        <v>125.52</v>
       </c>
       <c r="D8" t="n">
-        <v>4.43</v>
+        <v>4.71</v>
       </c>
       <c r="E8" t="n">
-        <v>67.90000000000001</v>
+        <v>27.6</v>
       </c>
       <c r="F8" t="n">
-        <v>67.90000000000001</v>
+        <v>27.6</v>
       </c>
       <c r="G8" t="n">
-        <v>67.90000000000001</v>
+        <v>27.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>16.58</v>
+        <v>15.46</v>
       </c>
       <c r="D9" t="n">
-        <v>2.46</v>
+        <v>1.26</v>
       </c>
       <c r="E9" t="n">
-        <v>66.09999999999999</v>
+        <v>19</v>
       </c>
       <c r="F9" t="n">
-        <v>67.90000000000001</v>
+        <v>17.2</v>
       </c>
       <c r="G9" t="n">
-        <v>67</v>
+        <v>17.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>20.39</v>
+        <v>12.04</v>
       </c>
       <c r="D10" t="n">
-        <v>1.9</v>
+        <v>1.09</v>
       </c>
       <c r="E10" t="n">
-        <v>67.90000000000001</v>
+        <v>10.3</v>
       </c>
       <c r="F10" t="n">
-        <v>64.3</v>
+        <v>20.7</v>
       </c>
       <c r="G10" t="n">
-        <v>66.09999999999999</v>
+        <v>17.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>15.25</v>
+        <v>26.47</v>
       </c>
       <c r="D11" t="n">
-        <v>1.44</v>
+        <v>2.45</v>
       </c>
       <c r="E11" t="n">
-        <v>50</v>
+        <v>27.6</v>
       </c>
       <c r="F11" t="n">
-        <v>50</v>
+        <v>12.1</v>
       </c>
       <c r="G11" t="n">
-        <v>50</v>
+        <v>16.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15.49</v>
+        <v>36.61</v>
       </c>
       <c r="D12" t="n">
-        <v>1.27</v>
+        <v>3.95</v>
       </c>
       <c r="E12" t="n">
-        <v>35.7</v>
+        <v>24.1</v>
       </c>
       <c r="F12" t="n">
-        <v>44.6</v>
+        <v>10.3</v>
       </c>
       <c r="G12" t="n">
-        <v>40.2</v>
+        <v>14.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>18.58</v>
+        <v>20.7</v>
       </c>
       <c r="D13" t="n">
-        <v>1.7</v>
+        <v>3.6</v>
       </c>
       <c r="E13" t="n">
-        <v>35.7</v>
+        <v>34.5</v>
       </c>
       <c r="F13" t="n">
-        <v>39.3</v>
+        <v>3.4</v>
       </c>
       <c r="G13" t="n">
-        <v>37.5</v>
+        <v>12.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>23.82</v>
+        <v>6.75</v>
       </c>
       <c r="D14" t="n">
-        <v>1.75</v>
+        <v>0.64</v>
       </c>
       <c r="E14" t="n">
-        <v>3.6</v>
+        <v>8.6</v>
       </c>
       <c r="F14" t="n">
-        <v>44.6</v>
+        <v>13.8</v>
       </c>
       <c r="G14" t="n">
-        <v>24.1</v>
+        <v>12.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>11.7</v>
+        <v>28.61</v>
       </c>
       <c r="D15" t="n">
-        <v>0.75</v>
+        <v>2.63</v>
       </c>
       <c r="E15" t="n">
-        <v>28.6</v>
+        <v>13.8</v>
       </c>
       <c r="F15" t="n">
-        <v>21.4</v>
+        <v>10.3</v>
       </c>
       <c r="G15" t="n">
-        <v>23.6</v>
+        <v>11.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>12.43</v>
+        <v>25.03</v>
       </c>
       <c r="D16" t="n">
-        <v>1.13</v>
+        <v>2.27</v>
       </c>
       <c r="E16" t="n">
-        <v>10.7</v>
+        <v>24.1</v>
       </c>
       <c r="F16" t="n">
-        <v>23.2</v>
+        <v>3.4</v>
       </c>
       <c r="G16" t="n">
-        <v>19.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25.58</v>
+        <v>11.39</v>
       </c>
       <c r="D17" t="n">
-        <v>2.32</v>
+        <v>0.73</v>
       </c>
       <c r="E17" t="n">
-        <v>28.6</v>
+        <v>19</v>
       </c>
       <c r="F17" t="n">
-        <v>14.3</v>
+        <v>3.4</v>
       </c>
       <c r="G17" t="n">
-        <v>18.6</v>
+        <v>8.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>20.88</v>
+        <v>51.48</v>
       </c>
       <c r="D18" t="n">
-        <v>3.63</v>
+        <v>4.28</v>
       </c>
       <c r="E18" t="n">
-        <v>50</v>
+        <v>10.3</v>
       </c>
       <c r="F18" t="n">
-        <v>3.6</v>
+        <v>6.9</v>
       </c>
       <c r="G18" t="n">
-        <v>17.5</v>
+        <v>7.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>21.39</v>
+        <v>63.4</v>
       </c>
       <c r="D19" t="n">
-        <v>1.8</v>
+        <v>4.12</v>
       </c>
       <c r="E19" t="n">
-        <v>21.4</v>
+        <v>3.4</v>
       </c>
       <c r="F19" t="n">
-        <v>8.9</v>
+        <v>6.9</v>
       </c>
       <c r="G19" t="n">
-        <v>12.7</v>
+        <v>5.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>26.38</v>
+        <v>10.01</v>
       </c>
       <c r="D20" t="n">
-        <v>2.44</v>
+        <v>1.22</v>
       </c>
       <c r="E20" t="n">
-        <v>25</v>
+        <v>3.4</v>
       </c>
       <c r="F20" t="n">
-        <v>5.4</v>
+        <v>6.9</v>
       </c>
       <c r="G20" t="n">
-        <v>11.2</v>
+        <v>5.9</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>6.7</v>
+        <v>18.08</v>
       </c>
       <c r="D21" t="n">
-        <v>0.64</v>
+        <v>1.66</v>
       </c>
       <c r="E21" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="F21" t="n">
-        <v>12.5</v>
+        <v>6.9</v>
       </c>
       <c r="G21" t="n">
-        <v>9.800000000000001</v>
+        <v>5.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28.58</v>
+        <v>20.96</v>
       </c>
       <c r="D22" t="n">
-        <v>2.63</v>
+        <v>1.76</v>
       </c>
       <c r="E22" t="n">
-        <v>8.9</v>
+        <v>6.9</v>
       </c>
       <c r="F22" t="n">
-        <v>8.9</v>
+        <v>5.2</v>
       </c>
       <c r="G22" t="n">
-        <v>8.9</v>
+        <v>5.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>21.81</v>
+        <v>29.26</v>
       </c>
       <c r="D23" t="n">
-        <v>3.7</v>
+        <v>2.17</v>
       </c>
       <c r="E23" t="n">
-        <v>5.4</v>
+        <v>6.9</v>
       </c>
       <c r="F23" t="n">
-        <v>8.9</v>
+        <v>3.4</v>
       </c>
       <c r="G23" t="n">
-        <v>7.9</v>
+        <v>4.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>25.15</v>
+        <v>26.94</v>
       </c>
       <c r="D24" t="n">
-        <v>2.07</v>
+        <v>2.21</v>
       </c>
       <c r="E24" t="n">
-        <v>3.6</v>
+        <v>6.9</v>
       </c>
       <c r="F24" t="n">
-        <v>8.9</v>
+        <v>3.4</v>
       </c>
       <c r="G24" t="n">
-        <v>7.3</v>
+        <v>4.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.35</v>
+        <v>24.49</v>
       </c>
       <c r="D25" t="n">
-        <v>2.6</v>
+        <v>2.01</v>
       </c>
       <c r="E25" t="n">
-        <v>7.1</v>
+        <v>3.4</v>
       </c>
       <c r="F25" t="n">
-        <v>7.1</v>
+        <v>3.4</v>
       </c>
       <c r="G25" t="n">
-        <v>7.1</v>
+        <v>3.4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>64.98999999999999</v>
+        <v>27.4</v>
       </c>
       <c r="D26" t="n">
-        <v>4.23</v>
+        <v>2.52</v>
       </c>
       <c r="E26" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="F26" t="n">
-        <v>7.1</v>
+        <v>3.4</v>
       </c>
       <c r="G26" t="n">
-        <v>6.1</v>
+        <v>3.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>10.06</v>
+        <v>18.06</v>
       </c>
       <c r="D27" t="n">
-        <v>1.22</v>
+        <v>1.01</v>
       </c>
       <c r="E27" t="n">
-        <v>5.4</v>
+        <v>3.4</v>
       </c>
       <c r="F27" t="n">
-        <v>5.4</v>
+        <v>3.4</v>
       </c>
       <c r="G27" t="n">
-        <v>5.4</v>
+        <v>3.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29.83</v>
+        <v>21.36</v>
       </c>
       <c r="D28" t="n">
-        <v>2.21</v>
+        <v>3.62</v>
       </c>
       <c r="E28" t="n">
-        <v>7.1</v>
+        <v>3.4</v>
       </c>
       <c r="F28" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="G28" t="n">
-        <v>4.6</v>
+        <v>3.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>27.66</v>
+        <v>32.52</v>
       </c>
       <c r="D29" t="n">
-        <v>2.26</v>
+        <v>2.49</v>
       </c>
       <c r="E29" t="n">
-        <v>7.1</v>
+        <v>3.4</v>
       </c>
       <c r="F29" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="G29" t="n">
-        <v>4.6</v>
+        <v>3.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>18.43</v>
+        <v>14.77</v>
       </c>
       <c r="D30" t="n">
-        <v>1.02</v>
+        <v>1.39</v>
       </c>
       <c r="E30" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="F30" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="G30" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>33.07</v>
+        <v>23.08</v>
       </c>
       <c r="D31" t="n">
-        <v>2.52</v>
+        <v>1.7</v>
       </c>
       <c r="E31" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="F31" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="G31" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>30.83</v>
+        <v>30.27</v>
       </c>
       <c r="D32" t="n">
-        <v>2.59</v>
+        <v>2.55</v>
       </c>
       <c r="E32" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="F32" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="G32" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri May 22 12:07:59 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>69.89</v>
+        <v>72.86</v>
       </c>
       <c r="D2" t="n">
-        <v>7.23</v>
+        <v>7.54</v>
       </c>
       <c r="E2" t="n">
-        <v>89.7</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>89.7</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>89.7</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="3">
@@ -516,892 +516,892 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>41.44</v>
+        <v>42.92</v>
       </c>
       <c r="D3" t="n">
-        <v>3.5</v>
+        <v>3.63</v>
       </c>
       <c r="E3" t="n">
-        <v>82.8</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>79.3</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30.51</v>
+        <v>36.39</v>
       </c>
       <c r="D4" t="n">
-        <v>2.89</v>
+        <v>2.03</v>
       </c>
       <c r="E4" t="n">
-        <v>65.5</v>
+        <v>90</v>
       </c>
       <c r="F4" t="n">
-        <v>65.5</v>
+        <v>91.7</v>
       </c>
       <c r="G4" t="n">
-        <v>65.5</v>
+        <v>90.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>34.55</v>
+        <v>31.19</v>
       </c>
       <c r="D5" t="n">
-        <v>1.92</v>
+        <v>2.95</v>
       </c>
       <c r="E5" t="n">
-        <v>51.7</v>
+        <v>70</v>
       </c>
       <c r="F5" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="G5" t="n">
-        <v>50.9</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.51</v>
+        <v>131.92</v>
       </c>
       <c r="D6" t="n">
-        <v>2.44</v>
+        <v>4.95</v>
       </c>
       <c r="E6" t="n">
-        <v>58.6</v>
+        <v>63.3</v>
       </c>
       <c r="F6" t="n">
-        <v>37.9</v>
+        <v>63.3</v>
       </c>
       <c r="G6" t="n">
-        <v>48.3</v>
+        <v>63.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.01</v>
+        <v>37.15</v>
       </c>
       <c r="D7" t="n">
-        <v>1.87</v>
+        <v>4.01</v>
       </c>
       <c r="E7" t="n">
-        <v>51.7</v>
+        <v>63.3</v>
       </c>
       <c r="F7" t="n">
-        <v>29.3</v>
+        <v>53.3</v>
       </c>
       <c r="G7" t="n">
-        <v>36</v>
+        <v>58.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>125.52</v>
+        <v>16.52</v>
       </c>
       <c r="D8" t="n">
-        <v>4.71</v>
+        <v>2.45</v>
       </c>
       <c r="E8" t="n">
-        <v>27.6</v>
+        <v>60</v>
       </c>
       <c r="F8" t="n">
-        <v>27.6</v>
+        <v>48.3</v>
       </c>
       <c r="G8" t="n">
-        <v>27.6</v>
+        <v>54.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15.46</v>
+        <v>20.05</v>
       </c>
       <c r="D9" t="n">
-        <v>1.26</v>
+        <v>1.87</v>
       </c>
       <c r="E9" t="n">
-        <v>19</v>
+        <v>53.3</v>
       </c>
       <c r="F9" t="n">
-        <v>17.2</v>
+        <v>30</v>
       </c>
       <c r="G9" t="n">
-        <v>17.8</v>
+        <v>41.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>12.04</v>
+        <v>26.7</v>
       </c>
       <c r="D10" t="n">
-        <v>1.09</v>
+        <v>2.48</v>
       </c>
       <c r="E10" t="n">
-        <v>10.3</v>
+        <v>33.3</v>
       </c>
       <c r="F10" t="n">
-        <v>20.7</v>
+        <v>45</v>
       </c>
       <c r="G10" t="n">
-        <v>17.6</v>
+        <v>39.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>26.47</v>
+        <v>52.03</v>
       </c>
       <c r="D11" t="n">
-        <v>2.45</v>
+        <v>4.33</v>
       </c>
       <c r="E11" t="n">
-        <v>27.6</v>
+        <v>30</v>
       </c>
       <c r="F11" t="n">
-        <v>12.1</v>
+        <v>33.3</v>
       </c>
       <c r="G11" t="n">
-        <v>16.7</v>
+        <v>31.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>36.61</v>
+        <v>12.14</v>
       </c>
       <c r="D12" t="n">
-        <v>3.95</v>
+        <v>1.09</v>
       </c>
       <c r="E12" t="n">
-        <v>24.1</v>
+        <v>13.3</v>
       </c>
       <c r="F12" t="n">
-        <v>10.3</v>
+        <v>21.7</v>
       </c>
       <c r="G12" t="n">
-        <v>14.5</v>
+        <v>19.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>20.7</v>
+        <v>22.11</v>
       </c>
       <c r="D13" t="n">
-        <v>3.6</v>
+        <v>3.75</v>
       </c>
       <c r="E13" t="n">
-        <v>34.5</v>
+        <v>16.7</v>
       </c>
       <c r="F13" t="n">
-        <v>3.4</v>
+        <v>20</v>
       </c>
       <c r="G13" t="n">
-        <v>12.8</v>
+        <v>19</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6.75</v>
+        <v>15.44</v>
       </c>
       <c r="D14" t="n">
-        <v>0.64</v>
+        <v>1.26</v>
       </c>
       <c r="E14" t="n">
-        <v>8.6</v>
+        <v>11.7</v>
       </c>
       <c r="F14" t="n">
-        <v>13.8</v>
+        <v>18.3</v>
       </c>
       <c r="G14" t="n">
-        <v>12.2</v>
+        <v>16.3</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>28.61</v>
+        <v>6.75</v>
       </c>
       <c r="D15" t="n">
-        <v>2.63</v>
+        <v>0.64</v>
       </c>
       <c r="E15" t="n">
-        <v>13.8</v>
+        <v>10</v>
       </c>
       <c r="F15" t="n">
-        <v>10.3</v>
+        <v>15</v>
       </c>
       <c r="G15" t="n">
-        <v>11.4</v>
+        <v>13.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>25.03</v>
+        <v>21.01</v>
       </c>
       <c r="D16" t="n">
-        <v>2.27</v>
+        <v>1.78</v>
       </c>
       <c r="E16" t="n">
-        <v>24.1</v>
+        <v>20</v>
       </c>
       <c r="F16" t="n">
-        <v>3.4</v>
+        <v>10</v>
       </c>
       <c r="G16" t="n">
-        <v>9.699999999999999</v>
+        <v>13</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>11.39</v>
+        <v>25.09</v>
       </c>
       <c r="D17" t="n">
-        <v>0.73</v>
+        <v>2.28</v>
       </c>
       <c r="E17" t="n">
-        <v>19</v>
+        <v>26.7</v>
       </c>
       <c r="F17" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="G17" t="n">
-        <v>8.1</v>
+        <v>12.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>51.48</v>
+        <v>11.41</v>
       </c>
       <c r="D18" t="n">
-        <v>4.28</v>
+        <v>0.73</v>
       </c>
       <c r="E18" t="n">
-        <v>10.3</v>
+        <v>30</v>
       </c>
       <c r="F18" t="n">
-        <v>6.9</v>
+        <v>5</v>
       </c>
       <c r="G18" t="n">
-        <v>7.9</v>
+        <v>12.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>63.4</v>
+        <v>20.41</v>
       </c>
       <c r="D19" t="n">
-        <v>4.12</v>
+        <v>3.55</v>
       </c>
       <c r="E19" t="n">
-        <v>3.4</v>
+        <v>33.3</v>
       </c>
       <c r="F19" t="n">
-        <v>6.9</v>
+        <v>3.3</v>
       </c>
       <c r="G19" t="n">
-        <v>5.9</v>
+        <v>12.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>10.01</v>
+        <v>64.18000000000001</v>
       </c>
       <c r="D20" t="n">
-        <v>1.22</v>
+        <v>4.17</v>
       </c>
       <c r="E20" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="F20" t="n">
-        <v>6.9</v>
+        <v>10</v>
       </c>
       <c r="G20" t="n">
-        <v>5.9</v>
+        <v>9</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>18.08</v>
+        <v>23.43</v>
       </c>
       <c r="D21" t="n">
-        <v>1.66</v>
+        <v>1.72</v>
       </c>
       <c r="E21" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="F21" t="n">
-        <v>6.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>5.9</v>
+        <v>7.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20.96</v>
+        <v>28.1</v>
       </c>
       <c r="D22" t="n">
-        <v>1.76</v>
+        <v>2.58</v>
       </c>
       <c r="E22" t="n">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="F22" t="n">
-        <v>5.2</v>
+        <v>6.7</v>
       </c>
       <c r="G22" t="n">
-        <v>5.7</v>
+        <v>6.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>29.26</v>
+        <v>32.65</v>
       </c>
       <c r="D23" t="n">
-        <v>2.17</v>
+        <v>2.5</v>
       </c>
       <c r="E23" t="n">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="F23" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="G23" t="n">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>26.94</v>
+        <v>24.53</v>
       </c>
       <c r="D24" t="n">
-        <v>2.21</v>
+        <v>2.02</v>
       </c>
       <c r="E24" t="n">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="F24" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="G24" t="n">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>24.49</v>
+        <v>18.07</v>
       </c>
       <c r="D25" t="n">
-        <v>2.01</v>
+        <v>1.01</v>
       </c>
       <c r="E25" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="F25" t="n">
-        <v>3.4</v>
+        <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>3.4</v>
+        <v>5.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>27.4</v>
+        <v>28.4</v>
       </c>
       <c r="D26" t="n">
-        <v>2.52</v>
+        <v>2.62</v>
       </c>
       <c r="E26" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="F26" t="n">
-        <v>3.4</v>
+        <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>3.4</v>
+        <v>5.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18.06</v>
+        <v>30.31</v>
       </c>
       <c r="D27" t="n">
-        <v>1.01</v>
+        <v>2.55</v>
       </c>
       <c r="E27" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="F27" t="n">
-        <v>3.4</v>
+        <v>5</v>
       </c>
       <c r="G27" t="n">
-        <v>3.4</v>
+        <v>5.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>21.36</v>
+        <v>29.02</v>
       </c>
       <c r="D28" t="n">
-        <v>3.62</v>
+        <v>2.16</v>
       </c>
       <c r="E28" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="F28" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="G28" t="n">
-        <v>3.4</v>
+        <v>4.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>32.52</v>
+        <v>26.85</v>
       </c>
       <c r="D29" t="n">
-        <v>2.49</v>
+        <v>2.2</v>
       </c>
       <c r="E29" t="n">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="F29" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="G29" t="n">
-        <v>3.4</v>
+        <v>4.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>14.77</v>
+        <v>9.9</v>
       </c>
       <c r="D30" t="n">
-        <v>1.39</v>
+        <v>1.2</v>
       </c>
       <c r="E30" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="F30" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="G30" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>23.08</v>
+        <v>14.57</v>
       </c>
       <c r="D31" t="n">
-        <v>1.7</v>
+        <v>1.37</v>
       </c>
       <c r="E31" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="F31" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="G31" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>30.27</v>
+        <v>17.91</v>
       </c>
       <c r="D32" t="n">
-        <v>2.55</v>
+        <v>1.64</v>
       </c>
       <c r="E32" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="F32" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="G32" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat May 23 11:01:53 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>7.54</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.63</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.03</v>
       </c>
       <c r="E4" t="n">
-        <v>90</v>
+        <v>88.7</v>
       </c>
       <c r="F4" t="n">
-        <v>91.7</v>
+        <v>90.3</v>
       </c>
       <c r="G4" t="n">
-        <v>90.8</v>
+        <v>89.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.95</v>
       </c>
       <c r="E5" t="n">
-        <v>70</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>70</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>70</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>4.95</v>
       </c>
       <c r="E6" t="n">
-        <v>63.3</v>
+        <v>62.9</v>
       </c>
       <c r="F6" t="n">
-        <v>63.3</v>
+        <v>62.9</v>
       </c>
       <c r="G6" t="n">
-        <v>63.3</v>
+        <v>62.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>4.01</v>
       </c>
       <c r="E7" t="n">
-        <v>63.3</v>
+        <v>62.9</v>
       </c>
       <c r="F7" t="n">
-        <v>53.3</v>
+        <v>53.2</v>
       </c>
       <c r="G7" t="n">
-        <v>58.3</v>
+        <v>58.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.45</v>
       </c>
       <c r="E8" t="n">
-        <v>60</v>
+        <v>59.7</v>
       </c>
       <c r="F8" t="n">
-        <v>48.3</v>
+        <v>48.4</v>
       </c>
       <c r="G8" t="n">
-        <v>54.2</v>
+        <v>54</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.87</v>
       </c>
       <c r="E9" t="n">
-        <v>53.3</v>
+        <v>53.2</v>
       </c>
       <c r="F9" t="n">
-        <v>30</v>
+        <v>30.6</v>
       </c>
       <c r="G9" t="n">
-        <v>41.7</v>
+        <v>41.9</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.48</v>
       </c>
       <c r="E10" t="n">
-        <v>33.3</v>
+        <v>33.9</v>
       </c>
       <c r="F10" t="n">
-        <v>45</v>
+        <v>45.2</v>
       </c>
       <c r="G10" t="n">
-        <v>39.2</v>
+        <v>39.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>4.33</v>
       </c>
       <c r="E11" t="n">
-        <v>30</v>
+        <v>30.6</v>
       </c>
       <c r="F11" t="n">
-        <v>33.3</v>
+        <v>33.9</v>
       </c>
       <c r="G11" t="n">
-        <v>31.7</v>
+        <v>32.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.09</v>
       </c>
       <c r="E12" t="n">
-        <v>13.3</v>
+        <v>14.5</v>
       </c>
       <c r="F12" t="n">
-        <v>21.7</v>
+        <v>22.6</v>
       </c>
       <c r="G12" t="n">
-        <v>19.2</v>
+        <v>20.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>3.75</v>
       </c>
       <c r="E13" t="n">
-        <v>16.7</v>
+        <v>17.7</v>
       </c>
       <c r="F13" t="n">
+        <v>21</v>
+      </c>
+      <c r="G13" t="n">
         <v>20</v>
       </c>
-      <c r="G13" t="n">
-        <v>19</v>
-      </c>
       <c r="H13" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.26</v>
       </c>
       <c r="E14" t="n">
-        <v>11.7</v>
+        <v>12.9</v>
       </c>
       <c r="F14" t="n">
-        <v>18.3</v>
+        <v>19.4</v>
       </c>
       <c r="G14" t="n">
-        <v>16.3</v>
+        <v>17.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>0.64</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>11.3</v>
       </c>
       <c r="F15" t="n">
-        <v>15</v>
+        <v>16.1</v>
       </c>
       <c r="G15" t="n">
-        <v>13.5</v>
+        <v>14.7</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.78</v>
       </c>
       <c r="E16" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F16" t="n">
-        <v>10</v>
+        <v>11.3</v>
       </c>
       <c r="G16" t="n">
-        <v>13</v>
+        <v>14.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.28</v>
       </c>
       <c r="E17" t="n">
-        <v>26.7</v>
+        <v>27.4</v>
       </c>
       <c r="F17" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="G17" t="n">
-        <v>12.7</v>
+        <v>13.9</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>0.73</v>
       </c>
       <c r="E18" t="n">
-        <v>30</v>
+        <v>30.6</v>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="G18" t="n">
-        <v>12.5</v>
+        <v>13.7</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>3.55</v>
       </c>
       <c r="E19" t="n">
-        <v>33.3</v>
+        <v>33.9</v>
       </c>
       <c r="F19" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="G19" t="n">
-        <v>12.3</v>
+        <v>13.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>4.17</v>
       </c>
       <c r="E20" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F20" t="n">
-        <v>10</v>
+        <v>11.3</v>
       </c>
       <c r="G20" t="n">
-        <v>9</v>
+        <v>10.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.72</v>
       </c>
       <c r="E21" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F21" t="n">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>7.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.58</v>
       </c>
       <c r="E22" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F22" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="G22" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.5</v>
       </c>
       <c r="E23" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F23" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="G23" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.02</v>
       </c>
       <c r="E24" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F24" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="G24" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.01</v>
       </c>
       <c r="E25" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="G25" t="n">
-        <v>5.5</v>
+        <v>6.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.62</v>
       </c>
       <c r="E26" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="G26" t="n">
-        <v>5.5</v>
+        <v>6.9</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.55</v>
       </c>
       <c r="E27" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F27" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="G27" t="n">
-        <v>5.5</v>
+        <v>6.9</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.16</v>
       </c>
       <c r="E28" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F28" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="G28" t="n">
-        <v>4.3</v>
+        <v>5.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>2.2</v>
       </c>
       <c r="E29" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="F29" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="G29" t="n">
-        <v>4.3</v>
+        <v>5.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.2</v>
       </c>
       <c r="E30" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="F30" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="G30" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.37</v>
       </c>
       <c r="E31" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="F31" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="G31" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.64</v>
       </c>
       <c r="E32" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="F32" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="G32" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun May 24 11:03:24 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>7.54</v>
       </c>
       <c r="E2" t="n">
-        <v>98.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>98.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>98.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.63</v>
       </c>
       <c r="E3" t="n">
-        <v>98.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>98.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>98.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.03</v>
       </c>
       <c r="E4" t="n">
-        <v>88.7</v>
+        <v>87.5</v>
       </c>
       <c r="F4" t="n">
-        <v>90.3</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>89.5</v>
+        <v>88.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.95</v>
       </c>
       <c r="E5" t="n">
-        <v>69.40000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="F5" t="n">
-        <v>69.40000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="G5" t="n">
-        <v>69.40000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>4.95</v>
       </c>
       <c r="E6" t="n">
-        <v>62.9</v>
+        <v>62.5</v>
       </c>
       <c r="F6" t="n">
-        <v>62.9</v>
+        <v>62.5</v>
       </c>
       <c r="G6" t="n">
-        <v>62.9</v>
+        <v>62.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>4.01</v>
       </c>
       <c r="E7" t="n">
-        <v>62.9</v>
+        <v>62.5</v>
       </c>
       <c r="F7" t="n">
-        <v>53.2</v>
+        <v>53.1</v>
       </c>
       <c r="G7" t="n">
-        <v>58.1</v>
+        <v>57.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.45</v>
       </c>
       <c r="E8" t="n">
-        <v>59.7</v>
+        <v>59.4</v>
       </c>
       <c r="F8" t="n">
         <v>48.4</v>
       </c>
       <c r="G8" t="n">
-        <v>54</v>
+        <v>53.9</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.87</v>
       </c>
       <c r="E9" t="n">
-        <v>53.2</v>
+        <v>53.1</v>
       </c>
       <c r="F9" t="n">
-        <v>30.6</v>
+        <v>31.2</v>
       </c>
       <c r="G9" t="n">
-        <v>41.9</v>
+        <v>42.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.48</v>
       </c>
       <c r="E10" t="n">
-        <v>33.9</v>
+        <v>34.4</v>
       </c>
       <c r="F10" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="G10" t="n">
-        <v>39.5</v>
+        <v>39.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>4.33</v>
       </c>
       <c r="E11" t="n">
-        <v>30.6</v>
+        <v>31.2</v>
       </c>
       <c r="F11" t="n">
-        <v>33.9</v>
+        <v>34.4</v>
       </c>
       <c r="G11" t="n">
-        <v>32.3</v>
+        <v>32.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.09</v>
       </c>
       <c r="E12" t="n">
-        <v>14.5</v>
+        <v>15.6</v>
       </c>
       <c r="F12" t="n">
-        <v>22.6</v>
+        <v>23.4</v>
       </c>
       <c r="G12" t="n">
-        <v>20.2</v>
+        <v>21.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>3.75</v>
       </c>
       <c r="E13" t="n">
-        <v>17.7</v>
+        <v>18.8</v>
       </c>
       <c r="F13" t="n">
-        <v>21</v>
+        <v>21.9</v>
       </c>
       <c r="G13" t="n">
-        <v>20</v>
+        <v>20.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.26</v>
       </c>
       <c r="E14" t="n">
-        <v>12.9</v>
+        <v>14.1</v>
       </c>
       <c r="F14" t="n">
-        <v>19.4</v>
+        <v>20.3</v>
       </c>
       <c r="G14" t="n">
-        <v>17.4</v>
+        <v>18.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>0.64</v>
       </c>
       <c r="E15" t="n">
-        <v>11.3</v>
+        <v>12.5</v>
       </c>
       <c r="F15" t="n">
-        <v>16.1</v>
+        <v>17.2</v>
       </c>
       <c r="G15" t="n">
-        <v>14.7</v>
+        <v>15.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.78</v>
       </c>
       <c r="E16" t="n">
-        <v>21</v>
+        <v>21.9</v>
       </c>
       <c r="F16" t="n">
-        <v>11.3</v>
+        <v>12.5</v>
       </c>
       <c r="G16" t="n">
-        <v>14.2</v>
+        <v>15.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.28</v>
       </c>
       <c r="E17" t="n">
-        <v>27.4</v>
+        <v>28.1</v>
       </c>
       <c r="F17" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="G17" t="n">
-        <v>13.9</v>
+        <v>15</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>0.73</v>
       </c>
       <c r="E18" t="n">
-        <v>30.6</v>
+        <v>31.2</v>
       </c>
       <c r="F18" t="n">
-        <v>6.5</v>
+        <v>7.8</v>
       </c>
       <c r="G18" t="n">
-        <v>13.7</v>
+        <v>14.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>3.55</v>
       </c>
       <c r="E19" t="n">
-        <v>33.9</v>
+        <v>34.4</v>
       </c>
       <c r="F19" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="G19" t="n">
-        <v>13.5</v>
+        <v>14.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>4.17</v>
       </c>
       <c r="E20" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F20" t="n">
-        <v>11.3</v>
+        <v>12.5</v>
       </c>
       <c r="G20" t="n">
-        <v>10.3</v>
+        <v>11.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.72</v>
       </c>
       <c r="E21" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F21" t="n">
-        <v>9.699999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="G21" t="n">
-        <v>9.199999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.58</v>
       </c>
       <c r="E22" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F22" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="G22" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.5</v>
       </c>
       <c r="E23" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F23" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="G23" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.02</v>
       </c>
       <c r="E24" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F24" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="G24" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.01</v>
       </c>
       <c r="E25" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F25" t="n">
-        <v>6.5</v>
+        <v>7.8</v>
       </c>
       <c r="G25" t="n">
-        <v>6.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.62</v>
       </c>
       <c r="E26" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F26" t="n">
-        <v>6.5</v>
+        <v>7.8</v>
       </c>
       <c r="G26" t="n">
-        <v>6.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.55</v>
       </c>
       <c r="E27" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F27" t="n">
-        <v>6.5</v>
+        <v>7.8</v>
       </c>
       <c r="G27" t="n">
-        <v>6.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.16</v>
       </c>
       <c r="E28" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F28" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="G28" t="n">
-        <v>5.8</v>
+        <v>7.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>2.2</v>
       </c>
       <c r="E29" t="n">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="F29" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="G29" t="n">
-        <v>5.8</v>
+        <v>7.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.2</v>
       </c>
       <c r="E30" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="F30" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="G30" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.37</v>
       </c>
       <c r="E31" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="F31" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="G31" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.64</v>
       </c>
       <c r="E32" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="F32" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="G32" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon May 25 12:53:35 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,82 +486,82 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>72.86</v>
+        <v>77</v>
       </c>
       <c r="D2" t="n">
-        <v>7.54</v>
+        <v>7.97</v>
       </c>
       <c r="E2" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42.92</v>
+        <v>37.54</v>
       </c>
       <c r="D3" t="n">
-        <v>3.63</v>
+        <v>2.09</v>
       </c>
       <c r="E3" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>36.39</v>
+        <v>43.41</v>
       </c>
       <c r="D4" t="n">
-        <v>2.03</v>
+        <v>3.67</v>
       </c>
       <c r="E4" t="n">
-        <v>87.5</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>89.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>88.3</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="5">
@@ -576,532 +576,532 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>31.19</v>
+        <v>31.95</v>
       </c>
       <c r="D5" t="n">
-        <v>2.95</v>
+        <v>3.03</v>
       </c>
       <c r="E5" t="n">
-        <v>68.8</v>
+        <v>84.8</v>
       </c>
       <c r="F5" t="n">
-        <v>68.8</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>68.8</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>131.92</v>
+        <v>20.46</v>
       </c>
       <c r="D6" t="n">
-        <v>4.95</v>
+        <v>1.91</v>
       </c>
       <c r="E6" t="n">
-        <v>62.5</v>
+        <v>72.7</v>
       </c>
       <c r="F6" t="n">
-        <v>62.5</v>
+        <v>71.2</v>
       </c>
       <c r="G6" t="n">
-        <v>62.5</v>
+        <v>72</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>37.15</v>
+        <v>52.51</v>
       </c>
       <c r="D7" t="n">
-        <v>4.01</v>
+        <v>4.37</v>
       </c>
       <c r="E7" t="n">
-        <v>62.5</v>
+        <v>54.5</v>
       </c>
       <c r="F7" t="n">
-        <v>53.1</v>
+        <v>54.5</v>
       </c>
       <c r="G7" t="n">
-        <v>57.8</v>
+        <v>54.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>16.52</v>
+        <v>26.76</v>
       </c>
       <c r="D8" t="n">
-        <v>2.45</v>
+        <v>2.48</v>
       </c>
       <c r="E8" t="n">
-        <v>59.4</v>
+        <v>59.1</v>
       </c>
       <c r="F8" t="n">
-        <v>48.4</v>
+        <v>45.5</v>
       </c>
       <c r="G8" t="n">
-        <v>53.9</v>
+        <v>52.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20.05</v>
+        <v>15.49</v>
       </c>
       <c r="D9" t="n">
-        <v>1.87</v>
+        <v>1.27</v>
       </c>
       <c r="E9" t="n">
-        <v>53.1</v>
+        <v>43.9</v>
       </c>
       <c r="F9" t="n">
-        <v>31.2</v>
+        <v>51.5</v>
       </c>
       <c r="G9" t="n">
-        <v>42.2</v>
+        <v>47.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>26.7</v>
+        <v>16.47</v>
       </c>
       <c r="D10" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="E10" t="n">
-        <v>34.4</v>
+        <v>51.5</v>
       </c>
       <c r="F10" t="n">
-        <v>45.3</v>
+        <v>30.3</v>
       </c>
       <c r="G10" t="n">
-        <v>39.8</v>
+        <v>40.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>52.03</v>
+        <v>36.96</v>
       </c>
       <c r="D11" t="n">
-        <v>4.33</v>
+        <v>3.99</v>
       </c>
       <c r="E11" t="n">
-        <v>31.2</v>
+        <v>45.5</v>
       </c>
       <c r="F11" t="n">
-        <v>34.4</v>
+        <v>25.8</v>
       </c>
       <c r="G11" t="n">
-        <v>32.8</v>
+        <v>31.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>12.14</v>
+        <v>22.24</v>
       </c>
       <c r="D12" t="n">
-        <v>1.09</v>
+        <v>3.77</v>
       </c>
       <c r="E12" t="n">
-        <v>15.6</v>
+        <v>24.2</v>
       </c>
       <c r="F12" t="n">
-        <v>23.4</v>
+        <v>31.8</v>
       </c>
       <c r="G12" t="n">
-        <v>21.1</v>
+        <v>28</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>22.11</v>
+        <v>129.89</v>
       </c>
       <c r="D13" t="n">
-        <v>3.75</v>
+        <v>4.87</v>
       </c>
       <c r="E13" t="n">
-        <v>18.8</v>
+        <v>27.3</v>
       </c>
       <c r="F13" t="n">
-        <v>21.9</v>
+        <v>27.3</v>
       </c>
       <c r="G13" t="n">
-        <v>20.9</v>
+        <v>27.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.44</v>
+        <v>12.23</v>
       </c>
       <c r="D14" t="n">
-        <v>1.26</v>
+        <v>1.1</v>
       </c>
       <c r="E14" t="n">
-        <v>14.1</v>
+        <v>21.2</v>
       </c>
       <c r="F14" t="n">
-        <v>20.3</v>
+        <v>30.3</v>
       </c>
       <c r="G14" t="n">
-        <v>18.4</v>
+        <v>25.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6.75</v>
+        <v>20.45</v>
       </c>
       <c r="D15" t="n">
-        <v>0.64</v>
+        <v>3.56</v>
       </c>
       <c r="E15" t="n">
-        <v>12.5</v>
+        <v>39.4</v>
       </c>
       <c r="F15" t="n">
-        <v>17.2</v>
+        <v>12.1</v>
       </c>
       <c r="G15" t="n">
-        <v>15.8</v>
+        <v>20.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>21.01</v>
+        <v>6.76</v>
       </c>
       <c r="D16" t="n">
-        <v>1.78</v>
+        <v>0.64</v>
       </c>
       <c r="E16" t="n">
-        <v>21.9</v>
+        <v>21.2</v>
       </c>
       <c r="F16" t="n">
-        <v>12.5</v>
+        <v>18.2</v>
       </c>
       <c r="G16" t="n">
-        <v>15.3</v>
+        <v>19.1</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25.09</v>
+        <v>64.54000000000001</v>
       </c>
       <c r="D17" t="n">
-        <v>2.28</v>
+        <v>4.2</v>
       </c>
       <c r="E17" t="n">
-        <v>28.1</v>
+        <v>15.2</v>
       </c>
       <c r="F17" t="n">
-        <v>9.4</v>
+        <v>18.2</v>
       </c>
       <c r="G17" t="n">
-        <v>15</v>
+        <v>17.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>11.41</v>
+        <v>23.52</v>
       </c>
       <c r="D18" t="n">
-        <v>0.73</v>
+        <v>1.73</v>
       </c>
       <c r="E18" t="n">
-        <v>31.2</v>
+        <v>15.2</v>
       </c>
       <c r="F18" t="n">
-        <v>7.8</v>
+        <v>18.2</v>
       </c>
       <c r="G18" t="n">
-        <v>14.8</v>
+        <v>17.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20.41</v>
+        <v>11.45</v>
       </c>
       <c r="D19" t="n">
-        <v>3.55</v>
+        <v>0.73</v>
       </c>
       <c r="E19" t="n">
-        <v>34.4</v>
+        <v>36.4</v>
       </c>
       <c r="F19" t="n">
-        <v>6.2</v>
+        <v>9.1</v>
       </c>
       <c r="G19" t="n">
-        <v>14.7</v>
+        <v>17.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>64.18000000000001</v>
+        <v>18.13</v>
       </c>
       <c r="D20" t="n">
-        <v>4.17</v>
+        <v>1.66</v>
       </c>
       <c r="E20" t="n">
-        <v>9.4</v>
+        <v>15.2</v>
       </c>
       <c r="F20" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="G20" t="n">
-        <v>11.6</v>
+        <v>16.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>23.43</v>
+        <v>30.28</v>
       </c>
       <c r="D21" t="n">
-        <v>1.72</v>
+        <v>2.56</v>
       </c>
       <c r="E21" t="n">
-        <v>9.4</v>
+        <v>6.1</v>
       </c>
       <c r="F21" t="n">
-        <v>10.9</v>
+        <v>15.2</v>
       </c>
       <c r="G21" t="n">
-        <v>10.5</v>
+        <v>12.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28.1</v>
+        <v>9.98</v>
       </c>
       <c r="D22" t="n">
-        <v>2.58</v>
+        <v>1.21</v>
       </c>
       <c r="E22" t="n">
-        <v>9.4</v>
+        <v>12.1</v>
       </c>
       <c r="F22" t="n">
-        <v>9.4</v>
+        <v>12.1</v>
       </c>
       <c r="G22" t="n">
-        <v>9.4</v>
+        <v>12.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.5</v>
       </c>
       <c r="E23" t="n">
-        <v>9.4</v>
+        <v>10.6</v>
       </c>
       <c r="F23" t="n">
-        <v>9.4</v>
+        <v>10.6</v>
       </c>
       <c r="G23" t="n">
-        <v>9.4</v>
+        <v>10.6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="24">
@@ -1146,112 +1146,112 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>24.53</v>
+        <v>24.5</v>
       </c>
       <c r="D24" t="n">
         <v>2.02</v>
       </c>
       <c r="E24" t="n">
-        <v>9.4</v>
+        <v>6.1</v>
       </c>
       <c r="F24" t="n">
-        <v>9.4</v>
+        <v>10.6</v>
       </c>
       <c r="G24" t="n">
-        <v>9.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>18.07</v>
+        <v>20.91</v>
       </c>
       <c r="D25" t="n">
-        <v>1.01</v>
+        <v>1.77</v>
       </c>
       <c r="E25" t="n">
-        <v>9.4</v>
+        <v>6.1</v>
       </c>
       <c r="F25" t="n">
-        <v>7.8</v>
+        <v>9.1</v>
       </c>
       <c r="G25" t="n">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>28.4</v>
+        <v>24.83</v>
       </c>
       <c r="D26" t="n">
-        <v>2.62</v>
+        <v>2.26</v>
       </c>
       <c r="E26" t="n">
-        <v>9.4</v>
+        <v>18.2</v>
       </c>
       <c r="F26" t="n">
-        <v>7.8</v>
+        <v>3</v>
       </c>
       <c r="G26" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>30.31</v>
+        <v>27.76</v>
       </c>
       <c r="D27" t="n">
         <v>2.55</v>
       </c>
       <c r="E27" t="n">
-        <v>9.4</v>
+        <v>6.1</v>
       </c>
       <c r="F27" t="n">
-        <v>7.8</v>
+        <v>6.1</v>
       </c>
       <c r="G27" t="n">
-        <v>8.300000000000001</v>
+        <v>6.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="28">
@@ -1266,22 +1266,22 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29.02</v>
+        <v>28.85</v>
       </c>
       <c r="D28" t="n">
-        <v>2.16</v>
+        <v>2.14</v>
       </c>
       <c r="E28" t="n">
-        <v>9.4</v>
+        <v>6.1</v>
       </c>
       <c r="F28" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="G28" t="n">
-        <v>7.2</v>
+        <v>3.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="29">
@@ -1296,112 +1296,112 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26.85</v>
+        <v>26.49</v>
       </c>
       <c r="D29" t="n">
-        <v>2.2</v>
+        <v>2.17</v>
       </c>
       <c r="E29" t="n">
-        <v>9.4</v>
+        <v>6.1</v>
       </c>
       <c r="F29" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="G29" t="n">
-        <v>7.2</v>
+        <v>3.9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9.9</v>
+        <v>28.23</v>
       </c>
       <c r="D30" t="n">
-        <v>1.2</v>
+        <v>2.6</v>
       </c>
       <c r="E30" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="F30" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="G30" t="n">
-        <v>6.2</v>
+        <v>3.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>14.57</v>
+        <v>17.97</v>
       </c>
       <c r="D31" t="n">
-        <v>1.37</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="G31" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>17.91</v>
+        <v>14.18</v>
       </c>
       <c r="D32" t="n">
-        <v>1.64</v>
+        <v>1.34</v>
       </c>
       <c r="E32" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="G32" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu May 28 12:55:38 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>77</v>
+        <v>77.08</v>
       </c>
       <c r="D2" t="n">
-        <v>7.97</v>
+        <v>7.99</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,25 +501,25 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>37.54</v>
+        <v>32.63</v>
       </c>
       <c r="D3" t="n">
-        <v>2.09</v>
+        <v>3.1</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -531,25 +531,25 @@
         <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>43.41</v>
+        <v>39.2</v>
       </c>
       <c r="D4" t="n">
-        <v>3.67</v>
+        <v>2.19</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
@@ -561,847 +561,847 @@
         <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>31.95</v>
+        <v>21.08</v>
       </c>
       <c r="D5" t="n">
-        <v>3.03</v>
+        <v>1.97</v>
       </c>
       <c r="E5" t="n">
-        <v>84.8</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>87.90000000000001</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>86.40000000000001</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>20.46</v>
+        <v>42.54</v>
       </c>
       <c r="D6" t="n">
-        <v>1.91</v>
+        <v>3.6</v>
       </c>
       <c r="E6" t="n">
-        <v>72.7</v>
+        <v>88.2</v>
       </c>
       <c r="F6" t="n">
-        <v>71.2</v>
+        <v>88.2</v>
       </c>
       <c r="G6" t="n">
-        <v>72</v>
+        <v>88.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>52.51</v>
+        <v>37.32</v>
       </c>
       <c r="D7" t="n">
-        <v>4.37</v>
+        <v>4.03</v>
       </c>
       <c r="E7" t="n">
-        <v>54.5</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>54.5</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>54.5</v>
+        <v>71.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>26.76</v>
+        <v>18.57</v>
       </c>
       <c r="D8" t="n">
-        <v>2.48</v>
+        <v>1.7</v>
       </c>
       <c r="E8" t="n">
-        <v>59.1</v>
+        <v>44.1</v>
       </c>
       <c r="F8" t="n">
-        <v>45.5</v>
+        <v>48.5</v>
       </c>
       <c r="G8" t="n">
-        <v>52.3</v>
+        <v>46.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15.49</v>
+        <v>130.25</v>
       </c>
       <c r="D9" t="n">
-        <v>1.27</v>
+        <v>4.89</v>
       </c>
       <c r="E9" t="n">
-        <v>43.9</v>
+        <v>41.2</v>
       </c>
       <c r="F9" t="n">
-        <v>51.5</v>
+        <v>41.2</v>
       </c>
       <c r="G9" t="n">
-        <v>47.7</v>
+        <v>41.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>16.47</v>
+        <v>22.02</v>
       </c>
       <c r="D10" t="n">
-        <v>2.43</v>
+        <v>3.75</v>
       </c>
       <c r="E10" t="n">
-        <v>51.5</v>
+        <v>11.8</v>
       </c>
       <c r="F10" t="n">
-        <v>30.3</v>
+        <v>22.1</v>
       </c>
       <c r="G10" t="n">
-        <v>40.9</v>
+        <v>19</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>36.96</v>
+        <v>11.83</v>
       </c>
       <c r="D11" t="n">
-        <v>3.99</v>
+        <v>1.07</v>
       </c>
       <c r="E11" t="n">
-        <v>45.5</v>
+        <v>5.9</v>
       </c>
       <c r="F11" t="n">
-        <v>25.8</v>
+        <v>17.6</v>
       </c>
       <c r="G11" t="n">
-        <v>31.7</v>
+        <v>14.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>22.24</v>
+        <v>25.91</v>
       </c>
       <c r="D12" t="n">
-        <v>3.77</v>
+        <v>2.4</v>
       </c>
       <c r="E12" t="n">
-        <v>24.2</v>
+        <v>20.6</v>
       </c>
       <c r="F12" t="n">
-        <v>31.8</v>
+        <v>2.9</v>
       </c>
       <c r="G12" t="n">
-        <v>28</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>129.89</v>
+        <v>15.9</v>
       </c>
       <c r="D13" t="n">
-        <v>4.87</v>
+        <v>2.36</v>
       </c>
       <c r="E13" t="n">
-        <v>27.3</v>
+        <v>20.6</v>
       </c>
       <c r="F13" t="n">
-        <v>27.3</v>
+        <v>2.9</v>
       </c>
       <c r="G13" t="n">
-        <v>27.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12.23</v>
+        <v>62.94</v>
       </c>
       <c r="D14" t="n">
-        <v>1.1</v>
+        <v>4.11</v>
       </c>
       <c r="E14" t="n">
-        <v>21.2</v>
+        <v>2.9</v>
       </c>
       <c r="F14" t="n">
-        <v>30.3</v>
+        <v>5.9</v>
       </c>
       <c r="G14" t="n">
-        <v>25.8</v>
+        <v>5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>20.45</v>
+        <v>27.26</v>
       </c>
       <c r="D15" t="n">
-        <v>3.56</v>
+        <v>2.52</v>
       </c>
       <c r="E15" t="n">
-        <v>39.4</v>
+        <v>2.9</v>
       </c>
       <c r="F15" t="n">
-        <v>12.1</v>
+        <v>4.4</v>
       </c>
       <c r="G15" t="n">
-        <v>20.3</v>
+        <v>4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6.76</v>
+        <v>27.55</v>
       </c>
       <c r="D16" t="n">
-        <v>0.64</v>
+        <v>2.55</v>
       </c>
       <c r="E16" t="n">
-        <v>21.2</v>
+        <v>5.9</v>
       </c>
       <c r="F16" t="n">
-        <v>18.2</v>
+        <v>2.9</v>
       </c>
       <c r="G16" t="n">
-        <v>19.1</v>
+        <v>3.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>64.54000000000001</v>
+        <v>25.91</v>
       </c>
       <c r="D17" t="n">
-        <v>4.2</v>
+        <v>2.13</v>
       </c>
       <c r="E17" t="n">
-        <v>15.2</v>
+        <v>5.9</v>
       </c>
       <c r="F17" t="n">
-        <v>18.2</v>
+        <v>2.9</v>
       </c>
       <c r="G17" t="n">
-        <v>17.3</v>
+        <v>3.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23.52</v>
+        <v>50.14</v>
       </c>
       <c r="D18" t="n">
-        <v>1.73</v>
+        <v>4.19</v>
       </c>
       <c r="E18" t="n">
-        <v>15.2</v>
+        <v>5.9</v>
       </c>
       <c r="F18" t="n">
-        <v>18.2</v>
+        <v>2.9</v>
       </c>
       <c r="G18" t="n">
-        <v>17.3</v>
+        <v>3.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>11.45</v>
+        <v>28.17</v>
       </c>
       <c r="D19" t="n">
-        <v>0.73</v>
+        <v>2.12</v>
       </c>
       <c r="E19" t="n">
-        <v>36.4</v>
+        <v>5.9</v>
       </c>
       <c r="F19" t="n">
-        <v>9.1</v>
+        <v>2.9</v>
       </c>
       <c r="G19" t="n">
-        <v>17.3</v>
+        <v>3.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>18.13</v>
+        <v>24.24</v>
       </c>
       <c r="D20" t="n">
-        <v>1.66</v>
+        <v>2.21</v>
       </c>
       <c r="E20" t="n">
-        <v>15.2</v>
+        <v>5.9</v>
       </c>
       <c r="F20" t="n">
-        <v>16.7</v>
+        <v>2.9</v>
       </c>
       <c r="G20" t="n">
-        <v>16.2</v>
+        <v>3.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>30.28</v>
+        <v>20.02</v>
       </c>
       <c r="D21" t="n">
-        <v>2.56</v>
+        <v>1.7</v>
       </c>
       <c r="E21" t="n">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
       <c r="F21" t="n">
-        <v>15.2</v>
+        <v>2.9</v>
       </c>
       <c r="G21" t="n">
-        <v>12.4</v>
+        <v>3.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9.98</v>
+        <v>20.14</v>
       </c>
       <c r="D22" t="n">
-        <v>1.21</v>
+        <v>3.52</v>
       </c>
       <c r="E22" t="n">
-        <v>12.1</v>
+        <v>5.9</v>
       </c>
       <c r="F22" t="n">
-        <v>12.1</v>
+        <v>2.9</v>
       </c>
       <c r="G22" t="n">
-        <v>12.1</v>
+        <v>3.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>32.65</v>
+        <v>11.19</v>
       </c>
       <c r="D23" t="n">
-        <v>2.5</v>
+        <v>0.71</v>
       </c>
       <c r="E23" t="n">
-        <v>10.6</v>
+        <v>5.9</v>
       </c>
       <c r="F23" t="n">
-        <v>10.6</v>
+        <v>2.9</v>
       </c>
       <c r="G23" t="n">
-        <v>10.6</v>
+        <v>3.8</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>24.5</v>
+        <v>17.8</v>
       </c>
       <c r="D24" t="n">
-        <v>2.02</v>
+        <v>0.99</v>
       </c>
       <c r="E24" t="n">
-        <v>6.1</v>
+        <v>2.9</v>
       </c>
       <c r="F24" t="n">
-        <v>10.6</v>
+        <v>2.9</v>
       </c>
       <c r="G24" t="n">
-        <v>9.199999999999999</v>
+        <v>2.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20.91</v>
+        <v>23.58</v>
       </c>
       <c r="D25" t="n">
-        <v>1.77</v>
+        <v>1.95</v>
       </c>
       <c r="E25" t="n">
-        <v>6.1</v>
+        <v>2.9</v>
       </c>
       <c r="F25" t="n">
-        <v>9.1</v>
+        <v>2.9</v>
       </c>
       <c r="G25" t="n">
-        <v>8.199999999999999</v>
+        <v>2.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>24.83</v>
+        <v>15.09</v>
       </c>
       <c r="D26" t="n">
-        <v>2.26</v>
+        <v>1.23</v>
       </c>
       <c r="E26" t="n">
-        <v>18.2</v>
+        <v>2.9</v>
       </c>
       <c r="F26" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="G26" t="n">
-        <v>7.6</v>
+        <v>2.9</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>27.76</v>
+        <v>9.75</v>
       </c>
       <c r="D27" t="n">
-        <v>2.55</v>
+        <v>1.18</v>
       </c>
       <c r="E27" t="n">
-        <v>6.1</v>
+        <v>2.9</v>
       </c>
       <c r="F27" t="n">
-        <v>6.1</v>
+        <v>2.9</v>
       </c>
       <c r="G27" t="n">
-        <v>6.1</v>
+        <v>2.9</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>28.85</v>
+        <v>32.18</v>
       </c>
       <c r="D28" t="n">
-        <v>2.14</v>
+        <v>2.47</v>
       </c>
       <c r="E28" t="n">
-        <v>6.1</v>
+        <v>2.9</v>
       </c>
       <c r="F28" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="G28" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26.49</v>
+        <v>6.67</v>
       </c>
       <c r="D29" t="n">
-        <v>2.17</v>
+        <v>0.63</v>
       </c>
       <c r="E29" t="n">
-        <v>6.1</v>
+        <v>2.9</v>
       </c>
       <c r="F29" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="G29" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>28.23</v>
+        <v>14.1</v>
       </c>
       <c r="D30" t="n">
-        <v>2.6</v>
+        <v>1.33</v>
       </c>
       <c r="E30" t="n">
-        <v>6.1</v>
+        <v>2.9</v>
       </c>
       <c r="F30" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="G30" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>17.97</v>
+        <v>22.89</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>1.69</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="F31" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="G31" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>14.18</v>
+        <v>29.31</v>
       </c>
       <c r="D32" t="n">
-        <v>1.34</v>
+        <v>2.48</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="F32" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="G32" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri May 29 12:36:17 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>77.08</v>
+        <v>21.69</v>
       </c>
       <c r="D2" t="n">
-        <v>7.99</v>
+        <v>2.03</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,7 +501,7 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>32.63</v>
+        <v>32.5</v>
       </c>
       <c r="D3" t="n">
-        <v>3.1</v>
+        <v>3.08</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="4">
@@ -546,142 +546,142 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>39.2</v>
+        <v>38.51</v>
       </c>
       <c r="D4" t="n">
-        <v>2.19</v>
+        <v>2.15</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21.08</v>
+        <v>73.81</v>
       </c>
       <c r="D5" t="n">
-        <v>1.97</v>
+        <v>7.66</v>
       </c>
       <c r="E5" t="n">
-        <v>94.09999999999999</v>
+        <v>94.3</v>
       </c>
       <c r="F5" t="n">
-        <v>95.59999999999999</v>
+        <v>94.3</v>
       </c>
       <c r="G5" t="n">
-        <v>94.90000000000001</v>
+        <v>94.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>42.54</v>
+        <v>18.96</v>
       </c>
       <c r="D6" t="n">
-        <v>3.6</v>
+        <v>1.74</v>
       </c>
       <c r="E6" t="n">
-        <v>88.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>88.2</v>
+        <v>61.4</v>
       </c>
       <c r="G6" t="n">
-        <v>88.2</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>37.32</v>
+        <v>40.95</v>
       </c>
       <c r="D7" t="n">
-        <v>4.03</v>
+        <v>3.47</v>
       </c>
       <c r="E7" t="n">
-        <v>70.59999999999999</v>
+        <v>57.1</v>
       </c>
       <c r="F7" t="n">
-        <v>72.09999999999999</v>
+        <v>57.1</v>
       </c>
       <c r="G7" t="n">
-        <v>71.3</v>
+        <v>57.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>18.57</v>
+        <v>20.76</v>
       </c>
       <c r="D8" t="n">
-        <v>1.7</v>
+        <v>3.63</v>
       </c>
       <c r="E8" t="n">
-        <v>44.1</v>
+        <v>57.1</v>
       </c>
       <c r="F8" t="n">
-        <v>48.5</v>
+        <v>21.4</v>
       </c>
       <c r="G8" t="n">
-        <v>46.3</v>
+        <v>32.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="9">
@@ -696,52 +696,52 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>130.25</v>
+        <v>121.94</v>
       </c>
       <c r="D9" t="n">
-        <v>4.89</v>
+        <v>4.59</v>
       </c>
       <c r="E9" t="n">
-        <v>41.2</v>
+        <v>22.9</v>
       </c>
       <c r="F9" t="n">
-        <v>41.2</v>
+        <v>22.9</v>
       </c>
       <c r="G9" t="n">
-        <v>41.2</v>
+        <v>22.9</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>22.02</v>
+        <v>6.75</v>
       </c>
       <c r="D10" t="n">
-        <v>3.75</v>
+        <v>0.64</v>
       </c>
       <c r="E10" t="n">
-        <v>11.8</v>
+        <v>15.7</v>
       </c>
       <c r="F10" t="n">
-        <v>22.1</v>
+        <v>21.4</v>
       </c>
       <c r="G10" t="n">
-        <v>19</v>
+        <v>19.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="11">
@@ -756,520 +756,520 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>11.83</v>
+        <v>11.94</v>
       </c>
       <c r="D11" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="E11" t="n">
-        <v>5.9</v>
+        <v>11.4</v>
       </c>
       <c r="F11" t="n">
-        <v>17.6</v>
+        <v>20</v>
       </c>
       <c r="G11" t="n">
-        <v>14.1</v>
+        <v>17.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>25.91</v>
+        <v>36.47</v>
       </c>
       <c r="D12" t="n">
-        <v>2.4</v>
+        <v>3.94</v>
       </c>
       <c r="E12" t="n">
-        <v>20.6</v>
+        <v>20</v>
       </c>
       <c r="F12" t="n">
-        <v>2.9</v>
+        <v>8.6</v>
       </c>
       <c r="G12" t="n">
-        <v>8.199999999999999</v>
+        <v>12</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>15.9</v>
+        <v>30.08</v>
       </c>
       <c r="D13" t="n">
-        <v>2.36</v>
+        <v>2.55</v>
       </c>
       <c r="E13" t="n">
-        <v>20.6</v>
+        <v>5.7</v>
       </c>
       <c r="F13" t="n">
-        <v>2.9</v>
+        <v>11.4</v>
       </c>
       <c r="G13" t="n">
-        <v>8.199999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>62.94</v>
+        <v>15.9</v>
       </c>
       <c r="D14" t="n">
-        <v>4.11</v>
+        <v>2.36</v>
       </c>
       <c r="E14" t="n">
-        <v>2.9</v>
+        <v>21.4</v>
       </c>
       <c r="F14" t="n">
-        <v>5.9</v>
+        <v>4.3</v>
       </c>
       <c r="G14" t="n">
-        <v>5</v>
+        <v>9.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>27.26</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>2.52</v>
+        <v>1.2</v>
       </c>
       <c r="E15" t="n">
-        <v>2.9</v>
+        <v>5.7</v>
       </c>
       <c r="F15" t="n">
-        <v>4.4</v>
+        <v>10</v>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>27.55</v>
+        <v>28.53</v>
       </c>
       <c r="D16" t="n">
-        <v>2.55</v>
+        <v>2.15</v>
       </c>
       <c r="E16" t="n">
-        <v>5.9</v>
+        <v>8.6</v>
       </c>
       <c r="F16" t="n">
-        <v>2.9</v>
+        <v>8.6</v>
       </c>
       <c r="G16" t="n">
-        <v>3.8</v>
+        <v>8.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25.91</v>
+        <v>21.61</v>
       </c>
       <c r="D17" t="n">
-        <v>2.13</v>
+        <v>3.69</v>
       </c>
       <c r="E17" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="F17" t="n">
-        <v>2.9</v>
+        <v>7.1</v>
       </c>
       <c r="G17" t="n">
-        <v>3.8</v>
+        <v>6.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>50.14</v>
+        <v>17.86</v>
       </c>
       <c r="D18" t="n">
-        <v>4.19</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="F18" t="n">
-        <v>2.9</v>
+        <v>7.1</v>
       </c>
       <c r="G18" t="n">
-        <v>3.8</v>
+        <v>6.7</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>28.17</v>
+        <v>27.85</v>
       </c>
       <c r="D19" t="n">
-        <v>2.12</v>
+        <v>2.59</v>
       </c>
       <c r="E19" t="n">
-        <v>5.9</v>
+        <v>8.6</v>
       </c>
       <c r="F19" t="n">
-        <v>2.9</v>
+        <v>5.7</v>
       </c>
       <c r="G19" t="n">
-        <v>3.8</v>
+        <v>6.6</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>24.24</v>
+        <v>11.21</v>
       </c>
       <c r="D20" t="n">
-        <v>2.21</v>
+        <v>0.72</v>
       </c>
       <c r="E20" t="n">
-        <v>5.9</v>
+        <v>8.6</v>
       </c>
       <c r="F20" t="n">
-        <v>2.9</v>
+        <v>5.7</v>
       </c>
       <c r="G20" t="n">
-        <v>3.8</v>
+        <v>6.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20.02</v>
+        <v>24.16</v>
       </c>
       <c r="D21" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="F21" t="n">
-        <v>2.9</v>
+        <v>5.7</v>
       </c>
       <c r="G21" t="n">
-        <v>3.8</v>
+        <v>5.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20.14</v>
+        <v>15.2</v>
       </c>
       <c r="D22" t="n">
-        <v>3.52</v>
+        <v>1.24</v>
       </c>
       <c r="E22" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="F22" t="n">
-        <v>2.9</v>
+        <v>5.7</v>
       </c>
       <c r="G22" t="n">
-        <v>3.8</v>
+        <v>5.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>11.19</v>
+        <v>25.98</v>
       </c>
       <c r="D23" t="n">
-        <v>0.71</v>
+        <v>2.13</v>
       </c>
       <c r="E23" t="n">
-        <v>5.9</v>
+        <v>8.6</v>
       </c>
       <c r="F23" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
       <c r="G23" t="n">
-        <v>3.8</v>
+        <v>5.6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>17.8</v>
+        <v>20.03</v>
       </c>
       <c r="D24" t="n">
-        <v>0.99</v>
+        <v>1.7</v>
       </c>
       <c r="E24" t="n">
-        <v>2.9</v>
+        <v>8.6</v>
       </c>
       <c r="F24" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
       <c r="G24" t="n">
-        <v>2.9</v>
+        <v>5.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>23.58</v>
+        <v>14.13</v>
       </c>
       <c r="D25" t="n">
-        <v>1.95</v>
+        <v>1.33</v>
       </c>
       <c r="E25" t="n">
-        <v>2.9</v>
+        <v>5.7</v>
       </c>
       <c r="F25" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
       <c r="G25" t="n">
-        <v>2.9</v>
+        <v>4.7</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>15.09</v>
+        <v>25.45</v>
       </c>
       <c r="D26" t="n">
-        <v>1.23</v>
+        <v>2.36</v>
       </c>
       <c r="E26" t="n">
-        <v>2.9</v>
+        <v>5.7</v>
       </c>
       <c r="F26" t="n">
         <v>2.9</v>
       </c>
       <c r="G26" t="n">
-        <v>2.9</v>
+        <v>3.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9.75</v>
+        <v>23.97</v>
       </c>
       <c r="D27" t="n">
-        <v>1.18</v>
+        <v>2.18</v>
       </c>
       <c r="E27" t="n">
-        <v>2.9</v>
+        <v>5.7</v>
       </c>
       <c r="F27" t="n">
         <v>2.9</v>
       </c>
       <c r="G27" t="n">
-        <v>2.9</v>
+        <v>3.7</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>32.18</v>
+        <v>26.49</v>
       </c>
       <c r="D28" t="n">
-        <v>2.47</v>
+        <v>2.45</v>
       </c>
       <c r="E28" t="n">
         <v>2.9</v>
@@ -1281,25 +1281,25 @@
         <v>2.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6.67</v>
+        <v>31.99</v>
       </c>
       <c r="D29" t="n">
-        <v>0.63</v>
+        <v>2.45</v>
       </c>
       <c r="E29" t="n">
         <v>2.9</v>
@@ -1311,25 +1311,25 @@
         <v>2.9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>14.1</v>
+        <v>48.55</v>
       </c>
       <c r="D30" t="n">
-        <v>1.33</v>
+        <v>4.06</v>
       </c>
       <c r="E30" t="n">
         <v>2.9</v>
@@ -1341,25 +1341,25 @@
         <v>2.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22.89</v>
+        <v>60.34</v>
       </c>
       <c r="D31" t="n">
-        <v>1.69</v>
+        <v>3.93</v>
       </c>
       <c r="E31" t="n">
         <v>2.9</v>
@@ -1371,25 +1371,25 @@
         <v>2.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>29.31</v>
+        <v>22.58</v>
       </c>
       <c r="D32" t="n">
-        <v>2.48</v>
+        <v>1.67</v>
       </c>
       <c r="E32" t="n">
         <v>2.9</v>
@@ -1401,7 +1401,7 @@
         <v>2.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat May 30 11:06:23 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.03</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.08</v>
       </c>
       <c r="E3" t="n">
-        <v>97.09999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="F3" t="n">
-        <v>97.09999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="G3" t="n">
-        <v>97.09999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.15</v>
       </c>
       <c r="E4" t="n">
-        <v>97.09999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="F4" t="n">
-        <v>97.09999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="G4" t="n">
-        <v>97.09999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>7.66</v>
       </c>
       <c r="E5" t="n">
-        <v>94.3</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>94.3</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>94.3</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.74</v>
       </c>
       <c r="E6" t="n">
-        <v>71.40000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="F6" t="n">
-        <v>61.4</v>
+        <v>61.1</v>
       </c>
       <c r="G6" t="n">
-        <v>66.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>3.47</v>
       </c>
       <c r="E7" t="n">
-        <v>57.1</v>
+        <v>56.9</v>
       </c>
       <c r="F7" t="n">
-        <v>57.1</v>
+        <v>56.9</v>
       </c>
       <c r="G7" t="n">
-        <v>57.1</v>
+        <v>56.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>3.63</v>
       </c>
       <c r="E8" t="n">
-        <v>57.1</v>
+        <v>56.9</v>
       </c>
       <c r="F8" t="n">
-        <v>21.4</v>
+        <v>22.2</v>
       </c>
       <c r="G8" t="n">
-        <v>32.1</v>
+        <v>32.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>4.59</v>
       </c>
       <c r="E9" t="n">
-        <v>22.9</v>
+        <v>23.6</v>
       </c>
       <c r="F9" t="n">
-        <v>22.9</v>
+        <v>23.6</v>
       </c>
       <c r="G9" t="n">
-        <v>22.9</v>
+        <v>23.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>0.64</v>
       </c>
       <c r="E10" t="n">
-        <v>15.7</v>
+        <v>16.7</v>
       </c>
       <c r="F10" t="n">
-        <v>21.4</v>
+        <v>22.2</v>
       </c>
       <c r="G10" t="n">
-        <v>19.7</v>
+        <v>20.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.08</v>
       </c>
       <c r="E11" t="n">
-        <v>11.4</v>
+        <v>12.5</v>
       </c>
       <c r="F11" t="n">
-        <v>20</v>
+        <v>20.8</v>
       </c>
       <c r="G11" t="n">
-        <v>17.4</v>
+        <v>18.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.94</v>
       </c>
       <c r="E12" t="n">
-        <v>20</v>
+        <v>20.8</v>
       </c>
       <c r="F12" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>12</v>
+        <v>13.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>2.55</v>
       </c>
       <c r="E13" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="F13" t="n">
-        <v>11.4</v>
+        <v>12.5</v>
       </c>
       <c r="G13" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.36</v>
       </c>
       <c r="E14" t="n">
-        <v>21.4</v>
+        <v>22.2</v>
       </c>
       <c r="F14" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="G14" t="n">
-        <v>9.4</v>
+        <v>10.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.2</v>
       </c>
       <c r="E15" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="F15" t="n">
-        <v>10</v>
+        <v>11.1</v>
       </c>
       <c r="G15" t="n">
-        <v>8.699999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.15</v>
       </c>
       <c r="E16" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.69</v>
       </c>
       <c r="E17" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="F17" t="n">
-        <v>7.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>6.7</v>
+        <v>7.9</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="F18" t="n">
-        <v>7.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>6.7</v>
+        <v>7.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.59</v>
       </c>
       <c r="E19" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F19" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="G19" t="n">
-        <v>6.6</v>
+        <v>7.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.72</v>
       </c>
       <c r="E20" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="G20" t="n">
-        <v>6.6</v>
+        <v>7.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="F21" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="G21" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.24</v>
       </c>
       <c r="E22" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="F22" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="G22" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.13</v>
       </c>
       <c r="E23" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="G23" t="n">
-        <v>5.6</v>
+        <v>6.8</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.7</v>
       </c>
       <c r="E24" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="G24" t="n">
-        <v>5.6</v>
+        <v>6.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.33</v>
       </c>
       <c r="E25" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="F25" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="G25" t="n">
-        <v>4.7</v>
+        <v>6</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.36</v>
       </c>
       <c r="E26" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="F26" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="G26" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.18</v>
       </c>
       <c r="E27" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="F27" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="G27" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.45</v>
       </c>
       <c r="E28" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="F28" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="G28" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>2.45</v>
       </c>
       <c r="E29" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="F29" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="G29" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>4.06</v>
       </c>
       <c r="E30" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="F30" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="G30" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.93</v>
       </c>
       <c r="E31" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="F31" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="G31" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.67</v>
       </c>
       <c r="E32" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="F32" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="G32" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun May 31 11:20:58 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.03</v>
       </c>
       <c r="E2" t="n">
-        <v>98.59999999999999</v>
+        <v>97.3</v>
       </c>
       <c r="F2" t="n">
-        <v>98.59999999999999</v>
+        <v>97.3</v>
       </c>
       <c r="G2" t="n">
-        <v>98.59999999999999</v>
+        <v>97.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.08</v>
       </c>
       <c r="E3" t="n">
-        <v>95.8</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>95.8</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>95.8</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.15</v>
       </c>
       <c r="E4" t="n">
-        <v>95.8</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>95.8</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>95.8</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>7.66</v>
       </c>
       <c r="E5" t="n">
-        <v>93.09999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>93.09999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>93.09999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.74</v>
       </c>
       <c r="E6" t="n">
-        <v>70.8</v>
+        <v>70.3</v>
       </c>
       <c r="F6" t="n">
-        <v>61.1</v>
+        <v>60.8</v>
       </c>
       <c r="G6" t="n">
-        <v>66</v>
+        <v>65.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>3.47</v>
       </c>
       <c r="E7" t="n">
-        <v>56.9</v>
+        <v>56.8</v>
       </c>
       <c r="F7" t="n">
-        <v>56.9</v>
+        <v>56.8</v>
       </c>
       <c r="G7" t="n">
-        <v>56.9</v>
+        <v>56.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>3.63</v>
       </c>
       <c r="E8" t="n">
-        <v>56.9</v>
+        <v>56.8</v>
       </c>
       <c r="F8" t="n">
-        <v>22.2</v>
+        <v>23</v>
       </c>
       <c r="G8" t="n">
-        <v>32.6</v>
+        <v>33.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>4.59</v>
       </c>
       <c r="E9" t="n">
-        <v>23.6</v>
+        <v>24.3</v>
       </c>
       <c r="F9" t="n">
-        <v>23.6</v>
+        <v>24.3</v>
       </c>
       <c r="G9" t="n">
-        <v>23.6</v>
+        <v>24.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>0.64</v>
       </c>
       <c r="E10" t="n">
-        <v>16.7</v>
+        <v>17.6</v>
       </c>
       <c r="F10" t="n">
-        <v>22.2</v>
+        <v>23</v>
       </c>
       <c r="G10" t="n">
-        <v>20.6</v>
+        <v>21.4</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.08</v>
       </c>
       <c r="E11" t="n">
-        <v>12.5</v>
+        <v>13.5</v>
       </c>
       <c r="F11" t="n">
-        <v>20.8</v>
+        <v>21.6</v>
       </c>
       <c r="G11" t="n">
-        <v>18.3</v>
+        <v>19.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.94</v>
       </c>
       <c r="E12" t="n">
-        <v>20.8</v>
+        <v>21.6</v>
       </c>
       <c r="F12" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="G12" t="n">
-        <v>13.1</v>
+        <v>14.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>2.55</v>
       </c>
       <c r="E13" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="F13" t="n">
-        <v>12.5</v>
+        <v>13.5</v>
       </c>
       <c r="G13" t="n">
-        <v>10.8</v>
+        <v>11.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.36</v>
       </c>
       <c r="E14" t="n">
-        <v>22.2</v>
+        <v>23</v>
       </c>
       <c r="F14" t="n">
-        <v>5.6</v>
+        <v>6.8</v>
       </c>
       <c r="G14" t="n">
-        <v>10.6</v>
+        <v>11.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.2</v>
       </c>
       <c r="E15" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="F15" t="n">
-        <v>11.1</v>
+        <v>12.2</v>
       </c>
       <c r="G15" t="n">
-        <v>9.9</v>
+        <v>10.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.15</v>
       </c>
       <c r="E16" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="F16" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="G16" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.69</v>
       </c>
       <c r="E17" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="F17" t="n">
-        <v>8.300000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="G17" t="n">
-        <v>7.9</v>
+        <v>9.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="F18" t="n">
-        <v>8.300000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="G18" t="n">
-        <v>7.9</v>
+        <v>9.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.59</v>
       </c>
       <c r="E19" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="F19" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="G19" t="n">
-        <v>7.8</v>
+        <v>8.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.72</v>
       </c>
       <c r="E20" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="F20" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="G20" t="n">
-        <v>7.8</v>
+        <v>8.9</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="F21" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="G21" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.24</v>
       </c>
       <c r="E22" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="F22" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="G22" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>2.13</v>
       </c>
       <c r="E23" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="F23" t="n">
-        <v>5.6</v>
+        <v>6.8</v>
       </c>
       <c r="G23" t="n">
-        <v>6.8</v>
+        <v>8</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.7</v>
       </c>
       <c r="E24" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="F24" t="n">
-        <v>5.6</v>
+        <v>6.8</v>
       </c>
       <c r="G24" t="n">
-        <v>6.8</v>
+        <v>8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.33</v>
       </c>
       <c r="E25" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="F25" t="n">
-        <v>5.6</v>
+        <v>6.8</v>
       </c>
       <c r="G25" t="n">
-        <v>6</v>
+        <v>7.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.36</v>
       </c>
       <c r="E26" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="F26" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="G26" t="n">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.18</v>
       </c>
       <c r="E27" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="F27" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="G27" t="n">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.45</v>
       </c>
       <c r="E28" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="F28" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="G28" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>2.45</v>
       </c>
       <c r="E29" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="F29" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="G29" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>4.06</v>
       </c>
       <c r="E30" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="F30" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="G30" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.93</v>
       </c>
       <c r="E31" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="F31" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="G31" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.67</v>
       </c>
       <c r="E32" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="F32" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="G32" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Jun  1 15:43:46 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,52 +486,52 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>21.69</v>
+        <v>22</v>
       </c>
       <c r="D2" t="n">
-        <v>2.03</v>
+        <v>2.06</v>
       </c>
       <c r="E2" t="n">
-        <v>97.3</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>97.3</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>97.3</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>32.5</v>
+        <v>20.03</v>
       </c>
       <c r="D3" t="n">
-        <v>3.08</v>
+        <v>1.83</v>
       </c>
       <c r="E3" t="n">
-        <v>94.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>94.59999999999999</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>94.59999999999999</v>
+        <v>98.7</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +546,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>38.51</v>
+        <v>36.8</v>
       </c>
       <c r="D4" t="n">
-        <v>2.15</v>
+        <v>2.06</v>
       </c>
       <c r="E4" t="n">
-        <v>94.59999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="F4" t="n">
-        <v>94.59999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="G4" t="n">
-        <v>94.59999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="5">
@@ -576,112 +576,112 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>73.81</v>
+        <v>70.81</v>
       </c>
       <c r="D5" t="n">
-        <v>7.66</v>
+        <v>7.35</v>
       </c>
       <c r="E5" t="n">
-        <v>91.90000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="F5" t="n">
-        <v>91.90000000000001</v>
+        <v>76.3</v>
       </c>
       <c r="G5" t="n">
-        <v>91.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>18.96</v>
+        <v>31.72</v>
       </c>
       <c r="D6" t="n">
-        <v>1.74</v>
+        <v>3.01</v>
       </c>
       <c r="E6" t="n">
-        <v>70.3</v>
+        <v>73.7</v>
       </c>
       <c r="F6" t="n">
-        <v>60.8</v>
+        <v>73.7</v>
       </c>
       <c r="G6" t="n">
-        <v>65.5</v>
+        <v>73.7</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>40.95</v>
+        <v>6.84</v>
       </c>
       <c r="D7" t="n">
-        <v>3.47</v>
+        <v>0.65</v>
       </c>
       <c r="E7" t="n">
-        <v>56.8</v>
+        <v>51.3</v>
       </c>
       <c r="F7" t="n">
-        <v>56.8</v>
+        <v>53.9</v>
       </c>
       <c r="G7" t="n">
-        <v>56.8</v>
+        <v>52.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20.76</v>
+        <v>40.45</v>
       </c>
       <c r="D8" t="n">
-        <v>3.63</v>
+        <v>3.42</v>
       </c>
       <c r="E8" t="n">
-        <v>56.8</v>
+        <v>44.7</v>
       </c>
       <c r="F8" t="n">
-        <v>23</v>
+        <v>44.7</v>
       </c>
       <c r="G8" t="n">
-        <v>33.1</v>
+        <v>44.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="9">
@@ -696,52 +696,52 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>121.94</v>
+        <v>123.15</v>
       </c>
       <c r="D9" t="n">
-        <v>4.59</v>
+        <v>4.63</v>
       </c>
       <c r="E9" t="n">
-        <v>24.3</v>
+        <v>28.9</v>
       </c>
       <c r="F9" t="n">
-        <v>24.3</v>
+        <v>28.9</v>
       </c>
       <c r="G9" t="n">
-        <v>24.3</v>
+        <v>28.9</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6.75</v>
+        <v>30.77</v>
       </c>
       <c r="D10" t="n">
-        <v>0.64</v>
+        <v>2.61</v>
       </c>
       <c r="E10" t="n">
-        <v>17.6</v>
+        <v>26.3</v>
       </c>
       <c r="F10" t="n">
-        <v>23</v>
+        <v>30.3</v>
       </c>
       <c r="G10" t="n">
-        <v>21.4</v>
+        <v>28.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="11">
@@ -756,502 +756,502 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>11.94</v>
+        <v>12.05</v>
       </c>
       <c r="D11" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="E11" t="n">
-        <v>13.5</v>
+        <v>21.1</v>
       </c>
       <c r="F11" t="n">
-        <v>21.6</v>
+        <v>31.6</v>
       </c>
       <c r="G11" t="n">
-        <v>19.2</v>
+        <v>26.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>36.47</v>
+        <v>29.05</v>
       </c>
       <c r="D12" t="n">
-        <v>3.94</v>
+        <v>2.19</v>
       </c>
       <c r="E12" t="n">
-        <v>21.6</v>
+        <v>26.3</v>
       </c>
       <c r="F12" t="n">
-        <v>10.8</v>
+        <v>26.3</v>
       </c>
       <c r="G12" t="n">
-        <v>14.1</v>
+        <v>26.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>30.08</v>
+        <v>20.69</v>
       </c>
       <c r="D13" t="n">
-        <v>2.55</v>
+        <v>3.61</v>
       </c>
       <c r="E13" t="n">
-        <v>8.1</v>
+        <v>39.5</v>
       </c>
       <c r="F13" t="n">
-        <v>13.5</v>
+        <v>18.4</v>
       </c>
       <c r="G13" t="n">
-        <v>11.9</v>
+        <v>24.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.9</v>
+        <v>26.84</v>
       </c>
       <c r="D14" t="n">
-        <v>2.36</v>
+        <v>2.21</v>
       </c>
       <c r="E14" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>25</v>
+      </c>
+      <c r="G14" t="n">
         <v>23</v>
       </c>
-      <c r="F14" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="G14" t="n">
-        <v>11.6</v>
-      </c>
       <c r="H14" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9.869999999999999</v>
+        <v>24.48</v>
       </c>
       <c r="D15" t="n">
-        <v>1.2</v>
+        <v>2.02</v>
       </c>
       <c r="E15" t="n">
-        <v>8.1</v>
+        <v>13.2</v>
       </c>
       <c r="F15" t="n">
-        <v>12.2</v>
+        <v>21.1</v>
       </c>
       <c r="G15" t="n">
-        <v>10.9</v>
+        <v>18.7</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>28.53</v>
+        <v>14.22</v>
       </c>
       <c r="D16" t="n">
-        <v>2.15</v>
+        <v>1.34</v>
       </c>
       <c r="E16" t="n">
-        <v>10.8</v>
+        <v>15.8</v>
       </c>
       <c r="F16" t="n">
-        <v>10.8</v>
+        <v>14.5</v>
       </c>
       <c r="G16" t="n">
-        <v>10.8</v>
+        <v>14.9</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>21.61</v>
+        <v>15.92</v>
       </c>
       <c r="D17" t="n">
-        <v>3.69</v>
+        <v>2.36</v>
       </c>
       <c r="E17" t="n">
-        <v>8.1</v>
+        <v>28.9</v>
       </c>
       <c r="F17" t="n">
-        <v>9.5</v>
+        <v>7.9</v>
       </c>
       <c r="G17" t="n">
-        <v>9.1</v>
+        <v>14.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>17.86</v>
+        <v>15.3</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E18" t="n">
-        <v>8.1</v>
+        <v>13.2</v>
       </c>
       <c r="F18" t="n">
-        <v>9.5</v>
+        <v>14.5</v>
       </c>
       <c r="G18" t="n">
-        <v>9.1</v>
+        <v>14.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>27.85</v>
+        <v>20.4</v>
       </c>
       <c r="D19" t="n">
-        <v>2.59</v>
+        <v>1.73</v>
       </c>
       <c r="E19" t="n">
-        <v>10.8</v>
+        <v>15.8</v>
       </c>
       <c r="F19" t="n">
-        <v>8.1</v>
+        <v>13.2</v>
       </c>
       <c r="G19" t="n">
-        <v>8.9</v>
+        <v>13.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>11.21</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="D20" t="n">
-        <v>0.72</v>
+        <v>1.2</v>
       </c>
       <c r="E20" t="n">
-        <v>10.8</v>
+        <v>13.2</v>
       </c>
       <c r="F20" t="n">
-        <v>8.1</v>
+        <v>13.2</v>
       </c>
       <c r="G20" t="n">
-        <v>8.9</v>
+        <v>13.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>24.16</v>
+        <v>24.28</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>2.21</v>
       </c>
       <c r="E21" t="n">
-        <v>8.1</v>
+        <v>15.8</v>
       </c>
       <c r="F21" t="n">
-        <v>8.1</v>
+        <v>11.8</v>
       </c>
       <c r="G21" t="n">
-        <v>8.1</v>
+        <v>13</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>15.2</v>
+        <v>32.18</v>
       </c>
       <c r="D22" t="n">
-        <v>1.24</v>
+        <v>2.47</v>
       </c>
       <c r="E22" t="n">
-        <v>8.1</v>
+        <v>11.8</v>
       </c>
       <c r="F22" t="n">
-        <v>8.1</v>
+        <v>11.8</v>
       </c>
       <c r="G22" t="n">
-        <v>8.1</v>
+        <v>11.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>25.98</v>
+        <v>17.89</v>
       </c>
       <c r="D23" t="n">
-        <v>2.13</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>10.8</v>
+        <v>13.2</v>
       </c>
       <c r="F23" t="n">
-        <v>6.8</v>
+        <v>10.5</v>
       </c>
       <c r="G23" t="n">
-        <v>8</v>
+        <v>11.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>20.03</v>
+        <v>49.31</v>
       </c>
       <c r="D24" t="n">
-        <v>1.7</v>
+        <v>4.12</v>
       </c>
       <c r="E24" t="n">
-        <v>10.8</v>
+        <v>13.2</v>
       </c>
       <c r="F24" t="n">
-        <v>6.8</v>
+        <v>10.5</v>
       </c>
       <c r="G24" t="n">
-        <v>8</v>
+        <v>11.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>14.13</v>
+        <v>11.25</v>
       </c>
       <c r="D25" t="n">
-        <v>1.33</v>
+        <v>0.72</v>
       </c>
       <c r="E25" t="n">
-        <v>8.1</v>
+        <v>15.8</v>
       </c>
       <c r="F25" t="n">
-        <v>6.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G25" t="n">
-        <v>7.2</v>
+        <v>11.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25.45</v>
+        <v>36.32</v>
       </c>
       <c r="D26" t="n">
-        <v>2.36</v>
+        <v>3.93</v>
       </c>
       <c r="E26" t="n">
-        <v>8.1</v>
+        <v>18.4</v>
       </c>
       <c r="F26" t="n">
-        <v>5.4</v>
+        <v>7.9</v>
       </c>
       <c r="G26" t="n">
-        <v>6.2</v>
+        <v>11.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>23.97</v>
+        <v>22.72</v>
       </c>
       <c r="D27" t="n">
-        <v>2.18</v>
+        <v>1.68</v>
       </c>
       <c r="E27" t="n">
-        <v>8.1</v>
+        <v>10.5</v>
       </c>
       <c r="F27" t="n">
-        <v>5.4</v>
+        <v>10.5</v>
       </c>
       <c r="G27" t="n">
-        <v>6.2</v>
+        <v>10.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="28">
@@ -1266,142 +1266,142 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>26.49</v>
+        <v>26.85</v>
       </c>
       <c r="D28" t="n">
-        <v>2.45</v>
+        <v>2.48</v>
       </c>
       <c r="E28" t="n">
-        <v>5.4</v>
+        <v>10.5</v>
       </c>
       <c r="F28" t="n">
-        <v>5.4</v>
+        <v>10.5</v>
       </c>
       <c r="G28" t="n">
-        <v>5.4</v>
+        <v>10.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>31.99</v>
+        <v>27.67</v>
       </c>
       <c r="D29" t="n">
-        <v>2.45</v>
+        <v>2.57</v>
       </c>
       <c r="E29" t="n">
-        <v>5.4</v>
+        <v>7.9</v>
       </c>
       <c r="F29" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="G29" t="n">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>48.55</v>
+        <v>21.41</v>
       </c>
       <c r="D30" t="n">
-        <v>4.06</v>
+        <v>3.66</v>
       </c>
       <c r="E30" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="F30" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="G30" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>60.34</v>
+        <v>25.25</v>
       </c>
       <c r="D31" t="n">
-        <v>3.93</v>
+        <v>2.35</v>
       </c>
       <c r="E31" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="F31" t="n">
-        <v>5.4</v>
+        <v>2.6</v>
       </c>
       <c r="G31" t="n">
-        <v>5.4</v>
+        <v>3.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>22.58</v>
+        <v>59.42</v>
       </c>
       <c r="D32" t="n">
-        <v>1.67</v>
+        <v>3.87</v>
       </c>
       <c r="E32" t="n">
-        <v>5.4</v>
+        <v>2.6</v>
       </c>
       <c r="F32" t="n">
-        <v>5.4</v>
+        <v>2.6</v>
       </c>
       <c r="G32" t="n">
-        <v>5.4</v>
+        <v>2.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Jun  2 13:01:59 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22</v>
+        <v>33.11</v>
       </c>
       <c r="D2" t="n">
-        <v>2.06</v>
+        <v>3.14</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,127 +501,127 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.03</v>
+        <v>21.82</v>
       </c>
       <c r="D3" t="n">
-        <v>1.83</v>
+        <v>2.04</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="F3" t="n">
         <v>97.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>98.7</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>36.8</v>
+        <v>19.75</v>
       </c>
       <c r="D4" t="n">
-        <v>2.06</v>
+        <v>1.81</v>
       </c>
       <c r="E4" t="n">
-        <v>86.8</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>86.8</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>86.8</v>
+        <v>96.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>70.81</v>
+        <v>37.39</v>
       </c>
       <c r="D5" t="n">
-        <v>7.35</v>
+        <v>2.09</v>
       </c>
       <c r="E5" t="n">
-        <v>73.7</v>
+        <v>87.2</v>
       </c>
       <c r="F5" t="n">
-        <v>76.3</v>
+        <v>88.5</v>
       </c>
       <c r="G5" t="n">
-        <v>75</v>
+        <v>87.8</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>31.72</v>
+        <v>72.94</v>
       </c>
       <c r="D6" t="n">
-        <v>3.01</v>
+        <v>7.57</v>
       </c>
       <c r="E6" t="n">
-        <v>73.7</v>
+        <v>87.2</v>
       </c>
       <c r="F6" t="n">
-        <v>73.7</v>
+        <v>87.2</v>
       </c>
       <c r="G6" t="n">
-        <v>73.7</v>
+        <v>87.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="7">
@@ -636,22 +636,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6.84</v>
+        <v>6.87</v>
       </c>
       <c r="D7" t="n">
         <v>0.65</v>
       </c>
       <c r="E7" t="n">
-        <v>51.3</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>53.9</v>
+        <v>53.8</v>
       </c>
       <c r="G7" t="n">
-        <v>52.6</v>
+        <v>60.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="8">
@@ -666,712 +666,712 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>40.45</v>
+        <v>40.96</v>
       </c>
       <c r="D8" t="n">
-        <v>3.42</v>
+        <v>3.47</v>
       </c>
       <c r="E8" t="n">
-        <v>44.7</v>
+        <v>61.5</v>
       </c>
       <c r="F8" t="n">
-        <v>44.7</v>
+        <v>57.7</v>
       </c>
       <c r="G8" t="n">
-        <v>44.7</v>
+        <v>59.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>123.15</v>
+        <v>22.12</v>
       </c>
       <c r="D9" t="n">
-        <v>4.63</v>
+        <v>3.78</v>
       </c>
       <c r="E9" t="n">
-        <v>28.9</v>
+        <v>33.3</v>
       </c>
       <c r="F9" t="n">
-        <v>28.9</v>
+        <v>46.2</v>
       </c>
       <c r="G9" t="n">
-        <v>28.9</v>
+        <v>39.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>30.77</v>
+        <v>20.47</v>
       </c>
       <c r="D10" t="n">
-        <v>2.61</v>
+        <v>3.58</v>
       </c>
       <c r="E10" t="n">
-        <v>26.3</v>
+        <v>38.5</v>
       </c>
       <c r="F10" t="n">
-        <v>30.3</v>
+        <v>15.4</v>
       </c>
       <c r="G10" t="n">
-        <v>28.3</v>
+        <v>22.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>12.05</v>
+        <v>16.04</v>
       </c>
       <c r="D11" t="n">
-        <v>1.09</v>
+        <v>2.38</v>
       </c>
       <c r="E11" t="n">
-        <v>21.1</v>
+        <v>30.8</v>
       </c>
       <c r="F11" t="n">
-        <v>31.6</v>
+        <v>16.7</v>
       </c>
       <c r="G11" t="n">
-        <v>26.3</v>
+        <v>20.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>29.05</v>
+        <v>121.81</v>
       </c>
       <c r="D12" t="n">
-        <v>2.19</v>
+        <v>4.58</v>
       </c>
       <c r="E12" t="n">
-        <v>26.3</v>
+        <v>20.5</v>
       </c>
       <c r="F12" t="n">
-        <v>26.3</v>
+        <v>20.5</v>
       </c>
       <c r="G12" t="n">
-        <v>26.3</v>
+        <v>20.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>20.69</v>
+        <v>15.23</v>
       </c>
       <c r="D13" t="n">
-        <v>3.61</v>
+        <v>1.25</v>
       </c>
       <c r="E13" t="n">
-        <v>39.5</v>
+        <v>12.8</v>
       </c>
       <c r="F13" t="n">
-        <v>18.4</v>
+        <v>15.4</v>
       </c>
       <c r="G13" t="n">
-        <v>24.7</v>
+        <v>14.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>26.84</v>
+        <v>11.84</v>
       </c>
       <c r="D14" t="n">
-        <v>2.21</v>
+        <v>1.07</v>
       </c>
       <c r="E14" t="n">
-        <v>18.4</v>
+        <v>7.7</v>
       </c>
       <c r="F14" t="n">
-        <v>25</v>
+        <v>16.7</v>
       </c>
       <c r="G14" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>24.48</v>
+        <v>20.16</v>
       </c>
       <c r="D15" t="n">
-        <v>2.02</v>
+        <v>1.71</v>
       </c>
       <c r="E15" t="n">
-        <v>13.2</v>
+        <v>15.4</v>
       </c>
       <c r="F15" t="n">
-        <v>21.1</v>
+        <v>12.8</v>
       </c>
       <c r="G15" t="n">
-        <v>18.7</v>
+        <v>13.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14.22</v>
+        <v>26.12</v>
       </c>
       <c r="D16" t="n">
-        <v>1.34</v>
+        <v>2.15</v>
       </c>
       <c r="E16" t="n">
-        <v>15.8</v>
+        <v>15.4</v>
       </c>
       <c r="F16" t="n">
-        <v>14.5</v>
+        <v>12.8</v>
       </c>
       <c r="G16" t="n">
-        <v>14.9</v>
+        <v>13.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>15.92</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="D17" t="n">
-        <v>2.36</v>
+        <v>1.2</v>
       </c>
       <c r="E17" t="n">
-        <v>28.9</v>
+        <v>9</v>
       </c>
       <c r="F17" t="n">
-        <v>7.9</v>
+        <v>14.1</v>
       </c>
       <c r="G17" t="n">
-        <v>14.2</v>
+        <v>12.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>15.3</v>
+        <v>26.84</v>
       </c>
       <c r="D18" t="n">
-        <v>1.25</v>
+        <v>2.48</v>
       </c>
       <c r="E18" t="n">
-        <v>13.2</v>
+        <v>10.3</v>
       </c>
       <c r="F18" t="n">
-        <v>14.5</v>
+        <v>11.5</v>
       </c>
       <c r="G18" t="n">
-        <v>14.1</v>
+        <v>11.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20.4</v>
+        <v>49.17</v>
       </c>
       <c r="D19" t="n">
-        <v>1.73</v>
+        <v>4.11</v>
       </c>
       <c r="E19" t="n">
-        <v>15.8</v>
+        <v>12.8</v>
       </c>
       <c r="F19" t="n">
-        <v>13.2</v>
+        <v>10.3</v>
       </c>
       <c r="G19" t="n">
-        <v>13.9</v>
+        <v>11</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>9.880000000000001</v>
+        <v>36.29</v>
       </c>
       <c r="D20" t="n">
-        <v>1.2</v>
+        <v>3.92</v>
       </c>
       <c r="E20" t="n">
-        <v>13.2</v>
+        <v>17.9</v>
       </c>
       <c r="F20" t="n">
-        <v>13.2</v>
+        <v>6.4</v>
       </c>
       <c r="G20" t="n">
-        <v>13.2</v>
+        <v>9.9</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>24.28</v>
+        <v>14.15</v>
       </c>
       <c r="D21" t="n">
-        <v>2.21</v>
+        <v>1.33</v>
       </c>
       <c r="E21" t="n">
-        <v>15.8</v>
+        <v>12.8</v>
       </c>
       <c r="F21" t="n">
-        <v>11.8</v>
+        <v>7.7</v>
       </c>
       <c r="G21" t="n">
-        <v>13</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>32.18</v>
+        <v>25.42</v>
       </c>
       <c r="D22" t="n">
-        <v>2.47</v>
+        <v>2.36</v>
       </c>
       <c r="E22" t="n">
-        <v>11.8</v>
+        <v>7.7</v>
       </c>
       <c r="F22" t="n">
-        <v>11.8</v>
+        <v>9</v>
       </c>
       <c r="G22" t="n">
-        <v>11.8</v>
+        <v>8.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>17.89</v>
+        <v>22.58</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>1.67</v>
       </c>
       <c r="E23" t="n">
-        <v>13.2</v>
+        <v>6.4</v>
       </c>
       <c r="F23" t="n">
-        <v>10.5</v>
+        <v>6.4</v>
       </c>
       <c r="G23" t="n">
-        <v>11.3</v>
+        <v>6.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>49.31</v>
+        <v>23.88</v>
       </c>
       <c r="D24" t="n">
-        <v>4.12</v>
+        <v>2.18</v>
       </c>
       <c r="E24" t="n">
-        <v>13.2</v>
+        <v>5.1</v>
       </c>
       <c r="F24" t="n">
-        <v>10.5</v>
+        <v>6.4</v>
       </c>
       <c r="G24" t="n">
-        <v>11.3</v>
+        <v>6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>11.25</v>
+        <v>28.36</v>
       </c>
       <c r="D25" t="n">
-        <v>0.72</v>
+        <v>2.13</v>
       </c>
       <c r="E25" t="n">
-        <v>15.8</v>
+        <v>7.7</v>
       </c>
       <c r="F25" t="n">
-        <v>9.199999999999999</v>
+        <v>5.1</v>
       </c>
       <c r="G25" t="n">
-        <v>11.2</v>
+        <v>5.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>36.32</v>
+        <v>31.84</v>
       </c>
       <c r="D26" t="n">
-        <v>3.93</v>
+        <v>2.45</v>
       </c>
       <c r="E26" t="n">
-        <v>18.4</v>
+        <v>2.6</v>
       </c>
       <c r="F26" t="n">
-        <v>7.9</v>
+        <v>6.4</v>
       </c>
       <c r="G26" t="n">
-        <v>11.1</v>
+        <v>5.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.72</v>
+        <v>23.99</v>
       </c>
       <c r="D27" t="n">
-        <v>1.68</v>
+        <v>1.98</v>
       </c>
       <c r="E27" t="n">
-        <v>10.5</v>
+        <v>5.1</v>
       </c>
       <c r="F27" t="n">
-        <v>10.5</v>
+        <v>5.1</v>
       </c>
       <c r="G27" t="n">
-        <v>10.5</v>
+        <v>5.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>26.85</v>
+        <v>29.87</v>
       </c>
       <c r="D28" t="n">
-        <v>2.48</v>
+        <v>2.53</v>
       </c>
       <c r="E28" t="n">
-        <v>10.5</v>
+        <v>5.1</v>
       </c>
       <c r="F28" t="n">
-        <v>10.5</v>
+        <v>5.1</v>
       </c>
       <c r="G28" t="n">
-        <v>10.5</v>
+        <v>5.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>27.67</v>
+        <v>11.17</v>
       </c>
       <c r="D29" t="n">
-        <v>2.57</v>
+        <v>0.71</v>
       </c>
       <c r="E29" t="n">
-        <v>7.9</v>
+        <v>5.1</v>
       </c>
       <c r="F29" t="n">
-        <v>5.3</v>
+        <v>3.8</v>
       </c>
       <c r="G29" t="n">
-        <v>6.1</v>
+        <v>4.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>21.41</v>
+        <v>17.7</v>
       </c>
       <c r="D30" t="n">
-        <v>3.66</v>
+        <v>0.99</v>
       </c>
       <c r="E30" t="n">
-        <v>5.3</v>
+        <v>2.6</v>
       </c>
       <c r="F30" t="n">
-        <v>5.3</v>
+        <v>3.8</v>
       </c>
       <c r="G30" t="n">
-        <v>5.3</v>
+        <v>3.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>25.25</v>
+        <v>27.24</v>
       </c>
       <c r="D31" t="n">
-        <v>2.35</v>
+        <v>2.53</v>
       </c>
       <c r="E31" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="F31" t="n">
         <v>2.6</v>
       </c>
       <c r="G31" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="32">
@@ -1386,10 +1386,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>59.42</v>
+        <v>59.22</v>
       </c>
       <c r="D32" t="n">
-        <v>3.87</v>
+        <v>3.86</v>
       </c>
       <c r="E32" t="n">
         <v>2.6</v>
@@ -1401,7 +1401,7 @@
         <v>2.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Jun  3 14:17:13 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>33.11</v>
+        <v>34.2</v>
       </c>
       <c r="D2" t="n">
-        <v>3.14</v>
+        <v>3.25</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,187 +501,187 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>21.82</v>
+        <v>20.46</v>
       </c>
       <c r="D3" t="n">
-        <v>2.04</v>
+        <v>1.86</v>
       </c>
       <c r="E3" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>97.40000000000001</v>
+        <v>98.8</v>
       </c>
       <c r="G3" t="n">
-        <v>97.40000000000001</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>19.75</v>
+        <v>21.9</v>
       </c>
       <c r="D4" t="n">
-        <v>1.81</v>
+        <v>2.05</v>
       </c>
       <c r="E4" t="n">
-        <v>97.40000000000001</v>
+        <v>97.5</v>
       </c>
       <c r="F4" t="n">
-        <v>94.90000000000001</v>
+        <v>97.5</v>
       </c>
       <c r="G4" t="n">
-        <v>96.2</v>
+        <v>97.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>37.39</v>
+        <v>74.45999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>2.09</v>
+        <v>7.73</v>
       </c>
       <c r="E5" t="n">
-        <v>87.2</v>
+        <v>95</v>
       </c>
       <c r="F5" t="n">
-        <v>88.5</v>
+        <v>95</v>
       </c>
       <c r="G5" t="n">
-        <v>87.8</v>
+        <v>95</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>72.94</v>
+        <v>36.62</v>
       </c>
       <c r="D6" t="n">
-        <v>7.57</v>
+        <v>2.05</v>
       </c>
       <c r="E6" t="n">
-        <v>87.2</v>
+        <v>80</v>
       </c>
       <c r="F6" t="n">
-        <v>87.2</v>
+        <v>82.5</v>
       </c>
       <c r="G6" t="n">
-        <v>87.2</v>
+        <v>81.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6.87</v>
+        <v>41.41</v>
       </c>
       <c r="D7" t="n">
-        <v>0.65</v>
+        <v>3.51</v>
       </c>
       <c r="E7" t="n">
-        <v>67.90000000000001</v>
+        <v>65</v>
       </c>
       <c r="F7" t="n">
-        <v>53.8</v>
+        <v>78.8</v>
       </c>
       <c r="G7" t="n">
-        <v>60.9</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>40.96</v>
+        <v>6.81</v>
       </c>
       <c r="D8" t="n">
-        <v>3.47</v>
+        <v>0.65</v>
       </c>
       <c r="E8" t="n">
-        <v>61.5</v>
+        <v>42.5</v>
       </c>
       <c r="F8" t="n">
-        <v>57.7</v>
+        <v>53.8</v>
       </c>
       <c r="G8" t="n">
-        <v>59.6</v>
+        <v>48.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="9">
@@ -696,82 +696,82 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>22.12</v>
+        <v>22.27</v>
       </c>
       <c r="D9" t="n">
-        <v>3.78</v>
+        <v>3.8</v>
       </c>
       <c r="E9" t="n">
-        <v>33.3</v>
+        <v>37.5</v>
       </c>
       <c r="F9" t="n">
-        <v>46.2</v>
+        <v>47.5</v>
       </c>
       <c r="G9" t="n">
-        <v>39.7</v>
+        <v>42.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>20.47</v>
+        <v>15.99</v>
       </c>
       <c r="D10" t="n">
-        <v>3.58</v>
+        <v>2.38</v>
       </c>
       <c r="E10" t="n">
-        <v>38.5</v>
+        <v>30</v>
       </c>
       <c r="F10" t="n">
-        <v>15.4</v>
+        <v>17.5</v>
       </c>
       <c r="G10" t="n">
-        <v>22.3</v>
+        <v>21.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16.04</v>
+        <v>14.42</v>
       </c>
       <c r="D11" t="n">
-        <v>2.38</v>
+        <v>1.36</v>
       </c>
       <c r="E11" t="n">
-        <v>30.8</v>
+        <v>20</v>
       </c>
       <c r="F11" t="n">
-        <v>16.7</v>
+        <v>20</v>
       </c>
       <c r="G11" t="n">
-        <v>20.9</v>
+        <v>20</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="12">
@@ -786,52 +786,52 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>121.81</v>
+        <v>119.5</v>
       </c>
       <c r="D12" t="n">
-        <v>4.58</v>
+        <v>4.5</v>
       </c>
       <c r="E12" t="n">
-        <v>20.5</v>
+        <v>20</v>
       </c>
       <c r="F12" t="n">
-        <v>20.5</v>
+        <v>20</v>
       </c>
       <c r="G12" t="n">
-        <v>20.5</v>
+        <v>20</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>15.23</v>
+        <v>26.87</v>
       </c>
       <c r="D13" t="n">
-        <v>1.25</v>
+        <v>2.49</v>
       </c>
       <c r="E13" t="n">
-        <v>12.8</v>
+        <v>15</v>
       </c>
       <c r="F13" t="n">
-        <v>15.4</v>
+        <v>15</v>
       </c>
       <c r="G13" t="n">
-        <v>14.6</v>
+        <v>15</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="14">
@@ -846,232 +846,232 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11.84</v>
+        <v>11.6</v>
       </c>
       <c r="D14" t="n">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
       <c r="E14" t="n">
-        <v>7.7</v>
+        <v>2.5</v>
       </c>
       <c r="F14" t="n">
-        <v>16.7</v>
+        <v>15</v>
       </c>
       <c r="G14" t="n">
-        <v>14</v>
+        <v>11.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>20.16</v>
+        <v>48.71</v>
       </c>
       <c r="D15" t="n">
-        <v>1.71</v>
+        <v>4.07</v>
       </c>
       <c r="E15" t="n">
-        <v>15.4</v>
+        <v>10</v>
       </c>
       <c r="F15" t="n">
-        <v>12.8</v>
+        <v>10</v>
       </c>
       <c r="G15" t="n">
-        <v>13.6</v>
+        <v>10</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26.12</v>
+        <v>59.74</v>
       </c>
       <c r="D16" t="n">
-        <v>2.15</v>
+        <v>3.9</v>
       </c>
       <c r="E16" t="n">
-        <v>15.4</v>
+        <v>7.5</v>
       </c>
       <c r="F16" t="n">
-        <v>12.8</v>
+        <v>7.5</v>
       </c>
       <c r="G16" t="n">
-        <v>13.6</v>
+        <v>7.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>9.869999999999999</v>
+        <v>20.13</v>
       </c>
       <c r="D17" t="n">
-        <v>1.2</v>
+        <v>3.53</v>
       </c>
       <c r="E17" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F17" t="n">
-        <v>14.1</v>
+        <v>5</v>
       </c>
       <c r="G17" t="n">
-        <v>12.6</v>
+        <v>5</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>26.84</v>
+        <v>29.33</v>
       </c>
       <c r="D18" t="n">
-        <v>2.48</v>
+        <v>2.49</v>
       </c>
       <c r="E18" t="n">
-        <v>10.3</v>
+        <v>5</v>
       </c>
       <c r="F18" t="n">
-        <v>11.5</v>
+        <v>5</v>
       </c>
       <c r="G18" t="n">
-        <v>11.2</v>
+        <v>5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>49.17</v>
+        <v>9.81</v>
       </c>
       <c r="D19" t="n">
-        <v>4.11</v>
+        <v>1.19</v>
       </c>
       <c r="E19" t="n">
-        <v>12.8</v>
+        <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>10.3</v>
+        <v>5</v>
       </c>
       <c r="G19" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>36.29</v>
+        <v>11.08</v>
       </c>
       <c r="D20" t="n">
-        <v>3.92</v>
+        <v>0.71</v>
       </c>
       <c r="E20" t="n">
-        <v>17.9</v>
+        <v>5</v>
       </c>
       <c r="F20" t="n">
-        <v>6.4</v>
+        <v>5</v>
       </c>
       <c r="G20" t="n">
-        <v>9.9</v>
+        <v>5</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>14.15</v>
+        <v>23.79</v>
       </c>
       <c r="D21" t="n">
-        <v>1.33</v>
+        <v>1.97</v>
       </c>
       <c r="E21" t="n">
-        <v>12.8</v>
+        <v>5</v>
       </c>
       <c r="F21" t="n">
-        <v>7.7</v>
+        <v>5</v>
       </c>
       <c r="G21" t="n">
-        <v>9.199999999999999</v>
+        <v>5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="22">
@@ -1086,82 +1086,82 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>25.42</v>
+        <v>25.23</v>
       </c>
       <c r="D22" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
       <c r="E22" t="n">
-        <v>7.7</v>
+        <v>5</v>
       </c>
       <c r="F22" t="n">
-        <v>9</v>
+        <v>3.8</v>
       </c>
       <c r="G22" t="n">
-        <v>8.6</v>
+        <v>4.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22.58</v>
+        <v>35.96</v>
       </c>
       <c r="D23" t="n">
-        <v>1.67</v>
+        <v>3.89</v>
       </c>
       <c r="E23" t="n">
-        <v>6.4</v>
+        <v>7.5</v>
       </c>
       <c r="F23" t="n">
-        <v>6.4</v>
+        <v>2.5</v>
       </c>
       <c r="G23" t="n">
-        <v>6.4</v>
+        <v>4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>23.88</v>
+        <v>14.99</v>
       </c>
       <c r="D24" t="n">
-        <v>2.18</v>
+        <v>1.23</v>
       </c>
       <c r="E24" t="n">
-        <v>5.1</v>
+        <v>2.5</v>
       </c>
       <c r="F24" t="n">
-        <v>6.4</v>
+        <v>3.8</v>
       </c>
       <c r="G24" t="n">
-        <v>6</v>
+        <v>3.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="25">
@@ -1176,142 +1176,142 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.36</v>
+        <v>28.05</v>
       </c>
       <c r="D25" t="n">
-        <v>2.13</v>
+        <v>2.11</v>
       </c>
       <c r="E25" t="n">
-        <v>7.7</v>
+        <v>5</v>
       </c>
       <c r="F25" t="n">
-        <v>5.1</v>
+        <v>2.5</v>
       </c>
       <c r="G25" t="n">
-        <v>5.9</v>
+        <v>3.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>31.84</v>
+        <v>25.77</v>
       </c>
       <c r="D26" t="n">
-        <v>2.45</v>
+        <v>2.12</v>
       </c>
       <c r="E26" t="n">
-        <v>2.6</v>
+        <v>5</v>
       </c>
       <c r="F26" t="n">
-        <v>6.4</v>
+        <v>2.5</v>
       </c>
       <c r="G26" t="n">
-        <v>5.3</v>
+        <v>3.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>23.99</v>
+        <v>19.87</v>
       </c>
       <c r="D27" t="n">
-        <v>1.98</v>
+        <v>1.69</v>
       </c>
       <c r="E27" t="n">
-        <v>5.1</v>
+        <v>5</v>
       </c>
       <c r="F27" t="n">
-        <v>5.1</v>
+        <v>2.5</v>
       </c>
       <c r="G27" t="n">
-        <v>5.1</v>
+        <v>3.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29.87</v>
+        <v>23.67</v>
       </c>
       <c r="D28" t="n">
-        <v>2.53</v>
+        <v>2.16</v>
       </c>
       <c r="E28" t="n">
-        <v>5.1</v>
+        <v>5</v>
       </c>
       <c r="F28" t="n">
-        <v>5.1</v>
+        <v>2.5</v>
       </c>
       <c r="G28" t="n">
-        <v>5.1</v>
+        <v>3.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>11.17</v>
+        <v>26.89</v>
       </c>
       <c r="D29" t="n">
-        <v>0.71</v>
+        <v>2.5</v>
       </c>
       <c r="E29" t="n">
-        <v>5.1</v>
+        <v>2.5</v>
       </c>
       <c r="F29" t="n">
-        <v>3.8</v>
+        <v>2.5</v>
       </c>
       <c r="G29" t="n">
-        <v>4.2</v>
+        <v>2.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="30">
@@ -1326,82 +1326,82 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>17.7</v>
+        <v>17.55</v>
       </c>
       <c r="D30" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="E30" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="F30" t="n">
-        <v>3.8</v>
+        <v>2.5</v>
       </c>
       <c r="G30" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>27.24</v>
+        <v>31.63</v>
       </c>
       <c r="D31" t="n">
-        <v>2.53</v>
+        <v>2.43</v>
       </c>
       <c r="E31" t="n">
-        <v>5.1</v>
+        <v>2.5</v>
       </c>
       <c r="F31" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="G31" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>59.22</v>
+        <v>22.5</v>
       </c>
       <c r="D32" t="n">
-        <v>3.86</v>
+        <v>1.66</v>
       </c>
       <c r="E32" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="F32" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="G32" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Jun  4 12:33:40 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>34.2</v>
+        <v>20.68</v>
       </c>
       <c r="D2" t="n">
-        <v>3.25</v>
+        <v>1.88</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,157 +501,157 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.46</v>
+        <v>34.45</v>
       </c>
       <c r="D3" t="n">
-        <v>1.86</v>
+        <v>3.27</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>98.8</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>21.9</v>
+        <v>75.83</v>
       </c>
       <c r="D4" t="n">
-        <v>2.05</v>
+        <v>7.87</v>
       </c>
       <c r="E4" t="n">
-        <v>97.5</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>97.5</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>97.5</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>74.45999999999999</v>
+        <v>21.63</v>
       </c>
       <c r="D5" t="n">
-        <v>7.73</v>
+        <v>2.02</v>
       </c>
       <c r="E5" t="n">
-        <v>95</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>95</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>95</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>36.62</v>
+        <v>41.96</v>
       </c>
       <c r="D6" t="n">
-        <v>2.05</v>
+        <v>3.56</v>
       </c>
       <c r="E6" t="n">
-        <v>80</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>82.5</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>81.2</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>41.41</v>
+        <v>36.5</v>
       </c>
       <c r="D7" t="n">
-        <v>3.51</v>
+        <v>2.05</v>
       </c>
       <c r="E7" t="n">
-        <v>65</v>
+        <v>73.2</v>
       </c>
       <c r="F7" t="n">
-        <v>78.8</v>
+        <v>81.7</v>
       </c>
       <c r="G7" t="n">
-        <v>71.90000000000001</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="8">
@@ -666,52 +666,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.81</v>
+        <v>6.75</v>
       </c>
       <c r="D8" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="E8" t="n">
-        <v>42.5</v>
+        <v>17.1</v>
       </c>
       <c r="F8" t="n">
-        <v>53.8</v>
+        <v>22</v>
       </c>
       <c r="G8" t="n">
-        <v>48.1</v>
+        <v>20.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>22.27</v>
+        <v>115.62</v>
       </c>
       <c r="D9" t="n">
-        <v>3.8</v>
+        <v>4.36</v>
       </c>
       <c r="E9" t="n">
-        <v>37.5</v>
+        <v>19.5</v>
       </c>
       <c r="F9" t="n">
-        <v>47.5</v>
+        <v>19.5</v>
       </c>
       <c r="G9" t="n">
-        <v>42.5</v>
+        <v>19.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="10">
@@ -726,502 +726,502 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>15.99</v>
+        <v>15.95</v>
       </c>
       <c r="D10" t="n">
-        <v>2.38</v>
+        <v>2.37</v>
       </c>
       <c r="E10" t="n">
-        <v>30</v>
+        <v>29.3</v>
       </c>
       <c r="F10" t="n">
-        <v>17.5</v>
+        <v>14.6</v>
       </c>
       <c r="G10" t="n">
-        <v>21.2</v>
+        <v>19</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>14.42</v>
+        <v>26.79</v>
       </c>
       <c r="D11" t="n">
-        <v>1.36</v>
+        <v>2.48</v>
       </c>
       <c r="E11" t="n">
-        <v>20</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>20</v>
+        <v>12.2</v>
       </c>
       <c r="G11" t="n">
-        <v>20</v>
+        <v>11.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>119.5</v>
+        <v>11.49</v>
       </c>
       <c r="D12" t="n">
-        <v>4.5</v>
+        <v>1.03</v>
       </c>
       <c r="E12" t="n">
-        <v>20</v>
+        <v>2.4</v>
       </c>
       <c r="F12" t="n">
-        <v>20</v>
+        <v>14.6</v>
       </c>
       <c r="G12" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>26.87</v>
+        <v>21.59</v>
       </c>
       <c r="D13" t="n">
-        <v>2.49</v>
+        <v>3.69</v>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>7.3</v>
       </c>
       <c r="F13" t="n">
-        <v>15</v>
+        <v>12.2</v>
       </c>
       <c r="G13" t="n">
-        <v>15</v>
+        <v>10.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11.6</v>
+        <v>59.91</v>
       </c>
       <c r="D14" t="n">
-        <v>1.05</v>
+        <v>3.91</v>
       </c>
       <c r="E14" t="n">
-        <v>2.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>15</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>11.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>48.71</v>
+        <v>14.14</v>
       </c>
       <c r="D15" t="n">
-        <v>4.07</v>
+        <v>1.33</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>12.2</v>
       </c>
       <c r="F15" t="n">
-        <v>10</v>
+        <v>8.5</v>
       </c>
       <c r="G15" t="n">
-        <v>10</v>
+        <v>9.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>59.74</v>
+        <v>9.68</v>
       </c>
       <c r="D16" t="n">
-        <v>3.9</v>
+        <v>1.18</v>
       </c>
       <c r="E16" t="n">
-        <v>7.5</v>
+        <v>2.4</v>
       </c>
       <c r="F16" t="n">
-        <v>7.5</v>
+        <v>3.7</v>
       </c>
       <c r="G16" t="n">
-        <v>7.5</v>
+        <v>3.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>20.13</v>
+        <v>27.3</v>
       </c>
       <c r="D17" t="n">
-        <v>3.53</v>
+        <v>2.06</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="F17" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="G17" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>29.33</v>
+        <v>10.98</v>
       </c>
       <c r="D18" t="n">
-        <v>2.49</v>
+        <v>0.7</v>
       </c>
       <c r="E18" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="G18" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>9.81</v>
+        <v>35.26</v>
       </c>
       <c r="D19" t="n">
-        <v>1.19</v>
+        <v>3.81</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="F19" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="G19" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>11.08</v>
+        <v>19.82</v>
       </c>
       <c r="D20" t="n">
-        <v>0.71</v>
+        <v>3.48</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="G20" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>23.79</v>
+        <v>25.18</v>
       </c>
       <c r="D21" t="n">
-        <v>1.97</v>
+        <v>2.34</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="F21" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="G21" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>25.23</v>
+        <v>23.23</v>
       </c>
       <c r="D22" t="n">
-        <v>2.35</v>
+        <v>2.15</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="F22" t="n">
-        <v>3.8</v>
+        <v>2.4</v>
       </c>
       <c r="G22" t="n">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>35.96</v>
+        <v>17.32</v>
       </c>
       <c r="D23" t="n">
-        <v>3.89</v>
+        <v>0.97</v>
       </c>
       <c r="E23" t="n">
-        <v>7.5</v>
+        <v>2.4</v>
       </c>
       <c r="F23" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="G23" t="n">
-        <v>4</v>
+        <v>2.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>14.99</v>
+        <v>26.56</v>
       </c>
       <c r="D24" t="n">
-        <v>1.23</v>
+        <v>2.47</v>
       </c>
       <c r="E24" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="F24" t="n">
-        <v>3.8</v>
+        <v>2.4</v>
       </c>
       <c r="G24" t="n">
-        <v>3.4</v>
+        <v>2.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.05</v>
+        <v>23.1</v>
       </c>
       <c r="D25" t="n">
-        <v>2.11</v>
+        <v>1.91</v>
       </c>
       <c r="E25" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="F25" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="G25" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25.77</v>
+        <v>14.8</v>
       </c>
       <c r="D26" t="n">
-        <v>2.12</v>
+        <v>1.21</v>
       </c>
       <c r="E26" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="F26" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="G26" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="27">
@@ -1236,172 +1236,172 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>19.87</v>
+        <v>19.56</v>
       </c>
       <c r="D27" t="n">
-        <v>1.69</v>
+        <v>1.66</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="F27" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="G27" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>23.67</v>
+        <v>31.16</v>
       </c>
       <c r="D28" t="n">
-        <v>2.16</v>
+        <v>2.4</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="F28" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="G28" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26.89</v>
+        <v>25.31</v>
       </c>
       <c r="D29" t="n">
-        <v>2.5</v>
+        <v>2.08</v>
       </c>
       <c r="E29" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="F29" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="G29" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>17.55</v>
+        <v>47.83</v>
       </c>
       <c r="D30" t="n">
-        <v>0.98</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="F30" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="G30" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>31.63</v>
+        <v>22.29</v>
       </c>
       <c r="D31" t="n">
-        <v>2.43</v>
+        <v>1.65</v>
       </c>
       <c r="E31" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="F31" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="G31" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>22.5</v>
+        <v>28.81</v>
       </c>
       <c r="D32" t="n">
-        <v>1.66</v>
+        <v>2.44</v>
       </c>
       <c r="E32" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="F32" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="G32" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Jun  5 12:27:50 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,151 +477,151 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>20.68</v>
+        <v>33.53</v>
       </c>
       <c r="D2" t="n">
-        <v>1.88</v>
+        <v>3.23</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>34.45</v>
+        <v>20.26</v>
       </c>
       <c r="D3" t="n">
-        <v>3.27</v>
+        <v>1.84</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>75.83</v>
+        <v>42.04</v>
       </c>
       <c r="D4" t="n">
-        <v>7.87</v>
+        <v>3.57</v>
       </c>
       <c r="E4" t="n">
-        <v>95.09999999999999</v>
+        <v>85.7</v>
       </c>
       <c r="F4" t="n">
-        <v>95.09999999999999</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>95.09999999999999</v>
+        <v>86.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21.63</v>
+        <v>72.79000000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>2.02</v>
+        <v>7.57</v>
       </c>
       <c r="E5" t="n">
-        <v>85.40000000000001</v>
+        <v>73.8</v>
       </c>
       <c r="F5" t="n">
-        <v>85.40000000000001</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>85.40000000000001</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>41.96</v>
+        <v>20.83</v>
       </c>
       <c r="D6" t="n">
-        <v>3.56</v>
+        <v>1.95</v>
       </c>
       <c r="E6" t="n">
-        <v>82.90000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="F6" t="n">
-        <v>85.40000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="G6" t="n">
-        <v>84.09999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="7">
@@ -636,22 +636,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>36.5</v>
+        <v>36.35</v>
       </c>
       <c r="D7" t="n">
-        <v>2.05</v>
+        <v>2.03</v>
       </c>
       <c r="E7" t="n">
-        <v>73.2</v>
+        <v>64.3</v>
       </c>
       <c r="F7" t="n">
-        <v>81.7</v>
+        <v>69</v>
       </c>
       <c r="G7" t="n">
-        <v>77.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="8">
@@ -666,52 +666,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.75</v>
+        <v>6.85</v>
       </c>
       <c r="D8" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="E8" t="n">
-        <v>17.1</v>
+        <v>59.5</v>
       </c>
       <c r="F8" t="n">
-        <v>22</v>
+        <v>54.8</v>
       </c>
       <c r="G8" t="n">
-        <v>20.5</v>
+        <v>57.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>115.62</v>
+        <v>26.96</v>
       </c>
       <c r="D9" t="n">
-        <v>4.36</v>
+        <v>2.5</v>
       </c>
       <c r="E9" t="n">
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="F9" t="n">
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="G9" t="n">
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="10">
@@ -726,352 +726,352 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>15.95</v>
+        <v>15.92</v>
       </c>
       <c r="D10" t="n">
         <v>2.37</v>
       </c>
       <c r="E10" t="n">
-        <v>29.3</v>
+        <v>27.4</v>
       </c>
       <c r="F10" t="n">
-        <v>14.6</v>
+        <v>15.5</v>
       </c>
       <c r="G10" t="n">
         <v>19</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>26.79</v>
+        <v>114.88</v>
       </c>
       <c r="D11" t="n">
-        <v>2.48</v>
+        <v>4.33</v>
       </c>
       <c r="E11" t="n">
-        <v>9.800000000000001</v>
+        <v>19</v>
       </c>
       <c r="F11" t="n">
-        <v>12.2</v>
+        <v>19</v>
       </c>
       <c r="G11" t="n">
-        <v>11.5</v>
+        <v>19</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>11.49</v>
+        <v>60.03</v>
       </c>
       <c r="D12" t="n">
-        <v>1.03</v>
+        <v>3.92</v>
       </c>
       <c r="E12" t="n">
-        <v>2.4</v>
+        <v>11.9</v>
       </c>
       <c r="F12" t="n">
-        <v>14.6</v>
+        <v>11.9</v>
       </c>
       <c r="G12" t="n">
-        <v>11</v>
+        <v>11.9</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>21.59</v>
+        <v>11.39</v>
       </c>
       <c r="D13" t="n">
-        <v>3.69</v>
+        <v>1.03</v>
       </c>
       <c r="E13" t="n">
-        <v>7.3</v>
+        <v>2.4</v>
       </c>
       <c r="F13" t="n">
-        <v>12.2</v>
+        <v>15.5</v>
       </c>
       <c r="G13" t="n">
-        <v>10.7</v>
+        <v>11.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>59.91</v>
+        <v>14.13</v>
       </c>
       <c r="D14" t="n">
-        <v>3.91</v>
+        <v>1.33</v>
       </c>
       <c r="E14" t="n">
-        <v>9.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="G14" t="n">
-        <v>9.800000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14.14</v>
+        <v>19.66</v>
       </c>
       <c r="D15" t="n">
-        <v>1.33</v>
+        <v>1.68</v>
       </c>
       <c r="E15" t="n">
-        <v>12.2</v>
+        <v>7.1</v>
       </c>
       <c r="F15" t="n">
-        <v>8.5</v>
+        <v>4.8</v>
       </c>
       <c r="G15" t="n">
-        <v>9.6</v>
+        <v>5.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9.68</v>
+        <v>19.83</v>
       </c>
       <c r="D16" t="n">
-        <v>1.18</v>
+        <v>3.5</v>
       </c>
       <c r="E16" t="n">
-        <v>2.4</v>
+        <v>7.1</v>
       </c>
       <c r="F16" t="n">
-        <v>3.7</v>
+        <v>4.8</v>
       </c>
       <c r="G16" t="n">
-        <v>3.3</v>
+        <v>5.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>27.3</v>
+        <v>28.91</v>
       </c>
       <c r="D17" t="n">
-        <v>2.06</v>
+        <v>2.46</v>
       </c>
       <c r="E17" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="F17" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="G17" t="n">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>10.98</v>
+        <v>25.44</v>
       </c>
       <c r="D18" t="n">
-        <v>0.7</v>
+        <v>2.1</v>
       </c>
       <c r="E18" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="F18" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="G18" t="n">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>35.26</v>
+        <v>31.5</v>
       </c>
       <c r="D19" t="n">
-        <v>3.81</v>
+        <v>2.42</v>
       </c>
       <c r="E19" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="F19" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="G19" t="n">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>19.82</v>
+        <v>14.87</v>
       </c>
       <c r="D20" t="n">
-        <v>3.48</v>
+        <v>1.22</v>
       </c>
       <c r="E20" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="F20" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="G20" t="n">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>25.18</v>
+        <v>23.21</v>
       </c>
       <c r="D21" t="n">
-        <v>2.34</v>
+        <v>1.92</v>
       </c>
       <c r="E21" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="F21" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="G21" t="n">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="22">
@@ -1086,160 +1086,160 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>23.23</v>
+        <v>23.28</v>
       </c>
       <c r="D22" t="n">
         <v>2.15</v>
       </c>
       <c r="E22" t="n">
-        <v>4.9</v>
+        <v>7.1</v>
       </c>
       <c r="F22" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
       <c r="G22" t="n">
-        <v>3.2</v>
+        <v>4.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>17.32</v>
+        <v>11</v>
       </c>
       <c r="D23" t="n">
-        <v>0.97</v>
+        <v>0.7</v>
       </c>
       <c r="E23" t="n">
-        <v>2.4</v>
+        <v>7.1</v>
       </c>
       <c r="F23" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
       <c r="G23" t="n">
-        <v>2.4</v>
+        <v>4.6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>26.56</v>
+        <v>17.37</v>
       </c>
       <c r="D24" t="n">
-        <v>2.47</v>
+        <v>0.97</v>
       </c>
       <c r="E24" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="F24" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
       <c r="G24" t="n">
-        <v>2.4</v>
+        <v>3.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>23.1</v>
+        <v>26.55</v>
       </c>
       <c r="D25" t="n">
-        <v>1.91</v>
+        <v>2.47</v>
       </c>
       <c r="E25" t="n">
         <v>2.4</v>
       </c>
       <c r="F25" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
       <c r="G25" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>14.8</v>
+        <v>27.27</v>
       </c>
       <c r="D26" t="n">
-        <v>1.21</v>
+        <v>2.05</v>
       </c>
       <c r="E26" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="F26" t="n">
         <v>2.4</v>
       </c>
       <c r="G26" t="n">
-        <v>2.4</v>
+        <v>3.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>19.56</v>
+        <v>21.13</v>
       </c>
       <c r="D27" t="n">
-        <v>1.66</v>
+        <v>3.61</v>
       </c>
       <c r="E27" t="n">
         <v>2.4</v>
@@ -1251,25 +1251,25 @@
         <v>2.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>31.16</v>
+        <v>25.04</v>
       </c>
       <c r="D28" t="n">
-        <v>2.4</v>
+        <v>2.33</v>
       </c>
       <c r="E28" t="n">
         <v>2.4</v>
@@ -1281,25 +1281,25 @@
         <v>2.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>25.31</v>
+        <v>34.63</v>
       </c>
       <c r="D29" t="n">
-        <v>2.08</v>
+        <v>3.75</v>
       </c>
       <c r="E29" t="n">
         <v>2.4</v>
@@ -1311,25 +1311,25 @@
         <v>2.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>47.83</v>
+        <v>9.66</v>
       </c>
       <c r="D30" t="n">
-        <v>4</v>
+        <v>1.17</v>
       </c>
       <c r="E30" t="n">
         <v>2.4</v>
@@ -1341,25 +1341,25 @@
         <v>2.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22.29</v>
+        <v>47.6</v>
       </c>
       <c r="D31" t="n">
-        <v>1.65</v>
+        <v>3.99</v>
       </c>
       <c r="E31" t="n">
         <v>2.4</v>
@@ -1371,25 +1371,25 @@
         <v>2.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>28.81</v>
+        <v>22.13</v>
       </c>
       <c r="D32" t="n">
-        <v>2.44</v>
+        <v>1.63</v>
       </c>
       <c r="E32" t="n">
         <v>2.4</v>
@@ -1401,7 +1401,7 @@
         <v>2.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Jun  6 11:11:26 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>3.23</v>
       </c>
       <c r="E2" t="n">
-        <v>95.2</v>
+        <v>94.2</v>
       </c>
       <c r="F2" t="n">
-        <v>95.2</v>
+        <v>94.2</v>
       </c>
       <c r="G2" t="n">
-        <v>95.2</v>
+        <v>94.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.84</v>
       </c>
       <c r="E3" t="n">
-        <v>95.2</v>
+        <v>94.2</v>
       </c>
       <c r="F3" t="n">
-        <v>92.90000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.57</v>
       </c>
       <c r="E4" t="n">
-        <v>85.7</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>86.90000000000001</v>
+        <v>86</v>
       </c>
       <c r="G4" t="n">
-        <v>86.3</v>
+        <v>85.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>7.57</v>
       </c>
       <c r="E5" t="n">
-        <v>73.8</v>
+        <v>73.3</v>
       </c>
       <c r="F5" t="n">
-        <v>82.09999999999999</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>78</v>
+        <v>77.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.95</v>
       </c>
       <c r="E6" t="n">
-        <v>76.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>76.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>76.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.03</v>
       </c>
       <c r="E7" t="n">
-        <v>64.3</v>
+        <v>64</v>
       </c>
       <c r="F7" t="n">
-        <v>69</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>66.7</v>
+        <v>66.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>0.65</v>
       </c>
       <c r="E8" t="n">
-        <v>59.5</v>
+        <v>59.3</v>
       </c>
       <c r="F8" t="n">
-        <v>54.8</v>
+        <v>54.7</v>
       </c>
       <c r="G8" t="n">
-        <v>57.1</v>
+        <v>57</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.5</v>
       </c>
       <c r="E9" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="F9" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="G9" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.37</v>
       </c>
       <c r="E10" t="n">
-        <v>27.4</v>
+        <v>27.9</v>
       </c>
       <c r="F10" t="n">
-        <v>15.5</v>
+        <v>16.3</v>
       </c>
       <c r="G10" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>4.33</v>
       </c>
       <c r="E11" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="F11" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="G11" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.92</v>
       </c>
       <c r="E12" t="n">
-        <v>11.9</v>
+        <v>12.8</v>
       </c>
       <c r="F12" t="n">
-        <v>11.9</v>
+        <v>12.8</v>
       </c>
       <c r="G12" t="n">
-        <v>11.9</v>
+        <v>12.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.03</v>
       </c>
       <c r="E13" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="F13" t="n">
-        <v>15.5</v>
+        <v>16.3</v>
       </c>
       <c r="G13" t="n">
-        <v>11.5</v>
+        <v>12.4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.33</v>
       </c>
       <c r="E14" t="n">
-        <v>8.300000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="G14" t="n">
-        <v>9.199999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.68</v>
       </c>
       <c r="E15" t="n">
-        <v>7.1</v>
+        <v>8.1</v>
       </c>
       <c r="F15" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="G15" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>3.5</v>
       </c>
       <c r="E16" t="n">
-        <v>7.1</v>
+        <v>8.1</v>
       </c>
       <c r="F16" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="G16" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.46</v>
       </c>
       <c r="E17" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="F17" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="G17" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.1</v>
       </c>
       <c r="E18" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="F18" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="G18" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.42</v>
       </c>
       <c r="E19" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="F19" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="G19" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.22</v>
       </c>
       <c r="E20" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="F20" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="G20" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.92</v>
       </c>
       <c r="E21" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="F21" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="G21" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.15</v>
       </c>
       <c r="E22" t="n">
-        <v>7.1</v>
+        <v>8.1</v>
       </c>
       <c r="F22" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="G22" t="n">
-        <v>4.6</v>
+        <v>5.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.7</v>
       </c>
       <c r="E23" t="n">
-        <v>7.1</v>
+        <v>8.1</v>
       </c>
       <c r="F23" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="G23" t="n">
-        <v>4.6</v>
+        <v>5.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>0.97</v>
       </c>
       <c r="E24" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="F24" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="G24" t="n">
-        <v>3.9</v>
+        <v>5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.47</v>
       </c>
       <c r="E25" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="F25" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="G25" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.05</v>
       </c>
       <c r="E26" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="F26" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G26" t="n">
-        <v>3.1</v>
+        <v>4.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.61</v>
       </c>
       <c r="E27" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="F27" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G27" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.33</v>
       </c>
       <c r="E28" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="F28" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G28" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.75</v>
       </c>
       <c r="E29" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="F29" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G29" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.17</v>
       </c>
       <c r="E30" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="F30" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G30" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.99</v>
       </c>
       <c r="E31" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="F31" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G31" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.63</v>
       </c>
       <c r="E32" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="F32" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G32" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Jun  7 11:27:47 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>3.23</v>
       </c>
       <c r="E2" t="n">
-        <v>94.2</v>
+        <v>93.2</v>
       </c>
       <c r="F2" t="n">
-        <v>94.2</v>
+        <v>93.2</v>
       </c>
       <c r="G2" t="n">
-        <v>94.2</v>
+        <v>93.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.84</v>
       </c>
       <c r="E3" t="n">
-        <v>94.2</v>
+        <v>93.2</v>
       </c>
       <c r="F3" t="n">
-        <v>91.90000000000001</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.57</v>
       </c>
       <c r="E4" t="n">
-        <v>84.90000000000001</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>86</v>
+        <v>85.2</v>
       </c>
       <c r="G4" t="n">
-        <v>85.5</v>
+        <v>84.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>7.57</v>
       </c>
       <c r="E5" t="n">
-        <v>73.3</v>
+        <v>72.7</v>
       </c>
       <c r="F5" t="n">
-        <v>81.40000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="G5" t="n">
-        <v>77.3</v>
+        <v>76.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.95</v>
       </c>
       <c r="E6" t="n">
-        <v>75.59999999999999</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>75.59999999999999</v>
+        <v>75</v>
       </c>
       <c r="G6" t="n">
-        <v>75.59999999999999</v>
+        <v>75</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>2.03</v>
       </c>
       <c r="E7" t="n">
-        <v>64</v>
+        <v>63.6</v>
       </c>
       <c r="F7" t="n">
-        <v>68.59999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="G7" t="n">
-        <v>66.3</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>0.65</v>
       </c>
       <c r="E8" t="n">
-        <v>59.3</v>
+        <v>59.1</v>
       </c>
       <c r="F8" t="n">
-        <v>54.7</v>
+        <v>54.5</v>
       </c>
       <c r="G8" t="n">
-        <v>57</v>
+        <v>56.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.5</v>
       </c>
       <c r="E9" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="F9" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="G9" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.37</v>
       </c>
       <c r="E10" t="n">
-        <v>27.9</v>
+        <v>28.4</v>
       </c>
       <c r="F10" t="n">
-        <v>16.3</v>
+        <v>17</v>
       </c>
       <c r="G10" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>4.33</v>
       </c>
       <c r="E11" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="F11" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="G11" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.92</v>
       </c>
       <c r="E12" t="n">
-        <v>12.8</v>
+        <v>13.6</v>
       </c>
       <c r="F12" t="n">
-        <v>12.8</v>
+        <v>13.6</v>
       </c>
       <c r="G12" t="n">
-        <v>12.8</v>
+        <v>13.6</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.03</v>
       </c>
       <c r="E13" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F13" t="n">
-        <v>16.3</v>
+        <v>17</v>
       </c>
       <c r="G13" t="n">
-        <v>12.4</v>
+        <v>13.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.33</v>
       </c>
       <c r="E14" t="n">
-        <v>9.300000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="F14" t="n">
-        <v>10.5</v>
+        <v>11.4</v>
       </c>
       <c r="G14" t="n">
-        <v>10.1</v>
+        <v>11</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.68</v>
       </c>
       <c r="E15" t="n">
-        <v>8.1</v>
+        <v>9.1</v>
       </c>
       <c r="F15" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G15" t="n">
-        <v>6.5</v>
+        <v>7.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>3.5</v>
       </c>
       <c r="E16" t="n">
-        <v>8.1</v>
+        <v>9.1</v>
       </c>
       <c r="F16" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G16" t="n">
-        <v>6.5</v>
+        <v>7.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.46</v>
       </c>
       <c r="E17" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="F17" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G17" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.1</v>
       </c>
       <c r="E18" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="F18" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G18" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.42</v>
       </c>
       <c r="E19" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="F19" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G19" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.22</v>
       </c>
       <c r="E20" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="F20" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G20" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.92</v>
       </c>
       <c r="E21" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="F21" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G21" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.15</v>
       </c>
       <c r="E22" t="n">
-        <v>8.1</v>
+        <v>9.1</v>
       </c>
       <c r="F22" t="n">
-        <v>4.7</v>
+        <v>5.7</v>
       </c>
       <c r="G22" t="n">
-        <v>5.7</v>
+        <v>6.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.7</v>
       </c>
       <c r="E23" t="n">
-        <v>8.1</v>
+        <v>9.1</v>
       </c>
       <c r="F23" t="n">
-        <v>4.7</v>
+        <v>5.7</v>
       </c>
       <c r="G23" t="n">
-        <v>5.7</v>
+        <v>6.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>0.97</v>
       </c>
       <c r="E24" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="F24" t="n">
-        <v>4.7</v>
+        <v>5.7</v>
       </c>
       <c r="G24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.47</v>
       </c>
       <c r="E25" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F25" t="n">
-        <v>4.7</v>
+        <v>5.7</v>
       </c>
       <c r="G25" t="n">
-        <v>4.3</v>
+        <v>5.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.05</v>
       </c>
       <c r="E26" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="F26" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G26" t="n">
-        <v>4.2</v>
+        <v>5.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.61</v>
       </c>
       <c r="E27" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F27" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G27" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.33</v>
       </c>
       <c r="E28" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F28" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G28" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.75</v>
       </c>
       <c r="E29" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F29" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G29" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.17</v>
       </c>
       <c r="E30" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F30" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G30" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.99</v>
       </c>
       <c r="E31" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F31" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G31" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.63</v>
       </c>
       <c r="E32" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F32" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G32" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Jun  8 13:54:16 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,931 +477,931 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>33.53</v>
+        <v>20.68</v>
       </c>
       <c r="D2" t="n">
-        <v>3.23</v>
+        <v>1.88</v>
       </c>
       <c r="E2" t="n">
-        <v>93.2</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>93.2</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>93.2</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.26</v>
+        <v>32.75</v>
       </c>
       <c r="D3" t="n">
-        <v>1.84</v>
+        <v>3.16</v>
       </c>
       <c r="E3" t="n">
-        <v>93.2</v>
+        <v>86.7</v>
       </c>
       <c r="F3" t="n">
-        <v>90.90000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>92</v>
+        <v>87.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42.04</v>
+        <v>6.95</v>
       </c>
       <c r="D4" t="n">
-        <v>3.57</v>
+        <v>0.66</v>
       </c>
       <c r="E4" t="n">
-        <v>84.09999999999999</v>
+        <v>86.7</v>
       </c>
       <c r="F4" t="n">
-        <v>85.2</v>
+        <v>77.8</v>
       </c>
       <c r="G4" t="n">
-        <v>84.7</v>
+        <v>82.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>72.79000000000001</v>
+        <v>41.63</v>
       </c>
       <c r="D5" t="n">
-        <v>7.57</v>
+        <v>3.54</v>
       </c>
       <c r="E5" t="n">
-        <v>72.7</v>
+        <v>73.3</v>
       </c>
       <c r="F5" t="n">
-        <v>80.7</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>76.7</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>20.83</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>1.95</v>
+        <v>7.25</v>
       </c>
       <c r="E6" t="n">
-        <v>75</v>
+        <v>57.8</v>
       </c>
       <c r="F6" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="G6" t="n">
-        <v>75</v>
+        <v>58.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>36.35</v>
+        <v>20.35</v>
       </c>
       <c r="D7" t="n">
-        <v>2.03</v>
+        <v>1.9</v>
       </c>
       <c r="E7" t="n">
-        <v>63.6</v>
+        <v>51.1</v>
       </c>
       <c r="F7" t="n">
-        <v>68.2</v>
+        <v>50</v>
       </c>
       <c r="G7" t="n">
-        <v>65.90000000000001</v>
+        <v>50.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.85</v>
+        <v>35.23</v>
       </c>
       <c r="D8" t="n">
-        <v>0.65</v>
+        <v>1.97</v>
       </c>
       <c r="E8" t="n">
-        <v>59.1</v>
+        <v>46.7</v>
       </c>
       <c r="F8" t="n">
-        <v>54.5</v>
+        <v>48.9</v>
       </c>
       <c r="G8" t="n">
-        <v>56.8</v>
+        <v>47.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>26.96</v>
+        <v>14.46</v>
       </c>
       <c r="D9" t="n">
-        <v>2.5</v>
+        <v>1.36</v>
       </c>
       <c r="E9" t="n">
-        <v>20.5</v>
+        <v>28.9</v>
       </c>
       <c r="F9" t="n">
-        <v>20.5</v>
+        <v>27.8</v>
       </c>
       <c r="G9" t="n">
-        <v>20.5</v>
+        <v>28.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>15.92</v>
+        <v>111.37</v>
       </c>
       <c r="D10" t="n">
-        <v>2.37</v>
+        <v>4.2</v>
       </c>
       <c r="E10" t="n">
-        <v>28.4</v>
+        <v>17.8</v>
       </c>
       <c r="F10" t="n">
-        <v>17</v>
+        <v>17.8</v>
       </c>
       <c r="G10" t="n">
-        <v>20.5</v>
+        <v>17.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>114.88</v>
+        <v>11.05</v>
       </c>
       <c r="D11" t="n">
-        <v>4.33</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>20.5</v>
+        <v>2.2</v>
       </c>
       <c r="F11" t="n">
-        <v>20.5</v>
+        <v>13.3</v>
       </c>
       <c r="G11" t="n">
-        <v>20.5</v>
+        <v>10</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>60.03</v>
+        <v>15.82</v>
       </c>
       <c r="D12" t="n">
-        <v>3.92</v>
+        <v>2.35</v>
       </c>
       <c r="E12" t="n">
-        <v>13.6</v>
+        <v>15.6</v>
       </c>
       <c r="F12" t="n">
-        <v>13.6</v>
+        <v>2.2</v>
       </c>
       <c r="G12" t="n">
-        <v>13.6</v>
+        <v>6.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11.39</v>
+        <v>10.73</v>
       </c>
       <c r="D13" t="n">
-        <v>1.03</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="F13" t="n">
-        <v>17</v>
+        <v>2.2</v>
       </c>
       <c r="G13" t="n">
-        <v>13.3</v>
+        <v>2.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14.13</v>
+        <v>26.8</v>
       </c>
       <c r="D14" t="n">
-        <v>1.33</v>
+        <v>2.02</v>
       </c>
       <c r="E14" t="n">
-        <v>10.2</v>
+        <v>4.4</v>
       </c>
       <c r="F14" t="n">
-        <v>11.4</v>
+        <v>2.2</v>
       </c>
       <c r="G14" t="n">
-        <v>11</v>
+        <v>2.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>19.66</v>
+        <v>16.96</v>
       </c>
       <c r="D15" t="n">
-        <v>1.68</v>
+        <v>0.95</v>
       </c>
       <c r="E15" t="n">
-        <v>9.1</v>
+        <v>2.2</v>
       </c>
       <c r="F15" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="G15" t="n">
-        <v>7.5</v>
+        <v>2.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>19.83</v>
+        <v>26.13</v>
       </c>
       <c r="D16" t="n">
-        <v>3.5</v>
+        <v>2.42</v>
       </c>
       <c r="E16" t="n">
-        <v>9.1</v>
+        <v>2.2</v>
       </c>
       <c r="F16" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="G16" t="n">
-        <v>7.5</v>
+        <v>2.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>28.91</v>
+        <v>22.58</v>
       </c>
       <c r="D17" t="n">
-        <v>2.46</v>
+        <v>1.87</v>
       </c>
       <c r="E17" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="F17" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="G17" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>25.44</v>
+        <v>14.55</v>
       </c>
       <c r="D18" t="n">
-        <v>2.1</v>
+        <v>1.19</v>
       </c>
       <c r="E18" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="F18" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="G18" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>31.5</v>
+        <v>22.75</v>
       </c>
       <c r="D19" t="n">
-        <v>2.42</v>
+        <v>2.11</v>
       </c>
       <c r="E19" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="F19" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="G19" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>14.87</v>
+        <v>25.96</v>
       </c>
       <c r="D20" t="n">
-        <v>1.22</v>
+        <v>2.42</v>
       </c>
       <c r="E20" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="F20" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="G20" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>23.21</v>
+        <v>19.28</v>
       </c>
       <c r="D21" t="n">
-        <v>1.92</v>
+        <v>1.65</v>
       </c>
       <c r="E21" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="F21" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="G21" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>23.28</v>
+        <v>19.6</v>
       </c>
       <c r="D22" t="n">
-        <v>2.15</v>
+        <v>3.46</v>
       </c>
       <c r="E22" t="n">
-        <v>9.1</v>
+        <v>2.2</v>
       </c>
       <c r="F22" t="n">
-        <v>5.7</v>
+        <v>2.2</v>
       </c>
       <c r="G22" t="n">
-        <v>6.7</v>
+        <v>2.2</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>11</v>
+        <v>19.95</v>
       </c>
       <c r="D23" t="n">
-        <v>0.7</v>
+        <v>3.41</v>
       </c>
       <c r="E23" t="n">
-        <v>9.1</v>
+        <v>2.2</v>
       </c>
       <c r="F23" t="n">
-        <v>5.7</v>
+        <v>2.2</v>
       </c>
       <c r="G23" t="n">
-        <v>6.7</v>
+        <v>2.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>17.37</v>
+        <v>24.58</v>
       </c>
       <c r="D24" t="n">
-        <v>0.97</v>
+        <v>2.29</v>
       </c>
       <c r="E24" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="F24" t="n">
-        <v>5.7</v>
+        <v>2.2</v>
       </c>
       <c r="G24" t="n">
-        <v>6</v>
+        <v>2.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>26.55</v>
+        <v>33.43</v>
       </c>
       <c r="D25" t="n">
-        <v>2.47</v>
+        <v>3.61</v>
       </c>
       <c r="E25" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="F25" t="n">
-        <v>5.7</v>
+        <v>2.2</v>
       </c>
       <c r="G25" t="n">
-        <v>5.3</v>
+        <v>2.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>27.27</v>
+        <v>9.57</v>
       </c>
       <c r="D26" t="n">
-        <v>2.05</v>
+        <v>1.16</v>
       </c>
       <c r="E26" t="n">
-        <v>6.8</v>
+        <v>2.2</v>
       </c>
       <c r="F26" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="G26" t="n">
-        <v>5.2</v>
+        <v>2.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>21.13</v>
+        <v>30.7</v>
       </c>
       <c r="D27" t="n">
-        <v>3.61</v>
+        <v>2.36</v>
       </c>
       <c r="E27" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="F27" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="G27" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25.04</v>
+        <v>57.94</v>
       </c>
       <c r="D28" t="n">
-        <v>2.33</v>
+        <v>3.78</v>
       </c>
       <c r="E28" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="F28" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="G28" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>34.63</v>
+        <v>24.92</v>
       </c>
       <c r="D29" t="n">
-        <v>3.75</v>
+        <v>2.05</v>
       </c>
       <c r="E29" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="F29" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="G29" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9.66</v>
+        <v>46.24</v>
       </c>
       <c r="D30" t="n">
-        <v>1.17</v>
+        <v>3.87</v>
       </c>
       <c r="E30" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="F30" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="G30" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>47.6</v>
+        <v>21.52</v>
       </c>
       <c r="D31" t="n">
-        <v>3.99</v>
+        <v>1.59</v>
       </c>
       <c r="E31" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="F31" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="G31" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>22.13</v>
+        <v>28.16</v>
       </c>
       <c r="D32" t="n">
-        <v>1.63</v>
+        <v>2.39</v>
       </c>
       <c r="E32" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="F32" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="G32" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Jun  9 12:27:10 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,121 +477,121 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>20.68</v>
+        <v>33.78</v>
       </c>
       <c r="D2" t="n">
-        <v>1.88</v>
+        <v>3.26</v>
       </c>
       <c r="E2" t="n">
-        <v>98.90000000000001</v>
+        <v>95.7</v>
       </c>
       <c r="F2" t="n">
-        <v>98.90000000000001</v>
+        <v>97.8</v>
       </c>
       <c r="G2" t="n">
-        <v>98.90000000000001</v>
+        <v>96.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>32.75</v>
+        <v>42.58</v>
       </c>
       <c r="D3" t="n">
-        <v>3.16</v>
+        <v>3.63</v>
       </c>
       <c r="E3" t="n">
-        <v>86.7</v>
+        <v>91.3</v>
       </c>
       <c r="F3" t="n">
-        <v>88.90000000000001</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>87.8</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6.95</v>
+        <v>37.24</v>
       </c>
       <c r="D4" t="n">
-        <v>0.66</v>
+        <v>2.08</v>
       </c>
       <c r="E4" t="n">
-        <v>86.7</v>
+        <v>87</v>
       </c>
       <c r="F4" t="n">
-        <v>77.8</v>
+        <v>87</v>
       </c>
       <c r="G4" t="n">
-        <v>82.2</v>
+        <v>87</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>41.63</v>
+        <v>20.06</v>
       </c>
       <c r="D5" t="n">
-        <v>3.54</v>
+        <v>1.83</v>
       </c>
       <c r="E5" t="n">
-        <v>73.3</v>
+        <v>87</v>
       </c>
       <c r="F5" t="n">
-        <v>74.40000000000001</v>
+        <v>83.7</v>
       </c>
       <c r="G5" t="n">
-        <v>73.90000000000001</v>
+        <v>85.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="6">
@@ -606,172 +606,172 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>69.70999999999999</v>
+        <v>73.42</v>
       </c>
       <c r="D6" t="n">
-        <v>7.25</v>
+        <v>7.63</v>
       </c>
       <c r="E6" t="n">
-        <v>57.8</v>
+        <v>84.8</v>
       </c>
       <c r="F6" t="n">
-        <v>60</v>
+        <v>84.8</v>
       </c>
       <c r="G6" t="n">
-        <v>58.9</v>
+        <v>84.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.35</v>
+        <v>6.97</v>
       </c>
       <c r="D7" t="n">
-        <v>1.9</v>
+        <v>0.66</v>
       </c>
       <c r="E7" t="n">
-        <v>51.1</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>50</v>
+        <v>77.2</v>
       </c>
       <c r="G7" t="n">
-        <v>50.6</v>
+        <v>83.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>35.23</v>
+        <v>20.52</v>
       </c>
       <c r="D8" t="n">
-        <v>1.97</v>
+        <v>1.92</v>
       </c>
       <c r="E8" t="n">
-        <v>46.7</v>
+        <v>58.7</v>
       </c>
       <c r="F8" t="n">
-        <v>48.9</v>
+        <v>59.8</v>
       </c>
       <c r="G8" t="n">
-        <v>47.8</v>
+        <v>59.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.46</v>
+        <v>118.94</v>
       </c>
       <c r="D9" t="n">
-        <v>1.36</v>
+        <v>4.48</v>
       </c>
       <c r="E9" t="n">
-        <v>28.9</v>
+        <v>28.3</v>
       </c>
       <c r="F9" t="n">
-        <v>27.8</v>
+        <v>28.3</v>
       </c>
       <c r="G9" t="n">
-        <v>28.1</v>
+        <v>28.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>111.37</v>
+        <v>11.14</v>
       </c>
       <c r="D10" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>17.8</v>
+        <v>4.3</v>
       </c>
       <c r="F10" t="n">
-        <v>17.8</v>
+        <v>14.1</v>
       </c>
       <c r="G10" t="n">
-        <v>17.8</v>
+        <v>11.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>11.05</v>
+        <v>26.69</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2.47</v>
       </c>
       <c r="E11" t="n">
-        <v>2.2</v>
+        <v>10.9</v>
       </c>
       <c r="F11" t="n">
-        <v>13.3</v>
+        <v>10.9</v>
       </c>
       <c r="G11" t="n">
-        <v>10</v>
+        <v>10.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="12">
@@ -786,550 +786,550 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15.82</v>
+        <v>15.83</v>
       </c>
       <c r="D12" t="n">
         <v>2.35</v>
       </c>
       <c r="E12" t="n">
-        <v>15.6</v>
+        <v>17.4</v>
       </c>
       <c r="F12" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="G12" t="n">
-        <v>6.2</v>
+        <v>7.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.73</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.17</v>
       </c>
       <c r="E13" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="F13" t="n">
-        <v>2.2</v>
+        <v>7.6</v>
       </c>
       <c r="G13" t="n">
-        <v>2.9</v>
+        <v>6.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>26.8</v>
+        <v>19.43</v>
       </c>
       <c r="D14" t="n">
-        <v>2.02</v>
+        <v>1.66</v>
       </c>
       <c r="E14" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="F14" t="n">
-        <v>2.2</v>
+        <v>5.4</v>
       </c>
       <c r="G14" t="n">
-        <v>2.9</v>
+        <v>5.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>16.96</v>
+        <v>14.6</v>
       </c>
       <c r="D15" t="n">
-        <v>0.95</v>
+        <v>1.2</v>
       </c>
       <c r="E15" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F15" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G15" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26.13</v>
+        <v>20.46</v>
       </c>
       <c r="D16" t="n">
-        <v>2.42</v>
+        <v>3.5</v>
       </c>
       <c r="E16" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F16" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G16" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>22.58</v>
+        <v>25.09</v>
       </c>
       <c r="D17" t="n">
-        <v>1.87</v>
+        <v>2.07</v>
       </c>
       <c r="E17" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F17" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G17" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>14.55</v>
+        <v>21.69</v>
       </c>
       <c r="D18" t="n">
-        <v>1.19</v>
+        <v>1.6</v>
       </c>
       <c r="E18" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F18" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G18" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22.75</v>
+        <v>46.96</v>
       </c>
       <c r="D19" t="n">
-        <v>2.11</v>
+        <v>3.94</v>
       </c>
       <c r="E19" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F19" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G19" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>25.96</v>
+        <v>58.55</v>
       </c>
       <c r="D20" t="n">
-        <v>2.42</v>
+        <v>3.82</v>
       </c>
       <c r="E20" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F20" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G20" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>19.28</v>
+        <v>22.92</v>
       </c>
       <c r="D21" t="n">
-        <v>1.65</v>
+        <v>2.13</v>
       </c>
       <c r="E21" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F21" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G21" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>19.6</v>
+        <v>17.11</v>
       </c>
       <c r="D22" t="n">
-        <v>3.46</v>
+        <v>0.96</v>
       </c>
       <c r="E22" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F22" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G22" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>19.95</v>
+        <v>24.72</v>
       </c>
       <c r="D23" t="n">
-        <v>3.41</v>
+        <v>2.3</v>
       </c>
       <c r="E23" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F23" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G23" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>24.58</v>
+        <v>34.35</v>
       </c>
       <c r="D24" t="n">
-        <v>2.29</v>
+        <v>3.71</v>
       </c>
       <c r="E24" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F24" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G24" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>33.43</v>
+        <v>10.8</v>
       </c>
       <c r="D25" t="n">
-        <v>3.61</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E25" t="n">
-        <v>2.2</v>
+        <v>6.5</v>
       </c>
       <c r="F25" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="G25" t="n">
-        <v>2.2</v>
+        <v>4.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>9.57</v>
+        <v>26.82</v>
       </c>
       <c r="D26" t="n">
-        <v>1.16</v>
+        <v>2.02</v>
       </c>
       <c r="E26" t="n">
-        <v>2.2</v>
+        <v>6.5</v>
       </c>
       <c r="F26" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="G26" t="n">
-        <v>2.2</v>
+        <v>4.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>30.7</v>
+        <v>25.98</v>
       </c>
       <c r="D27" t="n">
-        <v>2.36</v>
+        <v>2.42</v>
       </c>
       <c r="E27" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F27" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="G27" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>57.94</v>
+        <v>30.73</v>
       </c>
       <c r="D28" t="n">
-        <v>3.78</v>
+        <v>2.36</v>
       </c>
       <c r="E28" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F28" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="G28" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>24.92</v>
+        <v>22.54</v>
       </c>
       <c r="D29" t="n">
-        <v>2.05</v>
+        <v>1.87</v>
       </c>
       <c r="E29" t="n">
         <v>2.2</v>
       </c>
       <c r="F29" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="G29" t="n">
-        <v>2.2</v>
+        <v>2.9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>46.24</v>
+        <v>19.5</v>
       </c>
       <c r="D30" t="n">
-        <v>3.87</v>
+        <v>3.45</v>
       </c>
       <c r="E30" t="n">
         <v>2.2</v>
@@ -1341,25 +1341,25 @@
         <v>2.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>21.52</v>
+        <v>13.86</v>
       </c>
       <c r="D31" t="n">
-        <v>1.59</v>
+        <v>1.31</v>
       </c>
       <c r="E31" t="n">
         <v>2.2</v>
@@ -1371,7 +1371,7 @@
         <v>2.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
     <row r="32">
@@ -1386,10 +1386,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>28.16</v>
+        <v>27.95</v>
       </c>
       <c r="D32" t="n">
-        <v>2.39</v>
+        <v>2.38</v>
       </c>
       <c r="E32" t="n">
         <v>2.2</v>
@@ -1401,7 +1401,7 @@
         <v>2.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Jun 10 12:46:31 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,61 +477,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>33.78</v>
+        <v>7.08</v>
       </c>
       <c r="D2" t="n">
-        <v>3.26</v>
+        <v>0.67</v>
       </c>
       <c r="E2" t="n">
-        <v>95.7</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>97.8</v>
+        <v>88.3</v>
       </c>
       <c r="G2" t="n">
-        <v>96.7</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42.58</v>
+        <v>33.23</v>
       </c>
       <c r="D3" t="n">
-        <v>3.63</v>
+        <v>3.22</v>
       </c>
       <c r="E3" t="n">
-        <v>91.3</v>
+        <v>87.2</v>
       </c>
       <c r="F3" t="n">
-        <v>94.59999999999999</v>
+        <v>87.2</v>
       </c>
       <c r="G3" t="n">
-        <v>92.90000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="4">
@@ -546,112 +546,112 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37.24</v>
+        <v>36.57</v>
       </c>
       <c r="D4" t="n">
-        <v>2.08</v>
+        <v>2.04</v>
       </c>
       <c r="E4" t="n">
-        <v>87</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>87</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>87</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20.06</v>
+        <v>71.87</v>
       </c>
       <c r="D5" t="n">
-        <v>1.83</v>
+        <v>7.48</v>
       </c>
       <c r="E5" t="n">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="F5" t="n">
-        <v>83.7</v>
+        <v>66</v>
       </c>
       <c r="G5" t="n">
-        <v>85.3</v>
+        <v>66</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>73.42</v>
+        <v>41.23</v>
       </c>
       <c r="D6" t="n">
-        <v>7.63</v>
+        <v>3.51</v>
       </c>
       <c r="E6" t="n">
-        <v>84.8</v>
+        <v>55.3</v>
       </c>
       <c r="F6" t="n">
-        <v>84.8</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>84.8</v>
+        <v>61.7</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6.97</v>
+        <v>19.44</v>
       </c>
       <c r="D7" t="n">
-        <v>0.66</v>
+        <v>1.77</v>
       </c>
       <c r="E7" t="n">
-        <v>89.09999999999999</v>
+        <v>61.7</v>
       </c>
       <c r="F7" t="n">
-        <v>77.2</v>
+        <v>53.2</v>
       </c>
       <c r="G7" t="n">
-        <v>83.2</v>
+        <v>57.4</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="8">
@@ -666,22 +666,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20.52</v>
+        <v>20.07</v>
       </c>
       <c r="D8" t="n">
-        <v>1.92</v>
+        <v>1.88</v>
       </c>
       <c r="E8" t="n">
-        <v>58.7</v>
+        <v>40.4</v>
       </c>
       <c r="F8" t="n">
-        <v>59.8</v>
+        <v>30.9</v>
       </c>
       <c r="G8" t="n">
-        <v>59.2</v>
+        <v>35.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="9">
@@ -696,400 +696,400 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>118.94</v>
+        <v>116.74</v>
       </c>
       <c r="D9" t="n">
-        <v>4.48</v>
+        <v>4.4</v>
       </c>
       <c r="E9" t="n">
-        <v>28.3</v>
+        <v>27.7</v>
       </c>
       <c r="F9" t="n">
-        <v>28.3</v>
+        <v>27.7</v>
       </c>
       <c r="G9" t="n">
-        <v>28.3</v>
+        <v>27.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>11.14</v>
+        <v>26.84</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2.49</v>
       </c>
       <c r="E10" t="n">
-        <v>4.3</v>
+        <v>16</v>
       </c>
       <c r="F10" t="n">
-        <v>14.1</v>
+        <v>20.2</v>
       </c>
       <c r="G10" t="n">
-        <v>11.2</v>
+        <v>18.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>26.69</v>
+        <v>9.77</v>
       </c>
       <c r="D11" t="n">
-        <v>2.47</v>
+        <v>1.19</v>
       </c>
       <c r="E11" t="n">
-        <v>10.9</v>
+        <v>17</v>
       </c>
       <c r="F11" t="n">
-        <v>10.9</v>
+        <v>18.1</v>
       </c>
       <c r="G11" t="n">
-        <v>10.9</v>
+        <v>17.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15.83</v>
+        <v>11.25</v>
       </c>
       <c r="D12" t="n">
-        <v>2.35</v>
+        <v>1.01</v>
       </c>
       <c r="E12" t="n">
-        <v>17.4</v>
+        <v>6.4</v>
       </c>
       <c r="F12" t="n">
-        <v>3.3</v>
+        <v>17</v>
       </c>
       <c r="G12" t="n">
-        <v>7.5</v>
+        <v>13.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9.619999999999999</v>
+        <v>19.76</v>
       </c>
       <c r="D13" t="n">
-        <v>1.17</v>
+        <v>3.49</v>
       </c>
       <c r="E13" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="F13" t="n">
-        <v>7.6</v>
+        <v>8.5</v>
       </c>
       <c r="G13" t="n">
-        <v>6.6</v>
+        <v>8.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>19.43</v>
+        <v>15.78</v>
       </c>
       <c r="D14" t="n">
-        <v>1.66</v>
+        <v>2.35</v>
       </c>
       <c r="E14" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="F14" t="n">
         <v>4.3</v>
       </c>
-      <c r="F14" t="n">
-        <v>5.4</v>
-      </c>
       <c r="G14" t="n">
-        <v>5.1</v>
+        <v>7.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14.6</v>
+        <v>26.9</v>
       </c>
       <c r="D15" t="n">
-        <v>1.2</v>
+        <v>2.03</v>
       </c>
       <c r="E15" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="F15" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="G15" t="n">
-        <v>4.3</v>
+        <v>7</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>20.46</v>
+        <v>26.11</v>
       </c>
       <c r="D16" t="n">
-        <v>3.5</v>
+        <v>2.44</v>
       </c>
       <c r="E16" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="F16" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="G16" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25.09</v>
+        <v>30.81</v>
       </c>
       <c r="D17" t="n">
-        <v>2.07</v>
+        <v>2.37</v>
       </c>
       <c r="E17" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="F17" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="G17" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>21.69</v>
+        <v>14.65</v>
       </c>
       <c r="D18" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="E18" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="F18" t="n">
-        <v>4.3</v>
+        <v>5.3</v>
       </c>
       <c r="G18" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>46.96</v>
+        <v>21.62</v>
       </c>
       <c r="D19" t="n">
-        <v>3.94</v>
+        <v>1.6</v>
       </c>
       <c r="E19" t="n">
         <v>4.3</v>
       </c>
       <c r="F19" t="n">
-        <v>4.3</v>
+        <v>5.3</v>
       </c>
       <c r="G19" t="n">
-        <v>4.3</v>
+        <v>5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>58.55</v>
+        <v>28.11</v>
       </c>
       <c r="D20" t="n">
-        <v>3.82</v>
+        <v>2.39</v>
       </c>
       <c r="E20" t="n">
         <v>4.3</v>
       </c>
       <c r="F20" t="n">
-        <v>4.3</v>
+        <v>5.3</v>
       </c>
       <c r="G20" t="n">
-        <v>4.3</v>
+        <v>5</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>22.92</v>
+        <v>10.76</v>
       </c>
       <c r="D21" t="n">
-        <v>2.13</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E21" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="F21" t="n">
         <v>4.3</v>
       </c>
       <c r="G21" t="n">
-        <v>4.3</v>
+        <v>4.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>17.11</v>
+        <v>20.15</v>
       </c>
       <c r="D22" t="n">
-        <v>0.96</v>
+        <v>3.45</v>
       </c>
       <c r="E22" t="n">
         <v>4.3</v>
@@ -1101,187 +1101,187 @@
         <v>4.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24.72</v>
+        <v>17.03</v>
       </c>
       <c r="D23" t="n">
-        <v>2.3</v>
+        <v>0.95</v>
       </c>
       <c r="E23" t="n">
         <v>4.3</v>
       </c>
       <c r="F23" t="n">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
       <c r="G23" t="n">
-        <v>4.3</v>
+        <v>3.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>34.35</v>
+        <v>19.33</v>
       </c>
       <c r="D24" t="n">
-        <v>3.71</v>
+        <v>1.65</v>
       </c>
       <c r="E24" t="n">
         <v>4.3</v>
       </c>
       <c r="F24" t="n">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
       <c r="G24" t="n">
-        <v>4.3</v>
+        <v>3.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10.8</v>
+        <v>57.97</v>
       </c>
       <c r="D25" t="n">
-        <v>0.6899999999999999</v>
+        <v>3.78</v>
       </c>
       <c r="E25" t="n">
-        <v>6.5</v>
+        <v>4.3</v>
       </c>
       <c r="F25" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="G25" t="n">
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>26.82</v>
+        <v>24.89</v>
       </c>
       <c r="D26" t="n">
-        <v>2.02</v>
+        <v>2.05</v>
       </c>
       <c r="E26" t="n">
-        <v>6.5</v>
+        <v>2.1</v>
       </c>
       <c r="F26" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="G26" t="n">
-        <v>4.2</v>
+        <v>2.9</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25.98</v>
+        <v>22.74</v>
       </c>
       <c r="D27" t="n">
-        <v>2.42</v>
+        <v>2.11</v>
       </c>
       <c r="E27" t="n">
-        <v>4.3</v>
+        <v>2.1</v>
       </c>
       <c r="F27" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="G27" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>30.73</v>
+        <v>24.06</v>
       </c>
       <c r="D28" t="n">
-        <v>2.36</v>
+        <v>2.24</v>
       </c>
       <c r="E28" t="n">
-        <v>4.3</v>
+        <v>2.1</v>
       </c>
       <c r="F28" t="n">
-        <v>3.3</v>
+        <v>2.1</v>
       </c>
       <c r="G28" t="n">
-        <v>3.6</v>
+        <v>2.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="29">
@@ -1296,112 +1296,112 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>22.54</v>
+        <v>22.34</v>
       </c>
       <c r="D29" t="n">
-        <v>1.87</v>
+        <v>1.85</v>
       </c>
       <c r="E29" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="F29" t="n">
-        <v>3.3</v>
+        <v>2.1</v>
       </c>
       <c r="G29" t="n">
-        <v>2.9</v>
+        <v>2.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.5</v>
+        <v>33.3</v>
       </c>
       <c r="D30" t="n">
-        <v>3.45</v>
+        <v>3.59</v>
       </c>
       <c r="E30" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="F30" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="G30" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>13.86</v>
+        <v>46.06</v>
       </c>
       <c r="D31" t="n">
-        <v>1.31</v>
+        <v>3.86</v>
       </c>
       <c r="E31" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="F31" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="G31" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>27.95</v>
+        <v>13.67</v>
       </c>
       <c r="D32" t="n">
-        <v>2.38</v>
+        <v>1.28</v>
       </c>
       <c r="E32" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="F32" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="G32" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Jun 11 13:06:01 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,82 +486,82 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.08</v>
+        <v>7.07</v>
       </c>
       <c r="D2" t="n">
         <v>0.67</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>88.3</v>
+        <v>87.5</v>
       </c>
       <c r="G2" t="n">
-        <v>94.09999999999999</v>
+        <v>92.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>33.23</v>
+        <v>37.35</v>
       </c>
       <c r="D3" t="n">
-        <v>3.22</v>
+        <v>2.09</v>
       </c>
       <c r="E3" t="n">
-        <v>87.2</v>
+        <v>87.5</v>
       </c>
       <c r="F3" t="n">
-        <v>87.2</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>87.2</v>
+        <v>88.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>36.57</v>
+        <v>32.66</v>
       </c>
       <c r="D4" t="n">
-        <v>2.04</v>
+        <v>3.16</v>
       </c>
       <c r="E4" t="n">
-        <v>76.59999999999999</v>
+        <v>81.2</v>
       </c>
       <c r="F4" t="n">
-        <v>76.59999999999999</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>76.59999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="5">
@@ -576,82 +576,82 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>71.87</v>
+        <v>72.3</v>
       </c>
       <c r="D5" t="n">
-        <v>7.48</v>
+        <v>7.53</v>
       </c>
       <c r="E5" t="n">
-        <v>66</v>
+        <v>66.7</v>
       </c>
       <c r="F5" t="n">
-        <v>66</v>
+        <v>68.8</v>
       </c>
       <c r="G5" t="n">
-        <v>66</v>
+        <v>67.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>41.23</v>
+        <v>19.47</v>
       </c>
       <c r="D6" t="n">
-        <v>3.51</v>
+        <v>1.77</v>
       </c>
       <c r="E6" t="n">
-        <v>55.3</v>
+        <v>62.5</v>
       </c>
       <c r="F6" t="n">
-        <v>68.09999999999999</v>
+        <v>53.1</v>
       </c>
       <c r="G6" t="n">
-        <v>61.7</v>
+        <v>57.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.44</v>
+        <v>40.74</v>
       </c>
       <c r="D7" t="n">
-        <v>1.77</v>
+        <v>3.47</v>
       </c>
       <c r="E7" t="n">
-        <v>61.7</v>
+        <v>41.7</v>
       </c>
       <c r="F7" t="n">
-        <v>53.2</v>
+        <v>47.9</v>
       </c>
       <c r="G7" t="n">
-        <v>57.4</v>
+        <v>44.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="8">
@@ -666,562 +666,562 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20.07</v>
+        <v>20.09</v>
       </c>
       <c r="D8" t="n">
         <v>1.88</v>
       </c>
       <c r="E8" t="n">
-        <v>40.4</v>
+        <v>41.7</v>
       </c>
       <c r="F8" t="n">
-        <v>30.9</v>
+        <v>31.2</v>
       </c>
       <c r="G8" t="n">
-        <v>35.6</v>
+        <v>36.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>116.74</v>
+        <v>15.96</v>
       </c>
       <c r="D9" t="n">
-        <v>4.4</v>
+        <v>2.37</v>
       </c>
       <c r="E9" t="n">
-        <v>27.7</v>
+        <v>39.6</v>
       </c>
       <c r="F9" t="n">
-        <v>27.7</v>
+        <v>22.9</v>
       </c>
       <c r="G9" t="n">
-        <v>27.7</v>
+        <v>27.9</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>26.84</v>
+        <v>116.6</v>
       </c>
       <c r="D10" t="n">
-        <v>2.49</v>
+        <v>4.4</v>
       </c>
       <c r="E10" t="n">
-        <v>16</v>
+        <v>27.1</v>
       </c>
       <c r="F10" t="n">
-        <v>20.2</v>
+        <v>28.1</v>
       </c>
       <c r="G10" t="n">
-        <v>18.9</v>
+        <v>27.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9.77</v>
+        <v>26.97</v>
       </c>
       <c r="D11" t="n">
-        <v>1.19</v>
+        <v>2.5</v>
       </c>
       <c r="E11" t="n">
-        <v>17</v>
+        <v>29.2</v>
       </c>
       <c r="F11" t="n">
-        <v>18.1</v>
+        <v>26</v>
       </c>
       <c r="G11" t="n">
-        <v>17.8</v>
+        <v>27</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>11.25</v>
+        <v>9.68</v>
       </c>
       <c r="D12" t="n">
-        <v>1.01</v>
+        <v>1.18</v>
       </c>
       <c r="E12" t="n">
-        <v>6.4</v>
+        <v>13.5</v>
       </c>
       <c r="F12" t="n">
-        <v>17</v>
+        <v>14.6</v>
       </c>
       <c r="G12" t="n">
-        <v>13.8</v>
+        <v>14.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.76</v>
+        <v>11.15</v>
       </c>
       <c r="D13" t="n">
-        <v>3.49</v>
+        <v>1.01</v>
       </c>
       <c r="E13" t="n">
-        <v>8.5</v>
+        <v>6.2</v>
       </c>
       <c r="F13" t="n">
-        <v>8.5</v>
+        <v>17.7</v>
       </c>
       <c r="G13" t="n">
-        <v>8.5</v>
+        <v>14.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.78</v>
+        <v>19.78</v>
       </c>
       <c r="D14" t="n">
-        <v>2.35</v>
+        <v>3.49</v>
       </c>
       <c r="E14" t="n">
-        <v>14.9</v>
+        <v>10.4</v>
       </c>
       <c r="F14" t="n">
-        <v>4.3</v>
+        <v>9.4</v>
       </c>
       <c r="G14" t="n">
-        <v>7.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26.9</v>
+        <v>20.53</v>
       </c>
       <c r="D15" t="n">
-        <v>2.03</v>
+        <v>3.52</v>
       </c>
       <c r="E15" t="n">
-        <v>8.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>6.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26.11</v>
+        <v>17.18</v>
       </c>
       <c r="D16" t="n">
-        <v>2.44</v>
+        <v>0.96</v>
       </c>
       <c r="E16" t="n">
-        <v>6.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>6.4</v>
+        <v>7.3</v>
       </c>
       <c r="G16" t="n">
-        <v>6.4</v>
+        <v>7.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>30.81</v>
+        <v>26</v>
       </c>
       <c r="D17" t="n">
-        <v>2.37</v>
+        <v>2.43</v>
       </c>
       <c r="E17" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="F17" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="G17" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>14.65</v>
+        <v>58.16</v>
       </c>
       <c r="D18" t="n">
-        <v>1.2</v>
+        <v>3.79</v>
       </c>
       <c r="E18" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="F18" t="n">
-        <v>5.3</v>
+        <v>6.2</v>
       </c>
       <c r="G18" t="n">
-        <v>5.6</v>
+        <v>6.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>21.62</v>
+        <v>13.69</v>
       </c>
       <c r="D19" t="n">
-        <v>1.6</v>
+        <v>1.29</v>
       </c>
       <c r="E19" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="F19" t="n">
-        <v>5.3</v>
+        <v>4.2</v>
       </c>
       <c r="G19" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>28.11</v>
+        <v>26.78</v>
       </c>
       <c r="D20" t="n">
-        <v>2.39</v>
+        <v>2.02</v>
       </c>
       <c r="E20" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="F20" t="n">
-        <v>5.3</v>
+        <v>4.2</v>
       </c>
       <c r="G20" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10.76</v>
+        <v>19.2</v>
       </c>
       <c r="D21" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.65</v>
       </c>
       <c r="E21" t="n">
-        <v>6.4</v>
+        <v>2.1</v>
       </c>
       <c r="F21" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="G21" t="n">
-        <v>4.9</v>
+        <v>3.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20.15</v>
+        <v>21.44</v>
       </c>
       <c r="D22" t="n">
-        <v>3.45</v>
+        <v>1.59</v>
       </c>
       <c r="E22" t="n">
-        <v>4.3</v>
+        <v>2.1</v>
       </c>
       <c r="F22" t="n">
-        <v>4.3</v>
+        <v>3.1</v>
       </c>
       <c r="G22" t="n">
-        <v>4.3</v>
+        <v>2.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>17.03</v>
+        <v>10.7</v>
       </c>
       <c r="D23" t="n">
-        <v>0.95</v>
+        <v>0.68</v>
       </c>
       <c r="E23" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="F23" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
       <c r="G23" t="n">
-        <v>3.5</v>
+        <v>2.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>19.33</v>
+        <v>23.71</v>
       </c>
       <c r="D24" t="n">
-        <v>1.65</v>
+        <v>2.21</v>
       </c>
       <c r="E24" t="n">
-        <v>4.3</v>
+        <v>2.1</v>
       </c>
       <c r="F24" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
       <c r="G24" t="n">
-        <v>3.5</v>
+        <v>2.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>57.97</v>
+        <v>22.09</v>
       </c>
       <c r="D25" t="n">
-        <v>3.78</v>
+        <v>1.83</v>
       </c>
       <c r="E25" t="n">
-        <v>4.3</v>
+        <v>2.1</v>
       </c>
       <c r="F25" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
       <c r="G25" t="n">
-        <v>3.5</v>
+        <v>2.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>24.89</v>
+        <v>14.47</v>
       </c>
       <c r="D26" t="n">
-        <v>2.05</v>
+        <v>1.18</v>
       </c>
       <c r="E26" t="n">
         <v>2.1</v>
       </c>
       <c r="F26" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
       <c r="G26" t="n">
-        <v>2.9</v>
+        <v>2.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="27">
@@ -1236,40 +1236,40 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.74</v>
+        <v>22.59</v>
       </c>
       <c r="D27" t="n">
-        <v>2.11</v>
+        <v>2.1</v>
       </c>
       <c r="E27" t="n">
         <v>2.1</v>
       </c>
       <c r="F27" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
       <c r="G27" t="n">
-        <v>2.9</v>
+        <v>2.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>24.06</v>
+        <v>30.31</v>
       </c>
       <c r="D28" t="n">
-        <v>2.24</v>
+        <v>2.33</v>
       </c>
       <c r="E28" t="n">
         <v>2.1</v>
@@ -1281,25 +1281,25 @@
         <v>2.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>22.34</v>
+        <v>32.95</v>
       </c>
       <c r="D29" t="n">
-        <v>1.85</v>
+        <v>3.56</v>
       </c>
       <c r="E29" t="n">
         <v>2.1</v>
@@ -1311,25 +1311,25 @@
         <v>2.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>33.3</v>
+        <v>44.68</v>
       </c>
       <c r="D30" t="n">
-        <v>3.59</v>
+        <v>3.75</v>
       </c>
       <c r="E30" t="n">
         <v>2.1</v>
@@ -1341,25 +1341,25 @@
         <v>2.1</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>46.06</v>
+        <v>24.17</v>
       </c>
       <c r="D31" t="n">
-        <v>3.86</v>
+        <v>1.99</v>
       </c>
       <c r="E31" t="n">
         <v>2.1</v>
@@ -1371,25 +1371,25 @@
         <v>2.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>13.67</v>
+        <v>27.82</v>
       </c>
       <c r="D32" t="n">
-        <v>1.28</v>
+        <v>2.36</v>
       </c>
       <c r="E32" t="n">
         <v>2.1</v>
@@ -1401,7 +1401,7 @@
         <v>2.1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Jun 12 12:44:20 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.07</v>
+        <v>7.17</v>
       </c>
       <c r="D2" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="E2" t="n">
-        <v>97.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>87.5</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>92.7</v>
+        <v>98</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>37.35</v>
+        <v>37.64</v>
       </c>
       <c r="D3" t="n">
-        <v>2.09</v>
+        <v>2.11</v>
       </c>
       <c r="E3" t="n">
-        <v>87.5</v>
+        <v>91.8</v>
       </c>
       <c r="F3" t="n">
-        <v>89.59999999999999</v>
+        <v>91.8</v>
       </c>
       <c r="G3" t="n">
-        <v>88.5</v>
+        <v>91.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +546,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>32.66</v>
+        <v>32.3</v>
       </c>
       <c r="D4" t="n">
-        <v>3.16</v>
+        <v>3.13</v>
       </c>
       <c r="E4" t="n">
-        <v>81.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>84.40000000000001</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>82.8</v>
+        <v>75.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="5">
@@ -576,22 +576,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>72.3</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>7.53</v>
+        <v>7.47</v>
       </c>
       <c r="E5" t="n">
-        <v>66.7</v>
+        <v>63.3</v>
       </c>
       <c r="F5" t="n">
-        <v>68.8</v>
+        <v>63.3</v>
       </c>
       <c r="G5" t="n">
-        <v>67.7</v>
+        <v>63.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="6">
@@ -606,742 +606,742 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>19.47</v>
+        <v>19.3</v>
       </c>
       <c r="D6" t="n">
-        <v>1.77</v>
+        <v>1.76</v>
       </c>
       <c r="E6" t="n">
-        <v>62.5</v>
+        <v>59.2</v>
       </c>
       <c r="F6" t="n">
-        <v>53.1</v>
+        <v>51</v>
       </c>
       <c r="G6" t="n">
-        <v>57.8</v>
+        <v>55.1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>40.74</v>
+        <v>20.3</v>
       </c>
       <c r="D7" t="n">
-        <v>3.47</v>
+        <v>1.9</v>
       </c>
       <c r="E7" t="n">
-        <v>41.7</v>
+        <v>51</v>
       </c>
       <c r="F7" t="n">
-        <v>47.9</v>
+        <v>51</v>
       </c>
       <c r="G7" t="n">
-        <v>44.8</v>
+        <v>51</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20.09</v>
+        <v>40.86</v>
       </c>
       <c r="D8" t="n">
-        <v>1.88</v>
+        <v>3.48</v>
       </c>
       <c r="E8" t="n">
-        <v>41.7</v>
+        <v>42.9</v>
       </c>
       <c r="F8" t="n">
-        <v>31.2</v>
+        <v>54.1</v>
       </c>
       <c r="G8" t="n">
-        <v>36.5</v>
+        <v>48.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15.96</v>
+        <v>10.02</v>
       </c>
       <c r="D9" t="n">
-        <v>2.37</v>
+        <v>1.22</v>
       </c>
       <c r="E9" t="n">
-        <v>39.6</v>
+        <v>42.9</v>
       </c>
       <c r="F9" t="n">
-        <v>22.9</v>
+        <v>43.9</v>
       </c>
       <c r="G9" t="n">
-        <v>27.9</v>
+        <v>43.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>116.6</v>
+        <v>27.37</v>
       </c>
       <c r="D10" t="n">
-        <v>4.4</v>
+        <v>2.55</v>
       </c>
       <c r="E10" t="n">
-        <v>27.1</v>
+        <v>32.7</v>
       </c>
       <c r="F10" t="n">
-        <v>28.1</v>
+        <v>35.7</v>
       </c>
       <c r="G10" t="n">
-        <v>27.8</v>
+        <v>34.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>26.97</v>
+        <v>19.92</v>
       </c>
       <c r="D11" t="n">
-        <v>2.5</v>
+        <v>3.53</v>
       </c>
       <c r="E11" t="n">
-        <v>29.2</v>
+        <v>20.4</v>
       </c>
       <c r="F11" t="n">
-        <v>26</v>
+        <v>21.4</v>
       </c>
       <c r="G11" t="n">
-        <v>27</v>
+        <v>21.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9.68</v>
+        <v>21.48</v>
       </c>
       <c r="D12" t="n">
-        <v>1.18</v>
+        <v>3.68</v>
       </c>
       <c r="E12" t="n">
-        <v>13.5</v>
+        <v>20.4</v>
       </c>
       <c r="F12" t="n">
-        <v>14.6</v>
+        <v>20.4</v>
       </c>
       <c r="G12" t="n">
-        <v>14.3</v>
+        <v>20.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11.15</v>
+        <v>17.62</v>
       </c>
       <c r="D13" t="n">
-        <v>1.01</v>
+        <v>0.98</v>
       </c>
       <c r="E13" t="n">
-        <v>6.2</v>
+        <v>20.4</v>
       </c>
       <c r="F13" t="n">
-        <v>17.7</v>
+        <v>19.4</v>
       </c>
       <c r="G13" t="n">
-        <v>14.3</v>
+        <v>19.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>19.78</v>
+        <v>27.46</v>
       </c>
       <c r="D14" t="n">
-        <v>3.49</v>
+        <v>2.07</v>
       </c>
       <c r="E14" t="n">
-        <v>10.4</v>
+        <v>20.4</v>
       </c>
       <c r="F14" t="n">
-        <v>9.4</v>
+        <v>18.4</v>
       </c>
       <c r="G14" t="n">
-        <v>9.699999999999999</v>
+        <v>19</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>20.53</v>
+        <v>26.57</v>
       </c>
       <c r="D15" t="n">
-        <v>3.52</v>
+        <v>2.48</v>
       </c>
       <c r="E15" t="n">
-        <v>8.300000000000001</v>
+        <v>18.4</v>
       </c>
       <c r="F15" t="n">
-        <v>8.300000000000001</v>
+        <v>18.4</v>
       </c>
       <c r="G15" t="n">
-        <v>8.300000000000001</v>
+        <v>18.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>17.18</v>
+        <v>111.64</v>
       </c>
       <c r="D16" t="n">
-        <v>0.96</v>
+        <v>4.21</v>
       </c>
       <c r="E16" t="n">
-        <v>8.300000000000001</v>
+        <v>18.4</v>
       </c>
       <c r="F16" t="n">
-        <v>7.3</v>
+        <v>18.4</v>
       </c>
       <c r="G16" t="n">
-        <v>7.6</v>
+        <v>18.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>26</v>
+        <v>11.31</v>
       </c>
       <c r="D17" t="n">
-        <v>2.43</v>
+        <v>1.02</v>
       </c>
       <c r="E17" t="n">
-        <v>6.2</v>
+        <v>10.2</v>
       </c>
       <c r="F17" t="n">
-        <v>6.2</v>
+        <v>20.4</v>
       </c>
       <c r="G17" t="n">
-        <v>6.2</v>
+        <v>17.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>58.16</v>
+        <v>15.83</v>
       </c>
       <c r="D18" t="n">
-        <v>3.79</v>
+        <v>2.36</v>
       </c>
       <c r="E18" t="n">
-        <v>6.2</v>
+        <v>19.4</v>
       </c>
       <c r="F18" t="n">
-        <v>6.2</v>
+        <v>13.3</v>
       </c>
       <c r="G18" t="n">
-        <v>6.2</v>
+        <v>15.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>13.69</v>
+        <v>59.66</v>
       </c>
       <c r="D19" t="n">
-        <v>1.29</v>
+        <v>3.9</v>
       </c>
       <c r="E19" t="n">
-        <v>4.2</v>
+        <v>14.3</v>
       </c>
       <c r="F19" t="n">
-        <v>4.2</v>
+        <v>15.3</v>
       </c>
       <c r="G19" t="n">
-        <v>4.2</v>
+        <v>15</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>26.78</v>
+        <v>19.58</v>
       </c>
       <c r="D20" t="n">
-        <v>2.02</v>
+        <v>1.68</v>
       </c>
       <c r="E20" t="n">
-        <v>4.2</v>
+        <v>12.2</v>
       </c>
       <c r="F20" t="n">
-        <v>4.2</v>
+        <v>15.3</v>
       </c>
       <c r="G20" t="n">
-        <v>4.2</v>
+        <v>14.4</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>19.2</v>
+        <v>30.97</v>
       </c>
       <c r="D21" t="n">
-        <v>1.65</v>
+        <v>2.4</v>
       </c>
       <c r="E21" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="F21" t="n">
-        <v>4.2</v>
+        <v>11.2</v>
       </c>
       <c r="G21" t="n">
-        <v>3.5</v>
+        <v>10.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21.44</v>
+        <v>28.75</v>
       </c>
       <c r="D22" t="n">
-        <v>1.59</v>
+        <v>2.44</v>
       </c>
       <c r="E22" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="F22" t="n">
-        <v>3.1</v>
+        <v>11.2</v>
       </c>
       <c r="G22" t="n">
-        <v>2.8</v>
+        <v>10.9</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10.7</v>
+        <v>14.76</v>
       </c>
       <c r="D23" t="n">
-        <v>0.68</v>
+        <v>1.21</v>
       </c>
       <c r="E23" t="n">
-        <v>4.2</v>
+        <v>10.2</v>
       </c>
       <c r="F23" t="n">
-        <v>2.1</v>
+        <v>11.2</v>
       </c>
       <c r="G23" t="n">
-        <v>2.7</v>
+        <v>10.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>23.71</v>
+        <v>22.66</v>
       </c>
       <c r="D24" t="n">
-        <v>2.21</v>
+        <v>1.88</v>
       </c>
       <c r="E24" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="F24" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="G24" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>22.09</v>
+        <v>21.87</v>
       </c>
       <c r="D25" t="n">
-        <v>1.83</v>
+        <v>1.62</v>
       </c>
       <c r="E25" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="F25" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="G25" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>14.47</v>
+        <v>22.95</v>
       </c>
       <c r="D26" t="n">
-        <v>1.18</v>
+        <v>2.13</v>
       </c>
       <c r="E26" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="F26" t="n">
-        <v>2.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>2.1</v>
+        <v>9.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.59</v>
+        <v>33.66</v>
       </c>
       <c r="D27" t="n">
-        <v>2.1</v>
+        <v>3.64</v>
       </c>
       <c r="E27" t="n">
-        <v>2.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F27" t="n">
-        <v>2.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G27" t="n">
-        <v>2.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>30.31</v>
+        <v>10.78</v>
       </c>
       <c r="D28" t="n">
-        <v>2.33</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E28" t="n">
-        <v>2.1</v>
+        <v>10.2</v>
       </c>
       <c r="F28" t="n">
-        <v>2.1</v>
+        <v>7.1</v>
       </c>
       <c r="G28" t="n">
-        <v>2.1</v>
+        <v>8.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>32.95</v>
+        <v>13.76</v>
       </c>
       <c r="D29" t="n">
-        <v>3.56</v>
+        <v>1.3</v>
       </c>
       <c r="E29" t="n">
-        <v>2.1</v>
+        <v>6.1</v>
       </c>
       <c r="F29" t="n">
-        <v>2.1</v>
+        <v>6.1</v>
       </c>
       <c r="G29" t="n">
-        <v>2.1</v>
+        <v>6.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>44.68</v>
+        <v>24.03</v>
       </c>
       <c r="D30" t="n">
-        <v>3.75</v>
+        <v>2.24</v>
       </c>
       <c r="E30" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
       <c r="F30" t="n">
-        <v>2.1</v>
+        <v>5.1</v>
       </c>
       <c r="G30" t="n">
-        <v>2.1</v>
+        <v>4.8</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="31">
@@ -1356,52 +1356,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>24.17</v>
+        <v>24.27</v>
       </c>
       <c r="D31" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
       <c r="E31" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
       <c r="F31" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
       <c r="G31" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>27.82</v>
+        <v>45.52</v>
       </c>
       <c r="D32" t="n">
-        <v>2.36</v>
+        <v>3.82</v>
       </c>
       <c r="E32" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
       <c r="F32" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
       <c r="G32" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Jun 13 11:32:27 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.68</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F2" t="n">
-        <v>95.90000000000001</v>
+        <v>95</v>
       </c>
       <c r="G2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.11</v>
       </c>
       <c r="E3" t="n">
-        <v>91.8</v>
+        <v>91</v>
       </c>
       <c r="F3" t="n">
-        <v>91.8</v>
+        <v>91</v>
       </c>
       <c r="G3" t="n">
-        <v>91.8</v>
+        <v>91</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.13</v>
       </c>
       <c r="E4" t="n">
-        <v>71.40000000000001</v>
+        <v>71</v>
       </c>
       <c r="F4" t="n">
-        <v>79.59999999999999</v>
+        <v>79</v>
       </c>
       <c r="G4" t="n">
-        <v>75.5</v>
+        <v>75</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>7.47</v>
       </c>
       <c r="E5" t="n">
-        <v>63.3</v>
+        <v>63</v>
       </c>
       <c r="F5" t="n">
-        <v>63.3</v>
+        <v>63</v>
       </c>
       <c r="G5" t="n">
-        <v>63.3</v>
+        <v>63</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.76</v>
       </c>
       <c r="E6" t="n">
-        <v>59.2</v>
+        <v>59</v>
       </c>
       <c r="F6" t="n">
         <v>51</v>
       </c>
       <c r="G6" t="n">
-        <v>55.1</v>
+        <v>55</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         <v>51</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>3.48</v>
       </c>
       <c r="E8" t="n">
-        <v>42.9</v>
+        <v>43</v>
       </c>
       <c r="F8" t="n">
-        <v>54.1</v>
+        <v>54</v>
       </c>
       <c r="G8" t="n">
         <v>48.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.22</v>
       </c>
       <c r="E9" t="n">
-        <v>42.9</v>
+        <v>43</v>
       </c>
       <c r="F9" t="n">
-        <v>43.9</v>
+        <v>44</v>
       </c>
       <c r="G9" t="n">
-        <v>43.4</v>
+        <v>43.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.55</v>
       </c>
       <c r="E10" t="n">
-        <v>32.7</v>
+        <v>33</v>
       </c>
       <c r="F10" t="n">
-        <v>35.7</v>
+        <v>36</v>
       </c>
       <c r="G10" t="n">
-        <v>34.2</v>
+        <v>34.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>3.53</v>
       </c>
       <c r="E11" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="F11" t="n">
-        <v>21.4</v>
+        <v>22</v>
       </c>
       <c r="G11" t="n">
-        <v>21.1</v>
+        <v>21.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.68</v>
       </c>
       <c r="E12" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="F12" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="G12" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>0.98</v>
       </c>
       <c r="E13" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="F13" t="n">
-        <v>19.4</v>
+        <v>20</v>
       </c>
       <c r="G13" t="n">
-        <v>19.7</v>
+        <v>20.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.07</v>
       </c>
       <c r="E14" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="F14" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="G14" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.48</v>
       </c>
       <c r="E15" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="F15" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="G15" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>4.21</v>
       </c>
       <c r="E16" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="F16" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="G16" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.02</v>
       </c>
       <c r="E17" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="F17" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="G17" t="n">
-        <v>17.3</v>
+        <v>18</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.36</v>
       </c>
       <c r="E18" t="n">
-        <v>19.4</v>
+        <v>20</v>
       </c>
       <c r="F18" t="n">
-        <v>13.3</v>
+        <v>14</v>
       </c>
       <c r="G18" t="n">
-        <v>15.1</v>
+        <v>15.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>3.9</v>
       </c>
       <c r="E19" t="n">
-        <v>14.3</v>
+        <v>15</v>
       </c>
       <c r="F19" t="n">
-        <v>15.3</v>
+        <v>16</v>
       </c>
       <c r="G19" t="n">
-        <v>15</v>
+        <v>15.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.68</v>
       </c>
       <c r="E20" t="n">
-        <v>12.2</v>
+        <v>13</v>
       </c>
       <c r="F20" t="n">
-        <v>15.3</v>
+        <v>16</v>
       </c>
       <c r="G20" t="n">
-        <v>14.4</v>
+        <v>15.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.4</v>
       </c>
       <c r="E21" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="F21" t="n">
-        <v>11.2</v>
+        <v>12</v>
       </c>
       <c r="G21" t="n">
-        <v>10.9</v>
+        <v>11.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.44</v>
       </c>
       <c r="E22" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="F22" t="n">
-        <v>11.2</v>
+        <v>12</v>
       </c>
       <c r="G22" t="n">
-        <v>10.9</v>
+        <v>11.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.21</v>
       </c>
       <c r="E23" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="F23" t="n">
-        <v>11.2</v>
+        <v>12</v>
       </c>
       <c r="G23" t="n">
-        <v>10.9</v>
+        <v>11.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.88</v>
       </c>
       <c r="E24" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="F24" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="G24" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.62</v>
       </c>
       <c r="E25" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="F25" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="G25" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.13</v>
       </c>
       <c r="E26" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="F26" t="n">
-        <v>9.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="G26" t="n">
-        <v>9.5</v>
+        <v>10.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.64</v>
       </c>
       <c r="E27" t="n">
-        <v>8.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="F27" t="n">
-        <v>8.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="G27" t="n">
-        <v>8.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E28" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="F28" t="n">
-        <v>7.1</v>
+        <v>8</v>
       </c>
       <c r="G28" t="n">
-        <v>8.1</v>
+        <v>8.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.3</v>
       </c>
       <c r="E29" t="n">
-        <v>6.1</v>
+        <v>7</v>
       </c>
       <c r="F29" t="n">
-        <v>6.1</v>
+        <v>7</v>
       </c>
       <c r="G29" t="n">
-        <v>6.1</v>
+        <v>7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.24</v>
       </c>
       <c r="E30" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="F30" t="n">
-        <v>5.1</v>
+        <v>6</v>
       </c>
       <c r="G30" t="n">
-        <v>4.8</v>
+        <v>5.7</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>2</v>
       </c>
       <c r="E31" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="F31" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="G31" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>3.82</v>
       </c>
       <c r="E32" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="G32" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Jun 14 11:47:18 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.68</v>
       </c>
       <c r="E2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F2" t="n">
-        <v>95</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>97</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.11</v>
       </c>
       <c r="E3" t="n">
-        <v>91</v>
+        <v>90.2</v>
       </c>
       <c r="F3" t="n">
-        <v>91</v>
+        <v>90.2</v>
       </c>
       <c r="G3" t="n">
-        <v>91</v>
+        <v>90.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.13</v>
       </c>
       <c r="E4" t="n">
-        <v>71</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>79</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>75</v>
+        <v>74.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>7.47</v>
       </c>
       <c r="E5" t="n">
-        <v>63</v>
+        <v>62.7</v>
       </c>
       <c r="F5" t="n">
-        <v>63</v>
+        <v>62.7</v>
       </c>
       <c r="G5" t="n">
-        <v>63</v>
+        <v>62.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.76</v>
       </c>
       <c r="E6" t="n">
-        <v>59</v>
+        <v>58.8</v>
       </c>
       <c r="F6" t="n">
         <v>51</v>
       </c>
       <c r="G6" t="n">
-        <v>55</v>
+        <v>54.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         <v>51</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>3.48</v>
       </c>
       <c r="E8" t="n">
-        <v>43</v>
+        <v>43.1</v>
       </c>
       <c r="F8" t="n">
-        <v>54</v>
+        <v>53.9</v>
       </c>
       <c r="G8" t="n">
         <v>48.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.22</v>
       </c>
       <c r="E9" t="n">
-        <v>43</v>
+        <v>43.1</v>
       </c>
       <c r="F9" t="n">
-        <v>44</v>
+        <v>44.1</v>
       </c>
       <c r="G9" t="n">
-        <v>43.5</v>
+        <v>43.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.55</v>
       </c>
       <c r="E10" t="n">
-        <v>33</v>
+        <v>33.3</v>
       </c>
       <c r="F10" t="n">
-        <v>36</v>
+        <v>36.3</v>
       </c>
       <c r="G10" t="n">
-        <v>34.5</v>
+        <v>34.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>3.53</v>
       </c>
       <c r="E11" t="n">
-        <v>21</v>
+        <v>21.6</v>
       </c>
       <c r="F11" t="n">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="G11" t="n">
-        <v>21.7</v>
+        <v>22.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.68</v>
       </c>
       <c r="E12" t="n">
-        <v>21</v>
+        <v>21.6</v>
       </c>
       <c r="F12" t="n">
-        <v>21</v>
+        <v>21.6</v>
       </c>
       <c r="G12" t="n">
-        <v>21</v>
+        <v>21.6</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>0.98</v>
       </c>
       <c r="E13" t="n">
-        <v>21</v>
+        <v>21.6</v>
       </c>
       <c r="F13" t="n">
-        <v>20</v>
+        <v>20.6</v>
       </c>
       <c r="G13" t="n">
-        <v>20.3</v>
+        <v>20.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.07</v>
       </c>
       <c r="E14" t="n">
-        <v>21</v>
+        <v>21.6</v>
       </c>
       <c r="F14" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="G14" t="n">
-        <v>19.6</v>
+        <v>20.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.48</v>
       </c>
       <c r="E15" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="F15" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="G15" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>4.21</v>
       </c>
       <c r="E16" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="F16" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="G16" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.02</v>
       </c>
       <c r="E17" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="F17" t="n">
-        <v>21</v>
+        <v>21.6</v>
       </c>
       <c r="G17" t="n">
-        <v>18</v>
+        <v>18.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.36</v>
       </c>
       <c r="E18" t="n">
-        <v>20</v>
+        <v>20.6</v>
       </c>
       <c r="F18" t="n">
-        <v>14</v>
+        <v>14.7</v>
       </c>
       <c r="G18" t="n">
-        <v>15.8</v>
+        <v>16.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>3.9</v>
       </c>
       <c r="E19" t="n">
-        <v>15</v>
+        <v>15.7</v>
       </c>
       <c r="F19" t="n">
-        <v>16</v>
+        <v>16.7</v>
       </c>
       <c r="G19" t="n">
-        <v>15.7</v>
+        <v>16.4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.68</v>
       </c>
       <c r="E20" t="n">
-        <v>13</v>
+        <v>13.7</v>
       </c>
       <c r="F20" t="n">
-        <v>16</v>
+        <v>16.7</v>
       </c>
       <c r="G20" t="n">
-        <v>15.1</v>
+        <v>15.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.4</v>
       </c>
       <c r="E21" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="F21" t="n">
-        <v>12</v>
+        <v>12.7</v>
       </c>
       <c r="G21" t="n">
-        <v>11.7</v>
+        <v>12.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.44</v>
       </c>
       <c r="E22" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="F22" t="n">
-        <v>12</v>
+        <v>12.7</v>
       </c>
       <c r="G22" t="n">
-        <v>11.7</v>
+        <v>12.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.21</v>
       </c>
       <c r="E23" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="F23" t="n">
-        <v>12</v>
+        <v>12.7</v>
       </c>
       <c r="G23" t="n">
-        <v>11.7</v>
+        <v>12.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.88</v>
       </c>
       <c r="E24" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="F24" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="G24" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.62</v>
       </c>
       <c r="E25" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="F25" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="G25" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.13</v>
       </c>
       <c r="E26" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="F26" t="n">
-        <v>10</v>
+        <v>10.8</v>
       </c>
       <c r="G26" t="n">
-        <v>10.3</v>
+        <v>11.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.64</v>
       </c>
       <c r="E27" t="n">
-        <v>9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F27" t="n">
-        <v>9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G27" t="n">
-        <v>9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E28" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="F28" t="n">
-        <v>8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>8.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.3</v>
       </c>
       <c r="E29" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="F29" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="G29" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.24</v>
       </c>
       <c r="E30" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="F30" t="n">
-        <v>6</v>
+        <v>6.9</v>
       </c>
       <c r="G30" t="n">
-        <v>5.7</v>
+        <v>6.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>2</v>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="F31" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="G31" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>3.82</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="F32" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="G32" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Jun 15 15:32:30 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,241 +477,241 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.17</v>
+        <v>40.32</v>
       </c>
       <c r="D2" t="n">
-        <v>0.68</v>
+        <v>2.25</v>
       </c>
       <c r="E2" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>96.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>37.64</v>
+        <v>33.65</v>
       </c>
       <c r="D3" t="n">
-        <v>2.11</v>
+        <v>3.27</v>
       </c>
       <c r="E3" t="n">
-        <v>90.2</v>
+        <v>94.2</v>
       </c>
       <c r="F3" t="n">
-        <v>90.2</v>
+        <v>99</v>
       </c>
       <c r="G3" t="n">
-        <v>90.2</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>32.3</v>
+        <v>76.15000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>3.13</v>
+        <v>7.94</v>
       </c>
       <c r="E4" t="n">
-        <v>70.59999999999999</v>
+        <v>96.2</v>
       </c>
       <c r="F4" t="n">
-        <v>78.40000000000001</v>
+        <v>96.2</v>
       </c>
       <c r="G4" t="n">
-        <v>74.5</v>
+        <v>96.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>71.59999999999999</v>
+        <v>42.82</v>
       </c>
       <c r="D5" t="n">
-        <v>7.47</v>
+        <v>3.65</v>
       </c>
       <c r="E5" t="n">
-        <v>62.7</v>
+        <v>92.3</v>
       </c>
       <c r="F5" t="n">
-        <v>62.7</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>62.7</v>
+        <v>95.2</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>19.3</v>
+        <v>7.02</v>
       </c>
       <c r="D6" t="n">
-        <v>1.76</v>
+        <v>0.67</v>
       </c>
       <c r="E6" t="n">
-        <v>58.8</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>51</v>
+        <v>81.7</v>
       </c>
       <c r="G6" t="n">
-        <v>54.9</v>
+        <v>83.7</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.3</v>
+        <v>22.54</v>
       </c>
       <c r="D7" t="n">
-        <v>1.9</v>
+        <v>3.86</v>
       </c>
       <c r="E7" t="n">
-        <v>51</v>
+        <v>57.7</v>
       </c>
       <c r="F7" t="n">
-        <v>51</v>
+        <v>67.3</v>
       </c>
       <c r="G7" t="n">
-        <v>51</v>
+        <v>62.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>40.86</v>
+        <v>10.23</v>
       </c>
       <c r="D8" t="n">
-        <v>3.48</v>
+        <v>1.25</v>
       </c>
       <c r="E8" t="n">
-        <v>43.1</v>
+        <v>63.5</v>
       </c>
       <c r="F8" t="n">
-        <v>53.9</v>
+        <v>57.7</v>
       </c>
       <c r="G8" t="n">
-        <v>48.5</v>
+        <v>60.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10.02</v>
+        <v>20.36</v>
       </c>
       <c r="D9" t="n">
-        <v>1.22</v>
+        <v>1.9</v>
       </c>
       <c r="E9" t="n">
-        <v>43.1</v>
+        <v>55.8</v>
       </c>
       <c r="F9" t="n">
-        <v>44.1</v>
+        <v>51</v>
       </c>
       <c r="G9" t="n">
-        <v>43.6</v>
+        <v>53.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="10">
@@ -726,412 +726,412 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>27.37</v>
+        <v>28.15</v>
       </c>
       <c r="D10" t="n">
-        <v>2.55</v>
+        <v>2.62</v>
       </c>
       <c r="E10" t="n">
-        <v>33.3</v>
+        <v>46.2</v>
       </c>
       <c r="F10" t="n">
-        <v>36.3</v>
+        <v>51.9</v>
       </c>
       <c r="G10" t="n">
-        <v>34.8</v>
+        <v>49</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.92</v>
+        <v>60.49</v>
       </c>
       <c r="D11" t="n">
-        <v>3.53</v>
+        <v>3.95</v>
       </c>
       <c r="E11" t="n">
-        <v>21.6</v>
+        <v>34.6</v>
       </c>
       <c r="F11" t="n">
-        <v>22.5</v>
+        <v>34.6</v>
       </c>
       <c r="G11" t="n">
-        <v>22.3</v>
+        <v>34.6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>21.48</v>
+        <v>115.1</v>
       </c>
       <c r="D12" t="n">
-        <v>3.68</v>
+        <v>4.34</v>
       </c>
       <c r="E12" t="n">
-        <v>21.6</v>
+        <v>28.8</v>
       </c>
       <c r="F12" t="n">
-        <v>21.6</v>
+        <v>28.8</v>
       </c>
       <c r="G12" t="n">
-        <v>21.6</v>
+        <v>28.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>17.62</v>
+        <v>31.8</v>
       </c>
       <c r="D13" t="n">
-        <v>0.98</v>
+        <v>2.46</v>
       </c>
       <c r="E13" t="n">
-        <v>21.6</v>
+        <v>25</v>
       </c>
       <c r="F13" t="n">
-        <v>20.6</v>
+        <v>32.7</v>
       </c>
       <c r="G13" t="n">
-        <v>20.9</v>
+        <v>28.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>27.46</v>
+        <v>19.85</v>
       </c>
       <c r="D14" t="n">
-        <v>2.07</v>
+        <v>1.7</v>
       </c>
       <c r="E14" t="n">
-        <v>21.6</v>
+        <v>25</v>
       </c>
       <c r="F14" t="n">
-        <v>19.6</v>
+        <v>28.8</v>
       </c>
       <c r="G14" t="n">
-        <v>20.2</v>
+        <v>27.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26.57</v>
+        <v>17.68</v>
       </c>
       <c r="D15" t="n">
-        <v>2.48</v>
+        <v>0.99</v>
       </c>
       <c r="E15" t="n">
-        <v>19.6</v>
+        <v>25</v>
       </c>
       <c r="F15" t="n">
-        <v>19.6</v>
+        <v>26.9</v>
       </c>
       <c r="G15" t="n">
-        <v>19.6</v>
+        <v>26.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>111.64</v>
+        <v>27.63</v>
       </c>
       <c r="D16" t="n">
-        <v>4.21</v>
+        <v>2.08</v>
       </c>
       <c r="E16" t="n">
-        <v>19.6</v>
+        <v>25</v>
       </c>
       <c r="F16" t="n">
-        <v>19.6</v>
+        <v>23.1</v>
       </c>
       <c r="G16" t="n">
-        <v>19.6</v>
+        <v>23.7</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>11.31</v>
+        <v>22.24</v>
       </c>
       <c r="D17" t="n">
-        <v>1.02</v>
+        <v>1.65</v>
       </c>
       <c r="E17" t="n">
-        <v>11.8</v>
+        <v>21.2</v>
       </c>
       <c r="F17" t="n">
-        <v>21.6</v>
+        <v>22.1</v>
       </c>
       <c r="G17" t="n">
-        <v>18.6</v>
+        <v>21.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>15.83</v>
+        <v>14.89</v>
       </c>
       <c r="D18" t="n">
-        <v>2.36</v>
+        <v>1.22</v>
       </c>
       <c r="E18" t="n">
-        <v>20.6</v>
+        <v>23.1</v>
       </c>
       <c r="F18" t="n">
-        <v>14.7</v>
+        <v>20.2</v>
       </c>
       <c r="G18" t="n">
-        <v>16.5</v>
+        <v>21.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>59.66</v>
+        <v>11.35</v>
       </c>
       <c r="D19" t="n">
-        <v>3.9</v>
+        <v>1.02</v>
       </c>
       <c r="E19" t="n">
-        <v>15.7</v>
+        <v>15.4</v>
       </c>
       <c r="F19" t="n">
-        <v>16.7</v>
+        <v>22.1</v>
       </c>
       <c r="G19" t="n">
-        <v>16.4</v>
+        <v>20.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>19.58</v>
+        <v>10.91</v>
       </c>
       <c r="D20" t="n">
-        <v>1.68</v>
+        <v>0.7</v>
       </c>
       <c r="E20" t="n">
-        <v>13.7</v>
+        <v>17.3</v>
       </c>
       <c r="F20" t="n">
-        <v>16.7</v>
+        <v>19.2</v>
       </c>
       <c r="G20" t="n">
-        <v>15.8</v>
+        <v>18.7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>30.97</v>
+        <v>26.55</v>
       </c>
       <c r="D21" t="n">
-        <v>2.4</v>
+        <v>2.48</v>
       </c>
       <c r="E21" t="n">
-        <v>11.8</v>
+        <v>12.5</v>
       </c>
       <c r="F21" t="n">
-        <v>12.7</v>
+        <v>20.2</v>
       </c>
       <c r="G21" t="n">
-        <v>12.5</v>
+        <v>17.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28.75</v>
+        <v>22.98</v>
       </c>
       <c r="D22" t="n">
-        <v>2.44</v>
+        <v>2.14</v>
       </c>
       <c r="E22" t="n">
-        <v>11.8</v>
+        <v>15.4</v>
       </c>
       <c r="F22" t="n">
-        <v>12.7</v>
+        <v>15.4</v>
       </c>
       <c r="G22" t="n">
-        <v>12.5</v>
+        <v>15.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>14.76</v>
+        <v>34.61</v>
       </c>
       <c r="D23" t="n">
-        <v>1.21</v>
+        <v>3.74</v>
       </c>
       <c r="E23" t="n">
-        <v>11.8</v>
+        <v>15.4</v>
       </c>
       <c r="F23" t="n">
-        <v>12.7</v>
+        <v>15.4</v>
       </c>
       <c r="G23" t="n">
-        <v>12.5</v>
+        <v>15.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="24">
@@ -1146,262 +1146,262 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.66</v>
+        <v>22.94</v>
       </c>
       <c r="D24" t="n">
-        <v>1.88</v>
+        <v>1.9</v>
       </c>
       <c r="E24" t="n">
-        <v>11.8</v>
+        <v>15.4</v>
       </c>
       <c r="F24" t="n">
-        <v>11.8</v>
+        <v>15.4</v>
       </c>
       <c r="G24" t="n">
-        <v>11.8</v>
+        <v>15.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21.87</v>
+        <v>28.77</v>
       </c>
       <c r="D25" t="n">
-        <v>1.62</v>
+        <v>2.44</v>
       </c>
       <c r="E25" t="n">
-        <v>11.8</v>
+        <v>15.4</v>
       </c>
       <c r="F25" t="n">
-        <v>11.8</v>
+        <v>13.5</v>
       </c>
       <c r="G25" t="n">
-        <v>11.8</v>
+        <v>14</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>22.95</v>
+        <v>46.89</v>
       </c>
       <c r="D26" t="n">
-        <v>2.13</v>
+        <v>3.93</v>
       </c>
       <c r="E26" t="n">
-        <v>11.8</v>
+        <v>13.5</v>
       </c>
       <c r="F26" t="n">
-        <v>10.8</v>
+        <v>13.5</v>
       </c>
       <c r="G26" t="n">
-        <v>11.1</v>
+        <v>13.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>33.66</v>
+        <v>19.7</v>
       </c>
       <c r="D27" t="n">
-        <v>3.64</v>
+        <v>3.5</v>
       </c>
       <c r="E27" t="n">
-        <v>9.800000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="F27" t="n">
-        <v>9.800000000000001</v>
+        <v>14.4</v>
       </c>
       <c r="G27" t="n">
-        <v>9.800000000000001</v>
+        <v>12.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>10.78</v>
+        <v>18.18</v>
       </c>
       <c r="D28" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.66</v>
       </c>
       <c r="E28" t="n">
-        <v>11.8</v>
+        <v>13.5</v>
       </c>
       <c r="F28" t="n">
-        <v>8.800000000000001</v>
+        <v>11.5</v>
       </c>
       <c r="G28" t="n">
-        <v>9.699999999999999</v>
+        <v>12.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>13.76</v>
+        <v>24.48</v>
       </c>
       <c r="D29" t="n">
-        <v>1.3</v>
+        <v>2.28</v>
       </c>
       <c r="E29" t="n">
-        <v>7.8</v>
+        <v>11.5</v>
       </c>
       <c r="F29" t="n">
-        <v>7.8</v>
+        <v>11.5</v>
       </c>
       <c r="G29" t="n">
-        <v>7.8</v>
+        <v>11.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>24.03</v>
+        <v>24.52</v>
       </c>
       <c r="D30" t="n">
-        <v>2.24</v>
+        <v>2.02</v>
       </c>
       <c r="E30" t="n">
-        <v>5.9</v>
+        <v>9.6</v>
       </c>
       <c r="F30" t="n">
-        <v>6.9</v>
+        <v>9.6</v>
       </c>
       <c r="G30" t="n">
-        <v>6.6</v>
+        <v>9.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>24.27</v>
+        <v>15.8</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>2.35</v>
       </c>
       <c r="E31" t="n">
-        <v>5.9</v>
+        <v>15.4</v>
       </c>
       <c r="F31" t="n">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="G31" t="n">
-        <v>5.9</v>
+        <v>8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>45.52</v>
+        <v>13.49</v>
       </c>
       <c r="D32" t="n">
-        <v>3.82</v>
+        <v>1.27</v>
       </c>
       <c r="E32" t="n">
-        <v>5.9</v>
+        <v>1.9</v>
       </c>
       <c r="F32" t="n">
-        <v>5.9</v>
+        <v>1.9</v>
       </c>
       <c r="G32" t="n">
-        <v>5.9</v>
+        <v>1.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Jun 16 14:33:55 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>40.32</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>2.25</v>
+        <v>8.08</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,127 +501,127 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>33.65</v>
+        <v>42.74</v>
       </c>
       <c r="D3" t="n">
-        <v>3.27</v>
+        <v>2.38</v>
       </c>
       <c r="E3" t="n">
-        <v>94.2</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>96.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>76.15000000000001</v>
+        <v>43.52</v>
       </c>
       <c r="D4" t="n">
-        <v>7.94</v>
+        <v>3.68</v>
       </c>
       <c r="E4" t="n">
-        <v>96.2</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>96.2</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>96.2</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>42.82</v>
+        <v>34.17</v>
       </c>
       <c r="D5" t="n">
-        <v>3.65</v>
+        <v>3.24</v>
       </c>
       <c r="E5" t="n">
-        <v>92.3</v>
+        <v>96.2</v>
       </c>
       <c r="F5" t="n">
-        <v>98.09999999999999</v>
+        <v>92.5</v>
       </c>
       <c r="G5" t="n">
-        <v>95.2</v>
+        <v>94.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7.02</v>
+        <v>10.21</v>
       </c>
       <c r="D6" t="n">
-        <v>0.67</v>
+        <v>1.24</v>
       </c>
       <c r="E6" t="n">
-        <v>85.59999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="F6" t="n">
-        <v>81.7</v>
+        <v>56.6</v>
       </c>
       <c r="G6" t="n">
-        <v>83.7</v>
+        <v>59.4</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="7">
@@ -636,112 +636,112 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>22.54</v>
+        <v>22.87</v>
       </c>
       <c r="D7" t="n">
-        <v>3.86</v>
+        <v>3.78</v>
       </c>
       <c r="E7" t="n">
-        <v>57.7</v>
+        <v>58.5</v>
       </c>
       <c r="F7" t="n">
-        <v>67.3</v>
+        <v>55.7</v>
       </c>
       <c r="G7" t="n">
-        <v>62.5</v>
+        <v>57.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10.23</v>
+        <v>6.91</v>
       </c>
       <c r="D8" t="n">
-        <v>1.25</v>
+        <v>0.65</v>
       </c>
       <c r="E8" t="n">
-        <v>63.5</v>
+        <v>62.3</v>
       </c>
       <c r="F8" t="n">
-        <v>57.7</v>
+        <v>46.2</v>
       </c>
       <c r="G8" t="n">
-        <v>60.6</v>
+        <v>54.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20.36</v>
+        <v>28.18</v>
       </c>
       <c r="D9" t="n">
-        <v>1.9</v>
+        <v>2.58</v>
       </c>
       <c r="E9" t="n">
-        <v>55.8</v>
+        <v>47.2</v>
       </c>
       <c r="F9" t="n">
-        <v>51</v>
+        <v>42.5</v>
       </c>
       <c r="G9" t="n">
-        <v>53.4</v>
+        <v>44.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28.15</v>
+        <v>20.22</v>
       </c>
       <c r="D10" t="n">
-        <v>2.62</v>
+        <v>1.89</v>
       </c>
       <c r="E10" t="n">
-        <v>46.2</v>
+        <v>47.2</v>
       </c>
       <c r="F10" t="n">
-        <v>51.9</v>
+        <v>39.6</v>
       </c>
       <c r="G10" t="n">
-        <v>49</v>
+        <v>43.4</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="11">
@@ -756,232 +756,232 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>60.49</v>
+        <v>61.07</v>
       </c>
       <c r="D11" t="n">
-        <v>3.95</v>
+        <v>3.92</v>
       </c>
       <c r="E11" t="n">
-        <v>34.6</v>
+        <v>35.8</v>
       </c>
       <c r="F11" t="n">
-        <v>34.6</v>
+        <v>25.5</v>
       </c>
       <c r="G11" t="n">
-        <v>34.6</v>
+        <v>28.6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>115.1</v>
+        <v>35.56</v>
       </c>
       <c r="D12" t="n">
-        <v>4.34</v>
+        <v>3.84</v>
       </c>
       <c r="E12" t="n">
-        <v>28.8</v>
+        <v>28.3</v>
       </c>
       <c r="F12" t="n">
-        <v>28.8</v>
+        <v>24.5</v>
       </c>
       <c r="G12" t="n">
-        <v>28.8</v>
+        <v>25.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>31.8</v>
+        <v>113.92</v>
       </c>
       <c r="D13" t="n">
-        <v>2.46</v>
+        <v>4.28</v>
       </c>
       <c r="E13" t="n">
-        <v>25</v>
+        <v>22.6</v>
       </c>
       <c r="F13" t="n">
-        <v>32.7</v>
+        <v>22.6</v>
       </c>
       <c r="G13" t="n">
-        <v>28.8</v>
+        <v>22.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>19.85</v>
+        <v>22.29</v>
       </c>
       <c r="D14" t="n">
-        <v>1.7</v>
+        <v>1.64</v>
       </c>
       <c r="E14" t="n">
-        <v>25</v>
+        <v>23.6</v>
       </c>
       <c r="F14" t="n">
-        <v>28.8</v>
+        <v>20.8</v>
       </c>
       <c r="G14" t="n">
-        <v>27.7</v>
+        <v>21.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>17.68</v>
+        <v>31.8</v>
       </c>
       <c r="D15" t="n">
-        <v>0.99</v>
+        <v>2.42</v>
       </c>
       <c r="E15" t="n">
-        <v>25</v>
+        <v>25.5</v>
       </c>
       <c r="F15" t="n">
-        <v>26.9</v>
+        <v>19.8</v>
       </c>
       <c r="G15" t="n">
-        <v>26.3</v>
+        <v>21.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>27.63</v>
+        <v>10.89</v>
       </c>
       <c r="D16" t="n">
-        <v>2.08</v>
+        <v>0.7</v>
       </c>
       <c r="E16" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F16" t="n">
-        <v>23.1</v>
+        <v>19.8</v>
       </c>
       <c r="G16" t="n">
-        <v>23.7</v>
+        <v>19</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>22.24</v>
+        <v>23</v>
       </c>
       <c r="D17" t="n">
-        <v>1.65</v>
+        <v>1.89</v>
       </c>
       <c r="E17" t="n">
-        <v>21.2</v>
+        <v>17</v>
       </c>
       <c r="F17" t="n">
-        <v>22.1</v>
+        <v>15.1</v>
       </c>
       <c r="G17" t="n">
-        <v>21.8</v>
+        <v>15.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>14.89</v>
+        <v>47.47</v>
       </c>
       <c r="D18" t="n">
-        <v>1.22</v>
+        <v>3.89</v>
       </c>
       <c r="E18" t="n">
-        <v>23.1</v>
+        <v>17</v>
       </c>
       <c r="F18" t="n">
-        <v>20.2</v>
+        <v>13.2</v>
       </c>
       <c r="G18" t="n">
-        <v>21.1</v>
+        <v>14.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="19">
@@ -996,322 +996,322 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>11.35</v>
+        <v>11.16</v>
       </c>
       <c r="D19" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>15.4</v>
+        <v>7.5</v>
       </c>
       <c r="F19" t="n">
-        <v>22.1</v>
+        <v>13.2</v>
       </c>
       <c r="G19" t="n">
-        <v>20.1</v>
+        <v>11.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>10.91</v>
+        <v>17.36</v>
       </c>
       <c r="D20" t="n">
-        <v>0.7</v>
+        <v>0.96</v>
       </c>
       <c r="E20" t="n">
-        <v>17.3</v>
+        <v>11.3</v>
       </c>
       <c r="F20" t="n">
-        <v>19.2</v>
+        <v>7.5</v>
       </c>
       <c r="G20" t="n">
-        <v>18.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>26.55</v>
+        <v>19.69</v>
       </c>
       <c r="D21" t="n">
-        <v>2.48</v>
+        <v>1.64</v>
       </c>
       <c r="E21" t="n">
-        <v>12.5</v>
+        <v>24.5</v>
       </c>
       <c r="F21" t="n">
-        <v>20.2</v>
+        <v>1.9</v>
       </c>
       <c r="G21" t="n">
-        <v>17.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22.98</v>
+        <v>27.27</v>
       </c>
       <c r="D22" t="n">
-        <v>2.14</v>
+        <v>2.02</v>
       </c>
       <c r="E22" t="n">
-        <v>15.4</v>
+        <v>14.2</v>
       </c>
       <c r="F22" t="n">
-        <v>15.4</v>
+        <v>4.7</v>
       </c>
       <c r="G22" t="n">
-        <v>15.4</v>
+        <v>7.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>34.61</v>
+        <v>28.49</v>
       </c>
       <c r="D23" t="n">
-        <v>3.74</v>
+        <v>2.38</v>
       </c>
       <c r="E23" t="n">
-        <v>15.4</v>
+        <v>9.4</v>
       </c>
       <c r="F23" t="n">
-        <v>15.4</v>
+        <v>4.7</v>
       </c>
       <c r="G23" t="n">
-        <v>15.4</v>
+        <v>6.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.94</v>
+        <v>24.19</v>
       </c>
       <c r="D24" t="n">
-        <v>1.9</v>
+        <v>2.23</v>
       </c>
       <c r="E24" t="n">
-        <v>15.4</v>
+        <v>11.3</v>
       </c>
       <c r="F24" t="n">
-        <v>15.4</v>
+        <v>3.8</v>
       </c>
       <c r="G24" t="n">
-        <v>15.4</v>
+        <v>6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.77</v>
+        <v>17.79</v>
       </c>
       <c r="D25" t="n">
-        <v>2.44</v>
+        <v>1.65</v>
       </c>
       <c r="E25" t="n">
-        <v>15.4</v>
+        <v>1.9</v>
       </c>
       <c r="F25" t="n">
-        <v>13.5</v>
+        <v>7.5</v>
       </c>
       <c r="G25" t="n">
-        <v>14</v>
+        <v>5.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>46.89</v>
+        <v>15.63</v>
       </c>
       <c r="D26" t="n">
-        <v>3.93</v>
+        <v>2.31</v>
       </c>
       <c r="E26" t="n">
-        <v>13.5</v>
+        <v>13.2</v>
       </c>
       <c r="F26" t="n">
-        <v>13.5</v>
+        <v>1.9</v>
       </c>
       <c r="G26" t="n">
-        <v>13.5</v>
+        <v>5.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>19.7</v>
+        <v>14.59</v>
       </c>
       <c r="D27" t="n">
-        <v>3.5</v>
+        <v>1.19</v>
       </c>
       <c r="E27" t="n">
-        <v>7.7</v>
+        <v>5.7</v>
       </c>
       <c r="F27" t="n">
-        <v>14.4</v>
+        <v>4.7</v>
       </c>
       <c r="G27" t="n">
-        <v>12.4</v>
+        <v>5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18.18</v>
+        <v>22.87</v>
       </c>
       <c r="D28" t="n">
-        <v>1.66</v>
+        <v>2.07</v>
       </c>
       <c r="E28" t="n">
-        <v>13.5</v>
+        <v>7.5</v>
       </c>
       <c r="F28" t="n">
-        <v>11.5</v>
+        <v>1.9</v>
       </c>
       <c r="G28" t="n">
-        <v>12.1</v>
+        <v>3.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>24.48</v>
+        <v>26.08</v>
       </c>
       <c r="D29" t="n">
-        <v>2.28</v>
+        <v>2.39</v>
       </c>
       <c r="E29" t="n">
-        <v>11.5</v>
+        <v>7.5</v>
       </c>
       <c r="F29" t="n">
-        <v>11.5</v>
+        <v>1.9</v>
       </c>
       <c r="G29" t="n">
-        <v>11.5</v>
+        <v>3.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="30">
@@ -1326,52 +1326,52 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>24.52</v>
+        <v>24.23</v>
       </c>
       <c r="D30" t="n">
-        <v>2.02</v>
+        <v>1.98</v>
       </c>
       <c r="E30" t="n">
-        <v>9.6</v>
+        <v>3.8</v>
       </c>
       <c r="F30" t="n">
-        <v>9.6</v>
+        <v>1.9</v>
       </c>
       <c r="G30" t="n">
-        <v>9.6</v>
+        <v>2.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>15.8</v>
+        <v>19.42</v>
       </c>
       <c r="D31" t="n">
-        <v>2.35</v>
+        <v>3.36</v>
       </c>
       <c r="E31" t="n">
-        <v>15.4</v>
+        <v>1.9</v>
       </c>
       <c r="F31" t="n">
-        <v>4.8</v>
+        <v>1.9</v>
       </c>
       <c r="G31" t="n">
-        <v>8</v>
+        <v>1.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="32">
@@ -1386,10 +1386,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>13.49</v>
+        <v>13.27</v>
       </c>
       <c r="D32" t="n">
-        <v>1.27</v>
+        <v>1.25</v>
       </c>
       <c r="E32" t="n">
         <v>1.9</v>
@@ -1401,7 +1401,7 @@
         <v>1.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Jun 17 13:03:36 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>77.40000000000001</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>8.08</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,7 +501,7 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="3">
@@ -516,10 +516,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42.74</v>
+        <v>44.69</v>
       </c>
       <c r="D3" t="n">
-        <v>2.38</v>
+        <v>2.48</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -531,7 +531,7 @@
         <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="4">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>43.52</v>
+        <v>44.15</v>
       </c>
       <c r="D4" t="n">
-        <v>3.68</v>
+        <v>3.74</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
@@ -561,7 +561,7 @@
         <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="5">
@@ -576,22 +576,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>34.17</v>
+        <v>34.42</v>
       </c>
       <c r="D5" t="n">
-        <v>3.24</v>
+        <v>3.26</v>
       </c>
       <c r="E5" t="n">
-        <v>96.2</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>92.5</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>94.3</v>
+        <v>96.8</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="6">
@@ -606,22 +606,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.21</v>
+        <v>10.16</v>
       </c>
       <c r="D6" t="n">
-        <v>1.24</v>
+        <v>1.23</v>
       </c>
       <c r="E6" t="n">
-        <v>62.3</v>
+        <v>55.6</v>
       </c>
       <c r="F6" t="n">
-        <v>56.6</v>
+        <v>51.9</v>
       </c>
       <c r="G6" t="n">
-        <v>59.4</v>
+        <v>53.7</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="7">
@@ -636,22 +636,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>22.87</v>
+        <v>22.8</v>
       </c>
       <c r="D7" t="n">
-        <v>3.78</v>
+        <v>3.77</v>
       </c>
       <c r="E7" t="n">
-        <v>58.5</v>
+        <v>57.4</v>
       </c>
       <c r="F7" t="n">
-        <v>55.7</v>
+        <v>50</v>
       </c>
       <c r="G7" t="n">
-        <v>57.1</v>
+        <v>53.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="8">
@@ -666,22 +666,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.91</v>
+        <v>6.85</v>
       </c>
       <c r="D8" t="n">
         <v>0.65</v>
       </c>
       <c r="E8" t="n">
-        <v>62.3</v>
+        <v>49.1</v>
       </c>
       <c r="F8" t="n">
-        <v>46.2</v>
+        <v>46.3</v>
       </c>
       <c r="G8" t="n">
-        <v>54.2</v>
+        <v>47.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="9">
@@ -696,52 +696,52 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28.18</v>
+        <v>28.19</v>
       </c>
       <c r="D9" t="n">
         <v>2.58</v>
       </c>
       <c r="E9" t="n">
-        <v>47.2</v>
+        <v>48.1</v>
       </c>
       <c r="F9" t="n">
-        <v>42.5</v>
+        <v>42.6</v>
       </c>
       <c r="G9" t="n">
-        <v>44.8</v>
+        <v>45.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>20.22</v>
+        <v>120.14</v>
       </c>
       <c r="D10" t="n">
-        <v>1.89</v>
+        <v>4.5</v>
       </c>
       <c r="E10" t="n">
-        <v>47.2</v>
+        <v>40.7</v>
       </c>
       <c r="F10" t="n">
-        <v>39.6</v>
+        <v>39.8</v>
       </c>
       <c r="G10" t="n">
-        <v>43.4</v>
+        <v>40.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="11">
@@ -756,382 +756,382 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>61.07</v>
+        <v>61.72</v>
       </c>
       <c r="D11" t="n">
-        <v>3.92</v>
+        <v>3.97</v>
       </c>
       <c r="E11" t="n">
-        <v>35.8</v>
+        <v>37</v>
       </c>
       <c r="F11" t="n">
-        <v>25.5</v>
+        <v>37</v>
       </c>
       <c r="G11" t="n">
-        <v>28.6</v>
+        <v>37</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>35.56</v>
+        <v>11.14</v>
       </c>
       <c r="D12" t="n">
-        <v>3.84</v>
+        <v>0.71</v>
       </c>
       <c r="E12" t="n">
-        <v>28.3</v>
+        <v>29.6</v>
       </c>
       <c r="F12" t="n">
-        <v>24.5</v>
+        <v>28.7</v>
       </c>
       <c r="G12" t="n">
-        <v>25.7</v>
+        <v>29</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>113.92</v>
+        <v>35.48</v>
       </c>
       <c r="D13" t="n">
-        <v>4.28</v>
+        <v>3.83</v>
       </c>
       <c r="E13" t="n">
-        <v>22.6</v>
+        <v>25.9</v>
       </c>
       <c r="F13" t="n">
-        <v>22.6</v>
+        <v>24.1</v>
       </c>
       <c r="G13" t="n">
-        <v>22.6</v>
+        <v>24.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>22.29</v>
+        <v>20.07</v>
       </c>
       <c r="D14" t="n">
-        <v>1.64</v>
+        <v>1.87</v>
       </c>
       <c r="E14" t="n">
-        <v>23.6</v>
+        <v>36.1</v>
       </c>
       <c r="F14" t="n">
-        <v>20.8</v>
+        <v>19.4</v>
       </c>
       <c r="G14" t="n">
-        <v>21.6</v>
+        <v>24.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>31.8</v>
+        <v>22.17</v>
       </c>
       <c r="D15" t="n">
-        <v>2.42</v>
+        <v>1.63</v>
       </c>
       <c r="E15" t="n">
-        <v>25.5</v>
+        <v>20.4</v>
       </c>
       <c r="F15" t="n">
-        <v>19.8</v>
+        <v>17.6</v>
       </c>
       <c r="G15" t="n">
-        <v>21.5</v>
+        <v>18.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.89</v>
+        <v>47.7</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7</v>
+        <v>3.91</v>
       </c>
       <c r="E16" t="n">
-        <v>17</v>
+        <v>24.1</v>
       </c>
       <c r="F16" t="n">
-        <v>19.8</v>
+        <v>14.8</v>
       </c>
       <c r="G16" t="n">
-        <v>19</v>
+        <v>17.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23</v>
+        <v>31.44</v>
       </c>
       <c r="D17" t="n">
-        <v>1.89</v>
+        <v>2.39</v>
       </c>
       <c r="E17" t="n">
-        <v>17</v>
+        <v>16.7</v>
       </c>
       <c r="F17" t="n">
-        <v>15.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>15.7</v>
+        <v>11.5</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>47.47</v>
+        <v>11.03</v>
       </c>
       <c r="D18" t="n">
-        <v>3.89</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>17</v>
+        <v>1.9</v>
       </c>
       <c r="F18" t="n">
-        <v>13.2</v>
+        <v>13.9</v>
       </c>
       <c r="G18" t="n">
-        <v>14.3</v>
+        <v>10.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>11.16</v>
+        <v>14.65</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>1.19</v>
       </c>
       <c r="E19" t="n">
-        <v>7.5</v>
+        <v>10.2</v>
       </c>
       <c r="F19" t="n">
-        <v>13.2</v>
+        <v>5.6</v>
       </c>
       <c r="G19" t="n">
-        <v>11.5</v>
+        <v>6.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.36</v>
+        <v>15.54</v>
       </c>
       <c r="D20" t="n">
-        <v>0.96</v>
+        <v>2.3</v>
       </c>
       <c r="E20" t="n">
-        <v>11.3</v>
+        <v>13</v>
       </c>
       <c r="F20" t="n">
-        <v>7.5</v>
+        <v>1.9</v>
       </c>
       <c r="G20" t="n">
-        <v>8.699999999999999</v>
+        <v>5.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>19.69</v>
+        <v>26.93</v>
       </c>
       <c r="D21" t="n">
-        <v>1.64</v>
+        <v>1.99</v>
       </c>
       <c r="E21" t="n">
-        <v>24.5</v>
+        <v>11.1</v>
       </c>
       <c r="F21" t="n">
         <v>1.9</v>
       </c>
       <c r="G21" t="n">
-        <v>8.699999999999999</v>
+        <v>4.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>27.27</v>
+        <v>22.43</v>
       </c>
       <c r="D22" t="n">
-        <v>2.02</v>
+        <v>1.84</v>
       </c>
       <c r="E22" t="n">
-        <v>14.2</v>
+        <v>5.6</v>
       </c>
       <c r="F22" t="n">
-        <v>4.7</v>
+        <v>3.7</v>
       </c>
       <c r="G22" t="n">
-        <v>7.5</v>
+        <v>4.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>28.49</v>
+        <v>19.45</v>
       </c>
       <c r="D23" t="n">
-        <v>2.38</v>
+        <v>1.62</v>
       </c>
       <c r="E23" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>4.7</v>
+        <v>1.9</v>
       </c>
       <c r="G23" t="n">
-        <v>6.1</v>
+        <v>4.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="24">
@@ -1146,172 +1146,172 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>24.19</v>
+        <v>23.96</v>
       </c>
       <c r="D24" t="n">
-        <v>2.23</v>
+        <v>2.21</v>
       </c>
       <c r="E24" t="n">
-        <v>11.3</v>
+        <v>3.7</v>
       </c>
       <c r="F24" t="n">
-        <v>3.8</v>
+        <v>2.8</v>
       </c>
       <c r="G24" t="n">
-        <v>6</v>
+        <v>3.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>17.79</v>
+        <v>28.07</v>
       </c>
       <c r="D25" t="n">
-        <v>1.65</v>
+        <v>2.34</v>
       </c>
       <c r="E25" t="n">
-        <v>1.9</v>
+        <v>5.6</v>
       </c>
       <c r="F25" t="n">
-        <v>7.5</v>
+        <v>1.9</v>
       </c>
       <c r="G25" t="n">
-        <v>5.8</v>
+        <v>3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>15.63</v>
+        <v>22.66</v>
       </c>
       <c r="D26" t="n">
-        <v>2.31</v>
+        <v>2.05</v>
       </c>
       <c r="E26" t="n">
-        <v>13.2</v>
+        <v>3.7</v>
       </c>
       <c r="F26" t="n">
         <v>1.9</v>
       </c>
       <c r="G26" t="n">
-        <v>5.3</v>
+        <v>2.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>14.59</v>
+        <v>16.96</v>
       </c>
       <c r="D27" t="n">
-        <v>1.19</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E27" t="n">
-        <v>5.7</v>
+        <v>2.8</v>
       </c>
       <c r="F27" t="n">
-        <v>4.7</v>
+        <v>1.9</v>
       </c>
       <c r="G27" t="n">
-        <v>5</v>
+        <v>2.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22.87</v>
+        <v>25.93</v>
       </c>
       <c r="D28" t="n">
-        <v>2.07</v>
+        <v>2.38</v>
       </c>
       <c r="E28" t="n">
-        <v>7.5</v>
+        <v>1.9</v>
       </c>
       <c r="F28" t="n">
         <v>1.9</v>
       </c>
       <c r="G28" t="n">
-        <v>3.6</v>
+        <v>1.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26.08</v>
+        <v>19.2</v>
       </c>
       <c r="D29" t="n">
-        <v>2.39</v>
+        <v>3.32</v>
       </c>
       <c r="E29" t="n">
-        <v>7.5</v>
+        <v>1.9</v>
       </c>
       <c r="F29" t="n">
         <v>1.9</v>
       </c>
       <c r="G29" t="n">
-        <v>3.6</v>
+        <v>1.9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="30">
@@ -1326,40 +1326,40 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>24.23</v>
+        <v>23.85</v>
       </c>
       <c r="D30" t="n">
-        <v>1.98</v>
+        <v>1.95</v>
       </c>
       <c r="E30" t="n">
-        <v>3.8</v>
+        <v>1.9</v>
       </c>
       <c r="F30" t="n">
         <v>1.9</v>
       </c>
       <c r="G30" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>19.42</v>
+        <v>13.14</v>
       </c>
       <c r="D31" t="n">
-        <v>3.36</v>
+        <v>1.23</v>
       </c>
       <c r="E31" t="n">
         <v>1.9</v>
@@ -1371,25 +1371,25 @@
         <v>1.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>13.27</v>
+        <v>17.41</v>
       </c>
       <c r="D32" t="n">
-        <v>1.25</v>
+        <v>1.61</v>
       </c>
       <c r="E32" t="n">
         <v>1.9</v>
@@ -1401,7 +1401,7 @@
         <v>1.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Jun 18 12:40:44 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>80.90000000000001</v>
+        <v>83.83</v>
       </c>
       <c r="D2" t="n">
-        <v>8.449999999999999</v>
+        <v>8.76</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,25 +501,25 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>44.69</v>
+        <v>35.18</v>
       </c>
       <c r="D3" t="n">
-        <v>2.48</v>
+        <v>3.34</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -531,7 +531,7 @@
         <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="4">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>44.15</v>
+        <v>44.85</v>
       </c>
       <c r="D4" t="n">
-        <v>3.74</v>
+        <v>3.79</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
@@ -561,217 +561,217 @@
         <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>34.42</v>
+        <v>43.88</v>
       </c>
       <c r="D5" t="n">
-        <v>3.26</v>
+        <v>2.44</v>
       </c>
       <c r="E5" t="n">
-        <v>98.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="F5" t="n">
-        <v>95.40000000000001</v>
+        <v>98.2</v>
       </c>
       <c r="G5" t="n">
-        <v>96.8</v>
+        <v>98.2</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.16</v>
+        <v>22.87</v>
       </c>
       <c r="D6" t="n">
-        <v>1.23</v>
+        <v>3.78</v>
       </c>
       <c r="E6" t="n">
-        <v>55.6</v>
+        <v>59.1</v>
       </c>
       <c r="F6" t="n">
-        <v>51.9</v>
+        <v>56.4</v>
       </c>
       <c r="G6" t="n">
-        <v>53.7</v>
+        <v>57.7</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>22.8</v>
+        <v>120.55</v>
       </c>
       <c r="D7" t="n">
-        <v>3.77</v>
+        <v>4.52</v>
       </c>
       <c r="E7" t="n">
-        <v>57.4</v>
+        <v>41.8</v>
       </c>
       <c r="F7" t="n">
-        <v>50</v>
+        <v>41.8</v>
       </c>
       <c r="G7" t="n">
-        <v>53.7</v>
+        <v>41.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.85</v>
+        <v>27.89</v>
       </c>
       <c r="D8" t="n">
-        <v>0.65</v>
+        <v>2.55</v>
       </c>
       <c r="E8" t="n">
-        <v>49.1</v>
+        <v>38.2</v>
       </c>
       <c r="F8" t="n">
-        <v>46.3</v>
+        <v>34.5</v>
       </c>
       <c r="G8" t="n">
-        <v>47.7</v>
+        <v>36.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28.19</v>
+        <v>61.47</v>
       </c>
       <c r="D9" t="n">
-        <v>2.58</v>
+        <v>3.95</v>
       </c>
       <c r="E9" t="n">
-        <v>48.1</v>
+        <v>36.4</v>
       </c>
       <c r="F9" t="n">
-        <v>42.6</v>
+        <v>35.5</v>
       </c>
       <c r="G9" t="n">
-        <v>45.4</v>
+        <v>35.9</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>120.14</v>
+        <v>35.31</v>
       </c>
       <c r="D10" t="n">
-        <v>4.5</v>
+        <v>3.81</v>
       </c>
       <c r="E10" t="n">
-        <v>40.7</v>
+        <v>25.5</v>
       </c>
       <c r="F10" t="n">
-        <v>39.8</v>
+        <v>22.7</v>
       </c>
       <c r="G10" t="n">
-        <v>40.3</v>
+        <v>23.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>61.72</v>
+        <v>48.05</v>
       </c>
       <c r="D11" t="n">
-        <v>3.97</v>
+        <v>3.93</v>
       </c>
       <c r="E11" t="n">
-        <v>37</v>
+        <v>27.3</v>
       </c>
       <c r="F11" t="n">
-        <v>37</v>
+        <v>17.3</v>
       </c>
       <c r="G11" t="n">
-        <v>37</v>
+        <v>20.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="12">
@@ -786,502 +786,502 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>11.14</v>
+        <v>10.89</v>
       </c>
       <c r="D12" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="E12" t="n">
-        <v>29.6</v>
+        <v>17.3</v>
       </c>
       <c r="F12" t="n">
-        <v>28.7</v>
+        <v>20</v>
       </c>
       <c r="G12" t="n">
-        <v>29</v>
+        <v>19.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>35.48</v>
+        <v>9.74</v>
       </c>
       <c r="D13" t="n">
-        <v>3.83</v>
+        <v>1.18</v>
       </c>
       <c r="E13" t="n">
-        <v>25.9</v>
+        <v>14.5</v>
       </c>
       <c r="F13" t="n">
-        <v>24.1</v>
+        <v>13.6</v>
       </c>
       <c r="G13" t="n">
-        <v>24.6</v>
+        <v>13.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>20.07</v>
+        <v>22.1</v>
       </c>
       <c r="D14" t="n">
-        <v>1.87</v>
+        <v>1.62</v>
       </c>
       <c r="E14" t="n">
-        <v>36.1</v>
+        <v>14.5</v>
       </c>
       <c r="F14" t="n">
-        <v>19.4</v>
+        <v>11.8</v>
       </c>
       <c r="G14" t="n">
-        <v>24.4</v>
+        <v>12.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>22.17</v>
+        <v>31.39</v>
       </c>
       <c r="D15" t="n">
-        <v>1.63</v>
+        <v>2.39</v>
       </c>
       <c r="E15" t="n">
-        <v>20.4</v>
+        <v>16.4</v>
       </c>
       <c r="F15" t="n">
-        <v>17.6</v>
+        <v>10</v>
       </c>
       <c r="G15" t="n">
-        <v>18.4</v>
+        <v>11.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>47.7</v>
+        <v>10.87</v>
       </c>
       <c r="D16" t="n">
-        <v>3.91</v>
+        <v>0.98</v>
       </c>
       <c r="E16" t="n">
-        <v>24.1</v>
+        <v>1.8</v>
       </c>
       <c r="F16" t="n">
-        <v>14.8</v>
+        <v>10.9</v>
       </c>
       <c r="G16" t="n">
-        <v>17.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>31.44</v>
+        <v>26.23</v>
       </c>
       <c r="D17" t="n">
-        <v>2.39</v>
+        <v>2.41</v>
       </c>
       <c r="E17" t="n">
-        <v>16.7</v>
+        <v>12.7</v>
       </c>
       <c r="F17" t="n">
-        <v>9.300000000000001</v>
+        <v>5.5</v>
       </c>
       <c r="G17" t="n">
-        <v>11.5</v>
+        <v>7.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>11.03</v>
+        <v>24.05</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2.22</v>
       </c>
       <c r="E18" t="n">
-        <v>1.9</v>
+        <v>10.9</v>
       </c>
       <c r="F18" t="n">
-        <v>13.9</v>
+        <v>5.5</v>
       </c>
       <c r="G18" t="n">
-        <v>10.3</v>
+        <v>7.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>14.65</v>
+        <v>15.37</v>
       </c>
       <c r="D19" t="n">
-        <v>1.19</v>
+        <v>2.27</v>
       </c>
       <c r="E19" t="n">
-        <v>10.2</v>
+        <v>10.9</v>
       </c>
       <c r="F19" t="n">
-        <v>5.6</v>
+        <v>1.8</v>
       </c>
       <c r="G19" t="n">
-        <v>6.9</v>
+        <v>4.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>15.54</v>
+        <v>6.67</v>
       </c>
       <c r="D20" t="n">
-        <v>2.3</v>
+        <v>0.63</v>
       </c>
       <c r="E20" t="n">
-        <v>13</v>
+        <v>2.7</v>
       </c>
       <c r="F20" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="G20" t="n">
-        <v>5.2</v>
+        <v>2.7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>26.93</v>
+        <v>23.84</v>
       </c>
       <c r="D21" t="n">
-        <v>1.99</v>
+        <v>1.95</v>
       </c>
       <c r="E21" t="n">
-        <v>11.1</v>
+        <v>1.8</v>
       </c>
       <c r="F21" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="G21" t="n">
-        <v>4.6</v>
+        <v>2.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22.43</v>
+        <v>27.93</v>
       </c>
       <c r="D22" t="n">
-        <v>1.84</v>
+        <v>2.33</v>
       </c>
       <c r="E22" t="n">
-        <v>5.6</v>
+        <v>3.6</v>
       </c>
       <c r="F22" t="n">
-        <v>3.7</v>
+        <v>1.8</v>
       </c>
       <c r="G22" t="n">
-        <v>4.3</v>
+        <v>2.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>19.45</v>
+        <v>26.49</v>
       </c>
       <c r="D23" t="n">
-        <v>1.62</v>
+        <v>1.96</v>
       </c>
       <c r="E23" t="n">
-        <v>9.300000000000001</v>
+        <v>3.6</v>
       </c>
       <c r="F23" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G23" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>23.96</v>
+        <v>19.27</v>
       </c>
       <c r="D24" t="n">
-        <v>2.21</v>
+        <v>1.61</v>
       </c>
       <c r="E24" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="F24" t="n">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="G24" t="n">
-        <v>3.1</v>
+        <v>2.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.07</v>
+        <v>22.01</v>
       </c>
       <c r="D25" t="n">
-        <v>2.34</v>
+        <v>1.8</v>
       </c>
       <c r="E25" t="n">
-        <v>5.6</v>
+        <v>1.8</v>
       </c>
       <c r="F25" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G25" t="n">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>22.66</v>
+        <v>14.37</v>
       </c>
       <c r="D26" t="n">
-        <v>2.05</v>
+        <v>1.17</v>
       </c>
       <c r="E26" t="n">
-        <v>3.7</v>
+        <v>1.8</v>
       </c>
       <c r="F26" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G26" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>16.96</v>
+        <v>19.36</v>
       </c>
       <c r="D27" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.8</v>
       </c>
       <c r="E27" t="n">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="F27" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G27" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25.93</v>
+        <v>22.49</v>
       </c>
       <c r="D28" t="n">
-        <v>2.38</v>
+        <v>2.03</v>
       </c>
       <c r="E28" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="F28" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G28" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="29">
@@ -1296,52 +1296,52 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>19.2</v>
+        <v>18.8</v>
       </c>
       <c r="D29" t="n">
-        <v>3.32</v>
+        <v>3.25</v>
       </c>
       <c r="E29" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="F29" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G29" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>23.85</v>
+        <v>16.77</v>
       </c>
       <c r="D30" t="n">
-        <v>1.95</v>
+        <v>0.93</v>
       </c>
       <c r="E30" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="F30" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G30" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>13.14</v>
+        <v>12.83</v>
       </c>
       <c r="D31" t="n">
-        <v>1.23</v>
+        <v>1.21</v>
       </c>
       <c r="E31" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="F31" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G31" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>17.41</v>
+        <v>17.02</v>
       </c>
       <c r="D32" t="n">
-        <v>1.61</v>
+        <v>1.58</v>
       </c>
       <c r="E32" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="F32" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G32" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Jun 19 13:01:48 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>8.76</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.34</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.79</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.44</v>
       </c>
       <c r="E5" t="n">
-        <v>98.2</v>
+        <v>97.3</v>
       </c>
       <c r="F5" t="n">
-        <v>98.2</v>
+        <v>97.3</v>
       </c>
       <c r="G5" t="n">
-        <v>98.2</v>
+        <v>97.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>3.78</v>
       </c>
       <c r="E6" t="n">
-        <v>59.1</v>
+        <v>58.9</v>
       </c>
       <c r="F6" t="n">
-        <v>56.4</v>
+        <v>56.2</v>
       </c>
       <c r="G6" t="n">
-        <v>57.7</v>
+        <v>57.6</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>4.52</v>
       </c>
       <c r="E7" t="n">
-        <v>41.8</v>
+        <v>42</v>
       </c>
       <c r="F7" t="n">
-        <v>41.8</v>
+        <v>42</v>
       </c>
       <c r="G7" t="n">
-        <v>41.8</v>
+        <v>42</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.55</v>
       </c>
       <c r="E8" t="n">
-        <v>38.2</v>
+        <v>38.4</v>
       </c>
       <c r="F8" t="n">
-        <v>34.5</v>
+        <v>34.8</v>
       </c>
       <c r="G8" t="n">
-        <v>36.4</v>
+        <v>36.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>3.95</v>
       </c>
       <c r="E9" t="n">
-        <v>36.4</v>
+        <v>36.6</v>
       </c>
       <c r="F9" t="n">
-        <v>35.5</v>
+        <v>35.7</v>
       </c>
       <c r="G9" t="n">
-        <v>35.9</v>
+        <v>36.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>3.81</v>
       </c>
       <c r="E10" t="n">
-        <v>25.5</v>
+        <v>25.9</v>
       </c>
       <c r="F10" t="n">
-        <v>22.7</v>
+        <v>23.2</v>
       </c>
       <c r="G10" t="n">
-        <v>23.5</v>
+        <v>24</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>3.93</v>
       </c>
       <c r="E11" t="n">
-        <v>27.3</v>
+        <v>27.7</v>
       </c>
       <c r="F11" t="n">
-        <v>17.3</v>
+        <v>17.9</v>
       </c>
       <c r="G11" t="n">
-        <v>20.3</v>
+        <v>20.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>0.7</v>
       </c>
       <c r="E12" t="n">
-        <v>17.3</v>
+        <v>17.9</v>
       </c>
       <c r="F12" t="n">
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="G12" t="n">
-        <v>19.2</v>
+        <v>19.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.18</v>
       </c>
       <c r="E13" t="n">
-        <v>14.5</v>
+        <v>15.2</v>
       </c>
       <c r="F13" t="n">
-        <v>13.6</v>
+        <v>14.3</v>
       </c>
       <c r="G13" t="n">
-        <v>13.9</v>
+        <v>14.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.62</v>
       </c>
       <c r="E14" t="n">
-        <v>14.5</v>
+        <v>15.2</v>
       </c>
       <c r="F14" t="n">
-        <v>11.8</v>
+        <v>12.5</v>
       </c>
       <c r="G14" t="n">
-        <v>12.6</v>
+        <v>13.3</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.39</v>
       </c>
       <c r="E15" t="n">
-        <v>16.4</v>
+        <v>17</v>
       </c>
       <c r="F15" t="n">
-        <v>10</v>
+        <v>10.7</v>
       </c>
       <c r="G15" t="n">
-        <v>11.9</v>
+        <v>12.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>0.98</v>
       </c>
       <c r="E16" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F16" t="n">
-        <v>10.9</v>
+        <v>11.6</v>
       </c>
       <c r="G16" t="n">
-        <v>8.199999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.41</v>
       </c>
       <c r="E17" t="n">
-        <v>12.7</v>
+        <v>13.4</v>
       </c>
       <c r="F17" t="n">
-        <v>5.5</v>
+        <v>6.2</v>
       </c>
       <c r="G17" t="n">
-        <v>7.6</v>
+        <v>8.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.22</v>
       </c>
       <c r="E18" t="n">
-        <v>10.9</v>
+        <v>11.6</v>
       </c>
       <c r="F18" t="n">
-        <v>5.5</v>
+        <v>6.2</v>
       </c>
       <c r="G18" t="n">
-        <v>7.1</v>
+        <v>7.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.27</v>
       </c>
       <c r="E19" t="n">
-        <v>10.9</v>
+        <v>11.6</v>
       </c>
       <c r="F19" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G19" t="n">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.63</v>
       </c>
       <c r="E20" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="F20" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="G20" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.95</v>
       </c>
       <c r="E21" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F21" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="G21" t="n">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.33</v>
       </c>
       <c r="E22" t="n">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="F22" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G22" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.96</v>
       </c>
       <c r="E23" t="n">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="F23" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G23" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.61</v>
       </c>
       <c r="E24" t="n">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="F24" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G24" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.8</v>
       </c>
       <c r="E25" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F25" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G25" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>1.17</v>
       </c>
       <c r="E26" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F26" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G26" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>1.8</v>
       </c>
       <c r="E27" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F27" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G27" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.03</v>
       </c>
       <c r="E28" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F28" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G28" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.25</v>
       </c>
       <c r="E29" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F29" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G29" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>0.93</v>
       </c>
       <c r="E30" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F30" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G30" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.21</v>
       </c>
       <c r="E31" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F31" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G31" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.58</v>
       </c>
       <c r="E32" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="F32" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="G32" t="n">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Jun 20 11:34:51 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>8.76</v>
       </c>
       <c r="E2" t="n">
-        <v>99.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="F2" t="n">
-        <v>99.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="G2" t="n">
-        <v>99.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.34</v>
       </c>
       <c r="E3" t="n">
-        <v>99.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="F3" t="n">
-        <v>99.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="G3" t="n">
-        <v>99.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.79</v>
       </c>
       <c r="E4" t="n">
-        <v>99.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="F4" t="n">
-        <v>99.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="G4" t="n">
-        <v>99.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.44</v>
       </c>
       <c r="E5" t="n">
-        <v>97.3</v>
+        <v>96.5</v>
       </c>
       <c r="F5" t="n">
-        <v>97.3</v>
+        <v>96.5</v>
       </c>
       <c r="G5" t="n">
-        <v>97.3</v>
+        <v>96.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>3.78</v>
       </c>
       <c r="E6" t="n">
-        <v>58.9</v>
+        <v>58.8</v>
       </c>
       <c r="F6" t="n">
-        <v>56.2</v>
+        <v>56.1</v>
       </c>
       <c r="G6" t="n">
-        <v>57.6</v>
+        <v>57.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>4.52</v>
       </c>
       <c r="E7" t="n">
-        <v>42</v>
+        <v>42.1</v>
       </c>
       <c r="F7" t="n">
-        <v>42</v>
+        <v>42.1</v>
       </c>
       <c r="G7" t="n">
-        <v>42</v>
+        <v>42.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.55</v>
       </c>
       <c r="E8" t="n">
-        <v>38.4</v>
+        <v>38.6</v>
       </c>
       <c r="F8" t="n">
-        <v>34.8</v>
+        <v>35.1</v>
       </c>
       <c r="G8" t="n">
-        <v>36.6</v>
+        <v>36.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>3.95</v>
       </c>
       <c r="E9" t="n">
-        <v>36.6</v>
+        <v>36.8</v>
       </c>
       <c r="F9" t="n">
-        <v>35.7</v>
+        <v>36</v>
       </c>
       <c r="G9" t="n">
-        <v>36.2</v>
+        <v>36.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>3.81</v>
       </c>
       <c r="E10" t="n">
-        <v>25.9</v>
+        <v>26.3</v>
       </c>
       <c r="F10" t="n">
-        <v>23.2</v>
+        <v>23.7</v>
       </c>
       <c r="G10" t="n">
-        <v>24</v>
+        <v>24.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>3.93</v>
       </c>
       <c r="E11" t="n">
-        <v>27.7</v>
+        <v>28.1</v>
       </c>
       <c r="F11" t="n">
-        <v>17.9</v>
+        <v>18.4</v>
       </c>
       <c r="G11" t="n">
-        <v>20.8</v>
+        <v>21.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>0.7</v>
       </c>
       <c r="E12" t="n">
-        <v>17.9</v>
+        <v>18.4</v>
       </c>
       <c r="F12" t="n">
-        <v>20.5</v>
+        <v>21.1</v>
       </c>
       <c r="G12" t="n">
-        <v>19.7</v>
+        <v>20.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.18</v>
       </c>
       <c r="E13" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="F13" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="G13" t="n">
         <v>15.2</v>
       </c>
-      <c r="F13" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="G13" t="n">
-        <v>14.6</v>
-      </c>
       <c r="H13" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.62</v>
       </c>
       <c r="E14" t="n">
-        <v>15.2</v>
+        <v>15.8</v>
       </c>
       <c r="F14" t="n">
-        <v>12.5</v>
+        <v>13.2</v>
       </c>
       <c r="G14" t="n">
-        <v>13.3</v>
+        <v>13.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.39</v>
       </c>
       <c r="E15" t="n">
-        <v>17</v>
+        <v>17.5</v>
       </c>
       <c r="F15" t="n">
-        <v>10.7</v>
+        <v>11.4</v>
       </c>
       <c r="G15" t="n">
-        <v>12.6</v>
+        <v>13.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>0.98</v>
       </c>
       <c r="E16" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F16" t="n">
-        <v>11.6</v>
+        <v>12.3</v>
       </c>
       <c r="G16" t="n">
-        <v>8.9</v>
+        <v>9.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.41</v>
       </c>
       <c r="E17" t="n">
-        <v>13.4</v>
+        <v>14</v>
       </c>
       <c r="F17" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="G17" t="n">
-        <v>8.4</v>
+        <v>9.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.22</v>
       </c>
       <c r="E18" t="n">
-        <v>11.6</v>
+        <v>12.3</v>
       </c>
       <c r="F18" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="G18" t="n">
-        <v>7.9</v>
+        <v>8.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.27</v>
       </c>
       <c r="E19" t="n">
-        <v>11.6</v>
+        <v>12.3</v>
       </c>
       <c r="F19" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G19" t="n">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.63</v>
       </c>
       <c r="E20" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="F20" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="G20" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.95</v>
       </c>
       <c r="E21" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F21" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="G21" t="n">
-        <v>3.3</v>
+        <v>4.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.33</v>
       </c>
       <c r="E22" t="n">
-        <v>4.5</v>
+        <v>5.3</v>
       </c>
       <c r="F22" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G22" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.96</v>
       </c>
       <c r="E23" t="n">
-        <v>4.5</v>
+        <v>5.3</v>
       </c>
       <c r="F23" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G23" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.61</v>
       </c>
       <c r="E24" t="n">
-        <v>4.5</v>
+        <v>5.3</v>
       </c>
       <c r="F24" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G24" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.8</v>
       </c>
       <c r="E25" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F25" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G25" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>1.17</v>
       </c>
       <c r="E26" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F26" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G26" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>1.8</v>
       </c>
       <c r="E27" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F27" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G27" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.03</v>
       </c>
       <c r="E28" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F28" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G28" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.25</v>
       </c>
       <c r="E29" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F29" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G29" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>0.93</v>
       </c>
       <c r="E30" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F30" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G30" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.21</v>
       </c>
       <c r="E31" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F31" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G31" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.58</v>
       </c>
       <c r="E32" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F32" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="G32" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Jun 21 12:02:04 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>8.76</v>
       </c>
       <c r="E2" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.34</v>
       </c>
       <c r="E3" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.79</v>
       </c>
       <c r="E4" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.44</v>
       </c>
       <c r="E5" t="n">
-        <v>96.5</v>
+        <v>95.7</v>
       </c>
       <c r="F5" t="n">
-        <v>96.5</v>
+        <v>95.7</v>
       </c>
       <c r="G5" t="n">
-        <v>96.5</v>
+        <v>95.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>3.78</v>
       </c>
       <c r="E6" t="n">
-        <v>58.8</v>
+        <v>58.6</v>
       </c>
       <c r="F6" t="n">
-        <v>56.1</v>
+        <v>56</v>
       </c>
       <c r="G6" t="n">
-        <v>57.5</v>
+        <v>57.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>4.52</v>
       </c>
       <c r="E7" t="n">
-        <v>42.1</v>
+        <v>42.2</v>
       </c>
       <c r="F7" t="n">
-        <v>42.1</v>
+        <v>42.2</v>
       </c>
       <c r="G7" t="n">
-        <v>42.1</v>
+        <v>42.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.55</v>
       </c>
       <c r="E8" t="n">
-        <v>38.6</v>
+        <v>38.8</v>
       </c>
       <c r="F8" t="n">
-        <v>35.1</v>
+        <v>35.3</v>
       </c>
       <c r="G8" t="n">
-        <v>36.8</v>
+        <v>37.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>3.95</v>
       </c>
       <c r="E9" t="n">
-        <v>36.8</v>
+        <v>37.1</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>36.2</v>
       </c>
       <c r="G9" t="n">
-        <v>36.4</v>
+        <v>36.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>3.81</v>
       </c>
       <c r="E10" t="n">
-        <v>26.3</v>
+        <v>26.7</v>
       </c>
       <c r="F10" t="n">
-        <v>23.7</v>
+        <v>24.1</v>
       </c>
       <c r="G10" t="n">
-        <v>24.5</v>
+        <v>24.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>3.93</v>
       </c>
       <c r="E11" t="n">
-        <v>28.1</v>
+        <v>28.4</v>
       </c>
       <c r="F11" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="G11" t="n">
-        <v>21.3</v>
+        <v>21.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>0.7</v>
       </c>
       <c r="E12" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="F12" t="n">
-        <v>21.1</v>
+        <v>21.6</v>
       </c>
       <c r="G12" t="n">
-        <v>20.3</v>
+        <v>20.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.18</v>
       </c>
       <c r="E13" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="F13" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G13" t="n">
         <v>15.8</v>
       </c>
-      <c r="F13" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="G13" t="n">
-        <v>15.2</v>
-      </c>
       <c r="H13" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.62</v>
       </c>
       <c r="E14" t="n">
-        <v>15.8</v>
+        <v>16.4</v>
       </c>
       <c r="F14" t="n">
-        <v>13.2</v>
+        <v>13.8</v>
       </c>
       <c r="G14" t="n">
-        <v>13.9</v>
+        <v>14.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.39</v>
       </c>
       <c r="E15" t="n">
-        <v>17.5</v>
+        <v>18.1</v>
       </c>
       <c r="F15" t="n">
-        <v>11.4</v>
+        <v>12.1</v>
       </c>
       <c r="G15" t="n">
-        <v>13.2</v>
+        <v>13.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>0.98</v>
       </c>
       <c r="E16" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F16" t="n">
-        <v>12.3</v>
+        <v>12.9</v>
       </c>
       <c r="G16" t="n">
-        <v>9.6</v>
+        <v>10.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.41</v>
       </c>
       <c r="E17" t="n">
-        <v>14</v>
+        <v>14.7</v>
       </c>
       <c r="F17" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="G17" t="n">
-        <v>9.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.22</v>
       </c>
       <c r="E18" t="n">
-        <v>12.3</v>
+        <v>12.9</v>
       </c>
       <c r="F18" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="G18" t="n">
-        <v>8.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.27</v>
       </c>
       <c r="E19" t="n">
-        <v>12.3</v>
+        <v>12.9</v>
       </c>
       <c r="F19" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G19" t="n">
-        <v>6.1</v>
+        <v>6.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>0.63</v>
       </c>
       <c r="E20" t="n">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="F20" t="n">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="G20" t="n">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.95</v>
       </c>
       <c r="E21" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F21" t="n">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="G21" t="n">
-        <v>4.1</v>
+        <v>4.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>2.33</v>
       </c>
       <c r="E22" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.96</v>
       </c>
       <c r="E23" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G23" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.61</v>
       </c>
       <c r="E24" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
       <c r="F24" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G24" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.8</v>
       </c>
       <c r="E25" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F25" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G25" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>1.17</v>
       </c>
       <c r="E26" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F26" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G26" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>1.8</v>
       </c>
       <c r="E27" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F27" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G27" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.03</v>
       </c>
       <c r="E28" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F28" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G28" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.25</v>
       </c>
       <c r="E29" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F29" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G29" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>0.93</v>
       </c>
       <c r="E30" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F30" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G30" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.21</v>
       </c>
       <c r="E31" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F31" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G31" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.58</v>
       </c>
       <c r="E32" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F32" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="G32" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Jun 22 15:09:44 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,52 +486,52 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>83.83</v>
+        <v>85.18000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>8.76</v>
+        <v>8.9</v>
       </c>
       <c r="E2" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>35.18</v>
+        <v>45.32</v>
       </c>
       <c r="D3" t="n">
-        <v>3.34</v>
+        <v>2.52</v>
       </c>
       <c r="E3" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="4">
@@ -546,52 +546,52 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>44.85</v>
+        <v>45</v>
       </c>
       <c r="D4" t="n">
-        <v>3.79</v>
+        <v>3.81</v>
       </c>
       <c r="E4" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>97.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>43.88</v>
+        <v>35.77</v>
       </c>
       <c r="D5" t="n">
-        <v>2.44</v>
+        <v>3.39</v>
       </c>
       <c r="E5" t="n">
-        <v>95.7</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>95.7</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>95.7</v>
+        <v>100</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="6">
@@ -606,142 +606,142 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22.87</v>
+        <v>23.95</v>
       </c>
       <c r="D6" t="n">
-        <v>3.78</v>
+        <v>3.96</v>
       </c>
       <c r="E6" t="n">
-        <v>58.6</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>56</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>57.3</v>
+        <v>87.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>120.55</v>
+        <v>29.04</v>
       </c>
       <c r="D7" t="n">
-        <v>4.52</v>
+        <v>2.66</v>
       </c>
       <c r="E7" t="n">
-        <v>42.2</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>42.2</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>42.2</v>
+        <v>73.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>27.89</v>
+        <v>10.39</v>
       </c>
       <c r="D8" t="n">
-        <v>2.55</v>
+        <v>1.26</v>
       </c>
       <c r="E8" t="n">
-        <v>38.8</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>35.3</v>
+        <v>63.6</v>
       </c>
       <c r="G8" t="n">
-        <v>37.1</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>61.47</v>
+        <v>36.47</v>
       </c>
       <c r="D9" t="n">
-        <v>3.95</v>
+        <v>3.94</v>
       </c>
       <c r="E9" t="n">
-        <v>37.1</v>
+        <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>36.2</v>
+        <v>43.2</v>
       </c>
       <c r="G9" t="n">
-        <v>36.6</v>
+        <v>46.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>35.31</v>
+        <v>61.55</v>
       </c>
       <c r="D10" t="n">
-        <v>3.81</v>
+        <v>3.96</v>
       </c>
       <c r="E10" t="n">
-        <v>26.7</v>
+        <v>40.7</v>
       </c>
       <c r="F10" t="n">
-        <v>24.1</v>
+        <v>40.7</v>
       </c>
       <c r="G10" t="n">
-        <v>24.9</v>
+        <v>40.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="11">
@@ -756,172 +756,172 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>48.05</v>
+        <v>49.09</v>
       </c>
       <c r="D11" t="n">
-        <v>3.93</v>
+        <v>4.02</v>
       </c>
       <c r="E11" t="n">
-        <v>28.4</v>
+        <v>40.7</v>
       </c>
       <c r="F11" t="n">
-        <v>19</v>
+        <v>32.2</v>
       </c>
       <c r="G11" t="n">
-        <v>21.8</v>
+        <v>36.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10.89</v>
+        <v>119.35</v>
       </c>
       <c r="D12" t="n">
-        <v>0.7</v>
+        <v>4.48</v>
       </c>
       <c r="E12" t="n">
-        <v>19</v>
+        <v>35.6</v>
       </c>
       <c r="F12" t="n">
-        <v>21.6</v>
+        <v>34.7</v>
       </c>
       <c r="G12" t="n">
-        <v>20.8</v>
+        <v>35.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9.74</v>
+        <v>22.39</v>
       </c>
       <c r="D13" t="n">
-        <v>1.18</v>
+        <v>1.64</v>
       </c>
       <c r="E13" t="n">
-        <v>16.4</v>
+        <v>32.2</v>
       </c>
       <c r="F13" t="n">
-        <v>15.5</v>
+        <v>28</v>
       </c>
       <c r="G13" t="n">
-        <v>15.8</v>
+        <v>29.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>22.1</v>
+        <v>31.73</v>
       </c>
       <c r="D14" t="n">
-        <v>1.62</v>
+        <v>2.41</v>
       </c>
       <c r="E14" t="n">
-        <v>16.4</v>
+        <v>30.5</v>
       </c>
       <c r="F14" t="n">
-        <v>13.8</v>
+        <v>23.7</v>
       </c>
       <c r="G14" t="n">
-        <v>14.6</v>
+        <v>25.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>31.39</v>
+        <v>10.98</v>
       </c>
       <c r="D15" t="n">
-        <v>2.39</v>
+        <v>0.7</v>
       </c>
       <c r="E15" t="n">
-        <v>18.1</v>
+        <v>26.3</v>
       </c>
       <c r="F15" t="n">
-        <v>12.1</v>
+        <v>22</v>
       </c>
       <c r="G15" t="n">
-        <v>13.9</v>
+        <v>23.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.87</v>
+        <v>6.73</v>
       </c>
       <c r="D16" t="n">
-        <v>0.98</v>
+        <v>0.64</v>
       </c>
       <c r="E16" t="n">
-        <v>4.3</v>
+        <v>11.9</v>
       </c>
       <c r="F16" t="n">
-        <v>12.9</v>
+        <v>22.9</v>
       </c>
       <c r="G16" t="n">
-        <v>10.3</v>
+        <v>19.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="17">
@@ -936,292 +936,292 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>26.23</v>
+        <v>26.42</v>
       </c>
       <c r="D17" t="n">
-        <v>2.41</v>
+        <v>2.43</v>
       </c>
       <c r="E17" t="n">
-        <v>14.7</v>
+        <v>18.6</v>
       </c>
       <c r="F17" t="n">
-        <v>7.8</v>
+        <v>16.1</v>
       </c>
       <c r="G17" t="n">
-        <v>9.800000000000001</v>
+        <v>16.9</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>24.05</v>
+        <v>24.39</v>
       </c>
       <c r="D18" t="n">
-        <v>2.22</v>
+        <v>1.99</v>
       </c>
       <c r="E18" t="n">
-        <v>12.9</v>
+        <v>18.6</v>
       </c>
       <c r="F18" t="n">
-        <v>7.8</v>
+        <v>12.7</v>
       </c>
       <c r="G18" t="n">
-        <v>9.300000000000001</v>
+        <v>14.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15.37</v>
+        <v>14.53</v>
       </c>
       <c r="D19" t="n">
-        <v>2.27</v>
+        <v>1.19</v>
       </c>
       <c r="E19" t="n">
-        <v>12.9</v>
+        <v>10.2</v>
       </c>
       <c r="F19" t="n">
-        <v>4.3</v>
+        <v>12.7</v>
       </c>
       <c r="G19" t="n">
-        <v>6.9</v>
+        <v>11.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6.67</v>
+        <v>15.38</v>
       </c>
       <c r="D20" t="n">
-        <v>0.63</v>
+        <v>2.28</v>
       </c>
       <c r="E20" t="n">
-        <v>5.2</v>
+        <v>16.9</v>
       </c>
       <c r="F20" t="n">
-        <v>5.2</v>
+        <v>8.5</v>
       </c>
       <c r="G20" t="n">
-        <v>5.2</v>
+        <v>11</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>23.84</v>
+        <v>19.37</v>
       </c>
       <c r="D21" t="n">
-        <v>1.95</v>
+        <v>1.62</v>
       </c>
       <c r="E21" t="n">
-        <v>4.3</v>
+        <v>13.6</v>
       </c>
       <c r="F21" t="n">
-        <v>5.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>4.9</v>
+        <v>10.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>27.93</v>
+        <v>17.01</v>
       </c>
       <c r="D22" t="n">
-        <v>2.33</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>11.9</v>
       </c>
       <c r="F22" t="n">
-        <v>4.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>4.8</v>
+        <v>10.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>26.49</v>
+        <v>10.84</v>
       </c>
       <c r="D23" t="n">
-        <v>1.96</v>
+        <v>0.98</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>1.7</v>
       </c>
       <c r="F23" t="n">
-        <v>4.3</v>
+        <v>13.6</v>
       </c>
       <c r="G23" t="n">
-        <v>4.8</v>
+        <v>10</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>19.27</v>
+        <v>22.25</v>
       </c>
       <c r="D24" t="n">
-        <v>1.61</v>
+        <v>1.83</v>
       </c>
       <c r="E24" t="n">
-        <v>6</v>
+        <v>10.2</v>
       </c>
       <c r="F24" t="n">
-        <v>4.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G24" t="n">
-        <v>4.8</v>
+        <v>9.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>22.01</v>
+        <v>19.08</v>
       </c>
       <c r="D25" t="n">
-        <v>1.8</v>
+        <v>3.3</v>
       </c>
       <c r="E25" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="F25" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="G25" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>14.37</v>
+        <v>17.28</v>
       </c>
       <c r="D26" t="n">
-        <v>1.17</v>
+        <v>1.6</v>
       </c>
       <c r="E26" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="F26" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="G26" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="27">
@@ -1236,22 +1236,22 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>19.36</v>
+        <v>19.47</v>
       </c>
       <c r="D27" t="n">
-        <v>1.8</v>
+        <v>1.82</v>
       </c>
       <c r="E27" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="F27" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="G27" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="28">
@@ -1266,142 +1266,142 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22.49</v>
+        <v>22.57</v>
       </c>
       <c r="D28" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
       <c r="E28" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="F28" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="G28" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.8</v>
+        <v>12.98</v>
       </c>
       <c r="D29" t="n">
-        <v>3.25</v>
+        <v>1.22</v>
       </c>
       <c r="E29" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="F29" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="G29" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>16.77</v>
+        <v>26.54</v>
       </c>
       <c r="D30" t="n">
-        <v>0.93</v>
+        <v>1.96</v>
       </c>
       <c r="E30" t="n">
-        <v>4.3</v>
+        <v>10.2</v>
       </c>
       <c r="F30" t="n">
-        <v>4.3</v>
+        <v>5.1</v>
       </c>
       <c r="G30" t="n">
-        <v>4.3</v>
+        <v>6.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>12.83</v>
+        <v>23.84</v>
       </c>
       <c r="D31" t="n">
-        <v>1.21</v>
+        <v>2.2</v>
       </c>
       <c r="E31" t="n">
-        <v>4.3</v>
+        <v>3.4</v>
       </c>
       <c r="F31" t="n">
-        <v>4.3</v>
+        <v>1.7</v>
       </c>
       <c r="G31" t="n">
-        <v>4.3</v>
+        <v>2.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>17.02</v>
+        <v>27.59</v>
       </c>
       <c r="D32" t="n">
-        <v>1.58</v>
+        <v>2.31</v>
       </c>
       <c r="E32" t="n">
-        <v>4.3</v>
+        <v>1.7</v>
       </c>
       <c r="F32" t="n">
-        <v>4.3</v>
+        <v>1.7</v>
       </c>
       <c r="G32" t="n">
-        <v>4.3</v>
+        <v>1.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Jun 23 12:25:19 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,52 +486,52 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>85.18000000000001</v>
+        <v>82.97</v>
       </c>
       <c r="D2" t="n">
-        <v>8.9</v>
+        <v>8.67</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>91.7</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>91.7</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>91.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>45.32</v>
+        <v>34.95</v>
       </c>
       <c r="D3" t="n">
-        <v>2.52</v>
+        <v>3.31</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>91.7</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>91.7</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>91.7</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="4">
@@ -546,82 +546,82 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>45</v>
+        <v>43.98</v>
       </c>
       <c r="D4" t="n">
-        <v>3.81</v>
+        <v>3.72</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>35.77</v>
+        <v>43.56</v>
       </c>
       <c r="D5" t="n">
-        <v>3.39</v>
+        <v>2.42</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>23.95</v>
+        <v>10.34</v>
       </c>
       <c r="D6" t="n">
-        <v>3.96</v>
+        <v>1.25</v>
       </c>
       <c r="E6" t="n">
-        <v>88.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="F6" t="n">
-        <v>86.40000000000001</v>
+        <v>60.8</v>
       </c>
       <c r="G6" t="n">
-        <v>87.3</v>
+        <v>66.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="7">
@@ -636,760 +636,760 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>29.04</v>
+        <v>28.52</v>
       </c>
       <c r="D7" t="n">
-        <v>2.66</v>
+        <v>2.61</v>
       </c>
       <c r="E7" t="n">
-        <v>74.59999999999999</v>
+        <v>56.7</v>
       </c>
       <c r="F7" t="n">
-        <v>72.90000000000001</v>
+        <v>54.2</v>
       </c>
       <c r="G7" t="n">
-        <v>73.7</v>
+        <v>55.4</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10.39</v>
+        <v>6.86</v>
       </c>
       <c r="D8" t="n">
-        <v>1.26</v>
+        <v>0.65</v>
       </c>
       <c r="E8" t="n">
-        <v>74.59999999999999</v>
+        <v>60</v>
       </c>
       <c r="F8" t="n">
-        <v>63.6</v>
+        <v>50.8</v>
       </c>
       <c r="G8" t="n">
-        <v>69.09999999999999</v>
+        <v>55.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>36.47</v>
+        <v>117.24</v>
       </c>
       <c r="D9" t="n">
-        <v>3.94</v>
+        <v>4.4</v>
       </c>
       <c r="E9" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="F9" t="n">
-        <v>43.2</v>
+        <v>31.7</v>
       </c>
       <c r="G9" t="n">
-        <v>46.6</v>
+        <v>32.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>61.55</v>
+        <v>22.19</v>
       </c>
       <c r="D10" t="n">
-        <v>3.96</v>
+        <v>1.63</v>
       </c>
       <c r="E10" t="n">
-        <v>40.7</v>
+        <v>26.7</v>
       </c>
       <c r="F10" t="n">
-        <v>40.7</v>
+        <v>23.3</v>
       </c>
       <c r="G10" t="n">
-        <v>40.7</v>
+        <v>24.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>49.09</v>
+        <v>22.19</v>
       </c>
       <c r="D11" t="n">
-        <v>4.02</v>
+        <v>3.67</v>
       </c>
       <c r="E11" t="n">
-        <v>40.7</v>
+        <v>41.7</v>
       </c>
       <c r="F11" t="n">
-        <v>32.2</v>
+        <v>16.7</v>
       </c>
       <c r="G11" t="n">
-        <v>36.4</v>
+        <v>24.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>119.35</v>
+        <v>26.69</v>
       </c>
       <c r="D12" t="n">
-        <v>4.48</v>
+        <v>2.45</v>
       </c>
       <c r="E12" t="n">
-        <v>35.6</v>
+        <v>33.3</v>
       </c>
       <c r="F12" t="n">
-        <v>34.7</v>
+        <v>20</v>
       </c>
       <c r="G12" t="n">
-        <v>35.2</v>
+        <v>24</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>22.39</v>
+        <v>31.55</v>
       </c>
       <c r="D13" t="n">
-        <v>1.64</v>
+        <v>2.4</v>
       </c>
       <c r="E13" t="n">
-        <v>32.2</v>
+        <v>28.3</v>
       </c>
       <c r="F13" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G13" t="n">
-        <v>29.2</v>
+        <v>22.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>31.73</v>
+        <v>47.96</v>
       </c>
       <c r="D14" t="n">
-        <v>2.41</v>
+        <v>3.93</v>
       </c>
       <c r="E14" t="n">
-        <v>30.5</v>
+        <v>25</v>
       </c>
       <c r="F14" t="n">
-        <v>23.7</v>
+        <v>19.2</v>
       </c>
       <c r="G14" t="n">
-        <v>25.8</v>
+        <v>20.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10.98</v>
+        <v>34.96</v>
       </c>
       <c r="D15" t="n">
-        <v>0.7</v>
+        <v>3.78</v>
       </c>
       <c r="E15" t="n">
-        <v>26.3</v>
+        <v>20</v>
       </c>
       <c r="F15" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G15" t="n">
-        <v>23.3</v>
+        <v>20</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6.73</v>
+        <v>14.6</v>
       </c>
       <c r="D16" t="n">
-        <v>0.64</v>
+        <v>1.19</v>
       </c>
       <c r="E16" t="n">
-        <v>11.9</v>
+        <v>15.8</v>
       </c>
       <c r="F16" t="n">
-        <v>22.9</v>
+        <v>13.3</v>
       </c>
       <c r="G16" t="n">
-        <v>19.6</v>
+        <v>14.1</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>26.42</v>
+        <v>19.49</v>
       </c>
       <c r="D17" t="n">
-        <v>2.43</v>
+        <v>1.63</v>
       </c>
       <c r="E17" t="n">
-        <v>18.6</v>
+        <v>18.3</v>
       </c>
       <c r="F17" t="n">
-        <v>16.1</v>
+        <v>11.7</v>
       </c>
       <c r="G17" t="n">
-        <v>16.9</v>
+        <v>13.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>24.39</v>
+        <v>22.62</v>
       </c>
       <c r="D18" t="n">
-        <v>1.99</v>
+        <v>2.05</v>
       </c>
       <c r="E18" t="n">
-        <v>18.6</v>
+        <v>11.7</v>
       </c>
       <c r="F18" t="n">
-        <v>12.7</v>
+        <v>10.8</v>
       </c>
       <c r="G18" t="n">
-        <v>14.5</v>
+        <v>11.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>14.53</v>
+        <v>10.81</v>
       </c>
       <c r="D19" t="n">
-        <v>1.19</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>10.2</v>
+        <v>15</v>
       </c>
       <c r="F19" t="n">
-        <v>12.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>11.9</v>
+        <v>10.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>15.38</v>
+        <v>59.42</v>
       </c>
       <c r="D20" t="n">
-        <v>2.28</v>
+        <v>3.82</v>
       </c>
       <c r="E20" t="n">
-        <v>16.9</v>
+        <v>10.8</v>
       </c>
       <c r="F20" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G20" t="n">
         <v>8.5</v>
       </c>
-      <c r="G20" t="n">
-        <v>11</v>
-      </c>
       <c r="H20" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>19.37</v>
+        <v>18.84</v>
       </c>
       <c r="D21" t="n">
-        <v>1.62</v>
+        <v>3.26</v>
       </c>
       <c r="E21" t="n">
-        <v>13.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>9.300000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>10.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>17.01</v>
+        <v>10.72</v>
       </c>
       <c r="D22" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="E22" t="n">
-        <v>11.9</v>
+        <v>1.7</v>
       </c>
       <c r="F22" t="n">
-        <v>9.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="G22" t="n">
-        <v>10.1</v>
+        <v>7.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10.84</v>
+        <v>23.85</v>
       </c>
       <c r="D23" t="n">
-        <v>0.98</v>
+        <v>1.95</v>
       </c>
       <c r="E23" t="n">
-        <v>1.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>13.6</v>
+        <v>5.8</v>
       </c>
       <c r="G23" t="n">
-        <v>10</v>
+        <v>6.8</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.25</v>
+        <v>19.32</v>
       </c>
       <c r="D24" t="n">
-        <v>1.83</v>
+        <v>1.8</v>
       </c>
       <c r="E24" t="n">
-        <v>10.2</v>
+        <v>1.7</v>
       </c>
       <c r="F24" t="n">
-        <v>9.300000000000001</v>
+        <v>5</v>
       </c>
       <c r="G24" t="n">
-        <v>9.6</v>
+        <v>4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>19.08</v>
+        <v>21.96</v>
       </c>
       <c r="D25" t="n">
-        <v>3.3</v>
+        <v>1.8</v>
       </c>
       <c r="E25" t="n">
-        <v>8.5</v>
+        <v>1.7</v>
       </c>
       <c r="F25" t="n">
-        <v>8.5</v>
+        <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>8.5</v>
+        <v>4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>17.28</v>
+        <v>15.24</v>
       </c>
       <c r="D26" t="n">
-        <v>1.6</v>
+        <v>2.25</v>
       </c>
       <c r="E26" t="n">
-        <v>8.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F26" t="n">
-        <v>8.5</v>
+        <v>1.7</v>
       </c>
       <c r="G26" t="n">
-        <v>8.5</v>
+        <v>3.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>19.47</v>
+        <v>27.64</v>
       </c>
       <c r="D27" t="n">
-        <v>1.82</v>
+        <v>2.31</v>
       </c>
       <c r="E27" t="n">
-        <v>8.5</v>
+        <v>3.3</v>
       </c>
       <c r="F27" t="n">
-        <v>8.5</v>
+        <v>2.5</v>
       </c>
       <c r="G27" t="n">
-        <v>8.5</v>
+        <v>2.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22.57</v>
+        <v>26.22</v>
       </c>
       <c r="D28" t="n">
-        <v>2.04</v>
+        <v>1.94</v>
       </c>
       <c r="E28" t="n">
-        <v>8.5</v>
+        <v>3.3</v>
       </c>
       <c r="F28" t="n">
-        <v>8.5</v>
+        <v>1.7</v>
       </c>
       <c r="G28" t="n">
-        <v>8.5</v>
+        <v>2.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>12.98</v>
+        <v>16.66</v>
       </c>
       <c r="D29" t="n">
-        <v>1.22</v>
+        <v>0.92</v>
       </c>
       <c r="E29" t="n">
-        <v>8.5</v>
+        <v>1.7</v>
       </c>
       <c r="F29" t="n">
-        <v>8.5</v>
+        <v>1.7</v>
       </c>
       <c r="G29" t="n">
-        <v>8.5</v>
+        <v>1.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>26.54</v>
+        <v>23.44</v>
       </c>
       <c r="D30" t="n">
-        <v>1.96</v>
+        <v>2.16</v>
       </c>
       <c r="E30" t="n">
-        <v>10.2</v>
+        <v>1.7</v>
       </c>
       <c r="F30" t="n">
-        <v>5.1</v>
+        <v>1.7</v>
       </c>
       <c r="G30" t="n">
-        <v>6.6</v>
+        <v>1.7</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>23.84</v>
+        <v>12.65</v>
       </c>
       <c r="D31" t="n">
-        <v>2.2</v>
+        <v>1.19</v>
       </c>
       <c r="E31" t="n">
-        <v>3.4</v>
+        <v>1.7</v>
       </c>
       <c r="F31" t="n">
         <v>1.7</v>
       </c>
       <c r="G31" t="n">
-        <v>2.2</v>
+        <v>1.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>27.59</v>
+        <v>16.92</v>
       </c>
       <c r="D32" t="n">
-        <v>2.31</v>
+        <v>1.57</v>
       </c>
       <c r="E32" t="n">
         <v>1.7</v>
@@ -1401,7 +1401,7 @@
         <v>1.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Jun 24 12:10:13 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,52 +486,52 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>82.97</v>
+        <v>86.81</v>
       </c>
       <c r="D2" t="n">
-        <v>8.67</v>
+        <v>9.07</v>
       </c>
       <c r="E2" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>34.95</v>
+        <v>46.35</v>
       </c>
       <c r="D3" t="n">
-        <v>3.31</v>
+        <v>2.57</v>
       </c>
       <c r="E3" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="4">
@@ -546,622 +546,622 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>43.98</v>
+        <v>44.44</v>
       </c>
       <c r="D4" t="n">
-        <v>3.72</v>
+        <v>3.76</v>
       </c>
       <c r="E4" t="n">
-        <v>90</v>
+        <v>91.8</v>
       </c>
       <c r="F4" t="n">
-        <v>90</v>
+        <v>91.8</v>
       </c>
       <c r="G4" t="n">
-        <v>90</v>
+        <v>91.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>43.56</v>
+        <v>35</v>
       </c>
       <c r="D5" t="n">
-        <v>2.42</v>
+        <v>3.31</v>
       </c>
       <c r="E5" t="n">
-        <v>90</v>
+        <v>91.8</v>
       </c>
       <c r="F5" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G5" t="n">
-        <v>90</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.34</v>
+        <v>29.16</v>
       </c>
       <c r="D6" t="n">
-        <v>1.25</v>
+        <v>2.67</v>
       </c>
       <c r="E6" t="n">
-        <v>71.7</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>60.8</v>
+        <v>82.8</v>
       </c>
       <c r="G6" t="n">
-        <v>66.2</v>
+        <v>84.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.52</v>
+        <v>10.15</v>
       </c>
       <c r="D7" t="n">
-        <v>2.61</v>
+        <v>1.23</v>
       </c>
       <c r="E7" t="n">
-        <v>56.7</v>
+        <v>55.7</v>
       </c>
       <c r="F7" t="n">
-        <v>54.2</v>
+        <v>53.3</v>
       </c>
       <c r="G7" t="n">
-        <v>55.4</v>
+        <v>54.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.86</v>
+        <v>122.31</v>
       </c>
       <c r="D8" t="n">
-        <v>0.65</v>
+        <v>4.59</v>
       </c>
       <c r="E8" t="n">
-        <v>60</v>
+        <v>54.1</v>
       </c>
       <c r="F8" t="n">
-        <v>50.8</v>
+        <v>51.6</v>
       </c>
       <c r="G8" t="n">
-        <v>55.4</v>
+        <v>52.9</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>117.24</v>
+        <v>48.2</v>
       </c>
       <c r="D9" t="n">
-        <v>4.4</v>
+        <v>3.95</v>
       </c>
       <c r="E9" t="n">
-        <v>33.3</v>
+        <v>32.8</v>
       </c>
       <c r="F9" t="n">
-        <v>31.7</v>
+        <v>26.2</v>
       </c>
       <c r="G9" t="n">
-        <v>32.5</v>
+        <v>28.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>22.19</v>
+        <v>22.25</v>
       </c>
       <c r="D10" t="n">
-        <v>1.63</v>
+        <v>3.68</v>
       </c>
       <c r="E10" t="n">
-        <v>26.7</v>
+        <v>44.3</v>
       </c>
       <c r="F10" t="n">
-        <v>23.3</v>
+        <v>20.5</v>
       </c>
       <c r="G10" t="n">
-        <v>24.3</v>
+        <v>27.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>22.19</v>
+        <v>26.88</v>
       </c>
       <c r="D11" t="n">
-        <v>3.67</v>
+        <v>2.47</v>
       </c>
       <c r="E11" t="n">
-        <v>41.7</v>
+        <v>34.4</v>
       </c>
       <c r="F11" t="n">
-        <v>16.7</v>
+        <v>24.6</v>
       </c>
       <c r="G11" t="n">
-        <v>24.2</v>
+        <v>27.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>26.69</v>
+        <v>35.16</v>
       </c>
       <c r="D12" t="n">
-        <v>2.45</v>
+        <v>3.8</v>
       </c>
       <c r="E12" t="n">
-        <v>33.3</v>
+        <v>23</v>
       </c>
       <c r="F12" t="n">
-        <v>20</v>
+        <v>21.3</v>
       </c>
       <c r="G12" t="n">
-        <v>24</v>
+        <v>21.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>31.55</v>
+        <v>14.59</v>
       </c>
       <c r="D13" t="n">
-        <v>2.4</v>
+        <v>1.19</v>
       </c>
       <c r="E13" t="n">
-        <v>28.3</v>
+        <v>13.9</v>
       </c>
       <c r="F13" t="n">
-        <v>20</v>
+        <v>13.9</v>
       </c>
       <c r="G13" t="n">
-        <v>22.5</v>
+        <v>13.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>47.96</v>
+        <v>59.84</v>
       </c>
       <c r="D14" t="n">
-        <v>3.93</v>
+        <v>3.85</v>
       </c>
       <c r="E14" t="n">
-        <v>25</v>
+        <v>19.7</v>
       </c>
       <c r="F14" t="n">
-        <v>19.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>20.9</v>
+        <v>12.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>34.96</v>
+        <v>19.34</v>
       </c>
       <c r="D15" t="n">
-        <v>3.78</v>
+        <v>1.62</v>
       </c>
       <c r="E15" t="n">
-        <v>20</v>
+        <v>13.1</v>
       </c>
       <c r="F15" t="n">
-        <v>20</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>20</v>
+        <v>10.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14.6</v>
+        <v>21.99</v>
       </c>
       <c r="D16" t="n">
-        <v>1.19</v>
+        <v>1.61</v>
       </c>
       <c r="E16" t="n">
-        <v>15.8</v>
+        <v>13.1</v>
       </c>
       <c r="F16" t="n">
-        <v>13.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>14.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>19.49</v>
+        <v>31.19</v>
       </c>
       <c r="D17" t="n">
-        <v>1.63</v>
+        <v>2.37</v>
       </c>
       <c r="E17" t="n">
-        <v>18.3</v>
+        <v>14.8</v>
       </c>
       <c r="F17" t="n">
-        <v>11.7</v>
+        <v>7.4</v>
       </c>
       <c r="G17" t="n">
-        <v>13.7</v>
+        <v>9.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>22.62</v>
+        <v>10.77</v>
       </c>
       <c r="D18" t="n">
-        <v>2.05</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>11.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F18" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
       <c r="G18" t="n">
-        <v>11.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.81</v>
+        <v>10.47</v>
       </c>
       <c r="D19" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E19" t="n">
-        <v>15</v>
+        <v>1.6</v>
       </c>
       <c r="F19" t="n">
-        <v>8.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>10.3</v>
+        <v>7.4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>59.42</v>
+        <v>6.69</v>
       </c>
       <c r="D20" t="n">
-        <v>3.82</v>
+        <v>0.63</v>
       </c>
       <c r="E20" t="n">
-        <v>10.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F20" t="n">
-        <v>7.5</v>
+        <v>5.7</v>
       </c>
       <c r="G20" t="n">
-        <v>8.5</v>
+        <v>7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>18.84</v>
+        <v>22.44</v>
       </c>
       <c r="D21" t="n">
-        <v>3.26</v>
+        <v>2.03</v>
       </c>
       <c r="E21" t="n">
-        <v>8.300000000000001</v>
+        <v>1.6</v>
       </c>
       <c r="F21" t="n">
-        <v>8.300000000000001</v>
+        <v>4.9</v>
       </c>
       <c r="G21" t="n">
-        <v>8.300000000000001</v>
+        <v>3.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10.72</v>
+        <v>12.63</v>
       </c>
       <c r="D22" t="n">
-        <v>0.97</v>
+        <v>1.19</v>
       </c>
       <c r="E22" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="F22" t="n">
-        <v>10</v>
+        <v>2.5</v>
       </c>
       <c r="G22" t="n">
-        <v>7.5</v>
+        <v>2.2</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>23.85</v>
+        <v>15.04</v>
       </c>
       <c r="D23" t="n">
-        <v>1.95</v>
+        <v>2.22</v>
       </c>
       <c r="E23" t="n">
-        <v>9.199999999999999</v>
+        <v>3.3</v>
       </c>
       <c r="F23" t="n">
-        <v>5.8</v>
+        <v>1.6</v>
       </c>
       <c r="G23" t="n">
-        <v>6.8</v>
+        <v>2.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>19.32</v>
+        <v>25.54</v>
       </c>
       <c r="D24" t="n">
-        <v>1.8</v>
+        <v>1.89</v>
       </c>
       <c r="E24" t="n">
-        <v>1.7</v>
+        <v>3.3</v>
       </c>
       <c r="F24" t="n">
-        <v>5</v>
+        <v>1.6</v>
       </c>
       <c r="G24" t="n">
-        <v>4</v>
+        <v>2.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="25">
@@ -1176,112 +1176,112 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21.96</v>
+        <v>21.55</v>
       </c>
       <c r="D25" t="n">
-        <v>1.8</v>
+        <v>1.77</v>
       </c>
       <c r="E25" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>1.6</v>
       </c>
       <c r="G25" t="n">
-        <v>4</v>
+        <v>1.6</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>15.24</v>
+        <v>18.95</v>
       </c>
       <c r="D26" t="n">
-        <v>2.25</v>
+        <v>1.77</v>
       </c>
       <c r="E26" t="n">
-        <v>8.300000000000001</v>
+        <v>1.6</v>
       </c>
       <c r="F26" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="G26" t="n">
-        <v>3.7</v>
+        <v>1.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>27.64</v>
+        <v>18.62</v>
       </c>
       <c r="D27" t="n">
-        <v>2.31</v>
+        <v>3.22</v>
       </c>
       <c r="E27" t="n">
-        <v>3.3</v>
+        <v>1.6</v>
       </c>
       <c r="F27" t="n">
-        <v>2.5</v>
+        <v>1.6</v>
       </c>
       <c r="G27" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>26.22</v>
+        <v>23.16</v>
       </c>
       <c r="D28" t="n">
-        <v>1.94</v>
+        <v>2.14</v>
       </c>
       <c r="E28" t="n">
-        <v>3.3</v>
+        <v>1.6</v>
       </c>
       <c r="F28" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="G28" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="29">
@@ -1296,112 +1296,112 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>16.66</v>
+        <v>16.52</v>
       </c>
       <c r="D29" t="n">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
       <c r="E29" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="F29" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="G29" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>23.44</v>
+        <v>23.57</v>
       </c>
       <c r="D30" t="n">
-        <v>2.16</v>
+        <v>1.93</v>
       </c>
       <c r="E30" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="F30" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="G30" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>12.65</v>
+        <v>16.61</v>
       </c>
       <c r="D31" t="n">
-        <v>1.19</v>
+        <v>1.54</v>
       </c>
       <c r="E31" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="F31" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="G31" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>16.92</v>
+        <v>26.83</v>
       </c>
       <c r="D32" t="n">
-        <v>1.57</v>
+        <v>2.24</v>
       </c>
       <c r="E32" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="F32" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="G32" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Jun 25 12:06:22 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>86.81</v>
+        <v>90.23</v>
       </c>
       <c r="D2" t="n">
-        <v>9.07</v>
+        <v>9.43</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,7 +501,7 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="3">
@@ -516,10 +516,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>46.35</v>
+        <v>48.44</v>
       </c>
       <c r="D3" t="n">
-        <v>2.57</v>
+        <v>2.69</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -531,127 +531,127 @@
         <v>100</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>44.44</v>
+        <v>35.45</v>
       </c>
       <c r="D4" t="n">
-        <v>3.76</v>
+        <v>3.37</v>
       </c>
       <c r="E4" t="n">
-        <v>91.8</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>91.8</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>91.8</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>35</v>
+        <v>44.82</v>
       </c>
       <c r="D5" t="n">
-        <v>3.31</v>
+        <v>3.79</v>
       </c>
       <c r="E5" t="n">
-        <v>91.8</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>91</v>
+        <v>95.2</v>
       </c>
       <c r="G5" t="n">
-        <v>91.40000000000001</v>
+        <v>93.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>29.16</v>
+        <v>10.41</v>
       </c>
       <c r="D6" t="n">
-        <v>2.67</v>
+        <v>1.26</v>
       </c>
       <c r="E6" t="n">
-        <v>86.90000000000001</v>
+        <v>75.8</v>
       </c>
       <c r="F6" t="n">
-        <v>82.8</v>
+        <v>64.5</v>
       </c>
       <c r="G6" t="n">
-        <v>84.8</v>
+        <v>70.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10.15</v>
+        <v>28.92</v>
       </c>
       <c r="D7" t="n">
-        <v>1.23</v>
+        <v>2.65</v>
       </c>
       <c r="E7" t="n">
-        <v>55.7</v>
+        <v>67.7</v>
       </c>
       <c r="F7" t="n">
-        <v>53.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>54.5</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="8">
@@ -666,22 +666,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>122.31</v>
+        <v>121.75</v>
       </c>
       <c r="D8" t="n">
-        <v>4.59</v>
+        <v>4.57</v>
       </c>
       <c r="E8" t="n">
-        <v>54.1</v>
+        <v>46.8</v>
       </c>
       <c r="F8" t="n">
-        <v>51.6</v>
+        <v>46.8</v>
       </c>
       <c r="G8" t="n">
-        <v>52.9</v>
+        <v>46.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="9">
@@ -696,472 +696,472 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>48.2</v>
+        <v>48.27</v>
       </c>
       <c r="D9" t="n">
         <v>3.95</v>
       </c>
       <c r="E9" t="n">
-        <v>32.8</v>
+        <v>33.9</v>
       </c>
       <c r="F9" t="n">
-        <v>26.2</v>
+        <v>26.6</v>
       </c>
       <c r="G9" t="n">
-        <v>28.2</v>
+        <v>28.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>22.25</v>
+        <v>26.82</v>
       </c>
       <c r="D10" t="n">
-        <v>3.68</v>
+        <v>2.46</v>
       </c>
       <c r="E10" t="n">
-        <v>44.3</v>
+        <v>33.9</v>
       </c>
       <c r="F10" t="n">
-        <v>20.5</v>
+        <v>21</v>
       </c>
       <c r="G10" t="n">
-        <v>27.6</v>
+        <v>24.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>26.88</v>
+        <v>35.09</v>
       </c>
       <c r="D11" t="n">
-        <v>2.47</v>
+        <v>3.79</v>
       </c>
       <c r="E11" t="n">
-        <v>34.4</v>
+        <v>21</v>
       </c>
       <c r="F11" t="n">
-        <v>24.6</v>
+        <v>21</v>
       </c>
       <c r="G11" t="n">
-        <v>27.5</v>
+        <v>21</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>35.16</v>
+        <v>21.75</v>
       </c>
       <c r="D12" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="E12" t="n">
-        <v>23</v>
+        <v>27.4</v>
       </c>
       <c r="F12" t="n">
-        <v>21.3</v>
+        <v>8.1</v>
       </c>
       <c r="G12" t="n">
-        <v>21.8</v>
+        <v>13.9</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14.59</v>
+        <v>59.59</v>
       </c>
       <c r="D13" t="n">
-        <v>1.19</v>
+        <v>3.83</v>
       </c>
       <c r="E13" t="n">
-        <v>13.9</v>
+        <v>12.9</v>
       </c>
       <c r="F13" t="n">
-        <v>13.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>13.9</v>
+        <v>10.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>59.84</v>
+        <v>21.92</v>
       </c>
       <c r="D14" t="n">
-        <v>3.85</v>
+        <v>1.61</v>
       </c>
       <c r="E14" t="n">
-        <v>19.7</v>
+        <v>12.9</v>
       </c>
       <c r="F14" t="n">
-        <v>9.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="G14" t="n">
-        <v>12.8</v>
+        <v>10.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>19.34</v>
+        <v>14.54</v>
       </c>
       <c r="D15" t="n">
-        <v>1.62</v>
+        <v>1.18</v>
       </c>
       <c r="E15" t="n">
-        <v>13.1</v>
+        <v>11.3</v>
       </c>
       <c r="F15" t="n">
-        <v>9.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="G15" t="n">
-        <v>10.8</v>
+        <v>9.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>21.99</v>
+        <v>10.73</v>
       </c>
       <c r="D16" t="n">
-        <v>1.61</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>13.1</v>
+        <v>5.6</v>
       </c>
       <c r="F16" t="n">
-        <v>8.199999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>9.699999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>31.19</v>
+        <v>10.34</v>
       </c>
       <c r="D17" t="n">
-        <v>2.37</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E17" t="n">
-        <v>14.8</v>
+        <v>1.6</v>
       </c>
       <c r="F17" t="n">
-        <v>7.4</v>
+        <v>8.9</v>
       </c>
       <c r="G17" t="n">
-        <v>9.6</v>
+        <v>6.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>10.77</v>
+        <v>30.9</v>
       </c>
       <c r="D18" t="n">
-        <v>0.6899999999999999</v>
+        <v>2.35</v>
       </c>
       <c r="E18" t="n">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="F18" t="n">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="G18" t="n">
-        <v>8.800000000000001</v>
+        <v>4.7</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.47</v>
+        <v>18.69</v>
       </c>
       <c r="D19" t="n">
-        <v>0.95</v>
+        <v>3.23</v>
       </c>
       <c r="E19" t="n">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="F19" t="n">
-        <v>9.800000000000001</v>
+        <v>3.2</v>
       </c>
       <c r="G19" t="n">
-        <v>7.4</v>
+        <v>3.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6.69</v>
+        <v>23.64</v>
       </c>
       <c r="D20" t="n">
-        <v>0.63</v>
+        <v>1.93</v>
       </c>
       <c r="E20" t="n">
-        <v>9.800000000000001</v>
+        <v>3.2</v>
       </c>
       <c r="F20" t="n">
-        <v>5.7</v>
+        <v>2.4</v>
       </c>
       <c r="G20" t="n">
-        <v>7</v>
+        <v>2.7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>22.44</v>
+        <v>15.03</v>
       </c>
       <c r="D21" t="n">
-        <v>2.03</v>
+        <v>2.22</v>
       </c>
       <c r="E21" t="n">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="F21" t="n">
-        <v>4.9</v>
+        <v>2.4</v>
       </c>
       <c r="G21" t="n">
-        <v>3.9</v>
+        <v>2.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>12.63</v>
+        <v>25.36</v>
       </c>
       <c r="D22" t="n">
-        <v>1.19</v>
+        <v>1.88</v>
       </c>
       <c r="E22" t="n">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="F22" t="n">
-        <v>2.5</v>
+        <v>1.6</v>
       </c>
       <c r="G22" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>15.04</v>
+        <v>16.3</v>
       </c>
       <c r="D23" t="n">
-        <v>2.22</v>
+        <v>0.9</v>
       </c>
       <c r="E23" t="n">
-        <v>3.3</v>
+        <v>1.6</v>
       </c>
       <c r="F23" t="n">
         <v>1.6</v>
       </c>
       <c r="G23" t="n">
-        <v>2.1</v>
+        <v>1.6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>25.54</v>
+        <v>22.83</v>
       </c>
       <c r="D24" t="n">
-        <v>1.89</v>
+        <v>2.1</v>
       </c>
       <c r="E24" t="n">
-        <v>3.3</v>
+        <v>1.6</v>
       </c>
       <c r="F24" t="n">
         <v>1.6</v>
       </c>
       <c r="G24" t="n">
-        <v>2.1</v>
+        <v>1.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="25">
@@ -1176,10 +1176,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21.55</v>
+        <v>21.36</v>
       </c>
       <c r="D25" t="n">
-        <v>1.77</v>
+        <v>1.75</v>
       </c>
       <c r="E25" t="n">
         <v>1.6</v>
@@ -1191,7 +1191,7 @@
         <v>1.6</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="26">
@@ -1206,10 +1206,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18.95</v>
+        <v>18.57</v>
       </c>
       <c r="D26" t="n">
-        <v>1.77</v>
+        <v>1.73</v>
       </c>
       <c r="E26" t="n">
         <v>1.6</v>
@@ -1221,25 +1221,25 @@
         <v>1.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18.62</v>
+        <v>19.18</v>
       </c>
       <c r="D27" t="n">
-        <v>3.22</v>
+        <v>1.6</v>
       </c>
       <c r="E27" t="n">
         <v>1.6</v>
@@ -1251,25 +1251,25 @@
         <v>1.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>23.16</v>
+        <v>22.14</v>
       </c>
       <c r="D28" t="n">
-        <v>2.14</v>
+        <v>2</v>
       </c>
       <c r="E28" t="n">
         <v>1.6</v>
@@ -1281,25 +1281,25 @@
         <v>1.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>16.52</v>
+        <v>6.61</v>
       </c>
       <c r="D29" t="n">
-        <v>0.91</v>
+        <v>0.62</v>
       </c>
       <c r="E29" t="n">
         <v>1.6</v>
@@ -1311,25 +1311,25 @@
         <v>1.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>23.57</v>
+        <v>16.27</v>
       </c>
       <c r="D30" t="n">
-        <v>1.93</v>
+        <v>1.51</v>
       </c>
       <c r="E30" t="n">
         <v>1.6</v>
@@ -1341,25 +1341,25 @@
         <v>1.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>16.61</v>
+        <v>12.16</v>
       </c>
       <c r="D31" t="n">
-        <v>1.54</v>
+        <v>1.14</v>
       </c>
       <c r="E31" t="n">
         <v>1.6</v>
@@ -1371,7 +1371,7 @@
         <v>1.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="32">
@@ -1386,10 +1386,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>26.83</v>
+        <v>26.63</v>
       </c>
       <c r="D32" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
       <c r="E32" t="n">
         <v>1.6</v>
@@ -1401,7 +1401,7 @@
         <v>1.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Jun 26 12:02:11 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>90.23</v>
+        <v>50.21</v>
       </c>
       <c r="D2" t="n">
-        <v>9.43</v>
+        <v>2.78</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -501,157 +501,157 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>48.44</v>
+        <v>87.76000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>2.69</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35.45</v>
+        <v>43.46</v>
       </c>
       <c r="D4" t="n">
-        <v>3.37</v>
+        <v>3.68</v>
       </c>
       <c r="E4" t="n">
-        <v>98.40000000000001</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>98.40000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>98.40000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>44.82</v>
+        <v>33.66</v>
       </c>
       <c r="D5" t="n">
-        <v>3.79</v>
+        <v>3.18</v>
       </c>
       <c r="E5" t="n">
-        <v>91.90000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>95.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>93.5</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.41</v>
+        <v>28.17</v>
       </c>
       <c r="D6" t="n">
-        <v>1.26</v>
+        <v>2.58</v>
       </c>
       <c r="E6" t="n">
-        <v>75.8</v>
+        <v>46</v>
       </c>
       <c r="F6" t="n">
-        <v>64.5</v>
+        <v>43.7</v>
       </c>
       <c r="G6" t="n">
-        <v>70.2</v>
+        <v>44.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.92</v>
+        <v>9.99</v>
       </c>
       <c r="D7" t="n">
-        <v>2.65</v>
+        <v>1.21</v>
       </c>
       <c r="E7" t="n">
-        <v>67.7</v>
+        <v>38.1</v>
       </c>
       <c r="F7" t="n">
-        <v>66.09999999999999</v>
+        <v>37.3</v>
       </c>
       <c r="G7" t="n">
-        <v>66.90000000000001</v>
+        <v>37.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="8">
@@ -666,112 +666,112 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>121.75</v>
+        <v>116.68</v>
       </c>
       <c r="D8" t="n">
-        <v>4.57</v>
+        <v>4.38</v>
       </c>
       <c r="E8" t="n">
-        <v>46.8</v>
+        <v>30.2</v>
       </c>
       <c r="F8" t="n">
-        <v>46.8</v>
+        <v>28.6</v>
       </c>
       <c r="G8" t="n">
-        <v>46.8</v>
+        <v>29</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>48.27</v>
+        <v>59.23</v>
       </c>
       <c r="D9" t="n">
-        <v>3.95</v>
+        <v>3.81</v>
       </c>
       <c r="E9" t="n">
-        <v>33.9</v>
+        <v>9.5</v>
       </c>
       <c r="F9" t="n">
-        <v>26.6</v>
+        <v>6.3</v>
       </c>
       <c r="G9" t="n">
-        <v>28.8</v>
+        <v>7.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>26.82</v>
+        <v>33.62</v>
       </c>
       <c r="D10" t="n">
-        <v>2.46</v>
+        <v>3.63</v>
       </c>
       <c r="E10" t="n">
-        <v>33.9</v>
+        <v>6.3</v>
       </c>
       <c r="F10" t="n">
-        <v>21</v>
+        <v>6.3</v>
       </c>
       <c r="G10" t="n">
-        <v>24.8</v>
+        <v>6.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>35.09</v>
+        <v>10.1</v>
       </c>
       <c r="D11" t="n">
-        <v>3.79</v>
+        <v>0.92</v>
       </c>
       <c r="E11" t="n">
-        <v>21</v>
+        <v>1.6</v>
       </c>
       <c r="F11" t="n">
-        <v>21</v>
+        <v>7.9</v>
       </c>
       <c r="G11" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="12">
@@ -786,112 +786,112 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>21.75</v>
+        <v>20.84</v>
       </c>
       <c r="D12" t="n">
-        <v>3.6</v>
+        <v>3.45</v>
       </c>
       <c r="E12" t="n">
-        <v>27.4</v>
+        <v>7.9</v>
       </c>
       <c r="F12" t="n">
-        <v>8.1</v>
+        <v>4</v>
       </c>
       <c r="G12" t="n">
-        <v>13.9</v>
+        <v>5.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>59.59</v>
+        <v>46.21</v>
       </c>
       <c r="D13" t="n">
-        <v>3.83</v>
+        <v>3.79</v>
       </c>
       <c r="E13" t="n">
-        <v>12.9</v>
+        <v>9.5</v>
       </c>
       <c r="F13" t="n">
-        <v>9.699999999999999</v>
+        <v>3.2</v>
       </c>
       <c r="G13" t="n">
-        <v>10.6</v>
+        <v>5.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21.92</v>
+        <v>25.98</v>
       </c>
       <c r="D14" t="n">
-        <v>1.61</v>
+        <v>2.39</v>
       </c>
       <c r="E14" t="n">
-        <v>12.9</v>
+        <v>5.6</v>
       </c>
       <c r="F14" t="n">
-        <v>8.9</v>
+        <v>4</v>
       </c>
       <c r="G14" t="n">
-        <v>10.1</v>
+        <v>4.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14.54</v>
+        <v>25.4</v>
       </c>
       <c r="D15" t="n">
-        <v>1.18</v>
+        <v>1.88</v>
       </c>
       <c r="E15" t="n">
-        <v>11.3</v>
+        <v>4.8</v>
       </c>
       <c r="F15" t="n">
-        <v>8.9</v>
+        <v>2.4</v>
       </c>
       <c r="G15" t="n">
-        <v>9.6</v>
+        <v>3.1</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="16">
@@ -906,202 +906,202 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.73</v>
+        <v>10.57</v>
       </c>
       <c r="D16" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="E16" t="n">
-        <v>5.6</v>
+        <v>3.2</v>
       </c>
       <c r="F16" t="n">
-        <v>9.699999999999999</v>
+        <v>2.4</v>
       </c>
       <c r="G16" t="n">
-        <v>8.5</v>
+        <v>2.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.34</v>
+        <v>14.93</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.21</v>
       </c>
       <c r="E17" t="n">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="F17" t="n">
-        <v>8.9</v>
+        <v>1.6</v>
       </c>
       <c r="G17" t="n">
-        <v>6.7</v>
+        <v>2.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>30.9</v>
+        <v>6.56</v>
       </c>
       <c r="D18" t="n">
-        <v>2.35</v>
+        <v>0.62</v>
       </c>
       <c r="E18" t="n">
-        <v>8.1</v>
+        <v>1.6</v>
       </c>
       <c r="F18" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="G18" t="n">
-        <v>4.7</v>
+        <v>2.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18.69</v>
+        <v>18.48</v>
       </c>
       <c r="D19" t="n">
-        <v>3.23</v>
+        <v>1.72</v>
       </c>
       <c r="E19" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="F19" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="G19" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>23.64</v>
+        <v>21.79</v>
       </c>
       <c r="D20" t="n">
-        <v>1.93</v>
+        <v>1.97</v>
       </c>
       <c r="E20" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="F20" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="G20" t="n">
-        <v>2.7</v>
+        <v>1.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>15.03</v>
+        <v>18.16</v>
       </c>
       <c r="D21" t="n">
-        <v>2.22</v>
+        <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="F21" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="G21" t="n">
-        <v>2.7</v>
+        <v>1.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>25.36</v>
+        <v>18.83</v>
       </c>
       <c r="D22" t="n">
-        <v>1.88</v>
+        <v>1.57</v>
       </c>
       <c r="E22" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="F22" t="n">
         <v>1.6</v>
       </c>
       <c r="G22" t="n">
-        <v>2.1</v>
+        <v>1.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="23">
@@ -1116,10 +1116,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>16.3</v>
+        <v>15.76</v>
       </c>
       <c r="D23" t="n">
-        <v>0.9</v>
+        <v>0.87</v>
       </c>
       <c r="E23" t="n">
         <v>1.6</v>
@@ -1131,7 +1131,7 @@
         <v>1.6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="24">
@@ -1146,10 +1146,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.83</v>
+        <v>22.1</v>
       </c>
       <c r="D24" t="n">
-        <v>2.1</v>
+        <v>2.04</v>
       </c>
       <c r="E24" t="n">
         <v>1.6</v>
@@ -1161,7 +1161,7 @@
         <v>1.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="25">
@@ -1176,10 +1176,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21.36</v>
+        <v>20.68</v>
       </c>
       <c r="D25" t="n">
-        <v>1.75</v>
+        <v>1.7</v>
       </c>
       <c r="E25" t="n">
         <v>1.6</v>
@@ -1191,25 +1191,25 @@
         <v>1.6</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18.57</v>
+        <v>14.17</v>
       </c>
       <c r="D26" t="n">
-        <v>1.73</v>
+        <v>1.15</v>
       </c>
       <c r="E26" t="n">
         <v>1.6</v>
@@ -1221,25 +1221,25 @@
         <v>1.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>19.18</v>
+        <v>30.29</v>
       </c>
       <c r="D27" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="E27" t="n">
         <v>1.6</v>
@@ -1251,25 +1251,25 @@
         <v>1.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22.14</v>
+        <v>22.98</v>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>1.88</v>
       </c>
       <c r="E28" t="n">
         <v>1.6</v>
@@ -1281,25 +1281,25 @@
         <v>1.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6.61</v>
+        <v>16.04</v>
       </c>
       <c r="D29" t="n">
-        <v>0.62</v>
+        <v>1.48</v>
       </c>
       <c r="E29" t="n">
         <v>1.6</v>
@@ -1311,25 +1311,25 @@
         <v>1.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>16.27</v>
+        <v>12.01</v>
       </c>
       <c r="D30" t="n">
-        <v>1.51</v>
+        <v>1.13</v>
       </c>
       <c r="E30" t="n">
         <v>1.6</v>
@@ -1341,25 +1341,25 @@
         <v>1.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>12.16</v>
+        <v>21.28</v>
       </c>
       <c r="D31" t="n">
-        <v>1.14</v>
+        <v>1.56</v>
       </c>
       <c r="E31" t="n">
         <v>1.6</v>
@@ -1371,7 +1371,7 @@
         <v>1.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="32">
@@ -1386,10 +1386,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>26.63</v>
+        <v>26.07</v>
       </c>
       <c r="D32" t="n">
-        <v>2.23</v>
+        <v>2.18</v>
       </c>
       <c r="E32" t="n">
         <v>1.6</v>
@@ -1401,7 +1401,7 @@
         <v>1.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Jun 27 11:15:42 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.78</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>99.2</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>99.2</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>99.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>9.210000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>98.40000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="F3" t="n">
-        <v>98.40000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="G3" t="n">
-        <v>98.40000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.68</v>
       </c>
       <c r="E4" t="n">
-        <v>84.09999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>84.90000000000001</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>84.5</v>
+        <v>84</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>3.18</v>
       </c>
       <c r="E5" t="n">
-        <v>79.40000000000001</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>71.40000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>75.40000000000001</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.58</v>
       </c>
       <c r="E6" t="n">
-        <v>46</v>
+        <v>46.1</v>
       </c>
       <c r="F6" t="n">
-        <v>43.7</v>
+        <v>43.8</v>
       </c>
       <c r="G6" t="n">
-        <v>44.8</v>
+        <v>44.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.21</v>
       </c>
       <c r="E7" t="n">
-        <v>38.1</v>
+        <v>38.3</v>
       </c>
       <c r="F7" t="n">
-        <v>37.3</v>
+        <v>37.5</v>
       </c>
       <c r="G7" t="n">
-        <v>37.7</v>
+        <v>37.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>4.38</v>
       </c>
       <c r="E8" t="n">
-        <v>30.2</v>
+        <v>30.5</v>
       </c>
       <c r="F8" t="n">
-        <v>28.6</v>
+        <v>28.9</v>
       </c>
       <c r="G8" t="n">
-        <v>29</v>
+        <v>29.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>3.81</v>
       </c>
       <c r="E9" t="n">
-        <v>9.5</v>
+        <v>10.2</v>
       </c>
       <c r="F9" t="n">
-        <v>6.3</v>
+        <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>7.3</v>
+        <v>8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>3.63</v>
       </c>
       <c r="E10" t="n">
-        <v>6.3</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>6.3</v>
+        <v>7</v>
       </c>
       <c r="G10" t="n">
-        <v>6.3</v>
+        <v>7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>0.92</v>
       </c>
       <c r="E11" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F11" t="n">
-        <v>7.9</v>
+        <v>8.6</v>
       </c>
       <c r="G11" t="n">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.45</v>
       </c>
       <c r="E12" t="n">
-        <v>7.9</v>
+        <v>8.6</v>
       </c>
       <c r="F12" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="G12" t="n">
-        <v>5.2</v>
+        <v>5.9</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>3.79</v>
       </c>
       <c r="E13" t="n">
-        <v>9.5</v>
+        <v>10.2</v>
       </c>
       <c r="F13" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="G13" t="n">
-        <v>5.1</v>
+        <v>5.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.39</v>
       </c>
       <c r="E14" t="n">
-        <v>5.6</v>
+        <v>6.2</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="G14" t="n">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.88</v>
       </c>
       <c r="E15" t="n">
-        <v>4.8</v>
+        <v>5.5</v>
       </c>
       <c r="F15" t="n">
-        <v>2.4</v>
+        <v>3.1</v>
       </c>
       <c r="G15" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="16">
@@ -912,76 +912,76 @@
         <v>0.68</v>
       </c>
       <c r="E16" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="F16" t="n">
-        <v>2.4</v>
+        <v>3.1</v>
       </c>
       <c r="G16" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14.93</v>
+        <v>6.56</v>
       </c>
       <c r="D17" t="n">
-        <v>2.21</v>
+        <v>0.62</v>
       </c>
       <c r="E17" t="n">
-        <v>3.2</v>
+        <v>2.3</v>
       </c>
       <c r="F17" t="n">
-        <v>1.6</v>
+        <v>3.1</v>
       </c>
       <c r="G17" t="n">
-        <v>2.1</v>
+        <v>2.9</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6.56</v>
+        <v>14.93</v>
       </c>
       <c r="D18" t="n">
-        <v>0.62</v>
+        <v>2.21</v>
       </c>
       <c r="E18" t="n">
-        <v>1.6</v>
+        <v>3.9</v>
       </c>
       <c r="F18" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="G18" t="n">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.72</v>
       </c>
       <c r="E19" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F19" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G19" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.97</v>
       </c>
       <c r="E20" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F20" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G20" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F21" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G21" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.57</v>
       </c>
       <c r="E22" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F22" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G22" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.87</v>
       </c>
       <c r="E23" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F23" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G23" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.04</v>
       </c>
       <c r="E24" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F24" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G24" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.7</v>
       </c>
       <c r="E25" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F25" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G25" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>1.15</v>
       </c>
       <c r="E26" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F26" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G26" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.3</v>
       </c>
       <c r="E27" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F27" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G27" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.88</v>
       </c>
       <c r="E28" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F28" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G28" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.48</v>
       </c>
       <c r="E29" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F29" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G29" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.13</v>
       </c>
       <c r="E30" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F30" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G30" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.56</v>
       </c>
       <c r="E31" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F31" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G31" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.18</v>
       </c>
       <c r="E32" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="F32" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G32" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Jun 28 11:25:37 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.78</v>
       </c>
       <c r="E2" t="n">
-        <v>99.2</v>
+        <v>98.5</v>
       </c>
       <c r="F2" t="n">
-        <v>99.2</v>
+        <v>98.5</v>
       </c>
       <c r="G2" t="n">
-        <v>99.2</v>
+        <v>98.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>9.210000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>97.7</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>97.7</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>97.7</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.68</v>
       </c>
       <c r="E4" t="n">
-        <v>83.59999999999999</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>84.40000000000001</v>
+        <v>83.8</v>
       </c>
       <c r="G4" t="n">
-        <v>84</v>
+        <v>83.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>3.18</v>
       </c>
       <c r="E5" t="n">
-        <v>78.90000000000001</v>
+        <v>78.5</v>
       </c>
       <c r="F5" t="n">
-        <v>71.09999999999999</v>
+        <v>70.8</v>
       </c>
       <c r="G5" t="n">
-        <v>75</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.58</v>
       </c>
       <c r="E6" t="n">
-        <v>46.1</v>
+        <v>46.2</v>
       </c>
       <c r="F6" t="n">
         <v>43.8</v>
       </c>
       <c r="G6" t="n">
-        <v>44.9</v>
+        <v>45</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.21</v>
       </c>
       <c r="E7" t="n">
-        <v>38.3</v>
+        <v>38.5</v>
       </c>
       <c r="F7" t="n">
-        <v>37.5</v>
+        <v>37.7</v>
       </c>
       <c r="G7" t="n">
-        <v>37.9</v>
+        <v>38.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>4.38</v>
       </c>
       <c r="E8" t="n">
-        <v>30.5</v>
+        <v>30.8</v>
       </c>
       <c r="F8" t="n">
-        <v>28.9</v>
+        <v>29.2</v>
       </c>
       <c r="G8" t="n">
-        <v>29.4</v>
+        <v>29.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>3.81</v>
       </c>
       <c r="E9" t="n">
-        <v>10.2</v>
+        <v>10.8</v>
       </c>
       <c r="F9" t="n">
-        <v>7</v>
+        <v>7.7</v>
       </c>
       <c r="G9" t="n">
-        <v>8</v>
+        <v>8.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>3.63</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>7.7</v>
       </c>
       <c r="F10" t="n">
-        <v>7</v>
+        <v>7.7</v>
       </c>
       <c r="G10" t="n">
-        <v>7</v>
+        <v>7.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="11">
@@ -762,76 +762,76 @@
         <v>0.92</v>
       </c>
       <c r="E11" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F11" t="n">
-        <v>8.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>6.7</v>
+        <v>7.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>20.84</v>
+        <v>46.21</v>
       </c>
       <c r="D12" t="n">
-        <v>3.45</v>
+        <v>3.79</v>
       </c>
       <c r="E12" t="n">
-        <v>8.6</v>
+        <v>10.8</v>
       </c>
       <c r="F12" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="G12" t="n">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>46.21</v>
+        <v>20.84</v>
       </c>
       <c r="D13" t="n">
-        <v>3.79</v>
+        <v>3.45</v>
       </c>
       <c r="E13" t="n">
-        <v>10.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>3.9</v>
+        <v>5.4</v>
       </c>
       <c r="G13" t="n">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.39</v>
       </c>
       <c r="E14" t="n">
-        <v>6.2</v>
+        <v>6.9</v>
       </c>
       <c r="F14" t="n">
-        <v>4.7</v>
+        <v>5.4</v>
       </c>
       <c r="G14" t="n">
-        <v>5.2</v>
+        <v>5.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.88</v>
       </c>
       <c r="E15" t="n">
-        <v>5.5</v>
+        <v>6.2</v>
       </c>
       <c r="F15" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="G15" t="n">
-        <v>3.8</v>
+        <v>4.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>0.68</v>
       </c>
       <c r="E16" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
       <c r="F16" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="G16" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>0.62</v>
       </c>
       <c r="E17" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F17" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="G17" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.21</v>
       </c>
       <c r="E18" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
       <c r="F18" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G18" t="n">
-        <v>2.8</v>
+        <v>3.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.72</v>
       </c>
       <c r="E19" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G19" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.97</v>
       </c>
       <c r="E20" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F20" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G20" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F21" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G21" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.57</v>
       </c>
       <c r="E22" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F22" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G22" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.87</v>
       </c>
       <c r="E23" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F23" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G23" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.04</v>
       </c>
       <c r="E24" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F24" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G24" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.7</v>
       </c>
       <c r="E25" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F25" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G25" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>1.15</v>
       </c>
       <c r="E26" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F26" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G26" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.3</v>
       </c>
       <c r="E27" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F27" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G27" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.88</v>
       </c>
       <c r="E28" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F28" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G28" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.48</v>
       </c>
       <c r="E29" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F29" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G29" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.13</v>
       </c>
       <c r="E30" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F30" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G30" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.56</v>
       </c>
       <c r="E31" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F31" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G31" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.18</v>
       </c>
       <c r="E32" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="F32" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="G32" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Jun 29 13:54:57 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,19 +477,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50.21</v>
+        <v>88.91</v>
       </c>
       <c r="D2" t="n">
-        <v>2.78</v>
+        <v>9.33</v>
       </c>
       <c r="E2" t="n">
         <v>98.5</v>
@@ -501,37 +501,37 @@
         <v>98.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>87.76000000000001</v>
+        <v>47.71</v>
       </c>
       <c r="D3" t="n">
-        <v>9.210000000000001</v>
+        <v>2.65</v>
       </c>
       <c r="E3" t="n">
-        <v>96.90000000000001</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>96.90000000000001</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>96.90000000000001</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +546,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>43.46</v>
+        <v>43.12</v>
       </c>
       <c r="D4" t="n">
-        <v>3.68</v>
+        <v>3.65</v>
       </c>
       <c r="E4" t="n">
-        <v>83.09999999999999</v>
+        <v>78.8</v>
       </c>
       <c r="F4" t="n">
-        <v>83.8</v>
+        <v>78</v>
       </c>
       <c r="G4" t="n">
-        <v>83.5</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="5">
@@ -576,442 +576,442 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>33.66</v>
+        <v>33.07</v>
       </c>
       <c r="D5" t="n">
-        <v>3.18</v>
+        <v>3.13</v>
       </c>
       <c r="E5" t="n">
-        <v>78.5</v>
+        <v>66.7</v>
       </c>
       <c r="F5" t="n">
-        <v>70.8</v>
+        <v>61.4</v>
       </c>
       <c r="G5" t="n">
-        <v>74.59999999999999</v>
+        <v>64</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28.17</v>
+        <v>10.15</v>
       </c>
       <c r="D6" t="n">
-        <v>2.58</v>
+        <v>1.23</v>
       </c>
       <c r="E6" t="n">
-        <v>46.2</v>
+        <v>56.8</v>
       </c>
       <c r="F6" t="n">
-        <v>43.8</v>
+        <v>54.5</v>
       </c>
       <c r="G6" t="n">
-        <v>45</v>
+        <v>55.7</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9.99</v>
+        <v>27.63</v>
       </c>
       <c r="D7" t="n">
-        <v>1.21</v>
+        <v>2.54</v>
       </c>
       <c r="E7" t="n">
-        <v>38.5</v>
+        <v>45.5</v>
       </c>
       <c r="F7" t="n">
-        <v>37.7</v>
+        <v>42.4</v>
       </c>
       <c r="G7" t="n">
-        <v>38.1</v>
+        <v>43.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>116.68</v>
+        <v>28.04</v>
       </c>
       <c r="D8" t="n">
-        <v>4.38</v>
+        <v>2.56</v>
       </c>
       <c r="E8" t="n">
-        <v>30.8</v>
+        <v>37.9</v>
       </c>
       <c r="F8" t="n">
-        <v>29.2</v>
+        <v>37.9</v>
       </c>
       <c r="G8" t="n">
-        <v>29.7</v>
+        <v>37.9</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>59.23</v>
+        <v>33.96</v>
       </c>
       <c r="D9" t="n">
-        <v>3.81</v>
+        <v>3.67</v>
       </c>
       <c r="E9" t="n">
-        <v>10.8</v>
+        <v>15.2</v>
       </c>
       <c r="F9" t="n">
-        <v>7.7</v>
+        <v>15.2</v>
       </c>
       <c r="G9" t="n">
-        <v>8.6</v>
+        <v>15.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>33.62</v>
+        <v>111.22</v>
       </c>
       <c r="D10" t="n">
-        <v>3.63</v>
+        <v>4.18</v>
       </c>
       <c r="E10" t="n">
-        <v>7.7</v>
+        <v>12.1</v>
       </c>
       <c r="F10" t="n">
-        <v>7.7</v>
+        <v>12.1</v>
       </c>
       <c r="G10" t="n">
-        <v>7.7</v>
+        <v>12.1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10.1</v>
+        <v>21.14</v>
       </c>
       <c r="D11" t="n">
-        <v>0.92</v>
+        <v>3.5</v>
       </c>
       <c r="E11" t="n">
-        <v>3.1</v>
+        <v>16.7</v>
       </c>
       <c r="F11" t="n">
-        <v>9.199999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>7.4</v>
+        <v>11.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>46.21</v>
+        <v>26.19</v>
       </c>
       <c r="D12" t="n">
-        <v>3.79</v>
+        <v>1.94</v>
       </c>
       <c r="E12" t="n">
-        <v>10.8</v>
+        <v>10.6</v>
       </c>
       <c r="F12" t="n">
-        <v>4.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>6.5</v>
+        <v>10.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>20.84</v>
+        <v>26.99</v>
       </c>
       <c r="D13" t="n">
-        <v>3.45</v>
+        <v>2.26</v>
       </c>
       <c r="E13" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="F13" t="n">
-        <v>5.4</v>
+        <v>9.1</v>
       </c>
       <c r="G13" t="n">
-        <v>6.5</v>
+        <v>9.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>25.98</v>
+        <v>10.13</v>
       </c>
       <c r="D14" t="n">
-        <v>2.39</v>
+        <v>0.92</v>
       </c>
       <c r="E14" t="n">
-        <v>6.9</v>
+        <v>6.1</v>
       </c>
       <c r="F14" t="n">
-        <v>5.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>5.8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>25.4</v>
+        <v>59.22</v>
       </c>
       <c r="D15" t="n">
-        <v>1.88</v>
+        <v>3.81</v>
       </c>
       <c r="E15" t="n">
-        <v>6.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>3.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>4.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.57</v>
+        <v>15.01</v>
       </c>
       <c r="D16" t="n">
-        <v>0.68</v>
+        <v>2.22</v>
       </c>
       <c r="E16" t="n">
-        <v>4.6</v>
+        <v>7.6</v>
       </c>
       <c r="F16" t="n">
-        <v>3.8</v>
+        <v>7.6</v>
       </c>
       <c r="G16" t="n">
-        <v>4.1</v>
+        <v>7.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6.56</v>
+        <v>16.25</v>
       </c>
       <c r="D17" t="n">
-        <v>0.62</v>
+        <v>1.5</v>
       </c>
       <c r="E17" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="F17" t="n">
-        <v>3.8</v>
+        <v>6.1</v>
       </c>
       <c r="G17" t="n">
-        <v>3.6</v>
+        <v>6.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>14.93</v>
+        <v>23.17</v>
       </c>
       <c r="D18" t="n">
-        <v>2.21</v>
+        <v>1.89</v>
       </c>
       <c r="E18" t="n">
-        <v>4.6</v>
+        <v>6.1</v>
       </c>
       <c r="F18" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="G18" t="n">
-        <v>3.5</v>
+        <v>6.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18.48</v>
+        <v>20.93</v>
       </c>
       <c r="D19" t="n">
         <v>1.72</v>
       </c>
       <c r="E19" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="F19" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="G19" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="20">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>21.79</v>
+        <v>21.97</v>
       </c>
       <c r="D20" t="n">
-        <v>1.97</v>
+        <v>1.99</v>
       </c>
       <c r="E20" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="F20" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="G20" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="21">
@@ -1056,22 +1056,22 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>18.16</v>
+        <v>18.54</v>
       </c>
       <c r="D21" t="n">
-        <v>3.14</v>
+        <v>3.21</v>
       </c>
       <c r="E21" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="F21" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="G21" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="22">
@@ -1086,22 +1086,22 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>18.83</v>
+        <v>18.9</v>
       </c>
       <c r="D22" t="n">
-        <v>1.57</v>
+        <v>1.58</v>
       </c>
       <c r="E22" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="F22" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="G22" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="23">
@@ -1116,22 +1116,22 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>15.76</v>
+        <v>15.89</v>
       </c>
       <c r="D23" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="E23" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="F23" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="G23" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="24">
@@ -1146,262 +1146,262 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.1</v>
+        <v>22.14</v>
       </c>
       <c r="D24" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="E24" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="F24" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="G24" t="n">
-        <v>3.1</v>
+        <v>6.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20.68</v>
+        <v>10.64</v>
       </c>
       <c r="D25" t="n">
-        <v>1.7</v>
+        <v>0.68</v>
       </c>
       <c r="E25" t="n">
-        <v>3.1</v>
+        <v>7.6</v>
       </c>
       <c r="F25" t="n">
-        <v>3.1</v>
+        <v>4.5</v>
       </c>
       <c r="G25" t="n">
-        <v>3.1</v>
+        <v>5.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>14.17</v>
+        <v>6.61</v>
       </c>
       <c r="D26" t="n">
-        <v>1.15</v>
+        <v>0.62</v>
       </c>
       <c r="E26" t="n">
-        <v>3.1</v>
+        <v>6.8</v>
       </c>
       <c r="F26" t="n">
-        <v>3.1</v>
+        <v>4.5</v>
       </c>
       <c r="G26" t="n">
-        <v>3.1</v>
+        <v>5.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>30.29</v>
+        <v>46.14</v>
       </c>
       <c r="D27" t="n">
-        <v>2.3</v>
+        <v>3.78</v>
       </c>
       <c r="E27" t="n">
-        <v>3.1</v>
+        <v>9.1</v>
       </c>
       <c r="F27" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="G27" t="n">
-        <v>3.1</v>
+        <v>4.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22.98</v>
+        <v>12.01</v>
       </c>
       <c r="D28" t="n">
-        <v>1.88</v>
+        <v>1.13</v>
       </c>
       <c r="E28" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="F28" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="G28" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>16.04</v>
+        <v>18.47</v>
       </c>
       <c r="D29" t="n">
-        <v>1.48</v>
+        <v>1.72</v>
       </c>
       <c r="E29" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="F29" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="G29" t="n">
         <v>3.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>12.01</v>
+        <v>14.13</v>
       </c>
       <c r="D30" t="n">
-        <v>1.13</v>
+        <v>1.15</v>
       </c>
       <c r="E30" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="F30" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="G30" t="n">
         <v>3.1</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>21.28</v>
+        <v>30.23</v>
       </c>
       <c r="D31" t="n">
-        <v>1.56</v>
+        <v>2.3</v>
       </c>
       <c r="E31" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="F31" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="G31" t="n">
         <v>3.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>26.07</v>
+        <v>21.07</v>
       </c>
       <c r="D32" t="n">
-        <v>2.18</v>
+        <v>1.55</v>
       </c>
       <c r="E32" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="F32" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="G32" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Jun 30 12:01:01 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>88.91</v>
+        <v>92.72</v>
       </c>
       <c r="D2" t="n">
-        <v>9.33</v>
+        <v>9.73</v>
       </c>
       <c r="E2" t="n">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>47.71</v>
+        <v>47.86</v>
       </c>
       <c r="D3" t="n">
         <v>2.65</v>
       </c>
       <c r="E3" t="n">
-        <v>93.90000000000001</v>
+        <v>94</v>
       </c>
       <c r="F3" t="n">
-        <v>93.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="G3" t="n">
-        <v>93.90000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +546,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>43.12</v>
+        <v>44.28</v>
       </c>
       <c r="D4" t="n">
-        <v>3.65</v>
+        <v>3.75</v>
       </c>
       <c r="E4" t="n">
-        <v>78.8</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>78</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>78.40000000000001</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="5">
@@ -576,22 +576,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>33.07</v>
+        <v>34.08</v>
       </c>
       <c r="D5" t="n">
-        <v>3.13</v>
+        <v>3.22</v>
       </c>
       <c r="E5" t="n">
-        <v>66.7</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>61.4</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="6">
@@ -606,22 +606,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.15</v>
+        <v>10.07</v>
       </c>
       <c r="D6" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="E6" t="n">
-        <v>56.8</v>
+        <v>49.3</v>
       </c>
       <c r="F6" t="n">
-        <v>54.5</v>
+        <v>44.8</v>
       </c>
       <c r="G6" t="n">
-        <v>55.7</v>
+        <v>47</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="7">
@@ -636,22 +636,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>27.63</v>
+        <v>27.25</v>
       </c>
       <c r="D7" t="n">
-        <v>2.54</v>
+        <v>2.5</v>
       </c>
       <c r="E7" t="n">
-        <v>45.5</v>
+        <v>43.3</v>
       </c>
       <c r="F7" t="n">
-        <v>42.4</v>
+        <v>39.6</v>
       </c>
       <c r="G7" t="n">
-        <v>43.9</v>
+        <v>41.4</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="8">
@@ -666,292 +666,292 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28.04</v>
+        <v>28.13</v>
       </c>
       <c r="D8" t="n">
-        <v>2.56</v>
+        <v>2.57</v>
       </c>
       <c r="E8" t="n">
-        <v>37.9</v>
+        <v>43.3</v>
       </c>
       <c r="F8" t="n">
-        <v>37.9</v>
+        <v>38.8</v>
       </c>
       <c r="G8" t="n">
-        <v>37.9</v>
+        <v>41</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>33.96</v>
+        <v>61.16</v>
       </c>
       <c r="D9" t="n">
-        <v>3.67</v>
+        <v>3.93</v>
       </c>
       <c r="E9" t="n">
-        <v>15.2</v>
+        <v>40.3</v>
       </c>
       <c r="F9" t="n">
-        <v>15.2</v>
+        <v>36.6</v>
       </c>
       <c r="G9" t="n">
-        <v>15.2</v>
+        <v>38.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>111.22</v>
+        <v>34.68</v>
       </c>
       <c r="D10" t="n">
-        <v>4.18</v>
+        <v>3.75</v>
       </c>
       <c r="E10" t="n">
-        <v>12.1</v>
+        <v>23.9</v>
       </c>
       <c r="F10" t="n">
-        <v>12.1</v>
+        <v>21.6</v>
       </c>
       <c r="G10" t="n">
-        <v>12.1</v>
+        <v>22.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>21.14</v>
+        <v>47.78</v>
       </c>
       <c r="D11" t="n">
-        <v>3.5</v>
+        <v>3.91</v>
       </c>
       <c r="E11" t="n">
-        <v>16.7</v>
+        <v>26.9</v>
       </c>
       <c r="F11" t="n">
-        <v>9.800000000000001</v>
+        <v>18.7</v>
       </c>
       <c r="G11" t="n">
-        <v>11.9</v>
+        <v>21.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>26.19</v>
+        <v>114.55</v>
       </c>
       <c r="D12" t="n">
-        <v>1.94</v>
+        <v>4.29</v>
       </c>
       <c r="E12" t="n">
-        <v>10.6</v>
+        <v>20.9</v>
       </c>
       <c r="F12" t="n">
-        <v>9.800000000000001</v>
+        <v>20.9</v>
       </c>
       <c r="G12" t="n">
-        <v>10.1</v>
+        <v>20.9</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>26.99</v>
+        <v>15.05</v>
       </c>
       <c r="D13" t="n">
-        <v>2.26</v>
+        <v>2.23</v>
       </c>
       <c r="E13" t="n">
-        <v>9.1</v>
+        <v>11.9</v>
       </c>
       <c r="F13" t="n">
-        <v>9.1</v>
+        <v>10.4</v>
       </c>
       <c r="G13" t="n">
-        <v>9.1</v>
+        <v>10.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10.13</v>
+        <v>20.98</v>
       </c>
       <c r="D14" t="n">
-        <v>0.92</v>
+        <v>3.47</v>
       </c>
       <c r="E14" t="n">
-        <v>6.1</v>
+        <v>11.9</v>
       </c>
       <c r="F14" t="n">
-        <v>9.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="G14" t="n">
-        <v>8.699999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>59.22</v>
+        <v>27.02</v>
       </c>
       <c r="D15" t="n">
-        <v>3.81</v>
+        <v>2.26</v>
       </c>
       <c r="E15" t="n">
-        <v>8.300000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="F15" t="n">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>8.300000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15.01</v>
+        <v>10.23</v>
       </c>
       <c r="D16" t="n">
-        <v>2.22</v>
+        <v>0.92</v>
       </c>
       <c r="E16" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="F16" t="n">
-        <v>7.6</v>
+        <v>10.4</v>
       </c>
       <c r="G16" t="n">
-        <v>7.6</v>
+        <v>9.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>16.25</v>
+        <v>25.85</v>
       </c>
       <c r="D17" t="n">
-        <v>1.5</v>
+        <v>1.91</v>
       </c>
       <c r="E17" t="n">
-        <v>6.1</v>
+        <v>10.4</v>
       </c>
       <c r="F17" t="n">
-        <v>6.1</v>
+        <v>9</v>
       </c>
       <c r="G17" t="n">
-        <v>6.1</v>
+        <v>9.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="18">
@@ -966,430 +966,430 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23.17</v>
+        <v>23.26</v>
       </c>
       <c r="D18" t="n">
-        <v>1.89</v>
+        <v>1.9</v>
       </c>
       <c r="E18" t="n">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
       <c r="F18" t="n">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
       <c r="G18" t="n">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20.93</v>
+        <v>22.42</v>
       </c>
       <c r="D19" t="n">
-        <v>1.72</v>
+        <v>2.07</v>
       </c>
       <c r="E19" t="n">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
       <c r="F19" t="n">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
       <c r="G19" t="n">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>21.97</v>
+        <v>20.97</v>
       </c>
       <c r="D20" t="n">
-        <v>1.99</v>
+        <v>1.72</v>
       </c>
       <c r="E20" t="n">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
       <c r="F20" t="n">
-        <v>6.1</v>
+        <v>6.7</v>
       </c>
       <c r="G20" t="n">
-        <v>6.1</v>
+        <v>6.9</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>18.54</v>
+        <v>15.8</v>
       </c>
       <c r="D21" t="n">
-        <v>3.21</v>
+        <v>0.88</v>
       </c>
       <c r="E21" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="F21" t="n">
-        <v>6.1</v>
+        <v>6.7</v>
       </c>
       <c r="G21" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>18.9</v>
+        <v>18.35</v>
       </c>
       <c r="D22" t="n">
-        <v>1.58</v>
+        <v>3.17</v>
       </c>
       <c r="E22" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="G22" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>15.89</v>
+        <v>21.95</v>
       </c>
       <c r="D23" t="n">
-        <v>0.88</v>
+        <v>1.98</v>
       </c>
       <c r="E23" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="G23" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.14</v>
+        <v>10.56</v>
       </c>
       <c r="D24" t="n">
-        <v>2.05</v>
+        <v>0.68</v>
       </c>
       <c r="E24" t="n">
-        <v>6.1</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>6.1</v>
+        <v>5.2</v>
       </c>
       <c r="G24" t="n">
-        <v>6.1</v>
+        <v>4.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10.64</v>
+        <v>18.76</v>
       </c>
       <c r="D25" t="n">
-        <v>0.68</v>
+        <v>1.57</v>
       </c>
       <c r="E25" t="n">
-        <v>7.6</v>
+        <v>1.5</v>
       </c>
       <c r="F25" t="n">
-        <v>4.5</v>
+        <v>3.7</v>
       </c>
       <c r="G25" t="n">
-        <v>5.5</v>
+        <v>3.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6.61</v>
+        <v>21.14</v>
       </c>
       <c r="D26" t="n">
-        <v>0.62</v>
+        <v>1.55</v>
       </c>
       <c r="E26" t="n">
-        <v>6.8</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="G26" t="n">
-        <v>5.2</v>
+        <v>2.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>46.14</v>
+        <v>18.32</v>
       </c>
       <c r="D27" t="n">
-        <v>3.78</v>
+        <v>1.71</v>
       </c>
       <c r="E27" t="n">
-        <v>9.1</v>
+        <v>1.5</v>
       </c>
       <c r="F27" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="G27" t="n">
-        <v>4.8</v>
+        <v>1.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>12.01</v>
+        <v>13.89</v>
       </c>
       <c r="D28" t="n">
         <v>1.13</v>
       </c>
       <c r="E28" t="n">
-        <v>3.8</v>
+        <v>1.5</v>
       </c>
       <c r="F28" t="n">
-        <v>3.8</v>
+        <v>1.5</v>
       </c>
       <c r="G28" t="n">
-        <v>3.8</v>
+        <v>1.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.47</v>
+        <v>6.46</v>
       </c>
       <c r="D29" t="n">
-        <v>1.72</v>
+        <v>0.61</v>
       </c>
       <c r="E29" t="n">
         <v>1.5</v>
       </c>
       <c r="F29" t="n">
-        <v>3.8</v>
+        <v>1.5</v>
       </c>
       <c r="G29" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>14.13</v>
+        <v>30.15</v>
       </c>
       <c r="D30" t="n">
-        <v>1.15</v>
+        <v>2.29</v>
       </c>
       <c r="E30" t="n">
         <v>1.5</v>
       </c>
       <c r="F30" t="n">
-        <v>3.8</v>
+        <v>1.5</v>
       </c>
       <c r="G30" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>30.23</v>
+        <v>11.74</v>
       </c>
       <c r="D31" t="n">
-        <v>2.3</v>
+        <v>1.11</v>
       </c>
       <c r="E31" t="n">
         <v>1.5</v>
       </c>
       <c r="F31" t="n">
-        <v>3.8</v>
+        <v>1.5</v>
       </c>
       <c r="G31" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>21.07</v>
+        <v>15.78</v>
       </c>
       <c r="D32" t="n">
-        <v>1.55</v>
+        <v>1.46</v>
       </c>
       <c r="E32" t="n">
         <v>1.5</v>
@@ -1401,7 +1401,7 @@
         <v>1.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Jul  1 12:22:26 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>92.72</v>
+        <v>91.08</v>
       </c>
       <c r="D2" t="n">
-        <v>9.73</v>
+        <v>9.56</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>98.5</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>98.5</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>98.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="3">
@@ -516,232 +516,232 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>47.86</v>
+        <v>47.23</v>
       </c>
       <c r="D3" t="n">
-        <v>2.65</v>
+        <v>2.62</v>
       </c>
       <c r="E3" t="n">
-        <v>94</v>
+        <v>91.2</v>
       </c>
       <c r="F3" t="n">
-        <v>93.3</v>
+        <v>91.2</v>
       </c>
       <c r="G3" t="n">
-        <v>93.7</v>
+        <v>91.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>44.28</v>
+        <v>10.62</v>
       </c>
       <c r="D4" t="n">
-        <v>3.75</v>
+        <v>1.29</v>
       </c>
       <c r="E4" t="n">
-        <v>89.59999999999999</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>89.59999999999999</v>
+        <v>88.2</v>
       </c>
       <c r="G4" t="n">
-        <v>89.59999999999999</v>
+        <v>91.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>34.08</v>
+        <v>44.19</v>
       </c>
       <c r="D5" t="n">
-        <v>3.22</v>
+        <v>3.74</v>
       </c>
       <c r="E5" t="n">
-        <v>82.09999999999999</v>
+        <v>88.2</v>
       </c>
       <c r="F5" t="n">
-        <v>73.90000000000001</v>
+        <v>87.5</v>
       </c>
       <c r="G5" t="n">
-        <v>78</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.07</v>
+        <v>33.24</v>
       </c>
       <c r="D6" t="n">
-        <v>1.22</v>
+        <v>3.15</v>
       </c>
       <c r="E6" t="n">
-        <v>49.3</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>44.8</v>
+        <v>64.7</v>
       </c>
       <c r="G6" t="n">
-        <v>47</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>27.25</v>
+        <v>28.78</v>
       </c>
       <c r="D7" t="n">
-        <v>2.5</v>
+        <v>2.63</v>
       </c>
       <c r="E7" t="n">
-        <v>43.3</v>
+        <v>66.2</v>
       </c>
       <c r="F7" t="n">
-        <v>39.6</v>
+        <v>62.5</v>
       </c>
       <c r="G7" t="n">
-        <v>41.4</v>
+        <v>64.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28.13</v>
+        <v>123.16</v>
       </c>
       <c r="D8" t="n">
-        <v>2.57</v>
+        <v>4.62</v>
       </c>
       <c r="E8" t="n">
-        <v>43.3</v>
+        <v>60.3</v>
       </c>
       <c r="F8" t="n">
-        <v>38.8</v>
+        <v>58.8</v>
       </c>
       <c r="G8" t="n">
-        <v>41</v>
+        <v>59.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>61.16</v>
+        <v>28.26</v>
       </c>
       <c r="D9" t="n">
-        <v>3.93</v>
+        <v>2.6</v>
       </c>
       <c r="E9" t="n">
-        <v>40.3</v>
+        <v>54.4</v>
       </c>
       <c r="F9" t="n">
-        <v>36.6</v>
+        <v>52.2</v>
       </c>
       <c r="G9" t="n">
-        <v>38.4</v>
+        <v>53.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>34.68</v>
+        <v>61.66</v>
       </c>
       <c r="D10" t="n">
-        <v>3.75</v>
+        <v>3.96</v>
       </c>
       <c r="E10" t="n">
-        <v>23.9</v>
+        <v>48.5</v>
       </c>
       <c r="F10" t="n">
-        <v>21.6</v>
+        <v>47.8</v>
       </c>
       <c r="G10" t="n">
-        <v>22.3</v>
+        <v>48.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="11">
@@ -756,142 +756,142 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>47.78</v>
+        <v>48.44</v>
       </c>
       <c r="D11" t="n">
-        <v>3.91</v>
+        <v>3.97</v>
       </c>
       <c r="E11" t="n">
-        <v>26.9</v>
+        <v>39.7</v>
       </c>
       <c r="F11" t="n">
-        <v>18.7</v>
+        <v>33.8</v>
       </c>
       <c r="G11" t="n">
-        <v>21.1</v>
+        <v>36.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>114.55</v>
+        <v>26.99</v>
       </c>
       <c r="D12" t="n">
-        <v>4.29</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>20.9</v>
+        <v>29.4</v>
       </c>
       <c r="F12" t="n">
-        <v>20.9</v>
+        <v>22.1</v>
       </c>
       <c r="G12" t="n">
-        <v>20.9</v>
+        <v>24.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>15.05</v>
+        <v>34.11</v>
       </c>
       <c r="D13" t="n">
-        <v>2.23</v>
+        <v>3.68</v>
       </c>
       <c r="E13" t="n">
-        <v>11.9</v>
+        <v>16.2</v>
       </c>
       <c r="F13" t="n">
-        <v>10.4</v>
+        <v>16.2</v>
       </c>
       <c r="G13" t="n">
-        <v>10.9</v>
+        <v>16.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>20.98</v>
+        <v>10.73</v>
       </c>
       <c r="D14" t="n">
-        <v>3.47</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>11.9</v>
+        <v>13.2</v>
       </c>
       <c r="F14" t="n">
-        <v>9</v>
+        <v>16.9</v>
       </c>
       <c r="G14" t="n">
-        <v>9.9</v>
+        <v>15.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>27.02</v>
+        <v>31.06</v>
       </c>
       <c r="D15" t="n">
-        <v>2.26</v>
+        <v>2.36</v>
       </c>
       <c r="E15" t="n">
-        <v>10.4</v>
+        <v>20.6</v>
       </c>
       <c r="F15" t="n">
-        <v>9.699999999999999</v>
+        <v>13.2</v>
       </c>
       <c r="G15" t="n">
-        <v>9.9</v>
+        <v>15.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="16">
@@ -906,112 +906,112 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.23</v>
+        <v>10.47</v>
       </c>
       <c r="D16" t="n">
-        <v>0.92</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>7.5</v>
+        <v>11</v>
       </c>
       <c r="F16" t="n">
-        <v>10.4</v>
+        <v>16.2</v>
       </c>
       <c r="G16" t="n">
-        <v>9.6</v>
+        <v>14.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25.85</v>
+        <v>15.19</v>
       </c>
       <c r="D17" t="n">
-        <v>1.91</v>
+        <v>2.25</v>
       </c>
       <c r="E17" t="n">
-        <v>10.4</v>
+        <v>17.6</v>
       </c>
       <c r="F17" t="n">
-        <v>9</v>
+        <v>12.5</v>
       </c>
       <c r="G17" t="n">
-        <v>9.4</v>
+        <v>14</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23.26</v>
+        <v>27.63</v>
       </c>
       <c r="D18" t="n">
-        <v>1.9</v>
+        <v>2.31</v>
       </c>
       <c r="E18" t="n">
-        <v>7.5</v>
+        <v>13.2</v>
       </c>
       <c r="F18" t="n">
-        <v>7.5</v>
+        <v>13.2</v>
       </c>
       <c r="G18" t="n">
-        <v>7.5</v>
+        <v>13.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22.42</v>
+        <v>19.24</v>
       </c>
       <c r="D19" t="n">
-        <v>2.07</v>
+        <v>1.61</v>
       </c>
       <c r="E19" t="n">
-        <v>7.5</v>
+        <v>11.8</v>
       </c>
       <c r="F19" t="n">
-        <v>7.5</v>
+        <v>13.2</v>
       </c>
       <c r="G19" t="n">
-        <v>7.5</v>
+        <v>12.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="20">
@@ -1026,322 +1026,322 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>20.97</v>
+        <v>21.58</v>
       </c>
       <c r="D20" t="n">
-        <v>1.72</v>
+        <v>1.77</v>
       </c>
       <c r="E20" t="n">
-        <v>7.5</v>
+        <v>11.8</v>
       </c>
       <c r="F20" t="n">
-        <v>6.7</v>
+        <v>11</v>
       </c>
       <c r="G20" t="n">
-        <v>6.9</v>
+        <v>11.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>15.8</v>
+        <v>21</v>
       </c>
       <c r="D21" t="n">
-        <v>0.88</v>
+        <v>3.47</v>
       </c>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>13.2</v>
       </c>
       <c r="F21" t="n">
-        <v>6.7</v>
+        <v>9.6</v>
       </c>
       <c r="G21" t="n">
-        <v>6.5</v>
+        <v>10.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>18.35</v>
+        <v>22.28</v>
       </c>
       <c r="D22" t="n">
-        <v>3.17</v>
+        <v>2.02</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>10.3</v>
       </c>
       <c r="F22" t="n">
-        <v>6</v>
+        <v>10.3</v>
       </c>
       <c r="G22" t="n">
-        <v>6</v>
+        <v>10.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>21.95</v>
+        <v>18.61</v>
       </c>
       <c r="D23" t="n">
-        <v>1.98</v>
+        <v>1.73</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>10.3</v>
       </c>
       <c r="F23" t="n">
-        <v>6</v>
+        <v>9.6</v>
       </c>
       <c r="G23" t="n">
-        <v>6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10.56</v>
+        <v>16.17</v>
       </c>
       <c r="D24" t="n">
-        <v>0.68</v>
+        <v>0.9</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>5.2</v>
+        <v>9.6</v>
       </c>
       <c r="G24" t="n">
-        <v>4.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>18.76</v>
+        <v>21.47</v>
       </c>
       <c r="D25" t="n">
-        <v>1.57</v>
+        <v>1.58</v>
       </c>
       <c r="E25" t="n">
-        <v>1.5</v>
+        <v>10.3</v>
       </c>
       <c r="F25" t="n">
-        <v>3.7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G25" t="n">
-        <v>3.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>21.14</v>
+        <v>23.53</v>
       </c>
       <c r="D26" t="n">
-        <v>1.55</v>
+        <v>1.92</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F26" t="n">
-        <v>2.2</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G26" t="n">
-        <v>2.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18.32</v>
+        <v>22.68</v>
       </c>
       <c r="D27" t="n">
-        <v>1.71</v>
+        <v>2.09</v>
       </c>
       <c r="E27" t="n">
-        <v>1.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F27" t="n">
-        <v>1.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G27" t="n">
-        <v>1.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>13.89</v>
+        <v>18.55</v>
       </c>
       <c r="D28" t="n">
-        <v>1.13</v>
+        <v>3.21</v>
       </c>
       <c r="E28" t="n">
-        <v>1.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F28" t="n">
-        <v>1.5</v>
+        <v>8.1</v>
       </c>
       <c r="G28" t="n">
-        <v>1.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6.46</v>
+        <v>16.07</v>
       </c>
       <c r="D29" t="n">
-        <v>0.61</v>
+        <v>1.49</v>
       </c>
       <c r="E29" t="n">
-        <v>1.5</v>
+        <v>7.4</v>
       </c>
       <c r="F29" t="n">
-        <v>1.5</v>
+        <v>7.4</v>
       </c>
       <c r="G29" t="n">
-        <v>1.5</v>
+        <v>7.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>30.15</v>
+        <v>14.08</v>
       </c>
       <c r="D30" t="n">
-        <v>2.29</v>
+        <v>1.15</v>
       </c>
       <c r="E30" t="n">
-        <v>1.5</v>
+        <v>2.9</v>
       </c>
       <c r="F30" t="n">
-        <v>1.5</v>
+        <v>5.9</v>
       </c>
       <c r="G30" t="n">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="31">
@@ -1356,52 +1356,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>11.74</v>
+        <v>11.84</v>
       </c>
       <c r="D31" t="n">
         <v>1.11</v>
       </c>
       <c r="E31" t="n">
-        <v>1.5</v>
+        <v>2.9</v>
       </c>
       <c r="F31" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="G31" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>15.78</v>
+        <v>6.46</v>
       </c>
       <c r="D32" t="n">
-        <v>1.46</v>
+        <v>0.61</v>
       </c>
       <c r="E32" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="F32" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="G32" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Jul  2 11:56:49 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>91.08</v>
+        <v>84.58</v>
       </c>
       <c r="D2" t="n">
-        <v>9.56</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>98.5</v>
+        <v>87</v>
       </c>
       <c r="F2" t="n">
-        <v>98.5</v>
+        <v>87</v>
       </c>
       <c r="G2" t="n">
-        <v>98.5</v>
+        <v>87</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="3">
@@ -516,142 +516,142 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>47.23</v>
+        <v>45.18</v>
       </c>
       <c r="D3" t="n">
-        <v>2.62</v>
+        <v>2.5</v>
       </c>
       <c r="E3" t="n">
-        <v>91.2</v>
+        <v>87</v>
       </c>
       <c r="F3" t="n">
-        <v>91.2</v>
+        <v>87</v>
       </c>
       <c r="G3" t="n">
-        <v>91.2</v>
+        <v>87</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.62</v>
+        <v>43.17</v>
       </c>
       <c r="D4" t="n">
-        <v>1.29</v>
+        <v>3.65</v>
       </c>
       <c r="E4" t="n">
-        <v>94.09999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="F4" t="n">
-        <v>88.2</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>91.2</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>44.19</v>
+        <v>10.42</v>
       </c>
       <c r="D5" t="n">
-        <v>3.74</v>
+        <v>1.26</v>
       </c>
       <c r="E5" t="n">
-        <v>88.2</v>
+        <v>77.5</v>
       </c>
       <c r="F5" t="n">
-        <v>87.5</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>87.90000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>33.24</v>
+        <v>28.61</v>
       </c>
       <c r="D6" t="n">
-        <v>3.15</v>
+        <v>2.62</v>
       </c>
       <c r="E6" t="n">
-        <v>69.09999999999999</v>
+        <v>58.7</v>
       </c>
       <c r="F6" t="n">
-        <v>64.7</v>
+        <v>57.2</v>
       </c>
       <c r="G6" t="n">
-        <v>66.90000000000001</v>
+        <v>58</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.78</v>
+        <v>28.16</v>
       </c>
       <c r="D7" t="n">
-        <v>2.63</v>
+        <v>2.59</v>
       </c>
       <c r="E7" t="n">
-        <v>66.2</v>
+        <v>52.2</v>
       </c>
       <c r="F7" t="n">
-        <v>62.5</v>
+        <v>48.6</v>
       </c>
       <c r="G7" t="n">
-        <v>64.3</v>
+        <v>50.4</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="8">
@@ -666,712 +666,712 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>123.16</v>
+        <v>121.43</v>
       </c>
       <c r="D8" t="n">
-        <v>4.62</v>
+        <v>4.55</v>
       </c>
       <c r="E8" t="n">
-        <v>60.3</v>
+        <v>49.3</v>
       </c>
       <c r="F8" t="n">
-        <v>58.8</v>
+        <v>49.3</v>
       </c>
       <c r="G8" t="n">
-        <v>59.6</v>
+        <v>49.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28.26</v>
+        <v>31.71</v>
       </c>
       <c r="D9" t="n">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>54.4</v>
+        <v>40.6</v>
       </c>
       <c r="F9" t="n">
-        <v>52.2</v>
+        <v>40.6</v>
       </c>
       <c r="G9" t="n">
-        <v>53.3</v>
+        <v>40.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>61.66</v>
+        <v>19.59</v>
       </c>
       <c r="D10" t="n">
-        <v>3.96</v>
+        <v>1.63</v>
       </c>
       <c r="E10" t="n">
-        <v>48.5</v>
+        <v>34.8</v>
       </c>
       <c r="F10" t="n">
-        <v>47.8</v>
+        <v>22.5</v>
       </c>
       <c r="G10" t="n">
-        <v>48.2</v>
+        <v>26.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>48.44</v>
+        <v>27.11</v>
       </c>
       <c r="D11" t="n">
-        <v>3.97</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>39.7</v>
+        <v>30.4</v>
       </c>
       <c r="F11" t="n">
-        <v>33.8</v>
+        <v>22.5</v>
       </c>
       <c r="G11" t="n">
-        <v>36.8</v>
+        <v>24.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>26.99</v>
+        <v>60.31</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3.88</v>
       </c>
       <c r="E12" t="n">
-        <v>29.4</v>
+        <v>31.9</v>
       </c>
       <c r="F12" t="n">
-        <v>22.1</v>
+        <v>20.3</v>
       </c>
       <c r="G12" t="n">
-        <v>24.3</v>
+        <v>23.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>34.11</v>
+        <v>27.81</v>
       </c>
       <c r="D13" t="n">
-        <v>3.68</v>
+        <v>2.32</v>
       </c>
       <c r="E13" t="n">
-        <v>16.2</v>
+        <v>15.9</v>
       </c>
       <c r="F13" t="n">
-        <v>16.2</v>
+        <v>15.9</v>
       </c>
       <c r="G13" t="n">
-        <v>16.2</v>
+        <v>15.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10.73</v>
+        <v>47.08</v>
       </c>
       <c r="D14" t="n">
-        <v>0.6899999999999999</v>
+        <v>3.86</v>
       </c>
       <c r="E14" t="n">
-        <v>13.2</v>
+        <v>18.8</v>
       </c>
       <c r="F14" t="n">
-        <v>16.9</v>
+        <v>13.8</v>
       </c>
       <c r="G14" t="n">
-        <v>15.8</v>
+        <v>15.3</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>31.06</v>
+        <v>15.19</v>
       </c>
       <c r="D15" t="n">
-        <v>2.36</v>
+        <v>2.25</v>
       </c>
       <c r="E15" t="n">
-        <v>20.6</v>
+        <v>18.1</v>
       </c>
       <c r="F15" t="n">
-        <v>13.2</v>
+        <v>13</v>
       </c>
       <c r="G15" t="n">
-        <v>15.4</v>
+        <v>14.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.47</v>
+        <v>21.07</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9399999999999999</v>
+        <v>3.49</v>
       </c>
       <c r="E16" t="n">
-        <v>11</v>
+        <v>14.5</v>
       </c>
       <c r="F16" t="n">
-        <v>16.2</v>
+        <v>11.6</v>
       </c>
       <c r="G16" t="n">
-        <v>14.6</v>
+        <v>12.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>15.19</v>
+        <v>10.23</v>
       </c>
       <c r="D17" t="n">
-        <v>2.25</v>
+        <v>0.93</v>
       </c>
       <c r="E17" t="n">
-        <v>17.6</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G17" t="n">
         <v>12.5</v>
       </c>
-      <c r="G17" t="n">
-        <v>14</v>
-      </c>
       <c r="H17" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>27.63</v>
+        <v>23.6</v>
       </c>
       <c r="D18" t="n">
-        <v>2.31</v>
+        <v>1.93</v>
       </c>
       <c r="E18" t="n">
-        <v>13.2</v>
+        <v>11.6</v>
       </c>
       <c r="F18" t="n">
-        <v>13.2</v>
+        <v>11.6</v>
       </c>
       <c r="G18" t="n">
-        <v>13.2</v>
+        <v>11.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>19.24</v>
+        <v>16.36</v>
       </c>
       <c r="D19" t="n">
-        <v>1.61</v>
+        <v>1.52</v>
       </c>
       <c r="E19" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="F19" t="n">
-        <v>13.2</v>
+        <v>11.6</v>
       </c>
       <c r="G19" t="n">
-        <v>12.8</v>
+        <v>11.6</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>21.58</v>
+        <v>22.81</v>
       </c>
       <c r="D20" t="n">
-        <v>1.77</v>
+        <v>2.11</v>
       </c>
       <c r="E20" t="n">
-        <v>11.8</v>
+        <v>10.1</v>
       </c>
       <c r="F20" t="n">
-        <v>11</v>
+        <v>11.6</v>
       </c>
       <c r="G20" t="n">
         <v>11.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>21</v>
+        <v>30.74</v>
       </c>
       <c r="D21" t="n">
-        <v>3.47</v>
+        <v>2.34</v>
       </c>
       <c r="E21" t="n">
-        <v>13.2</v>
+        <v>13</v>
       </c>
       <c r="F21" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="G21" t="n">
-        <v>10.7</v>
+        <v>11</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22.28</v>
+        <v>16.31</v>
       </c>
       <c r="D22" t="n">
-        <v>2.02</v>
+        <v>0.9</v>
       </c>
       <c r="E22" t="n">
-        <v>10.3</v>
+        <v>11.6</v>
       </c>
       <c r="F22" t="n">
-        <v>10.3</v>
+        <v>10.1</v>
       </c>
       <c r="G22" t="n">
-        <v>10.3</v>
+        <v>10.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>18.61</v>
+        <v>21.46</v>
       </c>
       <c r="D23" t="n">
-        <v>1.73</v>
+        <v>1.76</v>
       </c>
       <c r="E23" t="n">
-        <v>10.3</v>
+        <v>10.1</v>
       </c>
       <c r="F23" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="G23" t="n">
-        <v>9.800000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>16.17</v>
+        <v>22.12</v>
       </c>
       <c r="D24" t="n">
-        <v>0.9</v>
+        <v>2</v>
       </c>
       <c r="E24" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>9.6</v>
+        <v>9.4</v>
       </c>
       <c r="G24" t="n">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21.47</v>
+        <v>18.56</v>
       </c>
       <c r="D25" t="n">
-        <v>1.58</v>
+        <v>3.21</v>
       </c>
       <c r="E25" t="n">
-        <v>10.3</v>
+        <v>10.1</v>
       </c>
       <c r="F25" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G25" t="n">
-        <v>9.300000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>23.53</v>
+        <v>21.35</v>
       </c>
       <c r="D26" t="n">
-        <v>1.92</v>
+        <v>1.57</v>
       </c>
       <c r="E26" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F26" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.68</v>
+        <v>10.61</v>
       </c>
       <c r="D27" t="n">
-        <v>2.09</v>
+        <v>0.68</v>
       </c>
       <c r="E27" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F27" t="n">
-        <v>8.800000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="G27" t="n">
-        <v>8.800000000000001</v>
+        <v>6.7</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18.55</v>
+        <v>14.15</v>
       </c>
       <c r="D28" t="n">
-        <v>3.21</v>
+        <v>1.15</v>
       </c>
       <c r="E28" t="n">
-        <v>8.800000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="F28" t="n">
-        <v>8.1</v>
+        <v>6.5</v>
       </c>
       <c r="G28" t="n">
-        <v>8.300000000000001</v>
+        <v>6.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>16.07</v>
+        <v>18.48</v>
       </c>
       <c r="D29" t="n">
-        <v>1.49</v>
+        <v>1.72</v>
       </c>
       <c r="E29" t="n">
-        <v>7.4</v>
+        <v>6.5</v>
       </c>
       <c r="F29" t="n">
-        <v>7.4</v>
+        <v>5.8</v>
       </c>
       <c r="G29" t="n">
-        <v>7.4</v>
+        <v>6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>14.08</v>
+        <v>11.87</v>
       </c>
       <c r="D30" t="n">
-        <v>1.15</v>
+        <v>1.12</v>
       </c>
       <c r="E30" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
       <c r="F30" t="n">
-        <v>5.9</v>
+        <v>4.3</v>
       </c>
       <c r="G30" t="n">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>11.84</v>
+        <v>33.28</v>
       </c>
       <c r="D31" t="n">
-        <v>1.11</v>
+        <v>3.59</v>
       </c>
       <c r="E31" t="n">
         <v>2.9</v>
       </c>
       <c r="F31" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="G31" t="n">
-        <v>2.4</v>
+        <v>3.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6.46</v>
+        <v>6.47</v>
       </c>
       <c r="D32" t="n">
         <v>0.61</v>
       </c>
       <c r="E32" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="F32" t="n">
-        <v>2.2</v>
+        <v>2.9</v>
       </c>
       <c r="G32" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Jul  3 11:55:58 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,91 +477,91 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>84.58</v>
+        <v>46.41</v>
       </c>
       <c r="D2" t="n">
-        <v>8.869999999999999</v>
+        <v>2.58</v>
       </c>
       <c r="E2" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F2" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="G2" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>45.18</v>
+        <v>44.29</v>
       </c>
       <c r="D3" t="n">
-        <v>2.5</v>
+        <v>3.75</v>
       </c>
       <c r="E3" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F3" t="n">
-        <v>87</v>
+        <v>89.3</v>
       </c>
       <c r="G3" t="n">
-        <v>87</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>43.17</v>
+        <v>84.05</v>
       </c>
       <c r="D4" t="n">
-        <v>3.65</v>
+        <v>8.82</v>
       </c>
       <c r="E4" t="n">
-        <v>76.8</v>
+        <v>85.7</v>
       </c>
       <c r="F4" t="n">
-        <v>75.40000000000001</v>
+        <v>85.7</v>
       </c>
       <c r="G4" t="n">
-        <v>76.09999999999999</v>
+        <v>85.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="5">
@@ -576,82 +576,82 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10.42</v>
+        <v>10.47</v>
       </c>
       <c r="D5" t="n">
-        <v>1.26</v>
+        <v>1.27</v>
       </c>
       <c r="E5" t="n">
-        <v>77.5</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>65.90000000000001</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>71.7</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28.61</v>
+        <v>28.71</v>
       </c>
       <c r="D6" t="n">
-        <v>2.62</v>
+        <v>2.64</v>
       </c>
       <c r="E6" t="n">
-        <v>58.7</v>
+        <v>64.3</v>
       </c>
       <c r="F6" t="n">
-        <v>57.2</v>
+        <v>65</v>
       </c>
       <c r="G6" t="n">
-        <v>58</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.16</v>
+        <v>62.49</v>
       </c>
       <c r="D7" t="n">
-        <v>2.59</v>
+        <v>4.02</v>
       </c>
       <c r="E7" t="n">
-        <v>52.2</v>
+        <v>51.4</v>
       </c>
       <c r="F7" t="n">
-        <v>48.6</v>
+        <v>51.4</v>
       </c>
       <c r="G7" t="n">
-        <v>50.4</v>
+        <v>51.4</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="8">
@@ -666,232 +666,232 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>121.43</v>
+        <v>120.43</v>
       </c>
       <c r="D8" t="n">
-        <v>4.55</v>
+        <v>4.52</v>
       </c>
       <c r="E8" t="n">
-        <v>49.3</v>
+        <v>42.9</v>
       </c>
       <c r="F8" t="n">
-        <v>49.3</v>
+        <v>45.7</v>
       </c>
       <c r="G8" t="n">
-        <v>49.3</v>
+        <v>44.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>31.71</v>
+        <v>19.87</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>1.66</v>
       </c>
       <c r="E9" t="n">
-        <v>40.6</v>
+        <v>45</v>
       </c>
       <c r="F9" t="n">
-        <v>40.6</v>
+        <v>31.4</v>
       </c>
       <c r="G9" t="n">
-        <v>40.6</v>
+        <v>38.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.59</v>
+        <v>31.57</v>
       </c>
       <c r="D10" t="n">
-        <v>1.63</v>
+        <v>2.99</v>
       </c>
       <c r="E10" t="n">
-        <v>34.8</v>
+        <v>37.9</v>
       </c>
       <c r="F10" t="n">
-        <v>22.5</v>
+        <v>37.9</v>
       </c>
       <c r="G10" t="n">
-        <v>26.2</v>
+        <v>37.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.11</v>
+        <v>28.01</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>2.56</v>
       </c>
       <c r="E11" t="n">
-        <v>30.4</v>
+        <v>35.7</v>
       </c>
       <c r="F11" t="n">
-        <v>22.5</v>
+        <v>36.4</v>
       </c>
       <c r="G11" t="n">
-        <v>24.9</v>
+        <v>36.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>60.31</v>
+        <v>28.19</v>
       </c>
       <c r="D12" t="n">
-        <v>3.88</v>
+        <v>2.36</v>
       </c>
       <c r="E12" t="n">
-        <v>31.9</v>
+        <v>30</v>
       </c>
       <c r="F12" t="n">
-        <v>20.3</v>
+        <v>25</v>
       </c>
       <c r="G12" t="n">
-        <v>23.8</v>
+        <v>26.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>27.81</v>
+        <v>15.51</v>
       </c>
       <c r="D13" t="n">
-        <v>2.32</v>
+        <v>2.29</v>
       </c>
       <c r="E13" t="n">
-        <v>15.9</v>
+        <v>30</v>
       </c>
       <c r="F13" t="n">
-        <v>15.9</v>
+        <v>22.9</v>
       </c>
       <c r="G13" t="n">
-        <v>15.9</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>47.08</v>
+        <v>27.09</v>
       </c>
       <c r="D14" t="n">
-        <v>3.86</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>18.8</v>
+        <v>30</v>
       </c>
       <c r="F14" t="n">
-        <v>13.8</v>
+        <v>22.9</v>
       </c>
       <c r="G14" t="n">
-        <v>15.3</v>
+        <v>25</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>15.19</v>
+        <v>47.33</v>
       </c>
       <c r="D15" t="n">
-        <v>2.25</v>
+        <v>3.88</v>
       </c>
       <c r="E15" t="n">
-        <v>18.1</v>
+        <v>20</v>
       </c>
       <c r="F15" t="n">
-        <v>13</v>
+        <v>17.1</v>
       </c>
       <c r="G15" t="n">
-        <v>14.6</v>
+        <v>18</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="16">
@@ -906,232 +906,232 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>21.07</v>
+        <v>21.3</v>
       </c>
       <c r="D16" t="n">
-        <v>3.49</v>
+        <v>3.52</v>
       </c>
       <c r="E16" t="n">
-        <v>14.5</v>
+        <v>21.4</v>
       </c>
       <c r="F16" t="n">
-        <v>11.6</v>
+        <v>16.4</v>
       </c>
       <c r="G16" t="n">
-        <v>12.5</v>
+        <v>17.9</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.23</v>
+        <v>23.85</v>
       </c>
       <c r="D17" t="n">
-        <v>0.93</v>
+        <v>2.2</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>18.6</v>
       </c>
       <c r="F17" t="n">
-        <v>14.5</v>
+        <v>16.4</v>
       </c>
       <c r="G17" t="n">
-        <v>12.5</v>
+        <v>17.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23.6</v>
+        <v>10.7</v>
       </c>
       <c r="D18" t="n">
-        <v>1.93</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>11.6</v>
+        <v>12.1</v>
       </c>
       <c r="F18" t="n">
-        <v>11.6</v>
+        <v>18.6</v>
       </c>
       <c r="G18" t="n">
-        <v>11.6</v>
+        <v>16.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>16.36</v>
+        <v>10.45</v>
       </c>
       <c r="D19" t="n">
-        <v>1.52</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="F19" t="n">
-        <v>11.6</v>
+        <v>17.9</v>
       </c>
       <c r="G19" t="n">
-        <v>11.6</v>
+        <v>15.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>22.81</v>
+        <v>21.7</v>
       </c>
       <c r="D20" t="n">
-        <v>2.11</v>
+        <v>1.59</v>
       </c>
       <c r="E20" t="n">
-        <v>10.1</v>
+        <v>17.1</v>
       </c>
       <c r="F20" t="n">
-        <v>11.6</v>
+        <v>12.9</v>
       </c>
       <c r="G20" t="n">
-        <v>11.2</v>
+        <v>14.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>30.74</v>
+        <v>14.32</v>
       </c>
       <c r="D21" t="n">
-        <v>2.34</v>
+        <v>1.17</v>
       </c>
       <c r="E21" t="n">
-        <v>13</v>
+        <v>11.4</v>
       </c>
       <c r="F21" t="n">
-        <v>10.1</v>
+        <v>14.3</v>
       </c>
       <c r="G21" t="n">
-        <v>11</v>
+        <v>13.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>16.31</v>
+        <v>21.58</v>
       </c>
       <c r="D22" t="n">
-        <v>0.9</v>
+        <v>1.77</v>
       </c>
       <c r="E22" t="n">
-        <v>11.6</v>
+        <v>13.6</v>
       </c>
       <c r="F22" t="n">
-        <v>10.1</v>
+        <v>12.9</v>
       </c>
       <c r="G22" t="n">
-        <v>10.6</v>
+        <v>13.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>21.46</v>
+        <v>16.44</v>
       </c>
       <c r="D23" t="n">
-        <v>1.76</v>
+        <v>1.52</v>
       </c>
       <c r="E23" t="n">
-        <v>10.1</v>
+        <v>12.9</v>
       </c>
       <c r="F23" t="n">
-        <v>10.1</v>
+        <v>12.1</v>
       </c>
       <c r="G23" t="n">
-        <v>10.1</v>
+        <v>12.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="24">
@@ -1146,202 +1146,202 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.12</v>
+        <v>22.29</v>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>2.02</v>
       </c>
       <c r="E24" t="n">
-        <v>8.699999999999999</v>
+        <v>12.9</v>
       </c>
       <c r="F24" t="n">
-        <v>9.4</v>
+        <v>12.1</v>
       </c>
       <c r="G24" t="n">
-        <v>9.199999999999999</v>
+        <v>12.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>18.56</v>
+        <v>12.15</v>
       </c>
       <c r="D25" t="n">
-        <v>3.21</v>
+        <v>1.14</v>
       </c>
       <c r="E25" t="n">
-        <v>10.1</v>
+        <v>11.4</v>
       </c>
       <c r="F25" t="n">
-        <v>8.699999999999999</v>
+        <v>12.1</v>
       </c>
       <c r="G25" t="n">
-        <v>9.1</v>
+        <v>11.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>21.35</v>
+        <v>18.53</v>
       </c>
       <c r="D26" t="n">
-        <v>1.57</v>
+        <v>1.73</v>
       </c>
       <c r="E26" t="n">
-        <v>8.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>8.699999999999999</v>
+        <v>11.4</v>
       </c>
       <c r="G26" t="n">
-        <v>8.699999999999999</v>
+        <v>11</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>10.61</v>
+        <v>16.27</v>
       </c>
       <c r="D27" t="n">
-        <v>0.68</v>
+        <v>0.9</v>
       </c>
       <c r="E27" t="n">
-        <v>8.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="F27" t="n">
-        <v>5.8</v>
+        <v>10.7</v>
       </c>
       <c r="G27" t="n">
-        <v>6.7</v>
+        <v>10.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>14.15</v>
+        <v>30.73</v>
       </c>
       <c r="D28" t="n">
-        <v>1.15</v>
+        <v>2.33</v>
       </c>
       <c r="E28" t="n">
-        <v>5.8</v>
+        <v>12.1</v>
       </c>
       <c r="F28" t="n">
-        <v>6.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>6.3</v>
+        <v>10.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.48</v>
+        <v>18.56</v>
       </c>
       <c r="D29" t="n">
-        <v>1.72</v>
+        <v>3.21</v>
       </c>
       <c r="E29" t="n">
-        <v>6.5</v>
+        <v>10.7</v>
       </c>
       <c r="F29" t="n">
-        <v>5.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G29" t="n">
-        <v>6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>11.87</v>
+        <v>23.36</v>
       </c>
       <c r="D30" t="n">
-        <v>1.12</v>
+        <v>1.91</v>
       </c>
       <c r="E30" t="n">
-        <v>4.3</v>
+        <v>8.6</v>
       </c>
       <c r="F30" t="n">
-        <v>4.3</v>
+        <v>8.6</v>
       </c>
       <c r="G30" t="n">
-        <v>4.3</v>
+        <v>8.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>33.28</v>
+        <v>33.54</v>
       </c>
       <c r="D31" t="n">
-        <v>3.59</v>
+        <v>3.62</v>
       </c>
       <c r="E31" t="n">
-        <v>2.9</v>
+        <v>7.1</v>
       </c>
       <c r="F31" t="n">
-        <v>3.6</v>
+        <v>7.1</v>
       </c>
       <c r="G31" t="n">
-        <v>3.4</v>
+        <v>7.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6.47</v>
+        <v>6.45</v>
       </c>
       <c r="D32" t="n">
         <v>0.61</v>
       </c>
       <c r="E32" t="n">
-        <v>4.3</v>
+        <v>1.4</v>
       </c>
       <c r="F32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G32" t="n">
         <v>2.9</v>
       </c>
-      <c r="G32" t="n">
-        <v>3.3</v>
-      </c>
       <c r="H32" s="2" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Jul  4 11:12:20 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.58</v>
       </c>
       <c r="E2" t="n">
-        <v>90</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>90</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>90</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.75</v>
       </c>
       <c r="E3" t="n">
-        <v>90</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>89.3</v>
+        <v>88.7</v>
       </c>
       <c r="G3" t="n">
-        <v>89.59999999999999</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>8.82</v>
       </c>
       <c r="E4" t="n">
-        <v>85.7</v>
+        <v>85.2</v>
       </c>
       <c r="F4" t="n">
-        <v>85.7</v>
+        <v>85.2</v>
       </c>
       <c r="G4" t="n">
-        <v>85.7</v>
+        <v>85.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>1.27</v>
       </c>
       <c r="E5" t="n">
-        <v>78.59999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="F5" t="n">
-        <v>68.59999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="G5" t="n">
-        <v>73.59999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.64</v>
       </c>
       <c r="E6" t="n">
-        <v>64.3</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>65</v>
+        <v>64.8</v>
       </c>
       <c r="G6" t="n">
-        <v>64.59999999999999</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         <v>51.4</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>4.52</v>
       </c>
       <c r="E8" t="n">
-        <v>42.9</v>
+        <v>43</v>
       </c>
       <c r="F8" t="n">
-        <v>45.7</v>
+        <v>45.8</v>
       </c>
       <c r="G8" t="n">
-        <v>44.3</v>
+        <v>44.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.66</v>
       </c>
       <c r="E9" t="n">
-        <v>45</v>
+        <v>45.1</v>
       </c>
       <c r="F9" t="n">
-        <v>31.4</v>
+        <v>31.7</v>
       </c>
       <c r="G9" t="n">
-        <v>38.2</v>
+        <v>38.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.99</v>
       </c>
       <c r="E10" t="n">
-        <v>37.9</v>
+        <v>38</v>
       </c>
       <c r="F10" t="n">
-        <v>37.9</v>
+        <v>38</v>
       </c>
       <c r="G10" t="n">
-        <v>37.9</v>
+        <v>38</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.56</v>
       </c>
       <c r="E11" t="n">
-        <v>35.7</v>
+        <v>35.9</v>
       </c>
       <c r="F11" t="n">
-        <v>36.4</v>
+        <v>36.6</v>
       </c>
       <c r="G11" t="n">
-        <v>36.1</v>
+        <v>36.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.36</v>
       </c>
       <c r="E12" t="n">
-        <v>30</v>
+        <v>30.3</v>
       </c>
       <c r="F12" t="n">
-        <v>25</v>
+        <v>25.4</v>
       </c>
       <c r="G12" t="n">
-        <v>26.5</v>
+        <v>26.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>2.29</v>
       </c>
       <c r="E13" t="n">
-        <v>30</v>
+        <v>30.3</v>
       </c>
       <c r="F13" t="n">
-        <v>22.9</v>
+        <v>23.2</v>
       </c>
       <c r="G13" t="n">
-        <v>25</v>
+        <v>25.4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>30</v>
+        <v>30.3</v>
       </c>
       <c r="F14" t="n">
-        <v>22.9</v>
+        <v>23.2</v>
       </c>
       <c r="G14" t="n">
-        <v>25</v>
+        <v>25.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>3.88</v>
       </c>
       <c r="E15" t="n">
-        <v>20</v>
+        <v>20.4</v>
       </c>
       <c r="F15" t="n">
-        <v>17.1</v>
+        <v>17.6</v>
       </c>
       <c r="G15" t="n">
-        <v>18</v>
+        <v>18.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>3.52</v>
       </c>
       <c r="E16" t="n">
-        <v>21.4</v>
+        <v>21.8</v>
       </c>
       <c r="F16" t="n">
-        <v>16.4</v>
+        <v>16.9</v>
       </c>
       <c r="G16" t="n">
-        <v>17.9</v>
+        <v>18.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.2</v>
       </c>
       <c r="E17" t="n">
-        <v>18.6</v>
+        <v>19</v>
       </c>
       <c r="F17" t="n">
-        <v>16.4</v>
+        <v>16.9</v>
       </c>
       <c r="G17" t="n">
-        <v>17.1</v>
+        <v>17.5</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>12.1</v>
+        <v>12.7</v>
       </c>
       <c r="F18" t="n">
-        <v>18.6</v>
+        <v>19</v>
       </c>
       <c r="G18" t="n">
-        <v>16.6</v>
+        <v>17.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="F19" t="n">
-        <v>17.9</v>
+        <v>18.3</v>
       </c>
       <c r="G19" t="n">
-        <v>15.9</v>
+        <v>16.4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.59</v>
       </c>
       <c r="E20" t="n">
-        <v>17.1</v>
+        <v>17.6</v>
       </c>
       <c r="F20" t="n">
-        <v>12.9</v>
+        <v>13.4</v>
       </c>
       <c r="G20" t="n">
-        <v>14.1</v>
+        <v>14.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.17</v>
       </c>
       <c r="E21" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="F21" t="n">
-        <v>14.3</v>
+        <v>14.8</v>
       </c>
       <c r="G21" t="n">
-        <v>13.4</v>
+        <v>13.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.77</v>
       </c>
       <c r="E22" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G22" t="n">
         <v>13.6</v>
       </c>
-      <c r="F22" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="G22" t="n">
-        <v>13.1</v>
-      </c>
       <c r="H22" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.52</v>
       </c>
       <c r="E23" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="F23" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G23" t="n">
         <v>12.9</v>
       </c>
-      <c r="F23" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="G23" t="n">
-        <v>12.4</v>
-      </c>
       <c r="H23" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.02</v>
       </c>
       <c r="E24" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="F24" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G24" t="n">
         <v>12.9</v>
       </c>
-      <c r="F24" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="G24" t="n">
-        <v>12.4</v>
-      </c>
       <c r="H24" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.14</v>
       </c>
       <c r="E25" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="F25" t="n">
-        <v>12.1</v>
+        <v>12.7</v>
       </c>
       <c r="G25" t="n">
-        <v>11.9</v>
+        <v>12.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>1.73</v>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>10.6</v>
       </c>
       <c r="F26" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="G26" t="n">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>0.9</v>
       </c>
       <c r="E27" t="n">
-        <v>10</v>
+        <v>10.6</v>
       </c>
       <c r="F27" t="n">
-        <v>10.7</v>
+        <v>11.3</v>
       </c>
       <c r="G27" t="n">
-        <v>10.5</v>
+        <v>11.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.33</v>
       </c>
       <c r="E28" t="n">
-        <v>12.1</v>
+        <v>12.7</v>
       </c>
       <c r="F28" t="n">
-        <v>9.300000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="G28" t="n">
-        <v>10.1</v>
+        <v>10.7</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.21</v>
       </c>
       <c r="E29" t="n">
-        <v>10.7</v>
+        <v>11.3</v>
       </c>
       <c r="F29" t="n">
-        <v>9.300000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="G29" t="n">
-        <v>9.699999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.91</v>
       </c>
       <c r="E30" t="n">
-        <v>8.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F30" t="n">
-        <v>8.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G30" t="n">
-        <v>8.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.62</v>
       </c>
       <c r="E31" t="n">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="F31" t="n">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="G31" t="n">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>0.61</v>
       </c>
       <c r="E32" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="F32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G32" t="n">
         <v>3.6</v>
       </c>
-      <c r="G32" t="n">
-        <v>2.9</v>
-      </c>
       <c r="H32" s="2" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Jul  5 11:19:52 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>2.58</v>
       </c>
       <c r="E2" t="n">
-        <v>89.40000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>89.40000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>89.40000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.75</v>
       </c>
       <c r="E3" t="n">
-        <v>89.40000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>88.7</v>
+        <v>88.2</v>
       </c>
       <c r="G3" t="n">
-        <v>89.09999999999999</v>
+        <v>88.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>8.82</v>
       </c>
       <c r="E4" t="n">
-        <v>85.2</v>
+        <v>84.7</v>
       </c>
       <c r="F4" t="n">
-        <v>85.2</v>
+        <v>84.7</v>
       </c>
       <c r="G4" t="n">
-        <v>85.2</v>
+        <v>84.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>1.27</v>
       </c>
       <c r="E5" t="n">
-        <v>78.2</v>
+        <v>77.8</v>
       </c>
       <c r="F5" t="n">
-        <v>68.3</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>73.2</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.64</v>
       </c>
       <c r="E6" t="n">
-        <v>64.09999999999999</v>
+        <v>63.9</v>
       </c>
       <c r="F6" t="n">
-        <v>64.8</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>64.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         <v>51.4</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="8">
@@ -672,7 +672,7 @@
         <v>4.52</v>
       </c>
       <c r="E8" t="n">
-        <v>43</v>
+        <v>43.1</v>
       </c>
       <c r="F8" t="n">
         <v>45.8</v>
@@ -681,7 +681,7 @@
         <v>44.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="9">
@@ -705,13 +705,13 @@
         <v>45.1</v>
       </c>
       <c r="F9" t="n">
-        <v>31.7</v>
+        <v>31.9</v>
       </c>
       <c r="G9" t="n">
-        <v>38.4</v>
+        <v>38.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.99</v>
       </c>
       <c r="E10" t="n">
-        <v>38</v>
+        <v>38.2</v>
       </c>
       <c r="F10" t="n">
-        <v>38</v>
+        <v>38.2</v>
       </c>
       <c r="G10" t="n">
-        <v>38</v>
+        <v>38.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.56</v>
       </c>
       <c r="E11" t="n">
-        <v>35.9</v>
+        <v>36.1</v>
       </c>
       <c r="F11" t="n">
-        <v>36.6</v>
+        <v>36.8</v>
       </c>
       <c r="G11" t="n">
-        <v>36.3</v>
+        <v>36.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.36</v>
       </c>
       <c r="E12" t="n">
-        <v>30.3</v>
+        <v>30.6</v>
       </c>
       <c r="F12" t="n">
-        <v>25.4</v>
+        <v>25.7</v>
       </c>
       <c r="G12" t="n">
-        <v>26.8</v>
+        <v>27.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>2.29</v>
       </c>
       <c r="E13" t="n">
-        <v>30.3</v>
+        <v>30.6</v>
       </c>
       <c r="F13" t="n">
-        <v>23.2</v>
+        <v>23.6</v>
       </c>
       <c r="G13" t="n">
-        <v>25.4</v>
+        <v>25.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>30.3</v>
+        <v>30.6</v>
       </c>
       <c r="F14" t="n">
-        <v>23.2</v>
+        <v>23.6</v>
       </c>
       <c r="G14" t="n">
-        <v>25.4</v>
+        <v>25.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>3.88</v>
       </c>
       <c r="E15" t="n">
-        <v>20.4</v>
+        <v>20.8</v>
       </c>
       <c r="F15" t="n">
-        <v>17.6</v>
+        <v>18.1</v>
       </c>
       <c r="G15" t="n">
-        <v>18.5</v>
+        <v>18.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>3.52</v>
       </c>
       <c r="E16" t="n">
-        <v>21.8</v>
+        <v>22.2</v>
       </c>
       <c r="F16" t="n">
-        <v>16.9</v>
+        <v>17.4</v>
       </c>
       <c r="G16" t="n">
-        <v>18.4</v>
+        <v>18.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.2</v>
       </c>
       <c r="E17" t="n">
-        <v>19</v>
+        <v>19.4</v>
       </c>
       <c r="F17" t="n">
-        <v>16.9</v>
+        <v>17.4</v>
       </c>
       <c r="G17" t="n">
-        <v>17.5</v>
+        <v>18</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>12.7</v>
+        <v>13.2</v>
       </c>
       <c r="F18" t="n">
-        <v>19</v>
+        <v>19.4</v>
       </c>
       <c r="G18" t="n">
-        <v>17.1</v>
+        <v>17.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="F19" t="n">
-        <v>18.3</v>
+        <v>18.8</v>
       </c>
       <c r="G19" t="n">
-        <v>16.4</v>
+        <v>16.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.59</v>
       </c>
       <c r="E20" t="n">
-        <v>17.6</v>
+        <v>18.1</v>
       </c>
       <c r="F20" t="n">
-        <v>13.4</v>
+        <v>13.9</v>
       </c>
       <c r="G20" t="n">
-        <v>14.6</v>
+        <v>15.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.17</v>
       </c>
       <c r="E21" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="F21" t="n">
-        <v>14.8</v>
+        <v>15.3</v>
       </c>
       <c r="G21" t="n">
-        <v>13.9</v>
+        <v>14.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.77</v>
       </c>
       <c r="E22" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="F22" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="G22" t="n">
         <v>14.1</v>
       </c>
-      <c r="F22" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="G22" t="n">
-        <v>13.6</v>
-      </c>
       <c r="H22" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.52</v>
       </c>
       <c r="E23" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="F23" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="G23" t="n">
         <v>13.4</v>
       </c>
-      <c r="F23" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="G23" t="n">
-        <v>12.9</v>
-      </c>
       <c r="H23" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.02</v>
       </c>
       <c r="E24" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="F24" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="G24" t="n">
         <v>13.4</v>
       </c>
-      <c r="F24" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="G24" t="n">
-        <v>12.9</v>
-      </c>
       <c r="H24" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.14</v>
       </c>
       <c r="E25" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="F25" t="n">
-        <v>12.7</v>
+        <v>13.2</v>
       </c>
       <c r="G25" t="n">
-        <v>12.5</v>
+        <v>13</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>1.73</v>
       </c>
       <c r="E26" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="F26" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="G26" t="n">
-        <v>11.5</v>
+        <v>12.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>0.9</v>
       </c>
       <c r="E27" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="F27" t="n">
-        <v>11.3</v>
+        <v>11.8</v>
       </c>
       <c r="G27" t="n">
-        <v>11.1</v>
+        <v>11.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.33</v>
       </c>
       <c r="E28" t="n">
-        <v>12.7</v>
+        <v>13.2</v>
       </c>
       <c r="F28" t="n">
-        <v>9.9</v>
+        <v>10.4</v>
       </c>
       <c r="G28" t="n">
-        <v>10.7</v>
+        <v>11.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.21</v>
       </c>
       <c r="E29" t="n">
-        <v>11.3</v>
+        <v>11.8</v>
       </c>
       <c r="F29" t="n">
-        <v>9.9</v>
+        <v>10.4</v>
       </c>
       <c r="G29" t="n">
-        <v>10.3</v>
+        <v>10.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.91</v>
       </c>
       <c r="E30" t="n">
-        <v>9.199999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F30" t="n">
-        <v>9.199999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G30" t="n">
-        <v>9.199999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.62</v>
       </c>
       <c r="E31" t="n">
-        <v>7.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F31" t="n">
-        <v>7.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>7.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>0.61</v>
       </c>
       <c r="E32" t="n">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="F32" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G32" t="n">
         <v>4.2</v>
       </c>
-      <c r="G32" t="n">
-        <v>3.6</v>
-      </c>
       <c r="H32" s="2" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Jul  6 13:30:14 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,31 +477,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>46.41</v>
+        <v>10.55</v>
       </c>
       <c r="D2" t="n">
-        <v>2.58</v>
+        <v>1.28</v>
       </c>
       <c r="E2" t="n">
-        <v>88.90000000000001</v>
+        <v>87.7</v>
       </c>
       <c r="F2" t="n">
-        <v>88.90000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="G2" t="n">
-        <v>88.90000000000001</v>
+        <v>81.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>44.29</v>
+        <v>43.46</v>
       </c>
       <c r="D3" t="n">
-        <v>3.75</v>
+        <v>3.68</v>
       </c>
       <c r="E3" t="n">
-        <v>88.90000000000001</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>88.2</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>88.5</v>
+        <v>77.7</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="4">
@@ -546,52 +546,52 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>84.05</v>
+        <v>83.14</v>
       </c>
       <c r="D4" t="n">
-        <v>8.82</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>84.7</v>
+        <v>76.7</v>
       </c>
       <c r="F4" t="n">
-        <v>84.7</v>
+        <v>76.7</v>
       </c>
       <c r="G4" t="n">
-        <v>84.7</v>
+        <v>76.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10.47</v>
+        <v>43.17</v>
       </c>
       <c r="D5" t="n">
-        <v>1.27</v>
+        <v>2.4</v>
       </c>
       <c r="E5" t="n">
-        <v>77.8</v>
+        <v>74</v>
       </c>
       <c r="F5" t="n">
-        <v>68.09999999999999</v>
+        <v>74</v>
       </c>
       <c r="G5" t="n">
-        <v>72.90000000000001</v>
+        <v>74</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="6">
@@ -606,202 +606,202 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28.71</v>
+        <v>28.96</v>
       </c>
       <c r="D6" t="n">
-        <v>2.64</v>
+        <v>2.66</v>
       </c>
       <c r="E6" t="n">
-        <v>63.9</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>64.59999999999999</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>64.2</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>62.49</v>
+        <v>121.47</v>
       </c>
       <c r="D7" t="n">
-        <v>4.02</v>
+        <v>4.55</v>
       </c>
       <c r="E7" t="n">
-        <v>51.4</v>
+        <v>52.1</v>
       </c>
       <c r="F7" t="n">
         <v>51.4</v>
       </c>
       <c r="G7" t="n">
-        <v>51.4</v>
+        <v>51.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>120.43</v>
+        <v>61.67</v>
       </c>
       <c r="D8" t="n">
-        <v>4.52</v>
+        <v>3.96</v>
       </c>
       <c r="E8" t="n">
-        <v>43.1</v>
+        <v>47.9</v>
       </c>
       <c r="F8" t="n">
-        <v>45.8</v>
+        <v>46.6</v>
       </c>
       <c r="G8" t="n">
-        <v>44.4</v>
+        <v>47.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19.87</v>
+        <v>27.79</v>
       </c>
       <c r="D9" t="n">
-        <v>1.66</v>
+        <v>2.05</v>
       </c>
       <c r="E9" t="n">
-        <v>45.1</v>
+        <v>46.6</v>
       </c>
       <c r="F9" t="n">
-        <v>31.9</v>
+        <v>36.3</v>
       </c>
       <c r="G9" t="n">
-        <v>38.5</v>
+        <v>41.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>31.57</v>
+        <v>19.76</v>
       </c>
       <c r="D10" t="n">
-        <v>2.99</v>
+        <v>1.65</v>
       </c>
       <c r="E10" t="n">
-        <v>38.2</v>
+        <v>41.1</v>
       </c>
       <c r="F10" t="n">
-        <v>38.2</v>
+        <v>26.7</v>
       </c>
       <c r="G10" t="n">
-        <v>38.2</v>
+        <v>31</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28.01</v>
+        <v>30.98</v>
       </c>
       <c r="D11" t="n">
-        <v>2.56</v>
+        <v>2.93</v>
       </c>
       <c r="E11" t="n">
-        <v>36.1</v>
+        <v>28.8</v>
       </c>
       <c r="F11" t="n">
-        <v>36.8</v>
+        <v>28.1</v>
       </c>
       <c r="G11" t="n">
-        <v>36.5</v>
+        <v>28.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>28.19</v>
+        <v>14.55</v>
       </c>
       <c r="D12" t="n">
-        <v>2.36</v>
+        <v>1.19</v>
       </c>
       <c r="E12" t="n">
-        <v>30.6</v>
+        <v>25.3</v>
       </c>
       <c r="F12" t="n">
-        <v>25.7</v>
+        <v>27.4</v>
       </c>
       <c r="G12" t="n">
-        <v>27.2</v>
+        <v>26.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="13">
@@ -822,586 +822,586 @@
         <v>2.29</v>
       </c>
       <c r="E13" t="n">
-        <v>30.6</v>
+        <v>30.8</v>
       </c>
       <c r="F13" t="n">
-        <v>23.6</v>
+        <v>24</v>
       </c>
       <c r="G13" t="n">
-        <v>25.7</v>
+        <v>26</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>27.09</v>
+        <v>27.73</v>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>2.54</v>
       </c>
       <c r="E14" t="n">
-        <v>30.6</v>
+        <v>27.4</v>
       </c>
       <c r="F14" t="n">
-        <v>23.6</v>
+        <v>23.3</v>
       </c>
       <c r="G14" t="n">
-        <v>25.7</v>
+        <v>24.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>47.33</v>
+        <v>28.05</v>
       </c>
       <c r="D15" t="n">
-        <v>3.88</v>
+        <v>2.34</v>
       </c>
       <c r="E15" t="n">
-        <v>20.8</v>
+        <v>24.7</v>
       </c>
       <c r="F15" t="n">
-        <v>18.1</v>
+        <v>22.6</v>
       </c>
       <c r="G15" t="n">
-        <v>18.9</v>
+        <v>23.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>21.3</v>
+        <v>17.08</v>
       </c>
       <c r="D16" t="n">
-        <v>3.52</v>
+        <v>1.58</v>
       </c>
       <c r="E16" t="n">
-        <v>22.2</v>
+        <v>24.7</v>
       </c>
       <c r="F16" t="n">
-        <v>17.4</v>
+        <v>21.9</v>
       </c>
       <c r="G16" t="n">
-        <v>18.8</v>
+        <v>22.7</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.85</v>
+        <v>10.47</v>
       </c>
       <c r="D17" t="n">
-        <v>2.2</v>
+        <v>0.95</v>
       </c>
       <c r="E17" t="n">
-        <v>19.4</v>
+        <v>16.4</v>
       </c>
       <c r="F17" t="n">
-        <v>17.4</v>
+        <v>24</v>
       </c>
       <c r="G17" t="n">
-        <v>18</v>
+        <v>21.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>10.7</v>
+        <v>18.75</v>
       </c>
       <c r="D18" t="n">
-        <v>0.6899999999999999</v>
+        <v>3.24</v>
       </c>
       <c r="E18" t="n">
-        <v>13.2</v>
+        <v>17.8</v>
       </c>
       <c r="F18" t="n">
-        <v>19.4</v>
+        <v>17.8</v>
       </c>
       <c r="G18" t="n">
-        <v>17.6</v>
+        <v>17.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.45</v>
+        <v>12.41</v>
       </c>
       <c r="D19" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.16</v>
       </c>
       <c r="E19" t="n">
-        <v>12.5</v>
+        <v>16.4</v>
       </c>
       <c r="F19" t="n">
-        <v>18.8</v>
+        <v>16.4</v>
       </c>
       <c r="G19" t="n">
-        <v>16.9</v>
+        <v>16.4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>21.7</v>
+        <v>23.76</v>
       </c>
       <c r="D20" t="n">
-        <v>1.59</v>
+        <v>2.19</v>
       </c>
       <c r="E20" t="n">
-        <v>18.1</v>
+        <v>16.4</v>
       </c>
       <c r="F20" t="n">
-        <v>13.9</v>
+        <v>15.1</v>
       </c>
       <c r="G20" t="n">
-        <v>15.1</v>
+        <v>15.5</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>14.32</v>
+        <v>21.59</v>
       </c>
       <c r="D21" t="n">
-        <v>1.17</v>
+        <v>1.77</v>
       </c>
       <c r="E21" t="n">
-        <v>12.5</v>
+        <v>17.8</v>
       </c>
       <c r="F21" t="n">
-        <v>15.3</v>
+        <v>14.4</v>
       </c>
       <c r="G21" t="n">
-        <v>14.4</v>
+        <v>15.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21.58</v>
+        <v>30.75</v>
       </c>
       <c r="D22" t="n">
-        <v>1.77</v>
+        <v>2.34</v>
       </c>
       <c r="E22" t="n">
-        <v>14.6</v>
+        <v>17.8</v>
       </c>
       <c r="F22" t="n">
-        <v>13.9</v>
+        <v>14.4</v>
       </c>
       <c r="G22" t="n">
-        <v>14.1</v>
+        <v>15.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>16.44</v>
+        <v>21.6</v>
       </c>
       <c r="D23" t="n">
-        <v>1.52</v>
+        <v>1.59</v>
       </c>
       <c r="E23" t="n">
-        <v>13.9</v>
+        <v>13.7</v>
       </c>
       <c r="F23" t="n">
-        <v>13.2</v>
+        <v>14.4</v>
       </c>
       <c r="G23" t="n">
-        <v>13.4</v>
+        <v>14.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.29</v>
+        <v>16.31</v>
       </c>
       <c r="D24" t="n">
-        <v>2.02</v>
+        <v>0.9</v>
       </c>
       <c r="E24" t="n">
-        <v>13.9</v>
+        <v>15.8</v>
       </c>
       <c r="F24" t="n">
-        <v>13.2</v>
+        <v>12.3</v>
       </c>
       <c r="G24" t="n">
         <v>13.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>12.15</v>
+        <v>46.89</v>
       </c>
       <c r="D25" t="n">
-        <v>1.14</v>
+        <v>3.84</v>
       </c>
       <c r="E25" t="n">
-        <v>12.5</v>
+        <v>15.8</v>
       </c>
       <c r="F25" t="n">
-        <v>13.2</v>
+        <v>12.3</v>
       </c>
       <c r="G25" t="n">
-        <v>13</v>
+        <v>13.4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18.53</v>
+        <v>6.55</v>
       </c>
       <c r="D26" t="n">
-        <v>1.73</v>
+        <v>0.62</v>
       </c>
       <c r="E26" t="n">
-        <v>11.1</v>
+        <v>9.6</v>
       </c>
       <c r="F26" t="n">
-        <v>12.5</v>
+        <v>13</v>
       </c>
       <c r="G26" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>16.27</v>
+        <v>23.42</v>
       </c>
       <c r="D27" t="n">
-        <v>0.9</v>
+        <v>1.91</v>
       </c>
       <c r="E27" t="n">
-        <v>11.1</v>
+        <v>12.3</v>
       </c>
       <c r="F27" t="n">
-        <v>11.8</v>
+        <v>10.3</v>
       </c>
       <c r="G27" t="n">
-        <v>11.6</v>
+        <v>10.9</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>30.73</v>
+        <v>22.16</v>
       </c>
       <c r="D28" t="n">
-        <v>2.33</v>
+        <v>2</v>
       </c>
       <c r="E28" t="n">
-        <v>13.2</v>
+        <v>11</v>
       </c>
       <c r="F28" t="n">
-        <v>10.4</v>
+        <v>9.6</v>
       </c>
       <c r="G28" t="n">
-        <v>11.2</v>
+        <v>10</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.56</v>
+        <v>20.93</v>
       </c>
       <c r="D29" t="n">
-        <v>3.21</v>
+        <v>3.46</v>
       </c>
       <c r="E29" t="n">
-        <v>11.8</v>
+        <v>11</v>
       </c>
       <c r="F29" t="n">
-        <v>10.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G29" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>23.36</v>
+        <v>10.61</v>
       </c>
       <c r="D30" t="n">
-        <v>1.91</v>
+        <v>0.68</v>
       </c>
       <c r="E30" t="n">
-        <v>9.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="F30" t="n">
-        <v>9.699999999999999</v>
+        <v>6.2</v>
       </c>
       <c r="G30" t="n">
-        <v>9.699999999999999</v>
+        <v>7</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>33.54</v>
+        <v>18.46</v>
       </c>
       <c r="D31" t="n">
-        <v>3.62</v>
+        <v>1.72</v>
       </c>
       <c r="E31" t="n">
-        <v>8.300000000000001</v>
+        <v>2.7</v>
       </c>
       <c r="F31" t="n">
-        <v>8.300000000000001</v>
+        <v>6.2</v>
       </c>
       <c r="G31" t="n">
-        <v>8.300000000000001</v>
+        <v>5.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6.45</v>
+        <v>32.92</v>
       </c>
       <c r="D32" t="n">
-        <v>0.61</v>
+        <v>3.56</v>
       </c>
       <c r="E32" t="n">
-        <v>2.8</v>
+        <v>1.4</v>
       </c>
       <c r="F32" t="n">
-        <v>4.9</v>
+        <v>2.1</v>
       </c>
       <c r="G32" t="n">
-        <v>4.2</v>
+        <v>1.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Jul  7 12:17:40 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,121 +477,121 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.55</v>
+        <v>82.81</v>
       </c>
       <c r="D2" t="n">
-        <v>1.28</v>
+        <v>8.69</v>
       </c>
       <c r="E2" t="n">
-        <v>87.7</v>
+        <v>74.3</v>
       </c>
       <c r="F2" t="n">
-        <v>75.3</v>
+        <v>75.7</v>
       </c>
       <c r="G2" t="n">
-        <v>81.5</v>
+        <v>75</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>43.46</v>
+        <v>41.93</v>
       </c>
       <c r="D3" t="n">
-        <v>3.68</v>
+        <v>2.32</v>
       </c>
       <c r="E3" t="n">
-        <v>77.40000000000001</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>78.09999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>77.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>83.14</v>
+        <v>42.7</v>
       </c>
       <c r="D4" t="n">
-        <v>8.720000000000001</v>
+        <v>3.61</v>
       </c>
       <c r="E4" t="n">
-        <v>76.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>76.7</v>
+        <v>63.5</v>
       </c>
       <c r="G4" t="n">
-        <v>76.7</v>
+        <v>64.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>43.17</v>
+        <v>10.27</v>
       </c>
       <c r="D5" t="n">
-        <v>2.4</v>
+        <v>1.25</v>
       </c>
       <c r="E5" t="n">
-        <v>74</v>
+        <v>64.2</v>
       </c>
       <c r="F5" t="n">
-        <v>74</v>
+        <v>58.1</v>
       </c>
       <c r="G5" t="n">
-        <v>74</v>
+        <v>61.1</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="6">
@@ -606,802 +606,802 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28.96</v>
+        <v>27.91</v>
       </c>
       <c r="D6" t="n">
-        <v>2.66</v>
+        <v>2.56</v>
       </c>
       <c r="E6" t="n">
-        <v>67.09999999999999</v>
+        <v>48.6</v>
       </c>
       <c r="F6" t="n">
-        <v>67.09999999999999</v>
+        <v>41.9</v>
       </c>
       <c r="G6" t="n">
-        <v>67.09999999999999</v>
+        <v>45.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>121.47</v>
+        <v>27.38</v>
       </c>
       <c r="D7" t="n">
-        <v>4.55</v>
+        <v>2.03</v>
       </c>
       <c r="E7" t="n">
-        <v>52.1</v>
+        <v>40.5</v>
       </c>
       <c r="F7" t="n">
-        <v>51.4</v>
+        <v>33.1</v>
       </c>
       <c r="G7" t="n">
-        <v>51.7</v>
+        <v>36.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>61.67</v>
+        <v>116.69</v>
       </c>
       <c r="D8" t="n">
-        <v>3.96</v>
+        <v>4.38</v>
       </c>
       <c r="E8" t="n">
-        <v>47.9</v>
+        <v>32.4</v>
       </c>
       <c r="F8" t="n">
-        <v>46.6</v>
+        <v>29.1</v>
       </c>
       <c r="G8" t="n">
-        <v>47.3</v>
+        <v>30.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27.79</v>
+        <v>30.96</v>
       </c>
       <c r="D9" t="n">
-        <v>2.05</v>
+        <v>2.94</v>
       </c>
       <c r="E9" t="n">
-        <v>46.6</v>
+        <v>28.4</v>
       </c>
       <c r="F9" t="n">
-        <v>36.3</v>
+        <v>29.7</v>
       </c>
       <c r="G9" t="n">
-        <v>41.4</v>
+        <v>29.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.76</v>
+        <v>60.31</v>
       </c>
       <c r="D10" t="n">
-        <v>1.65</v>
+        <v>3.88</v>
       </c>
       <c r="E10" t="n">
-        <v>41.1</v>
+        <v>30.4</v>
       </c>
       <c r="F10" t="n">
-        <v>26.7</v>
+        <v>19.6</v>
       </c>
       <c r="G10" t="n">
-        <v>31</v>
+        <v>22.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>30.98</v>
+        <v>6.63</v>
       </c>
       <c r="D11" t="n">
-        <v>2.93</v>
+        <v>0.63</v>
       </c>
       <c r="E11" t="n">
-        <v>28.8</v>
+        <v>17.6</v>
       </c>
       <c r="F11" t="n">
-        <v>28.1</v>
+        <v>21.6</v>
       </c>
       <c r="G11" t="n">
-        <v>28.3</v>
+        <v>20.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>14.55</v>
+        <v>16.84</v>
       </c>
       <c r="D12" t="n">
-        <v>1.19</v>
+        <v>1.56</v>
       </c>
       <c r="E12" t="n">
-        <v>25.3</v>
+        <v>17.6</v>
       </c>
       <c r="F12" t="n">
-        <v>27.4</v>
+        <v>17.6</v>
       </c>
       <c r="G12" t="n">
-        <v>26.8</v>
+        <v>17.6</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>15.51</v>
+        <v>12.31</v>
       </c>
       <c r="D13" t="n">
-        <v>2.29</v>
+        <v>1.16</v>
       </c>
       <c r="E13" t="n">
-        <v>30.8</v>
+        <v>16.2</v>
       </c>
       <c r="F13" t="n">
-        <v>24</v>
+        <v>16.9</v>
       </c>
       <c r="G13" t="n">
-        <v>26</v>
+        <v>16.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>27.73</v>
+        <v>15.25</v>
       </c>
       <c r="D14" t="n">
-        <v>2.54</v>
+        <v>2.25</v>
       </c>
       <c r="E14" t="n">
-        <v>27.4</v>
+        <v>20.3</v>
       </c>
       <c r="F14" t="n">
-        <v>23.3</v>
+        <v>12.8</v>
       </c>
       <c r="G14" t="n">
-        <v>24.5</v>
+        <v>15.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>28.05</v>
+        <v>23.31</v>
       </c>
       <c r="D15" t="n">
-        <v>2.34</v>
+        <v>2.15</v>
       </c>
       <c r="E15" t="n">
-        <v>24.7</v>
+        <v>13.5</v>
       </c>
       <c r="F15" t="n">
-        <v>22.6</v>
+        <v>13.5</v>
       </c>
       <c r="G15" t="n">
-        <v>23.2</v>
+        <v>13.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>17.08</v>
+        <v>19.26</v>
       </c>
       <c r="D16" t="n">
-        <v>1.58</v>
+        <v>1.61</v>
       </c>
       <c r="E16" t="n">
-        <v>24.7</v>
+        <v>12.2</v>
       </c>
       <c r="F16" t="n">
-        <v>21.9</v>
+        <v>12.8</v>
       </c>
       <c r="G16" t="n">
-        <v>22.7</v>
+        <v>12.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.47</v>
+        <v>14.27</v>
       </c>
       <c r="D17" t="n">
-        <v>0.95</v>
+        <v>1.16</v>
       </c>
       <c r="E17" t="n">
-        <v>16.4</v>
+        <v>10.8</v>
       </c>
       <c r="F17" t="n">
-        <v>24</v>
+        <v>10.8</v>
       </c>
       <c r="G17" t="n">
-        <v>21.7</v>
+        <v>10.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>18.75</v>
+        <v>27.37</v>
       </c>
       <c r="D18" t="n">
-        <v>3.24</v>
+        <v>2.29</v>
       </c>
       <c r="E18" t="n">
-        <v>17.8</v>
+        <v>10.8</v>
       </c>
       <c r="F18" t="n">
-        <v>17.8</v>
+        <v>10.8</v>
       </c>
       <c r="G18" t="n">
-        <v>17.8</v>
+        <v>10.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>12.41</v>
+        <v>23.31</v>
       </c>
       <c r="D19" t="n">
-        <v>1.16</v>
+        <v>1.91</v>
       </c>
       <c r="E19" t="n">
-        <v>16.4</v>
+        <v>8.1</v>
       </c>
       <c r="F19" t="n">
-        <v>16.4</v>
+        <v>10.8</v>
       </c>
       <c r="G19" t="n">
-        <v>16.4</v>
+        <v>10</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>23.76</v>
+        <v>26.95</v>
       </c>
       <c r="D20" t="n">
-        <v>2.19</v>
+        <v>2.47</v>
       </c>
       <c r="E20" t="n">
-        <v>16.4</v>
+        <v>14.9</v>
       </c>
       <c r="F20" t="n">
-        <v>15.1</v>
+        <v>7.4</v>
       </c>
       <c r="G20" t="n">
-        <v>15.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>21.59</v>
+        <v>10.17</v>
       </c>
       <c r="D21" t="n">
-        <v>1.77</v>
+        <v>0.92</v>
       </c>
       <c r="E21" t="n">
-        <v>17.8</v>
+        <v>6.8</v>
       </c>
       <c r="F21" t="n">
-        <v>14.4</v>
+        <v>10.1</v>
       </c>
       <c r="G21" t="n">
-        <v>15.4</v>
+        <v>9.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>30.75</v>
+        <v>15.92</v>
       </c>
       <c r="D22" t="n">
-        <v>2.34</v>
+        <v>0.88</v>
       </c>
       <c r="E22" t="n">
-        <v>17.8</v>
+        <v>8.1</v>
       </c>
       <c r="F22" t="n">
-        <v>14.4</v>
+        <v>6.8</v>
       </c>
       <c r="G22" t="n">
-        <v>15.4</v>
+        <v>7.2</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>21.6</v>
+        <v>20.97</v>
       </c>
       <c r="D23" t="n">
-        <v>1.59</v>
+        <v>1.72</v>
       </c>
       <c r="E23" t="n">
-        <v>13.7</v>
+        <v>7.4</v>
       </c>
       <c r="F23" t="n">
-        <v>14.4</v>
+        <v>6.8</v>
       </c>
       <c r="G23" t="n">
-        <v>14.2</v>
+        <v>7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>16.31</v>
+        <v>18.42</v>
       </c>
       <c r="D24" t="n">
-        <v>0.9</v>
+        <v>3.19</v>
       </c>
       <c r="E24" t="n">
-        <v>15.8</v>
+        <v>6.8</v>
       </c>
       <c r="F24" t="n">
-        <v>12.3</v>
+        <v>6.8</v>
       </c>
       <c r="G24" t="n">
-        <v>13.4</v>
+        <v>6.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>46.89</v>
+        <v>21.23</v>
       </c>
       <c r="D25" t="n">
-        <v>3.84</v>
+        <v>1.56</v>
       </c>
       <c r="E25" t="n">
-        <v>15.8</v>
+        <v>4.1</v>
       </c>
       <c r="F25" t="n">
-        <v>12.3</v>
+        <v>6.1</v>
       </c>
       <c r="G25" t="n">
-        <v>13.4</v>
+        <v>5.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6.55</v>
+        <v>45.9</v>
       </c>
       <c r="D26" t="n">
-        <v>0.62</v>
+        <v>3.76</v>
       </c>
       <c r="E26" t="n">
-        <v>9.6</v>
+        <v>6.8</v>
       </c>
       <c r="F26" t="n">
-        <v>13</v>
+        <v>2.7</v>
       </c>
       <c r="G26" t="n">
-        <v>12</v>
+        <v>3.9</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>23.42</v>
+        <v>21.72</v>
       </c>
       <c r="D27" t="n">
-        <v>1.91</v>
+        <v>1.97</v>
       </c>
       <c r="E27" t="n">
-        <v>12.3</v>
+        <v>1.4</v>
       </c>
       <c r="F27" t="n">
-        <v>10.3</v>
+        <v>3.4</v>
       </c>
       <c r="G27" t="n">
-        <v>10.9</v>
+        <v>2.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22.16</v>
+        <v>20.32</v>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>3.36</v>
       </c>
       <c r="E28" t="n">
-        <v>11</v>
+        <v>4.1</v>
       </c>
       <c r="F28" t="n">
-        <v>9.6</v>
+        <v>1.4</v>
       </c>
       <c r="G28" t="n">
-        <v>10</v>
+        <v>2.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>20.93</v>
+        <v>10.35</v>
       </c>
       <c r="D29" t="n">
-        <v>3.46</v>
+        <v>0.66</v>
       </c>
       <c r="E29" t="n">
-        <v>11</v>
+        <v>2.7</v>
       </c>
       <c r="F29" t="n">
-        <v>8.199999999999999</v>
+        <v>1.4</v>
       </c>
       <c r="G29" t="n">
-        <v>9</v>
+        <v>1.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>10.61</v>
+        <v>18.12</v>
       </c>
       <c r="D30" t="n">
-        <v>0.68</v>
+        <v>1.69</v>
       </c>
       <c r="E30" t="n">
-        <v>8.9</v>
+        <v>1.4</v>
       </c>
       <c r="F30" t="n">
-        <v>6.2</v>
+        <v>1.4</v>
       </c>
       <c r="G30" t="n">
-        <v>7</v>
+        <v>1.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>18.46</v>
+        <v>32.36</v>
       </c>
       <c r="D31" t="n">
-        <v>1.72</v>
+        <v>3.49</v>
       </c>
       <c r="E31" t="n">
-        <v>2.7</v>
+        <v>1.4</v>
       </c>
       <c r="F31" t="n">
-        <v>6.2</v>
+        <v>1.4</v>
       </c>
       <c r="G31" t="n">
-        <v>5.1</v>
+        <v>1.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>32.92</v>
+        <v>29.83</v>
       </c>
       <c r="D32" t="n">
-        <v>3.56</v>
+        <v>2.27</v>
       </c>
       <c r="E32" t="n">
         <v>1.4</v>
       </c>
       <c r="F32" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="G32" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Jul  8 11:31:35 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>82.81</v>
+        <v>82.41</v>
       </c>
       <c r="D2" t="n">
-        <v>8.69</v>
+        <v>8.65</v>
       </c>
       <c r="E2" t="n">
-        <v>74.3</v>
+        <v>73.3</v>
       </c>
       <c r="F2" t="n">
-        <v>75.7</v>
+        <v>73.3</v>
       </c>
       <c r="G2" t="n">
-        <v>75</v>
+        <v>73.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="3">
@@ -516,82 +516,82 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>41.93</v>
+        <v>40.1</v>
       </c>
       <c r="D3" t="n">
-        <v>2.32</v>
+        <v>2.23</v>
       </c>
       <c r="E3" t="n">
-        <v>71.59999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="F3" t="n">
-        <v>71.59999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="G3" t="n">
-        <v>71.59999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42.7</v>
+        <v>10.2</v>
       </c>
       <c r="D4" t="n">
-        <v>3.61</v>
+        <v>1.24</v>
       </c>
       <c r="E4" t="n">
-        <v>64.90000000000001</v>
+        <v>58.7</v>
       </c>
       <c r="F4" t="n">
-        <v>63.5</v>
+        <v>55.3</v>
       </c>
       <c r="G4" t="n">
-        <v>64.2</v>
+        <v>57</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10.27</v>
+        <v>41.21</v>
       </c>
       <c r="D5" t="n">
-        <v>1.25</v>
+        <v>3.49</v>
       </c>
       <c r="E5" t="n">
-        <v>64.2</v>
+        <v>40</v>
       </c>
       <c r="F5" t="n">
-        <v>58.1</v>
+        <v>40</v>
       </c>
       <c r="G5" t="n">
-        <v>61.1</v>
+        <v>40</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="6">
@@ -606,82 +606,82 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27.91</v>
+        <v>27.52</v>
       </c>
       <c r="D6" t="n">
-        <v>2.56</v>
+        <v>2.53</v>
       </c>
       <c r="E6" t="n">
-        <v>48.6</v>
+        <v>40</v>
       </c>
       <c r="F6" t="n">
-        <v>41.9</v>
+        <v>38</v>
       </c>
       <c r="G6" t="n">
-        <v>45.3</v>
+        <v>39</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>27.38</v>
+        <v>117.62</v>
       </c>
       <c r="D7" t="n">
-        <v>2.03</v>
+        <v>4.41</v>
       </c>
       <c r="E7" t="n">
-        <v>40.5</v>
+        <v>36</v>
       </c>
       <c r="F7" t="n">
-        <v>33.1</v>
+        <v>36</v>
       </c>
       <c r="G7" t="n">
-        <v>36.8</v>
+        <v>36</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>116.69</v>
+        <v>6.73</v>
       </c>
       <c r="D8" t="n">
-        <v>4.38</v>
+        <v>0.64</v>
       </c>
       <c r="E8" t="n">
-        <v>32.4</v>
+        <v>28.7</v>
       </c>
       <c r="F8" t="n">
-        <v>29.1</v>
+        <v>37.3</v>
       </c>
       <c r="G8" t="n">
-        <v>30.1</v>
+        <v>33</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="9">
@@ -696,562 +696,562 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30.96</v>
+        <v>31.08</v>
       </c>
       <c r="D9" t="n">
         <v>2.94</v>
       </c>
       <c r="E9" t="n">
-        <v>28.4</v>
+        <v>30.7</v>
       </c>
       <c r="F9" t="n">
-        <v>29.7</v>
+        <v>30</v>
       </c>
       <c r="G9" t="n">
-        <v>29.3</v>
+        <v>30.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>60.31</v>
+        <v>17.02</v>
       </c>
       <c r="D10" t="n">
-        <v>3.88</v>
+        <v>1.58</v>
       </c>
       <c r="E10" t="n">
-        <v>30.4</v>
+        <v>22.7</v>
       </c>
       <c r="F10" t="n">
-        <v>19.6</v>
+        <v>23.3</v>
       </c>
       <c r="G10" t="n">
-        <v>22.8</v>
+        <v>23.1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6.63</v>
+        <v>26.81</v>
       </c>
       <c r="D11" t="n">
-        <v>0.63</v>
+        <v>1.98</v>
       </c>
       <c r="E11" t="n">
-        <v>17.6</v>
+        <v>22.7</v>
       </c>
       <c r="F11" t="n">
-        <v>21.6</v>
+        <v>18.7</v>
       </c>
       <c r="G11" t="n">
-        <v>20.4</v>
+        <v>19.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>16.84</v>
+        <v>12.44</v>
       </c>
       <c r="D12" t="n">
-        <v>1.56</v>
+        <v>1.17</v>
       </c>
       <c r="E12" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="F12" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="G12" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12.31</v>
+        <v>46.96</v>
       </c>
       <c r="D13" t="n">
-        <v>1.16</v>
+        <v>3.85</v>
       </c>
       <c r="E13" t="n">
-        <v>16.2</v>
+        <v>19.3</v>
       </c>
       <c r="F13" t="n">
-        <v>16.9</v>
+        <v>14.7</v>
       </c>
       <c r="G13" t="n">
-        <v>16.7</v>
+        <v>16.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.25</v>
+        <v>14.29</v>
       </c>
       <c r="D14" t="n">
-        <v>2.25</v>
+        <v>1.16</v>
       </c>
       <c r="E14" t="n">
-        <v>20.3</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>12.8</v>
+        <v>11.3</v>
       </c>
       <c r="G14" t="n">
-        <v>15.1</v>
+        <v>11.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>23.31</v>
+        <v>27.38</v>
       </c>
       <c r="D15" t="n">
-        <v>2.15</v>
+        <v>2.29</v>
       </c>
       <c r="E15" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="F15" t="n">
-        <v>13.5</v>
+        <v>11.3</v>
       </c>
       <c r="G15" t="n">
-        <v>13.5</v>
+        <v>11.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>19.26</v>
+        <v>10.26</v>
       </c>
       <c r="D16" t="n">
-        <v>1.61</v>
+        <v>0.92</v>
       </c>
       <c r="E16" t="n">
-        <v>12.2</v>
+        <v>10.7</v>
       </c>
       <c r="F16" t="n">
-        <v>12.8</v>
+        <v>10.7</v>
       </c>
       <c r="G16" t="n">
-        <v>12.6</v>
+        <v>10.7</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14.27</v>
+        <v>15.07</v>
       </c>
       <c r="D17" t="n">
-        <v>1.16</v>
+        <v>2.23</v>
       </c>
       <c r="E17" t="n">
-        <v>10.8</v>
+        <v>12</v>
       </c>
       <c r="F17" t="n">
-        <v>10.8</v>
+        <v>10</v>
       </c>
       <c r="G17" t="n">
-        <v>10.8</v>
+        <v>10.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>27.37</v>
+        <v>22.8</v>
       </c>
       <c r="D18" t="n">
-        <v>2.29</v>
+        <v>2.1</v>
       </c>
       <c r="E18" t="n">
-        <v>10.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>10.8</v>
+        <v>10</v>
       </c>
       <c r="G18" t="n">
-        <v>10.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>23.31</v>
+        <v>18.5</v>
       </c>
       <c r="D19" t="n">
-        <v>1.91</v>
+        <v>3.2</v>
       </c>
       <c r="E19" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="F19" t="n">
-        <v>10.8</v>
+        <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>26.95</v>
+        <v>19.03</v>
       </c>
       <c r="D20" t="n">
-        <v>2.47</v>
+        <v>1.59</v>
       </c>
       <c r="E20" t="n">
-        <v>14.9</v>
+        <v>8</v>
       </c>
       <c r="F20" t="n">
-        <v>7.4</v>
+        <v>8</v>
       </c>
       <c r="G20" t="n">
-        <v>9.699999999999999</v>
+        <v>8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10.17</v>
+        <v>23.15</v>
       </c>
       <c r="D21" t="n">
-        <v>0.92</v>
+        <v>1.89</v>
       </c>
       <c r="E21" t="n">
-        <v>6.8</v>
+        <v>5.3</v>
       </c>
       <c r="F21" t="n">
-        <v>10.1</v>
+        <v>6</v>
       </c>
       <c r="G21" t="n">
-        <v>9.1</v>
+        <v>5.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>15.92</v>
+        <v>20.89</v>
       </c>
       <c r="D22" t="n">
-        <v>0.88</v>
+        <v>1.71</v>
       </c>
       <c r="E22" t="n">
-        <v>8.1</v>
+        <v>5.3</v>
       </c>
       <c r="F22" t="n">
-        <v>6.8</v>
+        <v>5.3</v>
       </c>
       <c r="G22" t="n">
-        <v>7.2</v>
+        <v>5.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>20.97</v>
+        <v>58.95</v>
       </c>
       <c r="D23" t="n">
-        <v>1.72</v>
+        <v>3.79</v>
       </c>
       <c r="E23" t="n">
-        <v>7.4</v>
+        <v>6.7</v>
       </c>
       <c r="F23" t="n">
-        <v>6.8</v>
+        <v>4.7</v>
       </c>
       <c r="G23" t="n">
-        <v>7</v>
+        <v>5.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>18.42</v>
+        <v>15.79</v>
       </c>
       <c r="D24" t="n">
-        <v>3.19</v>
+        <v>0.87</v>
       </c>
       <c r="E24" t="n">
-        <v>6.8</v>
+        <v>5.3</v>
       </c>
       <c r="F24" t="n">
-        <v>6.8</v>
+        <v>3.3</v>
       </c>
       <c r="G24" t="n">
-        <v>6.8</v>
+        <v>3.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21.23</v>
+        <v>10.33</v>
       </c>
       <c r="D25" t="n">
-        <v>1.56</v>
+        <v>0.66</v>
       </c>
       <c r="E25" t="n">
-        <v>4.1</v>
+        <v>2.7</v>
       </c>
       <c r="F25" t="n">
-        <v>6.1</v>
+        <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>5.5</v>
+        <v>2.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>45.9</v>
+        <v>18.12</v>
       </c>
       <c r="D26" t="n">
-        <v>3.76</v>
+        <v>1.69</v>
       </c>
       <c r="E26" t="n">
-        <v>6.8</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
-        <v>2.7</v>
+        <v>2</v>
       </c>
       <c r="G26" t="n">
-        <v>3.9</v>
+        <v>2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>21.72</v>
+        <v>26.05</v>
       </c>
       <c r="D27" t="n">
-        <v>1.97</v>
+        <v>2.38</v>
       </c>
       <c r="E27" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="F27" t="n">
-        <v>3.4</v>
+        <v>1.3</v>
       </c>
       <c r="G27" t="n">
-        <v>2.8</v>
+        <v>1.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="28">
@@ -1266,82 +1266,82 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>20.32</v>
+        <v>19.72</v>
       </c>
       <c r="D28" t="n">
-        <v>3.36</v>
+        <v>3.26</v>
       </c>
       <c r="E28" t="n">
-        <v>4.1</v>
+        <v>1.3</v>
       </c>
       <c r="F28" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G28" t="n">
-        <v>2.2</v>
+        <v>1.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>10.35</v>
+        <v>21.36</v>
       </c>
       <c r="D29" t="n">
-        <v>0.66</v>
+        <v>1.93</v>
       </c>
       <c r="E29" t="n">
-        <v>2.7</v>
+        <v>1.3</v>
       </c>
       <c r="F29" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G29" t="n">
-        <v>1.8</v>
+        <v>1.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>18.12</v>
+        <v>29.64</v>
       </c>
       <c r="D30" t="n">
-        <v>1.69</v>
+        <v>2.25</v>
       </c>
       <c r="E30" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="F30" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G30" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="31">
@@ -1356,52 +1356,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>32.36</v>
+        <v>31.04</v>
       </c>
       <c r="D31" t="n">
-        <v>3.49</v>
+        <v>3.35</v>
       </c>
       <c r="E31" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="F31" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G31" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>29.83</v>
+        <v>20.85</v>
       </c>
       <c r="D32" t="n">
-        <v>2.27</v>
+        <v>1.53</v>
       </c>
       <c r="E32" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="F32" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G32" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Jul 10 12:15:41 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>82.41</v>
+        <v>84.06999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>8.65</v>
+        <v>8.82</v>
       </c>
       <c r="E2" t="n">
-        <v>73.3</v>
+        <v>86.8</v>
       </c>
       <c r="F2" t="n">
-        <v>73.3</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>73.3</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>40.1</v>
+        <v>40.08</v>
       </c>
       <c r="D3" t="n">
         <v>2.23</v>
       </c>
       <c r="E3" t="n">
-        <v>69.3</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>69.3</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>69.3</v>
+        <v>68.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="4">
@@ -546,82 +546,82 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.2</v>
+        <v>10.19</v>
       </c>
       <c r="D4" t="n">
         <v>1.24</v>
       </c>
       <c r="E4" t="n">
-        <v>58.7</v>
+        <v>55.9</v>
       </c>
       <c r="F4" t="n">
         <v>55.3</v>
       </c>
       <c r="G4" t="n">
-        <v>57</v>
+        <v>55.6</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>41.21</v>
+        <v>28.37</v>
       </c>
       <c r="D5" t="n">
-        <v>3.49</v>
+        <v>2.6</v>
       </c>
       <c r="E5" t="n">
-        <v>40</v>
+        <v>53.9</v>
       </c>
       <c r="F5" t="n">
-        <v>40</v>
+        <v>51.3</v>
       </c>
       <c r="G5" t="n">
-        <v>40</v>
+        <v>52.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27.52</v>
+        <v>41.73</v>
       </c>
       <c r="D6" t="n">
-        <v>2.53</v>
+        <v>3.53</v>
       </c>
       <c r="E6" t="n">
-        <v>40</v>
+        <v>52.6</v>
       </c>
       <c r="F6" t="n">
-        <v>38</v>
+        <v>51.3</v>
       </c>
       <c r="G6" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="7">
@@ -636,112 +636,112 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>117.62</v>
+        <v>120.82</v>
       </c>
       <c r="D7" t="n">
-        <v>4.41</v>
+        <v>4.53</v>
       </c>
       <c r="E7" t="n">
-        <v>36</v>
+        <v>51.3</v>
       </c>
       <c r="F7" t="n">
-        <v>36</v>
+        <v>51.3</v>
       </c>
       <c r="G7" t="n">
-        <v>36</v>
+        <v>51.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.73</v>
+        <v>61.65</v>
       </c>
       <c r="D8" t="n">
-        <v>0.64</v>
+        <v>3.96</v>
       </c>
       <c r="E8" t="n">
-        <v>28.7</v>
+        <v>47.4</v>
       </c>
       <c r="F8" t="n">
-        <v>37.3</v>
+        <v>48</v>
       </c>
       <c r="G8" t="n">
-        <v>33</v>
+        <v>47.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>31.08</v>
+        <v>48.59</v>
       </c>
       <c r="D9" t="n">
-        <v>2.94</v>
+        <v>3.98</v>
       </c>
       <c r="E9" t="n">
-        <v>30.7</v>
+        <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>30</v>
+        <v>40.8</v>
       </c>
       <c r="G9" t="n">
-        <v>30.3</v>
+        <v>45.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>17.02</v>
+        <v>31.45</v>
       </c>
       <c r="D10" t="n">
-        <v>1.58</v>
+        <v>2.98</v>
       </c>
       <c r="E10" t="n">
-        <v>22.7</v>
+        <v>36.8</v>
       </c>
       <c r="F10" t="n">
-        <v>23.3</v>
+        <v>36.8</v>
       </c>
       <c r="G10" t="n">
-        <v>23.1</v>
+        <v>36.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="11">
@@ -756,322 +756,322 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>26.81</v>
+        <v>27.17</v>
       </c>
       <c r="D11" t="n">
-        <v>1.98</v>
+        <v>2.01</v>
       </c>
       <c r="E11" t="n">
-        <v>22.7</v>
+        <v>34.2</v>
       </c>
       <c r="F11" t="n">
-        <v>18.7</v>
+        <v>27.6</v>
       </c>
       <c r="G11" t="n">
-        <v>19.9</v>
+        <v>29.6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>12.44</v>
+        <v>6.68</v>
       </c>
       <c r="D12" t="n">
-        <v>1.17</v>
+        <v>0.63</v>
       </c>
       <c r="E12" t="n">
-        <v>18.7</v>
+        <v>25</v>
       </c>
       <c r="F12" t="n">
-        <v>18.7</v>
+        <v>21.7</v>
       </c>
       <c r="G12" t="n">
-        <v>18.7</v>
+        <v>22.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>46.96</v>
+        <v>10.46</v>
       </c>
       <c r="D13" t="n">
-        <v>3.85</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>19.3</v>
+        <v>17.1</v>
       </c>
       <c r="F13" t="n">
-        <v>14.7</v>
+        <v>21.1</v>
       </c>
       <c r="G13" t="n">
-        <v>16.1</v>
+        <v>19.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14.29</v>
+        <v>23.65</v>
       </c>
       <c r="D14" t="n">
-        <v>1.16</v>
+        <v>1.93</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>21.1</v>
       </c>
       <c r="F14" t="n">
-        <v>11.3</v>
+        <v>19.1</v>
       </c>
       <c r="G14" t="n">
-        <v>11.5</v>
+        <v>19.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>27.38</v>
+        <v>16.78</v>
       </c>
       <c r="D15" t="n">
-        <v>2.29</v>
+        <v>1.56</v>
       </c>
       <c r="E15" t="n">
-        <v>12</v>
+        <v>17.1</v>
       </c>
       <c r="F15" t="n">
-        <v>11.3</v>
+        <v>17.8</v>
       </c>
       <c r="G15" t="n">
-        <v>11.5</v>
+        <v>17.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.26</v>
+        <v>12.3</v>
       </c>
       <c r="D16" t="n">
-        <v>0.92</v>
+        <v>1.15</v>
       </c>
       <c r="E16" t="n">
-        <v>10.7</v>
+        <v>15.8</v>
       </c>
       <c r="F16" t="n">
-        <v>10.7</v>
+        <v>15.8</v>
       </c>
       <c r="G16" t="n">
-        <v>10.7</v>
+        <v>15.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>15.07</v>
+        <v>18.59</v>
       </c>
       <c r="D17" t="n">
-        <v>2.23</v>
+        <v>3.21</v>
       </c>
       <c r="E17" t="n">
-        <v>12</v>
+        <v>17.1</v>
       </c>
       <c r="F17" t="n">
-        <v>10</v>
+        <v>13.2</v>
       </c>
       <c r="G17" t="n">
-        <v>10.6</v>
+        <v>14.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>22.8</v>
+        <v>15.15</v>
       </c>
       <c r="D18" t="n">
-        <v>2.1</v>
+        <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>9.300000000000001</v>
+        <v>17.1</v>
       </c>
       <c r="F18" t="n">
-        <v>10</v>
+        <v>11.8</v>
       </c>
       <c r="G18" t="n">
-        <v>9.800000000000001</v>
+        <v>13.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18.5</v>
+        <v>23.04</v>
       </c>
       <c r="D19" t="n">
-        <v>3.2</v>
+        <v>2.13</v>
       </c>
       <c r="E19" t="n">
-        <v>8</v>
+        <v>13.2</v>
       </c>
       <c r="F19" t="n">
-        <v>8</v>
+        <v>13.2</v>
       </c>
       <c r="G19" t="n">
-        <v>8</v>
+        <v>13.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>19.03</v>
+        <v>27.43</v>
       </c>
       <c r="D20" t="n">
-        <v>1.59</v>
+        <v>2.29</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>13.2</v>
       </c>
       <c r="F20" t="n">
-        <v>8</v>
+        <v>11.8</v>
       </c>
       <c r="G20" t="n">
-        <v>8</v>
+        <v>12.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>23.15</v>
+        <v>14.18</v>
       </c>
       <c r="D21" t="n">
-        <v>1.89</v>
+        <v>1.16</v>
       </c>
       <c r="E21" t="n">
-        <v>5.3</v>
+        <v>10.5</v>
       </c>
       <c r="F21" t="n">
-        <v>6</v>
+        <v>11.8</v>
       </c>
       <c r="G21" t="n">
-        <v>5.8</v>
+        <v>11.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="22">
@@ -1086,220 +1086,220 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20.89</v>
+        <v>21.07</v>
       </c>
       <c r="D22" t="n">
-        <v>1.71</v>
+        <v>1.73</v>
       </c>
       <c r="E22" t="n">
-        <v>5.3</v>
+        <v>10.5</v>
       </c>
       <c r="F22" t="n">
-        <v>5.3</v>
+        <v>10.5</v>
       </c>
       <c r="G22" t="n">
-        <v>5.3</v>
+        <v>10.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>58.95</v>
+        <v>19.04</v>
       </c>
       <c r="D23" t="n">
-        <v>3.79</v>
+        <v>1.59</v>
       </c>
       <c r="E23" t="n">
-        <v>6.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>4.7</v>
+        <v>8.6</v>
       </c>
       <c r="G23" t="n">
-        <v>5.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>15.79</v>
+        <v>10.42</v>
       </c>
       <c r="D24" t="n">
-        <v>0.87</v>
+        <v>0.67</v>
       </c>
       <c r="E24" t="n">
         <v>5.3</v>
       </c>
       <c r="F24" t="n">
-        <v>3.3</v>
+        <v>3.9</v>
       </c>
       <c r="G24" t="n">
-        <v>3.9</v>
+        <v>4.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10.33</v>
+        <v>18.22</v>
       </c>
       <c r="D25" t="n">
-        <v>0.66</v>
+        <v>1.7</v>
       </c>
       <c r="E25" t="n">
-        <v>2.7</v>
+        <v>3.9</v>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>3.9</v>
       </c>
       <c r="G25" t="n">
-        <v>2.2</v>
+        <v>3.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18.12</v>
+        <v>19.74</v>
       </c>
       <c r="D26" t="n">
-        <v>1.69</v>
+        <v>3.27</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="G26" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>26.05</v>
+        <v>21.39</v>
       </c>
       <c r="D27" t="n">
-        <v>2.38</v>
+        <v>1.93</v>
       </c>
       <c r="E27" t="n">
-        <v>1.3</v>
+        <v>2.6</v>
       </c>
       <c r="F27" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="G27" t="n">
-        <v>1.3</v>
+        <v>2.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>19.72</v>
+        <v>20.77</v>
       </c>
       <c r="D28" t="n">
-        <v>3.26</v>
+        <v>1.53</v>
       </c>
       <c r="E28" t="n">
         <v>1.3</v>
       </c>
       <c r="F28" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="G28" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>21.36</v>
+        <v>15.59</v>
       </c>
       <c r="D29" t="n">
-        <v>1.93</v>
+        <v>0.86</v>
       </c>
       <c r="E29" t="n">
         <v>1.3</v>
@@ -1311,25 +1311,25 @@
         <v>1.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>29.64</v>
+        <v>25.74</v>
       </c>
       <c r="D30" t="n">
-        <v>2.25</v>
+        <v>2.35</v>
       </c>
       <c r="E30" t="n">
         <v>1.3</v>
@@ -1341,7 +1341,7 @@
         <v>1.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="31">
@@ -1356,10 +1356,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>31.04</v>
+        <v>30.52</v>
       </c>
       <c r="D31" t="n">
-        <v>3.35</v>
+        <v>3.3</v>
       </c>
       <c r="E31" t="n">
         <v>1.3</v>
@@ -1371,25 +1371,25 @@
         <v>1.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>20.85</v>
+        <v>29.35</v>
       </c>
       <c r="D32" t="n">
-        <v>1.53</v>
+        <v>2.23</v>
       </c>
       <c r="E32" t="n">
         <v>1.3</v>
@@ -1401,7 +1401,7 @@
         <v>1.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Jul 11 10:45:55 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>8.82</v>
       </c>
       <c r="E2" t="n">
-        <v>86.8</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>84.90000000000001</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>85.90000000000001</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.23</v>
       </c>
       <c r="E3" t="n">
-        <v>68.40000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="F3" t="n">
-        <v>69.09999999999999</v>
+        <v>68.8</v>
       </c>
       <c r="G3" t="n">
-        <v>68.8</v>
+        <v>68.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>1.24</v>
       </c>
       <c r="E4" t="n">
-        <v>55.9</v>
+        <v>55.8</v>
       </c>
       <c r="F4" t="n">
-        <v>55.3</v>
+        <v>55.2</v>
       </c>
       <c r="G4" t="n">
-        <v>55.6</v>
+        <v>55.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="5">
@@ -591,7 +591,7 @@
         <v>52.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="6">
@@ -618,10 +618,10 @@
         <v>51.3</v>
       </c>
       <c r="G6" t="n">
-        <v>52</v>
+        <v>51.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         <v>51.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="8">
@@ -675,13 +675,13 @@
         <v>47.4</v>
       </c>
       <c r="F8" t="n">
-        <v>48</v>
+        <v>48.1</v>
       </c>
       <c r="G8" t="n">
         <v>47.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="9">
@@ -705,13 +705,13 @@
         <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>40.8</v>
+        <v>40.9</v>
       </c>
       <c r="G9" t="n">
-        <v>45.4</v>
+        <v>45.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.98</v>
       </c>
       <c r="E10" t="n">
-        <v>36.8</v>
+        <v>37</v>
       </c>
       <c r="F10" t="n">
-        <v>36.8</v>
+        <v>37</v>
       </c>
       <c r="G10" t="n">
-        <v>36.8</v>
+        <v>37</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.01</v>
       </c>
       <c r="E11" t="n">
-        <v>34.2</v>
+        <v>34.4</v>
       </c>
       <c r="F11" t="n">
-        <v>27.6</v>
+        <v>27.9</v>
       </c>
       <c r="G11" t="n">
-        <v>29.6</v>
+        <v>29.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>0.63</v>
       </c>
       <c r="E12" t="n">
-        <v>25</v>
+        <v>25.3</v>
       </c>
       <c r="F12" t="n">
-        <v>21.7</v>
+        <v>22.1</v>
       </c>
       <c r="G12" t="n">
-        <v>22.7</v>
+        <v>23.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>17.1</v>
+        <v>17.5</v>
       </c>
       <c r="F13" t="n">
-        <v>21.1</v>
+        <v>21.4</v>
       </c>
       <c r="G13" t="n">
-        <v>19.9</v>
+        <v>20.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.93</v>
       </c>
       <c r="E14" t="n">
-        <v>21.1</v>
+        <v>21.4</v>
       </c>
       <c r="F14" t="n">
-        <v>19.1</v>
+        <v>19.5</v>
       </c>
       <c r="G14" t="n">
-        <v>19.7</v>
+        <v>20.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.56</v>
       </c>
       <c r="E15" t="n">
-        <v>17.1</v>
+        <v>17.5</v>
       </c>
       <c r="F15" t="n">
-        <v>17.8</v>
+        <v>18.2</v>
       </c>
       <c r="G15" t="n">
-        <v>17.6</v>
+        <v>18</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.15</v>
       </c>
       <c r="E16" t="n">
-        <v>15.8</v>
+        <v>16.2</v>
       </c>
       <c r="F16" t="n">
-        <v>15.8</v>
+        <v>16.2</v>
       </c>
       <c r="G16" t="n">
-        <v>15.8</v>
+        <v>16.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.21</v>
       </c>
       <c r="E17" t="n">
-        <v>17.1</v>
+        <v>17.5</v>
       </c>
       <c r="F17" t="n">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
       <c r="G17" t="n">
-        <v>14.3</v>
+        <v>14.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>17.1</v>
+        <v>17.5</v>
       </c>
       <c r="F18" t="n">
-        <v>11.8</v>
+        <v>12.3</v>
       </c>
       <c r="G18" t="n">
-        <v>13.4</v>
+        <v>13.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.13</v>
       </c>
       <c r="E19" t="n">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
       <c r="F19" t="n">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
       <c r="G19" t="n">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>2.29</v>
       </c>
       <c r="E20" t="n">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
       <c r="F20" t="n">
-        <v>11.8</v>
+        <v>12.3</v>
       </c>
       <c r="G20" t="n">
-        <v>12.2</v>
+        <v>12.7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.16</v>
       </c>
       <c r="E21" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="F21" t="n">
-        <v>11.8</v>
+        <v>12.3</v>
       </c>
       <c r="G21" t="n">
-        <v>11.4</v>
+        <v>11.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.73</v>
       </c>
       <c r="E22" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="F22" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="G22" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.59</v>
       </c>
       <c r="E23" t="n">
-        <v>9.199999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="G23" t="n">
-        <v>8.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>0.67</v>
       </c>
       <c r="E24" t="n">
-        <v>5.3</v>
+        <v>5.8</v>
       </c>
       <c r="F24" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="G24" t="n">
-        <v>4.3</v>
+        <v>4.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.7</v>
       </c>
       <c r="E25" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="F25" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="G25" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.27</v>
       </c>
       <c r="E26" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="F26" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="G26" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>1.93</v>
       </c>
       <c r="E27" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F27" t="n">
         <v>2.6</v>
       </c>
-      <c r="F27" t="n">
-        <v>2</v>
-      </c>
       <c r="G27" t="n">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.53</v>
       </c>
       <c r="E28" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="G28" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>0.86</v>
       </c>
       <c r="E29" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="F29" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="G29" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.35</v>
       </c>
       <c r="E30" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="F30" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="G30" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.3</v>
       </c>
       <c r="E31" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="F31" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="G31" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.23</v>
       </c>
       <c r="E32" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="F32" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="G32" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Jul 12 11:00:33 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>8.82</v>
       </c>
       <c r="E2" t="n">
-        <v>86.40000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>84.40000000000001</v>
+        <v>84</v>
       </c>
       <c r="G2" t="n">
-        <v>85.40000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.23</v>
       </c>
       <c r="E3" t="n">
-        <v>68.2</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>68.8</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>68.5</v>
+        <v>68.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="4">
@@ -555,13 +555,13 @@
         <v>55.8</v>
       </c>
       <c r="F4" t="n">
-        <v>55.2</v>
+        <v>55.1</v>
       </c>
       <c r="G4" t="n">
-        <v>55.5</v>
+        <v>55.4</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="5">
@@ -582,7 +582,7 @@
         <v>2.6</v>
       </c>
       <c r="E5" t="n">
-        <v>53.9</v>
+        <v>53.8</v>
       </c>
       <c r="F5" t="n">
         <v>51.3</v>
@@ -591,7 +591,7 @@
         <v>52.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="6">
@@ -621,7 +621,7 @@
         <v>51.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         <v>51.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="8">
@@ -678,10 +678,10 @@
         <v>48.1</v>
       </c>
       <c r="G8" t="n">
-        <v>47.7</v>
+        <v>47.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="9">
@@ -705,13 +705,13 @@
         <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>40.9</v>
+        <v>41</v>
       </c>
       <c r="G9" t="n">
         <v>45.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.98</v>
       </c>
       <c r="E10" t="n">
-        <v>37</v>
+        <v>37.2</v>
       </c>
       <c r="F10" t="n">
-        <v>37</v>
+        <v>37.2</v>
       </c>
       <c r="G10" t="n">
-        <v>37</v>
+        <v>37.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.01</v>
       </c>
       <c r="E11" t="n">
-        <v>34.4</v>
+        <v>34.6</v>
       </c>
       <c r="F11" t="n">
-        <v>27.9</v>
+        <v>28.2</v>
       </c>
       <c r="G11" t="n">
-        <v>29.9</v>
+        <v>30.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>0.63</v>
       </c>
       <c r="E12" t="n">
-        <v>25.3</v>
+        <v>25.6</v>
       </c>
       <c r="F12" t="n">
-        <v>22.1</v>
+        <v>22.4</v>
       </c>
       <c r="G12" t="n">
-        <v>23.1</v>
+        <v>23.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>17.5</v>
+        <v>17.9</v>
       </c>
       <c r="F13" t="n">
-        <v>21.4</v>
+        <v>21.8</v>
       </c>
       <c r="G13" t="n">
-        <v>20.3</v>
+        <v>20.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.93</v>
       </c>
       <c r="E14" t="n">
-        <v>21.4</v>
+        <v>21.8</v>
       </c>
       <c r="F14" t="n">
-        <v>19.5</v>
+        <v>19.9</v>
       </c>
       <c r="G14" t="n">
-        <v>20.1</v>
+        <v>20.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.56</v>
       </c>
       <c r="E15" t="n">
-        <v>17.5</v>
+        <v>17.9</v>
       </c>
       <c r="F15" t="n">
-        <v>18.2</v>
+        <v>18.6</v>
       </c>
       <c r="G15" t="n">
-        <v>18</v>
+        <v>18.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.15</v>
       </c>
       <c r="E16" t="n">
-        <v>16.2</v>
+        <v>16.7</v>
       </c>
       <c r="F16" t="n">
-        <v>16.2</v>
+        <v>16.7</v>
       </c>
       <c r="G16" t="n">
-        <v>16.2</v>
+        <v>16.7</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.21</v>
       </c>
       <c r="E17" t="n">
-        <v>17.5</v>
+        <v>17.9</v>
       </c>
       <c r="F17" t="n">
-        <v>13.6</v>
+        <v>14.1</v>
       </c>
       <c r="G17" t="n">
-        <v>14.8</v>
+        <v>15.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>17.5</v>
+        <v>17.9</v>
       </c>
       <c r="F18" t="n">
-        <v>12.3</v>
+        <v>12.8</v>
       </c>
       <c r="G18" t="n">
-        <v>13.9</v>
+        <v>14.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.13</v>
       </c>
       <c r="E19" t="n">
-        <v>13.6</v>
+        <v>14.1</v>
       </c>
       <c r="F19" t="n">
-        <v>13.6</v>
+        <v>14.1</v>
       </c>
       <c r="G19" t="n">
-        <v>13.6</v>
+        <v>14.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>2.29</v>
       </c>
       <c r="E20" t="n">
-        <v>13.6</v>
+        <v>14.1</v>
       </c>
       <c r="F20" t="n">
-        <v>12.3</v>
+        <v>12.8</v>
       </c>
       <c r="G20" t="n">
-        <v>12.7</v>
+        <v>13.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.16</v>
       </c>
       <c r="E21" t="n">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="F21" t="n">
-        <v>12.3</v>
+        <v>12.8</v>
       </c>
       <c r="G21" t="n">
-        <v>11.9</v>
+        <v>12.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.73</v>
       </c>
       <c r="E22" t="n">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="F22" t="n">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="G22" t="n">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.59</v>
       </c>
       <c r="E23" t="n">
-        <v>9.699999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="F23" t="n">
-        <v>9.1</v>
+        <v>9.6</v>
       </c>
       <c r="G23" t="n">
-        <v>9.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>0.67</v>
       </c>
       <c r="E24" t="n">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
       <c r="F24" t="n">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
       <c r="G24" t="n">
-        <v>4.9</v>
+        <v>5.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.7</v>
       </c>
       <c r="E25" t="n">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
       <c r="F25" t="n">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
       <c r="G25" t="n">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.27</v>
       </c>
       <c r="E26" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="F26" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="G26" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>1.93</v>
       </c>
       <c r="E27" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F27" t="n">
         <v>3.2</v>
       </c>
-      <c r="F27" t="n">
-        <v>2.6</v>
-      </c>
       <c r="G27" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.53</v>
       </c>
       <c r="E28" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="F28" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="G28" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>0.86</v>
       </c>
       <c r="E29" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="F29" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="G29" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.35</v>
       </c>
       <c r="E30" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="F30" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="G30" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.3</v>
       </c>
       <c r="E31" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="F31" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="G31" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.23</v>
       </c>
       <c r="E32" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="F32" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="G32" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Jul 13 12:23:04 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,82 +486,82 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>84.06999999999999</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>8.82</v>
+        <v>8.35</v>
       </c>
       <c r="E2" t="n">
-        <v>85.90000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>84</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>84.90000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>40.08</v>
+        <v>122.25</v>
       </c>
       <c r="D3" t="n">
-        <v>2.23</v>
+        <v>4.59</v>
       </c>
       <c r="E3" t="n">
-        <v>67.90000000000001</v>
+        <v>62</v>
       </c>
       <c r="F3" t="n">
-        <v>68.59999999999999</v>
+        <v>60.8</v>
       </c>
       <c r="G3" t="n">
-        <v>68.3</v>
+        <v>61.4</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.19</v>
+        <v>37.52</v>
       </c>
       <c r="D4" t="n">
-        <v>1.24</v>
+        <v>2.07</v>
       </c>
       <c r="E4" t="n">
-        <v>55.8</v>
+        <v>55.7</v>
       </c>
       <c r="F4" t="n">
-        <v>55.1</v>
+        <v>51.9</v>
       </c>
       <c r="G4" t="n">
-        <v>55.4</v>
+        <v>53.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="5">
@@ -576,412 +576,412 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28.37</v>
+        <v>28.21</v>
       </c>
       <c r="D5" t="n">
-        <v>2.6</v>
+        <v>2.59</v>
       </c>
       <c r="E5" t="n">
-        <v>53.8</v>
+        <v>49.4</v>
       </c>
       <c r="F5" t="n">
-        <v>51.3</v>
+        <v>45.6</v>
       </c>
       <c r="G5" t="n">
-        <v>52.6</v>
+        <v>47.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>41.73</v>
+        <v>6.81</v>
       </c>
       <c r="D6" t="n">
-        <v>3.53</v>
+        <v>0.64</v>
       </c>
       <c r="E6" t="n">
-        <v>52.6</v>
+        <v>52.5</v>
       </c>
       <c r="F6" t="n">
-        <v>51.3</v>
+        <v>39.9</v>
       </c>
       <c r="G6" t="n">
-        <v>51.9</v>
+        <v>46.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>120.82</v>
+        <v>10.13</v>
       </c>
       <c r="D7" t="n">
-        <v>4.53</v>
+        <v>1.23</v>
       </c>
       <c r="E7" t="n">
-        <v>51.3</v>
+        <v>44.3</v>
       </c>
       <c r="F7" t="n">
-        <v>51.3</v>
+        <v>47.5</v>
       </c>
       <c r="G7" t="n">
-        <v>51.3</v>
+        <v>45.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>61.65</v>
+        <v>27.11</v>
       </c>
       <c r="D8" t="n">
-        <v>3.96</v>
+        <v>2.01</v>
       </c>
       <c r="E8" t="n">
-        <v>47.4</v>
+        <v>32.3</v>
       </c>
       <c r="F8" t="n">
-        <v>48.1</v>
+        <v>28.5</v>
       </c>
       <c r="G8" t="n">
-        <v>47.8</v>
+        <v>29.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>48.59</v>
+        <v>30.86</v>
       </c>
       <c r="D9" t="n">
-        <v>3.98</v>
+        <v>2.92</v>
       </c>
       <c r="E9" t="n">
-        <v>50</v>
+        <v>25.3</v>
       </c>
       <c r="F9" t="n">
-        <v>41</v>
+        <v>25.3</v>
       </c>
       <c r="G9" t="n">
-        <v>45.5</v>
+        <v>25.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>31.45</v>
+        <v>12.59</v>
       </c>
       <c r="D10" t="n">
-        <v>2.98</v>
+        <v>1.18</v>
       </c>
       <c r="E10" t="n">
-        <v>37.2</v>
+        <v>22.8</v>
       </c>
       <c r="F10" t="n">
-        <v>37.2</v>
+        <v>22.8</v>
       </c>
       <c r="G10" t="n">
-        <v>37.2</v>
+        <v>22.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.17</v>
+        <v>16.96</v>
       </c>
       <c r="D11" t="n">
-        <v>2.01</v>
+        <v>1.57</v>
       </c>
       <c r="E11" t="n">
-        <v>34.6</v>
+        <v>22.8</v>
       </c>
       <c r="F11" t="n">
-        <v>28.2</v>
+        <v>22.2</v>
       </c>
       <c r="G11" t="n">
-        <v>30.1</v>
+        <v>22.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6.68</v>
+        <v>18.6</v>
       </c>
       <c r="D12" t="n">
-        <v>0.63</v>
+        <v>3.22</v>
       </c>
       <c r="E12" t="n">
-        <v>25.6</v>
+        <v>20.3</v>
       </c>
       <c r="F12" t="n">
-        <v>22.4</v>
+        <v>20.9</v>
       </c>
       <c r="G12" t="n">
-        <v>23.4</v>
+        <v>20.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.46</v>
+        <v>39.35</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9399999999999999</v>
+        <v>3.33</v>
       </c>
       <c r="E13" t="n">
-        <v>17.9</v>
+        <v>19</v>
       </c>
       <c r="F13" t="n">
-        <v>21.8</v>
+        <v>19</v>
       </c>
       <c r="G13" t="n">
-        <v>20.6</v>
+        <v>19</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>23.65</v>
+        <v>46.77</v>
       </c>
       <c r="D14" t="n">
-        <v>1.93</v>
+        <v>3.83</v>
       </c>
       <c r="E14" t="n">
-        <v>21.8</v>
+        <v>15.2</v>
       </c>
       <c r="F14" t="n">
-        <v>19.9</v>
+        <v>12.7</v>
       </c>
       <c r="G14" t="n">
-        <v>20.4</v>
+        <v>13.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>16.78</v>
+        <v>10.08</v>
       </c>
       <c r="D15" t="n">
-        <v>1.56</v>
+        <v>0.92</v>
       </c>
       <c r="E15" t="n">
-        <v>17.9</v>
+        <v>1.3</v>
       </c>
       <c r="F15" t="n">
-        <v>18.6</v>
+        <v>10.8</v>
       </c>
       <c r="G15" t="n">
-        <v>18.4</v>
+        <v>7.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>12.3</v>
+        <v>15.02</v>
       </c>
       <c r="D16" t="n">
-        <v>1.15</v>
+        <v>2.22</v>
       </c>
       <c r="E16" t="n">
-        <v>16.7</v>
+        <v>7.6</v>
       </c>
       <c r="F16" t="n">
-        <v>16.7</v>
+        <v>7</v>
       </c>
       <c r="G16" t="n">
-        <v>16.7</v>
+        <v>7.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>18.59</v>
+        <v>26.8</v>
       </c>
       <c r="D17" t="n">
-        <v>3.21</v>
+        <v>2.24</v>
       </c>
       <c r="E17" t="n">
-        <v>17.9</v>
+        <v>6.3</v>
       </c>
       <c r="F17" t="n">
-        <v>14.1</v>
+        <v>7</v>
       </c>
       <c r="G17" t="n">
-        <v>15.3</v>
+        <v>6.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>15.15</v>
+        <v>14.12</v>
       </c>
       <c r="D18" t="n">
-        <v>2.24</v>
+        <v>1.15</v>
       </c>
       <c r="E18" t="n">
-        <v>17.9</v>
+        <v>3.8</v>
       </c>
       <c r="F18" t="n">
-        <v>12.8</v>
+        <v>6.3</v>
       </c>
       <c r="G18" t="n">
-        <v>14.4</v>
+        <v>5.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="19">
@@ -996,412 +996,412 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>23.04</v>
+        <v>22.13</v>
       </c>
       <c r="D19" t="n">
-        <v>2.13</v>
+        <v>2.04</v>
       </c>
       <c r="E19" t="n">
-        <v>14.1</v>
+        <v>5.1</v>
       </c>
       <c r="F19" t="n">
-        <v>14.1</v>
+        <v>3.2</v>
       </c>
       <c r="G19" t="n">
-        <v>14.1</v>
+        <v>3.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>27.43</v>
+        <v>15.47</v>
       </c>
       <c r="D20" t="n">
-        <v>2.29</v>
+        <v>0.86</v>
       </c>
       <c r="E20" t="n">
-        <v>14.1</v>
+        <v>1.3</v>
       </c>
       <c r="F20" t="n">
-        <v>12.8</v>
+        <v>3.2</v>
       </c>
       <c r="G20" t="n">
-        <v>13.2</v>
+        <v>2.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>14.18</v>
+        <v>10.2</v>
       </c>
       <c r="D21" t="n">
-        <v>1.16</v>
+        <v>0.65</v>
       </c>
       <c r="E21" t="n">
-        <v>11.5</v>
+        <v>2.5</v>
       </c>
       <c r="F21" t="n">
-        <v>12.8</v>
+        <v>1.3</v>
       </c>
       <c r="G21" t="n">
-        <v>12.4</v>
+        <v>1.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21.07</v>
+        <v>57.95</v>
       </c>
       <c r="D22" t="n">
-        <v>1.73</v>
+        <v>3.72</v>
       </c>
       <c r="E22" t="n">
-        <v>11.5</v>
+        <v>2.5</v>
       </c>
       <c r="F22" t="n">
-        <v>11.5</v>
+        <v>1.3</v>
       </c>
       <c r="G22" t="n">
-        <v>11.5</v>
+        <v>1.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>19.04</v>
+        <v>24.76</v>
       </c>
       <c r="D23" t="n">
-        <v>1.59</v>
+        <v>2.27</v>
       </c>
       <c r="E23" t="n">
-        <v>10.3</v>
+        <v>1.3</v>
       </c>
       <c r="F23" t="n">
-        <v>9.6</v>
+        <v>1.3</v>
       </c>
       <c r="G23" t="n">
-        <v>9.800000000000001</v>
+        <v>1.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10.42</v>
+        <v>18.98</v>
       </c>
       <c r="D24" t="n">
-        <v>0.67</v>
+        <v>3.14</v>
       </c>
       <c r="E24" t="n">
-        <v>6.4</v>
+        <v>1.3</v>
       </c>
       <c r="F24" t="n">
-        <v>5.1</v>
+        <v>1.3</v>
       </c>
       <c r="G24" t="n">
-        <v>5.5</v>
+        <v>1.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>18.22</v>
+        <v>20.49</v>
       </c>
       <c r="D25" t="n">
-        <v>1.7</v>
+        <v>1.68</v>
       </c>
       <c r="E25" t="n">
-        <v>5.1</v>
+        <v>1.3</v>
       </c>
       <c r="F25" t="n">
-        <v>5.1</v>
+        <v>1.3</v>
       </c>
       <c r="G25" t="n">
-        <v>5.1</v>
+        <v>1.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>19.74</v>
+        <v>18.07</v>
       </c>
       <c r="D26" t="n">
-        <v>3.27</v>
+        <v>1.68</v>
       </c>
       <c r="E26" t="n">
-        <v>3.8</v>
+        <v>1.3</v>
       </c>
       <c r="F26" t="n">
-        <v>3.8</v>
+        <v>1.3</v>
       </c>
       <c r="G26" t="n">
-        <v>3.8</v>
+        <v>1.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>21.39</v>
+        <v>18.65</v>
       </c>
       <c r="D27" t="n">
-        <v>1.93</v>
+        <v>1.56</v>
       </c>
       <c r="E27" t="n">
-        <v>3.8</v>
+        <v>1.3</v>
       </c>
       <c r="F27" t="n">
-        <v>3.2</v>
+        <v>1.3</v>
       </c>
       <c r="G27" t="n">
-        <v>3.4</v>
+        <v>1.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>20.77</v>
+        <v>20.65</v>
       </c>
       <c r="D28" t="n">
-        <v>1.53</v>
+        <v>1.87</v>
       </c>
       <c r="E28" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="F28" t="n">
-        <v>3.2</v>
+        <v>1.3</v>
       </c>
       <c r="G28" t="n">
-        <v>3</v>
+        <v>1.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>15.59</v>
+        <v>29.54</v>
       </c>
       <c r="D29" t="n">
-        <v>0.86</v>
+        <v>3.19</v>
       </c>
       <c r="E29" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="F29" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="G29" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>25.74</v>
+        <v>28.13</v>
       </c>
       <c r="D30" t="n">
-        <v>2.35</v>
+        <v>2.14</v>
       </c>
       <c r="E30" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="F30" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="G30" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>30.52</v>
+        <v>22.79</v>
       </c>
       <c r="D31" t="n">
-        <v>3.3</v>
+        <v>1.86</v>
       </c>
       <c r="E31" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="F31" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="G31" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>29.35</v>
+        <v>20.08</v>
       </c>
       <c r="D32" t="n">
-        <v>2.23</v>
+        <v>1.47</v>
       </c>
       <c r="E32" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="F32" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="G32" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Jul 14 11:12:19 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,232 +486,232 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>79.59999999999999</v>
+        <v>81.52</v>
       </c>
       <c r="D2" t="n">
-        <v>8.35</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>68.40000000000001</v>
+        <v>70</v>
       </c>
       <c r="F2" t="n">
-        <v>68.40000000000001</v>
+        <v>70</v>
       </c>
       <c r="G2" t="n">
-        <v>68.40000000000001</v>
+        <v>70</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>122.25</v>
+        <v>28.9</v>
       </c>
       <c r="D3" t="n">
-        <v>4.59</v>
+        <v>2.66</v>
       </c>
       <c r="E3" t="n">
-        <v>62</v>
+        <v>68.8</v>
       </c>
       <c r="F3" t="n">
-        <v>60.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>61.4</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37.52</v>
+        <v>124.23</v>
       </c>
       <c r="D4" t="n">
-        <v>2.07</v>
+        <v>4.66</v>
       </c>
       <c r="E4" t="n">
-        <v>55.7</v>
+        <v>66.2</v>
       </c>
       <c r="F4" t="n">
-        <v>51.9</v>
+        <v>66.2</v>
       </c>
       <c r="G4" t="n">
-        <v>53.8</v>
+        <v>66.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28.21</v>
+        <v>39.89</v>
       </c>
       <c r="D5" t="n">
-        <v>2.59</v>
+        <v>2.21</v>
       </c>
       <c r="E5" t="n">
-        <v>49.4</v>
+        <v>66.2</v>
       </c>
       <c r="F5" t="n">
-        <v>45.6</v>
+        <v>66.2</v>
       </c>
       <c r="G5" t="n">
-        <v>47.5</v>
+        <v>66.2</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6.81</v>
+        <v>10.23</v>
       </c>
       <c r="D6" t="n">
-        <v>0.64</v>
+        <v>1.24</v>
       </c>
       <c r="E6" t="n">
-        <v>52.5</v>
+        <v>63.1</v>
       </c>
       <c r="F6" t="n">
-        <v>39.9</v>
+        <v>55.6</v>
       </c>
       <c r="G6" t="n">
-        <v>46.2</v>
+        <v>59.4</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10.13</v>
+        <v>31.93</v>
       </c>
       <c r="D7" t="n">
-        <v>1.23</v>
+        <v>3.02</v>
       </c>
       <c r="E7" t="n">
-        <v>44.3</v>
+        <v>50</v>
       </c>
       <c r="F7" t="n">
-        <v>47.5</v>
+        <v>50</v>
       </c>
       <c r="G7" t="n">
-        <v>45.9</v>
+        <v>50</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>27.11</v>
+        <v>6.78</v>
       </c>
       <c r="D8" t="n">
-        <v>2.01</v>
+        <v>0.64</v>
       </c>
       <c r="E8" t="n">
-        <v>32.3</v>
+        <v>46.2</v>
       </c>
       <c r="F8" t="n">
-        <v>28.5</v>
+        <v>40</v>
       </c>
       <c r="G8" t="n">
-        <v>29.6</v>
+        <v>43.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30.86</v>
+        <v>17.49</v>
       </c>
       <c r="D9" t="n">
-        <v>2.92</v>
+        <v>1.62</v>
       </c>
       <c r="E9" t="n">
-        <v>25.3</v>
+        <v>33.8</v>
       </c>
       <c r="F9" t="n">
-        <v>25.3</v>
+        <v>33.8</v>
       </c>
       <c r="G9" t="n">
-        <v>25.3</v>
+        <v>33.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="10">
@@ -726,52 +726,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>12.59</v>
+        <v>13.02</v>
       </c>
       <c r="D10" t="n">
-        <v>1.18</v>
+        <v>1.23</v>
       </c>
       <c r="E10" t="n">
-        <v>22.8</v>
+        <v>32.5</v>
       </c>
       <c r="F10" t="n">
-        <v>22.8</v>
+        <v>33.1</v>
       </c>
       <c r="G10" t="n">
-        <v>22.8</v>
+        <v>32.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16.96</v>
+        <v>27.21</v>
       </c>
       <c r="D11" t="n">
-        <v>1.57</v>
+        <v>2.01</v>
       </c>
       <c r="E11" t="n">
-        <v>22.8</v>
+        <v>37.5</v>
       </c>
       <c r="F11" t="n">
-        <v>22.2</v>
+        <v>28.7</v>
       </c>
       <c r="G11" t="n">
-        <v>22.3</v>
+        <v>31.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="12">
@@ -786,502 +786,502 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>18.6</v>
+        <v>18.69</v>
       </c>
       <c r="D12" t="n">
-        <v>3.22</v>
+        <v>3.23</v>
       </c>
       <c r="E12" t="n">
-        <v>20.3</v>
+        <v>23.1</v>
       </c>
       <c r="F12" t="n">
-        <v>20.9</v>
+        <v>23.1</v>
       </c>
       <c r="G12" t="n">
-        <v>20.7</v>
+        <v>23.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>39.35</v>
+        <v>14.36</v>
       </c>
       <c r="D13" t="n">
-        <v>3.33</v>
+        <v>1.17</v>
       </c>
       <c r="E13" t="n">
-        <v>19</v>
+        <v>21.2</v>
       </c>
       <c r="F13" t="n">
-        <v>19</v>
+        <v>21.9</v>
       </c>
       <c r="G13" t="n">
-        <v>19</v>
+        <v>21.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>46.77</v>
+        <v>40.27</v>
       </c>
       <c r="D14" t="n">
-        <v>3.83</v>
+        <v>3.41</v>
       </c>
       <c r="E14" t="n">
-        <v>15.2</v>
+        <v>20</v>
       </c>
       <c r="F14" t="n">
-        <v>12.7</v>
+        <v>21.2</v>
       </c>
       <c r="G14" t="n">
-        <v>13.4</v>
+        <v>20.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10.08</v>
+        <v>15.15</v>
       </c>
       <c r="D15" t="n">
-        <v>0.92</v>
+        <v>2.24</v>
       </c>
       <c r="E15" t="n">
-        <v>1.3</v>
+        <v>19.4</v>
       </c>
       <c r="F15" t="n">
-        <v>10.8</v>
+        <v>14.4</v>
       </c>
       <c r="G15" t="n">
-        <v>7.9</v>
+        <v>15.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15.02</v>
+        <v>15.8</v>
       </c>
       <c r="D16" t="n">
-        <v>2.22</v>
+        <v>0.88</v>
       </c>
       <c r="E16" t="n">
-        <v>7.6</v>
+        <v>11.9</v>
       </c>
       <c r="F16" t="n">
-        <v>7</v>
+        <v>13.1</v>
       </c>
       <c r="G16" t="n">
-        <v>7.2</v>
+        <v>12.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>26.8</v>
+        <v>46.34</v>
       </c>
       <c r="D17" t="n">
-        <v>2.24</v>
+        <v>3.8</v>
       </c>
       <c r="E17" t="n">
-        <v>6.3</v>
+        <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>6.8</v>
+        <v>10.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>14.12</v>
+        <v>18.99</v>
       </c>
       <c r="D18" t="n">
-        <v>1.15</v>
+        <v>1.59</v>
       </c>
       <c r="E18" t="n">
-        <v>3.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>6.3</v>
+        <v>11.2</v>
       </c>
       <c r="G18" t="n">
-        <v>5.6</v>
+        <v>10.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22.13</v>
+        <v>27.11</v>
       </c>
       <c r="D19" t="n">
-        <v>2.04</v>
+        <v>2.26</v>
       </c>
       <c r="E19" t="n">
-        <v>5.1</v>
+        <v>11.2</v>
       </c>
       <c r="F19" t="n">
-        <v>3.2</v>
+        <v>10</v>
       </c>
       <c r="G19" t="n">
-        <v>3.7</v>
+        <v>10.4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>15.47</v>
+        <v>10.17</v>
       </c>
       <c r="D20" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="E20" t="n">
-        <v>1.3</v>
+        <v>8.1</v>
       </c>
       <c r="F20" t="n">
-        <v>3.2</v>
+        <v>11.2</v>
       </c>
       <c r="G20" t="n">
-        <v>2.6</v>
+        <v>10.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10.2</v>
+        <v>22.5</v>
       </c>
       <c r="D21" t="n">
-        <v>0.65</v>
+        <v>2.07</v>
       </c>
       <c r="E21" t="n">
-        <v>2.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>1.3</v>
+        <v>8.1</v>
       </c>
       <c r="G21" t="n">
-        <v>1.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>57.95</v>
+        <v>20</v>
       </c>
       <c r="D22" t="n">
-        <v>3.72</v>
+        <v>3.31</v>
       </c>
       <c r="E22" t="n">
-        <v>2.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>1.3</v>
+        <v>7.5</v>
       </c>
       <c r="G22" t="n">
-        <v>1.6</v>
+        <v>7.9</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24.76</v>
+        <v>18.25</v>
       </c>
       <c r="D23" t="n">
-        <v>2.27</v>
+        <v>1.7</v>
       </c>
       <c r="E23" t="n">
-        <v>1.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>1.3</v>
+        <v>6.9</v>
       </c>
       <c r="G23" t="n">
-        <v>1.3</v>
+        <v>7.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>18.98</v>
+        <v>20.72</v>
       </c>
       <c r="D24" t="n">
-        <v>3.14</v>
+        <v>1.7</v>
       </c>
       <c r="E24" t="n">
-        <v>1.3</v>
+        <v>6.2</v>
       </c>
       <c r="F24" t="n">
-        <v>1.3</v>
+        <v>4.4</v>
       </c>
       <c r="G24" t="n">
-        <v>1.3</v>
+        <v>4.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20.49</v>
+        <v>10.33</v>
       </c>
       <c r="D25" t="n">
-        <v>1.68</v>
+        <v>0.66</v>
       </c>
       <c r="E25" t="n">
-        <v>1.3</v>
+        <v>4.4</v>
       </c>
       <c r="F25" t="n">
-        <v>1.3</v>
+        <v>3.8</v>
       </c>
       <c r="G25" t="n">
-        <v>1.3</v>
+        <v>3.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18.07</v>
+        <v>25.35</v>
       </c>
       <c r="D26" t="n">
-        <v>1.68</v>
+        <v>2.32</v>
       </c>
       <c r="E26" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="F26" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="G26" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18.65</v>
+        <v>20.94</v>
       </c>
       <c r="D27" t="n">
-        <v>1.56</v>
+        <v>1.89</v>
       </c>
       <c r="E27" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="F27" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="G27" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>20.65</v>
+        <v>28.59</v>
       </c>
       <c r="D28" t="n">
-        <v>1.87</v>
+        <v>2.17</v>
       </c>
       <c r="E28" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="F28" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="G28" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="29">
@@ -1296,52 +1296,52 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>29.54</v>
+        <v>30.02</v>
       </c>
       <c r="D29" t="n">
-        <v>3.19</v>
+        <v>3.24</v>
       </c>
       <c r="E29" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="F29" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="G29" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>28.13</v>
+        <v>20.53</v>
       </c>
       <c r="D30" t="n">
-        <v>2.14</v>
+        <v>1.51</v>
       </c>
       <c r="E30" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="F30" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="G30" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="31">
@@ -1356,52 +1356,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22.79</v>
+        <v>22.57</v>
       </c>
       <c r="D31" t="n">
-        <v>1.86</v>
+        <v>1.85</v>
       </c>
       <c r="E31" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="F31" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="G31" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>20.08</v>
+        <v>56.3</v>
       </c>
       <c r="D32" t="n">
-        <v>1.47</v>
+        <v>3.62</v>
       </c>
       <c r="E32" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="F32" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="G32" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Jul 15 11:16:00 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,31 +477,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>81.52</v>
+        <v>10.54</v>
       </c>
       <c r="D2" t="n">
-        <v>8.550000000000001</v>
+        <v>1.28</v>
       </c>
       <c r="E2" t="n">
-        <v>70</v>
+        <v>87.7</v>
       </c>
       <c r="F2" t="n">
-        <v>70</v>
+        <v>77.2</v>
       </c>
       <c r="G2" t="n">
-        <v>70</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="3">
@@ -516,52 +516,52 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.9</v>
+        <v>29.85</v>
       </c>
       <c r="D3" t="n">
-        <v>2.66</v>
+        <v>2.74</v>
       </c>
       <c r="E3" t="n">
-        <v>68.8</v>
+        <v>77.8</v>
       </c>
       <c r="F3" t="n">
-        <v>69.40000000000001</v>
+        <v>84</v>
       </c>
       <c r="G3" t="n">
-        <v>69.09999999999999</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>124.23</v>
+        <v>77.78</v>
       </c>
       <c r="D4" t="n">
-        <v>4.66</v>
+        <v>8.16</v>
       </c>
       <c r="E4" t="n">
-        <v>66.2</v>
+        <v>66.7</v>
       </c>
       <c r="F4" t="n">
-        <v>66.2</v>
+        <v>66.7</v>
       </c>
       <c r="G4" t="n">
-        <v>66.2</v>
+        <v>66.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="5">
@@ -576,292 +576,292 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>39.89</v>
+        <v>38.74</v>
       </c>
       <c r="D5" t="n">
-        <v>2.21</v>
+        <v>2.15</v>
       </c>
       <c r="E5" t="n">
-        <v>66.2</v>
+        <v>64.2</v>
       </c>
       <c r="F5" t="n">
-        <v>66.2</v>
+        <v>62.3</v>
       </c>
       <c r="G5" t="n">
-        <v>66.2</v>
+        <v>63.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.23</v>
+        <v>6.82</v>
       </c>
       <c r="D6" t="n">
-        <v>1.24</v>
+        <v>0.65</v>
       </c>
       <c r="E6" t="n">
-        <v>63.1</v>
+        <v>54.9</v>
       </c>
       <c r="F6" t="n">
-        <v>55.6</v>
+        <v>63</v>
       </c>
       <c r="G6" t="n">
-        <v>59.4</v>
+        <v>59</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>31.93</v>
+        <v>121.45</v>
       </c>
       <c r="D7" t="n">
-        <v>3.02</v>
+        <v>4.56</v>
       </c>
       <c r="E7" t="n">
-        <v>50</v>
+        <v>53.1</v>
       </c>
       <c r="F7" t="n">
-        <v>50</v>
+        <v>54.3</v>
       </c>
       <c r="G7" t="n">
-        <v>50</v>
+        <v>53.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.78</v>
+        <v>27.95</v>
       </c>
       <c r="D8" t="n">
-        <v>0.64</v>
+        <v>2.07</v>
       </c>
       <c r="E8" t="n">
-        <v>46.2</v>
+        <v>51.9</v>
       </c>
       <c r="F8" t="n">
-        <v>40</v>
+        <v>47.5</v>
       </c>
       <c r="G8" t="n">
-        <v>43.1</v>
+        <v>49.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>17.49</v>
+        <v>31.73</v>
       </c>
       <c r="D9" t="n">
-        <v>1.62</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>33.8</v>
+        <v>49.4</v>
       </c>
       <c r="F9" t="n">
-        <v>33.8</v>
+        <v>47.5</v>
       </c>
       <c r="G9" t="n">
-        <v>33.8</v>
+        <v>48.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>13.02</v>
+        <v>17.69</v>
       </c>
       <c r="D10" t="n">
-        <v>1.23</v>
+        <v>1.64</v>
       </c>
       <c r="E10" t="n">
-        <v>32.5</v>
+        <v>34.6</v>
       </c>
       <c r="F10" t="n">
-        <v>33.1</v>
+        <v>36.4</v>
       </c>
       <c r="G10" t="n">
-        <v>32.8</v>
+        <v>35.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.21</v>
+        <v>19.34</v>
       </c>
       <c r="D11" t="n">
-        <v>2.01</v>
+        <v>3.34</v>
       </c>
       <c r="E11" t="n">
-        <v>37.5</v>
+        <v>34.6</v>
       </c>
       <c r="F11" t="n">
-        <v>28.7</v>
+        <v>34.6</v>
       </c>
       <c r="G11" t="n">
-        <v>31.4</v>
+        <v>34.6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>18.69</v>
+        <v>28.19</v>
       </c>
       <c r="D12" t="n">
-        <v>3.23</v>
+        <v>2.35</v>
       </c>
       <c r="E12" t="n">
-        <v>23.1</v>
+        <v>37.7</v>
       </c>
       <c r="F12" t="n">
-        <v>23.1</v>
+        <v>30.9</v>
       </c>
       <c r="G12" t="n">
-        <v>23.1</v>
+        <v>34.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14.36</v>
+        <v>13.01</v>
       </c>
       <c r="D13" t="n">
-        <v>1.17</v>
+        <v>1.22</v>
       </c>
       <c r="E13" t="n">
-        <v>21.2</v>
+        <v>32.1</v>
       </c>
       <c r="F13" t="n">
-        <v>21.9</v>
+        <v>31.5</v>
       </c>
       <c r="G13" t="n">
-        <v>21.7</v>
+        <v>31.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>40.27</v>
+        <v>14.5</v>
       </c>
       <c r="D14" t="n">
-        <v>3.41</v>
+        <v>1.18</v>
       </c>
       <c r="E14" t="n">
-        <v>20</v>
+        <v>28.4</v>
       </c>
       <c r="F14" t="n">
-        <v>21.2</v>
+        <v>28.4</v>
       </c>
       <c r="G14" t="n">
-        <v>20.9</v>
+        <v>28.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="15">
@@ -876,292 +876,292 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>15.15</v>
+        <v>15.32</v>
       </c>
       <c r="D15" t="n">
-        <v>2.24</v>
+        <v>2.27</v>
       </c>
       <c r="E15" t="n">
-        <v>19.4</v>
+        <v>27.8</v>
       </c>
       <c r="F15" t="n">
-        <v>14.4</v>
+        <v>24.7</v>
       </c>
       <c r="G15" t="n">
-        <v>15.9</v>
+        <v>25.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15.8</v>
+        <v>10.38</v>
       </c>
       <c r="D16" t="n">
-        <v>0.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>11.9</v>
+        <v>14.8</v>
       </c>
       <c r="F16" t="n">
-        <v>13.1</v>
+        <v>24.1</v>
       </c>
       <c r="G16" t="n">
-        <v>12.8</v>
+        <v>21.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>46.34</v>
+        <v>39.7</v>
       </c>
       <c r="D17" t="n">
-        <v>3.8</v>
+        <v>3.36</v>
       </c>
       <c r="E17" t="n">
-        <v>15</v>
+        <v>19.8</v>
       </c>
       <c r="F17" t="n">
-        <v>8.800000000000001</v>
+        <v>19.8</v>
       </c>
       <c r="G17" t="n">
-        <v>10.6</v>
+        <v>19.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>18.99</v>
+        <v>21.5</v>
       </c>
       <c r="D18" t="n">
-        <v>1.59</v>
+        <v>1.76</v>
       </c>
       <c r="E18" t="n">
-        <v>8.800000000000001</v>
+        <v>18.5</v>
       </c>
       <c r="F18" t="n">
-        <v>11.2</v>
+        <v>17.9</v>
       </c>
       <c r="G18" t="n">
-        <v>10.5</v>
+        <v>18.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>27.11</v>
+        <v>23.46</v>
       </c>
       <c r="D19" t="n">
-        <v>2.26</v>
+        <v>1.92</v>
       </c>
       <c r="E19" t="n">
-        <v>11.2</v>
+        <v>17.3</v>
       </c>
       <c r="F19" t="n">
-        <v>10</v>
+        <v>17.9</v>
       </c>
       <c r="G19" t="n">
-        <v>10.4</v>
+        <v>17.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>10.17</v>
+        <v>19.23</v>
       </c>
       <c r="D20" t="n">
-        <v>0.92</v>
+        <v>1.6</v>
       </c>
       <c r="E20" t="n">
-        <v>8.1</v>
+        <v>17.3</v>
       </c>
       <c r="F20" t="n">
-        <v>11.2</v>
+        <v>15.4</v>
       </c>
       <c r="G20" t="n">
-        <v>10.3</v>
+        <v>16</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>22.5</v>
+        <v>16.15</v>
       </c>
       <c r="D21" t="n">
-        <v>2.07</v>
+        <v>0.89</v>
       </c>
       <c r="E21" t="n">
-        <v>8.800000000000001</v>
+        <v>16</v>
       </c>
       <c r="F21" t="n">
-        <v>8.1</v>
+        <v>16</v>
       </c>
       <c r="G21" t="n">
-        <v>8.300000000000001</v>
+        <v>16</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20</v>
+        <v>22.67</v>
       </c>
       <c r="D22" t="n">
-        <v>3.31</v>
+        <v>2.1</v>
       </c>
       <c r="E22" t="n">
-        <v>8.800000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="F22" t="n">
-        <v>7.5</v>
+        <v>12.3</v>
       </c>
       <c r="G22" t="n">
-        <v>7.9</v>
+        <v>11.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>18.25</v>
+        <v>46.4</v>
       </c>
       <c r="D23" t="n">
-        <v>1.7</v>
+        <v>3.8</v>
       </c>
       <c r="E23" t="n">
-        <v>8.800000000000001</v>
+        <v>16</v>
       </c>
       <c r="F23" t="n">
-        <v>6.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>7.4</v>
+        <v>11.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>20.72</v>
+        <v>18.37</v>
       </c>
       <c r="D24" t="n">
-        <v>1.7</v>
+        <v>1.71</v>
       </c>
       <c r="E24" t="n">
-        <v>6.2</v>
+        <v>11.1</v>
       </c>
       <c r="F24" t="n">
-        <v>4.4</v>
+        <v>10.5</v>
       </c>
       <c r="G24" t="n">
-        <v>4.9</v>
+        <v>10.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="25">
@@ -1176,52 +1176,52 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10.33</v>
+        <v>10.39</v>
       </c>
       <c r="D25" t="n">
         <v>0.66</v>
       </c>
       <c r="E25" t="n">
-        <v>4.4</v>
+        <v>7.4</v>
       </c>
       <c r="F25" t="n">
-        <v>3.8</v>
+        <v>4.3</v>
       </c>
       <c r="G25" t="n">
-        <v>3.9</v>
+        <v>5.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25.35</v>
+        <v>28.99</v>
       </c>
       <c r="D26" t="n">
-        <v>2.32</v>
+        <v>2.2</v>
       </c>
       <c r="E26" t="n">
-        <v>2.5</v>
+        <v>3.7</v>
       </c>
       <c r="F26" t="n">
-        <v>2.5</v>
+        <v>3.7</v>
       </c>
       <c r="G26" t="n">
-        <v>2.5</v>
+        <v>3.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="27">
@@ -1236,70 +1236,70 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>20.94</v>
+        <v>21.19</v>
       </c>
       <c r="D27" t="n">
-        <v>1.89</v>
+        <v>1.92</v>
       </c>
       <c r="E27" t="n">
-        <v>2.5</v>
+        <v>3.7</v>
       </c>
       <c r="F27" t="n">
-        <v>2.5</v>
+        <v>3.7</v>
       </c>
       <c r="G27" t="n">
-        <v>2.5</v>
+        <v>3.7</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>28.59</v>
+        <v>20.59</v>
       </c>
       <c r="D28" t="n">
-        <v>2.17</v>
+        <v>1.51</v>
       </c>
       <c r="E28" t="n">
-        <v>2.5</v>
+        <v>3.7</v>
       </c>
       <c r="F28" t="n">
-        <v>2.5</v>
+        <v>3.1</v>
       </c>
       <c r="G28" t="n">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>30.02</v>
+        <v>25.23</v>
       </c>
       <c r="D29" t="n">
-        <v>3.24</v>
+        <v>2.31</v>
       </c>
       <c r="E29" t="n">
         <v>2.5</v>
@@ -1311,25 +1311,25 @@
         <v>2.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>20.53</v>
+        <v>19.65</v>
       </c>
       <c r="D30" t="n">
-        <v>1.51</v>
+        <v>3.25</v>
       </c>
       <c r="E30" t="n">
         <v>2.5</v>
@@ -1341,37 +1341,37 @@
         <v>2.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22.57</v>
+        <v>29.85</v>
       </c>
       <c r="D31" t="n">
-        <v>1.85</v>
+        <v>3.22</v>
       </c>
       <c r="E31" t="n">
-        <v>1.2</v>
+        <v>2.5</v>
       </c>
       <c r="F31" t="n">
-        <v>1.2</v>
+        <v>2.5</v>
       </c>
       <c r="G31" t="n">
-        <v>1.2</v>
+        <v>2.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="32">
@@ -1386,10 +1386,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>56.3</v>
+        <v>55.51</v>
       </c>
       <c r="D32" t="n">
-        <v>3.62</v>
+        <v>3.57</v>
       </c>
       <c r="E32" t="n">
         <v>1.2</v>
@@ -1401,7 +1401,7 @@
         <v>1.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Jul 16 11:22:03 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,61 +477,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.54</v>
+        <v>29.95</v>
       </c>
       <c r="D2" t="n">
-        <v>1.28</v>
+        <v>2.75</v>
       </c>
       <c r="E2" t="n">
-        <v>87.7</v>
+        <v>81.7</v>
       </c>
       <c r="F2" t="n">
-        <v>77.2</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>82.40000000000001</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>29.85</v>
+        <v>10.34</v>
       </c>
       <c r="D3" t="n">
-        <v>2.74</v>
+        <v>1.25</v>
       </c>
       <c r="E3" t="n">
-        <v>77.8</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>84</v>
+        <v>60.4</v>
       </c>
       <c r="G3" t="n">
-        <v>80.90000000000001</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="4">
@@ -546,262 +546,262 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>77.78</v>
+        <v>75.02</v>
       </c>
       <c r="D4" t="n">
-        <v>8.16</v>
+        <v>7.87</v>
       </c>
       <c r="E4" t="n">
-        <v>66.7</v>
+        <v>59.8</v>
       </c>
       <c r="F4" t="n">
-        <v>66.7</v>
+        <v>60.4</v>
       </c>
       <c r="G4" t="n">
-        <v>66.7</v>
+        <v>60.1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>38.74</v>
+        <v>28.38</v>
       </c>
       <c r="D5" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="E5" t="n">
-        <v>64.2</v>
+        <v>56.1</v>
       </c>
       <c r="F5" t="n">
-        <v>62.3</v>
+        <v>51.2</v>
       </c>
       <c r="G5" t="n">
-        <v>63.3</v>
+        <v>53.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6.82</v>
+        <v>36.72</v>
       </c>
       <c r="D6" t="n">
-        <v>0.65</v>
+        <v>2.04</v>
       </c>
       <c r="E6" t="n">
-        <v>54.9</v>
+        <v>47.6</v>
       </c>
       <c r="F6" t="n">
-        <v>63</v>
+        <v>44.5</v>
       </c>
       <c r="G6" t="n">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>121.45</v>
+        <v>28.5</v>
       </c>
       <c r="D7" t="n">
-        <v>4.56</v>
+        <v>2.38</v>
       </c>
       <c r="E7" t="n">
-        <v>53.1</v>
+        <v>41.5</v>
       </c>
       <c r="F7" t="n">
-        <v>54.3</v>
+        <v>37.8</v>
       </c>
       <c r="G7" t="n">
-        <v>53.7</v>
+        <v>39.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>27.95</v>
+        <v>19.4</v>
       </c>
       <c r="D8" t="n">
-        <v>2.07</v>
+        <v>3.36</v>
       </c>
       <c r="E8" t="n">
-        <v>51.9</v>
+        <v>35.4</v>
       </c>
       <c r="F8" t="n">
-        <v>47.5</v>
+        <v>36</v>
       </c>
       <c r="G8" t="n">
-        <v>49.7</v>
+        <v>35.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>31.73</v>
+        <v>6.72</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>0.64</v>
       </c>
       <c r="E9" t="n">
-        <v>49.4</v>
+        <v>29.3</v>
       </c>
       <c r="F9" t="n">
-        <v>47.5</v>
+        <v>39.6</v>
       </c>
       <c r="G9" t="n">
-        <v>48.5</v>
+        <v>34.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>17.69</v>
+        <v>117.72</v>
       </c>
       <c r="D10" t="n">
-        <v>1.64</v>
+        <v>4.42</v>
       </c>
       <c r="E10" t="n">
-        <v>34.6</v>
+        <v>34.1</v>
       </c>
       <c r="F10" t="n">
-        <v>36.4</v>
+        <v>34.1</v>
       </c>
       <c r="G10" t="n">
-        <v>35.5</v>
+        <v>34.1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.34</v>
+        <v>17.32</v>
       </c>
       <c r="D11" t="n">
-        <v>3.34</v>
+        <v>1.6</v>
       </c>
       <c r="E11" t="n">
-        <v>34.6</v>
+        <v>31.7</v>
       </c>
       <c r="F11" t="n">
-        <v>34.6</v>
+        <v>31.1</v>
       </c>
       <c r="G11" t="n">
-        <v>34.6</v>
+        <v>31.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>28.19</v>
+        <v>10.56</v>
       </c>
       <c r="D12" t="n">
-        <v>2.35</v>
+        <v>0.95</v>
       </c>
       <c r="E12" t="n">
-        <v>37.7</v>
+        <v>26.8</v>
       </c>
       <c r="F12" t="n">
-        <v>30.9</v>
+        <v>31.7</v>
       </c>
       <c r="G12" t="n">
-        <v>34.3</v>
+        <v>29.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="13">
@@ -816,232 +816,232 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>13.01</v>
+        <v>12.84</v>
       </c>
       <c r="D13" t="n">
-        <v>1.22</v>
+        <v>1.21</v>
       </c>
       <c r="E13" t="n">
-        <v>32.1</v>
+        <v>30.5</v>
       </c>
       <c r="F13" t="n">
-        <v>31.5</v>
+        <v>28</v>
       </c>
       <c r="G13" t="n">
-        <v>31.8</v>
+        <v>28.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14.5</v>
+        <v>30.97</v>
       </c>
       <c r="D14" t="n">
-        <v>1.18</v>
+        <v>2.93</v>
       </c>
       <c r="E14" t="n">
-        <v>28.4</v>
+        <v>28</v>
       </c>
       <c r="F14" t="n">
-        <v>28.4</v>
+        <v>26.8</v>
       </c>
       <c r="G14" t="n">
-        <v>28.4</v>
+        <v>27.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>15.32</v>
+        <v>21.64</v>
       </c>
       <c r="D15" t="n">
-        <v>2.27</v>
+        <v>1.78</v>
       </c>
       <c r="E15" t="n">
-        <v>27.8</v>
+        <v>26.8</v>
       </c>
       <c r="F15" t="n">
-        <v>24.7</v>
+        <v>26.8</v>
       </c>
       <c r="G15" t="n">
-        <v>25.6</v>
+        <v>26.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.38</v>
+        <v>23.7</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.94</v>
       </c>
       <c r="E16" t="n">
-        <v>14.8</v>
+        <v>26.8</v>
       </c>
       <c r="F16" t="n">
-        <v>24.1</v>
+        <v>26.8</v>
       </c>
       <c r="G16" t="n">
-        <v>21.3</v>
+        <v>26.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>39.7</v>
+        <v>14.34</v>
       </c>
       <c r="D17" t="n">
-        <v>3.36</v>
+        <v>1.17</v>
       </c>
       <c r="E17" t="n">
-        <v>19.8</v>
+        <v>20.7</v>
       </c>
       <c r="F17" t="n">
-        <v>19.8</v>
+        <v>22</v>
       </c>
       <c r="G17" t="n">
-        <v>19.8</v>
+        <v>21.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C18" t="n">
+        <v>19.27</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="E18" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="G18" t="n">
         <v>21.5</v>
       </c>
-      <c r="D18" t="n">
-        <v>1.76</v>
-      </c>
-      <c r="E18" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="F18" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="G18" t="n">
-        <v>18.1</v>
-      </c>
       <c r="H18" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>23.46</v>
+        <v>15.24</v>
       </c>
       <c r="D19" t="n">
-        <v>1.92</v>
+        <v>2.25</v>
       </c>
       <c r="E19" t="n">
-        <v>17.3</v>
+        <v>25</v>
       </c>
       <c r="F19" t="n">
-        <v>17.9</v>
+        <v>19.5</v>
       </c>
       <c r="G19" t="n">
-        <v>17.7</v>
+        <v>21.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>19.23</v>
+        <v>38.56</v>
       </c>
       <c r="D20" t="n">
-        <v>1.6</v>
+        <v>3.26</v>
       </c>
       <c r="E20" t="n">
-        <v>17.3</v>
+        <v>17.1</v>
       </c>
       <c r="F20" t="n">
-        <v>15.4</v>
+        <v>17.1</v>
       </c>
       <c r="G20" t="n">
-        <v>16</v>
+        <v>17.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="21">
@@ -1056,292 +1056,292 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>16.15</v>
+        <v>16</v>
       </c>
       <c r="D21" t="n">
         <v>0.89</v>
       </c>
       <c r="E21" t="n">
-        <v>16</v>
+        <v>15.9</v>
       </c>
       <c r="F21" t="n">
-        <v>16</v>
+        <v>16.5</v>
       </c>
       <c r="G21" t="n">
-        <v>16</v>
+        <v>16.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22.67</v>
+        <v>46.72</v>
       </c>
       <c r="D22" t="n">
-        <v>2.1</v>
+        <v>3.83</v>
       </c>
       <c r="E22" t="n">
-        <v>9.9</v>
+        <v>17.1</v>
       </c>
       <c r="F22" t="n">
-        <v>12.3</v>
+        <v>15.2</v>
       </c>
       <c r="G22" t="n">
-        <v>11.6</v>
+        <v>15.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>46.4</v>
+        <v>22.78</v>
       </c>
       <c r="D23" t="n">
-        <v>3.8</v>
+        <v>2.1</v>
       </c>
       <c r="E23" t="n">
-        <v>16</v>
+        <v>12.2</v>
       </c>
       <c r="F23" t="n">
-        <v>9.300000000000001</v>
+        <v>12.8</v>
       </c>
       <c r="G23" t="n">
-        <v>11.3</v>
+        <v>12.6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>18.37</v>
+        <v>28.96</v>
       </c>
       <c r="D24" t="n">
-        <v>1.71</v>
+        <v>2.2</v>
       </c>
       <c r="E24" t="n">
-        <v>11.1</v>
+        <v>3.7</v>
       </c>
       <c r="F24" t="n">
-        <v>10.5</v>
+        <v>4.3</v>
       </c>
       <c r="G24" t="n">
-        <v>10.7</v>
+        <v>4.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10.39</v>
+        <v>21.14</v>
       </c>
       <c r="D25" t="n">
-        <v>0.66</v>
+        <v>1.91</v>
       </c>
       <c r="E25" t="n">
-        <v>7.4</v>
+        <v>3.7</v>
       </c>
       <c r="F25" t="n">
-        <v>4.3</v>
+        <v>3.7</v>
       </c>
       <c r="G25" t="n">
-        <v>5.2</v>
+        <v>3.7</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>28.99</v>
+        <v>20.36</v>
       </c>
       <c r="D26" t="n">
-        <v>2.2</v>
+        <v>1.49</v>
       </c>
       <c r="E26" t="n">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="F26" t="n">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="G26" t="n">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>21.19</v>
+        <v>19.44</v>
       </c>
       <c r="D27" t="n">
-        <v>1.92</v>
+        <v>3.21</v>
       </c>
       <c r="E27" t="n">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="F27" t="n">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="G27" t="n">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>20.59</v>
+        <v>10.21</v>
       </c>
       <c r="D28" t="n">
-        <v>1.51</v>
+        <v>0.65</v>
       </c>
       <c r="E28" t="n">
         <v>3.7</v>
       </c>
       <c r="F28" t="n">
-        <v>3.1</v>
+        <v>1.8</v>
       </c>
       <c r="G28" t="n">
-        <v>3.3</v>
+        <v>2.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>25.23</v>
+        <v>18.04</v>
       </c>
       <c r="D29" t="n">
-        <v>2.31</v>
+        <v>1.68</v>
       </c>
       <c r="E29" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="F29" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="G29" t="n">
-        <v>2.5</v>
+        <v>1.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.65</v>
+        <v>24.59</v>
       </c>
       <c r="D30" t="n">
-        <v>3.25</v>
+        <v>2.25</v>
       </c>
       <c r="E30" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="F30" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="G30" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>29.85</v>
+        <v>29.12</v>
       </c>
       <c r="D31" t="n">
-        <v>3.22</v>
+        <v>3.14</v>
       </c>
       <c r="E31" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="F31" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="G31" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="32">
@@ -1386,10 +1386,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>55.51</v>
+        <v>54.44</v>
       </c>
       <c r="D32" t="n">
-        <v>3.57</v>
+        <v>3.5</v>
       </c>
       <c r="E32" t="n">
         <v>1.2</v>
@@ -1401,7 +1401,7 @@
         <v>1.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Jul 17 11:09:50 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,31 +477,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>29.95</v>
+        <v>6.84</v>
       </c>
       <c r="D2" t="n">
-        <v>2.75</v>
+        <v>0.65</v>
       </c>
       <c r="E2" t="n">
-        <v>81.7</v>
+        <v>59</v>
       </c>
       <c r="F2" t="n">
-        <v>86.59999999999999</v>
+        <v>63.3</v>
       </c>
       <c r="G2" t="n">
-        <v>84.09999999999999</v>
+        <v>61.1</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="3">
@@ -516,142 +516,142 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.34</v>
+        <v>10.22</v>
       </c>
       <c r="D3" t="n">
-        <v>1.25</v>
+        <v>1.24</v>
       </c>
       <c r="E3" t="n">
-        <v>68.90000000000001</v>
+        <v>60.2</v>
       </c>
       <c r="F3" t="n">
-        <v>60.4</v>
+        <v>54.2</v>
       </c>
       <c r="G3" t="n">
-        <v>64.59999999999999</v>
+        <v>57.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>75.02</v>
+        <v>27.77</v>
       </c>
       <c r="D4" t="n">
-        <v>7.87</v>
+        <v>2.06</v>
       </c>
       <c r="E4" t="n">
-        <v>59.8</v>
+        <v>49.4</v>
       </c>
       <c r="F4" t="n">
-        <v>60.4</v>
+        <v>44</v>
       </c>
       <c r="G4" t="n">
-        <v>60.1</v>
+        <v>46.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28.38</v>
+        <v>28.18</v>
       </c>
       <c r="D5" t="n">
-        <v>2.1</v>
+        <v>2.59</v>
       </c>
       <c r="E5" t="n">
-        <v>56.1</v>
+        <v>47</v>
       </c>
       <c r="F5" t="n">
-        <v>51.2</v>
+        <v>44</v>
       </c>
       <c r="G5" t="n">
-        <v>53.7</v>
+        <v>45.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>36.72</v>
+        <v>13.03</v>
       </c>
       <c r="D6" t="n">
-        <v>2.04</v>
+        <v>1.22</v>
       </c>
       <c r="E6" t="n">
-        <v>47.6</v>
+        <v>34.9</v>
       </c>
       <c r="F6" t="n">
-        <v>44.5</v>
+        <v>32.5</v>
       </c>
       <c r="G6" t="n">
-        <v>46</v>
+        <v>33.7</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.5</v>
+        <v>17.38</v>
       </c>
       <c r="D7" t="n">
-        <v>2.38</v>
+        <v>1.61</v>
       </c>
       <c r="E7" t="n">
-        <v>41.5</v>
+        <v>32.5</v>
       </c>
       <c r="F7" t="n">
-        <v>37.8</v>
+        <v>33.1</v>
       </c>
       <c r="G7" t="n">
-        <v>39.6</v>
+        <v>32.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="8">
@@ -666,172 +666,172 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.4</v>
+        <v>19.14</v>
       </c>
       <c r="D8" t="n">
-        <v>3.36</v>
+        <v>3.31</v>
       </c>
       <c r="E8" t="n">
-        <v>35.4</v>
+        <v>32.5</v>
       </c>
       <c r="F8" t="n">
-        <v>36</v>
+        <v>32.5</v>
       </c>
       <c r="G8" t="n">
-        <v>35.7</v>
+        <v>32.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6.72</v>
+        <v>68.98</v>
       </c>
       <c r="D9" t="n">
-        <v>0.64</v>
+        <v>7.24</v>
       </c>
       <c r="E9" t="n">
-        <v>29.3</v>
+        <v>30.1</v>
       </c>
       <c r="F9" t="n">
-        <v>39.6</v>
+        <v>32.5</v>
       </c>
       <c r="G9" t="n">
-        <v>34.5</v>
+        <v>31.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>117.72</v>
+        <v>27.73</v>
       </c>
       <c r="D10" t="n">
-        <v>4.42</v>
+        <v>2.32</v>
       </c>
       <c r="E10" t="n">
-        <v>34.1</v>
+        <v>21.7</v>
       </c>
       <c r="F10" t="n">
-        <v>34.1</v>
+        <v>22.3</v>
       </c>
       <c r="G10" t="n">
-        <v>34.1</v>
+        <v>22.1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>17.32</v>
+        <v>34.65</v>
       </c>
       <c r="D11" t="n">
-        <v>1.6</v>
+        <v>1.92</v>
       </c>
       <c r="E11" t="n">
-        <v>31.7</v>
+        <v>24.1</v>
       </c>
       <c r="F11" t="n">
-        <v>31.1</v>
+        <v>18.1</v>
       </c>
       <c r="G11" t="n">
-        <v>31.4</v>
+        <v>19.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10.56</v>
+        <v>14.29</v>
       </c>
       <c r="D12" t="n">
-        <v>0.95</v>
+        <v>1.16</v>
       </c>
       <c r="E12" t="n">
-        <v>26.8</v>
+        <v>16.3</v>
       </c>
       <c r="F12" t="n">
-        <v>31.7</v>
+        <v>13.9</v>
       </c>
       <c r="G12" t="n">
-        <v>29.3</v>
+        <v>14.6</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12.84</v>
+        <v>15.84</v>
       </c>
       <c r="D13" t="n">
-        <v>1.21</v>
+        <v>0.88</v>
       </c>
       <c r="E13" t="n">
-        <v>30.5</v>
+        <v>13.3</v>
       </c>
       <c r="F13" t="n">
-        <v>28</v>
+        <v>13.3</v>
       </c>
       <c r="G13" t="n">
-        <v>28.8</v>
+        <v>13.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="14">
@@ -846,322 +846,322 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>30.97</v>
+        <v>28.98</v>
       </c>
       <c r="D14" t="n">
-        <v>2.93</v>
+        <v>2.74</v>
       </c>
       <c r="E14" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>26.8</v>
+        <v>12.7</v>
       </c>
       <c r="G14" t="n">
-        <v>27.2</v>
+        <v>12.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>21.64</v>
+        <v>109.21</v>
       </c>
       <c r="D15" t="n">
-        <v>1.78</v>
+        <v>4.1</v>
       </c>
       <c r="E15" t="n">
-        <v>26.8</v>
+        <v>8.4</v>
       </c>
       <c r="F15" t="n">
-        <v>26.8</v>
+        <v>9.6</v>
       </c>
       <c r="G15" t="n">
-        <v>26.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>23.7</v>
+        <v>10.1</v>
       </c>
       <c r="D16" t="n">
-        <v>1.94</v>
+        <v>0.92</v>
       </c>
       <c r="E16" t="n">
-        <v>26.8</v>
+        <v>4.2</v>
       </c>
       <c r="F16" t="n">
-        <v>26.8</v>
+        <v>11.4</v>
       </c>
       <c r="G16" t="n">
-        <v>26.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14.34</v>
+        <v>20.88</v>
       </c>
       <c r="D17" t="n">
-        <v>1.17</v>
+        <v>1.71</v>
       </c>
       <c r="E17" t="n">
-        <v>20.7</v>
+        <v>7.2</v>
       </c>
       <c r="F17" t="n">
-        <v>22</v>
+        <v>7.8</v>
       </c>
       <c r="G17" t="n">
-        <v>21.6</v>
+        <v>7.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19.27</v>
+        <v>14.99</v>
       </c>
       <c r="D18" t="n">
-        <v>1.61</v>
+        <v>2.22</v>
       </c>
       <c r="E18" t="n">
-        <v>23.2</v>
+        <v>6</v>
       </c>
       <c r="F18" t="n">
-        <v>20.7</v>
+        <v>7.2</v>
       </c>
       <c r="G18" t="n">
-        <v>21.5</v>
+        <v>6.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15.24</v>
+        <v>18.14</v>
       </c>
       <c r="D19" t="n">
-        <v>2.25</v>
+        <v>1.69</v>
       </c>
       <c r="E19" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="F19" t="n">
-        <v>19.5</v>
+        <v>4.8</v>
       </c>
       <c r="G19" t="n">
-        <v>21.2</v>
+        <v>5.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>38.56</v>
+        <v>22.79</v>
       </c>
       <c r="D20" t="n">
-        <v>3.26</v>
+        <v>1.86</v>
       </c>
       <c r="E20" t="n">
-        <v>17.1</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>17.1</v>
+        <v>3</v>
       </c>
       <c r="G20" t="n">
-        <v>17.1</v>
+        <v>3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>16</v>
+        <v>35.96</v>
       </c>
       <c r="D21" t="n">
-        <v>0.89</v>
+        <v>3.04</v>
       </c>
       <c r="E21" t="n">
-        <v>15.9</v>
+        <v>2.4</v>
       </c>
       <c r="F21" t="n">
-        <v>16.5</v>
+        <v>2.4</v>
       </c>
       <c r="G21" t="n">
-        <v>16.3</v>
+        <v>2.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>46.72</v>
+        <v>18.66</v>
       </c>
       <c r="D22" t="n">
-        <v>3.83</v>
+        <v>1.56</v>
       </c>
       <c r="E22" t="n">
-        <v>17.1</v>
+        <v>2.4</v>
       </c>
       <c r="F22" t="n">
-        <v>15.2</v>
+        <v>1.8</v>
       </c>
       <c r="G22" t="n">
-        <v>15.8</v>
+        <v>2</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22.78</v>
+        <v>10.03</v>
       </c>
       <c r="D23" t="n">
-        <v>2.1</v>
+        <v>0.64</v>
       </c>
       <c r="E23" t="n">
-        <v>12.2</v>
+        <v>2.4</v>
       </c>
       <c r="F23" t="n">
-        <v>12.8</v>
+        <v>1.2</v>
       </c>
       <c r="G23" t="n">
-        <v>12.6</v>
+        <v>1.6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>28.96</v>
+        <v>21.97</v>
       </c>
       <c r="D24" t="n">
-        <v>2.2</v>
+        <v>2.03</v>
       </c>
       <c r="E24" t="n">
-        <v>3.7</v>
+        <v>1.2</v>
       </c>
       <c r="F24" t="n">
-        <v>4.3</v>
+        <v>1.2</v>
       </c>
       <c r="G24" t="n">
-        <v>4.1</v>
+        <v>1.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="25">
@@ -1176,52 +1176,52 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21.14</v>
+        <v>20.31</v>
       </c>
       <c r="D25" t="n">
-        <v>1.91</v>
+        <v>1.84</v>
       </c>
       <c r="E25" t="n">
-        <v>3.7</v>
+        <v>1.2</v>
       </c>
       <c r="F25" t="n">
-        <v>3.7</v>
+        <v>1.2</v>
       </c>
       <c r="G25" t="n">
-        <v>3.7</v>
+        <v>1.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>20.36</v>
+        <v>23.94</v>
       </c>
       <c r="D26" t="n">
-        <v>1.49</v>
+        <v>2.19</v>
       </c>
       <c r="E26" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F26" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G26" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="27">
@@ -1236,100 +1236,100 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>19.44</v>
+        <v>18.5</v>
       </c>
       <c r="D27" t="n">
-        <v>3.21</v>
+        <v>3.06</v>
       </c>
       <c r="E27" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F27" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G27" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>10.21</v>
+        <v>27.82</v>
       </c>
       <c r="D28" t="n">
-        <v>0.65</v>
+        <v>2.12</v>
       </c>
       <c r="E28" t="n">
-        <v>3.7</v>
+        <v>1.2</v>
       </c>
       <c r="F28" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="G28" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.04</v>
+        <v>28.08</v>
       </c>
       <c r="D29" t="n">
-        <v>1.68</v>
+        <v>3.03</v>
       </c>
       <c r="E29" t="n">
         <v>1.2</v>
       </c>
       <c r="F29" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="G29" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>24.59</v>
+        <v>44.29</v>
       </c>
       <c r="D30" t="n">
-        <v>2.25</v>
+        <v>3.63</v>
       </c>
       <c r="E30" t="n">
         <v>1.2</v>
@@ -1341,25 +1341,25 @@
         <v>1.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>29.12</v>
+        <v>51.58</v>
       </c>
       <c r="D31" t="n">
-        <v>3.14</v>
+        <v>3.31</v>
       </c>
       <c r="E31" t="n">
         <v>1.2</v>
@@ -1371,25 +1371,25 @@
         <v>1.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>54.44</v>
+        <v>19.53</v>
       </c>
       <c r="D32" t="n">
-        <v>3.5</v>
+        <v>1.43</v>
       </c>
       <c r="E32" t="n">
         <v>1.2</v>
@@ -1401,7 +1401,7 @@
         <v>1.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Jul 18 10:49:50 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.65</v>
       </c>
       <c r="E2" t="n">
-        <v>59</v>
+        <v>58.9</v>
       </c>
       <c r="F2" t="n">
-        <v>63.3</v>
+        <v>63.1</v>
       </c>
       <c r="G2" t="n">
-        <v>61.1</v>
+        <v>61</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.24</v>
       </c>
       <c r="E3" t="n">
-        <v>60.2</v>
+        <v>60.1</v>
       </c>
       <c r="F3" t="n">
         <v>54.2</v>
       </c>
       <c r="G3" t="n">
-        <v>57.2</v>
+        <v>57.1</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="4">
@@ -561,7 +561,7 @@
         <v>46.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="5">
@@ -591,7 +591,7 @@
         <v>45.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.22</v>
       </c>
       <c r="E6" t="n">
-        <v>34.9</v>
+        <v>35.1</v>
       </c>
       <c r="F6" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="G6" t="n">
-        <v>33.7</v>
+        <v>33.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.61</v>
       </c>
       <c r="E7" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="F7" t="n">
-        <v>33.1</v>
+        <v>33.3</v>
       </c>
       <c r="G7" t="n">
-        <v>32.8</v>
+        <v>33</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>3.31</v>
       </c>
       <c r="E8" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="F8" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="G8" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>7.24</v>
       </c>
       <c r="E9" t="n">
-        <v>30.1</v>
+        <v>30.4</v>
       </c>
       <c r="F9" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="G9" t="n">
-        <v>31.3</v>
+        <v>31.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.32</v>
       </c>
       <c r="E10" t="n">
-        <v>21.7</v>
+        <v>22</v>
       </c>
       <c r="F10" t="n">
-        <v>22.3</v>
+        <v>22.6</v>
       </c>
       <c r="G10" t="n">
-        <v>22.1</v>
+        <v>22.4</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.92</v>
       </c>
       <c r="E11" t="n">
-        <v>24.1</v>
+        <v>24.4</v>
       </c>
       <c r="F11" t="n">
-        <v>18.1</v>
+        <v>18.5</v>
       </c>
       <c r="G11" t="n">
-        <v>19.9</v>
+        <v>20.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.16</v>
       </c>
       <c r="E12" t="n">
-        <v>16.3</v>
+        <v>16.7</v>
       </c>
       <c r="F12" t="n">
-        <v>13.9</v>
+        <v>14.3</v>
       </c>
       <c r="G12" t="n">
-        <v>14.6</v>
+        <v>15</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>0.88</v>
       </c>
       <c r="E13" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="F13" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="G13" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.74</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="F14" t="n">
-        <v>12.7</v>
+        <v>13.1</v>
       </c>
       <c r="G14" t="n">
-        <v>12.5</v>
+        <v>12.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>4.1</v>
       </c>
       <c r="E15" t="n">
-        <v>8.4</v>
+        <v>8.9</v>
       </c>
       <c r="F15" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="G15" t="n">
-        <v>9.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>0.92</v>
       </c>
       <c r="E16" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
       <c r="F16" t="n">
-        <v>11.4</v>
+        <v>11.9</v>
       </c>
       <c r="G16" t="n">
-        <v>9.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.71</v>
       </c>
       <c r="E17" t="n">
-        <v>7.2</v>
+        <v>7.7</v>
       </c>
       <c r="F17" t="n">
-        <v>7.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.22</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="F18" t="n">
-        <v>7.2</v>
+        <v>7.7</v>
       </c>
       <c r="G18" t="n">
-        <v>6.9</v>
+        <v>7.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.69</v>
       </c>
       <c r="E19" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="F19" t="n">
-        <v>4.8</v>
+        <v>5.4</v>
       </c>
       <c r="G19" t="n">
-        <v>5.2</v>
+        <v>5.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.86</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="G20" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.04</v>
       </c>
       <c r="E21" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.56</v>
       </c>
       <c r="E22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" t="n">
         <v>2.4</v>
       </c>
-      <c r="F22" t="n">
-        <v>1.8</v>
-      </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.64</v>
       </c>
       <c r="E23" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G23" t="n">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.03</v>
       </c>
       <c r="E24" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F24" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G24" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.84</v>
       </c>
       <c r="E25" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F25" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G25" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.19</v>
       </c>
       <c r="E26" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F26" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G26" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.06</v>
       </c>
       <c r="E27" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F27" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G27" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.12</v>
       </c>
       <c r="E28" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F28" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G28" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.03</v>
       </c>
       <c r="E29" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F29" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G29" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>3.63</v>
       </c>
       <c r="E30" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F30" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G30" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.31</v>
       </c>
       <c r="E31" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F31" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G31" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.43</v>
       </c>
       <c r="E32" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F32" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G32" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Jul 19 11:00:29 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.65</v>
       </c>
       <c r="E2" t="n">
-        <v>58.9</v>
+        <v>58.8</v>
       </c>
       <c r="F2" t="n">
-        <v>63.1</v>
+        <v>62.9</v>
       </c>
       <c r="G2" t="n">
-        <v>61</v>
+        <v>60.9</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.24</v>
       </c>
       <c r="E3" t="n">
-        <v>60.1</v>
+        <v>60</v>
       </c>
       <c r="F3" t="n">
-        <v>54.2</v>
+        <v>54.1</v>
       </c>
       <c r="G3" t="n">
         <v>57.1</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="4">
@@ -555,13 +555,13 @@
         <v>49.4</v>
       </c>
       <c r="F4" t="n">
-        <v>44</v>
+        <v>44.1</v>
       </c>
       <c r="G4" t="n">
-        <v>46.7</v>
+        <v>46.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.59</v>
       </c>
       <c r="E5" t="n">
-        <v>47</v>
+        <v>47.1</v>
       </c>
       <c r="F5" t="n">
-        <v>44</v>
+        <v>44.1</v>
       </c>
       <c r="G5" t="n">
-        <v>45.5</v>
+        <v>45.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.22</v>
       </c>
       <c r="E6" t="n">
-        <v>35.1</v>
+        <v>35.3</v>
       </c>
       <c r="F6" t="n">
-        <v>32.7</v>
+        <v>32.9</v>
       </c>
       <c r="G6" t="n">
-        <v>33.9</v>
+        <v>34.1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.61</v>
       </c>
       <c r="E7" t="n">
-        <v>32.7</v>
+        <v>32.9</v>
       </c>
       <c r="F7" t="n">
-        <v>33.3</v>
+        <v>33.5</v>
       </c>
       <c r="G7" t="n">
-        <v>33</v>
+        <v>33.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>3.31</v>
       </c>
       <c r="E8" t="n">
-        <v>32.7</v>
+        <v>32.9</v>
       </c>
       <c r="F8" t="n">
-        <v>32.7</v>
+        <v>32.9</v>
       </c>
       <c r="G8" t="n">
-        <v>32.7</v>
+        <v>32.9</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>7.24</v>
       </c>
       <c r="E9" t="n">
-        <v>30.4</v>
+        <v>30.6</v>
       </c>
       <c r="F9" t="n">
-        <v>32.7</v>
+        <v>32.9</v>
       </c>
       <c r="G9" t="n">
-        <v>31.5</v>
+        <v>31.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.32</v>
       </c>
       <c r="E10" t="n">
-        <v>22</v>
+        <v>22.4</v>
       </c>
       <c r="F10" t="n">
-        <v>22.6</v>
+        <v>22.9</v>
       </c>
       <c r="G10" t="n">
-        <v>22.4</v>
+        <v>22.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.92</v>
       </c>
       <c r="E11" t="n">
-        <v>24.4</v>
+        <v>24.7</v>
       </c>
       <c r="F11" t="n">
-        <v>18.5</v>
+        <v>18.8</v>
       </c>
       <c r="G11" t="n">
-        <v>20.2</v>
+        <v>20.6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.16</v>
       </c>
       <c r="E12" t="n">
-        <v>16.7</v>
+        <v>17.1</v>
       </c>
       <c r="F12" t="n">
-        <v>14.3</v>
+        <v>14.7</v>
       </c>
       <c r="G12" t="n">
-        <v>15</v>
+        <v>15.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>0.88</v>
       </c>
       <c r="E13" t="n">
-        <v>13.7</v>
+        <v>14.1</v>
       </c>
       <c r="F13" t="n">
-        <v>13.7</v>
+        <v>14.1</v>
       </c>
       <c r="G13" t="n">
-        <v>13.7</v>
+        <v>14.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.74</v>
       </c>
       <c r="E14" t="n">
-        <v>12.5</v>
+        <v>12.9</v>
       </c>
       <c r="F14" t="n">
-        <v>13.1</v>
+        <v>13.5</v>
       </c>
       <c r="G14" t="n">
-        <v>12.9</v>
+        <v>13.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>4.1</v>
       </c>
       <c r="E15" t="n">
-        <v>8.9</v>
+        <v>9.4</v>
       </c>
       <c r="F15" t="n">
-        <v>10.1</v>
+        <v>10.6</v>
       </c>
       <c r="G15" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>0.92</v>
       </c>
       <c r="E16" t="n">
-        <v>4.8</v>
+        <v>5.3</v>
       </c>
       <c r="F16" t="n">
-        <v>11.9</v>
+        <v>12.4</v>
       </c>
       <c r="G16" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.71</v>
       </c>
       <c r="E17" t="n">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>8.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>8.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.22</v>
       </c>
       <c r="E18" t="n">
-        <v>6.5</v>
+        <v>7.1</v>
       </c>
       <c r="F18" t="n">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.69</v>
       </c>
       <c r="E19" t="n">
-        <v>6.5</v>
+        <v>7.1</v>
       </c>
       <c r="F19" t="n">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="G19" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.86</v>
       </c>
       <c r="E20" t="n">
-        <v>3.6</v>
+        <v>4.1</v>
       </c>
       <c r="F20" t="n">
-        <v>3.6</v>
+        <v>4.1</v>
       </c>
       <c r="G20" t="n">
-        <v>3.6</v>
+        <v>4.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.04</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F21" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="G21" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.56</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F22" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="G22" t="n">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.64</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F23" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G23" t="n">
-        <v>2.1</v>
+        <v>2.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.03</v>
       </c>
       <c r="E24" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="F24" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G24" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.84</v>
       </c>
       <c r="E25" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="F25" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G25" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.19</v>
       </c>
       <c r="E26" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="F26" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G26" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.06</v>
       </c>
       <c r="E27" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="F27" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G27" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.12</v>
       </c>
       <c r="E28" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="F28" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G28" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.03</v>
       </c>
       <c r="E29" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="F29" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G29" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>3.63</v>
       </c>
       <c r="E30" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="F30" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G30" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.31</v>
       </c>
       <c r="E31" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="F31" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G31" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.43</v>
       </c>
       <c r="E32" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="F32" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="G32" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Jul 20 12:03:34 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6.84</v>
+        <v>7.01</v>
       </c>
       <c r="D2" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="E2" t="n">
-        <v>58.8</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>62.9</v>
+        <v>80.2</v>
       </c>
       <c r="G2" t="n">
-        <v>60.9</v>
+        <v>84.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="3">
@@ -516,142 +516,142 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.22</v>
+        <v>10.53</v>
       </c>
       <c r="D3" t="n">
-        <v>1.24</v>
+        <v>1.28</v>
       </c>
       <c r="E3" t="n">
-        <v>60</v>
+        <v>87.2</v>
       </c>
       <c r="F3" t="n">
-        <v>54.1</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>57.1</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>27.77</v>
+        <v>28.74</v>
       </c>
       <c r="D4" t="n">
-        <v>2.06</v>
+        <v>2.64</v>
       </c>
       <c r="E4" t="n">
-        <v>49.4</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>44.1</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>46.8</v>
+        <v>66.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28.18</v>
+        <v>18.39</v>
       </c>
       <c r="D5" t="n">
-        <v>2.59</v>
+        <v>1.7</v>
       </c>
       <c r="E5" t="n">
-        <v>47.1</v>
+        <v>50</v>
       </c>
       <c r="F5" t="n">
-        <v>44.1</v>
+        <v>59.3</v>
       </c>
       <c r="G5" t="n">
-        <v>45.6</v>
+        <v>54.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13.03</v>
+        <v>28.2</v>
       </c>
       <c r="D6" t="n">
-        <v>1.22</v>
+        <v>2.09</v>
       </c>
       <c r="E6" t="n">
-        <v>35.3</v>
+        <v>55.8</v>
       </c>
       <c r="F6" t="n">
-        <v>32.9</v>
+        <v>52.3</v>
       </c>
       <c r="G6" t="n">
-        <v>34.1</v>
+        <v>54.1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>17.38</v>
+        <v>13.94</v>
       </c>
       <c r="D7" t="n">
-        <v>1.61</v>
+        <v>1.31</v>
       </c>
       <c r="E7" t="n">
-        <v>32.9</v>
+        <v>47.7</v>
       </c>
       <c r="F7" t="n">
-        <v>33.5</v>
+        <v>47.1</v>
       </c>
       <c r="G7" t="n">
-        <v>33.2</v>
+        <v>47.4</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="8">
@@ -666,52 +666,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.14</v>
+        <v>19.92</v>
       </c>
       <c r="D8" t="n">
-        <v>3.31</v>
+        <v>3.45</v>
       </c>
       <c r="E8" t="n">
-        <v>32.9</v>
+        <v>52.9</v>
       </c>
       <c r="F8" t="n">
-        <v>32.9</v>
+        <v>40.1</v>
       </c>
       <c r="G8" t="n">
-        <v>32.9</v>
+        <v>46.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>68.98</v>
+        <v>14.57</v>
       </c>
       <c r="D9" t="n">
-        <v>7.24</v>
+        <v>1.19</v>
       </c>
       <c r="E9" t="n">
-        <v>30.6</v>
+        <v>37.2</v>
       </c>
       <c r="F9" t="n">
-        <v>32.9</v>
+        <v>37.8</v>
       </c>
       <c r="G9" t="n">
-        <v>31.8</v>
+        <v>37.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="10">
@@ -726,172 +726,172 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>27.73</v>
+        <v>27.98</v>
       </c>
       <c r="D10" t="n">
-        <v>2.32</v>
+        <v>2.34</v>
       </c>
       <c r="E10" t="n">
-        <v>22.4</v>
+        <v>32.6</v>
       </c>
       <c r="F10" t="n">
-        <v>22.9</v>
+        <v>31.4</v>
       </c>
       <c r="G10" t="n">
-        <v>22.8</v>
+        <v>32</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>34.65</v>
+        <v>18.91</v>
       </c>
       <c r="D11" t="n">
-        <v>1.92</v>
+        <v>1.76</v>
       </c>
       <c r="E11" t="n">
-        <v>24.7</v>
+        <v>29.1</v>
       </c>
       <c r="F11" t="n">
-        <v>18.8</v>
+        <v>29.1</v>
       </c>
       <c r="G11" t="n">
-        <v>20.6</v>
+        <v>29.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>14.29</v>
+        <v>66.37</v>
       </c>
       <c r="D12" t="n">
-        <v>1.16</v>
+        <v>6.97</v>
       </c>
       <c r="E12" t="n">
-        <v>17.1</v>
+        <v>20.9</v>
       </c>
       <c r="F12" t="n">
-        <v>14.7</v>
+        <v>22.1</v>
       </c>
       <c r="G12" t="n">
-        <v>15.4</v>
+        <v>21.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>15.84</v>
+        <v>29.34</v>
       </c>
       <c r="D13" t="n">
-        <v>0.88</v>
+        <v>2.78</v>
       </c>
       <c r="E13" t="n">
-        <v>14.1</v>
+        <v>20.9</v>
       </c>
       <c r="F13" t="n">
-        <v>14.1</v>
+        <v>20.9</v>
       </c>
       <c r="G13" t="n">
-        <v>14.1</v>
+        <v>20.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>28.98</v>
+        <v>16.09</v>
       </c>
       <c r="D14" t="n">
-        <v>2.74</v>
+        <v>0.89</v>
       </c>
       <c r="E14" t="n">
-        <v>12.9</v>
+        <v>19.8</v>
       </c>
       <c r="F14" t="n">
-        <v>13.5</v>
+        <v>19.8</v>
       </c>
       <c r="G14" t="n">
-        <v>13.4</v>
+        <v>19.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>109.21</v>
+        <v>21.07</v>
       </c>
       <c r="D15" t="n">
-        <v>4.1</v>
+        <v>1.73</v>
       </c>
       <c r="E15" t="n">
-        <v>9.4</v>
+        <v>16.9</v>
       </c>
       <c r="F15" t="n">
-        <v>10.6</v>
+        <v>16.9</v>
       </c>
       <c r="G15" t="n">
-        <v>10.2</v>
+        <v>16.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="16">
@@ -906,322 +906,322 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.1</v>
+        <v>10.22</v>
       </c>
       <c r="D16" t="n">
         <v>0.92</v>
       </c>
       <c r="E16" t="n">
-        <v>5.3</v>
+        <v>12.8</v>
       </c>
       <c r="F16" t="n">
-        <v>12.4</v>
+        <v>12.8</v>
       </c>
       <c r="G16" t="n">
-        <v>10.2</v>
+        <v>12.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>20.88</v>
+        <v>23.09</v>
       </c>
       <c r="D17" t="n">
-        <v>1.71</v>
+        <v>1.89</v>
       </c>
       <c r="E17" t="n">
-        <v>8.199999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="F17" t="n">
-        <v>8.800000000000001</v>
+        <v>11.6</v>
       </c>
       <c r="G17" t="n">
-        <v>8.6</v>
+        <v>11.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>14.99</v>
+        <v>101.63</v>
       </c>
       <c r="D18" t="n">
-        <v>2.22</v>
+        <v>3.81</v>
       </c>
       <c r="E18" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
-        <v>8.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>7.9</v>
+        <v>8.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18.14</v>
+        <v>14.97</v>
       </c>
       <c r="D19" t="n">
-        <v>1.69</v>
+        <v>2.22</v>
       </c>
       <c r="E19" t="n">
-        <v>7.1</v>
+        <v>5.8</v>
       </c>
       <c r="F19" t="n">
-        <v>5.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>6.2</v>
+        <v>7.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>22.79</v>
+        <v>10.07</v>
       </c>
       <c r="D20" t="n">
-        <v>1.86</v>
+        <v>0.65</v>
       </c>
       <c r="E20" t="n">
-        <v>4.1</v>
+        <v>5.8</v>
       </c>
       <c r="F20" t="n">
-        <v>4.1</v>
+        <v>5.8</v>
       </c>
       <c r="G20" t="n">
-        <v>4.1</v>
+        <v>5.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>35.96</v>
+        <v>45.04</v>
       </c>
       <c r="D21" t="n">
-        <v>3.04</v>
+        <v>3.7</v>
       </c>
       <c r="E21" t="n">
-        <v>3.5</v>
+        <v>5.8</v>
       </c>
       <c r="F21" t="n">
-        <v>3.5</v>
+        <v>4.7</v>
       </c>
       <c r="G21" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>18.66</v>
+        <v>51.63</v>
       </c>
       <c r="D22" t="n">
-        <v>1.56</v>
+        <v>3.32</v>
       </c>
       <c r="E22" t="n">
-        <v>3.5</v>
+        <v>4.7</v>
       </c>
       <c r="F22" t="n">
-        <v>2.9</v>
+        <v>4.7</v>
       </c>
       <c r="G22" t="n">
-        <v>3.1</v>
+        <v>4.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10.03</v>
+        <v>32.34</v>
       </c>
       <c r="D23" t="n">
-        <v>0.64</v>
+        <v>1.8</v>
       </c>
       <c r="E23" t="n">
         <v>3.5</v>
       </c>
       <c r="F23" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="G23" t="n">
         <v>2.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>21.97</v>
+        <v>19.48</v>
       </c>
       <c r="D24" t="n">
-        <v>2.03</v>
+        <v>1.43</v>
       </c>
       <c r="E24" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F24" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="G24" t="n">
         <v>2.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20.31</v>
+        <v>34.63</v>
       </c>
       <c r="D25" t="n">
-        <v>1.84</v>
+        <v>2.93</v>
       </c>
       <c r="E25" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="F25" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="G25" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>23.94</v>
+        <v>18.44</v>
       </c>
       <c r="D26" t="n">
-        <v>2.19</v>
+        <v>1.54</v>
       </c>
       <c r="E26" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F26" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G26" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="27">
@@ -1236,172 +1236,172 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18.5</v>
+        <v>18.48</v>
       </c>
       <c r="D27" t="n">
-        <v>3.06</v>
+        <v>3.05</v>
       </c>
       <c r="E27" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F27" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G27" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>27.82</v>
+        <v>21.88</v>
       </c>
       <c r="D28" t="n">
-        <v>2.12</v>
+        <v>2.02</v>
       </c>
       <c r="E28" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F28" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G28" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>28.08</v>
+        <v>23.61</v>
       </c>
       <c r="D29" t="n">
-        <v>3.03</v>
+        <v>2.16</v>
       </c>
       <c r="E29" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F29" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G29" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>44.29</v>
+        <v>20.17</v>
       </c>
       <c r="D30" t="n">
-        <v>3.63</v>
+        <v>1.82</v>
       </c>
       <c r="E30" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F30" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G30" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>51.58</v>
+        <v>27.92</v>
       </c>
       <c r="D31" t="n">
-        <v>3.31</v>
+        <v>3.02</v>
       </c>
       <c r="E31" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F31" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G31" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>19.53</v>
+        <v>27.54</v>
       </c>
       <c r="D32" t="n">
-        <v>1.43</v>
+        <v>2.09</v>
       </c>
       <c r="E32" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F32" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G32" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Jul 24 11:26:09 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.01</v>
+        <v>6.99</v>
       </c>
       <c r="D2" t="n">
         <v>0.66</v>
       </c>
       <c r="E2" t="n">
-        <v>88.40000000000001</v>
+        <v>86.8</v>
       </c>
       <c r="F2" t="n">
-        <v>80.2</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>84.3</v>
+        <v>83.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="3">
@@ -516,352 +516,352 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.53</v>
+        <v>10.32</v>
       </c>
       <c r="D3" t="n">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="E3" t="n">
-        <v>87.2</v>
+        <v>67.8</v>
       </c>
       <c r="F3" t="n">
-        <v>77.90000000000001</v>
+        <v>60.9</v>
       </c>
       <c r="G3" t="n">
-        <v>82.59999999999999</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28.74</v>
+        <v>17.88</v>
       </c>
       <c r="D4" t="n">
-        <v>2.64</v>
+        <v>1.73</v>
       </c>
       <c r="E4" t="n">
-        <v>67.40000000000001</v>
+        <v>39.1</v>
       </c>
       <c r="F4" t="n">
-        <v>65.09999999999999</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>66.3</v>
+        <v>51.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>18.39</v>
+        <v>13.94</v>
       </c>
       <c r="D5" t="n">
-        <v>1.7</v>
+        <v>1.31</v>
       </c>
       <c r="E5" t="n">
-        <v>50</v>
+        <v>47.7</v>
       </c>
       <c r="F5" t="n">
-        <v>59.3</v>
+        <v>47.1</v>
       </c>
       <c r="G5" t="n">
-        <v>54.7</v>
+        <v>47.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28.2</v>
+        <v>27.86</v>
       </c>
       <c r="D6" t="n">
-        <v>2.09</v>
+        <v>2.56</v>
       </c>
       <c r="E6" t="n">
-        <v>55.8</v>
+        <v>42.5</v>
       </c>
       <c r="F6" t="n">
-        <v>52.3</v>
+        <v>37.4</v>
       </c>
       <c r="G6" t="n">
-        <v>54.1</v>
+        <v>39.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>13.94</v>
+        <v>19.43</v>
       </c>
       <c r="D7" t="n">
-        <v>1.31</v>
+        <v>3.37</v>
       </c>
       <c r="E7" t="n">
-        <v>47.7</v>
+        <v>39.1</v>
       </c>
       <c r="F7" t="n">
-        <v>47.1</v>
+        <v>39.1</v>
       </c>
       <c r="G7" t="n">
-        <v>47.4</v>
+        <v>39.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.92</v>
+        <v>14.55</v>
       </c>
       <c r="D8" t="n">
-        <v>3.45</v>
+        <v>1.19</v>
       </c>
       <c r="E8" t="n">
-        <v>52.9</v>
+        <v>35.6</v>
       </c>
       <c r="F8" t="n">
-        <v>40.1</v>
+        <v>37.9</v>
       </c>
       <c r="G8" t="n">
-        <v>46.5</v>
+        <v>36.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.57</v>
+        <v>69.17</v>
       </c>
       <c r="D9" t="n">
-        <v>1.19</v>
+        <v>7.26</v>
       </c>
       <c r="E9" t="n">
-        <v>37.2</v>
+        <v>33.3</v>
       </c>
       <c r="F9" t="n">
-        <v>37.8</v>
+        <v>36.8</v>
       </c>
       <c r="G9" t="n">
-        <v>37.5</v>
+        <v>35.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>27.98</v>
+        <v>19.37</v>
       </c>
       <c r="D10" t="n">
-        <v>2.34</v>
+        <v>1.74</v>
       </c>
       <c r="E10" t="n">
-        <v>32.6</v>
+        <v>36.8</v>
       </c>
       <c r="F10" t="n">
-        <v>31.4</v>
+        <v>28.7</v>
       </c>
       <c r="G10" t="n">
-        <v>32</v>
+        <v>31.1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>18.91</v>
+        <v>27.08</v>
       </c>
       <c r="D11" t="n">
-        <v>1.76</v>
+        <v>2.02</v>
       </c>
       <c r="E11" t="n">
-        <v>29.1</v>
+        <v>25.3</v>
       </c>
       <c r="F11" t="n">
-        <v>29.1</v>
+        <v>32.2</v>
       </c>
       <c r="G11" t="n">
-        <v>29.1</v>
+        <v>28.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>66.37</v>
+        <v>29.29</v>
       </c>
       <c r="D12" t="n">
-        <v>6.97</v>
+        <v>2.77</v>
       </c>
       <c r="E12" t="n">
-        <v>20.9</v>
+        <v>19.5</v>
       </c>
       <c r="F12" t="n">
-        <v>22.1</v>
+        <v>20.7</v>
       </c>
       <c r="G12" t="n">
-        <v>21.7</v>
+        <v>20.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>29.34</v>
+        <v>16.08</v>
       </c>
       <c r="D13" t="n">
-        <v>2.78</v>
+        <v>0.89</v>
       </c>
       <c r="E13" t="n">
-        <v>20.9</v>
+        <v>19.5</v>
       </c>
       <c r="F13" t="n">
-        <v>20.9</v>
+        <v>20.1</v>
       </c>
       <c r="G13" t="n">
-        <v>20.9</v>
+        <v>19.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>16.09</v>
+        <v>27.18</v>
       </c>
       <c r="D14" t="n">
-        <v>0.89</v>
+        <v>2.28</v>
       </c>
       <c r="E14" t="n">
-        <v>19.8</v>
+        <v>11.5</v>
       </c>
       <c r="F14" t="n">
-        <v>19.8</v>
+        <v>11.5</v>
       </c>
       <c r="G14" t="n">
-        <v>19.8</v>
+        <v>11.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="15">
@@ -876,172 +876,172 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>21.07</v>
+        <v>20.83</v>
       </c>
       <c r="D15" t="n">
-        <v>1.73</v>
+        <v>1.71</v>
       </c>
       <c r="E15" t="n">
-        <v>16.9</v>
+        <v>6.9</v>
       </c>
       <c r="F15" t="n">
-        <v>16.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>16.9</v>
+        <v>8.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.22</v>
+        <v>19.31</v>
       </c>
       <c r="D16" t="n">
-        <v>0.92</v>
+        <v>3.17</v>
       </c>
       <c r="E16" t="n">
-        <v>12.8</v>
+        <v>6.9</v>
       </c>
       <c r="F16" t="n">
-        <v>12.8</v>
+        <v>6.9</v>
       </c>
       <c r="G16" t="n">
-        <v>12.8</v>
+        <v>6.9</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.09</v>
+        <v>28.85</v>
       </c>
       <c r="D17" t="n">
-        <v>1.89</v>
+        <v>3.1</v>
       </c>
       <c r="E17" t="n">
-        <v>10.5</v>
+        <v>5.7</v>
       </c>
       <c r="F17" t="n">
-        <v>11.6</v>
+        <v>5.7</v>
       </c>
       <c r="G17" t="n">
-        <v>11.3</v>
+        <v>5.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>101.63</v>
+        <v>23.99</v>
       </c>
       <c r="D18" t="n">
-        <v>3.81</v>
+        <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>5.7</v>
       </c>
       <c r="F18" t="n">
-        <v>9.300000000000001</v>
+        <v>5.7</v>
       </c>
       <c r="G18" t="n">
-        <v>8.6</v>
+        <v>5.7</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>14.97</v>
+        <v>52.76</v>
       </c>
       <c r="D19" t="n">
-        <v>2.22</v>
+        <v>3.4</v>
       </c>
       <c r="E19" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="F19" t="n">
-        <v>8.699999999999999</v>
+        <v>5.7</v>
       </c>
       <c r="G19" t="n">
-        <v>7.8</v>
+        <v>5.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>10.07</v>
+        <v>71.39</v>
       </c>
       <c r="D20" t="n">
-        <v>0.65</v>
+        <v>3.27</v>
       </c>
       <c r="E20" t="n">
-        <v>5.8</v>
+        <v>2.3</v>
       </c>
       <c r="F20" t="n">
-        <v>5.8</v>
+        <v>6.3</v>
       </c>
       <c r="G20" t="n">
-        <v>5.8</v>
+        <v>5.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="21">
@@ -1056,202 +1056,202 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>45.04</v>
+        <v>44.6</v>
       </c>
       <c r="D21" t="n">
-        <v>3.7</v>
+        <v>3.67</v>
       </c>
       <c r="E21" t="n">
-        <v>5.8</v>
+        <v>4.6</v>
       </c>
       <c r="F21" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="G21" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>51.63</v>
+        <v>35.42</v>
       </c>
       <c r="D22" t="n">
-        <v>3.32</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>4.7</v>
+        <v>3.4</v>
       </c>
       <c r="F22" t="n">
-        <v>4.7</v>
+        <v>3.4</v>
       </c>
       <c r="G22" t="n">
-        <v>4.7</v>
+        <v>3.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>32.34</v>
+        <v>20.22</v>
       </c>
       <c r="D23" t="n">
-        <v>1.8</v>
+        <v>1.83</v>
       </c>
       <c r="E23" t="n">
-        <v>3.5</v>
+        <v>2.3</v>
       </c>
       <c r="F23" t="n">
         <v>2.3</v>
       </c>
       <c r="G23" t="n">
-        <v>2.7</v>
+        <v>2.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>19.48</v>
+        <v>31.75</v>
       </c>
       <c r="D24" t="n">
-        <v>1.43</v>
+        <v>1.76</v>
       </c>
       <c r="E24" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="F24" t="n">
-        <v>2.9</v>
+        <v>2.3</v>
       </c>
       <c r="G24" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>34.63</v>
+        <v>27.33</v>
       </c>
       <c r="D25" t="n">
-        <v>2.93</v>
+        <v>2.11</v>
       </c>
       <c r="E25" t="n">
-        <v>2.3</v>
+        <v>1.1</v>
       </c>
       <c r="F25" t="n">
         <v>2.3</v>
       </c>
       <c r="G25" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18.44</v>
+        <v>9.85</v>
       </c>
       <c r="D26" t="n">
-        <v>1.54</v>
+        <v>0.63</v>
       </c>
       <c r="E26" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="F26" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="G26" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18.48</v>
+        <v>14.83</v>
       </c>
       <c r="D27" t="n">
-        <v>3.05</v>
+        <v>2.19</v>
       </c>
       <c r="E27" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="F27" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="G27" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="28">
@@ -1266,142 +1266,142 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>21.88</v>
+        <v>21.77</v>
       </c>
       <c r="D28" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
       <c r="E28" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="F28" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="G28" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>23.61</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="D29" t="n">
-        <v>2.16</v>
+        <v>0.9</v>
       </c>
       <c r="E29" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="F29" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="G29" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>20.17</v>
+        <v>18.07</v>
       </c>
       <c r="D30" t="n">
-        <v>1.82</v>
+        <v>1.51</v>
       </c>
       <c r="E30" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="F30" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="G30" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>27.92</v>
+        <v>21.91</v>
       </c>
       <c r="D31" t="n">
-        <v>3.02</v>
+        <v>1.79</v>
       </c>
       <c r="E31" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="F31" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="G31" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>27.54</v>
+        <v>18.56</v>
       </c>
       <c r="D32" t="n">
-        <v>2.09</v>
+        <v>1.38</v>
       </c>
       <c r="E32" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="F32" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="G32" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46223</v>
+        <v>46227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Jul 25 10:56:56 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.66</v>
       </c>
       <c r="E2" t="n">
-        <v>86.8</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>79.90000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="G2" t="n">
-        <v>83.3</v>
+        <v>83</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.25</v>
       </c>
       <c r="E3" t="n">
-        <v>67.8</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>60.9</v>
+        <v>60.8</v>
       </c>
       <c r="G3" t="n">
-        <v>64.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>1.73</v>
       </c>
       <c r="E4" t="n">
-        <v>39.1</v>
+        <v>39.2</v>
       </c>
       <c r="F4" t="n">
-        <v>64.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="G4" t="n">
         <v>51.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="5">
@@ -585,13 +585,13 @@
         <v>47.7</v>
       </c>
       <c r="F5" t="n">
-        <v>47.1</v>
+        <v>47.2</v>
       </c>
       <c r="G5" t="n">
         <v>47.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.56</v>
       </c>
       <c r="E6" t="n">
-        <v>42.5</v>
+        <v>42.6</v>
       </c>
       <c r="F6" t="n">
-        <v>37.4</v>
+        <v>37.5</v>
       </c>
       <c r="G6" t="n">
-        <v>39.9</v>
+        <v>40.1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>3.37</v>
       </c>
       <c r="E7" t="n">
-        <v>39.1</v>
+        <v>39.2</v>
       </c>
       <c r="F7" t="n">
-        <v>39.1</v>
+        <v>39.2</v>
       </c>
       <c r="G7" t="n">
-        <v>39.1</v>
+        <v>39.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.19</v>
       </c>
       <c r="E8" t="n">
-        <v>35.6</v>
+        <v>35.8</v>
       </c>
       <c r="F8" t="n">
-        <v>37.9</v>
+        <v>38.1</v>
       </c>
       <c r="G8" t="n">
-        <v>36.8</v>
+        <v>36.9</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>7.26</v>
       </c>
       <c r="E9" t="n">
-        <v>33.3</v>
+        <v>33.5</v>
       </c>
       <c r="F9" t="n">
-        <v>36.8</v>
+        <v>36.9</v>
       </c>
       <c r="G9" t="n">
-        <v>35.1</v>
+        <v>35.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>1.74</v>
       </c>
       <c r="E10" t="n">
-        <v>36.8</v>
+        <v>36.9</v>
       </c>
       <c r="F10" t="n">
-        <v>28.7</v>
+        <v>29</v>
       </c>
       <c r="G10" t="n">
-        <v>31.1</v>
+        <v>31.4</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.02</v>
       </c>
       <c r="E11" t="n">
-        <v>25.3</v>
+        <v>25.6</v>
       </c>
       <c r="F11" t="n">
-        <v>32.2</v>
+        <v>32.4</v>
       </c>
       <c r="G11" t="n">
-        <v>28.7</v>
+        <v>29</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.77</v>
       </c>
       <c r="E12" t="n">
-        <v>19.5</v>
+        <v>19.9</v>
       </c>
       <c r="F12" t="n">
+        <v>21</v>
+      </c>
+      <c r="G12" t="n">
         <v>20.7</v>
       </c>
-      <c r="G12" t="n">
-        <v>20.3</v>
-      </c>
       <c r="H12" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>0.89</v>
       </c>
       <c r="E13" t="n">
-        <v>19.5</v>
+        <v>19.9</v>
       </c>
       <c r="F13" t="n">
-        <v>20.1</v>
+        <v>20.5</v>
       </c>
       <c r="G13" t="n">
-        <v>19.9</v>
+        <v>20.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.28</v>
       </c>
       <c r="E14" t="n">
-        <v>11.5</v>
+        <v>11.9</v>
       </c>
       <c r="F14" t="n">
-        <v>11.5</v>
+        <v>11.9</v>
       </c>
       <c r="G14" t="n">
-        <v>11.5</v>
+        <v>11.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.71</v>
       </c>
       <c r="E15" t="n">
-        <v>6.9</v>
+        <v>7.4</v>
       </c>
       <c r="F15" t="n">
-        <v>9.199999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>3.17</v>
       </c>
       <c r="E16" t="n">
-        <v>6.9</v>
+        <v>7.4</v>
       </c>
       <c r="F16" t="n">
-        <v>6.9</v>
+        <v>7.4</v>
       </c>
       <c r="G16" t="n">
-        <v>6.9</v>
+        <v>7.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.1</v>
       </c>
       <c r="E17" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="F17" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="G17" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="F18" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="G18" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>3.4</v>
       </c>
       <c r="E19" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="F19" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="G19" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>3.27</v>
       </c>
       <c r="E20" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="F20" t="n">
-        <v>6.3</v>
+        <v>6.8</v>
       </c>
       <c r="G20" t="n">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.67</v>
       </c>
       <c r="E21" t="n">
-        <v>4.6</v>
+        <v>5.1</v>
       </c>
       <c r="F21" t="n">
-        <v>4.6</v>
+        <v>5.1</v>
       </c>
       <c r="G21" t="n">
-        <v>4.6</v>
+        <v>5.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.83</v>
       </c>
       <c r="E23" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="F23" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="G23" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.76</v>
       </c>
       <c r="E24" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="F24" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="G24" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.11</v>
       </c>
       <c r="E25" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="F25" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>0.63</v>
       </c>
       <c r="E26" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="F26" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="G26" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.19</v>
       </c>
       <c r="E27" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="F27" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="G27" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.01</v>
       </c>
       <c r="E28" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="F28" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="G28" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>0.9</v>
       </c>
       <c r="E29" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="F29" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="G29" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.51</v>
       </c>
       <c r="E30" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="F30" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="G30" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.79</v>
       </c>
       <c r="E31" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="F31" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="G31" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.38</v>
       </c>
       <c r="E32" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="F32" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="G32" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Jul 26 11:09:34 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.66</v>
       </c>
       <c r="E2" t="n">
-        <v>86.40000000000001</v>
+        <v>86</v>
       </c>
       <c r="F2" t="n">
-        <v>79.5</v>
+        <v>79.2</v>
       </c>
       <c r="G2" t="n">
-        <v>83</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.25</v>
       </c>
       <c r="E3" t="n">
-        <v>67.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>60.8</v>
+        <v>60.7</v>
       </c>
       <c r="G3" t="n">
-        <v>64.2</v>
+        <v>64</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>1.73</v>
       </c>
       <c r="E4" t="n">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="F4" t="n">
-        <v>64.2</v>
+        <v>64</v>
       </c>
       <c r="G4" t="n">
         <v>51.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>1.31</v>
       </c>
       <c r="E5" t="n">
-        <v>47.7</v>
+        <v>47.8</v>
       </c>
       <c r="F5" t="n">
         <v>47.2</v>
       </c>
       <c r="G5" t="n">
-        <v>47.4</v>
+        <v>47.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.56</v>
       </c>
       <c r="E6" t="n">
-        <v>42.6</v>
+        <v>42.7</v>
       </c>
       <c r="F6" t="n">
-        <v>37.5</v>
+        <v>37.6</v>
       </c>
       <c r="G6" t="n">
-        <v>40.1</v>
+        <v>40.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>3.37</v>
       </c>
       <c r="E7" t="n">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="F7" t="n">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="G7" t="n">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.19</v>
       </c>
       <c r="E8" t="n">
-        <v>35.8</v>
+        <v>36</v>
       </c>
       <c r="F8" t="n">
-        <v>38.1</v>
+        <v>38.2</v>
       </c>
       <c r="G8" t="n">
-        <v>36.9</v>
+        <v>37.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>7.26</v>
       </c>
       <c r="E9" t="n">
-        <v>33.5</v>
+        <v>33.7</v>
       </c>
       <c r="F9" t="n">
-        <v>36.9</v>
+        <v>37.1</v>
       </c>
       <c r="G9" t="n">
-        <v>35.2</v>
+        <v>35.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>1.74</v>
       </c>
       <c r="E10" t="n">
-        <v>36.9</v>
+        <v>37.1</v>
       </c>
       <c r="F10" t="n">
-        <v>29</v>
+        <v>29.2</v>
       </c>
       <c r="G10" t="n">
-        <v>31.4</v>
+        <v>31.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>2.02</v>
       </c>
       <c r="E11" t="n">
-        <v>25.6</v>
+        <v>25.8</v>
       </c>
       <c r="F11" t="n">
-        <v>32.4</v>
+        <v>32.6</v>
       </c>
       <c r="G11" t="n">
-        <v>29</v>
+        <v>29.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.77</v>
       </c>
       <c r="E12" t="n">
-        <v>19.9</v>
+        <v>20.2</v>
       </c>
       <c r="F12" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="G12" t="n">
         <v>21</v>
       </c>
-      <c r="G12" t="n">
-        <v>20.7</v>
-      </c>
       <c r="H12" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>0.89</v>
       </c>
       <c r="E13" t="n">
-        <v>19.9</v>
+        <v>20.2</v>
       </c>
       <c r="F13" t="n">
-        <v>20.5</v>
+        <v>20.8</v>
       </c>
       <c r="G13" t="n">
-        <v>20.3</v>
+        <v>20.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.28</v>
       </c>
       <c r="E14" t="n">
-        <v>11.9</v>
+        <v>12.4</v>
       </c>
       <c r="F14" t="n">
-        <v>11.9</v>
+        <v>12.4</v>
       </c>
       <c r="G14" t="n">
-        <v>11.9</v>
+        <v>12.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.71</v>
       </c>
       <c r="E15" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="F15" t="n">
-        <v>9.699999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="G15" t="n">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>3.17</v>
       </c>
       <c r="E16" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="F16" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="G16" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>3.1</v>
       </c>
       <c r="E17" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="F17" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="G17" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="F18" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="G18" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>3.4</v>
       </c>
       <c r="E19" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="F19" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="G19" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>3.27</v>
       </c>
       <c r="E20" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="F20" t="n">
-        <v>6.8</v>
+        <v>7.3</v>
       </c>
       <c r="G20" t="n">
-        <v>5.6</v>
+        <v>6.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.67</v>
       </c>
       <c r="E21" t="n">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="F21" t="n">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="G21" t="n">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="F22" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.83</v>
       </c>
       <c r="E23" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="F23" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="G23" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.76</v>
       </c>
       <c r="E24" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="F24" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="G24" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.11</v>
       </c>
       <c r="E25" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="F25" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="G25" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>0.63</v>
       </c>
       <c r="E26" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="F26" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="G26" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.19</v>
       </c>
       <c r="E27" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="F27" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.01</v>
       </c>
       <c r="E28" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="F28" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="G28" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>0.9</v>
       </c>
       <c r="E29" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="F29" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="G29" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.51</v>
       </c>
       <c r="E30" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="F30" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="G30" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>1.79</v>
       </c>
       <c r="E31" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="F31" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="G31" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>1.38</v>
       </c>
       <c r="E32" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="F32" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="G32" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Jul 27 12:45:25 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,322 +486,322 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6.99</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
         <v>0.66</v>
       </c>
       <c r="E2" t="n">
-        <v>86</v>
+        <v>87.8</v>
       </c>
       <c r="F2" t="n">
-        <v>79.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>82.59999999999999</v>
+        <v>83.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.32</v>
+        <v>75.36</v>
       </c>
       <c r="D3" t="n">
-        <v>1.25</v>
+        <v>8.5</v>
       </c>
       <c r="E3" t="n">
-        <v>67.40000000000001</v>
+        <v>63.3</v>
       </c>
       <c r="F3" t="n">
-        <v>60.7</v>
+        <v>72.2</v>
       </c>
       <c r="G3" t="n">
-        <v>64</v>
+        <v>67.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17.88</v>
+        <v>10.3</v>
       </c>
       <c r="D4" t="n">
-        <v>1.73</v>
+        <v>1.25</v>
       </c>
       <c r="E4" t="n">
-        <v>39.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>64</v>
+        <v>60.6</v>
       </c>
       <c r="G4" t="n">
-        <v>51.7</v>
+        <v>63.1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>13.94</v>
+        <v>28.47</v>
       </c>
       <c r="D5" t="n">
-        <v>1.31</v>
+        <v>2.61</v>
       </c>
       <c r="E5" t="n">
-        <v>47.8</v>
+        <v>60</v>
       </c>
       <c r="F5" t="n">
-        <v>47.2</v>
+        <v>55.6</v>
       </c>
       <c r="G5" t="n">
-        <v>47.5</v>
+        <v>57.8</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27.86</v>
+        <v>17.75</v>
       </c>
       <c r="D6" t="n">
-        <v>2.56</v>
+        <v>1.71</v>
       </c>
       <c r="E6" t="n">
-        <v>42.7</v>
+        <v>36.7</v>
       </c>
       <c r="F6" t="n">
-        <v>37.6</v>
+        <v>61.1</v>
       </c>
       <c r="G6" t="n">
-        <v>40.2</v>
+        <v>48.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.43</v>
+        <v>14.69</v>
       </c>
       <c r="D7" t="n">
-        <v>3.37</v>
+        <v>1.2</v>
       </c>
       <c r="E7" t="n">
-        <v>39.3</v>
+        <v>46.7</v>
       </c>
       <c r="F7" t="n">
-        <v>39.3</v>
+        <v>45.6</v>
       </c>
       <c r="G7" t="n">
-        <v>39.3</v>
+        <v>46.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14.55</v>
+        <v>28.5</v>
       </c>
       <c r="D8" t="n">
-        <v>1.19</v>
+        <v>2.39</v>
       </c>
       <c r="E8" t="n">
-        <v>36</v>
+        <v>46.1</v>
       </c>
       <c r="F8" t="n">
-        <v>38.2</v>
+        <v>45.6</v>
       </c>
       <c r="G8" t="n">
-        <v>37.1</v>
+        <v>45.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>69.17</v>
+        <v>13.82</v>
       </c>
       <c r="D9" t="n">
-        <v>7.26</v>
+        <v>1.3</v>
       </c>
       <c r="E9" t="n">
-        <v>33.7</v>
+        <v>44.4</v>
       </c>
       <c r="F9" t="n">
-        <v>37.1</v>
+        <v>42.8</v>
       </c>
       <c r="G9" t="n">
-        <v>35.4</v>
+        <v>43.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.37</v>
+        <v>27.47</v>
       </c>
       <c r="D10" t="n">
-        <v>1.74</v>
+        <v>2.04</v>
       </c>
       <c r="E10" t="n">
-        <v>37.1</v>
+        <v>47.8</v>
       </c>
       <c r="F10" t="n">
-        <v>29.2</v>
+        <v>38.9</v>
       </c>
       <c r="G10" t="n">
-        <v>31.6</v>
+        <v>43.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.08</v>
+        <v>19.45</v>
       </c>
       <c r="D11" t="n">
-        <v>2.02</v>
+        <v>3.37</v>
       </c>
       <c r="E11" t="n">
-        <v>25.8</v>
+        <v>41.1</v>
       </c>
       <c r="F11" t="n">
-        <v>32.6</v>
+        <v>39.4</v>
       </c>
       <c r="G11" t="n">
-        <v>29.2</v>
+        <v>40.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>29.29</v>
+        <v>19.49</v>
       </c>
       <c r="D12" t="n">
-        <v>2.77</v>
+        <v>1.75</v>
       </c>
       <c r="E12" t="n">
-        <v>20.2</v>
+        <v>40</v>
       </c>
       <c r="F12" t="n">
-        <v>21.3</v>
+        <v>31.1</v>
       </c>
       <c r="G12" t="n">
-        <v>21</v>
+        <v>35.6</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="13">
@@ -816,52 +816,52 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>16.08</v>
+        <v>16.29</v>
       </c>
       <c r="D13" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="E13" t="n">
-        <v>20.2</v>
+        <v>28.9</v>
       </c>
       <c r="F13" t="n">
-        <v>20.8</v>
+        <v>28.3</v>
       </c>
       <c r="G13" t="n">
-        <v>20.6</v>
+        <v>28.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>27.18</v>
+        <v>29.74</v>
       </c>
       <c r="D14" t="n">
-        <v>2.28</v>
+        <v>2.82</v>
       </c>
       <c r="E14" t="n">
-        <v>12.4</v>
+        <v>24.4</v>
       </c>
       <c r="F14" t="n">
-        <v>12.4</v>
+        <v>25.6</v>
       </c>
       <c r="G14" t="n">
-        <v>12.4</v>
+        <v>25.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="15">
@@ -876,472 +876,472 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>20.83</v>
+        <v>21.35</v>
       </c>
       <c r="D15" t="n">
-        <v>1.71</v>
+        <v>1.75</v>
       </c>
       <c r="E15" t="n">
-        <v>7.9</v>
+        <v>22.2</v>
       </c>
       <c r="F15" t="n">
-        <v>10.1</v>
+        <v>22.8</v>
       </c>
       <c r="G15" t="n">
-        <v>9.4</v>
+        <v>22.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>19.31</v>
+        <v>33.95</v>
       </c>
       <c r="D16" t="n">
-        <v>3.17</v>
+        <v>1.88</v>
       </c>
       <c r="E16" t="n">
-        <v>7.9</v>
+        <v>18.9</v>
       </c>
       <c r="F16" t="n">
-        <v>7.9</v>
+        <v>18.9</v>
       </c>
       <c r="G16" t="n">
-        <v>7.9</v>
+        <v>18.9</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>28.85</v>
+        <v>10.01</v>
       </c>
       <c r="D17" t="n">
-        <v>3.1</v>
+        <v>0.92</v>
       </c>
       <c r="E17" t="n">
-        <v>6.7</v>
+        <v>4.4</v>
       </c>
       <c r="F17" t="n">
-        <v>6.7</v>
+        <v>16.1</v>
       </c>
       <c r="G17" t="n">
-        <v>6.7</v>
+        <v>12.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23.99</v>
+        <v>19.74</v>
       </c>
       <c r="D18" t="n">
-        <v>2.24</v>
+        <v>3.24</v>
       </c>
       <c r="E18" t="n">
-        <v>6.7</v>
+        <v>15</v>
       </c>
       <c r="F18" t="n">
-        <v>6.7</v>
+        <v>11.1</v>
       </c>
       <c r="G18" t="n">
-        <v>6.7</v>
+        <v>12.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>52.76</v>
+        <v>22.17</v>
       </c>
       <c r="D19" t="n">
-        <v>3.4</v>
+        <v>2.04</v>
       </c>
       <c r="E19" t="n">
-        <v>6.7</v>
+        <v>14.4</v>
       </c>
       <c r="F19" t="n">
-        <v>6.7</v>
+        <v>11.1</v>
       </c>
       <c r="G19" t="n">
-        <v>6.7</v>
+        <v>12.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>71.39</v>
+        <v>36.49</v>
       </c>
       <c r="D20" t="n">
-        <v>3.27</v>
+        <v>3.09</v>
       </c>
       <c r="E20" t="n">
-        <v>3.4</v>
+        <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>7.3</v>
+        <v>11.7</v>
       </c>
       <c r="G20" t="n">
-        <v>6.1</v>
+        <v>11.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>44.6</v>
+        <v>28.25</v>
       </c>
       <c r="D21" t="n">
-        <v>3.67</v>
+        <v>2.18</v>
       </c>
       <c r="E21" t="n">
-        <v>5.6</v>
+        <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>5.6</v>
+        <v>11.1</v>
       </c>
       <c r="G21" t="n">
-        <v>5.6</v>
+        <v>10.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>35.42</v>
+        <v>24.55</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>2.29</v>
       </c>
       <c r="E22" t="n">
-        <v>4.5</v>
+        <v>8.9</v>
       </c>
       <c r="F22" t="n">
-        <v>4.5</v>
+        <v>11.1</v>
       </c>
       <c r="G22" t="n">
-        <v>4.5</v>
+        <v>10.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>20.22</v>
+        <v>75.48</v>
       </c>
       <c r="D23" t="n">
-        <v>1.83</v>
+        <v>3.46</v>
       </c>
       <c r="E23" t="n">
-        <v>3.4</v>
+        <v>5.6</v>
       </c>
       <c r="F23" t="n">
-        <v>3.4</v>
+        <v>12.2</v>
       </c>
       <c r="G23" t="n">
-        <v>3.4</v>
+        <v>10.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>31.75</v>
+        <v>44.64</v>
       </c>
       <c r="D24" t="n">
-        <v>1.76</v>
+        <v>3.77</v>
       </c>
       <c r="E24" t="n">
-        <v>3.4</v>
+        <v>7.8</v>
       </c>
       <c r="F24" t="n">
-        <v>3.4</v>
+        <v>11.1</v>
       </c>
       <c r="G24" t="n">
-        <v>3.4</v>
+        <v>10.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>27.33</v>
+        <v>29.11</v>
       </c>
       <c r="D25" t="n">
-        <v>2.11</v>
+        <v>3.17</v>
       </c>
       <c r="E25" t="n">
-        <v>2.2</v>
+        <v>8.9</v>
       </c>
       <c r="F25" t="n">
-        <v>3.4</v>
+        <v>10</v>
       </c>
       <c r="G25" t="n">
-        <v>3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>9.85</v>
+        <v>20.63</v>
       </c>
       <c r="D26" t="n">
-        <v>0.63</v>
+        <v>1.87</v>
       </c>
       <c r="E26" t="n">
-        <v>3.4</v>
+        <v>8.9</v>
       </c>
       <c r="F26" t="n">
-        <v>2.2</v>
+        <v>9.4</v>
       </c>
       <c r="G26" t="n">
-        <v>2.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>14.83</v>
+        <v>53.85</v>
       </c>
       <c r="D27" t="n">
-        <v>2.19</v>
+        <v>3.47</v>
       </c>
       <c r="E27" t="n">
-        <v>3.4</v>
+        <v>8.9</v>
       </c>
       <c r="F27" t="n">
-        <v>2.2</v>
+        <v>8.9</v>
       </c>
       <c r="G27" t="n">
-        <v>2.6</v>
+        <v>8.9</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>21.77</v>
+        <v>14.98</v>
       </c>
       <c r="D28" t="n">
-        <v>2.01</v>
+        <v>2.21</v>
       </c>
       <c r="E28" t="n">
-        <v>2.2</v>
+        <v>10</v>
       </c>
       <c r="F28" t="n">
-        <v>2.2</v>
+        <v>6.1</v>
       </c>
       <c r="G28" t="n">
-        <v>2.2</v>
+        <v>7.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9.779999999999999</v>
+        <v>18.64</v>
       </c>
       <c r="D29" t="n">
-        <v>0.9</v>
+        <v>1.56</v>
       </c>
       <c r="E29" t="n">
-        <v>2.2</v>
+        <v>5.6</v>
       </c>
       <c r="F29" t="n">
-        <v>2.2</v>
+        <v>7.8</v>
       </c>
       <c r="G29" t="n">
-        <v>2.2</v>
+        <v>7.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>18.07</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="D30" t="n">
-        <v>1.51</v>
+        <v>0.64</v>
       </c>
       <c r="E30" t="n">
-        <v>2.2</v>
+        <v>5.6</v>
       </c>
       <c r="F30" t="n">
-        <v>2.2</v>
+        <v>6.1</v>
       </c>
       <c r="G30" t="n">
-        <v>2.2</v>
+        <v>5.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>21.91</v>
+        <v>22.49</v>
       </c>
       <c r="D31" t="n">
-        <v>1.79</v>
+        <v>1.84</v>
       </c>
       <c r="E31" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
       <c r="F31" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
       <c r="G31" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18.56</v>
+        <v>18.91</v>
       </c>
       <c r="D32" t="n">
-        <v>1.38</v>
+        <v>1.41</v>
       </c>
       <c r="E32" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
       <c r="F32" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
       <c r="G32" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Jul 28 11:45:36 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,112 +486,112 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>7.16</v>
       </c>
       <c r="D2" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="E2" t="n">
-        <v>87.8</v>
+        <v>96.7</v>
       </c>
       <c r="F2" t="n">
-        <v>78.90000000000001</v>
+        <v>96.2</v>
       </c>
       <c r="G2" t="n">
-        <v>83.3</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>75.36</v>
+        <v>10.26</v>
       </c>
       <c r="D3" t="n">
-        <v>8.5</v>
+        <v>1.25</v>
       </c>
       <c r="E3" t="n">
-        <v>63.3</v>
+        <v>61.5</v>
       </c>
       <c r="F3" t="n">
-        <v>72.2</v>
+        <v>60.4</v>
       </c>
       <c r="G3" t="n">
-        <v>67.8</v>
+        <v>61</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.3</v>
+        <v>70.44</v>
       </c>
       <c r="D4" t="n">
-        <v>1.25</v>
+        <v>7.95</v>
       </c>
       <c r="E4" t="n">
-        <v>65.59999999999999</v>
+        <v>38.5</v>
       </c>
       <c r="F4" t="n">
-        <v>60.6</v>
+        <v>64.8</v>
       </c>
       <c r="G4" t="n">
-        <v>63.1</v>
+        <v>51.6</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28.47</v>
+        <v>14.82</v>
       </c>
       <c r="D5" t="n">
-        <v>2.61</v>
+        <v>1.21</v>
       </c>
       <c r="E5" t="n">
-        <v>60</v>
+        <v>51.6</v>
       </c>
       <c r="F5" t="n">
-        <v>55.6</v>
+        <v>49.5</v>
       </c>
       <c r="G5" t="n">
-        <v>57.8</v>
+        <v>50.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="6">
@@ -606,52 +606,52 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17.75</v>
+        <v>17.77</v>
       </c>
       <c r="D6" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="E6" t="n">
-        <v>36.7</v>
+        <v>37.4</v>
       </c>
       <c r="F6" t="n">
-        <v>61.1</v>
+        <v>62.6</v>
       </c>
       <c r="G6" t="n">
-        <v>48.9</v>
+        <v>50</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>14.69</v>
+        <v>19.9</v>
       </c>
       <c r="D7" t="n">
-        <v>1.2</v>
+        <v>3.45</v>
       </c>
       <c r="E7" t="n">
-        <v>46.7</v>
+        <v>52.7</v>
       </c>
       <c r="F7" t="n">
-        <v>45.6</v>
+        <v>42.9</v>
       </c>
       <c r="G7" t="n">
-        <v>46.1</v>
+        <v>47.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="8">
@@ -666,742 +666,742 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28.5</v>
+        <v>28.62</v>
       </c>
       <c r="D8" t="n">
-        <v>2.39</v>
+        <v>2.4</v>
       </c>
       <c r="E8" t="n">
-        <v>46.1</v>
+        <v>47.3</v>
       </c>
       <c r="F8" t="n">
-        <v>45.6</v>
+        <v>47.3</v>
       </c>
       <c r="G8" t="n">
-        <v>45.8</v>
+        <v>47.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>13.82</v>
+        <v>27.58</v>
       </c>
       <c r="D9" t="n">
-        <v>1.3</v>
+        <v>2.05</v>
       </c>
       <c r="E9" t="n">
-        <v>44.4</v>
+        <v>48.4</v>
       </c>
       <c r="F9" t="n">
-        <v>42.8</v>
+        <v>41.8</v>
       </c>
       <c r="G9" t="n">
-        <v>43.6</v>
+        <v>45.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>27.47</v>
+        <v>13.88</v>
       </c>
       <c r="D10" t="n">
-        <v>2.04</v>
+        <v>1.3</v>
       </c>
       <c r="E10" t="n">
-        <v>47.8</v>
+        <v>46.2</v>
       </c>
       <c r="F10" t="n">
-        <v>38.9</v>
+        <v>42.9</v>
       </c>
       <c r="G10" t="n">
-        <v>43.3</v>
+        <v>44.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.45</v>
+        <v>28.11</v>
       </c>
       <c r="D11" t="n">
-        <v>3.37</v>
+        <v>2.58</v>
       </c>
       <c r="E11" t="n">
-        <v>41.1</v>
+        <v>45.1</v>
       </c>
       <c r="F11" t="n">
-        <v>39.4</v>
+        <v>40.7</v>
       </c>
       <c r="G11" t="n">
-        <v>40.3</v>
+        <v>42.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>19.49</v>
+        <v>21.78</v>
       </c>
       <c r="D12" t="n">
-        <v>1.75</v>
+        <v>1.78</v>
       </c>
       <c r="E12" t="n">
-        <v>40</v>
+        <v>34.1</v>
       </c>
       <c r="F12" t="n">
-        <v>31.1</v>
+        <v>33.5</v>
       </c>
       <c r="G12" t="n">
-        <v>35.6</v>
+        <v>33.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>16.29</v>
+        <v>19.45</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9</v>
+        <v>1.74</v>
       </c>
       <c r="E13" t="n">
-        <v>28.9</v>
+        <v>38.5</v>
       </c>
       <c r="F13" t="n">
-        <v>28.3</v>
+        <v>29.1</v>
       </c>
       <c r="G13" t="n">
-        <v>28.5</v>
+        <v>31.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>29.74</v>
+        <v>16.31</v>
       </c>
       <c r="D14" t="n">
-        <v>2.82</v>
+        <v>0.9</v>
       </c>
       <c r="E14" t="n">
-        <v>24.4</v>
+        <v>31.9</v>
       </c>
       <c r="F14" t="n">
-        <v>25.6</v>
+        <v>28.6</v>
       </c>
       <c r="G14" t="n">
-        <v>25.2</v>
+        <v>29.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>21.35</v>
+        <v>10.15</v>
       </c>
       <c r="D15" t="n">
-        <v>1.75</v>
+        <v>0.93</v>
       </c>
       <c r="E15" t="n">
-        <v>22.2</v>
+        <v>14.3</v>
       </c>
       <c r="F15" t="n">
-        <v>22.8</v>
+        <v>24.7</v>
       </c>
       <c r="G15" t="n">
-        <v>22.6</v>
+        <v>21.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>33.95</v>
+        <v>15.1</v>
       </c>
       <c r="D16" t="n">
-        <v>1.88</v>
+        <v>2.23</v>
       </c>
       <c r="E16" t="n">
-        <v>18.9</v>
+        <v>20.9</v>
       </c>
       <c r="F16" t="n">
-        <v>18.9</v>
+        <v>18.7</v>
       </c>
       <c r="G16" t="n">
-        <v>18.9</v>
+        <v>19.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.01</v>
+        <v>18.83</v>
       </c>
       <c r="D17" t="n">
-        <v>0.92</v>
+        <v>1.57</v>
       </c>
       <c r="E17" t="n">
-        <v>4.4</v>
+        <v>13.7</v>
       </c>
       <c r="F17" t="n">
-        <v>16.1</v>
+        <v>13.2</v>
       </c>
       <c r="G17" t="n">
-        <v>12.6</v>
+        <v>13.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19.74</v>
+        <v>28.34</v>
       </c>
       <c r="D18" t="n">
-        <v>3.24</v>
+        <v>2.19</v>
       </c>
       <c r="E18" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F18" t="n">
-        <v>11.1</v>
+        <v>12.1</v>
       </c>
       <c r="G18" t="n">
-        <v>12.3</v>
+        <v>11.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22.17</v>
+        <v>20.71</v>
       </c>
       <c r="D19" t="n">
-        <v>2.04</v>
+        <v>1.87</v>
       </c>
       <c r="E19" t="n">
-        <v>14.4</v>
+        <v>11</v>
       </c>
       <c r="F19" t="n">
-        <v>11.1</v>
+        <v>9.9</v>
       </c>
       <c r="G19" t="n">
-        <v>12.1</v>
+        <v>10.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>36.49</v>
+        <v>24.18</v>
       </c>
       <c r="D20" t="n">
-        <v>3.09</v>
+        <v>2.26</v>
       </c>
       <c r="E20" t="n">
-        <v>10</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F20" t="n">
-        <v>11.7</v>
+        <v>9.9</v>
       </c>
       <c r="G20" t="n">
-        <v>11.2</v>
+        <v>9.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>28.25</v>
+        <v>71.7</v>
       </c>
       <c r="D21" t="n">
-        <v>2.18</v>
+        <v>3.29</v>
       </c>
       <c r="E21" t="n">
-        <v>10</v>
+        <v>5.5</v>
       </c>
       <c r="F21" t="n">
-        <v>11.1</v>
+        <v>10.4</v>
       </c>
       <c r="G21" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>24.55</v>
+        <v>32.53</v>
       </c>
       <c r="D22" t="n">
-        <v>2.29</v>
+        <v>1.8</v>
       </c>
       <c r="E22" t="n">
-        <v>8.9</v>
+        <v>12.1</v>
       </c>
       <c r="F22" t="n">
-        <v>11.1</v>
+        <v>6</v>
       </c>
       <c r="G22" t="n">
-        <v>10.4</v>
+        <v>7.9</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>75.48</v>
+        <v>19.23</v>
       </c>
       <c r="D23" t="n">
-        <v>3.46</v>
+        <v>3.17</v>
       </c>
       <c r="E23" t="n">
-        <v>5.6</v>
+        <v>6.6</v>
       </c>
       <c r="F23" t="n">
-        <v>12.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>10.2</v>
+        <v>7.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>44.64</v>
+        <v>22.02</v>
       </c>
       <c r="D24" t="n">
-        <v>3.77</v>
+        <v>2.03</v>
       </c>
       <c r="E24" t="n">
-        <v>7.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>11.1</v>
+        <v>7.1</v>
       </c>
       <c r="G24" t="n">
-        <v>10.1</v>
+        <v>7.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29.11</v>
+        <v>44.18</v>
       </c>
       <c r="D25" t="n">
-        <v>3.17</v>
+        <v>3.73</v>
       </c>
       <c r="E25" t="n">
-        <v>8.9</v>
+        <v>1.1</v>
       </c>
       <c r="F25" t="n">
-        <v>10</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G25" t="n">
-        <v>9.699999999999999</v>
+        <v>6.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>20.63</v>
+        <v>9.91</v>
       </c>
       <c r="D26" t="n">
-        <v>1.87</v>
+        <v>0.64</v>
       </c>
       <c r="E26" t="n">
-        <v>8.9</v>
+        <v>5.5</v>
       </c>
       <c r="F26" t="n">
-        <v>9.4</v>
+        <v>6.6</v>
       </c>
       <c r="G26" t="n">
-        <v>9.300000000000001</v>
+        <v>6.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>53.85</v>
+        <v>22.58</v>
       </c>
       <c r="D27" t="n">
-        <v>3.47</v>
+        <v>1.85</v>
       </c>
       <c r="E27" t="n">
-        <v>8.9</v>
+        <v>6.6</v>
       </c>
       <c r="F27" t="n">
-        <v>8.9</v>
+        <v>6</v>
       </c>
       <c r="G27" t="n">
-        <v>8.9</v>
+        <v>6.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>14.98</v>
+        <v>28.26</v>
       </c>
       <c r="D28" t="n">
-        <v>2.21</v>
+        <v>3.08</v>
       </c>
       <c r="E28" t="n">
-        <v>10</v>
+        <v>5.5</v>
       </c>
       <c r="F28" t="n">
-        <v>6.1</v>
+        <v>5.5</v>
       </c>
       <c r="G28" t="n">
-        <v>7.3</v>
+        <v>5.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.64</v>
+        <v>52.5</v>
       </c>
       <c r="D29" t="n">
-        <v>1.56</v>
+        <v>3.39</v>
       </c>
       <c r="E29" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="F29" t="n">
-        <v>7.8</v>
+        <v>5.5</v>
       </c>
       <c r="G29" t="n">
-        <v>7.1</v>
+        <v>5.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9.970000000000001</v>
+        <v>18.73</v>
       </c>
       <c r="D30" t="n">
-        <v>0.64</v>
+        <v>1.4</v>
       </c>
       <c r="E30" t="n">
-        <v>5.6</v>
+        <v>4.4</v>
       </c>
       <c r="F30" t="n">
-        <v>6.1</v>
+        <v>4.4</v>
       </c>
       <c r="G30" t="n">
-        <v>5.9</v>
+        <v>4.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22.49</v>
+        <v>34.13</v>
       </c>
       <c r="D31" t="n">
-        <v>1.84</v>
+        <v>2.96</v>
       </c>
       <c r="E31" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="F31" t="n">
-        <v>4.4</v>
+        <v>3.3</v>
       </c>
       <c r="G31" t="n">
-        <v>4.4</v>
+        <v>3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18.91</v>
+        <v>27.9</v>
       </c>
       <c r="D32" t="n">
-        <v>1.41</v>
+        <v>2.64</v>
       </c>
       <c r="E32" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="F32" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="G32" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Jul 29 11:49:19 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.16</v>
+        <v>7.14</v>
       </c>
       <c r="D2" t="n">
         <v>0.68</v>
       </c>
       <c r="E2" t="n">
-        <v>96.7</v>
+        <v>95.7</v>
       </c>
       <c r="F2" t="n">
-        <v>96.2</v>
+        <v>95.7</v>
       </c>
       <c r="G2" t="n">
-        <v>96.40000000000001</v>
+        <v>95.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="3">
@@ -516,52 +516,52 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.26</v>
+        <v>10.33</v>
       </c>
       <c r="D3" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
       <c r="E3" t="n">
-        <v>61.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>60.4</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>61</v>
+        <v>68.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>70.44</v>
+        <v>28.41</v>
       </c>
       <c r="D4" t="n">
-        <v>7.95</v>
+        <v>2.61</v>
       </c>
       <c r="E4" t="n">
-        <v>38.5</v>
+        <v>59.8</v>
       </c>
       <c r="F4" t="n">
-        <v>64.8</v>
+        <v>56</v>
       </c>
       <c r="G4" t="n">
-        <v>51.6</v>
+        <v>57.9</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="5">
@@ -576,52 +576,52 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14.82</v>
+        <v>14.95</v>
       </c>
       <c r="D5" t="n">
-        <v>1.21</v>
+        <v>1.22</v>
       </c>
       <c r="E5" t="n">
-        <v>51.6</v>
+        <v>56.5</v>
       </c>
       <c r="F5" t="n">
-        <v>49.5</v>
+        <v>54.3</v>
       </c>
       <c r="G5" t="n">
-        <v>50.5</v>
+        <v>55.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17.77</v>
+        <v>71.16</v>
       </c>
       <c r="D6" t="n">
-        <v>1.72</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>37.4</v>
+        <v>42.4</v>
       </c>
       <c r="F6" t="n">
-        <v>62.6</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>50</v>
+        <v>54.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="7">
@@ -636,22 +636,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.9</v>
+        <v>20.15</v>
       </c>
       <c r="D7" t="n">
-        <v>3.45</v>
+        <v>3.49</v>
       </c>
       <c r="E7" t="n">
-        <v>52.7</v>
+        <v>59.8</v>
       </c>
       <c r="F7" t="n">
-        <v>42.9</v>
+        <v>47.8</v>
       </c>
       <c r="G7" t="n">
-        <v>47.8</v>
+        <v>53.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="8">
@@ -666,22 +666,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28.62</v>
+        <v>28.98</v>
       </c>
       <c r="D8" t="n">
-        <v>2.4</v>
+        <v>2.43</v>
       </c>
       <c r="E8" t="n">
-        <v>47.3</v>
+        <v>56.5</v>
       </c>
       <c r="F8" t="n">
-        <v>47.3</v>
+        <v>47.8</v>
       </c>
       <c r="G8" t="n">
-        <v>47.3</v>
+        <v>52.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="9">
@@ -696,112 +696,112 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27.58</v>
+        <v>27.77</v>
       </c>
       <c r="D9" t="n">
-        <v>2.05</v>
+        <v>2.07</v>
       </c>
       <c r="E9" t="n">
-        <v>48.4</v>
+        <v>51.6</v>
       </c>
       <c r="F9" t="n">
-        <v>41.8</v>
+        <v>51.1</v>
       </c>
       <c r="G9" t="n">
-        <v>45.1</v>
+        <v>51.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>13.88</v>
+        <v>17.86</v>
       </c>
       <c r="D10" t="n">
-        <v>1.3</v>
+        <v>1.72</v>
       </c>
       <c r="E10" t="n">
-        <v>46.2</v>
+        <v>39.1</v>
       </c>
       <c r="F10" t="n">
-        <v>42.9</v>
+        <v>62.5</v>
       </c>
       <c r="G10" t="n">
-        <v>44.5</v>
+        <v>50.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28.11</v>
+        <v>22.45</v>
       </c>
       <c r="D11" t="n">
-        <v>2.58</v>
+        <v>1.84</v>
       </c>
       <c r="E11" t="n">
-        <v>45.1</v>
+        <v>44.6</v>
       </c>
       <c r="F11" t="n">
-        <v>40.7</v>
+        <v>42.9</v>
       </c>
       <c r="G11" t="n">
-        <v>42.9</v>
+        <v>43.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>21.78</v>
+        <v>13.85</v>
       </c>
       <c r="D12" t="n">
-        <v>1.78</v>
+        <v>1.3</v>
       </c>
       <c r="E12" t="n">
-        <v>34.1</v>
+        <v>44.6</v>
       </c>
       <c r="F12" t="n">
-        <v>33.5</v>
+        <v>42.9</v>
       </c>
       <c r="G12" t="n">
-        <v>33.8</v>
+        <v>43.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="13">
@@ -816,502 +816,502 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.45</v>
+        <v>19.67</v>
       </c>
       <c r="D13" t="n">
-        <v>1.74</v>
+        <v>1.76</v>
       </c>
       <c r="E13" t="n">
-        <v>38.5</v>
+        <v>52.2</v>
       </c>
       <c r="F13" t="n">
-        <v>29.1</v>
+        <v>33.2</v>
       </c>
       <c r="G13" t="n">
-        <v>31.9</v>
+        <v>42.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>16.31</v>
+        <v>15.37</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9</v>
+        <v>2.27</v>
       </c>
       <c r="E14" t="n">
-        <v>31.9</v>
+        <v>39.1</v>
       </c>
       <c r="F14" t="n">
-        <v>28.6</v>
+        <v>33.2</v>
       </c>
       <c r="G14" t="n">
-        <v>29.6</v>
+        <v>36.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10.15</v>
+        <v>16.7</v>
       </c>
       <c r="D15" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="E15" t="n">
-        <v>14.3</v>
+        <v>35.9</v>
       </c>
       <c r="F15" t="n">
-        <v>24.7</v>
+        <v>35.3</v>
       </c>
       <c r="G15" t="n">
-        <v>21.6</v>
+        <v>35.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15.1</v>
+        <v>10.44</v>
       </c>
       <c r="D16" t="n">
-        <v>2.23</v>
+        <v>0.96</v>
       </c>
       <c r="E16" t="n">
-        <v>20.9</v>
+        <v>23.9</v>
       </c>
       <c r="F16" t="n">
-        <v>18.7</v>
+        <v>40.2</v>
       </c>
       <c r="G16" t="n">
-        <v>19.3</v>
+        <v>32.1</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>18.83</v>
+        <v>23.4</v>
       </c>
       <c r="D17" t="n">
-        <v>1.57</v>
+        <v>1.91</v>
       </c>
       <c r="E17" t="n">
-        <v>13.7</v>
+        <v>23.9</v>
       </c>
       <c r="F17" t="n">
-        <v>13.2</v>
+        <v>22.3</v>
       </c>
       <c r="G17" t="n">
-        <v>13.4</v>
+        <v>22.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28.34</v>
+        <v>19.07</v>
       </c>
       <c r="D18" t="n">
-        <v>2.19</v>
+        <v>1.59</v>
       </c>
       <c r="E18" t="n">
-        <v>11</v>
+        <v>22.8</v>
       </c>
       <c r="F18" t="n">
-        <v>12.1</v>
+        <v>20.1</v>
       </c>
       <c r="G18" t="n">
-        <v>11.8</v>
+        <v>20.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20.71</v>
+        <v>22.39</v>
       </c>
       <c r="D19" t="n">
-        <v>1.87</v>
+        <v>2.06</v>
       </c>
       <c r="E19" t="n">
-        <v>11</v>
+        <v>16.3</v>
       </c>
       <c r="F19" t="n">
-        <v>9.9</v>
+        <v>16.3</v>
       </c>
       <c r="G19" t="n">
-        <v>10.2</v>
+        <v>16.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>24.18</v>
+        <v>28.91</v>
       </c>
       <c r="D20" t="n">
-        <v>2.26</v>
+        <v>2.23</v>
       </c>
       <c r="E20" t="n">
-        <v>8.800000000000001</v>
+        <v>13</v>
       </c>
       <c r="F20" t="n">
-        <v>9.9</v>
+        <v>16.8</v>
       </c>
       <c r="G20" t="n">
-        <v>9.6</v>
+        <v>15.7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>71.7</v>
+        <v>21.17</v>
       </c>
       <c r="D21" t="n">
-        <v>3.29</v>
+        <v>1.91</v>
       </c>
       <c r="E21" t="n">
-        <v>5.5</v>
+        <v>14.1</v>
       </c>
       <c r="F21" t="n">
-        <v>10.4</v>
+        <v>13.6</v>
       </c>
       <c r="G21" t="n">
-        <v>9</v>
+        <v>13.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>32.53</v>
+        <v>19.6</v>
       </c>
       <c r="D22" t="n">
-        <v>1.8</v>
+        <v>3.23</v>
       </c>
       <c r="E22" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="F22" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G22" t="n">
-        <v>7.9</v>
+        <v>12</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>19.23</v>
+        <v>24.45</v>
       </c>
       <c r="D23" t="n">
-        <v>3.17</v>
+        <v>2.28</v>
       </c>
       <c r="E23" t="n">
-        <v>6.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>8.199999999999999</v>
+        <v>12</v>
       </c>
       <c r="G23" t="n">
-        <v>7.7</v>
+        <v>11.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.02</v>
+        <v>32.72</v>
       </c>
       <c r="D24" t="n">
-        <v>2.03</v>
+        <v>1.82</v>
       </c>
       <c r="E24" t="n">
-        <v>8.800000000000001</v>
+        <v>13</v>
       </c>
       <c r="F24" t="n">
-        <v>7.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G24" t="n">
-        <v>7.6</v>
+        <v>10.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>44.18</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="D25" t="n">
-        <v>3.73</v>
+        <v>3.3</v>
       </c>
       <c r="E25" t="n">
-        <v>1.1</v>
+        <v>6.5</v>
       </c>
       <c r="F25" t="n">
-        <v>8.800000000000001</v>
+        <v>12</v>
       </c>
       <c r="G25" t="n">
-        <v>6.5</v>
+        <v>10.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>9.91</v>
+        <v>53.43</v>
       </c>
       <c r="D26" t="n">
-        <v>0.64</v>
+        <v>3.44</v>
       </c>
       <c r="E26" t="n">
-        <v>5.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F26" t="n">
-        <v>6.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G26" t="n">
-        <v>6.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.58</v>
+        <v>28.6</v>
       </c>
       <c r="D27" t="n">
-        <v>1.85</v>
+        <v>3.12</v>
       </c>
       <c r="E27" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="F27" t="n">
-        <v>6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G27" t="n">
-        <v>6.2</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>28.26</v>
+        <v>10</v>
       </c>
       <c r="D28" t="n">
-        <v>3.08</v>
+        <v>0.64</v>
       </c>
       <c r="E28" t="n">
-        <v>5.5</v>
+        <v>7.6</v>
       </c>
       <c r="F28" t="n">
-        <v>5.5</v>
+        <v>7.1</v>
       </c>
       <c r="G28" t="n">
-        <v>5.5</v>
+        <v>7.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>52.5</v>
+        <v>44.13</v>
       </c>
       <c r="D29" t="n">
-        <v>3.39</v>
+        <v>3.73</v>
       </c>
       <c r="E29" t="n">
-        <v>5.5</v>
+        <v>1.1</v>
       </c>
       <c r="F29" t="n">
-        <v>5.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G29" t="n">
-        <v>5.5</v>
+        <v>6.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="30">
@@ -1326,22 +1326,22 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>18.73</v>
+        <v>19.01</v>
       </c>
       <c r="D30" t="n">
-        <v>1.4</v>
+        <v>1.42</v>
       </c>
       <c r="E30" t="n">
-        <v>4.4</v>
+        <v>6.5</v>
       </c>
       <c r="F30" t="n">
-        <v>4.4</v>
+        <v>6.5</v>
       </c>
       <c r="G30" t="n">
-        <v>4.4</v>
+        <v>6.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>34.13</v>
+        <v>34.21</v>
       </c>
       <c r="D31" t="n">
-        <v>2.96</v>
+        <v>2.97</v>
       </c>
       <c r="E31" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="F31" t="n">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="G31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>27.9</v>
+        <v>28.06</v>
       </c>
       <c r="D32" t="n">
-        <v>2.64</v>
+        <v>2.65</v>
       </c>
       <c r="E32" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="F32" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="G32" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Jul 30 11:33:40 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.14</v>
+        <v>7.32</v>
       </c>
       <c r="D2" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>95.7</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>95.7</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>95.7</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="3">
@@ -516,382 +516,382 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.33</v>
+        <v>10.41</v>
       </c>
       <c r="D3" t="n">
-        <v>1.26</v>
+        <v>1.27</v>
       </c>
       <c r="E3" t="n">
-        <v>69.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="F3" t="n">
-        <v>67.40000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="G3" t="n">
-        <v>68.5</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28.41</v>
+        <v>20.7</v>
       </c>
       <c r="D4" t="n">
-        <v>2.61</v>
+        <v>3.59</v>
       </c>
       <c r="E4" t="n">
-        <v>59.8</v>
+        <v>75.8</v>
       </c>
       <c r="F4" t="n">
-        <v>56</v>
+        <v>64.5</v>
       </c>
       <c r="G4" t="n">
-        <v>57.9</v>
+        <v>70.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14.95</v>
+        <v>14.26</v>
       </c>
       <c r="D5" t="n">
-        <v>1.22</v>
+        <v>1.34</v>
       </c>
       <c r="E5" t="n">
-        <v>56.5</v>
+        <v>63.4</v>
       </c>
       <c r="F5" t="n">
-        <v>54.3</v>
+        <v>62.4</v>
       </c>
       <c r="G5" t="n">
-        <v>55.4</v>
+        <v>62.9</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>71.16</v>
+        <v>15.12</v>
       </c>
       <c r="D6" t="n">
-        <v>8.029999999999999</v>
+        <v>1.23</v>
       </c>
       <c r="E6" t="n">
-        <v>42.4</v>
+        <v>59.1</v>
       </c>
       <c r="F6" t="n">
-        <v>67.40000000000001</v>
+        <v>58.1</v>
       </c>
       <c r="G6" t="n">
-        <v>54.9</v>
+        <v>58.6</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.15</v>
+        <v>28.23</v>
       </c>
       <c r="D7" t="n">
-        <v>3.49</v>
+        <v>2.1</v>
       </c>
       <c r="E7" t="n">
-        <v>59.8</v>
+        <v>59.1</v>
       </c>
       <c r="F7" t="n">
-        <v>47.8</v>
+        <v>56.5</v>
       </c>
       <c r="G7" t="n">
-        <v>53.8</v>
+        <v>57.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28.98</v>
+        <v>18.04</v>
       </c>
       <c r="D8" t="n">
-        <v>2.43</v>
+        <v>1.74</v>
       </c>
       <c r="E8" t="n">
-        <v>56.5</v>
+        <v>46.2</v>
       </c>
       <c r="F8" t="n">
-        <v>47.8</v>
+        <v>68.8</v>
       </c>
       <c r="G8" t="n">
-        <v>52.2</v>
+        <v>57.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27.77</v>
+        <v>29.3</v>
       </c>
       <c r="D9" t="n">
-        <v>2.07</v>
+        <v>2.46</v>
       </c>
       <c r="E9" t="n">
-        <v>51.6</v>
+        <v>57</v>
       </c>
       <c r="F9" t="n">
-        <v>51.1</v>
+        <v>55.4</v>
       </c>
       <c r="G9" t="n">
-        <v>51.4</v>
+        <v>56.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>17.86</v>
+        <v>22.59</v>
       </c>
       <c r="D10" t="n">
-        <v>1.72</v>
+        <v>1.85</v>
       </c>
       <c r="E10" t="n">
-        <v>39.1</v>
+        <v>47.3</v>
       </c>
       <c r="F10" t="n">
-        <v>62.5</v>
+        <v>44.6</v>
       </c>
       <c r="G10" t="n">
-        <v>50.8</v>
+        <v>46</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>22.45</v>
+        <v>28.16</v>
       </c>
       <c r="D11" t="n">
-        <v>1.84</v>
+        <v>2.59</v>
       </c>
       <c r="E11" t="n">
-        <v>44.6</v>
+        <v>45.7</v>
       </c>
       <c r="F11" t="n">
-        <v>42.9</v>
+        <v>45.2</v>
       </c>
       <c r="G11" t="n">
-        <v>43.8</v>
+        <v>45.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>13.85</v>
+        <v>15.51</v>
       </c>
       <c r="D12" t="n">
-        <v>1.3</v>
+        <v>2.29</v>
       </c>
       <c r="E12" t="n">
-        <v>44.6</v>
+        <v>45.2</v>
       </c>
       <c r="F12" t="n">
-        <v>42.9</v>
+        <v>39.8</v>
       </c>
       <c r="G12" t="n">
-        <v>43.8</v>
+        <v>42.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.67</v>
+        <v>16.86</v>
       </c>
       <c r="D13" t="n">
-        <v>1.76</v>
+        <v>0.93</v>
       </c>
       <c r="E13" t="n">
-        <v>52.2</v>
+        <v>40.9</v>
       </c>
       <c r="F13" t="n">
-        <v>33.2</v>
+        <v>38.7</v>
       </c>
       <c r="G13" t="n">
-        <v>42.7</v>
+        <v>39.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.37</v>
+        <v>19.61</v>
       </c>
       <c r="D14" t="n">
-        <v>2.27</v>
+        <v>1.76</v>
       </c>
       <c r="E14" t="n">
-        <v>39.1</v>
+        <v>41.9</v>
       </c>
       <c r="F14" t="n">
-        <v>33.2</v>
+        <v>33.3</v>
       </c>
       <c r="G14" t="n">
-        <v>36.1</v>
+        <v>37.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>16.7</v>
+        <v>67.17</v>
       </c>
       <c r="D15" t="n">
-        <v>0.92</v>
+        <v>7.58</v>
       </c>
       <c r="E15" t="n">
-        <v>35.9</v>
+        <v>20.4</v>
       </c>
       <c r="F15" t="n">
-        <v>35.3</v>
+        <v>54.8</v>
       </c>
       <c r="G15" t="n">
-        <v>35.6</v>
+        <v>37.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="16">
@@ -906,22 +906,22 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.44</v>
+        <v>10.45</v>
       </c>
       <c r="D16" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="E16" t="n">
-        <v>23.9</v>
+        <v>26.3</v>
       </c>
       <c r="F16" t="n">
-        <v>40.2</v>
+        <v>41.4</v>
       </c>
       <c r="G16" t="n">
-        <v>32.1</v>
+        <v>33.9</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="17">
@@ -936,22 +936,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.4</v>
+        <v>23.42</v>
       </c>
       <c r="D17" t="n">
-        <v>1.91</v>
+        <v>1.92</v>
       </c>
       <c r="E17" t="n">
-        <v>23.9</v>
+        <v>25.3</v>
       </c>
       <c r="F17" t="n">
-        <v>22.3</v>
+        <v>26.9</v>
       </c>
       <c r="G17" t="n">
-        <v>22.8</v>
+        <v>26.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="18">
@@ -966,82 +966,82 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19.07</v>
+        <v>19.14</v>
       </c>
       <c r="D18" t="n">
-        <v>1.59</v>
+        <v>1.6</v>
       </c>
       <c r="E18" t="n">
-        <v>22.8</v>
+        <v>23.7</v>
       </c>
       <c r="F18" t="n">
-        <v>20.1</v>
+        <v>24.7</v>
       </c>
       <c r="G18" t="n">
-        <v>20.9</v>
+        <v>24.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22.39</v>
+        <v>28.99</v>
       </c>
       <c r="D19" t="n">
-        <v>2.06</v>
+        <v>2.24</v>
       </c>
       <c r="E19" t="n">
-        <v>16.3</v>
+        <v>15.6</v>
       </c>
       <c r="F19" t="n">
-        <v>16.3</v>
+        <v>19.4</v>
       </c>
       <c r="G19" t="n">
-        <v>16.3</v>
+        <v>18.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>28.91</v>
+        <v>22.41</v>
       </c>
       <c r="D20" t="n">
-        <v>2.23</v>
+        <v>2.07</v>
       </c>
       <c r="E20" t="n">
-        <v>13</v>
+        <v>17.2</v>
       </c>
       <c r="F20" t="n">
-        <v>16.8</v>
+        <v>18.3</v>
       </c>
       <c r="G20" t="n">
-        <v>15.7</v>
+        <v>18</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="21">
@@ -1056,22 +1056,22 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>21.17</v>
+        <v>21.01</v>
       </c>
       <c r="D21" t="n">
-        <v>1.91</v>
+        <v>1.9</v>
       </c>
       <c r="E21" t="n">
-        <v>14.1</v>
+        <v>12.9</v>
       </c>
       <c r="F21" t="n">
-        <v>13.6</v>
+        <v>12.9</v>
       </c>
       <c r="G21" t="n">
-        <v>13.7</v>
+        <v>12.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="22">
@@ -1086,22 +1086,22 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>19.6</v>
+        <v>19.32</v>
       </c>
       <c r="D22" t="n">
-        <v>3.23</v>
+        <v>3.2</v>
       </c>
       <c r="E22" t="n">
-        <v>12</v>
+        <v>10.8</v>
       </c>
       <c r="F22" t="n">
-        <v>12</v>
+        <v>10.8</v>
       </c>
       <c r="G22" t="n">
-        <v>12</v>
+        <v>10.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="23">
@@ -1116,172 +1116,172 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24.45</v>
+        <v>24.21</v>
       </c>
       <c r="D23" t="n">
-        <v>2.28</v>
+        <v>2.26</v>
       </c>
       <c r="E23" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>12</v>
+        <v>10.2</v>
       </c>
       <c r="G23" t="n">
-        <v>11.3</v>
+        <v>10.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>32.72</v>
+        <v>9.99</v>
       </c>
       <c r="D24" t="n">
-        <v>1.82</v>
+        <v>0.64</v>
       </c>
       <c r="E24" t="n">
-        <v>13</v>
+        <v>7.5</v>
       </c>
       <c r="F24" t="n">
-        <v>9.800000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="G24" t="n">
-        <v>10.8</v>
+        <v>7.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>72.09999999999999</v>
+        <v>28.2</v>
       </c>
       <c r="D25" t="n">
-        <v>3.3</v>
+        <v>3.08</v>
       </c>
       <c r="E25" t="n">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="F25" t="n">
-        <v>12</v>
+        <v>5.9</v>
       </c>
       <c r="G25" t="n">
-        <v>10.3</v>
+        <v>5.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>53.43</v>
+        <v>32.26</v>
       </c>
       <c r="D26" t="n">
-        <v>3.44</v>
+        <v>1.79</v>
       </c>
       <c r="E26" t="n">
-        <v>9.800000000000001</v>
+        <v>6.5</v>
       </c>
       <c r="F26" t="n">
-        <v>9.800000000000001</v>
+        <v>5.4</v>
       </c>
       <c r="G26" t="n">
-        <v>9.800000000000001</v>
+        <v>5.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>28.6</v>
+        <v>52.4</v>
       </c>
       <c r="D27" t="n">
-        <v>3.12</v>
+        <v>3.38</v>
       </c>
       <c r="E27" t="n">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="F27" t="n">
-        <v>9.800000000000001</v>
+        <v>5.4</v>
       </c>
       <c r="G27" t="n">
-        <v>8.800000000000001</v>
+        <v>5.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>10</v>
+        <v>18.78</v>
       </c>
       <c r="D28" t="n">
-        <v>0.64</v>
+        <v>1.4</v>
       </c>
       <c r="E28" t="n">
-        <v>7.6</v>
+        <v>5.4</v>
       </c>
       <c r="F28" t="n">
-        <v>7.1</v>
+        <v>4.8</v>
       </c>
       <c r="G28" t="n">
-        <v>7.2</v>
+        <v>5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="29">
@@ -1296,112 +1296,112 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>44.13</v>
+        <v>43.42</v>
       </c>
       <c r="D29" t="n">
-        <v>3.73</v>
+        <v>3.67</v>
       </c>
       <c r="E29" t="n">
         <v>1.1</v>
       </c>
       <c r="F29" t="n">
-        <v>9.199999999999999</v>
+        <v>5.9</v>
       </c>
       <c r="G29" t="n">
-        <v>6.8</v>
+        <v>4.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.01</v>
+        <v>68.78</v>
       </c>
       <c r="D30" t="n">
-        <v>1.42</v>
+        <v>3.16</v>
       </c>
       <c r="E30" t="n">
-        <v>6.5</v>
+        <v>2.2</v>
       </c>
       <c r="F30" t="n">
-        <v>6.5</v>
+        <v>2.2</v>
       </c>
       <c r="G30" t="n">
-        <v>6.5</v>
+        <v>2.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>34.21</v>
+        <v>26.99</v>
       </c>
       <c r="D31" t="n">
-        <v>2.97</v>
+        <v>2.55</v>
       </c>
       <c r="E31" t="n">
-        <v>3.3</v>
+        <v>2.2</v>
       </c>
       <c r="F31" t="n">
-        <v>4.3</v>
+        <v>2.2</v>
       </c>
       <c r="G31" t="n">
-        <v>4</v>
+        <v>2.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>28.06</v>
+        <v>32.86</v>
       </c>
       <c r="D32" t="n">
-        <v>2.65</v>
+        <v>2.85</v>
       </c>
       <c r="E32" t="n">
-        <v>3.3</v>
+        <v>1.1</v>
       </c>
       <c r="F32" t="n">
-        <v>3.3</v>
+        <v>1.1</v>
       </c>
       <c r="G32" t="n">
-        <v>3.3</v>
+        <v>1.1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Jul 31 11:49:14 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.32</v>
+        <v>7.2</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>96.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.41</v>
+        <v>10.36</v>
       </c>
       <c r="D3" t="n">
-        <v>1.27</v>
+        <v>1.26</v>
       </c>
       <c r="E3" t="n">
-        <v>74.7</v>
+        <v>71.8</v>
       </c>
       <c r="F3" t="n">
-        <v>71.5</v>
+        <v>66.5</v>
       </c>
       <c r="G3" t="n">
-        <v>73.09999999999999</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="4">
@@ -546,412 +546,412 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20.7</v>
+        <v>20.5</v>
       </c>
       <c r="D4" t="n">
-        <v>3.59</v>
+        <v>3.57</v>
       </c>
       <c r="E4" t="n">
-        <v>75.8</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>64.5</v>
+        <v>62.8</v>
       </c>
       <c r="G4" t="n">
-        <v>70.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14.26</v>
+        <v>28.31</v>
       </c>
       <c r="D5" t="n">
-        <v>1.34</v>
+        <v>2.11</v>
       </c>
       <c r="E5" t="n">
-        <v>63.4</v>
+        <v>59.6</v>
       </c>
       <c r="F5" t="n">
-        <v>62.4</v>
+        <v>58</v>
       </c>
       <c r="G5" t="n">
-        <v>62.9</v>
+        <v>58.8</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15.12</v>
+        <v>29.57</v>
       </c>
       <c r="D6" t="n">
-        <v>1.23</v>
+        <v>2.48</v>
       </c>
       <c r="E6" t="n">
-        <v>59.1</v>
+        <v>59.6</v>
       </c>
       <c r="F6" t="n">
-        <v>58.1</v>
+        <v>58</v>
       </c>
       <c r="G6" t="n">
-        <v>58.6</v>
+        <v>58.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.23</v>
+        <v>15.1</v>
       </c>
       <c r="D7" t="n">
-        <v>2.1</v>
+        <v>1.23</v>
       </c>
       <c r="E7" t="n">
-        <v>59.1</v>
+        <v>58.5</v>
       </c>
       <c r="F7" t="n">
-        <v>56.5</v>
+        <v>58</v>
       </c>
       <c r="G7" t="n">
-        <v>57.8</v>
+        <v>58.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>18.04</v>
+        <v>28.41</v>
       </c>
       <c r="D8" t="n">
-        <v>1.74</v>
+        <v>2.61</v>
       </c>
       <c r="E8" t="n">
-        <v>46.2</v>
+        <v>60.1</v>
       </c>
       <c r="F8" t="n">
-        <v>68.8</v>
+        <v>56.4</v>
       </c>
       <c r="G8" t="n">
-        <v>57.5</v>
+        <v>58.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>29.3</v>
+        <v>18.01</v>
       </c>
       <c r="D9" t="n">
-        <v>2.46</v>
+        <v>1.74</v>
       </c>
       <c r="E9" t="n">
-        <v>57</v>
+        <v>45.7</v>
       </c>
       <c r="F9" t="n">
-        <v>55.4</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>56.2</v>
+        <v>57.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>22.59</v>
+        <v>14.11</v>
       </c>
       <c r="D10" t="n">
-        <v>1.85</v>
+        <v>1.33</v>
       </c>
       <c r="E10" t="n">
-        <v>47.3</v>
+        <v>52.1</v>
       </c>
       <c r="F10" t="n">
-        <v>44.6</v>
+        <v>55.9</v>
       </c>
       <c r="G10" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28.16</v>
+        <v>22.77</v>
       </c>
       <c r="D11" t="n">
-        <v>2.59</v>
+        <v>1.86</v>
       </c>
       <c r="E11" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="F11" t="n">
         <v>45.7</v>
       </c>
-      <c r="F11" t="n">
-        <v>45.2</v>
-      </c>
       <c r="G11" t="n">
-        <v>45.4</v>
+        <v>48.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15.51</v>
+        <v>24.43</v>
       </c>
       <c r="D12" t="n">
-        <v>2.29</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>45.2</v>
+        <v>48.9</v>
       </c>
       <c r="F12" t="n">
-        <v>39.8</v>
+        <v>47.3</v>
       </c>
       <c r="G12" t="n">
-        <v>42.5</v>
+        <v>48.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>16.86</v>
+        <v>69.27</v>
       </c>
       <c r="D13" t="n">
-        <v>0.93</v>
+        <v>7.82</v>
       </c>
       <c r="E13" t="n">
-        <v>40.9</v>
+        <v>35.1</v>
       </c>
       <c r="F13" t="n">
-        <v>38.7</v>
+        <v>60.6</v>
       </c>
       <c r="G13" t="n">
-        <v>39.8</v>
+        <v>47.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>19.61</v>
+        <v>15.55</v>
       </c>
       <c r="D14" t="n">
-        <v>1.76</v>
+        <v>2.3</v>
       </c>
       <c r="E14" t="n">
-        <v>41.9</v>
+        <v>50</v>
       </c>
       <c r="F14" t="n">
-        <v>33.3</v>
+        <v>43.1</v>
       </c>
       <c r="G14" t="n">
-        <v>37.6</v>
+        <v>46.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>67.17</v>
+        <v>19.64</v>
       </c>
       <c r="D15" t="n">
-        <v>7.58</v>
+        <v>1.76</v>
       </c>
       <c r="E15" t="n">
-        <v>20.4</v>
+        <v>50.5</v>
       </c>
       <c r="F15" t="n">
-        <v>54.8</v>
+        <v>33.5</v>
       </c>
       <c r="G15" t="n">
-        <v>37.6</v>
+        <v>42</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.45</v>
+        <v>16.8</v>
       </c>
       <c r="D16" t="n">
-        <v>0.97</v>
+        <v>0.93</v>
       </c>
       <c r="E16" t="n">
-        <v>26.3</v>
+        <v>40.4</v>
       </c>
       <c r="F16" t="n">
-        <v>41.4</v>
+        <v>38.8</v>
       </c>
       <c r="G16" t="n">
-        <v>33.9</v>
+        <v>39.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.42</v>
+        <v>10.34</v>
       </c>
       <c r="D17" t="n">
-        <v>1.92</v>
+        <v>0.97</v>
       </c>
       <c r="E17" t="n">
-        <v>25.3</v>
+        <v>21.8</v>
       </c>
       <c r="F17" t="n">
-        <v>26.9</v>
+        <v>41.5</v>
       </c>
       <c r="G17" t="n">
-        <v>26.4</v>
+        <v>31.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="18">
@@ -966,52 +966,52 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19.14</v>
+        <v>19.24</v>
       </c>
       <c r="D18" t="n">
-        <v>1.6</v>
+        <v>1.61</v>
       </c>
       <c r="E18" t="n">
-        <v>23.7</v>
+        <v>28.2</v>
       </c>
       <c r="F18" t="n">
-        <v>24.7</v>
+        <v>30.3</v>
       </c>
       <c r="G18" t="n">
-        <v>24.4</v>
+        <v>29.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>28.99</v>
+        <v>45.78</v>
       </c>
       <c r="D19" t="n">
-        <v>2.24</v>
+        <v>3.87</v>
       </c>
       <c r="E19" t="n">
-        <v>15.6</v>
+        <v>17</v>
       </c>
       <c r="F19" t="n">
-        <v>19.4</v>
+        <v>31.4</v>
       </c>
       <c r="G19" t="n">
-        <v>18.2</v>
+        <v>24.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="20">
@@ -1026,382 +1026,382 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>22.41</v>
+        <v>22.76</v>
       </c>
       <c r="D20" t="n">
-        <v>2.07</v>
+        <v>2.1</v>
       </c>
       <c r="E20" t="n">
-        <v>17.2</v>
+        <v>22.3</v>
       </c>
       <c r="F20" t="n">
-        <v>18.3</v>
+        <v>23.4</v>
       </c>
       <c r="G20" t="n">
-        <v>18</v>
+        <v>23.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>21.01</v>
+        <v>29.53</v>
       </c>
       <c r="D21" t="n">
-        <v>1.9</v>
+        <v>2.28</v>
       </c>
       <c r="E21" t="n">
-        <v>12.9</v>
+        <v>20.2</v>
       </c>
       <c r="F21" t="n">
-        <v>12.9</v>
+        <v>22.3</v>
       </c>
       <c r="G21" t="n">
-        <v>12.9</v>
+        <v>21.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>19.32</v>
+        <v>21.19</v>
       </c>
       <c r="D22" t="n">
-        <v>3.2</v>
+        <v>1.92</v>
       </c>
       <c r="E22" t="n">
-        <v>10.8</v>
+        <v>16.5</v>
       </c>
       <c r="F22" t="n">
-        <v>10.8</v>
+        <v>16.5</v>
       </c>
       <c r="G22" t="n">
-        <v>10.8</v>
+        <v>16.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24.21</v>
+        <v>19.7</v>
       </c>
       <c r="D23" t="n">
-        <v>2.26</v>
+        <v>3.26</v>
       </c>
       <c r="E23" t="n">
-        <v>9.699999999999999</v>
+        <v>14.9</v>
       </c>
       <c r="F23" t="n">
-        <v>10.2</v>
+        <v>16.5</v>
       </c>
       <c r="G23" t="n">
-        <v>10.1</v>
+        <v>16</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9.99</v>
+        <v>72.8</v>
       </c>
       <c r="D24" t="n">
-        <v>0.64</v>
+        <v>3.34</v>
       </c>
       <c r="E24" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="F24" t="n">
-        <v>7.5</v>
+        <v>14.9</v>
       </c>
       <c r="G24" t="n">
-        <v>7.5</v>
+        <v>13</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.2</v>
+        <v>24.29</v>
       </c>
       <c r="D25" t="n">
-        <v>3.08</v>
+        <v>2.27</v>
       </c>
       <c r="E25" t="n">
-        <v>5.4</v>
+        <v>10.6</v>
       </c>
       <c r="F25" t="n">
-        <v>5.9</v>
+        <v>12.2</v>
       </c>
       <c r="G25" t="n">
-        <v>5.8</v>
+        <v>11.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>32.26</v>
+        <v>53.32</v>
       </c>
       <c r="D26" t="n">
-        <v>1.79</v>
+        <v>3.44</v>
       </c>
       <c r="E26" t="n">
-        <v>6.5</v>
+        <v>10.6</v>
       </c>
       <c r="F26" t="n">
-        <v>5.4</v>
+        <v>11.2</v>
       </c>
       <c r="G26" t="n">
-        <v>5.7</v>
+        <v>11</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>52.4</v>
+        <v>10.09</v>
       </c>
       <c r="D27" t="n">
-        <v>3.38</v>
+        <v>0.64</v>
       </c>
       <c r="E27" t="n">
-        <v>5.4</v>
+        <v>13.8</v>
       </c>
       <c r="F27" t="n">
-        <v>5.4</v>
+        <v>8</v>
       </c>
       <c r="G27" t="n">
-        <v>5.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18.78</v>
+        <v>32.44</v>
       </c>
       <c r="D28" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E28" t="n">
-        <v>5.4</v>
+        <v>12.8</v>
       </c>
       <c r="F28" t="n">
-        <v>4.8</v>
+        <v>7.4</v>
       </c>
       <c r="G28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>43.42</v>
+        <v>28.4</v>
       </c>
       <c r="D29" t="n">
-        <v>3.67</v>
+        <v>3.1</v>
       </c>
       <c r="E29" t="n">
-        <v>1.1</v>
+        <v>7.4</v>
       </c>
       <c r="F29" t="n">
-        <v>5.9</v>
+        <v>9</v>
       </c>
       <c r="G29" t="n">
-        <v>4.5</v>
+        <v>8.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>68.78</v>
+        <v>19.06</v>
       </c>
       <c r="D30" t="n">
-        <v>3.16</v>
+        <v>1.42</v>
       </c>
       <c r="E30" t="n">
-        <v>2.2</v>
+        <v>8.5</v>
       </c>
       <c r="F30" t="n">
-        <v>2.2</v>
+        <v>8</v>
       </c>
       <c r="G30" t="n">
-        <v>2.2</v>
+        <v>8.1</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>26.99</v>
+        <v>33.94</v>
       </c>
       <c r="D31" t="n">
-        <v>2.55</v>
+        <v>2.95</v>
       </c>
       <c r="E31" t="n">
-        <v>2.2</v>
+        <v>3.2</v>
       </c>
       <c r="F31" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G31" t="n">
-        <v>2.2</v>
+        <v>3.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>32.86</v>
+        <v>27.74</v>
       </c>
       <c r="D32" t="n">
-        <v>2.85</v>
+        <v>2.62</v>
       </c>
       <c r="E32" t="n">
-        <v>1.1</v>
+        <v>3.2</v>
       </c>
       <c r="F32" t="n">
-        <v>1.1</v>
+        <v>3.2</v>
       </c>
       <c r="G32" t="n">
-        <v>1.1</v>
+        <v>3.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Aug  1 11:05:46 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.68</v>
       </c>
       <c r="E2" t="n">
-        <v>98.90000000000001</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>94.09999999999999</v>
+        <v>93.7</v>
       </c>
       <c r="G2" t="n">
-        <v>96.5</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.26</v>
       </c>
       <c r="E3" t="n">
-        <v>71.8</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>66.5</v>
+        <v>66.3</v>
       </c>
       <c r="G3" t="n">
-        <v>69.09999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.57</v>
       </c>
       <c r="E4" t="n">
-        <v>73.40000000000001</v>
+        <v>73.2</v>
       </c>
       <c r="F4" t="n">
-        <v>62.8</v>
+        <v>62.6</v>
       </c>
       <c r="G4" t="n">
-        <v>68.09999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.11</v>
       </c>
       <c r="E5" t="n">
-        <v>59.6</v>
+        <v>59.5</v>
       </c>
       <c r="F5" t="n">
-        <v>58</v>
+        <v>57.9</v>
       </c>
       <c r="G5" t="n">
-        <v>58.8</v>
+        <v>58.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.48</v>
       </c>
       <c r="E6" t="n">
-        <v>59.6</v>
+        <v>59.5</v>
       </c>
       <c r="F6" t="n">
-        <v>58</v>
+        <v>57.9</v>
       </c>
       <c r="G6" t="n">
-        <v>58.8</v>
+        <v>58.7</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.23</v>
       </c>
       <c r="E7" t="n">
-        <v>58.5</v>
+        <v>58.4</v>
       </c>
       <c r="F7" t="n">
-        <v>58</v>
+        <v>57.9</v>
       </c>
       <c r="G7" t="n">
         <v>58.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.61</v>
       </c>
       <c r="E8" t="n">
-        <v>60.1</v>
+        <v>60</v>
       </c>
       <c r="F8" t="n">
-        <v>56.4</v>
+        <v>56.3</v>
       </c>
       <c r="G8" t="n">
         <v>58.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.74</v>
       </c>
       <c r="E9" t="n">
-        <v>45.7</v>
+        <v>45.8</v>
       </c>
       <c r="F9" t="n">
-        <v>68.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>57.2</v>
+        <v>57.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="10">
@@ -735,13 +735,13 @@
         <v>52.1</v>
       </c>
       <c r="F10" t="n">
-        <v>55.9</v>
+        <v>55.8</v>
       </c>
       <c r="G10" t="n">
-        <v>54</v>
+        <v>53.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="11">
@@ -765,13 +765,13 @@
         <v>51.1</v>
       </c>
       <c r="F11" t="n">
-        <v>45.7</v>
+        <v>45.8</v>
       </c>
       <c r="G11" t="n">
         <v>48.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="12">
@@ -795,13 +795,13 @@
         <v>48.9</v>
       </c>
       <c r="F12" t="n">
-        <v>47.3</v>
+        <v>47.4</v>
       </c>
       <c r="G12" t="n">
-        <v>48.1</v>
+        <v>48.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>7.82</v>
       </c>
       <c r="E13" t="n">
-        <v>35.1</v>
+        <v>35.3</v>
       </c>
       <c r="F13" t="n">
-        <v>60.6</v>
+        <v>60.5</v>
       </c>
       <c r="G13" t="n">
         <v>47.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="14">
@@ -855,13 +855,13 @@
         <v>50</v>
       </c>
       <c r="F14" t="n">
-        <v>43.1</v>
+        <v>43.2</v>
       </c>
       <c r="G14" t="n">
-        <v>46.5</v>
+        <v>46.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="15">
@@ -885,13 +885,13 @@
         <v>50.5</v>
       </c>
       <c r="F15" t="n">
-        <v>33.5</v>
+        <v>33.7</v>
       </c>
       <c r="G15" t="n">
-        <v>42</v>
+        <v>42.1</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>0.93</v>
       </c>
       <c r="E16" t="n">
-        <v>40.4</v>
+        <v>40.5</v>
       </c>
       <c r="F16" t="n">
-        <v>38.8</v>
+        <v>38.9</v>
       </c>
       <c r="G16" t="n">
-        <v>39.6</v>
+        <v>39.7</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>0.97</v>
       </c>
       <c r="E17" t="n">
-        <v>21.8</v>
+        <v>22.1</v>
       </c>
       <c r="F17" t="n">
-        <v>41.5</v>
+        <v>41.6</v>
       </c>
       <c r="G17" t="n">
-        <v>31.6</v>
+        <v>31.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.61</v>
       </c>
       <c r="E18" t="n">
-        <v>28.2</v>
+        <v>28.4</v>
       </c>
       <c r="F18" t="n">
-        <v>30.3</v>
+        <v>30.5</v>
       </c>
       <c r="G18" t="n">
-        <v>29.3</v>
+        <v>29.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>3.87</v>
       </c>
       <c r="E19" t="n">
-        <v>17</v>
+        <v>17.4</v>
       </c>
       <c r="F19" t="n">
-        <v>31.4</v>
+        <v>31.6</v>
       </c>
       <c r="G19" t="n">
-        <v>24.2</v>
+        <v>24.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>2.1</v>
       </c>
       <c r="E20" t="n">
-        <v>22.3</v>
+        <v>22.6</v>
       </c>
       <c r="F20" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="G20" t="n">
         <v>23.4</v>
       </c>
-      <c r="G20" t="n">
-        <v>23.1</v>
-      </c>
       <c r="H20" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.28</v>
       </c>
       <c r="E21" t="n">
-        <v>20.2</v>
+        <v>20.5</v>
       </c>
       <c r="F21" t="n">
-        <v>22.3</v>
+        <v>22.6</v>
       </c>
       <c r="G21" t="n">
-        <v>21.7</v>
+        <v>22</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.92</v>
       </c>
       <c r="E22" t="n">
-        <v>16.5</v>
+        <v>16.8</v>
       </c>
       <c r="F22" t="n">
-        <v>16.5</v>
+        <v>16.8</v>
       </c>
       <c r="G22" t="n">
-        <v>16.5</v>
+        <v>16.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.26</v>
       </c>
       <c r="E23" t="n">
-        <v>14.9</v>
+        <v>15.3</v>
       </c>
       <c r="F23" t="n">
-        <v>16.5</v>
+        <v>16.8</v>
       </c>
       <c r="G23" t="n">
-        <v>16</v>
+        <v>16.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>3.34</v>
       </c>
       <c r="E24" t="n">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="F24" t="n">
-        <v>14.9</v>
+        <v>15.3</v>
       </c>
       <c r="G24" t="n">
-        <v>13</v>
+        <v>13.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.27</v>
       </c>
       <c r="E25" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="F25" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="G25" t="n">
         <v>12.2</v>
       </c>
-      <c r="G25" t="n">
-        <v>11.8</v>
-      </c>
       <c r="H25" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.44</v>
       </c>
       <c r="E26" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="F26" t="n">
-        <v>11.2</v>
+        <v>11.6</v>
       </c>
       <c r="G26" t="n">
-        <v>11</v>
+        <v>11.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>0.64</v>
       </c>
       <c r="E27" t="n">
-        <v>13.8</v>
+        <v>14.2</v>
       </c>
       <c r="F27" t="n">
-        <v>8</v>
+        <v>8.4</v>
       </c>
       <c r="G27" t="n">
-        <v>9.699999999999999</v>
+        <v>10.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.8</v>
       </c>
       <c r="E28" t="n">
-        <v>12.8</v>
+        <v>13.2</v>
       </c>
       <c r="F28" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="G28" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.1</v>
       </c>
       <c r="E29" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="F29" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G29" t="n">
         <v>9</v>
       </c>
-      <c r="G29" t="n">
-        <v>8.6</v>
-      </c>
       <c r="H29" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.42</v>
       </c>
       <c r="E30" t="n">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="F30" t="n">
-        <v>8</v>
+        <v>8.4</v>
       </c>
       <c r="G30" t="n">
-        <v>8.1</v>
+        <v>8.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>2.95</v>
       </c>
       <c r="E31" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="F31" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="G31" t="n">
-        <v>3.9</v>
+        <v>4.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.62</v>
       </c>
       <c r="E32" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="F32" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="G32" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Aug  2 11:07:38 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.68</v>
       </c>
       <c r="E2" t="n">
-        <v>98.40000000000001</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>93.7</v>
+        <v>93.2</v>
       </c>
       <c r="G2" t="n">
-        <v>96.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.26</v>
       </c>
       <c r="E3" t="n">
-        <v>71.59999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>66.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>68.90000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>3.57</v>
       </c>
       <c r="E4" t="n">
-        <v>73.2</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>62.6</v>
+        <v>62.5</v>
       </c>
       <c r="G4" t="n">
-        <v>67.90000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.11</v>
       </c>
       <c r="E5" t="n">
-        <v>59.5</v>
+        <v>59.4</v>
       </c>
       <c r="F5" t="n">
-        <v>57.9</v>
+        <v>57.8</v>
       </c>
       <c r="G5" t="n">
-        <v>58.7</v>
+        <v>58.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>2.48</v>
       </c>
       <c r="E6" t="n">
-        <v>59.5</v>
+        <v>59.4</v>
       </c>
       <c r="F6" t="n">
-        <v>57.9</v>
+        <v>57.8</v>
       </c>
       <c r="G6" t="n">
-        <v>58.7</v>
+        <v>58.6</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.23</v>
       </c>
       <c r="E7" t="n">
-        <v>58.4</v>
+        <v>58.3</v>
       </c>
       <c r="F7" t="n">
-        <v>57.9</v>
+        <v>57.8</v>
       </c>
       <c r="G7" t="n">
-        <v>58.2</v>
+        <v>58.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.61</v>
       </c>
       <c r="E8" t="n">
-        <v>60</v>
+        <v>59.9</v>
       </c>
       <c r="F8" t="n">
-        <v>56.3</v>
+        <v>56.2</v>
       </c>
       <c r="G8" t="n">
-        <v>58.2</v>
+        <v>58.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="9">
@@ -705,13 +705,13 @@
         <v>45.8</v>
       </c>
       <c r="F9" t="n">
-        <v>68.40000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="G9" t="n">
-        <v>57.1</v>
+        <v>57</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="10">
@@ -735,13 +735,13 @@
         <v>52.1</v>
       </c>
       <c r="F10" t="n">
-        <v>55.8</v>
+        <v>55.7</v>
       </c>
       <c r="G10" t="n">
         <v>53.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="11">
@@ -762,7 +762,7 @@
         <v>1.86</v>
       </c>
       <c r="E11" t="n">
-        <v>51.1</v>
+        <v>51</v>
       </c>
       <c r="F11" t="n">
         <v>45.8</v>
@@ -771,7 +771,7 @@
         <v>48.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="12">
@@ -792,7 +792,7 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>48.9</v>
+        <v>49</v>
       </c>
       <c r="F12" t="n">
         <v>47.4</v>
@@ -801,7 +801,7 @@
         <v>48.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>7.82</v>
       </c>
       <c r="E13" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="F13" t="n">
-        <v>60.5</v>
+        <v>60.4</v>
       </c>
       <c r="G13" t="n">
         <v>47.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="14">
@@ -861,7 +861,7 @@
         <v>46.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="15">
@@ -885,13 +885,13 @@
         <v>50.5</v>
       </c>
       <c r="F15" t="n">
-        <v>33.7</v>
+        <v>33.9</v>
       </c>
       <c r="G15" t="n">
-        <v>42.1</v>
+        <v>42.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>0.93</v>
       </c>
       <c r="E16" t="n">
-        <v>40.5</v>
+        <v>40.6</v>
       </c>
       <c r="F16" t="n">
-        <v>38.9</v>
+        <v>39.1</v>
       </c>
       <c r="G16" t="n">
-        <v>39.7</v>
+        <v>39.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>0.97</v>
       </c>
       <c r="E17" t="n">
-        <v>22.1</v>
+        <v>22.4</v>
       </c>
       <c r="F17" t="n">
-        <v>41.6</v>
+        <v>41.7</v>
       </c>
       <c r="G17" t="n">
-        <v>31.8</v>
+        <v>32</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.61</v>
       </c>
       <c r="E18" t="n">
-        <v>28.4</v>
+        <v>28.6</v>
       </c>
       <c r="F18" t="n">
-        <v>30.5</v>
+        <v>30.7</v>
       </c>
       <c r="G18" t="n">
-        <v>29.5</v>
+        <v>29.7</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>3.87</v>
       </c>
       <c r="E19" t="n">
-        <v>17.4</v>
+        <v>17.7</v>
       </c>
       <c r="F19" t="n">
-        <v>31.6</v>
+        <v>31.8</v>
       </c>
       <c r="G19" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>2.1</v>
       </c>
       <c r="E20" t="n">
-        <v>22.6</v>
+        <v>22.9</v>
       </c>
       <c r="F20" t="n">
-        <v>23.7</v>
+        <v>24</v>
       </c>
       <c r="G20" t="n">
-        <v>23.4</v>
+        <v>23.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.28</v>
       </c>
       <c r="E21" t="n">
-        <v>20.5</v>
+        <v>20.8</v>
       </c>
       <c r="F21" t="n">
-        <v>22.6</v>
+        <v>22.9</v>
       </c>
       <c r="G21" t="n">
-        <v>22</v>
+        <v>22.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.92</v>
       </c>
       <c r="E22" t="n">
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="F22" t="n">
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="G22" t="n">
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.26</v>
       </c>
       <c r="E23" t="n">
-        <v>15.3</v>
+        <v>15.6</v>
       </c>
       <c r="F23" t="n">
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="G23" t="n">
-        <v>16.4</v>
+        <v>16.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>3.34</v>
       </c>
       <c r="E24" t="n">
-        <v>8.9</v>
+        <v>9.4</v>
       </c>
       <c r="F24" t="n">
-        <v>15.3</v>
+        <v>15.6</v>
       </c>
       <c r="G24" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.27</v>
       </c>
       <c r="E25" t="n">
-        <v>11.1</v>
+        <v>11.5</v>
       </c>
       <c r="F25" t="n">
+        <v>13</v>
+      </c>
+      <c r="G25" t="n">
         <v>12.6</v>
       </c>
-      <c r="G25" t="n">
-        <v>12.2</v>
-      </c>
       <c r="H25" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.44</v>
       </c>
       <c r="E26" t="n">
-        <v>11.1</v>
+        <v>11.5</v>
       </c>
       <c r="F26" t="n">
-        <v>11.6</v>
+        <v>12</v>
       </c>
       <c r="G26" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>0.64</v>
       </c>
       <c r="E27" t="n">
-        <v>14.2</v>
+        <v>14.6</v>
       </c>
       <c r="F27" t="n">
-        <v>8.4</v>
+        <v>8.9</v>
       </c>
       <c r="G27" t="n">
-        <v>10.2</v>
+        <v>10.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.8</v>
       </c>
       <c r="E28" t="n">
-        <v>13.2</v>
+        <v>13.5</v>
       </c>
       <c r="F28" t="n">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>9.5</v>
+        <v>9.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.1</v>
       </c>
       <c r="E29" t="n">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F29" t="n">
-        <v>9.5</v>
+        <v>9.9</v>
       </c>
       <c r="G29" t="n">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.42</v>
       </c>
       <c r="E30" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F30" t="n">
         <v>8.9</v>
       </c>
-      <c r="F30" t="n">
-        <v>8.4</v>
-      </c>
       <c r="G30" t="n">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>2.95</v>
       </c>
       <c r="E31" t="n">
-        <v>3.7</v>
+        <v>4.2</v>
       </c>
       <c r="F31" t="n">
-        <v>4.7</v>
+        <v>5.2</v>
       </c>
       <c r="G31" t="n">
-        <v>4.4</v>
+        <v>4.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.62</v>
       </c>
       <c r="E32" t="n">
-        <v>3.7</v>
+        <v>4.2</v>
       </c>
       <c r="F32" t="n">
-        <v>3.7</v>
+        <v>4.2</v>
       </c>
       <c r="G32" t="n">
-        <v>3.7</v>
+        <v>4.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Aug  3 12:45:22 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,502 +486,502 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.2</v>
+        <v>7.16</v>
       </c>
       <c r="D2" t="n">
         <v>0.68</v>
       </c>
       <c r="E2" t="n">
-        <v>97.90000000000001</v>
+        <v>92.3</v>
       </c>
       <c r="F2" t="n">
-        <v>93.2</v>
+        <v>92.8</v>
       </c>
       <c r="G2" t="n">
-        <v>95.59999999999999</v>
+        <v>92.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.36</v>
+        <v>20.51</v>
       </c>
       <c r="D3" t="n">
-        <v>1.26</v>
+        <v>3.57</v>
       </c>
       <c r="E3" t="n">
-        <v>71.40000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="F3" t="n">
-        <v>66.09999999999999</v>
+        <v>62.4</v>
       </c>
       <c r="G3" t="n">
-        <v>68.8</v>
+        <v>68.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20.5</v>
+        <v>10.33</v>
       </c>
       <c r="D4" t="n">
-        <v>3.57</v>
+        <v>1.26</v>
       </c>
       <c r="E4" t="n">
-        <v>72.90000000000001</v>
+        <v>66.5</v>
       </c>
       <c r="F4" t="n">
-        <v>62.5</v>
+        <v>66</v>
       </c>
       <c r="G4" t="n">
-        <v>67.7</v>
+        <v>66.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28.31</v>
+        <v>15.23</v>
       </c>
       <c r="D5" t="n">
-        <v>2.11</v>
+        <v>1.24</v>
       </c>
       <c r="E5" t="n">
-        <v>59.4</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>57.8</v>
+        <v>62.4</v>
       </c>
       <c r="G5" t="n">
-        <v>58.6</v>
+        <v>63.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>29.57</v>
+        <v>28.24</v>
       </c>
       <c r="D6" t="n">
-        <v>2.48</v>
+        <v>2.1</v>
       </c>
       <c r="E6" t="n">
-        <v>59.4</v>
+        <v>57.7</v>
       </c>
       <c r="F6" t="n">
-        <v>57.8</v>
+        <v>54.6</v>
       </c>
       <c r="G6" t="n">
-        <v>58.6</v>
+        <v>56.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>15.1</v>
+        <v>29.38</v>
       </c>
       <c r="D7" t="n">
-        <v>1.23</v>
+        <v>2.46</v>
       </c>
       <c r="E7" t="n">
-        <v>58.3</v>
+        <v>57.7</v>
       </c>
       <c r="F7" t="n">
-        <v>57.8</v>
+        <v>53.6</v>
       </c>
       <c r="G7" t="n">
-        <v>58.1</v>
+        <v>55.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28.41</v>
+        <v>24.66</v>
       </c>
       <c r="D8" t="n">
-        <v>2.61</v>
+        <v>2.02</v>
       </c>
       <c r="E8" t="n">
-        <v>59.9</v>
+        <v>51.5</v>
       </c>
       <c r="F8" t="n">
-        <v>56.2</v>
+        <v>51</v>
       </c>
       <c r="G8" t="n">
-        <v>58.1</v>
+        <v>51.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>18.01</v>
+        <v>14.06</v>
       </c>
       <c r="D9" t="n">
-        <v>1.74</v>
+        <v>1.32</v>
       </c>
       <c r="E9" t="n">
-        <v>45.8</v>
+        <v>49.5</v>
       </c>
       <c r="F9" t="n">
-        <v>68.2</v>
+        <v>49.5</v>
       </c>
       <c r="G9" t="n">
-        <v>57</v>
+        <v>49.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>14.11</v>
+        <v>22.74</v>
       </c>
       <c r="D10" t="n">
-        <v>1.33</v>
+        <v>1.86</v>
       </c>
       <c r="E10" t="n">
-        <v>52.1</v>
+        <v>49.5</v>
       </c>
       <c r="F10" t="n">
-        <v>55.7</v>
+        <v>45.9</v>
       </c>
       <c r="G10" t="n">
-        <v>53.9</v>
+        <v>47.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>22.77</v>
+        <v>28.24</v>
       </c>
       <c r="D11" t="n">
-        <v>1.86</v>
+        <v>2.59</v>
       </c>
       <c r="E11" t="n">
-        <v>51</v>
+        <v>50.5</v>
       </c>
       <c r="F11" t="n">
-        <v>45.8</v>
+        <v>43.8</v>
       </c>
       <c r="G11" t="n">
-        <v>48.4</v>
+        <v>47.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>24.43</v>
+        <v>19.85</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>1.78</v>
       </c>
       <c r="E12" t="n">
-        <v>49</v>
+        <v>55.7</v>
       </c>
       <c r="F12" t="n">
-        <v>47.4</v>
+        <v>38.1</v>
       </c>
       <c r="G12" t="n">
-        <v>48.2</v>
+        <v>46.9</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>69.27</v>
+        <v>10.49</v>
       </c>
       <c r="D13" t="n">
-        <v>7.82</v>
+        <v>0.98</v>
       </c>
       <c r="E13" t="n">
-        <v>35.4</v>
+        <v>37.1</v>
       </c>
       <c r="F13" t="n">
-        <v>60.4</v>
+        <v>46.9</v>
       </c>
       <c r="G13" t="n">
-        <v>47.9</v>
+        <v>42</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.55</v>
+        <v>16.88</v>
       </c>
       <c r="D14" t="n">
-        <v>2.3</v>
+        <v>0.93</v>
       </c>
       <c r="E14" t="n">
-        <v>50</v>
+        <v>43.3</v>
       </c>
       <c r="F14" t="n">
-        <v>43.2</v>
+        <v>39.2</v>
       </c>
       <c r="G14" t="n">
-        <v>46.6</v>
+        <v>41.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>19.64</v>
+        <v>19.36</v>
       </c>
       <c r="D15" t="n">
-        <v>1.76</v>
+        <v>1.62</v>
       </c>
       <c r="E15" t="n">
-        <v>50.5</v>
+        <v>40.2</v>
       </c>
       <c r="F15" t="n">
-        <v>33.9</v>
+        <v>37.6</v>
       </c>
       <c r="G15" t="n">
-        <v>42.2</v>
+        <v>38.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>16.8</v>
+        <v>15.42</v>
       </c>
       <c r="D16" t="n">
-        <v>0.93</v>
+        <v>2.28</v>
       </c>
       <c r="E16" t="n">
-        <v>40.6</v>
+        <v>41.2</v>
       </c>
       <c r="F16" t="n">
-        <v>39.1</v>
+        <v>35.6</v>
       </c>
       <c r="G16" t="n">
-        <v>39.8</v>
+        <v>38.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.34</v>
+        <v>17.38</v>
       </c>
       <c r="D17" t="n">
-        <v>0.97</v>
+        <v>1.68</v>
       </c>
       <c r="E17" t="n">
-        <v>22.4</v>
+        <v>29.4</v>
       </c>
       <c r="F17" t="n">
-        <v>41.7</v>
+        <v>43.8</v>
       </c>
       <c r="G17" t="n">
-        <v>32</v>
+        <v>36.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19.24</v>
+        <v>67.02</v>
       </c>
       <c r="D18" t="n">
-        <v>1.61</v>
+        <v>7.57</v>
       </c>
       <c r="E18" t="n">
-        <v>28.6</v>
+        <v>19.6</v>
       </c>
       <c r="F18" t="n">
-        <v>30.7</v>
+        <v>50.5</v>
       </c>
       <c r="G18" t="n">
-        <v>29.7</v>
+        <v>35.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="19">
@@ -996,82 +996,82 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>45.78</v>
+        <v>45.9</v>
       </c>
       <c r="D19" t="n">
-        <v>3.87</v>
+        <v>3.88</v>
       </c>
       <c r="E19" t="n">
-        <v>17.7</v>
+        <v>20.1</v>
       </c>
       <c r="F19" t="n">
-        <v>31.8</v>
+        <v>35.6</v>
       </c>
       <c r="G19" t="n">
-        <v>24.7</v>
+        <v>27.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>22.76</v>
+        <v>29.7</v>
       </c>
       <c r="D20" t="n">
-        <v>2.1</v>
+        <v>2.29</v>
       </c>
       <c r="E20" t="n">
-        <v>22.9</v>
+        <v>23.7</v>
       </c>
       <c r="F20" t="n">
-        <v>24</v>
+        <v>25.3</v>
       </c>
       <c r="G20" t="n">
-        <v>23.6</v>
+        <v>24.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>29.53</v>
+        <v>22.79</v>
       </c>
       <c r="D21" t="n">
-        <v>2.28</v>
+        <v>2.1</v>
       </c>
       <c r="E21" t="n">
-        <v>20.8</v>
+        <v>25.8</v>
       </c>
       <c r="F21" t="n">
-        <v>22.9</v>
+        <v>24.2</v>
       </c>
       <c r="G21" t="n">
-        <v>22.3</v>
+        <v>24.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="22">
@@ -1086,52 +1086,52 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21.19</v>
+        <v>21.38</v>
       </c>
       <c r="D22" t="n">
-        <v>1.92</v>
+        <v>1.94</v>
       </c>
       <c r="E22" t="n">
-        <v>17.2</v>
+        <v>20.6</v>
       </c>
       <c r="F22" t="n">
-        <v>17.2</v>
+        <v>23.7</v>
       </c>
       <c r="G22" t="n">
-        <v>17.2</v>
+        <v>22.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>19.7</v>
+        <v>10.15</v>
       </c>
       <c r="D23" t="n">
-        <v>3.26</v>
+        <v>0.65</v>
       </c>
       <c r="E23" t="n">
-        <v>15.6</v>
+        <v>16.5</v>
       </c>
       <c r="F23" t="n">
-        <v>17.2</v>
+        <v>16</v>
       </c>
       <c r="G23" t="n">
-        <v>16.7</v>
+        <v>16.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="24">
@@ -1146,202 +1146,202 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.8</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D24" t="n">
-        <v>3.34</v>
+        <v>3.43</v>
       </c>
       <c r="E24" t="n">
-        <v>9.4</v>
+        <v>11.3</v>
       </c>
       <c r="F24" t="n">
-        <v>15.6</v>
+        <v>17.5</v>
       </c>
       <c r="G24" t="n">
-        <v>13.8</v>
+        <v>15.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>24.29</v>
+        <v>53.83</v>
       </c>
       <c r="D25" t="n">
-        <v>2.27</v>
+        <v>3.47</v>
       </c>
       <c r="E25" t="n">
-        <v>11.5</v>
+        <v>14.4</v>
       </c>
       <c r="F25" t="n">
-        <v>13</v>
+        <v>14.9</v>
       </c>
       <c r="G25" t="n">
-        <v>12.6</v>
+        <v>14.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>53.32</v>
+        <v>19.49</v>
       </c>
       <c r="D26" t="n">
-        <v>3.44</v>
+        <v>1.45</v>
       </c>
       <c r="E26" t="n">
-        <v>11.5</v>
+        <v>12.4</v>
       </c>
       <c r="F26" t="n">
-        <v>12</v>
+        <v>15.5</v>
       </c>
       <c r="G26" t="n">
-        <v>11.8</v>
+        <v>14.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>10.09</v>
+        <v>28.64</v>
       </c>
       <c r="D27" t="n">
-        <v>0.64</v>
+        <v>3.12</v>
       </c>
       <c r="E27" t="n">
-        <v>14.6</v>
+        <v>11.3</v>
       </c>
       <c r="F27" t="n">
-        <v>8.9</v>
+        <v>13.9</v>
       </c>
       <c r="G27" t="n">
-        <v>10.6</v>
+        <v>13.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>32.44</v>
+        <v>19.5</v>
       </c>
       <c r="D28" t="n">
-        <v>1.8</v>
+        <v>3.23</v>
       </c>
       <c r="E28" t="n">
-        <v>13.5</v>
+        <v>12.4</v>
       </c>
       <c r="F28" t="n">
-        <v>8.300000000000001</v>
+        <v>12.9</v>
       </c>
       <c r="G28" t="n">
-        <v>9.9</v>
+        <v>12.7</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>28.4</v>
+        <v>24.21</v>
       </c>
       <c r="D29" t="n">
-        <v>3.1</v>
+        <v>2.27</v>
       </c>
       <c r="E29" t="n">
-        <v>8.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F29" t="n">
-        <v>9.9</v>
+        <v>13.4</v>
       </c>
       <c r="G29" t="n">
-        <v>9.4</v>
+        <v>12.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.06</v>
+        <v>27.93</v>
       </c>
       <c r="D30" t="n">
-        <v>1.42</v>
+        <v>2.65</v>
       </c>
       <c r="E30" t="n">
-        <v>9.4</v>
+        <v>7.2</v>
       </c>
       <c r="F30" t="n">
-        <v>8.9</v>
+        <v>7.7</v>
       </c>
       <c r="G30" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="31">
@@ -1356,52 +1356,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>33.94</v>
+        <v>33.84</v>
       </c>
       <c r="D31" t="n">
-        <v>2.95</v>
+        <v>2.94</v>
       </c>
       <c r="E31" t="n">
-        <v>4.2</v>
+        <v>3.1</v>
       </c>
       <c r="F31" t="n">
-        <v>5.2</v>
+        <v>4.1</v>
       </c>
       <c r="G31" t="n">
-        <v>4.9</v>
+        <v>3.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>27.74</v>
+        <v>30.79</v>
       </c>
       <c r="D32" t="n">
-        <v>2.62</v>
+        <v>1.71</v>
       </c>
       <c r="E32" t="n">
-        <v>4.2</v>
+        <v>2.1</v>
       </c>
       <c r="F32" t="n">
-        <v>4.2</v>
+        <v>2.1</v>
       </c>
       <c r="G32" t="n">
-        <v>4.2</v>
+        <v>2.1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Aug  4 11:49:25 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,292 +486,292 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.16</v>
+        <v>6.93</v>
       </c>
       <c r="D2" t="n">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="E2" t="n">
-        <v>92.3</v>
+        <v>67.3</v>
       </c>
       <c r="F2" t="n">
-        <v>92.8</v>
+        <v>73</v>
       </c>
       <c r="G2" t="n">
-        <v>92.5</v>
+        <v>70.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.51</v>
+        <v>28.63</v>
       </c>
       <c r="D3" t="n">
-        <v>3.57</v>
+        <v>2.65</v>
       </c>
       <c r="E3" t="n">
-        <v>74.2</v>
+        <v>66.3</v>
       </c>
       <c r="F3" t="n">
-        <v>62.4</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>68.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.33</v>
+        <v>25.22</v>
       </c>
       <c r="D4" t="n">
-        <v>1.26</v>
+        <v>2.06</v>
       </c>
       <c r="E4" t="n">
-        <v>66.5</v>
+        <v>55.1</v>
       </c>
       <c r="F4" t="n">
-        <v>66</v>
+        <v>54.1</v>
       </c>
       <c r="G4" t="n">
-        <v>66.2</v>
+        <v>54.6</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15.23</v>
+        <v>20.14</v>
       </c>
       <c r="D5" t="n">
-        <v>1.24</v>
+        <v>3.51</v>
       </c>
       <c r="E5" t="n">
-        <v>64.40000000000001</v>
+        <v>55.6</v>
       </c>
       <c r="F5" t="n">
-        <v>62.4</v>
+        <v>51</v>
       </c>
       <c r="G5" t="n">
-        <v>63.4</v>
+        <v>53.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28.24</v>
+        <v>70.25</v>
       </c>
       <c r="D6" t="n">
-        <v>2.1</v>
+        <v>7.95</v>
       </c>
       <c r="E6" t="n">
-        <v>57.7</v>
+        <v>40.8</v>
       </c>
       <c r="F6" t="n">
-        <v>54.6</v>
+        <v>65.8</v>
       </c>
       <c r="G6" t="n">
-        <v>56.2</v>
+        <v>53.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>29.38</v>
+        <v>14.97</v>
       </c>
       <c r="D7" t="n">
-        <v>2.46</v>
+        <v>1.22</v>
       </c>
       <c r="E7" t="n">
-        <v>57.7</v>
+        <v>54.1</v>
       </c>
       <c r="F7" t="n">
-        <v>53.6</v>
+        <v>51.5</v>
       </c>
       <c r="G7" t="n">
-        <v>55.7</v>
+        <v>52.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24.66</v>
+        <v>29.11</v>
       </c>
       <c r="D8" t="n">
-        <v>2.02</v>
+        <v>2.44</v>
       </c>
       <c r="E8" t="n">
-        <v>51.5</v>
+        <v>54.1</v>
       </c>
       <c r="F8" t="n">
-        <v>51</v>
+        <v>48.5</v>
       </c>
       <c r="G8" t="n">
         <v>51.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.06</v>
+        <v>27.83</v>
       </c>
       <c r="D9" t="n">
-        <v>1.32</v>
+        <v>2.07</v>
       </c>
       <c r="E9" t="n">
-        <v>49.5</v>
+        <v>52</v>
       </c>
       <c r="F9" t="n">
-        <v>49.5</v>
+        <v>48.5</v>
       </c>
       <c r="G9" t="n">
-        <v>49.5</v>
+        <v>50.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>22.74</v>
+        <v>10.21</v>
       </c>
       <c r="D10" t="n">
-        <v>1.86</v>
+        <v>1.24</v>
       </c>
       <c r="E10" t="n">
-        <v>49.5</v>
+        <v>50.5</v>
       </c>
       <c r="F10" t="n">
-        <v>45.9</v>
+        <v>47.4</v>
       </c>
       <c r="G10" t="n">
-        <v>47.7</v>
+        <v>49</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28.24</v>
+        <v>22.67</v>
       </c>
       <c r="D11" t="n">
-        <v>2.59</v>
+        <v>1.86</v>
       </c>
       <c r="E11" t="n">
-        <v>50.5</v>
+        <v>49</v>
       </c>
       <c r="F11" t="n">
-        <v>43.8</v>
+        <v>45.9</v>
       </c>
       <c r="G11" t="n">
-        <v>47.2</v>
+        <v>47.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="12">
@@ -786,112 +786,112 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>19.85</v>
+        <v>19.71</v>
       </c>
       <c r="D12" t="n">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
       <c r="E12" t="n">
-        <v>55.7</v>
+        <v>54.1</v>
       </c>
       <c r="F12" t="n">
-        <v>38.1</v>
+        <v>37.2</v>
       </c>
       <c r="G12" t="n">
-        <v>46.9</v>
+        <v>45.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.49</v>
+        <v>47.02</v>
       </c>
       <c r="D13" t="n">
-        <v>0.98</v>
+        <v>3.98</v>
       </c>
       <c r="E13" t="n">
-        <v>37.1</v>
+        <v>35.7</v>
       </c>
       <c r="F13" t="n">
-        <v>46.9</v>
+        <v>52.6</v>
       </c>
       <c r="G13" t="n">
-        <v>42</v>
+        <v>44.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>16.88</v>
+        <v>13.84</v>
       </c>
       <c r="D14" t="n">
-        <v>0.93</v>
+        <v>1.3</v>
       </c>
       <c r="E14" t="n">
-        <v>43.3</v>
+        <v>41.8</v>
       </c>
       <c r="F14" t="n">
-        <v>39.2</v>
+        <v>40.8</v>
       </c>
       <c r="G14" t="n">
-        <v>41.2</v>
+        <v>41.3</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>19.36</v>
+        <v>10.47</v>
       </c>
       <c r="D15" t="n">
-        <v>1.62</v>
+        <v>0.97</v>
       </c>
       <c r="E15" t="n">
-        <v>40.2</v>
+        <v>35.2</v>
       </c>
       <c r="F15" t="n">
-        <v>37.6</v>
+        <v>41.3</v>
       </c>
       <c r="G15" t="n">
-        <v>38.9</v>
+        <v>38.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="16">
@@ -906,112 +906,112 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15.42</v>
+        <v>15.38</v>
       </c>
       <c r="D16" t="n">
-        <v>2.28</v>
+        <v>2.27</v>
       </c>
       <c r="E16" t="n">
-        <v>41.2</v>
+        <v>40.3</v>
       </c>
       <c r="F16" t="n">
-        <v>35.6</v>
+        <v>31.6</v>
       </c>
       <c r="G16" t="n">
-        <v>38.4</v>
+        <v>36</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>17.38</v>
+        <v>16.62</v>
       </c>
       <c r="D17" t="n">
-        <v>1.68</v>
+        <v>0.92</v>
       </c>
       <c r="E17" t="n">
-        <v>29.4</v>
+        <v>32.7</v>
       </c>
       <c r="F17" t="n">
-        <v>43.8</v>
+        <v>33.7</v>
       </c>
       <c r="G17" t="n">
-        <v>36.6</v>
+        <v>33.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>67.02</v>
+        <v>17.24</v>
       </c>
       <c r="D18" t="n">
-        <v>7.57</v>
+        <v>1.66</v>
       </c>
       <c r="E18" t="n">
-        <v>19.6</v>
+        <v>25.5</v>
       </c>
       <c r="F18" t="n">
-        <v>50.5</v>
+        <v>40.3</v>
       </c>
       <c r="G18" t="n">
-        <v>35.1</v>
+        <v>32.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>45.9</v>
+        <v>19.26</v>
       </c>
       <c r="D19" t="n">
-        <v>3.88</v>
+        <v>1.61</v>
       </c>
       <c r="E19" t="n">
-        <v>20.1</v>
+        <v>31.1</v>
       </c>
       <c r="F19" t="n">
-        <v>35.6</v>
+        <v>30.6</v>
       </c>
       <c r="G19" t="n">
-        <v>27.8</v>
+        <v>30.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="20">
@@ -1026,52 +1026,52 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29.7</v>
+        <v>29.84</v>
       </c>
       <c r="D20" t="n">
-        <v>2.29</v>
+        <v>2.3</v>
       </c>
       <c r="E20" t="n">
-        <v>23.7</v>
+        <v>25.5</v>
       </c>
       <c r="F20" t="n">
-        <v>25.3</v>
+        <v>28.6</v>
       </c>
       <c r="G20" t="n">
-        <v>24.8</v>
+        <v>27.7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>22.79</v>
+        <v>29.22</v>
       </c>
       <c r="D21" t="n">
-        <v>2.1</v>
+        <v>2.77</v>
       </c>
       <c r="E21" t="n">
-        <v>25.8</v>
+        <v>24.5</v>
       </c>
       <c r="F21" t="n">
-        <v>24.2</v>
+        <v>27</v>
       </c>
       <c r="G21" t="n">
-        <v>24.7</v>
+        <v>26.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="22">
@@ -1086,262 +1086,262 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21.38</v>
+        <v>21.49</v>
       </c>
       <c r="D22" t="n">
-        <v>1.94</v>
+        <v>1.95</v>
       </c>
       <c r="E22" t="n">
-        <v>20.6</v>
+        <v>24.5</v>
       </c>
       <c r="F22" t="n">
-        <v>23.7</v>
+        <v>24.5</v>
       </c>
       <c r="G22" t="n">
-        <v>22.8</v>
+        <v>24.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10.15</v>
+        <v>19.81</v>
       </c>
       <c r="D23" t="n">
-        <v>0.65</v>
+        <v>3.28</v>
       </c>
       <c r="E23" t="n">
-        <v>16.5</v>
+        <v>23.5</v>
       </c>
       <c r="F23" t="n">
-        <v>16</v>
+        <v>23.5</v>
       </c>
       <c r="G23" t="n">
-        <v>16.1</v>
+        <v>23.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>74.90000000000001</v>
+        <v>22.62</v>
       </c>
       <c r="D24" t="n">
-        <v>3.43</v>
+        <v>2.09</v>
       </c>
       <c r="E24" t="n">
-        <v>11.3</v>
+        <v>19.4</v>
       </c>
       <c r="F24" t="n">
-        <v>17.5</v>
+        <v>19.9</v>
       </c>
       <c r="G24" t="n">
-        <v>15.7</v>
+        <v>19.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>53.83</v>
+        <v>79.27</v>
       </c>
       <c r="D25" t="n">
-        <v>3.47</v>
+        <v>3.63</v>
       </c>
       <c r="E25" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="F25" t="n">
-        <v>14.9</v>
+        <v>19.4</v>
       </c>
       <c r="G25" t="n">
-        <v>14.8</v>
+        <v>17.6</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>19.49</v>
+        <v>24.53</v>
       </c>
       <c r="D26" t="n">
-        <v>1.45</v>
+        <v>2.3</v>
       </c>
       <c r="E26" t="n">
-        <v>12.4</v>
+        <v>15.3</v>
       </c>
       <c r="F26" t="n">
-        <v>15.5</v>
+        <v>18.4</v>
       </c>
       <c r="G26" t="n">
-        <v>14.5</v>
+        <v>17.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>28.64</v>
+        <v>54.58</v>
       </c>
       <c r="D27" t="n">
-        <v>3.12</v>
+        <v>3.52</v>
       </c>
       <c r="E27" t="n">
-        <v>11.3</v>
+        <v>17.3</v>
       </c>
       <c r="F27" t="n">
-        <v>13.9</v>
+        <v>17.3</v>
       </c>
       <c r="G27" t="n">
-        <v>13.1</v>
+        <v>17.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>19.5</v>
+        <v>29.08</v>
       </c>
       <c r="D28" t="n">
-        <v>3.23</v>
+        <v>3.17</v>
       </c>
       <c r="E28" t="n">
-        <v>12.4</v>
+        <v>15.3</v>
       </c>
       <c r="F28" t="n">
-        <v>12.9</v>
+        <v>16.8</v>
       </c>
       <c r="G28" t="n">
-        <v>12.7</v>
+        <v>16.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>24.21</v>
+        <v>10.1</v>
       </c>
       <c r="D29" t="n">
-        <v>2.27</v>
+        <v>0.65</v>
       </c>
       <c r="E29" t="n">
-        <v>9.800000000000001</v>
+        <v>16.3</v>
       </c>
       <c r="F29" t="n">
-        <v>13.4</v>
+        <v>16.3</v>
       </c>
       <c r="G29" t="n">
-        <v>12.3</v>
+        <v>16.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>27.93</v>
+        <v>19.57</v>
       </c>
       <c r="D30" t="n">
-        <v>2.65</v>
+        <v>1.46</v>
       </c>
       <c r="E30" t="n">
-        <v>7.2</v>
+        <v>16.3</v>
       </c>
       <c r="F30" t="n">
-        <v>7.7</v>
+        <v>16.3</v>
       </c>
       <c r="G30" t="n">
-        <v>7.6</v>
+        <v>16.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>33.84</v>
+        <v>35.06</v>
       </c>
       <c r="D31" t="n">
-        <v>2.94</v>
+        <v>3.04</v>
       </c>
       <c r="E31" t="n">
-        <v>3.1</v>
+        <v>10.2</v>
       </c>
       <c r="F31" t="n">
-        <v>4.1</v>
+        <v>14.8</v>
       </c>
       <c r="G31" t="n">
-        <v>3.8</v>
+        <v>13.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>30.79</v>
+        <v>31.87</v>
       </c>
       <c r="D32" t="n">
-        <v>1.71</v>
+        <v>1.76</v>
       </c>
       <c r="E32" t="n">
-        <v>2.1</v>
+        <v>7.1</v>
       </c>
       <c r="F32" t="n">
-        <v>2.1</v>
+        <v>4.6</v>
       </c>
       <c r="G32" t="n">
-        <v>2.1</v>
+        <v>5.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Aug  5 11:45:38 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,151 +477,151 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6.93</v>
+        <v>28.92</v>
       </c>
       <c r="D2" t="n">
-        <v>0.66</v>
+        <v>2.68</v>
       </c>
       <c r="E2" t="n">
-        <v>67.3</v>
+        <v>72.7</v>
       </c>
       <c r="F2" t="n">
-        <v>73</v>
+        <v>75.3</v>
       </c>
       <c r="G2" t="n">
-        <v>70.2</v>
+        <v>74</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.63</v>
+        <v>73.48</v>
       </c>
       <c r="D3" t="n">
-        <v>2.65</v>
+        <v>8.32</v>
       </c>
       <c r="E3" t="n">
-        <v>66.3</v>
+        <v>60.6</v>
       </c>
       <c r="F3" t="n">
-        <v>71.40000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="G3" t="n">
-        <v>68.90000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>25.22</v>
+        <v>10.28</v>
       </c>
       <c r="D4" t="n">
-        <v>2.06</v>
+        <v>1.25</v>
       </c>
       <c r="E4" t="n">
-        <v>55.1</v>
+        <v>60.6</v>
       </c>
       <c r="F4" t="n">
-        <v>54.1</v>
+        <v>57.1</v>
       </c>
       <c r="G4" t="n">
-        <v>54.6</v>
+        <v>58.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20.14</v>
+        <v>48.18</v>
       </c>
       <c r="D5" t="n">
-        <v>3.51</v>
+        <v>4.07</v>
       </c>
       <c r="E5" t="n">
-        <v>55.6</v>
+        <v>52.5</v>
       </c>
       <c r="F5" t="n">
-        <v>51</v>
+        <v>63.1</v>
       </c>
       <c r="G5" t="n">
-        <v>53.3</v>
+        <v>57.8</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>70.25</v>
+        <v>25.24</v>
       </c>
       <c r="D6" t="n">
-        <v>7.95</v>
+        <v>2.06</v>
       </c>
       <c r="E6" t="n">
-        <v>40.8</v>
+        <v>55.6</v>
       </c>
       <c r="F6" t="n">
-        <v>65.8</v>
+        <v>54</v>
       </c>
       <c r="G6" t="n">
-        <v>53.3</v>
+        <v>54.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="7">
@@ -636,112 +636,112 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>14.97</v>
+        <v>15.02</v>
       </c>
       <c r="D7" t="n">
         <v>1.22</v>
       </c>
       <c r="E7" t="n">
-        <v>54.1</v>
+        <v>55.6</v>
       </c>
       <c r="F7" t="n">
         <v>51.5</v>
       </c>
       <c r="G7" t="n">
-        <v>52.8</v>
+        <v>53.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>29.11</v>
+        <v>27.93</v>
       </c>
       <c r="D8" t="n">
-        <v>2.44</v>
+        <v>2.08</v>
       </c>
       <c r="E8" t="n">
-        <v>54.1</v>
+        <v>52.5</v>
       </c>
       <c r="F8" t="n">
-        <v>48.5</v>
+        <v>52</v>
       </c>
       <c r="G8" t="n">
-        <v>51.3</v>
+        <v>52.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27.83</v>
+        <v>29.11</v>
       </c>
       <c r="D9" t="n">
-        <v>2.07</v>
+        <v>2.44</v>
       </c>
       <c r="E9" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F9" t="n">
         <v>48.5</v>
       </c>
       <c r="G9" t="n">
-        <v>50.3</v>
+        <v>51.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>10.21</v>
+        <v>6.83</v>
       </c>
       <c r="D10" t="n">
-        <v>1.24</v>
+        <v>0.65</v>
       </c>
       <c r="E10" t="n">
-        <v>50.5</v>
+        <v>47.5</v>
       </c>
       <c r="F10" t="n">
-        <v>47.4</v>
+        <v>54.5</v>
       </c>
       <c r="G10" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="11">
@@ -756,202 +756,202 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>22.67</v>
+        <v>22.77</v>
       </c>
       <c r="D11" t="n">
         <v>1.86</v>
       </c>
       <c r="E11" t="n">
+        <v>52</v>
+      </c>
+      <c r="F11" t="n">
+        <v>46</v>
+      </c>
+      <c r="G11" t="n">
         <v>49</v>
       </c>
-      <c r="F11" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="G11" t="n">
-        <v>47.4</v>
-      </c>
       <c r="H11" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>19.71</v>
+        <v>19.88</v>
       </c>
       <c r="D12" t="n">
-        <v>1.77</v>
+        <v>3.46</v>
       </c>
       <c r="E12" t="n">
-        <v>54.1</v>
+        <v>48.5</v>
       </c>
       <c r="F12" t="n">
-        <v>37.2</v>
+        <v>41.9</v>
       </c>
       <c r="G12" t="n">
-        <v>45.7</v>
+        <v>45.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>47.02</v>
+        <v>10.48</v>
       </c>
       <c r="D13" t="n">
-        <v>3.98</v>
+        <v>0.98</v>
       </c>
       <c r="E13" t="n">
-        <v>35.7</v>
+        <v>37.4</v>
       </c>
       <c r="F13" t="n">
-        <v>52.6</v>
+        <v>47.5</v>
       </c>
       <c r="G13" t="n">
-        <v>44.1</v>
+        <v>42.4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13.84</v>
+        <v>19.46</v>
       </c>
       <c r="D14" t="n">
-        <v>1.3</v>
+        <v>1.62</v>
       </c>
       <c r="E14" t="n">
-        <v>41.8</v>
+        <v>44.4</v>
       </c>
       <c r="F14" t="n">
-        <v>40.8</v>
+        <v>38.4</v>
       </c>
       <c r="G14" t="n">
-        <v>41.3</v>
+        <v>41.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10.47</v>
+        <v>15.45</v>
       </c>
       <c r="D15" t="n">
-        <v>0.97</v>
+        <v>2.28</v>
       </c>
       <c r="E15" t="n">
-        <v>35.2</v>
+        <v>42.4</v>
       </c>
       <c r="F15" t="n">
-        <v>41.3</v>
+        <v>36.4</v>
       </c>
       <c r="G15" t="n">
-        <v>38.3</v>
+        <v>39.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15.38</v>
+        <v>19.59</v>
       </c>
       <c r="D16" t="n">
-        <v>2.27</v>
+        <v>1.76</v>
       </c>
       <c r="E16" t="n">
-        <v>40.3</v>
+        <v>39.4</v>
       </c>
       <c r="F16" t="n">
-        <v>31.6</v>
+        <v>33.3</v>
       </c>
       <c r="G16" t="n">
-        <v>36</v>
+        <v>36.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>16.62</v>
+        <v>13.59</v>
       </c>
       <c r="D17" t="n">
-        <v>0.92</v>
+        <v>1.28</v>
       </c>
       <c r="E17" t="n">
-        <v>32.7</v>
+        <v>35.4</v>
       </c>
       <c r="F17" t="n">
-        <v>33.7</v>
+        <v>35.9</v>
       </c>
       <c r="G17" t="n">
-        <v>33.2</v>
+        <v>35.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="18">
@@ -966,52 +966,52 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>17.24</v>
+        <v>17.25</v>
       </c>
       <c r="D18" t="n">
         <v>1.66</v>
       </c>
       <c r="E18" t="n">
-        <v>25.5</v>
+        <v>26.3</v>
       </c>
       <c r="F18" t="n">
-        <v>40.3</v>
+        <v>40.4</v>
       </c>
       <c r="G18" t="n">
-        <v>32.9</v>
+        <v>33.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>19.26</v>
+        <v>16.58</v>
       </c>
       <c r="D19" t="n">
-        <v>1.61</v>
+        <v>0.91</v>
       </c>
       <c r="E19" t="n">
-        <v>31.1</v>
+        <v>32.3</v>
       </c>
       <c r="F19" t="n">
-        <v>30.6</v>
+        <v>31.8</v>
       </c>
       <c r="G19" t="n">
-        <v>30.9</v>
+        <v>32.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="20">
@@ -1026,382 +1026,382 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29.84</v>
+        <v>30.18</v>
       </c>
       <c r="D20" t="n">
-        <v>2.3</v>
+        <v>2.33</v>
       </c>
       <c r="E20" t="n">
-        <v>25.5</v>
+        <v>27.3</v>
       </c>
       <c r="F20" t="n">
-        <v>28.6</v>
+        <v>33.3</v>
       </c>
       <c r="G20" t="n">
-        <v>27.7</v>
+        <v>30.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>29.22</v>
+        <v>22.9</v>
       </c>
       <c r="D21" t="n">
-        <v>2.77</v>
+        <v>2.11</v>
       </c>
       <c r="E21" t="n">
-        <v>24.5</v>
+        <v>30.3</v>
       </c>
       <c r="F21" t="n">
-        <v>27</v>
+        <v>29.8</v>
       </c>
       <c r="G21" t="n">
-        <v>26.3</v>
+        <v>29.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21.49</v>
+        <v>20.76</v>
       </c>
       <c r="D22" t="n">
-        <v>1.95</v>
+        <v>3.45</v>
       </c>
       <c r="E22" t="n">
-        <v>24.5</v>
+        <v>30.3</v>
       </c>
       <c r="F22" t="n">
-        <v>24.5</v>
+        <v>29.3</v>
       </c>
       <c r="G22" t="n">
-        <v>24.5</v>
+        <v>29.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>19.81</v>
+        <v>21.67</v>
       </c>
       <c r="D23" t="n">
-        <v>3.28</v>
+        <v>1.97</v>
       </c>
       <c r="E23" t="n">
-        <v>23.5</v>
+        <v>25.3</v>
       </c>
       <c r="F23" t="n">
-        <v>23.5</v>
+        <v>27.3</v>
       </c>
       <c r="G23" t="n">
-        <v>23.5</v>
+        <v>26.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.62</v>
+        <v>33.67</v>
       </c>
       <c r="D24" t="n">
-        <v>2.09</v>
+        <v>1.86</v>
       </c>
       <c r="E24" t="n">
-        <v>19.4</v>
+        <v>25.3</v>
       </c>
       <c r="F24" t="n">
-        <v>19.9</v>
+        <v>22.2</v>
       </c>
       <c r="G24" t="n">
-        <v>19.7</v>
+        <v>23.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>79.27</v>
+        <v>25.13</v>
       </c>
       <c r="D25" t="n">
-        <v>3.63</v>
+        <v>2.36</v>
       </c>
       <c r="E25" t="n">
-        <v>13.3</v>
+        <v>19.2</v>
       </c>
       <c r="F25" t="n">
-        <v>19.4</v>
+        <v>24.2</v>
       </c>
       <c r="G25" t="n">
-        <v>17.6</v>
+        <v>22.7</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>24.53</v>
+        <v>29.01</v>
       </c>
       <c r="D26" t="n">
-        <v>2.3</v>
+        <v>2.75</v>
       </c>
       <c r="E26" t="n">
-        <v>15.3</v>
+        <v>20.2</v>
       </c>
       <c r="F26" t="n">
-        <v>18.4</v>
+        <v>23.2</v>
       </c>
       <c r="G26" t="n">
-        <v>17.4</v>
+        <v>22.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>54.58</v>
+        <v>29.77</v>
       </c>
       <c r="D27" t="n">
-        <v>3.52</v>
+        <v>3.25</v>
       </c>
       <c r="E27" t="n">
-        <v>17.3</v>
+        <v>19.2</v>
       </c>
       <c r="F27" t="n">
-        <v>17.3</v>
+        <v>21.2</v>
       </c>
       <c r="G27" t="n">
-        <v>17.3</v>
+        <v>20.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29.08</v>
+        <v>36.19</v>
       </c>
       <c r="D28" t="n">
-        <v>3.17</v>
+        <v>3.14</v>
       </c>
       <c r="E28" t="n">
-        <v>15.3</v>
+        <v>17.2</v>
       </c>
       <c r="F28" t="n">
-        <v>16.8</v>
+        <v>21.7</v>
       </c>
       <c r="G28" t="n">
-        <v>16.4</v>
+        <v>20.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>10.1</v>
+        <v>55.74</v>
       </c>
       <c r="D29" t="n">
-        <v>0.65</v>
+        <v>3.59</v>
       </c>
       <c r="E29" t="n">
-        <v>16.3</v>
+        <v>19.2</v>
       </c>
       <c r="F29" t="n">
-        <v>16.3</v>
+        <v>19.2</v>
       </c>
       <c r="G29" t="n">
-        <v>16.3</v>
+        <v>19.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.57</v>
+        <v>80.18000000000001</v>
       </c>
       <c r="D30" t="n">
-        <v>1.46</v>
+        <v>3.68</v>
       </c>
       <c r="E30" t="n">
-        <v>16.3</v>
+        <v>14.1</v>
       </c>
       <c r="F30" t="n">
-        <v>16.3</v>
+        <v>20.2</v>
       </c>
       <c r="G30" t="n">
-        <v>16.3</v>
+        <v>18.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>35.06</v>
+        <v>19.82</v>
       </c>
       <c r="D31" t="n">
-        <v>3.04</v>
+        <v>1.48</v>
       </c>
       <c r="E31" t="n">
-        <v>10.2</v>
+        <v>17.2</v>
       </c>
       <c r="F31" t="n">
-        <v>14.8</v>
+        <v>18.2</v>
       </c>
       <c r="G31" t="n">
-        <v>13.4</v>
+        <v>17.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>31.87</v>
+        <v>10.14</v>
       </c>
       <c r="D32" t="n">
-        <v>1.76</v>
+        <v>0.65</v>
       </c>
       <c r="E32" t="n">
-        <v>7.1</v>
+        <v>17.2</v>
       </c>
       <c r="F32" t="n">
-        <v>4.6</v>
+        <v>16.7</v>
       </c>
       <c r="G32" t="n">
-        <v>5.4</v>
+        <v>16.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Aug  6 11:51:58 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -477,691 +477,691 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>28.92</v>
+        <v>73.89</v>
       </c>
       <c r="D2" t="n">
-        <v>2.68</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>72.7</v>
+        <v>64</v>
       </c>
       <c r="F2" t="n">
-        <v>75.3</v>
+        <v>73</v>
       </c>
       <c r="G2" t="n">
-        <v>74</v>
+        <v>68.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>73.48</v>
+        <v>28.54</v>
       </c>
       <c r="D3" t="n">
-        <v>8.32</v>
+        <v>2.64</v>
       </c>
       <c r="E3" t="n">
-        <v>60.6</v>
+        <v>62</v>
       </c>
       <c r="F3" t="n">
-        <v>71.7</v>
+        <v>67.5</v>
       </c>
       <c r="G3" t="n">
-        <v>66.2</v>
+        <v>64.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801780.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.28</v>
+        <v>6.87</v>
       </c>
       <c r="D4" t="n">
-        <v>1.25</v>
+        <v>0.65</v>
       </c>
       <c r="E4" t="n">
-        <v>60.6</v>
+        <v>65</v>
       </c>
       <c r="F4" t="n">
-        <v>57.1</v>
+        <v>54.5</v>
       </c>
       <c r="G4" t="n">
-        <v>58.8</v>
+        <v>59.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>48.18</v>
+        <v>17.98</v>
       </c>
       <c r="D5" t="n">
-        <v>4.07</v>
+        <v>1.73</v>
       </c>
       <c r="E5" t="n">
-        <v>52.5</v>
+        <v>46</v>
       </c>
       <c r="F5" t="n">
-        <v>63.1</v>
+        <v>63.5</v>
       </c>
       <c r="G5" t="n">
-        <v>57.8</v>
+        <v>54.8</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>25.24</v>
+        <v>28.02</v>
       </c>
       <c r="D6" t="n">
-        <v>2.06</v>
+        <v>2.09</v>
       </c>
       <c r="E6" t="n">
-        <v>55.6</v>
+        <v>54</v>
       </c>
       <c r="F6" t="n">
-        <v>54</v>
+        <v>53.5</v>
       </c>
       <c r="G6" t="n">
-        <v>54.8</v>
+        <v>53.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>15.02</v>
+        <v>47.81</v>
       </c>
       <c r="D7" t="n">
-        <v>1.22</v>
+        <v>4.04</v>
       </c>
       <c r="E7" t="n">
-        <v>55.6</v>
+        <v>46</v>
       </c>
       <c r="F7" t="n">
-        <v>51.5</v>
+        <v>59</v>
       </c>
       <c r="G7" t="n">
-        <v>53.5</v>
+        <v>52.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>27.93</v>
+        <v>14.94</v>
       </c>
       <c r="D8" t="n">
-        <v>2.08</v>
+        <v>1.22</v>
       </c>
       <c r="E8" t="n">
-        <v>52.5</v>
+        <v>52</v>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>51.5</v>
       </c>
       <c r="G8" t="n">
-        <v>52.3</v>
+        <v>51.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>29.11</v>
+        <v>24.76</v>
       </c>
       <c r="D9" t="n">
-        <v>2.44</v>
+        <v>2.02</v>
       </c>
       <c r="E9" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F9" t="n">
-        <v>48.5</v>
+        <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>51.3</v>
+        <v>50.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801780.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6.83</v>
+        <v>19.58</v>
       </c>
       <c r="D10" t="n">
-        <v>0.65</v>
+        <v>1.64</v>
       </c>
       <c r="E10" t="n">
-        <v>47.5</v>
+        <v>48.5</v>
       </c>
       <c r="F10" t="n">
-        <v>54.5</v>
+        <v>43.5</v>
       </c>
       <c r="G10" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="11">
